<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-14
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$Y$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$AF$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y31"/>
+  <dimension ref="A1:AF31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -496,6 +496,13 @@
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="11" customWidth="1" min="24" max="24"/>
     <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="29" max="29"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
+    <col width="11" customWidth="1" min="31" max="31"/>
+    <col width="11" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -622,6 +629,41 @@
       <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300_4W</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>风险度</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>动量</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>DS信号</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>B距今</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>S距今</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>急杀</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>周线档</t>
         </is>
       </c>
     </row>
@@ -679,6 +721,23 @@
       <c r="Y2" s="2" t="n">
         <v>-7.43</v>
       </c>
+      <c r="Z2" s="2" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="AA2" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -730,6 +789,21 @@
       <c r="Y3" s="2" t="n">
         <v>2.78</v>
       </c>
+      <c r="Z3" s="2" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="AA3" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -783,6 +857,21 @@
       <c r="Y4" s="2" t="n">
         <v>3.22</v>
       </c>
+      <c r="Z4" s="2" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="AA4" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -841,6 +930,21 @@
       </c>
       <c r="Y5" s="2" t="n">
         <v>19.84</v>
+      </c>
+      <c r="Z5" s="2" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="AA5" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -893,6 +997,23 @@
       <c r="Y6" s="2" t="n">
         <v>-8.76</v>
       </c>
+      <c r="Z6" s="2" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="AA6" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -944,6 +1065,21 @@
       <c r="Y7" s="2" t="n">
         <v>2.4</v>
       </c>
+      <c r="Z7" s="2" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="AA7" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -995,6 +1131,21 @@
       <c r="Y8" s="2" t="n">
         <v>-2.43</v>
       </c>
+      <c r="Z8" s="2" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="AA8" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1057,6 +1208,27 @@
       </c>
       <c r="Y9" s="2" t="n">
         <v>7.46</v>
+      </c>
+      <c r="Z9" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="AA9" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="2" t="inlineStr"/>
+      <c r="AF9" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1109,6 +1281,21 @@
       <c r="Y10" s="2" t="n">
         <v>2.5</v>
       </c>
+      <c r="Z10" s="2" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="AA10" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AE10" s="2" t="inlineStr"/>
+      <c r="AF10" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1161,6 +1348,23 @@
       </c>
       <c r="Y11" s="2" t="n">
         <v>-3.06</v>
+      </c>
+      <c r="Z11" s="2" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="AA11" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1215,6 +1419,21 @@
       <c r="Y12" s="2" t="n">
         <v>5.48</v>
       </c>
+      <c r="Z12" s="2" t="n">
+        <v>78.7</v>
+      </c>
+      <c r="AA12" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="inlineStr"/>
+      <c r="AE12" s="2" t="inlineStr"/>
+      <c r="AF12" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1266,6 +1485,21 @@
       <c r="Y13" s="2" t="n">
         <v>-0.92</v>
       </c>
+      <c r="Z13" s="2" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="AA13" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AD13" s="2" t="inlineStr"/>
+      <c r="AE13" s="2" t="inlineStr"/>
+      <c r="AF13" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1318,6 +1552,23 @@
       </c>
       <c r="Y14" s="2" t="n">
         <v>-2.13</v>
+      </c>
+      <c r="Z14" s="2" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="AA14" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE14" s="2" t="inlineStr"/>
+      <c r="AF14" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1373,6 +1624,23 @@
       </c>
       <c r="Y15" s="2" t="n">
         <v>5.54</v>
+      </c>
+      <c r="Z15" s="2" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="AA15" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="inlineStr"/>
+      <c r="AF15" s="2" t="inlineStr">
+        <is>
+          <t>背离</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1429,6 +1697,21 @@
       <c r="Y16" s="2" t="n">
         <v>0.02</v>
       </c>
+      <c r="Z16" s="2" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="AA16" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="inlineStr"/>
+      <c r="AF16" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1482,6 +1765,23 @@
       <c r="Y17" s="2" t="n">
         <v>-13.25</v>
       </c>
+      <c r="Z17" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="AA17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="AD17" s="2" t="inlineStr"/>
+      <c r="AE17" s="2" t="inlineStr"/>
+      <c r="AF17" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1535,6 +1835,23 @@
       <c r="Y18" s="2" t="n">
         <v>10.89</v>
       </c>
+      <c r="Z18" s="2" t="n">
+        <v>100.1</v>
+      </c>
+      <c r="AA18" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AD18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE18" s="2" t="inlineStr"/>
+      <c r="AF18" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1588,6 +1905,21 @@
       <c r="Y19" s="2" t="n">
         <v>-0.75</v>
       </c>
+      <c r="Z19" s="2" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="AA19" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="AB19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AD19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="inlineStr"/>
+      <c r="AF19" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1641,6 +1973,21 @@
       <c r="Y20" s="2" t="n">
         <v>-1.14</v>
       </c>
+      <c r="Z20" s="2" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="AA20" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AE20" s="2" t="inlineStr"/>
+      <c r="AF20" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1695,6 +2042,23 @@
       </c>
       <c r="Y21" s="2" t="n">
         <v>-7.74</v>
+      </c>
+      <c r="Z21" s="2" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="AA21" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="AD21" s="2" t="inlineStr"/>
+      <c r="AE21" s="2" t="inlineStr"/>
+      <c r="AF21" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -1747,6 +2111,27 @@
       <c r="Y22" s="2" t="n">
         <v>-4.43</v>
       </c>
+      <c r="Z22" s="2" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="AA22" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="AB22" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="2" t="inlineStr"/>
+      <c r="AE22" s="2" t="inlineStr"/>
+      <c r="AF22" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1798,6 +2183,23 @@
       <c r="Y23" s="2" t="n">
         <v>-4.52</v>
       </c>
+      <c r="Z23" s="2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="AA23" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD23" s="2" t="inlineStr"/>
+      <c r="AE23" s="2" t="inlineStr"/>
+      <c r="AF23" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1849,6 +2251,27 @@
       <c r="Y24" s="2" t="n">
         <v>-3.75</v>
       </c>
+      <c r="Z24" s="2" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="AA24" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="AB24" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="2" t="inlineStr"/>
+      <c r="AE24" s="2" t="inlineStr"/>
+      <c r="AF24" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1901,6 +2324,21 @@
       </c>
       <c r="Y25" s="2" t="n">
         <v>-7.15</v>
+      </c>
+      <c r="Z25" s="2" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="AA25" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="AB25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AD25" s="2" t="inlineStr"/>
+      <c r="AE25" s="2" t="inlineStr"/>
+      <c r="AF25" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1953,6 +2391,19 @@
       <c r="Y26" s="2" t="n">
         <v>-5.1</v>
       </c>
+      <c r="Z26" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="AA26" s="2" t="inlineStr"/>
+      <c r="AB26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="inlineStr"/>
+      <c r="AD26" s="2" t="inlineStr"/>
+      <c r="AE26" s="2" t="inlineStr"/>
+      <c r="AF26" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2006,6 +2457,23 @@
       <c r="Y27" s="2" t="n">
         <v>-9.890000000000001</v>
       </c>
+      <c r="Z27" s="2" t="n">
+        <v>-7</v>
+      </c>
+      <c r="AA27" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="AB27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="AD27" s="2" t="inlineStr"/>
+      <c r="AE27" s="2" t="inlineStr"/>
+      <c r="AF27" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2055,6 +2523,23 @@
       <c r="Y28" s="2" t="n">
         <v>0.09</v>
       </c>
+      <c r="Z28" s="2" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="AA28" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="AB28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD28" s="2" t="inlineStr"/>
+      <c r="AE28" s="2" t="inlineStr"/>
+      <c r="AF28" s="2" t="inlineStr">
+        <is>
+          <t>无背离</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2104,6 +2589,23 @@
       <c r="Y29" s="2" t="n">
         <v>-5.38</v>
       </c>
+      <c r="Z29" s="2" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="AA29" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="AD29" s="2" t="inlineStr"/>
+      <c r="AE29" s="2" t="inlineStr"/>
+      <c r="AF29" s="2" t="inlineStr">
+        <is>
+          <t>背离</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2153,6 +2655,21 @@
       <c r="Y30" s="2" t="n">
         <v>5.27</v>
       </c>
+      <c r="Z30" s="2" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="AA30" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AD30" s="2" t="inlineStr"/>
+      <c r="AE30" s="2" t="inlineStr"/>
+      <c r="AF30" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2202,9 +2719,24 @@
       <c r="Y31" s="2" t="n">
         <v>5.32</v>
       </c>
+      <c r="Z31" s="2" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="AA31" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="AB31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AD31" s="2" t="inlineStr"/>
+      <c r="AE31" s="2" t="inlineStr"/>
+      <c r="AF31" s="2" t="inlineStr">
+        <is>
+          <t>柱≥0</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y1"/>
+  <autoFilter ref="A1:AF1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2215,7 +2747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2265,206 +2797,276 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>【② 趋势尾声 — 背离】</t>
+          <t>【⑥ 东吴风险趋势信号】(逆向复现v2, 最右7列)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  周KDJ背离/周MACD背离/周RSI背离: 价格新低(底背离)或新高(顶背离) vs 指标未新低/新高。周KDJ背离用J为指标且要求两极值点J&lt;10(底)/J&gt;90(顶)。过滤: 第二极值时效(周线近4周/日线近10日, 过期清除), 价差&gt;2%, 间距≥4根</t>
+          <t xml:space="preserve">  风险度: KDJ(75,20,15)J线(精确复现)。&lt;20超卖区, &gt;85超买区, &lt;0超跌勿接飞刀, &gt;100超涨易暴涨暴跌</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    波动率取消: 价格从第二极值沿背离方向走 &gt;6×20日收益标准差 → 视为已兑现→取消(银行低波~7%到位, 高波股~30%到位, 自适应)</t>
+          <t xml:space="preserve">  动量: 综合动量TREND(ztanh近似,R²=0.96)。&gt;50偏多; 历史不足1217根K线为空</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    反向取代: 若底/顶背离同时存在, 取第二极值更晚的那个(后来者取代前者)</t>
+          <t xml:space="preserve">  DS信号: B=底右强买(TR&lt;20且短期动量↑且济安线拐头) / b=底左早买(济安线未拐,动量&gt;50) /</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  日MACD背离/日RSI背离: 同上周线规则但日线级别, min_spacing=22, 无极值区约束</t>
+          <t xml:space="preserve">           S=顶右强卖(TR&gt;85且济安线↓且动量&lt;40) / s=顶左早卖。信号收盘确认,无重绘</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  周度背离: 周KDJ/MACD/RSI任一背离 → +1底/-1顶/±1双向。周J超卖(&lt;20)不显示顶背离; 超买(&gt;80)不显示底背离</t>
+          <t xml:space="preserve">  B距今/S距今: 最近一次买/卖信号距今天数(15日内,超龄留空) — B距今≤5为可操作窗口</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  日度背离: 日KDJ/MACD/RSI任一背离 → +1底/-1顶/±1双向</t>
+          <t xml:space="preserve">  急杀: 近10日跌量&gt;涨量 且 3/5/10/15日均线无纠缠 = 恐慌宣泄型底部(胜率+4pp;</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           仅A股/美股有效, HK/ETF留空)。回测: B+急杀 A股68.6%/中位+10.3% (2016-2026)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>【② 趋势尾声 — DeMark TD Sequential】</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  周线档: 上一完整周周线MACD状态。无背离=新鲜急杀(最优) / 背离=拖尾阴跌(A股降权,</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  周度DeMark / 日度DeMark: +9=买方setup完成(近8日/4周内, 非瞬时); +13=买方countdown完成(setup后数到13根 收盘&lt;2根前低, 近4周/8日内完成, 底反转); -9/-13=卖方对称(顶反转)。正=买方, 负=卖方</t>
+          <t xml:space="preserve">           美股反而加分) / 柱≥0=牛回调。回测口径: B进S出, 详见 D:/Project/risk_trend_model</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>【② 趋势尾声 — 背离】</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>【③ 多空平衡】(1=命中, 空=未命中)</t>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  周KDJ背离/周MACD背离/周RSI背离: 价格新低(底背离)或新高(顶背离) vs 指标未新低/新高。周KDJ背离用J为指标且要求两极值点J&lt;10(底)/J&gt;90(顶)。过滤: 第二极值时效(周线近4周/日线近10日, 过期清除), 价差&gt;2%, 间距≥4根</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  十字星(3d): 近3日十字星个数。十字星=实体/振幅≤10% 且 振幅/开盘≥0.5%(经典十字星), 或 实体绝对值≤0.02(价≥5)/≤0.01(价&lt;5)(小实体)</t>
+          <t xml:space="preserve">    波动率取消: 价格从第二极值沿背离方向走 &gt;6×20日收益标准差 → 视为已兑现→取消(银行低波~7%到位, 高波股~30%到位, 自适应)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  涨放量跌缩量: 近10日≥2上涨日且≥1下跌日; 上涨日均量≥1.5×下跌日均量; 且每个下跌日成交量&lt;当日20日量均(持续缩量)。多头承接信号</t>
+          <t xml:space="preserve">    反向取代: 若底/顶背离同时存在, 取第二极值更晚的那个(后来者取代前者)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置(位置门前): {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。位置门 = A OR B。A: 200日pos&lt;=0.80(200日数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5% 且距250日收盘高点回落≥5%(创新高处的平台突破归新高, 不算SOS)。仙股过滤: 信号K线收盘&lt;0.5(本币)不触发。强度: 放量+RS超额+阳线。捕获纠缠平台突破、次新股底部反强</t>
+          <t xml:space="preserve">  日MACD背离/日RSI背离: 同上周线规则但日线级别, min_spacing=22, 无极值区约束</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=2x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
+          <t xml:space="preserve">  周度背离: 周KDJ/MACD/RSI任一背离 → +1底/-1顶/±1双向。周J超卖(&lt;20)不显示顶背离; 超买(&gt;80)不显示底背离</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SOS: 仅最新一根K线命中阳线路径 → 1 (当日新鲜信号)</t>
+          <t xml:space="preserve">  日度背离: 日KDJ/MACD/RSI任一背离 → +1底/-1顶/±1双向</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SOS 过去3天: 最新一根之前的3根(不含最新)任一根命中信号 且 通过3日确认 → 1。确认=信号后已过交易日(至多3根): ①收盘未跌破信号K线OLC均值(O+L+C)/3的2%以内 ②回调日(OHLC均价较信号收盘跌&gt;=2%)成交量&lt;=信号日量60%, 上涨日不限量。与SOS独立, 可同时为1</t>
-        </is>
-      </c>
+      <c r="A25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>【② 趋势尾声 — DeMark TD Sequential】</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>【④ 企稳上行 — Cross】</t>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  周度DeMark / 日度DeMark: +9=买方setup完成(近8日/4周内, 非瞬时); +13=买方countdown完成(setup后数到13根 收盘&lt;2根前低, 近4周/8日内完成, 底反转); -9/-13=卖方对称(顶反转)。正=买方, 负=卖方</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
-        </is>
-      </c>
+      <c r="A28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>【③ 多空平衡】(1=命中, 空=未命中)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
+          <t xml:space="preserve">  十字星(3d): 近3日十字星个数。十字星=实体/振幅≤10% 且 振幅/开盘≥0.5%(经典十字星), 或 实体绝对值≤0.02(价≥5)/≤0.01(价&lt;5)(小实体)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
+          <t xml:space="preserve">  涨放量跌缩量: 近10日≥2上涨日且≥1下跌日; 上涨日均量≥1.5×下跌日均量; 且每个下跌日成交量&lt;当日20日量均(持续缩量)。多头承接信号</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
+          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置(位置门前): {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。位置门 = A OR B。A: 200日pos&lt;=0.80(200日数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5% 且距250日收盘高点回落≥5%(创新高处的平台突破归新高, 不算SOS)。仙股过滤: 信号K线收盘&lt;0.5(本币)不触发。强度: 放量+RS超额+阳线。捕获纠缠平台突破、次新股底部反强</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=2x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    有过零但不稳定(whipsaw/暴涨驱动等脏交叉) → 0; 无过零但两线持续重叠(近5日rel&lt;0.2%) → 0; 其余空</t>
+          <t xml:space="preserve">  SOS: 仅最新一根K线命中阳线路径 → 1 (当日新鲜信号)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr"/>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SOS 过去3天: 最新一根之前的3根(不含最新)任一根命中信号 且 通过3日确认 → 1。确认=信号后已过交易日(至多3根): ①收盘未跌破信号K线OLC均值(O+L+C)/3的2%以内 ②回调日(OHLC均价较信号收盘跌&gt;=2%)成交量&lt;=信号日量60%, 上涨日不限量。与SOS独立, 可同时为1</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>【⑤ ETF 专属 — 趋势/Mansfield RS】</t>
-        </is>
-      </c>
+      <c r="A36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>【④ 企稳上行 — Cross】</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
+          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    有过零但不稳定(whipsaw/暴涨驱动等脏交叉) → 0; 无过零但两线持续重叠(近5日rel&lt;0.2%) → 0; 其余空</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>【⑤ ETF 专属 — 趋势/Mansfield RS】</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  MRS_沪深300_1W / MRS_沪深300_4W: MRS_沪深300 分数的 5日 / 20日 变化</t>
         </is>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-15
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.304</v>
+        <v>3.268</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -708,26 +708,26 @@
       </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>9.539999999999999</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>0.93</v>
+        <v>0.46</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-1.53</v>
+        <v>-1.15</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-9.33</v>
+        <v>-9.06</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>2.9</v>
+        <v>1.6</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -740,19 +740,19 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.462</v>
+        <v>0.654</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>99.02</v>
+        <v>90.17</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -762,38 +762,40 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-13.08</v>
+        <v>-30.96</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-1.26</v>
+        <v>-8.81</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>0.01</v>
+        <v>-1.23</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>3.84</v>
+        <v>5.22</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>79</v>
+        <v>78.2</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -808,62 +810,68 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.657</v>
+        <v>1.787</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>90.17</v>
+        <v>101.36</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S4" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T4" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-30.67</v>
+        <v>49.76</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-9.109999999999999</v>
+        <v>30.57</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-1.09</v>
+        <v>5.1</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>5.83</v>
+        <v>21.59</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>79.7</v>
+        <v>97.5</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
@@ -878,70 +886,64 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.778</v>
+        <v>0.822</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>101.36</v>
+        <v>4.26</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>48.7</v>
+        <v>-10.42</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>29.23</v>
+        <v>0.79</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>9.01</v>
+        <v>-0.49</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>21.78</v>
+        <v>-3.89</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>95.3</v>
+        <v>59.2</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
         <is>
@@ -952,19 +954,19 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.83</v>
+        <v>2.958</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4.26</v>
+        <v>55.83</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -974,133 +976,145 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R6" s="2" t="inlineStr"/>
       <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-10.79</v>
+        <v>-3.87</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.01</v>
+        <v>1.87</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>1.11</v>
+        <v>0.47</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>-4.17</v>
+        <v>3.34</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>61.1</v>
+        <v>50.5</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="n">
-        <v>11</v>
-      </c>
+      <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.976</v>
+        <v>3.382</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>55.83</v>
+        <v>114.34</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L7" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="n">
+      <c r="R7" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-3.9</v>
+        <v>11</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.82</v>
+        <v>11.71</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.77</v>
+        <v>0.36</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>3.46</v>
+        <v>7.53</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>53.9</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7.598</v>
+        <v>0.501</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>33.48</v>
+        <v>6.73</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1110,36 +1124,36 @@
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>9.199999999999999</v>
+        <v>-17.86</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.73</v>
+        <v>-4.16</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.8</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-2.83</v>
+        <v>4.88</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>19.8</v>
+        <v>43.4</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr"/>
@@ -1147,84 +1161,72 @@
       <c r="AE8" s="2" t="inlineStr"/>
       <c r="AF8" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.404</v>
+        <v>0.369</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>114.34</v>
+        <v>89.56999999999999</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="n">
         <v>-9</v>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S9" s="2" t="inlineStr"/>
-      <c r="T9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>11.05</v>
+        <v>-10.54</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>11.74</v>
+        <v>1.02</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>2.56</v>
+        <v>0.08</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>9.039999999999999</v>
+        <v>-0.9</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>99.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr">
@@ -1236,19 +1238,19 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.503</v>
+        <v>0.779</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>6.73</v>
+        <v>79.75</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1272,22 +1274,22 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-17.65</v>
+        <v>-13.89</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-4.51</v>
+        <v>-2.97</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-1.26</v>
+        <v>-0</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>3.69</v>
+        <v>7.35</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>46.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
@@ -1302,19 +1304,19 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.372</v>
+        <v>0.332</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>89.56999999999999</v>
+        <v>98.59</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1340,27 +1342,27 @@
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-11.02</v>
+        <v>-9.43</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>1.1</v>
+        <v>1.03</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.86</v>
+        <v>0.09</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>-0.41</v>
+        <v>1.45</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>69.2</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
       <c r="AD11" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr">
@@ -1372,19 +1374,19 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.785</v>
+        <v>1.139</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>79.75</v>
+        <v>33.19</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1394,63 +1396,71 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N12" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="n">
+      <c r="R12" s="2" t="n">
         <v>-1</v>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-13.82</v>
+        <v>-1.24</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-2.93</v>
+        <v>-6.72</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-0.27</v>
+        <v>0.6</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>6.72</v>
+        <v>4.33</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>75.7</v>
+        <v>37.8</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
-      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.033</v>
+        <v>1.024</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>40.26</v>
+        <v>-3.59</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1462,41 +1472,39 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S13" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>2.9</v>
+        <v>32.3</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>0.22</v>
+        <v>11.57</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-0.03</v>
+        <v>-0.5</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-15.58</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>35.2</v>
+        <v>-7.2</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
-      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="AD13" s="2" t="inlineStr"/>
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="inlineStr">
@@ -1508,19 +1516,19 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.334</v>
+        <v>0.843</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>98.59</v>
+        <v>99.92</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1529,44 +1537,46 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-10.05</v>
+        <v>0.95</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>0.86</v>
+        <v>10.13</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>1.58</v>
+        <v>3.14</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>1.68</v>
+        <v>12.26</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>74.40000000000001</v>
+        <v>100.9</v>
       </c>
       <c r="AA14" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
@@ -1578,19 +1588,19 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.149</v>
+        <v>1.023</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>33.19</v>
+        <v>11.5</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1601,7 +1611,7 @@
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="n">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>2</v>
@@ -1610,61 +1620,59 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
+          <t>预1</t>
         </is>
       </c>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-1.06</v>
+        <v>-56.37</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-6.58</v>
+        <v>-19.46</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>2</v>
+        <v>1.08</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>4.59</v>
+        <v>0.36</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>37.2</v>
+        <v>42.1</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
-      <c r="AC15" s="2" t="n">
-        <v>11</v>
-      </c>
+      <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.412</v>
+        <v>2.196</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>80.06</v>
+        <v>85.05</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1674,40 +1682,38 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N16" s="2" t="n">
         <v>3</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S16" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-47.56</v>
+        <v>21.06</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-15.31</v>
+        <v>16.83</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-1.73</v>
+        <v>0.26</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>3.96</v>
+        <v>2.8</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>61.2</v>
+        <v>26.2</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
@@ -1715,94 +1721,108 @@
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.856</v>
+        <v>1.483</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>99.92</v>
+        <v>12.11</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N17" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="n">
-        <v>1</v>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>0.91</v>
+        <v>-28.55</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>11.1</v>
+        <v>-14.26</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>5.01</v>
+        <v>-1.32</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>14.36</v>
+        <v>-6.35</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>101.3</v>
+        <v>6.7</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>85</v>
+        <v>20</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
-      <c r="AC17" s="2" t="inlineStr"/>
-      <c r="AD17" s="2" t="n">
-        <v>3</v>
-      </c>
+      <c r="AC17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="AD17" s="2" t="inlineStr"/>
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.012</v>
+        <v>1.011</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>11.5</v>
+        <v>24.85</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1812,65 +1832,65 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-58.2</v>
+        <v>51.91</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-20.98</v>
+        <v>18.88</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-1.83</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-0.64</v>
+        <v>-8.289999999999999</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>43.7</v>
+        <v>17.5</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
-      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2.191</v>
+        <v>1.27</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>85.05</v>
+        <v>117.45</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1880,40 +1900,36 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>20.67</v>
+        <v>15.64</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>15.92</v>
+        <v>13.58</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-0.52</v>
+        <v>-0.6</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>0.41</v>
+        <v>5.32</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>26.8</v>
+        <v>67.3</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
@@ -1921,96 +1937,100 @@
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.506</v>
+        <v>0.787</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>12.11</v>
+        <v>35.77</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-28.9</v>
+        <v>-27.6</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-13.51</v>
+        <v>-16.28</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-1.18</v>
+        <v>-1.27</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-6.16</v>
+        <v>-5.37</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>8.1</v>
+        <v>8.5</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.016</v>
+        <v>0.653</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>24.85</v>
+        <v>26.58</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2022,40 +2042,38 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R21" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>52.45</v>
+        <v>49.65</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>18.86</v>
+        <v>16.47</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-2.48</v>
+        <v>-1.38</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-10.08</v>
+        <v>-7.57</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>17.6</v>
+        <v>19.9</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="inlineStr"/>
@@ -2068,19 +2086,19 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.273</v>
+        <v>2.299</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>117.45</v>
+        <v>10.28</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -2090,7 +2108,9 @@
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
       </c>
@@ -2099,27 +2119,25 @@
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>15.02</v>
+        <v>-30.34</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>13.19</v>
+        <v>-15.42</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>2.13</v>
+        <v>-0.22</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>6.46</v>
+        <v>-6.38</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>68.40000000000001</v>
+        <v>5.1</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
@@ -2127,26 +2145,26 @@
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.793</v>
+        <v>1.638</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>35.77</v>
+        <v>-4.94</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -2156,40 +2174,44 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N23" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="n">
-        <v>1</v>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>-28.63</v>
+        <v>17.81</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>-16.22</v>
+        <v>6.6</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-0.8</v>
+        <v>-0.52</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-4.64</v>
+        <v>-11.47</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>9.5</v>
+        <v>-9</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
@@ -2202,19 +2224,19 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.657</v>
+        <v>1.452</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>26.58</v>
+        <v>99.02</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -2231,60 +2253,54 @@
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R24" s="2" t="inlineStr"/>
       <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>50.3</v>
+        <v>-12.22</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>16.57</v>
+        <v>-1.21</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-2.14</v>
+        <v>0.23</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-9.140000000000001</v>
+        <v>3.58</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>19.9</v>
+        <v>76.8</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
-      <c r="AC24" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AC24" s="2" t="inlineStr"/>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2.324</v>
+        <v>4.523</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>10.28</v>
+        <v>10.81</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -2294,9 +2310,7 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
         <v>1</v>
       </c>
@@ -2308,49 +2322,51 @@
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>-31.17</v>
+        <v>-0.02</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-15.16</v>
+        <v>1.31</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-0.01</v>
+        <v>0.17</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-6.09</v>
+        <v>0.18</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>6.2</v>
+        <v>1.1</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.914</v>
+        <v>7.588</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>3.17</v>
+        <v>33.48</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -2367,58 +2383,54 @@
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S26" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-4.59</v>
+        <v>9.48</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-7.35</v>
+        <v>2.26</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-2.04</v>
+        <v>-0.38</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-4.6</v>
+        <v>-2.43</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA26" s="2" t="inlineStr"/>
+        <v>18.6</v>
+      </c>
+      <c r="AA26" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1.613</v>
+        <v>3.024</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>-4.94</v>
+        <v>40.26</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -2428,11 +2440,9 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
@@ -2442,27 +2452,25 @@
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>17.35</v>
+        <v>3.07</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>4.33</v>
+        <v>0.62</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-4.01</v>
+        <v>-0.25</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-13.54</v>
+        <v>-0.05</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>-8.300000000000001</v>
+        <v>34.6</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="AC27" s="2" t="inlineStr"/>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr">
@@ -2474,19 +2482,19 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>4.552</v>
+        <v>0.41</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>10.81</v>
+        <v>80.06</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2498,7 +2506,7 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
@@ -2508,32 +2516,30 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-0.2</v>
+        <v>-47.93</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>1.29</v>
+        <v>-15.06</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>0.27</v>
+        <v>-1.71</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>0.19</v>
+        <v>3.24</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>3.3</v>
+        <v>59.3</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2555,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.11</v>
+        <v>1.105</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>5.68</v>
@@ -2574,26 +2580,26 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-10.4</v>
+        <v>-10.31</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-6.81</v>
+        <v>-6.51</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-2.17</v>
+        <v>-0.77</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-4.25</v>
+        <v>-3.57</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>11.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AA29" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
@@ -2606,19 +2612,19 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.005</v>
+        <v>1.793</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-3.59</v>
+        <v>93.77</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2630,9 +2636,11 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O30" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="inlineStr"/>
@@ -2640,51 +2648,49 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>31.91</v>
+        <v>-20.76</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>8.869999999999999</v>
+        <v>-4.56</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-4.44</v>
+        <v>0.06</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-18.47</v>
+        <v>6.72</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-6.4</v>
+        <v>69.5</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.807</v>
+        <v>0.906</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>93.77</v>
+        <v>3.17</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2698,9 +2704,7 @@
       <c r="N31" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O31" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="inlineStr"/>
@@ -2708,30 +2712,28 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-21.6</v>
+        <v>-4.92</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-4.55</v>
+        <v>-7.51</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-1.16</v>
+        <v>-2.07</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>6.56</v>
+        <v>-6.41</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>73.59999999999999</v>
-      </c>
-      <c r="AA31" s="2" t="n">
-        <v>30</v>
-      </c>
+        <v>1.5</v>
+      </c>
+      <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2765,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-14 | 30 只</t>
+          <t>截至: 2026-09-15 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-16
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.268</v>
+        <v>3.33</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -700,34 +700,32 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>9.890000000000001</v>
+        <v>10.97</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>0.46</v>
+        <v>1.61</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-1.15</v>
+        <v>0.47</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-9.06</v>
+        <v>-4.24</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -749,7 +747,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.654</v>
+        <v>0.648</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>90.17</v>
@@ -772,30 +770,26 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T3" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-30.96</v>
+        <v>-31.49</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-8.81</v>
+        <v>-10.15</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-1.23</v>
+        <v>-1.85</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>5.22</v>
+        <v>2.13</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>78.2</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -819,7 +813,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.787</v>
+        <v>1.821</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>101.36</v>
@@ -842,36 +836,34 @@
         <v>-9</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>49.76</v>
+        <v>51.28</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>30.57</v>
+        <v>31.96</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>5.1</v>
+        <v>6.44</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>21.59</v>
+        <v>19.46</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>97.5</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
@@ -895,7 +887,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.822</v>
+        <v>0.826</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>4.26</v>
@@ -910,7 +902,7 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -922,27 +914,27 @@
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-10.42</v>
+        <v>-9.06</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>0.79</v>
+        <v>0.68</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-0.49</v>
+        <v>1.07</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>-3.89</v>
+        <v>-4.61</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>59.2</v>
+        <v>57.7</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
@@ -963,7 +955,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2.958</v>
+        <v>2.98</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>55.83</v>
@@ -985,27 +977,31 @@
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-3.87</v>
+        <v>-3.54</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.87</v>
+        <v>1.95</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>0.47</v>
+        <v>0.71</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>3.34</v>
+        <v>2.04</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>50.5</v>
+        <v>48.7</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
@@ -1020,40 +1016,28 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3.382</v>
+        <v>4.55</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>114.34</v>
+        <v>10.81</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
         <v>1</v>
@@ -1061,60 +1045,60 @@
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="n">
-        <v>-1</v>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>11</v>
+        <v>0.44</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>11.71</v>
+        <v>1.22</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.36</v>
+        <v>0.09</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>7.53</v>
+        <v>-0.03</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>97.40000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AC7" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.501</v>
+        <v>7.71</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>6.73</v>
+        <v>33.48</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1126,107 +1110,127 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>-17.86</v>
+        <v>10.55</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>-4.16</v>
+        <v>3.13</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-0.8</v>
+        <v>0.89</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>4.88</v>
+        <v>0.4</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>43.4</v>
+        <v>18.5</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="AB8" s="2" t="inlineStr"/>
-      <c r="AC8" s="2" t="inlineStr"/>
+        <v>58</v>
+      </c>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="AC8" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
       <c r="AF8" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.369</v>
+        <v>3.367</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>89.56999999999999</v>
+        <v>114.34</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="n">
         <v>-9</v>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R9" s="2" t="inlineStr"/>
       <c r="S9" s="2" t="inlineStr"/>
-      <c r="T9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>-10.54</v>
+        <v>10.65</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>1.02</v>
+        <v>10.4</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>0.08</v>
+        <v>-2.24</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-0.9</v>
+        <v>2.44</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>67.3</v>
+        <v>95.3</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="AB9" s="2" t="inlineStr"/>
+        <v>17</v>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr">
@@ -1238,19 +1242,19 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.779</v>
+        <v>0.503</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>79.75</v>
+        <v>6.73</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1262,34 +1266,36 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-13.89</v>
+        <v>-17.24</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-2.97</v>
+        <v>-4.35</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-0</v>
+        <v>-0.42</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>7.35</v>
+        <v>2.98</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>72.09999999999999</v>
+        <v>41.2</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
@@ -1304,19 +1310,19 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.332</v>
+        <v>0.369</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>98.59</v>
+        <v>89.56999999999999</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1342,27 +1348,27 @@
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-9.43</v>
+        <v>-9.42</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>1.03</v>
+        <v>0.42</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.09</v>
+        <v>1.08</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>1.45</v>
+        <v>-3.27</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>72.59999999999999</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
       <c r="AD11" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr">
@@ -1374,19 +1380,19 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1.139</v>
+        <v>0.78</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>33.19</v>
+        <v>79.75</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1396,71 +1402,65 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S12" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-1.24</v>
+        <v>-13.46</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-6.72</v>
+        <v>-3.43</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>0.6</v>
+        <v>-0.38</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>4.33</v>
+        <v>4.59</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>37.8</v>
+        <v>69</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
-      <c r="AC12" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1.024</v>
+        <v>3.082</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>-3.59</v>
+        <v>40.26</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1472,7 +1472,7 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
@@ -1484,27 +1484,25 @@
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>32.3</v>
+        <v>4.31</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>11.57</v>
+        <v>1.78</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-0.5</v>
+        <v>1.4</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>-15.58</v>
+        <v>3.38</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>-7.2</v>
+        <v>34.9</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
-      <c r="AC13" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="inlineStr">
@@ -1516,19 +1514,19 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.843</v>
+        <v>0.335</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>99.92</v>
+        <v>98.59</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1537,46 +1535,44 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>0.95</v>
+        <v>-7.95</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>10.13</v>
+        <v>1.29</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>3.14</v>
+        <v>1.82</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>12.26</v>
+        <v>1.26</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>100.9</v>
+        <v>71.5</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="AB14" s="2" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
@@ -1588,19 +1584,19 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.023</v>
+        <v>1.15</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>11.5</v>
+        <v>33.19</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1611,68 +1607,64 @@
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="n">
-        <v>9</v>
+        <v>-9</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-56.37</v>
+        <v>-1.2</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-19.46</v>
+        <v>-6.42</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>1.08</v>
+        <v>-0.29</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>0.36</v>
+        <v>6.69</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>42.1</v>
+        <v>39</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
-      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2.196</v>
+        <v>1.118</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>85.05</v>
+        <v>5.68</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1683,146 +1675,142 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="n">
-        <v>-13</v>
+        <v>9</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>21.06</v>
+        <v>-9.66</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>16.83</v>
+        <v>-6.04</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>0.26</v>
+        <v>0.75</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>2.8</v>
+        <v>-0.55</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>26.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
-      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.483</v>
+        <v>1.069</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>12.11</v>
+        <v>-3.59</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="n">
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="N17" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-28.55</v>
+        <v>34.14</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-14.26</v>
+        <v>15.51</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-1.32</v>
+        <v>4.46</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-6.35</v>
+        <v>-5.09</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>6.7</v>
+        <v>-6.9</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="AB17" s="2" t="inlineStr"/>
+        <v>73</v>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AC17" s="2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AD17" s="2" t="inlineStr"/>
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.011</v>
+        <v>0.839</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>24.85</v>
+        <v>99.92</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1834,7 +1822,7 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -1842,55 +1830,57 @@
       <c r="R18" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>51.91</v>
+        <v>1.14</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>18.88</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-1.83</v>
+        <v>1.8</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-8.289999999999999</v>
+        <v>6.36</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>17.5</v>
+        <v>100.1</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
-      <c r="AC18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AD18" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.27</v>
+        <v>1.015</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>117.45</v>
+        <v>11.5</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1900,36 +1890,36 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N19" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>15.64</v>
+        <v>-54.7</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>13.58</v>
+        <v>-20.5</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-0.6</v>
+        <v>1.14</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>5.32</v>
+        <v>-3.05</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>67.3</v>
+        <v>40.2</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
@@ -1944,93 +1934,89 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.787</v>
+        <v>1.796</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>35.77</v>
+        <v>93.77</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="n">
-        <v>-1</v>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-27.6</v>
+        <v>-19.59</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-16.28</v>
+        <v>-4.95</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-1.27</v>
+        <v>-0.17</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-5.37</v>
+        <v>4.21</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>8.5</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="AC20" s="2" t="inlineStr"/>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.653</v>
+        <v>2.218</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>26.58</v>
+        <v>85.05</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2040,41 +2026,43 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N21" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="n">
-        <v>-1</v>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>49.65</v>
+        <v>21.81</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>16.47</v>
+        <v>17.07</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-1.38</v>
+        <v>0.92</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-7.57</v>
+        <v>1.76</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>19.9</v>
+        <v>26.2</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
-      <c r="AC21" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AC21" s="2" t="inlineStr"/>
       <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="inlineStr"/>
       <c r="AF21" s="2" t="inlineStr">
@@ -2086,61 +2074,75 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2.299</v>
+        <v>1.484</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>10.28</v>
+        <v>12.11</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="n">
         <v>9</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-30.34</v>
+        <v>-27.12</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-15.42</v>
+        <v>-14.78</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.22</v>
+        <v>-1.56</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-6.38</v>
+        <v>-6.6</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>5.1</v>
+        <v>5.8</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="n">
+        <v>14</v>
+      </c>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
@@ -2152,19 +2154,19 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.638</v>
+        <v>1.05</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>-4.94</v>
+        <v>24.85</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -2174,44 +2176,44 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R23" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>17.81</v>
+        <v>52.5</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>6.6</v>
+        <v>22.4</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-0.52</v>
+        <v>1.14</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-11.47</v>
+        <v>2.3</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>-9</v>
+        <v>18.3</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="AB23" s="2" t="inlineStr"/>
+        <v>64</v>
+      </c>
+      <c r="AB23" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AC23" s="2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
@@ -2224,19 +2226,19 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.452</v>
+        <v>1.272</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>99.02</v>
+        <v>117.45</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -2255,25 +2257,27 @@
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="inlineStr"/>
       <c r="S24" s="2" t="inlineStr"/>
-      <c r="T24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-12.22</v>
+        <v>15.87</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-1.21</v>
+        <v>12.9</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>0.23</v>
+        <v>-4.24</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>3.58</v>
+        <v>1.12</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>76.8</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="inlineStr"/>
@@ -2288,56 +2292,64 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>4.523</v>
+        <v>0.798</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>10.81</v>
+        <v>35.77</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>-0.02</v>
+        <v>-25.09</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>1.31</v>
+        <v>-15.68</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>0.17</v>
+        <v>-0.21</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>0.18</v>
+        <v>-2.78</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>1.1</v>
+        <v>8</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="n">
@@ -2354,19 +2366,19 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>7.588</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>33.48</v>
+        <v>26.58</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -2376,37 +2388,51 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="V26" s="2" t="n">
-        <v>9.48</v>
+        <v>50.47</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>2.26</v>
+        <v>21.13</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-0.38</v>
+        <v>2.83</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-2.43</v>
+        <v>3.93</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>18.6</v>
+        <v>21</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="inlineStr"/>
+        <v>72</v>
+      </c>
+      <c r="AB26" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC26" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
@@ -2418,19 +2444,19 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>3.024</v>
+        <v>2.303</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>40.26</v>
+        <v>10.28</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -2440,9 +2466,11 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N27" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
@@ -2452,22 +2480,22 @@
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>3.07</v>
+        <v>-28.29</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>0.62</v>
+        <v>-15.87</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.25</v>
+        <v>-0.41</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-0.05</v>
+        <v>-5.82</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>34.6</v>
+        <v>4.3</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="inlineStr"/>
@@ -2475,26 +2503,26 @@
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.41</v>
+        <v>0.912</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>80.06</v>
+        <v>3.17</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2506,59 +2534,61 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-47.93</v>
+        <v>-4.84</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-15.06</v>
+        <v>-7.48</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-1.71</v>
+        <v>-0.9</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>3.24</v>
+        <v>-1.41</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="AA28" s="2" t="n">
-        <v>29</v>
-      </c>
+        <v>0.4</v>
+      </c>
+      <c r="AA28" s="2" t="inlineStr"/>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.105</v>
+        <v>1.708</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>5.68</v>
+        <v>-4.94</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2568,63 +2598,73 @@
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
-      <c r="S29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-10.31</v>
+        <v>19.64</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-6.51</v>
+        <v>10.31</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-0.77</v>
+        <v>4.24</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-3.57</v>
+        <v>-2.95</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>9.199999999999999</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="AA29" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="AB29" s="2" t="inlineStr"/>
+        <v>77</v>
+      </c>
+      <c r="AB29" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="AC29" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.793</v>
+        <v>1.451</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>93.77</v>
+        <v>99.02</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2638,9 +2678,7 @@
       <c r="N30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="inlineStr"/>
@@ -2648,22 +2686,22 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-20.76</v>
+        <v>-11.35</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-4.56</v>
+        <v>-1.91</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>0.06</v>
+        <v>0.17</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>6.72</v>
+        <v>0.1</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>69.5</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
@@ -2678,19 +2716,19 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.906</v>
+        <v>0.408</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>3.17</v>
+        <v>80.06</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2702,7 +2740,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2712,28 +2750,30 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-4.92</v>
+        <v>-48.28</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-7.51</v>
+        <v>-15.88</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-2.07</v>
+        <v>-1.21</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-6.41</v>
+        <v>1.45</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AA31" s="2" t="inlineStr"/>
+        <v>57.4</v>
+      </c>
+      <c r="AA31" s="2" t="n">
+        <v>31</v>
+      </c>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
@@ -2765,7 +2805,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-15 | 30 只</t>
+          <t>截至: 2026-09-16 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-17
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.33</v>
+        <v>3.319</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -702,30 +702,36 @@
       <c r="R2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>10.97</v>
+        <v>11.98</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>1.61</v>
+        <v>1.68</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>0.47</v>
+        <v>0.52</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-4.24</v>
+        <v>-4.39</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -747,7 +753,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.648</v>
+        <v>0.649</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>90.17</v>
@@ -774,22 +780,22 @@
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-31.49</v>
+        <v>-31.74</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-10.15</v>
+        <v>-9.5</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-1.85</v>
+        <v>-0.18</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>2.13</v>
+        <v>2.08</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>76.09999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -813,7 +819,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.821</v>
+        <v>1.772</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>101.36</v>
@@ -842,32 +848,38 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>51.28</v>
+        <v>51.18</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>31.96</v>
+        <v>28.82</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>6.44</v>
+        <v>1.84</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>19.46</v>
+        <v>16.65</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>99.90000000000001</v>
+        <v>100.5</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+        <v>56</v>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
@@ -887,7 +899,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.826</v>
+        <v>0.83</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>4.26</v>
@@ -902,39 +914,41 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-9.06</v>
+        <v>-7.97</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>0.68</v>
+        <v>1.71</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>1.07</v>
+        <v>3.41</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>-4.61</v>
+        <v>-8</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>57.7</v>
+        <v>56.6</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
@@ -955,7 +969,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2.98</v>
+        <v>2.958</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>55.83</v>
@@ -977,31 +991,27 @@
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R6" s="2" t="inlineStr"/>
       <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-3.54</v>
+        <v>-3.5</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.95</v>
+        <v>1.66</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>0.71</v>
+        <v>0.05</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>2.04</v>
+        <v>2.18</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>48.7</v>
+        <v>45.8</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
@@ -1025,7 +1035,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4.55</v>
+        <v>4.532</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>10.81</v>
@@ -1045,35 +1055,33 @@
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R7" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S7" s="2" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>0.44</v>
+        <v>0.8</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>-0.03</v>
+        <v>0.15</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>0.5</v>
+        <v>-0.3</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
@@ -1095,7 +1103,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7.71</v>
+        <v>7.681</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>33.48</v>
@@ -1122,30 +1130,26 @@
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>10.55</v>
+        <v>11.52</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>3.13</v>
+        <v>3.15</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.89</v>
+        <v>0.99</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>0.4</v>
+        <v>-0.22</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>18.5</v>
+        <v>18.2</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="AB8" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1167,7 +1171,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.367</v>
+        <v>3.347</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>114.34</v>
@@ -1194,7 +1198,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
@@ -1206,31 +1210,27 @@
       </c>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>10.65</v>
+        <v>10.41</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>10.4</v>
+        <v>10.19</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-2.24</v>
+        <v>-2.2</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>2.44</v>
+        <v>1.61</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>95.3</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="AA9" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="AB9" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.503</v>
+        <v>0.499</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>6.73</v>
@@ -1264,38 +1264,36 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N10" s="2" t="n">
         <v>3</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-17.24</v>
+        <v>-17.35</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-4.35</v>
+        <v>-4.61</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-0.42</v>
+        <v>-1.84</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>2.98</v>
+        <v>2.89</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>41.2</v>
+        <v>38.6</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
@@ -1319,7 +1317,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.369</v>
+        <v>0.372</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>89.56999999999999</v>
@@ -1341,34 +1339,36 @@
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-9.42</v>
+        <v>-8.58</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0.42</v>
+        <v>1.8</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>1.08</v>
+        <v>3.16</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>-3.27</v>
+        <v>-2.93</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>65.59999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
       <c r="AD11" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr">
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.78</v>
+        <v>0.773</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>79.75</v>
@@ -1402,38 +1402,36 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N12" s="2" t="n">
         <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R12" s="2" t="inlineStr"/>
       <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-13.46</v>
+        <v>-13.68</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-3.43</v>
+        <v>-3.82</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-0.38</v>
+        <v>-1.97</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>4.59</v>
+        <v>4.2</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>69</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1457,7 +1455,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.082</v>
+        <v>3.066</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>40.26</v>
@@ -1484,22 +1482,22 @@
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>4.31</v>
+        <v>5.35</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>1.78</v>
+        <v>1.68</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>1.4</v>
+        <v>1.38</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>3.38</v>
+        <v>2.59</v>
       </c>
       <c r="Z13" s="2" t="n">
         <v>34.9</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1523,7 +1521,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.335</v>
+        <v>0.337</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>98.59</v>
@@ -1545,34 +1543,38 @@
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="V14" s="2" t="n">
-        <v>-7.95</v>
+        <v>-6.86</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>1.29</v>
+        <v>2.39</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>1.82</v>
+        <v>3.46</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>1.26</v>
+        <v>-1.99</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>71.5</v>
+        <v>70.8</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
@@ -1593,7 +1595,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.15</v>
+        <v>1.142</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>33.19</v>
@@ -1610,36 +1612,42 @@
         <v>-9</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr"/>
-      <c r="T15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-1.2</v>
+        <v>-1.95</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-6.42</v>
+        <v>-6.64</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>-0.29</v>
+        <v>-1.04</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>6.69</v>
+        <v>7.34</v>
       </c>
       <c r="Z15" s="2" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="AA15" s="2" t="n">
         <v>39</v>
-      </c>
-      <c r="AA15" s="2" t="n">
-        <v>37</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
@@ -1661,7 +1669,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.118</v>
+        <v>1.114</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>5.68</v>
@@ -1692,26 +1700,26 @@
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-9.66</v>
+        <v>-9.32</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-6.04</v>
+        <v>-5.96</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>0.75</v>
+        <v>0.87</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-0.55</v>
+        <v>-0.5</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
@@ -1733,7 +1741,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.069</v>
+        <v>1.06</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>-3.59</v>
@@ -1762,30 +1770,26 @@
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>34.14</v>
+        <v>35.68</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>15.51</v>
+        <v>14.89</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>4.46</v>
+        <v>4.11</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-5.09</v>
+        <v>-4.3</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>-6.9</v>
+        <v>-6.8</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="AB17" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD17" s="2" t="inlineStr"/>
       <c r="AE17" s="2" t="inlineStr"/>
@@ -1807,7 +1811,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.839</v>
+        <v>0.837</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>99.92</v>
@@ -1836,27 +1840,27 @@
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>1.14</v>
+        <v>0.72</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>8.869999999999999</v>
+        <v>9.09</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>1.8</v>
+        <v>0.04</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>6.36</v>
+        <v>6.22</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>100.1</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
@@ -1877,7 +1881,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.015</v>
+        <v>1.003</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>11.5</v>
@@ -1899,27 +1903,29 @@
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-54.7</v>
+        <v>-54.15</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-20.5</v>
+        <v>-20.96</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>1.14</v>
+        <v>1.59</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-3.05</v>
+        <v>-4.82</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>40.2</v>
+        <v>37.8</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
@@ -1943,7 +1949,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.796</v>
+        <v>1.771</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>93.77</v>
@@ -1956,40 +1962,36 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N20" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O20" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-19.59</v>
+        <v>-19.48</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-4.95</v>
+        <v>-5.77</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-0.17</v>
+        <v>-1.81</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>4.21</v>
+        <v>2.89</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>65.90000000000001</v>
+        <v>61.1</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
@@ -2013,7 +2015,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.218</v>
+        <v>2.22</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>85.05</v>
@@ -2035,31 +2037,29 @@
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R21" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>21.81</v>
+        <v>22.49</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>17.07</v>
+        <v>17.57</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>0.92</v>
+        <v>1.69</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>1.76</v>
+        <v>1.81</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>26.2</v>
+        <v>29.1</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.484</v>
+        <v>1.483</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>12.11</v>
@@ -2091,57 +2091,45 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="n">
         <v>9</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-27.12</v>
+        <v>-24.59</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-14.78</v>
+        <v>-14.45</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-1.56</v>
+        <v>-0.44</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-6.6</v>
+        <v>-5.48</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>5.8</v>
+        <v>5.1</v>
       </c>
       <c r="AA22" s="2" t="n">
         <v>33</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
@@ -2163,7 +2151,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.05</v>
+        <v>1.044</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>24.85</v>
@@ -2176,9 +2164,11 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -2187,33 +2177,35 @@
         <v>1</v>
       </c>
       <c r="S23" s="2" t="inlineStr"/>
-      <c r="T23" s="2" t="inlineStr"/>
-      <c r="U23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="V23" s="2" t="n">
-        <v>52.5</v>
+        <v>53.46</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>22.4</v>
+        <v>22.03</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>1.14</v>
+        <v>1.29</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>2.3</v>
+        <v>1.01</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>18.3</v>
+        <v>19</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="AB23" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
@@ -2235,7 +2227,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.272</v>
+        <v>1.258</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>117.45</v>
@@ -2262,22 +2254,22 @@
       </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>15.87</v>
+        <v>16.92</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>12.9</v>
+        <v>12.05</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-4.24</v>
+        <v>-3.7</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>1.12</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>66.40000000000001</v>
+        <v>65</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="inlineStr"/>
@@ -2301,7 +2293,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.798</v>
+        <v>0.793</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>35.77</v>
@@ -2334,26 +2326,26 @@
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>-25.09</v>
+        <v>-22.83</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-15.68</v>
+        <v>-15.81</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-0.21</v>
+        <v>0.14</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-2.78</v>
+        <v>-3.24</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>8</v>
+        <v>7.4</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
@@ -2375,7 +2367,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.6860000000000001</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>26.58</v>
@@ -2402,36 +2394,30 @@
       </c>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="U26" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="V26" s="2" t="n">
-        <v>50.47</v>
+        <v>51.95</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>21.13</v>
+        <v>21.64</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>2.83</v>
+        <v>3.98</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>3.93</v>
+        <v>2.67</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>21</v>
+        <v>22.1</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="AB26" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
@@ -2453,7 +2439,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2.303</v>
+        <v>2.294</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>10.28</v>
@@ -2470,7 +2456,7 @@
         <v>9</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
@@ -2480,22 +2466,22 @@
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-28.29</v>
+        <v>-25.79</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-15.87</v>
+        <v>-15.85</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.41</v>
+        <v>-0.24</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-5.82</v>
+        <v>-5.1</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="inlineStr"/>
@@ -2519,7 +2505,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.912</v>
+        <v>0.916</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>3.17</v>
@@ -2534,33 +2520,35 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr">
+      <c r="R28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-4.84</v>
+        <v>-4.47</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-7.48</v>
+        <v>-6.62</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-0.9</v>
+        <v>1.01</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-1.41</v>
+        <v>-0.12</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>0.4</v>
+        <v>-0.4</v>
       </c>
       <c r="AA28" s="2" t="inlineStr"/>
       <c r="AB28" s="2" t="inlineStr"/>
@@ -2585,7 +2573,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.708</v>
+        <v>1.696</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>-4.94</v>
@@ -2616,26 +2604,26 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>19.64</v>
+        <v>21.18</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>10.31</v>
+        <v>9.94</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>4.24</v>
+        <v>4.14</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-2.95</v>
+        <v>-1.99</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>-8.199999999999999</v>
+        <v>-7.7</v>
       </c>
       <c r="AA29" s="2" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>B</t>
         </is>
       </c>
       <c r="AC29" s="2" t="n">
@@ -2661,7 +2649,7 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.451</v>
+        <v>1.441</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>99.02</v>
@@ -2676,7 +2664,7 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2686,22 +2674,22 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-11.35</v>
+        <v>-11</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-1.91</v>
+        <v>-2.15</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>0.17</v>
+        <v>0.32</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>0.1</v>
+        <v>-1.28</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>74.59999999999999</v>
+        <v>72</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
@@ -2750,22 +2738,22 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-48.28</v>
+        <v>-48</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-15.88</v>
+        <v>-15.36</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-1.21</v>
+        <v>0.29</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>1.45</v>
+        <v>1.69</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>57.4</v>
+        <v>55.7</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
@@ -2805,7 +2793,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-16 | 30 只</t>
+          <t>截至: 2026-09-17 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-18
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.319</v>
+        <v>3.391</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -708,30 +708,26 @@
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>11.98</v>
+        <v>13.01</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>1.68</v>
+        <v>2.73</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>0.52</v>
+        <v>1.29</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-4.39</v>
+        <v>-4.06</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="AB2" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -744,19 +740,19 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.649</v>
+        <v>1.452</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>90.17</v>
+        <v>93.48999999999999</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -766,36 +762,36 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
         <v>3</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-31.74</v>
+        <v>-11</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-9.5</v>
+        <v>-2.37</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-0.18</v>
+        <v>-0.11</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>2.08</v>
+        <v>-1.55</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>74.2</v>
+        <v>70.3</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -810,76 +806,66 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.772</v>
+        <v>0.652</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>101.36</v>
+        <v>90.17</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="n">
-        <v>-9</v>
+        <v>13</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="n">
-        <v>-1</v>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>51.18</v>
+        <v>-31.57</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>28.82</v>
+        <v>-9.92</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>1.84</v>
+        <v>-0.23</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>16.65</v>
+        <v>3.36</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>100.5</v>
+        <v>72.8</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="AB4" s="2" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
@@ -890,65 +876,77 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.83</v>
+        <v>1.742</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4.26</v>
+        <v>101.26</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N5" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>预1</t>
+          <t>预-1</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-7.97</v>
+        <v>50.68</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>1.71</v>
+        <v>25.16</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>3.41</v>
+        <v>-2.01</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>-8</v>
+        <v>12.3</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>56.6</v>
+        <v>100.1</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
@@ -960,19 +958,19 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2.958</v>
+        <v>0.835</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>55.83</v>
+        <v>4.26</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -982,63 +980,67 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-3.5</v>
+        <v>-6.51</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.66</v>
+        <v>1.33</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>0.05</v>
+        <v>4.31</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>2.18</v>
+        <v>-2.92</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>45.8</v>
+        <v>55.9</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="n">
+        <v>15</v>
+      </c>
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4.532</v>
+        <v>2.975</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>10.81</v>
+        <v>55.83</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -1048,41 +1050,43 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="n">
-        <v>1</v>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S7" s="2" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>0.8</v>
+        <v>-3.21</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.28</v>
+        <v>1.19</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.11</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.15</v>
+        <v>2.09</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>-0.3</v>
+        <v>44.2</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="n">
-        <v>8</v>
-      </c>
+      <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr">
@@ -1094,19 +1098,19 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7.681</v>
+        <v>4.582</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>33.48</v>
+        <v>10.81</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1126,30 +1130,38 @@
       <c r="R8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>11.52</v>
+        <v>1.28</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>3.15</v>
+        <v>1.3</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.99</v>
+        <v>0.09</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-0.22</v>
+        <v>0.18</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>18.2</v>
+        <v>0.1</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="AB8" s="2" t="inlineStr"/>
+        <v>57</v>
+      </c>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="AC8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1162,40 +1174,28 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.347</v>
+        <v>7.83</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>114.34</v>
+        <v>28.85</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1203,72 +1203,88 @@
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr"/>
-      <c r="T9" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>10.41</v>
+        <v>12.89</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>10.19</v>
+        <v>4.01</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-2.2</v>
+        <v>2.73</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>1.61</v>
+        <v>1.23</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>92.90000000000001</v>
+        <v>19</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="AB9" s="2" t="inlineStr"/>
-      <c r="AC9" s="2" t="inlineStr"/>
-      <c r="AD9" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.499</v>
+        <v>3.339</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>6.73</v>
+        <v>114.34</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L10" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
@@ -1278,26 +1294,28 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-17.35</v>
+        <v>10.07</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-4.61</v>
+        <v>8.76</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-1.84</v>
+        <v>-2.77</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>2.89</v>
+        <v>0.61</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>38.6</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
         <is>
@@ -1308,19 +1326,19 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.372</v>
+        <v>0.505</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>89.56999999999999</v>
+        <v>6.73</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1329,47 +1347,45 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N11" s="2" t="n">
         <v>3</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr">
+      <c r="R11" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
+      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-8.58</v>
+        <v>-16.49</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>1.8</v>
+        <v>-4.39</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>3.16</v>
+        <v>0.28</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>-2.93</v>
+        <v>3.54</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>64.5</v>
+        <v>37.1</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
-      <c r="AD11" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="AD11" s="2" t="inlineStr"/>
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr">
         <is>
@@ -1380,19 +1396,19 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.773</v>
+        <v>0.373</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>79.75</v>
+        <v>12.91</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1401,10 +1417,10 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L12" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
         <v>3</v>
       </c>
@@ -1416,26 +1432,28 @@
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-13.68</v>
+        <v>-7.6</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-3.82</v>
+        <v>1.09</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-1.97</v>
+        <v>2.66</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>4.2</v>
+        <v>0.01</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>65.09999999999999</v>
+        <v>63.6</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
-      <c r="AD12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="n">
+        <v>14</v>
+      </c>
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="inlineStr">
         <is>
@@ -1446,19 +1464,19 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.066</v>
+        <v>0.781</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>40.26</v>
+        <v>79.75</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1468,36 +1486,40 @@
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="n">
-        <v>1</v>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>5.35</v>
+        <v>-13.4</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>1.68</v>
+        <v>-3.78</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>1.38</v>
+        <v>-0.51</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>2.59</v>
+        <v>4.08</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>34.9</v>
+        <v>62.7</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1505,26 +1527,26 @@
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.337</v>
+        <v>3.129</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>98.59</v>
+        <v>43.79</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1533,72 +1555,66 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
-      <c r="S14" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-6.86</v>
+        <v>6.99</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>2.39</v>
+        <v>2.7</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>3.46</v>
+        <v>3.75</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>-1.99</v>
+        <v>3.92</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>70.8</v>
+        <v>36</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
-      <c r="AD14" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.142</v>
+        <v>0.34</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>33.19</v>
+        <v>40.85</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1607,12 +1623,12 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="n">
+      <c r="L15" s="2" t="n">
         <v>-9</v>
       </c>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
@@ -1620,59 +1636,61 @@
       <c r="R15" s="2" t="inlineStr"/>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
+          <t>预1</t>
         </is>
       </c>
       <c r="T15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-1.95</v>
+        <v>-5.06</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-6.64</v>
+        <v>2.34</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>-1.04</v>
+        <v>4.33</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>7.34</v>
+        <v>1.35</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>39.6</v>
+        <v>70.8</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
-      <c r="AC15" s="2" t="n">
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.114</v>
+        <v>1.16</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>5.68</v>
+        <v>33.19</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1682,11 +1700,9 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -1697,29 +1713,31 @@
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-9.32</v>
+        <v>-2.29</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-5.96</v>
+        <v>-6.15</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>0.87</v>
+        <v>-0.35</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-0.5</v>
+        <v>7.46</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>7.2</v>
+        <v>41</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
@@ -1732,19 +1750,19 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.06</v>
+        <v>0.411</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-3.59</v>
+        <v>76.56999999999999</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1756,65 +1774,63 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S17" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>35.68</v>
+        <v>-47.45</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>14.89</v>
+        <v>-15.48</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>4.11</v>
+        <v>0.54</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-4.3</v>
+        <v>3.28</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>-6.8</v>
+        <v>54.7</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
-      <c r="AC17" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AC17" s="2" t="inlineStr"/>
       <c r="AD17" s="2" t="inlineStr"/>
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.837</v>
+        <v>1.134</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>99.92</v>
+        <v>5.68</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1824,7 +1840,9 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N18" s="2" t="n">
         <v>2</v>
       </c>
@@ -1832,59 +1850,65 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S18" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>0.72</v>
+        <v>-8.18</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>9.09</v>
+        <v>-5.26</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>0.04</v>
+        <v>2.16</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>6.22</v>
+        <v>0.87</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>99.09999999999999</v>
+        <v>7.3</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="AB18" s="2" t="inlineStr"/>
-      <c r="AC18" s="2" t="inlineStr"/>
-      <c r="AD18" s="2" t="n">
-        <v>2</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="AC18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.003</v>
+        <v>1.1</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>11.5</v>
+        <v>-3.59</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1894,65 +1918,67 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-54.15</v>
+        <v>38.59</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-20.96</v>
+        <v>17.79</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>1.59</v>
+        <v>7.7</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-4.82</v>
+        <v>-1.05</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>37.8</v>
+        <v>-5.8</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
-      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.771</v>
+        <v>0.835</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>93.77</v>
+        <v>99.92</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1962,40 +1988,44 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-19.48</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-5.77</v>
+        <v>7.71</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-1.81</v>
+        <v>-1.5</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>2.89</v>
+        <v>5.71</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>61.1</v>
+        <v>98</v>
       </c>
       <c r="AA20" s="2" t="n">
         <v>25</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
@@ -2006,19 +2036,19 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.22</v>
+        <v>1.014</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>85.05</v>
+        <v>-2.39</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2027,12 +2057,14 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M21" s="2" t="n">
-        <v>-13</v>
+        <v>9</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -2040,26 +2072,30 @@
       <c r="R21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>22.49</v>
+        <v>-53.95</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>17.57</v>
+        <v>-20.8</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>1.69</v>
+        <v>0.59</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>1.81</v>
+        <v>-3.42</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>29.1</v>
+        <v>36.3</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2067,26 +2103,26 @@
       <c r="AE21" s="2" t="inlineStr"/>
       <c r="AF21" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.483</v>
+        <v>1.799</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>12.11</v>
+        <v>93.77</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -2100,61 +2136,63 @@
         <v>9</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-24.59</v>
+        <v>-18.78</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-14.45</v>
+        <v>-5.19</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.44</v>
+        <v>-0.26</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-5.48</v>
+        <v>3.21</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>5.1</v>
+        <v>58.5</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AC22" s="2" t="inlineStr"/>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.044</v>
+        <v>2.269</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>24.85</v>
+        <v>78.59</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -2164,11 +2202,9 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -2176,37 +2212,31 @@
       <c r="R23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S23" s="2" t="inlineStr"/>
-      <c r="T23" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="U23" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>53.46</v>
+        <v>22.67</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>22.03</v>
+        <v>18.78</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>1.29</v>
+        <v>2.98</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>1.01</v>
+        <v>4.63</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>19</v>
+        <v>33.7</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
@@ -2218,19 +2248,19 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.258</v>
+        <v>1.503</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>117.45</v>
+        <v>12.11</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -2240,79 +2270,85 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N24" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr"/>
-      <c r="T24" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>16.92</v>
+        <v>-22.67</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>12.05</v>
+        <v>-14.2</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-3.7</v>
+        <v>0.97</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>-6.07</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="AB24" s="2" t="inlineStr"/>
-      <c r="AC24" s="2" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="AB24" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="AC24" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.793</v>
+        <v>1.07</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>35.77</v>
+        <v>25.84</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N25" s="2" t="n">
         <v>2</v>
       </c>
@@ -2323,29 +2359,33 @@
         <v>1</v>
       </c>
       <c r="S25" s="2" t="inlineStr"/>
-      <c r="T25" s="2" t="inlineStr"/>
-      <c r="U25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V25" s="2" t="n">
-        <v>-22.83</v>
+        <v>54.36</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-15.81</v>
+        <v>23.5</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>0.14</v>
+        <v>1.61</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-3.24</v>
+        <v>0.3</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>7.4</v>
+        <v>20.3</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
@@ -2358,33 +2398,37 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>26.58</v>
+        <v>20.09</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
@@ -2392,32 +2436,36 @@
       <c r="R26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>51.95</v>
+        <v>-20.74</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>21.64</v>
+        <v>-14.36</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>3.98</v>
+        <v>2.43</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>2.67</v>
+        <v>-1.59</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>22.1</v>
+        <v>8</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="AB26" s="2" t="inlineStr"/>
+        <v>76</v>
+      </c>
+      <c r="AB26" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="AC26" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
@@ -2430,19 +2478,19 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2.294</v>
+        <v>0.704</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>10.28</v>
+        <v>30.88</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -2453,62 +2501,68 @@
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="n">
-        <v>9</v>
+        <v>-13</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
-      <c r="U27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V27" s="2" t="n">
-        <v>-25.79</v>
+        <v>53.33</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-15.85</v>
+        <v>23.27</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.24</v>
+        <v>4.11</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-5.1</v>
+        <v>2.95</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>3.5</v>
+        <v>23.8</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.916</v>
+        <v>2.334</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>3.17</v>
+        <v>10.28</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2518,16 +2572,16 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N28" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R28" s="2" t="inlineStr"/>
       <c r="S28" s="2" t="inlineStr">
         <is>
           <t>预1</t>
@@ -2536,23 +2590,31 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-4.47</v>
+        <v>-23.84</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-6.62</v>
+        <v>-15.31</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>1.01</v>
+        <v>1.11</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-0.12</v>
+        <v>-5.28</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="AA28" s="2" t="inlineStr"/>
-      <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="inlineStr"/>
+        <v>3.4</v>
+      </c>
+      <c r="AA28" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="AB28" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="AC28" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
@@ -2564,19 +2626,19 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.696</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>-4.94</v>
+        <v>3.17</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2586,11 +2648,9 @@
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2604,55 +2664,47 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>21.18</v>
+        <v>-3.38</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>9.94</v>
+        <v>-5.76</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>4.14</v>
+        <v>2.65</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-1.99</v>
+        <v>0.65</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>-7.7</v>
-      </c>
-      <c r="AA29" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="AB29" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="AC29" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>-0.3</v>
+      </c>
+      <c r="AA29" s="2" t="inlineStr"/>
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="inlineStr"/>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.441</v>
+        <v>1.744</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>99.02</v>
+        <v>-4.94</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2662,61 +2714,71 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N30" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
-      <c r="S30" s="2" t="inlineStr"/>
-      <c r="T30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-11</v>
+        <v>23.73</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-2.15</v>
+        <v>11.75</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>0.32</v>
+        <v>6.39</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-1.28</v>
+        <v>0.53</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>72</v>
+        <v>-6.3</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.408</v>
+        <v>1.249</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>80.06</v>
+        <v>117.45</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2728,7 +2790,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2738,22 +2800,22 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-48</v>
+        <v>17.3</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-15.36</v>
+        <v>10</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>0.29</v>
+        <v>-4.24</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>1.69</v>
+        <v>-1.36</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>55.7</v>
+        <v>63.8</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
@@ -2793,7 +2855,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-17 | 30 只</t>
+          <t>截至: 2026-09-18 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-21
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.391</v>
+        <v>3.418</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -694,40 +694,42 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
       <c r="S2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>13.01</v>
+        <v>14.07</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>2.73</v>
+        <v>2.76</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>1.29</v>
+        <v>1.83</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-4.06</v>
+        <v>-2.1</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+        <v>78</v>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -749,7 +751,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.452</v>
+        <v>1.462</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>93.48999999999999</v>
@@ -764,7 +766,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -772,26 +774,30 @@
       <c r="R3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-11</v>
+        <v>-11.1</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-2.37</v>
+        <v>-2.4</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-0.11</v>
+        <v>-1.14</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>-1.55</v>
+        <v>-1.15</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>70.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -815,7 +821,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.652</v>
+        <v>0.658</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>90.17</v>
@@ -837,31 +843,29 @@
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-31.57</v>
+        <v>-31.18</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-9.92</v>
+        <v>-9.619999999999999</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-0.23</v>
+        <v>-0.51</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>3.36</v>
+        <v>2.35</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>72.8</v>
+        <v>72.3</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
@@ -885,7 +889,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.742</v>
+        <v>1.748</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>101.26</v>
@@ -910,7 +914,7 @@
         <v>-9</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -918,35 +922,33 @@
       <c r="R5" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="S5" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>50.68</v>
+        <v>49.79</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>25.16</v>
+        <v>24.56</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-2.01</v>
+        <v>-4.68</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>12.3</v>
+        <v>10.78</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>100.1</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
@@ -967,7 +969,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.835</v>
+        <v>0.869</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>4.26</v>
@@ -982,42 +984,40 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="T6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-6.51</v>
+        <v>-5.42</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.33</v>
+        <v>4.78</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>4.31</v>
+        <v>3.77</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>-2.92</v>
+        <v>4.27</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>55.9</v>
+        <v>57.1</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr">
         <is>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.975</v>
+        <v>3.002</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>55.83</v>
@@ -1059,31 +1059,33 @@
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-3.21</v>
+        <v>-2.57</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.19</v>
+        <v>1.39</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-0.11</v>
+        <v>-0.44</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>2.09</v>
+        <v>1.51</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>44.2</v>
+        <v>44.3</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
@@ -1107,7 +1109,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.582</v>
+        <v>4.608</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>10.81</v>
@@ -1130,38 +1132,32 @@
       <c r="R8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="S8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>1.28</v>
+        <v>1.97</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.3</v>
+        <v>1.15</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>0.18</v>
+        <v>-0.05</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>0.1</v>
+        <v>1.1</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="AB8" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1183,7 +1179,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.83</v>
+        <v>7.872</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>28.85</v>
@@ -1198,44 +1194,40 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R9" s="2" t="inlineStr"/>
       <c r="S9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>12.89</v>
+        <v>14.28</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>4.01</v>
+        <v>3.77</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>2.73</v>
+        <v>2.04</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>1.23</v>
+        <v>1.44</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>19</v>
+        <v>20.1</v>
       </c>
       <c r="AA9" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="AB9" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+      <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
@@ -1257,7 +1249,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.339</v>
+        <v>3.385</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>114.34</v>
@@ -1289,32 +1281,36 @@
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>10.07</v>
+        <v>10.49</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>8.76</v>
+        <v>9.42</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-2.77</v>
+        <v>-2.31</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>0.61</v>
+        <v>-1.76</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>90.40000000000001</v>
+        <v>89.3</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
@@ -1335,7 +1331,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.505</v>
+        <v>0.51</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>6.73</v>
@@ -1357,31 +1353,33 @@
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr">
+      <c r="R11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-16.49</v>
+        <v>-15.14</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-4.39</v>
+        <v>-4.06</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.28</v>
+        <v>0.45</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>3.54</v>
+        <v>2.3</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>37.1</v>
+        <v>36.6</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1405,7 +1403,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.373</v>
+        <v>0.386</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>12.91</v>
@@ -1422,37 +1420,41 @@
       </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr"/>
-      <c r="T12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-7.6</v>
+        <v>-6.37</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>1.09</v>
+        <v>3.89</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>2.66</v>
+        <v>2.79</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>0.01</v>
+        <v>4.67</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>63.6</v>
+        <v>64.7</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="inlineStr">
@@ -1473,7 +1475,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.781</v>
+        <v>0.788</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>79.75</v>
@@ -1495,31 +1497,33 @@
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr">
+      <c r="R13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-13.4</v>
+        <v>-12.62</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-3.78</v>
+        <v>-3.54</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-0.51</v>
+        <v>-0.61</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>4.08</v>
+        <v>1.79</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>62.7</v>
+        <v>61.7</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1543,7 +1547,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>3.129</v>
+        <v>3.149</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>43.79</v>
@@ -1558,33 +1562,33 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R14" s="2" t="inlineStr"/>
       <c r="S14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>6.99</v>
+        <v>8.4</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>2.7</v>
+        <v>2.56</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>3.75</v>
+        <v>2.34</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>3.92</v>
+        <v>3.87</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>36</v>
+        <v>37.3</v>
       </c>
       <c r="AA14" s="2" t="n">
         <v>78</v>
@@ -1611,7 +1615,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.34</v>
+        <v>0.348</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>40.85</v>
@@ -1634,10 +1638,8 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="S15" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="T15" s="2" t="n">
         <v>0</v>
@@ -1646,27 +1648,27 @@
         <v>-1</v>
       </c>
       <c r="V15" s="2" t="n">
-        <v>-5.06</v>
+        <v>-3.52</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>2.34</v>
+        <v>3.97</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>4.33</v>
+        <v>3.11</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>1.35</v>
+        <v>4.67</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>70.8</v>
+        <v>72.2</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr">
@@ -1687,7 +1689,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.16</v>
+        <v>1.176</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>33.19</v>
@@ -1707,38 +1709,32 @@
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R16" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-2.29</v>
+        <v>-1.4</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-6.15</v>
+        <v>-5.52</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-0.35</v>
+        <v>1.06</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>7.46</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
-      <c r="AC16" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AC16" s="2" t="inlineStr"/>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr">
@@ -1759,7 +1755,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.411</v>
+        <v>0.416</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>76.56999999999999</v>
@@ -1779,31 +1775,33 @@
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr">
+      <c r="R17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-47.45</v>
+        <v>-46.79</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-15.48</v>
+        <v>-14.94</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>0.54</v>
+        <v>0.38</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>3.28</v>
+        <v>2.24</v>
       </c>
       <c r="Z17" s="2" t="n">
         <v>54.7</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
@@ -1827,7 +1825,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.134</v>
+        <v>1.142</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>5.68</v>
@@ -1844,7 +1842,7 @@
         <v>9</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -1852,38 +1850,32 @@
       <c r="R18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S18" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="S18" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-8.18</v>
+        <v>-7.11</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-5.26</v>
+        <v>-5.23</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>2.16</v>
+        <v>1.59</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>0.87</v>
+        <v>2.03</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>7.3</v>
+        <v>7.9</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="AB18" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
@@ -1905,7 +1897,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.1</v>
+        <v>1.102</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>-3.59</v>
@@ -1920,40 +1912,38 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="inlineStr"/>
-      <c r="S19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>38.59</v>
+        <v>41.51</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>17.79</v>
+        <v>16.97</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>7.7</v>
+        <v>8.09</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-1.05</v>
+        <v>1.02</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>-5.8</v>
+        <v>-4.7</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
@@ -1975,7 +1965,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.835</v>
+        <v>0.839</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>99.92</v>
@@ -1995,36 +1985,38 @@
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.52</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>7.71</v>
+        <v>7.46</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-1.5</v>
+        <v>-3.63</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>5.71</v>
+        <v>2.62</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>98</v>
+        <v>97.3</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
       <c r="AD20" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
@@ -2045,7 +2037,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.014</v>
+        <v>1.03</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>-2.39</v>
@@ -2064,7 +2056,7 @@
         <v>9</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -2080,22 +2072,22 @@
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-53.95</v>
+        <v>-53.63</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-20.8</v>
+        <v>-19.99</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>0.59</v>
+        <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-3.42</v>
+        <v>-0.15</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>36.3</v>
+        <v>35.7</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2119,7 +2111,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.799</v>
+        <v>1.809</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>93.77</v>
@@ -2136,36 +2128,34 @@
         <v>9</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R22" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-18.78</v>
+        <v>-17.97</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-5.19</v>
+        <v>-5.25</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.26</v>
+        <v>-0.7</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>3.21</v>
+        <v>1.86</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>58.5</v>
+        <v>56.7</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
@@ -2189,7 +2179,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.269</v>
+        <v>2.283</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>78.59</v>
@@ -2204,7 +2194,7 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -2215,25 +2205,27 @@
       <c r="S23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>22.67</v>
+        <v>22.66</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>18.78</v>
+        <v>18.53</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>2.98</v>
+        <v>2.61</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>4.63</v>
+        <v>4.58</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>33.7</v>
+        <v>38.5</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="inlineStr"/>
@@ -2257,7 +2249,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.503</v>
+        <v>1.504</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>12.11</v>
@@ -2280,38 +2272,30 @@
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-22.67</v>
+        <v>-20.8</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-14.2</v>
+        <v>-14.72</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>0.97</v>
+        <v>-1.21</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-6.07</v>
+        <v>-7.06</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="AB24" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
@@ -2333,7 +2317,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.07</v>
+        <v>1.081</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>25.84</v>
@@ -2350,42 +2334,40 @@
         <v>-13</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="V25" s="2" t="n">
-        <v>54.36</v>
+        <v>55.6</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>23.5</v>
+        <v>23.63</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>1.61</v>
+        <v>4.77</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>0.3</v>
+        <v>4.79</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>20.3</v>
+        <v>21.7</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
@@ -2398,35 +2380,31 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>1.282</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>20.09</v>
+        <v>117.45</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N26" s="2" t="n">
         <v>1</v>
       </c>
@@ -2436,108 +2414,106 @@
       <c r="R26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-20.74</v>
+        <v>18.96</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-14.36</v>
+        <v>12.01</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>2.43</v>
+        <v>-1.18</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-1.59</v>
+        <v>-3.38</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>8</v>
+        <v>64.3</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>76</v>
-      </c>
-      <c r="AB26" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
-      <c r="AC26" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="AB26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.704</v>
+        <v>0.82</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>30.88</v>
+        <v>20.09</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T27" s="2" t="inlineStr"/>
-      <c r="U27" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>53.33</v>
+        <v>-18.76</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>23.27</v>
+        <v>-14.41</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>4.11</v>
+        <v>1.81</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>2.95</v>
+        <v>-1.65</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>23.8</v>
+        <v>8.9</v>
       </c>
       <c r="AA27" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="AB27" s="2" t="inlineStr"/>
+      <c r="AB27" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AC27" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
@@ -2550,19 +2526,19 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2.334</v>
+        <v>0.712</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>10.28</v>
+        <v>30.88</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2573,72 +2549,66 @@
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="n">
-        <v>9</v>
+        <v>-13</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
-      <c r="U28" s="2" t="inlineStr"/>
+      <c r="U28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V28" s="2" t="n">
-        <v>-23.84</v>
+        <v>55.02</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-15.31</v>
+        <v>23.54</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>1.11</v>
+        <v>6.97</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-5.28</v>
+        <v>7.24</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>3.4</v>
+        <v>25.6</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="AB28" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.9340000000000001</v>
+        <v>2.335</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>3.17</v>
+        <v>10.28</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2650,37 +2620,39 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R29" s="2" t="inlineStr"/>
       <c r="S29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-3.38</v>
+        <v>-21.95</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-5.76</v>
+        <v>-15.76</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>2.65</v>
+        <v>-0.6</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>0.65</v>
+        <v>-5.87</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="AA29" s="2" t="inlineStr"/>
+        <v>3.4</v>
+      </c>
+      <c r="AA29" s="2" t="n">
+        <v>65</v>
+      </c>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
@@ -2692,19 +2664,19 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.744</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-4.94</v>
+        <v>3.17</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2714,11 +2686,9 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2729,56 +2699,50 @@
       <c r="S30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>23.73</v>
+        <v>-2.52</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>11.75</v>
+        <v>-6.2</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>6.39</v>
+        <v>1.15</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>0.53</v>
+        <v>1.6</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-6.3</v>
-      </c>
-      <c r="AA30" s="2" t="n">
-        <v>83</v>
-      </c>
+        <v>-0.1</v>
+      </c>
+      <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.249</v>
+        <v>1.749</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>117.45</v>
+        <v>-4.94</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2788,42 +2752,48 @@
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N31" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="inlineStr"/>
       <c r="S31" s="2" t="inlineStr"/>
-      <c r="T31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>17.3</v>
+        <v>26.33</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>10</v>
+        <v>11.16</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-4.24</v>
+        <v>6.83</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-1.36</v>
+        <v>2.2</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>63.8</v>
+        <v>-4.9</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2825,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-18 | 30 只</t>
+          <t>截至: 2026-09-21 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-22
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.418</v>
+        <v>3.42</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -694,42 +694,38 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>14.07</v>
+        <v>15.3</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>2.76</v>
+        <v>2.65</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>1.83</v>
+        <v>2.19</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-2.1</v>
+        <v>-1.21</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="AB2" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -751,7 +747,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.462</v>
+        <v>1.473</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>93.48999999999999</v>
@@ -782,22 +778,22 @@
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-11.1</v>
+        <v>-10.8</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-2.4</v>
+        <v>-1.71</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-1.14</v>
+        <v>-0.49</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>-1.15</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="Z3" s="2" t="n">
         <v>69.40000000000001</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -834,8 +830,10 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="n">
-        <v>13</v>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>+13/-13</t>
+        </is>
       </c>
       <c r="N4" s="2" t="n">
         <v>3</v>
@@ -850,22 +848,22 @@
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-31.18</v>
+        <v>-30.86</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-9.619999999999999</v>
+        <v>-9.609999999999999</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-0.51</v>
+        <v>-0.8</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>2.35</v>
+        <v>1.5</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>72.3</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
@@ -889,7 +887,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.748</v>
+        <v>1.743</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>101.26</v>
@@ -919,36 +917,36 @@
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R5" s="2" t="inlineStr"/>
       <c r="S5" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>49.79</v>
+        <v>48.59</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>24.56</v>
+        <v>23.92</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-4.68</v>
+        <v>-6.65</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>10.78</v>
+        <v>9.25</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>99.90000000000001</v>
+        <v>99.5</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
@@ -969,7 +967,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.869</v>
+        <v>0.867</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>4.26</v>
@@ -998,19 +996,19 @@
       </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-5.42</v>
+        <v>-4.02</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>4.78</v>
+        <v>4.51</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>3.77</v>
+        <v>3.71</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>4.27</v>
+        <v>1.55</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>57.1</v>
+        <v>58.2</v>
       </c>
       <c r="AA6" s="2" t="n">
         <v>80</v>
@@ -1037,7 +1035,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3.002</v>
+        <v>3.015</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>55.83</v>
@@ -1054,7 +1052,7 @@
         <v>9</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -1070,22 +1068,22 @@
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-2.57</v>
+        <v>-1.72</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.39</v>
+        <v>1.72</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-0.44</v>
+        <v>-0.15</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>44.3</v>
+        <v>45</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
@@ -1109,7 +1107,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.608</v>
+        <v>4.613</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>10.81</v>
@@ -1124,40 +1122,38 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
       <c r="S8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>1.97</v>
+        <v>2.76</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.15</v>
+        <v>1.13</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.18</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1179,7 +1175,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.872</v>
+        <v>7.85</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>28.85</v>
@@ -1208,26 +1204,26 @@
       </c>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>14.28</v>
+        <v>15.51</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>3.77</v>
+        <v>3.34</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>2.04</v>
+        <v>1.08</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>1.44</v>
+        <v>0.96</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>20.1</v>
+        <v>21</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
@@ -1249,7 +1245,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.385</v>
+        <v>3.38</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>114.34</v>
@@ -1276,41 +1272,39 @@
       </c>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>10.49</v>
+        <v>11.01</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>9.42</v>
+        <v>9.1</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-2.31</v>
+        <v>-2.6</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>-1.76</v>
+        <v>-1.36</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>89.3</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
@@ -1331,7 +1325,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.51</v>
+        <v>0.511</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>6.73</v>
@@ -1356,30 +1350,26 @@
       <c r="R11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S11" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-15.14</v>
+        <v>-13.74</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-4.06</v>
+        <v>-3.91</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.45</v>
+        <v>0.26</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>36.6</v>
+        <v>36.3</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1403,7 +1393,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.386</v>
+        <v>0.384</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>12.91</v>
@@ -1434,28 +1424,26 @@
       </c>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-6.37</v>
+        <v>-5.17</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>3.89</v>
+        <v>3.38</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>2.79</v>
+        <v>2.36</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>4.67</v>
+        <v>1.95</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>64.7</v>
+        <v>65.5</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
-      <c r="AD12" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="inlineStr">
         <is>
@@ -1475,7 +1463,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.788</v>
+        <v>0.791</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>79.75</v>
@@ -1508,22 +1496,22 @@
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-12.62</v>
+        <v>-11.5</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-3.54</v>
+        <v>-3.23</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-0.61</v>
+        <v>-0.26</v>
       </c>
       <c r="Y13" s="2" t="n">
         <v>1.79</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>61.7</v>
+        <v>61.2</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1547,7 +1535,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>3.149</v>
+        <v>3.148</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>43.79</v>
@@ -1576,19 +1564,19 @@
       </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>8.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>2.56</v>
+        <v>2.42</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>2.34</v>
+        <v>1.8</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>3.87</v>
+        <v>3.23</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>37.3</v>
+        <v>38.5</v>
       </c>
       <c r="AA14" s="2" t="n">
         <v>78</v>
@@ -1641,35 +1629,29 @@
       <c r="S15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-3.52</v>
+        <v>-1.84</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>3.97</v>
+        <v>3.93</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>3.11</v>
+        <v>2.9</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>4.67</v>
+        <v>1.96</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>72.2</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
-      <c r="AD15" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr">
         <is>
@@ -1689,7 +1671,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.176</v>
+        <v>1.168</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>33.19</v>
@@ -1704,7 +1686,7 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -1716,22 +1698,22 @@
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-1.4</v>
+        <v>-0.68</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-5.52</v>
+        <v>-6.25</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>1.06</v>
+        <v>0.48</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>8.300000000000001</v>
+        <v>6.89</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>43</v>
+        <v>44.4</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
@@ -1755,7 +1737,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.416</v>
+        <v>0.415</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>76.56999999999999</v>
@@ -1778,27 +1760,23 @@
       <c r="R17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S17" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-46.79</v>
+        <v>-46.21</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-14.94</v>
+        <v>-15.03</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>0.38</v>
+        <v>0.03</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>2.24</v>
+        <v>1.65</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>54.7</v>
+        <v>54.5</v>
       </c>
       <c r="AA17" s="2" t="n">
         <v>66</v>
@@ -1825,7 +1803,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.142</v>
+        <v>1.155</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>5.68</v>
@@ -1853,29 +1831,35 @@
       <c r="S18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-7.11</v>
+        <v>-5.8</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-5.23</v>
+        <v>-4.18</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>1.59</v>
+        <v>2.34</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>2.03</v>
+        <v>2.23</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>7.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="AB18" s="2" t="inlineStr"/>
+        <v>77</v>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AC18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
@@ -1888,19 +1872,19 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.102</v>
+        <v>0.839</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>-3.59</v>
+        <v>99.92</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1912,63 +1896,65 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>41.51</v>
+        <v>-0.42</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>16.97</v>
+        <v>7.34</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>8.09</v>
+        <v>-2.79</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>1.02</v>
+        <v>2.94</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>-4.7</v>
+        <v>96.7</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
-      <c r="AC19" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AD19" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.839</v>
+        <v>1.05</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>99.92</v>
+        <v>-2.39</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1977,47 +1963,51 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N20" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O20" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-0.52</v>
+        <v>-53.04</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>7.46</v>
+        <v>-18.38</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-3.63</v>
+        <v>1.08</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>2.62</v>
+        <v>1.05</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>97.3</v>
+        <v>36.4</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>40</v>
+        <v>79</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
@@ -2028,19 +2018,19 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.03</v>
+        <v>1.814</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-2.39</v>
+        <v>93.77</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2049,14 +2039,12 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="n">
         <v>9</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -2064,30 +2052,26 @@
       <c r="R21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-53.63</v>
+        <v>-16.69</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-19.99</v>
+        <v>-5</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>1</v>
+        <v>-0.44</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-0.15</v>
+        <v>1.86</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>35.7</v>
+        <v>55.3</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2102,19 +2086,19 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.809</v>
+        <v>2.316</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>93.77</v>
+        <v>78.59</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -2124,38 +2108,38 @@
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-17.97</v>
+        <v>23.96</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-5.25</v>
+        <v>19.96</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.7</v>
+        <v>3.13</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>1.86</v>
+        <v>4.28</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>56.7</v>
+        <v>44.2</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>56</v>
+        <v>85</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
@@ -2163,26 +2147,26 @@
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.283</v>
+        <v>1.514</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>78.59</v>
+        <v>12.11</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -2192,67 +2176,67 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R23" s="2" t="inlineStr"/>
       <c r="S23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T23" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>22.66</v>
+        <v>-18.9</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>18.53</v>
+        <v>-14.22</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>2.61</v>
+        <v>0.04</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>4.58</v>
+        <v>-5.51</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>38.5</v>
+        <v>5.2</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.504</v>
+        <v>1.079</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>12.11</v>
+        <v>25.84</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -2263,64 +2247,72 @@
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="n">
-        <v>9</v>
+        <v>-13</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S24" s="2" t="inlineStr"/>
-      <c r="T24" s="2" t="inlineStr"/>
-      <c r="U24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V24" s="2" t="n">
-        <v>-20.8</v>
+        <v>57</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-14.72</v>
+        <v>23.01</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-1.21</v>
+        <v>4.13</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-7.06</v>
+        <v>3.8</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>4.9</v>
+        <v>23</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.081</v>
+        <v>1.292</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>25.84</v>
+        <v>117.45</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -2334,186 +2326,188 @@
         <v>-13</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr"/>
-      <c r="T25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U25" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>55.6</v>
+        <v>20.21</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>23.63</v>
+        <v>12.68</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>4.77</v>
+        <v>-0.9</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>4.79</v>
+        <v>-2.48</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>21.7</v>
+        <v>65.7</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="n">
-        <v>3</v>
-      </c>
+      <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.282</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>117.45</v>
+        <v>20.09</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S26" s="2" t="inlineStr"/>
-      <c r="T26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>18.96</v>
+        <v>-17.06</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>12.01</v>
+        <v>-14.78</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-1.18</v>
+        <v>1.51</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-3.38</v>
+        <v>-1.81</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>64.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.82</v>
+        <v>0.707</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>20.09</v>
+        <v>30.88</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-18.76</v>
+        <v>56.68</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-14.41</v>
+        <v>22.29</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>1.81</v>
+        <v>5.82</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-1.65</v>
+        <v>5.96</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>8.9</v>
+        <v>27.1</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="AB27" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
@@ -2526,19 +2520,19 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.712</v>
+        <v>2.334</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>30.88</v>
+        <v>10.28</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2548,67 +2542,65 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T28" s="2" t="inlineStr"/>
-      <c r="U28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>55.02</v>
+        <v>-20.28</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>23.54</v>
+        <v>-15.94</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>6.97</v>
+        <v>-0.52</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>7.24</v>
+        <v>-4.73</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>25.6</v>
+        <v>3.4</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2.335</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>10.28</v>
+        <v>3.17</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2620,7 +2612,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2629,30 +2621,28 @@
       <c r="S29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-21.95</v>
+        <v>-1.77</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-15.76</v>
+        <v>-6.46</v>
       </c>
       <c r="X29" s="2" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="Y29" s="2" t="n">
         <v>-0.6</v>
       </c>
-      <c r="Y29" s="2" t="n">
-        <v>-5.87</v>
-      </c>
       <c r="Z29" s="2" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="AA29" s="2" t="n">
-        <v>65</v>
-      </c>
+        <v>0.1</v>
+      </c>
+      <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AC29" s="2" t="inlineStr"/>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
@@ -2664,19 +2654,19 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.9360000000000001</v>
+        <v>1.758</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>3.17</v>
+        <v>-4.94</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2686,63 +2676,65 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N30" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-2.52</v>
+        <v>28.46</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-6.2</v>
+        <v>11.5</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>1.15</v>
+        <v>4.9</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>1.6</v>
+        <v>2.27</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="AA30" s="2" t="inlineStr"/>
+        <v>-3.4</v>
+      </c>
+      <c r="AA30" s="2" t="n">
+        <v>80</v>
+      </c>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.749</v>
+        <v>1.112</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>-4.94</v>
+        <v>-3.59</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2752,9 +2744,7 @@
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
         <v>1</v>
       </c>
@@ -2763,31 +2753,29 @@
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="inlineStr"/>
       <c r="S31" s="2" t="inlineStr"/>
-      <c r="T31" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>26.33</v>
+        <v>43.89</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>11.16</v>
+        <v>17.71</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>6.83</v>
+        <v>6.14</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>2.2</v>
+        <v>1.69</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>-4.9</v>
+        <v>-3.5</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
@@ -2825,7 +2813,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-21 | 30 只</t>
+          <t>截至: 2026-09-22 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-23
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.42</v>
+        <v>3.399</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -699,33 +699,37 @@
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>15.3</v>
+        <v>14.83</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>2.65</v>
+        <v>2.57</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>2.19</v>
+        <v>0.96</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-1.21</v>
+        <v>-0.7</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -738,19 +742,19 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.473</v>
+        <v>0.656</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>93.48999999999999</v>
+        <v>90.17</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -760,9 +764,13 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>+13/-13</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -770,30 +778,26 @@
       <c r="R3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-10.8</v>
+        <v>-30.75</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-1.71</v>
+        <v>-9.220000000000001</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-0.49</v>
+        <v>0.93</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>-0.6899999999999999</v>
+        <v>2.39</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>69.40000000000001</v>
+        <v>71.2</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -808,66 +812,78 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.658</v>
+        <v>1.678</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>90.17</v>
+        <v>101.26</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>+13/-13</t>
-        </is>
-      </c>
+      <c r="L4" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S4" s="2" t="inlineStr"/>
-      <c r="T4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-30.86</v>
+        <v>45.25</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-9.609999999999999</v>
+        <v>19.9</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-0.8</v>
+        <v>-12.06</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>1.5</v>
+        <v>11.8</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>71.90000000000001</v>
+        <v>97.2</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
@@ -878,76 +894,62 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.743</v>
+        <v>0.87</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>101.26</v>
+        <v>4.26</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
       <c r="S5" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T5" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>48.59</v>
+        <v>-3.31</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>23.92</v>
+        <v>5.57</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-6.65</v>
+        <v>4.89</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>9.25</v>
+        <v>3.42</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>99.5</v>
+        <v>59.1</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="n">
-        <v>3</v>
-      </c>
+      <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
         <is>
@@ -958,19 +960,19 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.867</v>
+        <v>3</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4.26</v>
+        <v>55.83</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -980,38 +982,42 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-4.02</v>
+        <v>-1.65</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>4.51</v>
+        <v>1.83</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>3.71</v>
+        <v>-0.12</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>1.55</v>
+        <v>1.39</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>58.2</v>
+        <v>44.2</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
@@ -1019,26 +1025,26 @@
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3.015</v>
+        <v>4.59</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>55.83</v>
+        <v>10.81</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -1048,45 +1054,43 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S7" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="T7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-1.72</v>
+        <v>2.61</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.72</v>
+        <v>1.23</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-0.15</v>
+        <v>0.02</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>1.49</v>
+        <v>0.11</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>45</v>
+        <v>2.7</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr">
@@ -1098,19 +1102,19 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.613</v>
+        <v>7.818</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>10.81</v>
+        <v>28.85</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1122,38 +1126,40 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>2.76</v>
+        <v>15.18</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.13</v>
+        <v>3.49</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-0.18</v>
+        <v>0.35</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-0.06</v>
+        <v>1.21</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>2.2</v>
+        <v>21.5</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1166,28 +1172,40 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.85</v>
+        <v>3.35</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>28.85</v>
+        <v>114.34</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
         <v>1</v>
@@ -1195,84 +1213,72 @@
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T9" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R9" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>15.51</v>
+        <v>11.06</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>3.34</v>
+        <v>8.76</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>1.08</v>
+        <v>-1.64</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>0.96</v>
+        <v>-1.77</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>21</v>
+        <v>86.3</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
-      <c r="AC9" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.38</v>
+        <v>0.51</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>114.34</v>
+        <v>6.73</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
@@ -1281,31 +1287,31 @@
         <v>1</v>
       </c>
       <c r="S10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>11.01</v>
+        <v>-13.56</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>9.1</v>
+        <v>-3.45</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-2.6</v>
+        <v>0.9</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>-1.36</v>
+        <v>0.92</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>88.09999999999999</v>
+        <v>35.5</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
         <is>
@@ -1316,19 +1322,19 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.511</v>
+        <v>0.384</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6.73</v>
+        <v>12.91</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1337,39 +1343,39 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L11" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-13.74</v>
+        <v>-4.55</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-3.91</v>
+        <v>4.08</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.26</v>
+        <v>3.66</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>2.31</v>
+        <v>3.17</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>36.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1384,19 +1390,19 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.384</v>
+        <v>0.786</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>12.91</v>
+        <v>79.75</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1405,41 +1411,39 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-5.17</v>
+        <v>-11.51</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>3.38</v>
+        <v>-3.21</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>2.36</v>
+        <v>0.22</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>1.95</v>
+        <v>0.53</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>65.5</v>
+        <v>59.6</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1454,19 +1458,19 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.791</v>
+        <v>0.349</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>79.75</v>
+        <v>40.85</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1475,43 +1479,41 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L13" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
         <v>3</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="T13" s="2" t="inlineStr"/>
-      <c r="U13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V13" s="2" t="n">
-        <v>-11.5</v>
+        <v>-0.89</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-3.23</v>
+        <v>5.01</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-0.26</v>
+        <v>3.72</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>1.79</v>
+        <v>4.38</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>61.2</v>
+        <v>74.8</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1526,19 +1528,19 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>3.148</v>
+        <v>1.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>43.79</v>
+        <v>33.19</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1550,36 +1552,36 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
-      <c r="S14" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R14" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>9.699999999999999</v>
+        <v>-1.28</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>2.42</v>
+        <v>-7.12</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>1.8</v>
+        <v>-0.7</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>3.23</v>
+        <v>6.2</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>38.5</v>
+        <v>44.8</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
@@ -1587,26 +1589,26 @@
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.348</v>
+        <v>0.415</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>40.85</v>
+        <v>76.56999999999999</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1615,9 +1617,7 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
         <v>3</v>
@@ -1625,29 +1625,31 @@
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-1.84</v>
+        <v>-45.81</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>3.93</v>
+        <v>-14.36</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>2.9</v>
+        <v>1.51</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>1.96</v>
+        <v>2.66</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>73.40000000000001</v>
+        <v>54.3</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
@@ -1662,19 +1664,19 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.168</v>
+        <v>1.142</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>33.19</v>
+        <v>5.68</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1684,39 +1686,49 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N16" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-0.68</v>
+        <v>-5.93</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-6.25</v>
+        <v>-4.71</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>0.48</v>
+        <v>1.32</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>6.89</v>
+        <v>2.3</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>44.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="AB16" s="2" t="inlineStr"/>
-      <c r="AC16" s="2" t="inlineStr"/>
+        <v>69</v>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr">
@@ -1728,19 +1740,19 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.415</v>
+        <v>1.03</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>76.56999999999999</v>
+        <v>-2.39</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1749,37 +1761,47 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S17" s="2" t="inlineStr"/>
-      <c r="T17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-46.21</v>
+        <v>-53.49</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-15.03</v>
+        <v>-19.31</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>0.03</v>
+        <v>1.19</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>1.65</v>
+        <v>-0.28</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>54.5</v>
+        <v>35.8</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
@@ -1794,19 +1816,19 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.155</v>
+        <v>1.813</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>5.68</v>
+        <v>93.77</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1820,7 +1842,7 @@
         <v>9</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -1828,63 +1850,53 @@
       <c r="R18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-5.8</v>
+        <v>-16.55</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-4.18</v>
+        <v>-4.38</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>2.34</v>
+        <v>0.58</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>2.23</v>
+        <v>-0.29</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>9.199999999999999</v>
+        <v>53.9</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="AB18" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="AC18" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.839</v>
+        <v>1.504</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>99.92</v>
+        <v>12.11</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1894,67 +1906,69 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N19" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-0.42</v>
+        <v>-19.15</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>7.34</v>
+        <v>-14.23</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-2.79</v>
+        <v>0.54</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>2.94</v>
+        <v>-5.79</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>96.7</v>
+        <v>5.1</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
-      <c r="AC19" s="2" t="inlineStr"/>
-      <c r="AD19" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="AC19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.05</v>
+        <v>1.07</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-2.39</v>
+        <v>25.84</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1963,74 +1977,70 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="n">
-        <v>9</v>
+        <v>-13</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-53.04</v>
+        <v>56.01</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-18.38</v>
+        <v>22.47</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>1.08</v>
+        <v>0.06</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>1.05</v>
+        <v>4.05</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>36.4</v>
+        <v>24</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.814</v>
+        <v>1.262</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>93.77</v>
+        <v>117.45</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2041,37 +2051,39 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="n">
-        <v>9</v>
+        <v>-13</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="n">
-        <v>1</v>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-16.69</v>
+        <v>20.06</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-5</v>
+        <v>10.65</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-0.44</v>
+        <v>-2.25</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>1.86</v>
+        <v>-3.94</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>55.3</v>
+        <v>65.7</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2086,63 +2098,69 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2.316</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>78.59</v>
+        <v>20.09</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>23.96</v>
+        <v>-17.43</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>19.96</v>
+        <v>-14.54</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>3.13</v>
+        <v>1.13</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>4.28</v>
+        <v>-2.18</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>44.2</v>
+        <v>10.2</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
@@ -2154,19 +2172,19 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.514</v>
+        <v>0.701</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>12.11</v>
+        <v>30.88</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -2177,66 +2195,68 @@
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="n">
-        <v>9</v>
+        <v>-13</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>-18.9</v>
+        <v>55.72</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>-14.22</v>
+        <v>21.73</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>0.04</v>
+        <v>0.59</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-5.51</v>
+        <v>6.63</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>5.2</v>
+        <v>28.2</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.079</v>
+        <v>2.315</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>25.84</v>
+        <v>10.28</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -2246,9 +2266,7 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
         <v>2</v>
       </c>
@@ -2260,59 +2278,59 @@
           <t>预-1</t>
         </is>
       </c>
-      <c r="S24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U24" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>57</v>
+        <v>-20.79</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>23.01</v>
+        <v>-15.98</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>4.13</v>
+        <v>-0.11</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>3.8</v>
+        <v>-5.27</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>23</v>
+        <v>3.1</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.292</v>
+        <v>0.929</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>117.45</v>
+        <v>3.17</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -2322,120 +2340,104 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S25" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="T25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>20.21</v>
+        <v>-1.79</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>12.68</v>
+        <v>-6.36</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-0.9</v>
+        <v>1.12</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-2.48</v>
+        <v>0.46</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>65.7</v>
-      </c>
-      <c r="AA25" s="2" t="n">
-        <v>58</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AA25" s="2" t="inlineStr"/>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8169999999999999</v>
+        <v>1.755</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>20.09</v>
+        <v>-4.94</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T26" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-17.06</v>
+        <v>28.51</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-14.78</v>
+        <v>11.86</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>1.51</v>
+        <v>1.54</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-1.81</v>
+        <v>1.89</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>9.699999999999999</v>
+        <v>-2.1</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
@@ -2448,19 +2450,19 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.707</v>
+        <v>1.46</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>30.88</v>
+        <v>93.48999999999999</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -2470,69 +2472,61 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R27" s="2" t="inlineStr"/>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>56.68</v>
+        <v>-11.16</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>22.29</v>
+        <v>-1.96</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>5.82</v>
+        <v>-0.05</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>5.96</v>
+        <v>-0.97</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>27.1</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AC27" s="2" t="inlineStr"/>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2.334</v>
+        <v>3.146</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>10.28</v>
+        <v>43.79</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2544,63 +2538,59 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-20.28</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-15.94</v>
+        <v>2.92</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-0.52</v>
+        <v>1.14</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-4.73</v>
+        <v>4.23</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>3.4</v>
+        <v>39.6</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.9340000000000001</v>
+        <v>1.108</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>3.17</v>
+        <v>-3.59</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2612,61 +2602,61 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
       <c r="R29" s="2" t="inlineStr"/>
-      <c r="S29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T29" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-1.77</v>
+        <v>43.91</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-6.46</v>
+        <v>17.82</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>1.04</v>
+        <v>2.3</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-0.6</v>
+        <v>1.48</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AA29" s="2" t="inlineStr"/>
+        <v>-2.4</v>
+      </c>
+      <c r="AA29" s="2" t="n">
+        <v>76</v>
+      </c>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.758</v>
+        <v>0.833</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-4.94</v>
+        <v>99.92</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2676,11 +2666,9 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2690,51 +2678,51 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>28.46</v>
+        <v>-0.49</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>11.5</v>
+        <v>7.23</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>4.9</v>
+        <v>-1.64</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>2.27</v>
+        <v>2.63</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-3.4</v>
+        <v>95.5</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AD30" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.112</v>
+        <v>2.334</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>-3.59</v>
+        <v>78.59</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2746,7 +2734,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2756,27 +2744,25 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>43.89</v>
+        <v>24.21</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>17.71</v>
+        <v>21.47</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>6.14</v>
+        <v>4.4</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>1.69</v>
+        <v>6.43</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>-3.5</v>
+        <v>50.1</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
@@ -2813,7 +2799,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-22 | 30 只</t>
+          <t>截至: 2026-09-23 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-24
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.399</v>
+        <v>3.312</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -694,42 +694,38 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R2" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>14.83</v>
+        <v>13.55</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>2.57</v>
+        <v>1.65</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>0.96</v>
+        <v>-0.02</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-0.7</v>
+        <v>-2.5</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -742,19 +738,19 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.656</v>
+        <v>1.453</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>90.17</v>
+        <v>93.48999999999999</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -764,40 +760,40 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>+13/-13</t>
-        </is>
-      </c>
+      <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="n">
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-30.75</v>
+        <v>-11.25</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-9.220000000000001</v>
+        <v>-0.65</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>0.93</v>
+        <v>1.5</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>2.39</v>
+        <v>1.62</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>71.2</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -812,78 +808,68 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.678</v>
+        <v>0.646</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>101.26</v>
+        <v>90.17</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>+13/-13</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="n">
+      <c r="R4" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>45.25</v>
+        <v>-30.97</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>19.9</v>
+        <v>-8.91</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-12.06</v>
+        <v>0.59</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>11.8</v>
+        <v>3.34</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>97.2</v>
+        <v>69.2</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="AB4" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
@@ -894,62 +880,74 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.87</v>
+        <v>1.749</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4.26</v>
+        <v>101.26</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-3.31</v>
+        <v>44.25</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>5.57</v>
+        <v>27.01</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>4.89</v>
+        <v>-1.8</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>3.42</v>
+        <v>18.99</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>59.1</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>79</v>
+        <v>43</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
         <is>
@@ -960,19 +958,19 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3</v>
+        <v>0.841</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>55.83</v>
+        <v>4.26</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -982,42 +980,38 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-1.65</v>
+        <v>-3.37</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.83</v>
+        <v>3.92</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-0.12</v>
+        <v>2.21</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>1.39</v>
+        <v>1.74</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>44.2</v>
+        <v>58.2</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
@@ -1025,26 +1019,26 @@
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4.59</v>
+        <v>2.959</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>10.81</v>
+        <v>55.83</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -1054,43 +1048,47 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>2.61</v>
+        <v>-1.99</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.23</v>
+        <v>2.21</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.02</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.11</v>
+        <v>1.72</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>2.7</v>
+        <v>40.6</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="n">
-        <v>3</v>
-      </c>
+      <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr">
@@ -1102,19 +1100,19 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7.818</v>
+        <v>4.515</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>28.85</v>
+        <v>10.81</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1126,40 +1124,40 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R8" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>15.18</v>
+        <v>1.81</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>3.49</v>
+        <v>1.32</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.35</v>
+        <v>0.05</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>1.21</v>
+        <v>0.23</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>21.5</v>
+        <v>1.4</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1172,43 +1170,31 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.35</v>
+        <v>7.65</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>114.34</v>
+        <v>28.85</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
@@ -1220,65 +1206,75 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>11.06</v>
+        <v>14.34</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>8.76</v>
+        <v>3</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-1.64</v>
+        <v>-0.15</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-1.77</v>
+        <v>-0.77</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>86.3</v>
+        <v>20.8</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
-      <c r="AC9" s="2" t="inlineStr"/>
-      <c r="AD9" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="AC9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.51</v>
+        <v>3.357</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>6.73</v>
+        <v>114.34</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L10" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
@@ -1287,31 +1283,39 @@
         <v>1</v>
       </c>
       <c r="S10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="V10" s="2" t="n">
-        <v>-13.56</v>
+        <v>10.99</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-3.45</v>
+        <v>10.84</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>0.9</v>
+        <v>0.65</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>0.92</v>
+        <v>0.82</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>35.5</v>
+        <v>84.8</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="AB10" s="2" t="inlineStr"/>
+        <v>33</v>
+      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
         <is>
@@ -1322,19 +1326,19 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.384</v>
+        <v>0.501</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>12.91</v>
+        <v>6.73</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1343,39 +1347,43 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="n">
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-4.55</v>
+        <v>-13.66</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>4.08</v>
+        <v>-3.41</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>3.66</v>
+        <v>1.2</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>3.17</v>
+        <v>0.59</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>66.09999999999999</v>
+        <v>33.5</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1390,19 +1398,19 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.786</v>
+        <v>0.375</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>79.75</v>
+        <v>12.91</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1411,39 +1419,41 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L12" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
         <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="n">
-        <v>1</v>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-11.51</v>
+        <v>-4.42</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-3.21</v>
+        <v>3.45</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>0.22</v>
+        <v>1.65</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>0.53</v>
+        <v>2.85</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>59.6</v>
+        <v>65.2</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1458,19 +1468,19 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.349</v>
+        <v>0.772</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>40.85</v>
+        <v>79.75</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1479,41 +1489,41 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="n">
+      <c r="R13" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T13" s="2" t="inlineStr"/>
-      <c r="U13" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-0.89</v>
+        <v>-11.82</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>5.01</v>
+        <v>-3.23</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>3.72</v>
+        <v>0.59</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>4.38</v>
+        <v>0.66</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>74.8</v>
+        <v>55.2</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>78</v>
+        <v>26</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1528,19 +1538,19 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1.15</v>
+        <v>3.079</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>33.19</v>
+        <v>43.79</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1561,27 +1571,25 @@
         <v>-1</v>
       </c>
       <c r="S14" s="2" t="inlineStr"/>
-      <c r="T14" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-1.28</v>
+        <v>8.74</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-7.12</v>
+        <v>2.47</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-0.7</v>
+        <v>0.79</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>6.2</v>
+        <v>2.13</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>44.8</v>
+        <v>39.5</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
@@ -1589,26 +1597,26 @@
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.415</v>
+        <v>0.341</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>76.56999999999999</v>
+        <v>40.85</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1617,7 +1625,9 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
         <v>3</v>
@@ -1625,31 +1635,33 @@
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="n">
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S15" s="2" t="inlineStr"/>
-      <c r="T15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-45.81</v>
+        <v>-0.57</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-14.36</v>
+        <v>4.47</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>1.51</v>
+        <v>2.08</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>2.66</v>
+        <v>4.33</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>54.3</v>
+        <v>74.5</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
@@ -1664,19 +1676,19 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.142</v>
+        <v>1.129</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>5.68</v>
+        <v>33.19</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1686,49 +1698,43 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S16" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-5.93</v>
+        <v>-1.46</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-4.71</v>
+        <v>-7.2</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>1.32</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>2.3</v>
+        <v>5.23</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>9.699999999999999</v>
+        <v>44.1</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="AB16" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
-      <c r="AC16" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr"/>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr">
@@ -1740,19 +1746,19 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.03</v>
+        <v>0.408</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-2.39</v>
+        <v>76.56999999999999</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1761,14 +1767,10 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
@@ -1778,30 +1780,28 @@
           <t>预-1</t>
         </is>
       </c>
-      <c r="S17" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-53.49</v>
+        <v>-45.99</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-19.31</v>
+        <v>-14.2</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>1.19</v>
+        <v>1.16</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-0.28</v>
+        <v>3.76</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>35.8</v>
+        <v>52.8</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
@@ -1816,19 +1816,19 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.813</v>
+        <v>1.121</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>93.77</v>
+        <v>5.68</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1847,56 +1847,60 @@
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="n">
-        <v>1</v>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-16.55</v>
+        <v>-6.22</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-4.38</v>
+        <v>-4.79</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>0.58</v>
+        <v>1.17</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-0.29</v>
+        <v>0.13</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>53.9</v>
+        <v>9</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
-      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.504</v>
+        <v>1.083</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>12.11</v>
+        <v>-3.59</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1906,69 +1910,69 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O19" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr"/>
-      <c r="S19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-19.15</v>
+        <v>43.32</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-14.23</v>
+        <v>16.99</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>0.54</v>
+        <v>2.1</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-5.79</v>
+        <v>-2.84</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>5.1</v>
+        <v>-1.9</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.07</v>
+        <v>0.839</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>25.84</v>
+        <v>99.92</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1978,69 +1982,67 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
+          <t>预1</t>
         </is>
       </c>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>56.01</v>
+        <v>-0.65</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>22.47</v>
+        <v>9.9</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>0.06</v>
+        <v>0.8</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>4.05</v>
+        <v>7.37</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>24</v>
+        <v>95</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.262</v>
+        <v>1.025</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>117.45</v>
+        <v>-2.39</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2049,12 +2051,14 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M21" s="2" t="n">
-        <v>-13</v>
+        <v>13</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -2064,26 +2068,28 @@
           <t>预-1</t>
         </is>
       </c>
-      <c r="S21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>20.06</v>
+        <v>-53.25</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>10.65</v>
+        <v>-18.14</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-2.25</v>
+        <v>2.82</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-3.94</v>
+        <v>1.82</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>65.7</v>
+        <v>35.1</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2098,93 +2104,93 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.8139999999999999</v>
+        <v>1.782</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>20.09</v>
+        <v>93.77</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="n">
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-17.43</v>
+        <v>-16.43</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-14.54</v>
+        <v>-4.25</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>1.13</v>
+        <v>1.52</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-2.18</v>
+        <v>0.03</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>10.2</v>
+        <v>50.7</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AC22" s="2" t="inlineStr"/>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.701</v>
+        <v>2.312</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>30.88</v>
+        <v>78.59</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -2194,11 +2200,9 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -2212,27 +2216,25 @@
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>55.72</v>
+        <v>24.35</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>21.73</v>
+        <v>22.29</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>0.59</v>
+        <v>4.72</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>6.63</v>
+        <v>6.96</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>28.2</v>
+        <v>54.6</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
@@ -2244,19 +2246,19 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2.315</v>
+        <v>1.472</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>10.28</v>
+        <v>12.11</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -2268,7 +2270,7 @@
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
@@ -2286,26 +2288,26 @@
       </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-20.79</v>
+        <v>-20.35</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-15.98</v>
+        <v>-14.55</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-0.11</v>
+        <v>-0.1</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-5.27</v>
+        <v>-5.53</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>3.1</v>
+        <v>4.2</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
@@ -2318,19 +2320,19 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.929</v>
+        <v>1.038</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>3.17</v>
+        <v>25.84</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -2340,61 +2342,71 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N25" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr"/>
-      <c r="T25" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>-1.79</v>
+        <v>53.69</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-6.36</v>
+        <v>20.66</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>1.12</v>
+        <v>-1.36</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>0.46</v>
+        <v>-1.12</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA25" s="2" t="inlineStr"/>
+        <v>24.1</v>
+      </c>
+      <c r="AA25" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.755</v>
+        <v>1.266</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>-4.94</v>
+        <v>117.45</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -2405,7 +2417,7 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="n">
-        <v>9</v>
+        <v>-13</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>1</v>
@@ -2416,53 +2428,55 @@
       <c r="R26" s="2" t="inlineStr"/>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="V26" s="2" t="n">
-        <v>28.51</v>
+        <v>19.86</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>11.86</v>
+        <v>12.84</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>1.54</v>
+        <v>0.79</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>1.89</v>
+        <v>-3.57</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>-2.1</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1.46</v>
+        <v>0.792</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>93.48999999999999</v>
+        <v>20.09</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -2474,59 +2488,63 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-11.16</v>
+        <v>-18.31</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-1.96</v>
+        <v>-15.36</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.05</v>
+        <v>0.45</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-0.97</v>
+        <v>-1.73</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>68.40000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>3.146</v>
+        <v>0.679</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>43.79</v>
+        <v>30.88</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2536,37 +2554,47 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>9.369999999999999</v>
+        <v>53.08</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>2.92</v>
+        <v>19.76</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>1.14</v>
+        <v>-1.89</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>4.23</v>
+        <v>0.62</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>39.6</v>
+        <v>28.5</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
@@ -2578,19 +2606,19 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.108</v>
+        <v>2.265</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>-3.59</v>
+        <v>10.28</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2602,61 +2630,65 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S29" s="2" t="inlineStr"/>
-      <c r="T29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>43.91</v>
+        <v>-22</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>17.82</v>
+        <v>-16.39</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>2.3</v>
+        <v>-0.54</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>1.48</v>
+        <v>-4.55</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>-2.4</v>
+        <v>2</v>
       </c>
       <c r="AA29" s="2" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.833</v>
+        <v>0.919</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>99.92</v>
+        <v>3.17</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2673,56 +2705,56 @@
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-0.49</v>
+        <v>-2.22</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>7.23</v>
+        <v>-5.7</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-1.64</v>
+        <v>0.92</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>2.63</v>
+        <v>0.12</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>95.5</v>
-      </c>
-      <c r="AA30" s="2" t="n">
-        <v>29</v>
-      </c>
+        <v>-0.4</v>
+      </c>
+      <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
-      <c r="AD30" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>2.334</v>
+        <v>1.713</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>78.59</v>
+        <v>-4.94</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2732,37 +2764,45 @@
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N31" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S31" s="2" t="inlineStr"/>
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>24.21</v>
+        <v>28.06</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>21.47</v>
+        <v>10.99</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>4.4</v>
+        <v>1.05</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>6.43</v>
+        <v>-2.13</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>50.1</v>
+        <v>-1.6</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>85</v>
+        <v>48</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
@@ -2799,7 +2839,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-23 | 30 只</t>
+          <t>截至: 2026-09-24 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-25
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$AF$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$AR$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF31"/>
+  <dimension ref="A1:AR31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -503,6 +503,18 @@
     <col width="11" customWidth="1" min="30" max="30"/>
     <col width="11" customWidth="1" min="31" max="31"/>
     <col width="11" customWidth="1" min="32" max="32"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
+    <col width="11" customWidth="1" min="34" max="34"/>
+    <col width="11" customWidth="1" min="35" max="35"/>
+    <col width="11" customWidth="1" min="36" max="36"/>
+    <col width="11" customWidth="1" min="37" max="37"/>
+    <col width="11" customWidth="1" min="38" max="38"/>
+    <col width="11" customWidth="1" min="39" max="39"/>
+    <col width="11" customWidth="1" min="40" max="40"/>
+    <col width="11" customWidth="1" min="41" max="41"/>
+    <col width="11" customWidth="1" min="42" max="42"/>
+    <col width="11" customWidth="1" min="43" max="43"/>
+    <col width="11" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -664,6 +676,66 @@
       <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>周线档</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>5D MV</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>10D MV</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>20D MV</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>30D MV</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>50D MV</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>100D MV</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>200D MV</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>10D斜率</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>20D斜率</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>50D斜率</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>100D斜率</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>200D斜率</t>
         </is>
       </c>
     </row>
@@ -734,6 +806,42 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG2" s="2" t="n">
+        <v>3.388</v>
+      </c>
+      <c r="AH2" s="2" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="AI2" s="2" t="n">
+        <v>3.365</v>
+      </c>
+      <c r="AJ2" s="2" t="n">
+        <v>3.427</v>
+      </c>
+      <c r="AK2" s="2" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="AL2" s="2" t="n">
+        <v>3.739</v>
+      </c>
+      <c r="AM2" s="2" t="n">
+        <v>3.525</v>
+      </c>
+      <c r="AN2" s="2" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="AO2" s="2" t="n">
+        <v>-32.4</v>
+      </c>
+      <c r="AP2" s="2" t="n">
+        <v>-62.09</v>
+      </c>
+      <c r="AQ2" s="2" t="n">
+        <v>-20.54</v>
+      </c>
+      <c r="AR2" s="2" t="n">
+        <v>13.55</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -804,6 +912,42 @@
           <t>柱≥0</t>
         </is>
       </c>
+      <c r="AG3" s="2" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="AH3" s="2" t="n">
+        <v>1.456</v>
+      </c>
+      <c r="AI3" s="2" t="n">
+        <v>1.472</v>
+      </c>
+      <c r="AJ3" s="2" t="n">
+        <v>1.482</v>
+      </c>
+      <c r="AK3" s="2" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="AL3" s="2" t="n">
+        <v>1.473</v>
+      </c>
+      <c r="AM3" s="2" t="n">
+        <v>1.518</v>
+      </c>
+      <c r="AN3" s="2" t="n">
+        <v>-48.78</v>
+      </c>
+      <c r="AO3" s="2" t="n">
+        <v>-40.98</v>
+      </c>
+      <c r="AP3" s="2" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="AQ3" s="2" t="n">
+        <v>-12.35</v>
+      </c>
+      <c r="AR3" s="2" t="n">
+        <v>-11.25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -876,6 +1020,42 @@
           <t>柱≥0</t>
         </is>
       </c>
+      <c r="AG4" s="2" t="n">
+        <v>0.654</v>
+      </c>
+      <c r="AH4" s="2" t="n">
+        <v>0.654</v>
+      </c>
+      <c r="AI4" s="2" t="n">
+        <v>0.664</v>
+      </c>
+      <c r="AJ4" s="2" t="n">
+        <v>0.665</v>
+      </c>
+      <c r="AK4" s="2" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="AL4" s="2" t="n">
+        <v>0.665</v>
+      </c>
+      <c r="AM4" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AN4" s="2" t="n">
+        <v>-100.65</v>
+      </c>
+      <c r="AO4" s="2" t="n">
+        <v>-16.78</v>
+      </c>
+      <c r="AP4" s="2" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="AQ4" s="2" t="n">
+        <v>-33.18</v>
+      </c>
+      <c r="AR4" s="2" t="n">
+        <v>-30.97</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -953,6 +1133,42 @@
         <is>
           <t>柱≥0</t>
         </is>
+      </c>
+      <c r="AG5" s="2" t="n">
+        <v>1.732</v>
+      </c>
+      <c r="AH5" s="2" t="n">
+        <v>1.758</v>
+      </c>
+      <c r="AI5" s="2" t="n">
+        <v>1.719</v>
+      </c>
+      <c r="AJ5" s="2" t="n">
+        <v>1.664</v>
+      </c>
+      <c r="AK5" s="2" t="n">
+        <v>1.596</v>
+      </c>
+      <c r="AL5" s="2" t="n">
+        <v>1.573</v>
+      </c>
+      <c r="AM5" s="2" t="n">
+        <v>1.501</v>
+      </c>
+      <c r="AN5" s="2" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="AO5" s="2" t="n">
+        <v>137.53</v>
+      </c>
+      <c r="AP5" s="2" t="n">
+        <v>85.26000000000001</v>
+      </c>
+      <c r="AQ5" s="2" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="AR5" s="2" t="n">
+        <v>44.25</v>
       </c>
     </row>
     <row r="6">
@@ -1022,6 +1238,42 @@
           <t>柱≥0</t>
         </is>
       </c>
+      <c r="AG6" s="2" t="n">
+        <v>0.856</v>
+      </c>
+      <c r="AH6" s="2" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="AI6" s="2" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="AJ6" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AK6" s="2" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="AL6" s="2" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="AM6" s="2" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="AN6" s="2" t="n">
+        <v>55.73</v>
+      </c>
+      <c r="AO6" s="2" t="n">
+        <v>-22.14</v>
+      </c>
+      <c r="AP6" s="2" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="AQ6" s="2" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="AR6" s="2" t="n">
+        <v>-3.37</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1095,6 +1347,42 @@
         <is>
           <t>无背离</t>
         </is>
+      </c>
+      <c r="AG7" s="2" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="AH7" s="2" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="AI7" s="2" t="n">
+        <v>3.005</v>
+      </c>
+      <c r="AJ7" s="2" t="n">
+        <v>3.007</v>
+      </c>
+      <c r="AK7" s="2" t="n">
+        <v>3.018</v>
+      </c>
+      <c r="AL7" s="2" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="AM7" s="2" t="n">
+        <v>3.044</v>
+      </c>
+      <c r="AN7" s="2" t="n">
+        <v>-27.45</v>
+      </c>
+      <c r="AO7" s="2" t="n">
+        <v>-4.84</v>
+      </c>
+      <c r="AP7" s="2" t="n">
+        <v>-8.359999999999999</v>
+      </c>
+      <c r="AQ7" s="2" t="n">
+        <v>-4.98</v>
+      </c>
+      <c r="AR7" s="2" t="n">
+        <v>-1.99</v>
       </c>
     </row>
     <row r="8">
@@ -1166,6 +1454,42 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG8" s="2" t="n">
+        <v>4.582</v>
+      </c>
+      <c r="AH8" s="2" t="n">
+        <v>4.564</v>
+      </c>
+      <c r="AI8" s="2" t="n">
+        <v>4.603</v>
+      </c>
+      <c r="AJ8" s="2" t="n">
+        <v>4.632</v>
+      </c>
+      <c r="AK8" s="2" t="n">
+        <v>4.658</v>
+      </c>
+      <c r="AL8" s="2" t="n">
+        <v>4.777</v>
+      </c>
+      <c r="AM8" s="2" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="AN8" s="2" t="n">
+        <v>-24.96</v>
+      </c>
+      <c r="AO8" s="2" t="n">
+        <v>-20.16</v>
+      </c>
+      <c r="AP8" s="2" t="n">
+        <v>-24.29</v>
+      </c>
+      <c r="AQ8" s="2" t="n">
+        <v>-12.79</v>
+      </c>
+      <c r="AR8" s="2" t="n">
+        <v>1.81</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1234,6 +1558,42 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG9" s="2" t="n">
+        <v>7.803</v>
+      </c>
+      <c r="AH9" s="2" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="AI9" s="2" t="n">
+        <v>7.763</v>
+      </c>
+      <c r="AJ9" s="2" t="n">
+        <v>7.813</v>
+      </c>
+      <c r="AK9" s="2" t="n">
+        <v>7.768</v>
+      </c>
+      <c r="AL9" s="2" t="n">
+        <v>8.131</v>
+      </c>
+      <c r="AM9" s="2" t="n">
+        <v>8.004</v>
+      </c>
+      <c r="AN9" s="2" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="AO9" s="2" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="AP9" s="2" t="n">
+        <v>-27.17</v>
+      </c>
+      <c r="AQ9" s="2" t="n">
+        <v>-15.22</v>
+      </c>
+      <c r="AR9" s="2" t="n">
+        <v>14.34</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1321,6 +1681,42 @@
         <is>
           <t>柱≥0</t>
         </is>
+      </c>
+      <c r="AG10" s="2" t="n">
+        <v>3.362</v>
+      </c>
+      <c r="AH10" s="2" t="n">
+        <v>3.373</v>
+      </c>
+      <c r="AI10" s="2" t="n">
+        <v>3.414</v>
+      </c>
+      <c r="AJ10" s="2" t="n">
+        <v>3.403</v>
+      </c>
+      <c r="AK10" s="2" t="n">
+        <v>3.346</v>
+      </c>
+      <c r="AL10" s="2" t="n">
+        <v>3.256</v>
+      </c>
+      <c r="AM10" s="2" t="n">
+        <v>3.213</v>
+      </c>
+      <c r="AN10" s="2" t="n">
+        <v>-66.05</v>
+      </c>
+      <c r="AO10" s="2" t="n">
+        <v>-24.2</v>
+      </c>
+      <c r="AP10" s="2" t="n">
+        <v>38.55</v>
+      </c>
+      <c r="AQ10" s="2" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="AR10" s="2" t="n">
+        <v>10.99</v>
       </c>
     </row>
     <row r="11">
@@ -1394,6 +1790,42 @@
           <t>柱≥0</t>
         </is>
       </c>
+      <c r="AG11" s="2" t="n">
+        <v>0.507</v>
+      </c>
+      <c r="AH11" s="2" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="AI11" s="2" t="n">
+        <v>0.515</v>
+      </c>
+      <c r="AJ11" s="2" t="n">
+        <v>0.515</v>
+      </c>
+      <c r="AK11" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AL11" s="2" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="AM11" s="2" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="AN11" s="2" t="n">
+        <v>-74.11</v>
+      </c>
+      <c r="AO11" s="2" t="n">
+        <v>-21.13</v>
+      </c>
+      <c r="AP11" s="2" t="n">
+        <v>-23.89</v>
+      </c>
+      <c r="AQ11" s="2" t="n">
+        <v>-3.41</v>
+      </c>
+      <c r="AR11" s="2" t="n">
+        <v>-13.66</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1463,6 +1895,42 @@
         <is>
           <t>柱≥0</t>
         </is>
+      </c>
+      <c r="AG12" s="2" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="AH12" s="2" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="AI12" s="2" t="n">
+        <v>0.376</v>
+      </c>
+      <c r="AJ12" s="2" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="AK12" s="2" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="AL12" s="2" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="AM12" s="2" t="n">
+        <v>0.372</v>
+      </c>
+      <c r="AN12" s="2" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="AO12" s="2" t="n">
+        <v>-10.25</v>
+      </c>
+      <c r="AP12" s="2" t="n">
+        <v>15.07</v>
+      </c>
+      <c r="AQ12" s="2" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="AR12" s="2" t="n">
+        <v>-4.42</v>
       </c>
     </row>
     <row r="13">
@@ -1533,6 +2001,42 @@
         <is>
           <t>柱≥0</t>
         </is>
+      </c>
+      <c r="AG13" s="2" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="AH13" s="2" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="AI13" s="2" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="AJ13" s="2" t="n">
+        <v>0.793</v>
+      </c>
+      <c r="AK13" s="2" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="AL13" s="2" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="AM13" s="2" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="AN13" s="2" t="n">
+        <v>-79.61</v>
+      </c>
+      <c r="AO13" s="2" t="n">
+        <v>-17.88</v>
+      </c>
+      <c r="AP13" s="2" t="n">
+        <v>-5.97</v>
+      </c>
+      <c r="AQ13" s="2" t="n">
+        <v>-7.03</v>
+      </c>
+      <c r="AR13" s="2" t="n">
+        <v>-11.82</v>
       </c>
     </row>
     <row r="14">
@@ -1600,6 +2104,42 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG14" s="2" t="n">
+        <v>3.131</v>
+      </c>
+      <c r="AH14" s="2" t="n">
+        <v>3.087</v>
+      </c>
+      <c r="AI14" s="2" t="n">
+        <v>3.093</v>
+      </c>
+      <c r="AJ14" s="2" t="n">
+        <v>3.098</v>
+      </c>
+      <c r="AK14" s="2" t="n">
+        <v>3.042</v>
+      </c>
+      <c r="AL14" s="2" t="n">
+        <v>3.237</v>
+      </c>
+      <c r="AM14" s="2" t="n">
+        <v>3.216</v>
+      </c>
+      <c r="AN14" s="2" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="AO14" s="2" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="AP14" s="2" t="n">
+        <v>-9.800000000000001</v>
+      </c>
+      <c r="AQ14" s="2" t="n">
+        <v>-18.05</v>
+      </c>
+      <c r="AR14" s="2" t="n">
+        <v>8.74</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1671,6 +2211,42 @@
         <is>
           <t>柱≥0</t>
         </is>
+      </c>
+      <c r="AG15" s="2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="AH15" s="2" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="AI15" s="2" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="AJ15" s="2" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="AK15" s="2" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="AL15" s="2" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="AM15" s="2" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="AN15" s="2" t="n">
+        <v>60.67</v>
+      </c>
+      <c r="AO15" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AP15" s="2" t="n">
+        <v>35.53</v>
+      </c>
+      <c r="AQ15" s="2" t="n">
+        <v>7.19</v>
+      </c>
+      <c r="AR15" s="2" t="n">
+        <v>-0.57</v>
       </c>
     </row>
     <row r="16">
@@ -1742,6 +2318,42 @@
           <t>背离</t>
         </is>
       </c>
+      <c r="AG16" s="2" t="n">
+        <v>1.157</v>
+      </c>
+      <c r="AH16" s="2" t="n">
+        <v>1.153</v>
+      </c>
+      <c r="AI16" s="2" t="n">
+        <v>1.152</v>
+      </c>
+      <c r="AJ16" s="2" t="n">
+        <v>1.142</v>
+      </c>
+      <c r="AK16" s="2" t="n">
+        <v>1.129</v>
+      </c>
+      <c r="AL16" s="2" t="n">
+        <v>1.213</v>
+      </c>
+      <c r="AM16" s="2" t="n">
+        <v>1.303</v>
+      </c>
+      <c r="AN16" s="2" t="n">
+        <v>-17.08</v>
+      </c>
+      <c r="AO16" s="2" t="n">
+        <v>61.43</v>
+      </c>
+      <c r="AP16" s="2" t="n">
+        <v>-10.21</v>
+      </c>
+      <c r="AQ16" s="2" t="n">
+        <v>-50.41</v>
+      </c>
+      <c r="AR16" s="2" t="n">
+        <v>-1.46</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1812,6 +2424,42 @@
           <t>柱≥0</t>
         </is>
       </c>
+      <c r="AG17" s="2" t="n">
+        <v>0.413</v>
+      </c>
+      <c r="AH17" s="2" t="n">
+        <v>0.412</v>
+      </c>
+      <c r="AI17" s="2" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="AJ17" s="2" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="AK17" s="2" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="AL17" s="2" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="AM17" s="2" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="AN17" s="2" t="n">
+        <v>-96.73</v>
+      </c>
+      <c r="AO17" s="2" t="n">
+        <v>-25.26</v>
+      </c>
+      <c r="AP17" s="2" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="AQ17" s="2" t="n">
+        <v>-41.93</v>
+      </c>
+      <c r="AR17" s="2" t="n">
+        <v>-45.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1883,6 +2531,42 @@
         <is>
           <t>背离</t>
         </is>
+      </c>
+      <c r="AG18" s="2" t="n">
+        <v>1.139</v>
+      </c>
+      <c r="AH18" s="2" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="AI18" s="2" t="n">
+        <v>1.146</v>
+      </c>
+      <c r="AJ18" s="2" t="n">
+        <v>1.156</v>
+      </c>
+      <c r="AK18" s="2" t="n">
+        <v>1.172</v>
+      </c>
+      <c r="AL18" s="2" t="n">
+        <v>1.215</v>
+      </c>
+      <c r="AM18" s="2" t="n">
+        <v>1.234</v>
+      </c>
+      <c r="AN18" s="2" t="n">
+        <v>-18</v>
+      </c>
+      <c r="AO18" s="2" t="n">
+        <v>-13.38</v>
+      </c>
+      <c r="AP18" s="2" t="n">
+        <v>-44.15</v>
+      </c>
+      <c r="AQ18" s="2" t="n">
+        <v>-34.29</v>
+      </c>
+      <c r="AR18" s="2" t="n">
+        <v>-6.22</v>
       </c>
     </row>
     <row r="19">
@@ -1956,6 +2640,42 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG19" s="2" t="n">
+        <v>1.101</v>
+      </c>
+      <c r="AH19" s="2" t="n">
+        <v>1.068</v>
+      </c>
+      <c r="AI19" s="2" t="n">
+        <v>1.068</v>
+      </c>
+      <c r="AJ19" s="2" t="n">
+        <v>1.085</v>
+      </c>
+      <c r="AK19" s="2" t="n">
+        <v>1.107</v>
+      </c>
+      <c r="AL19" s="2" t="n">
+        <v>1.182</v>
+      </c>
+      <c r="AM19" s="2" t="n">
+        <v>1.021</v>
+      </c>
+      <c r="AN19" s="2" t="n">
+        <v>139.91</v>
+      </c>
+      <c r="AO19" s="2" t="n">
+        <v>15.79</v>
+      </c>
+      <c r="AP19" s="2" t="n">
+        <v>-117.87</v>
+      </c>
+      <c r="AQ19" s="2" t="n">
+        <v>28.58</v>
+      </c>
+      <c r="AR19" s="2" t="n">
+        <v>43.32</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2026,6 +2746,42 @@
           <t>柱≥0</t>
         </is>
       </c>
+      <c r="AG20" s="2" t="n">
+        <v>0.837</v>
+      </c>
+      <c r="AH20" s="2" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="AI20" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AJ20" s="2" t="n">
+        <v>0.831</v>
+      </c>
+      <c r="AK20" s="2" t="n">
+        <v>0.822</v>
+      </c>
+      <c r="AL20" s="2" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="AM20" s="2" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="AN20" s="2" t="n">
+        <v>-19.73</v>
+      </c>
+      <c r="AO20" s="2" t="n">
+        <v>23.02</v>
+      </c>
+      <c r="AP20" s="2" t="n">
+        <v>36.46</v>
+      </c>
+      <c r="AQ20" s="2" t="n">
+        <v>13.01</v>
+      </c>
+      <c r="AR20" s="2" t="n">
+        <v>-0.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2099,6 +2855,42 @@
         <is>
           <t>柱≥0</t>
         </is>
+      </c>
+      <c r="AG21" s="2" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="AH21" s="2" t="n">
+        <v>1.022</v>
+      </c>
+      <c r="AI21" s="2" t="n">
+        <v>1.035</v>
+      </c>
+      <c r="AJ21" s="2" t="n">
+        <v>1.057</v>
+      </c>
+      <c r="AK21" s="2" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="AL21" s="2" t="n">
+        <v>1.094</v>
+      </c>
+      <c r="AM21" s="2" t="n">
+        <v>1.233</v>
+      </c>
+      <c r="AN21" s="2" t="n">
+        <v>-18.76</v>
+      </c>
+      <c r="AO21" s="2" t="n">
+        <v>-68.89</v>
+      </c>
+      <c r="AP21" s="2" t="n">
+        <v>-35.91</v>
+      </c>
+      <c r="AQ21" s="2" t="n">
+        <v>-38.16</v>
+      </c>
+      <c r="AR21" s="2" t="n">
+        <v>-53.25</v>
       </c>
     </row>
     <row r="22">
@@ -2173,6 +2965,42 @@
         <is>
           <t>柱≥0</t>
         </is>
+      </c>
+      <c r="AG22" s="2" t="n">
+        <v>1.803</v>
+      </c>
+      <c r="AH22" s="2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AI22" s="2" t="n">
+        <v>1.838</v>
+      </c>
+      <c r="AJ22" s="2" t="n">
+        <v>1.837</v>
+      </c>
+      <c r="AK22" s="2" t="n">
+        <v>1.839</v>
+      </c>
+      <c r="AL22" s="2" t="n">
+        <v>1.821</v>
+      </c>
+      <c r="AM22" s="2" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="AN22" s="2" t="n">
+        <v>-88.33</v>
+      </c>
+      <c r="AO22" s="2" t="n">
+        <v>-36.8</v>
+      </c>
+      <c r="AP22" s="2" t="n">
+        <v>-5.59</v>
+      </c>
+      <c r="AQ22" s="2" t="n">
+        <v>-6.13</v>
+      </c>
+      <c r="AR22" s="2" t="n">
+        <v>-16.43</v>
       </c>
     </row>
     <row r="23">
@@ -2242,6 +3070,42 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG23" s="2" t="n">
+        <v>2.303</v>
+      </c>
+      <c r="AH23" s="2" t="n">
+        <v>2.254</v>
+      </c>
+      <c r="AI23" s="2" t="n">
+        <v>2.238</v>
+      </c>
+      <c r="AJ23" s="2" t="n">
+        <v>2.231</v>
+      </c>
+      <c r="AK23" s="2" t="n">
+        <v>2.202</v>
+      </c>
+      <c r="AL23" s="2" t="n">
+        <v>2.189</v>
+      </c>
+      <c r="AM23" s="2" t="n">
+        <v>2.023</v>
+      </c>
+      <c r="AN23" s="2" t="n">
+        <v>86.75</v>
+      </c>
+      <c r="AO23" s="2" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="AP23" s="2" t="n">
+        <v>30.73</v>
+      </c>
+      <c r="AQ23" s="2" t="n">
+        <v>40.08</v>
+      </c>
+      <c r="AR23" s="2" t="n">
+        <v>24.35</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2316,6 +3180,42 @@
           <t>背离</t>
         </is>
       </c>
+      <c r="AG24" s="2" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="AH24" s="2" t="n">
+        <v>1.494</v>
+      </c>
+      <c r="AI24" s="2" t="n">
+        <v>1.532</v>
+      </c>
+      <c r="AJ24" s="2" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="AK24" s="2" t="n">
+        <v>1.587</v>
+      </c>
+      <c r="AL24" s="2" t="n">
+        <v>1.747</v>
+      </c>
+      <c r="AM24" s="2" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="AN24" s="2" t="n">
+        <v>-75.12</v>
+      </c>
+      <c r="AO24" s="2" t="n">
+        <v>-108.87</v>
+      </c>
+      <c r="AP24" s="2" t="n">
+        <v>-40.7</v>
+      </c>
+      <c r="AQ24" s="2" t="n">
+        <v>-90.11</v>
+      </c>
+      <c r="AR24" s="2" t="n">
+        <v>-20.35</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2390,6 +3290,42 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG25" s="2" t="n">
+        <v>1.068</v>
+      </c>
+      <c r="AH25" s="2" t="n">
+        <v>1.051</v>
+      </c>
+      <c r="AI25" s="2" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="AJ25" s="2" t="n">
+        <v>1.042</v>
+      </c>
+      <c r="AK25" s="2" t="n">
+        <v>1.029</v>
+      </c>
+      <c r="AL25" s="2" t="n">
+        <v>1.126</v>
+      </c>
+      <c r="AM25" s="2" t="n">
+        <v>0.966</v>
+      </c>
+      <c r="AN25" s="2" t="n">
+        <v>82.45999999999999</v>
+      </c>
+      <c r="AO25" s="2" t="n">
+        <v>55.31</v>
+      </c>
+      <c r="AP25" s="2" t="n">
+        <v>-64.81</v>
+      </c>
+      <c r="AQ25" s="2" t="n">
+        <v>16.38</v>
+      </c>
+      <c r="AR25" s="2" t="n">
+        <v>53.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2459,6 +3395,42 @@
         <is>
           <t>柱≥0</t>
         </is>
+      </c>
+      <c r="AG26" s="2" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AH26" s="2" t="n">
+        <v>1.272</v>
+      </c>
+      <c r="AI26" s="2" t="n">
+        <v>1.296</v>
+      </c>
+      <c r="AJ26" s="2" t="n">
+        <v>1.293</v>
+      </c>
+      <c r="AK26" s="2" t="n">
+        <v>1.259</v>
+      </c>
+      <c r="AL26" s="2" t="n">
+        <v>1.238</v>
+      </c>
+      <c r="AM26" s="2" t="n">
+        <v>1.198</v>
+      </c>
+      <c r="AN26" s="2" t="n">
+        <v>-72.09999999999999</v>
+      </c>
+      <c r="AO26" s="2" t="n">
+        <v>-36.98</v>
+      </c>
+      <c r="AP26" s="2" t="n">
+        <v>50.13</v>
+      </c>
+      <c r="AQ26" s="2" t="n">
+        <v>-6.64</v>
+      </c>
+      <c r="AR26" s="2" t="n">
+        <v>19.86</v>
       </c>
     </row>
     <row r="27">
@@ -2528,6 +3500,42 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG27" s="2" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="AH27" s="2" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="AI27" s="2" t="n">
+        <v>0.8110000000000001</v>
+      </c>
+      <c r="AJ27" s="2" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="AK27" s="2" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="AL27" s="2" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="AM27" s="2" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="AN27" s="2" t="n">
+        <v>-5.83</v>
+      </c>
+      <c r="AO27" s="2" t="n">
+        <v>-54.26</v>
+      </c>
+      <c r="AP27" s="2" t="n">
+        <v>-27.21</v>
+      </c>
+      <c r="AQ27" s="2" t="n">
+        <v>-68.75</v>
+      </c>
+      <c r="AR27" s="2" t="n">
+        <v>-18.31</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2601,6 +3609,42 @@
         <is>
           <t>无背离</t>
         </is>
+      </c>
+      <c r="AG28" s="2" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="AH28" s="2" t="n">
+        <v>0.6860000000000001</v>
+      </c>
+      <c r="AI28" s="2" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="AJ28" s="2" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="AK28" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AL28" s="2" t="n">
+        <v>0.732</v>
+      </c>
+      <c r="AM28" s="2" t="n">
+        <v>0.639</v>
+      </c>
+      <c r="AN28" s="2" t="n">
+        <v>130.6</v>
+      </c>
+      <c r="AO28" s="2" t="n">
+        <v>79.86</v>
+      </c>
+      <c r="AP28" s="2" t="n">
+        <v>-44.51</v>
+      </c>
+      <c r="AQ28" s="2" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="AR28" s="2" t="n">
+        <v>53.08</v>
       </c>
     </row>
     <row r="29">
@@ -2672,6 +3716,42 @@
           <t>背离</t>
         </is>
       </c>
+      <c r="AG29" s="2" t="n">
+        <v>2.317</v>
+      </c>
+      <c r="AH29" s="2" t="n">
+        <v>2.311</v>
+      </c>
+      <c r="AI29" s="2" t="n">
+        <v>2.349</v>
+      </c>
+      <c r="AJ29" s="2" t="n">
+        <v>2.411</v>
+      </c>
+      <c r="AK29" s="2" t="n">
+        <v>2.434</v>
+      </c>
+      <c r="AL29" s="2" t="n">
+        <v>2.709</v>
+      </c>
+      <c r="AM29" s="2" t="n">
+        <v>2.867</v>
+      </c>
+      <c r="AN29" s="2" t="n">
+        <v>-46.18</v>
+      </c>
+      <c r="AO29" s="2" t="n">
+        <v>-99.40000000000001</v>
+      </c>
+      <c r="AP29" s="2" t="n">
+        <v>-36.79</v>
+      </c>
+      <c r="AQ29" s="2" t="n">
+        <v>-90.19</v>
+      </c>
+      <c r="AR29" s="2" t="n">
+        <v>-22</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2738,6 +3818,42 @@
           <t>背离</t>
         </is>
       </c>
+      <c r="AG30" s="2" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AH30" s="2" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="AI30" s="2" t="n">
+        <v>0.9360000000000001</v>
+      </c>
+      <c r="AJ30" s="2" t="n">
+        <v>0.948</v>
+      </c>
+      <c r="AK30" s="2" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="AL30" s="2" t="n">
+        <v>1.047</v>
+      </c>
+      <c r="AM30" s="2" t="n">
+        <v>1.029</v>
+      </c>
+      <c r="AN30" s="2" t="n">
+        <v>-34.21</v>
+      </c>
+      <c r="AO30" s="2" t="n">
+        <v>-27.36</v>
+      </c>
+      <c r="AP30" s="2" t="n">
+        <v>-66.81999999999999</v>
+      </c>
+      <c r="AQ30" s="2" t="n">
+        <v>-24.82</v>
+      </c>
+      <c r="AR30" s="2" t="n">
+        <v>-2.22</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2810,9 +3926,45 @@
           <t>无背离</t>
         </is>
       </c>
+      <c r="AG31" s="2" t="n">
+        <v>1.744</v>
+      </c>
+      <c r="AH31" s="2" t="n">
+        <v>1.701</v>
+      </c>
+      <c r="AI31" s="2" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="AJ31" s="2" t="n">
+        <v>1.727</v>
+      </c>
+      <c r="AK31" s="2" t="n">
+        <v>1.762</v>
+      </c>
+      <c r="AL31" s="2" t="n">
+        <v>1.857</v>
+      </c>
+      <c r="AM31" s="2" t="n">
+        <v>1.669</v>
+      </c>
+      <c r="AN31" s="2" t="n">
+        <v>104.45</v>
+      </c>
+      <c r="AO31" s="2" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="AP31" s="2" t="n">
+        <v>-97.76000000000001</v>
+      </c>
+      <c r="AQ31" s="2" t="n">
+        <v>16.49</v>
+      </c>
+      <c r="AR31" s="2" t="n">
+        <v>28.06</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF1"/>
+  <autoFilter ref="A1:AR1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2823,7 +3975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2873,7 +4025,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>【⑥ 东吴风险趋势信号】(逆向复现v2, 最右7列)</t>
+          <t>【⑥ 东吴风险趋势信号】(逆向复现v2)</t>
         </is>
       </c>
     </row>
@@ -3123,26 +4275,57 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>【⑤ ETF 专属 — 趋势/Mansfield RS】</t>
+          <t>【⑦ 均线 MV 与年化斜率】(最右 12 列)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
+          <t xml:space="preserve">  ND MV: N日收盘均线(前复权)最新值, N=5/10/20/30/50/100/200。历史不足N个交易日留空</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
+          <t xml:space="preserve">  ND斜率: (N日均线最新 ÷ 5个交易日前的N日均线 - 1) ×52, 年化%。N=10/20/50/100/200, 正值=均线上行</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           (200D斜率与【⑤】年线斜率同公式; 不足N+5个交易日留空)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>【⑤ ETF 专属 — 趋势/Mansfield RS】</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  MRS_沪深300_1W / MRS_沪深300_4W: MRS_沪深300 分数的 5日 / 20日 变化</t>
         </is>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-26
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -828,19 +828,19 @@
         <v>3.525</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>17.75</v>
+        <v>0.1775</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>-32.4</v>
+        <v>-0.324</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>-62.09</v>
+        <v>-0.6209</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>-20.54</v>
+        <v>-0.2054</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>13.55</v>
+        <v>0.1355</v>
       </c>
     </row>
     <row r="3">
@@ -934,19 +934,19 @@
         <v>1.518</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>-48.78</v>
+        <v>-0.4878</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>-40.98</v>
+        <v>-0.4098</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>1.93</v>
+        <v>0.0193</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>-12.35</v>
+        <v>-0.1235</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>-11.25</v>
+        <v>-0.1125</v>
       </c>
     </row>
     <row r="4">
@@ -1042,19 +1042,19 @@
         <v>0.72</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>-100.65</v>
+        <v>-1.0065</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>-16.78</v>
+        <v>-0.1678</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>8.4</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>-33.18</v>
+        <v>-0.3318</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>-30.97</v>
+        <v>-0.3097</v>
       </c>
     </row>
     <row r="5">
@@ -1156,19 +1156,19 @@
         <v>1.501</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>10.67</v>
+        <v>0.1067</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>137.53</v>
+        <v>1.3753</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>85.26000000000001</v>
+        <v>0.8526</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>1.32</v>
+        <v>0.0132</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>44.25</v>
+        <v>0.4425</v>
       </c>
     </row>
     <row r="6">
@@ -1260,19 +1260,19 @@
         <v>0.833</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>55.73</v>
+        <v>0.5573</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>-22.14</v>
+        <v>-0.2214</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>-14.4</v>
+        <v>-0.144</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>6.68</v>
+        <v>0.0668</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>-3.37</v>
+        <v>-0.0337</v>
       </c>
     </row>
     <row r="7">
@@ -1370,19 +1370,19 @@
         <v>3.044</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>-27.45</v>
+        <v>-0.2745</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>-4.84</v>
+        <v>-0.0484</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>-8.359999999999999</v>
+        <v>-0.08359999999999999</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>-4.98</v>
+        <v>-0.0498</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>-1.99</v>
+        <v>-0.0199</v>
       </c>
     </row>
     <row r="8">
@@ -1476,19 +1476,19 @@
         <v>4.72</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-24.96</v>
+        <v>-0.2496</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>-20.16</v>
+        <v>-0.2016</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>-24.29</v>
+        <v>-0.2429</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>-12.79</v>
+        <v>-0.1279</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>1.81</v>
+        <v>0.0181</v>
       </c>
     </row>
     <row r="9">
@@ -1580,19 +1580,19 @@
         <v>8.004</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>17.49</v>
+        <v>0.1749</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>-2.46</v>
+        <v>-0.0246</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>-27.17</v>
+        <v>-0.2717</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>-15.22</v>
+        <v>-0.1522</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>14.34</v>
+        <v>0.1434</v>
       </c>
     </row>
     <row r="10">
@@ -1704,19 +1704,19 @@
         <v>3.213</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>-66.05</v>
+        <v>-0.6605</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>-24.2</v>
+        <v>-0.242</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>38.55</v>
+        <v>0.3855</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>2.92</v>
+        <v>0.0292</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>10.99</v>
+        <v>0.1099</v>
       </c>
     </row>
     <row r="11">
@@ -1812,19 +1812,19 @@
         <v>0.533</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>-74.11</v>
+        <v>-0.7411</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>-21.13</v>
+        <v>-0.2113</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>-23.89</v>
+        <v>-0.2389</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>-3.41</v>
+        <v>-0.0341</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>-13.66</v>
+        <v>-0.1366</v>
       </c>
     </row>
     <row r="12">
@@ -1918,19 +1918,19 @@
         <v>0.372</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>31.08</v>
+        <v>0.3108</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>-10.25</v>
+        <v>-0.1025</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>15.07</v>
+        <v>0.1507</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>7.77</v>
+        <v>0.07770000000000001</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>-4.42</v>
+        <v>-0.0442</v>
       </c>
     </row>
     <row r="13">
@@ -2024,19 +2024,19 @@
         <v>0.829</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>-79.61</v>
+        <v>-0.7961</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>-17.88</v>
+        <v>-0.1788</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>-5.97</v>
+        <v>-0.0597</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>-7.03</v>
+        <v>-0.0703</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>-11.82</v>
+        <v>-0.1182</v>
       </c>
     </row>
     <row r="14">
@@ -2126,19 +2126,19 @@
         <v>3.216</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>37.8</v>
+        <v>0.378</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>23.8</v>
+        <v>0.238</v>
       </c>
       <c r="AP14" s="2" t="n">
-        <v>-9.800000000000001</v>
+        <v>-0.098</v>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>-18.05</v>
+        <v>-0.1805</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>8.74</v>
+        <v>0.08740000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -2234,19 +2234,19 @@
         <v>0.336</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>60.67</v>
+        <v>0.6067</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>0.25</v>
+        <v>0.0025</v>
       </c>
       <c r="AP15" s="2" t="n">
-        <v>35.53</v>
+        <v>0.3553</v>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>7.19</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="AR15" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.0057</v>
       </c>
     </row>
     <row r="16">
@@ -2340,19 +2340,19 @@
         <v>1.303</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>-17.08</v>
+        <v>-0.1708</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>61.43</v>
+        <v>0.6143</v>
       </c>
       <c r="AP16" s="2" t="n">
-        <v>-10.21</v>
+        <v>-0.1021</v>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>-50.41</v>
+        <v>-0.5041</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>-1.46</v>
+        <v>-0.0146</v>
       </c>
     </row>
     <row r="17">
@@ -2446,19 +2446,19 @@
         <v>0.475</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>-96.73</v>
+        <v>-0.9673</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>-25.26</v>
+        <v>-0.2526</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>10.53</v>
+        <v>0.1053</v>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>-41.93</v>
+        <v>-0.4193</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>-45.99</v>
+        <v>-0.4599</v>
       </c>
     </row>
     <row r="18">
@@ -2554,19 +2554,19 @@
         <v>1.234</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-18</v>
+        <v>-0.18</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>-13.38</v>
+        <v>-0.1338</v>
       </c>
       <c r="AP18" s="2" t="n">
-        <v>-44.15</v>
+        <v>-0.4415</v>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>-34.29</v>
+        <v>-0.3429</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>-6.22</v>
+        <v>-0.0622</v>
       </c>
     </row>
     <row r="19">
@@ -2662,19 +2662,19 @@
         <v>1.021</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>139.91</v>
+        <v>1.3991</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>15.79</v>
+        <v>0.1579</v>
       </c>
       <c r="AP19" s="2" t="n">
-        <v>-117.87</v>
+        <v>-1.1787</v>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>28.58</v>
+        <v>0.2858</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>43.32</v>
+        <v>0.4332</v>
       </c>
     </row>
     <row r="20">
@@ -2768,19 +2768,19 @@
         <v>0.798</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>-19.73</v>
+        <v>-0.1973</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>23.02</v>
+        <v>0.2302</v>
       </c>
       <c r="AP20" s="2" t="n">
-        <v>36.46</v>
+        <v>0.3646</v>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>13.01</v>
+        <v>0.1301</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>-0.65</v>
+        <v>-0.0065</v>
       </c>
     </row>
     <row r="21">
@@ -2878,19 +2878,19 @@
         <v>1.233</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>-18.76</v>
+        <v>-0.1876</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>-68.89</v>
+        <v>-0.6889</v>
       </c>
       <c r="AP21" s="2" t="n">
-        <v>-35.91</v>
+        <v>-0.3591</v>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>-38.16</v>
+        <v>-0.3816</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>-53.25</v>
+        <v>-0.5325</v>
       </c>
     </row>
     <row r="22">
@@ -2988,19 +2988,19 @@
         <v>1.89</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>-88.33</v>
+        <v>-0.8833</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>-36.8</v>
+        <v>-0.368</v>
       </c>
       <c r="AP22" s="2" t="n">
-        <v>-5.59</v>
+        <v>-0.0559</v>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>-6.13</v>
+        <v>-0.0613</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>-16.43</v>
+        <v>-0.1643</v>
       </c>
     </row>
     <row r="23">
@@ -3092,19 +3092,19 @@
         <v>2.023</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>86.75</v>
+        <v>0.8675</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>61.8</v>
+        <v>0.618</v>
       </c>
       <c r="AP23" s="2" t="n">
-        <v>30.73</v>
+        <v>0.3073</v>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>40.08</v>
+        <v>0.4008</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>24.35</v>
+        <v>0.2435</v>
       </c>
     </row>
     <row r="24">
@@ -3202,19 +3202,19 @@
         <v>1.816</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>-75.12</v>
+        <v>-0.7512</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>-108.87</v>
+        <v>-1.0887</v>
       </c>
       <c r="AP24" s="2" t="n">
-        <v>-40.7</v>
+        <v>-0.407</v>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>-90.11</v>
+        <v>-0.9011</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>-20.35</v>
+        <v>-0.2035</v>
       </c>
     </row>
     <row r="25">
@@ -3312,19 +3312,19 @@
         <v>0.966</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>82.45999999999999</v>
+        <v>0.8246</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>55.31</v>
+        <v>0.5531</v>
       </c>
       <c r="AP25" s="2" t="n">
-        <v>-64.81</v>
+        <v>-0.6481</v>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>16.38</v>
+        <v>0.1638</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>53.69</v>
+        <v>0.5369</v>
       </c>
     </row>
     <row r="26">
@@ -3418,19 +3418,19 @@
         <v>1.198</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>-72.09999999999999</v>
+        <v>-0.721</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>-36.98</v>
+        <v>-0.3698</v>
       </c>
       <c r="AP26" s="2" t="n">
-        <v>50.13</v>
+        <v>0.5013</v>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>-6.64</v>
+        <v>-0.0664</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>19.86</v>
+        <v>0.1986</v>
       </c>
     </row>
     <row r="27">
@@ -3522,19 +3522,19 @@
         <v>0.992</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>-5.83</v>
+        <v>-0.0583</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>-54.26</v>
+        <v>-0.5426</v>
       </c>
       <c r="AP27" s="2" t="n">
-        <v>-27.21</v>
+        <v>-0.2721</v>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>-68.75</v>
+        <v>-0.6875</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>-18.31</v>
+        <v>-0.1831</v>
       </c>
     </row>
     <row r="28">
@@ -3632,19 +3632,19 @@
         <v>0.639</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>130.6</v>
+        <v>1.306</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>79.86</v>
+        <v>0.7986</v>
       </c>
       <c r="AP28" s="2" t="n">
-        <v>-44.51</v>
+        <v>-0.4451</v>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>11.38</v>
+        <v>0.1138</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>53.08</v>
+        <v>0.5308</v>
       </c>
     </row>
     <row r="29">
@@ -3738,19 +3738,19 @@
         <v>2.867</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-46.18</v>
+        <v>-0.4618</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>-99.40000000000001</v>
+        <v>-0.994</v>
       </c>
       <c r="AP29" s="2" t="n">
-        <v>-36.79</v>
+        <v>-0.3679</v>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>-90.19</v>
+        <v>-0.9019</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>-22</v>
+        <v>-0.22</v>
       </c>
     </row>
     <row r="30">
@@ -3840,19 +3840,19 @@
         <v>1.029</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>-34.21</v>
+        <v>-0.3421</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>-27.36</v>
+        <v>-0.2736</v>
       </c>
       <c r="AP30" s="2" t="n">
-        <v>-66.81999999999999</v>
+        <v>-0.6682</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>-24.82</v>
+        <v>-0.2482</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>-2.22</v>
+        <v>-0.0222</v>
       </c>
     </row>
     <row r="31">
@@ -3948,19 +3948,19 @@
         <v>1.669</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>104.45</v>
+        <v>1.0445</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>12.39</v>
+        <v>0.1239</v>
       </c>
       <c r="AP31" s="2" t="n">
-        <v>-97.76000000000001</v>
+        <v>-0.9776</v>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>16.49</v>
+        <v>0.1649</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>28.06</v>
+        <v>0.2806</v>
       </c>
     </row>
   </sheetData>
@@ -4289,14 +4289,14 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ND斜率: (N日均线最新 ÷ 5个交易日前的N日均线 - 1) ×52, 年化%。N=10/20/50/100/200, 正值=均线上行</t>
+          <t xml:space="preserve">  ND斜率: (N日均线最新 ÷ 5个交易日前的N日均线 - 1) ×52, 年化小数(0.1=10%)。N=10/20/50/100/200, 正值=均线上行</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">           (200D斜率与【⑤】年线斜率同公式; 不足N+5个交易日留空)</t>
+          <t xml:space="preserve">           (与【⑤】年线斜率列的×100百分比口径不同, 本列为原始×52; 不足N+5个交易日留空)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-28
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.312</v>
+        <v>3.159</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -774,30 +774,32 @@
       <c r="R2" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>13.55</v>
+        <v>11.15</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>1.65</v>
+        <v>-0.88</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-0.02</v>
+        <v>-3.61</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-2.5</v>
+        <v>-3.89</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -807,40 +809,40 @@
         </is>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>3.388</v>
+        <v>3.342</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>3.35</v>
+        <v>3.332</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>3.365</v>
+        <v>3.351</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>3.427</v>
+        <v>3.41</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>3.46</v>
+        <v>3.454</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>3.739</v>
+        <v>3.732</v>
       </c>
       <c r="AM2" s="2" t="n">
         <v>3.525</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.1775</v>
+        <v>-0.2392</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>-0.324</v>
+        <v>-0.4133</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>-0.6209</v>
+        <v>-0.5729</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>-0.2054</v>
+        <v>-0.2645</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.1355</v>
+        <v>0.1115</v>
       </c>
     </row>
     <row r="3">
@@ -855,10 +857,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.453</v>
+        <v>1.452</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>93.48999999999999</v>
+        <v>7.34</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -868,7 +870,9 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N3" s="2" t="n">
         <v>2</v>
       </c>
@@ -886,22 +890,22 @@
       </c>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-11.25</v>
+        <v>-11.42</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-0.65</v>
+        <v>1.56</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>1.5</v>
+        <v>3.93</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>1.62</v>
+        <v>3.33</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>67.09999999999999</v>
+        <v>65.8</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -919,7 +923,7 @@
         <v>1.456</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>1.472</v>
+        <v>1.47</v>
       </c>
       <c r="AJ3" s="2" t="n">
         <v>1.482</v>
@@ -928,25 +932,25 @@
         <v>1.49</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>1.473</v>
+        <v>1.472</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>1.518</v>
+        <v>1.517</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>-0.4878</v>
+        <v>-0.3039</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>-0.4098</v>
+        <v>-0.3724</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>0.0193</v>
+        <v>0.0073</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>-0.1235</v>
+        <v>-0.1367</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>-0.1125</v>
+        <v>-0.1142</v>
       </c>
     </row>
     <row r="4">
@@ -961,10 +965,10 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.646</v>
+        <v>0.645</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>90.17</v>
+        <v>-2.04</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -994,22 +998,22 @@
       </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-30.97</v>
+        <v>-31.04</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-8.91</v>
+        <v>-6.88</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>0.59</v>
+        <v>3.04</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>3.34</v>
+        <v>4.06</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>69.2</v>
+        <v>67.2</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
@@ -1021,40 +1025,40 @@
         </is>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>0.654</v>
+        <v>0.653</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.654</v>
+        <v>0.652</v>
       </c>
       <c r="AI4" s="2" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="AJ4" s="2" t="n">
         <v>0.664</v>
-      </c>
-      <c r="AJ4" s="2" t="n">
-        <v>0.665</v>
       </c>
       <c r="AK4" s="2" t="n">
         <v>0.669</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>0.665</v>
+        <v>0.664</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>0.72</v>
+        <v>0.719</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>-1.0065</v>
+        <v>-0.8391999999999999</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>-0.1678</v>
+        <v>-0.2421</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.0404</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>-0.3318</v>
+        <v>-0.3439</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>-0.3097</v>
+        <v>-0.3104</v>
       </c>
     </row>
     <row r="5">
@@ -1069,7 +1073,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.749</v>
+        <v>1.751</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>101.26</v>
@@ -1092,7 +1096,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -1106,27 +1110,27 @@
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>44.25</v>
+        <v>43.86</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>27.01</v>
+        <v>29.85</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-1.8</v>
+        <v>4.68</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>18.99</v>
+        <v>19.15</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>97.09999999999999</v>
+        <v>97</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
@@ -1135,40 +1139,40 @@
         </is>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>1.732</v>
+        <v>1.734</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>1.758</v>
+        <v>1.757</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>1.719</v>
+        <v>1.729</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>1.664</v>
+        <v>1.672</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>1.596</v>
+        <v>1.601</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>1.573</v>
+        <v>1.574</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>1.501</v>
+        <v>1.503</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.1067</v>
+        <v>-0.124</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>1.3753</v>
+        <v>1.4322</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>0.8526</v>
+        <v>0.8235</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.0132</v>
+        <v>0.0264</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.4425</v>
+        <v>0.4386</v>
       </c>
     </row>
     <row r="6">
@@ -1183,7 +1187,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.841</v>
+        <v>0.845</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>4.26</v>
@@ -1203,31 +1207,29 @@
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R6" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-3.37</v>
+        <v>-2.84</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>3.92</v>
+        <v>6.83</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>2.21</v>
+        <v>5.5</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>1.74</v>
+        <v>5.63</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>58.2</v>
+        <v>57.6</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
@@ -1239,16 +1241,16 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>0.856</v>
+        <v>0.858</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>0.839</v>
+        <v>0.843</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>0.842</v>
+        <v>0.841</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>0.86</v>
+        <v>0.857</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>0.864</v>
@@ -1260,19 +1262,19 @@
         <v>0.833</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.5573</v>
+        <v>0.884</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>-0.2214</v>
+        <v>-0.09569999999999999</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>-0.144</v>
+        <v>-0.1177</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.0668</v>
+        <v>0.0643</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>-0.0337</v>
+        <v>-0.0284</v>
       </c>
     </row>
     <row r="7">
@@ -1287,10 +1289,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.959</v>
+        <v>2.922</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>55.83</v>
+        <v>2.95</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -1300,44 +1302,38 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R7" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S7" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T7" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-1.99</v>
+        <v>-2.55</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>2.21</v>
+        <v>3.21</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>2.02</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>1.72</v>
+        <v>2.33</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>40.6</v>
+        <v>35</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
@@ -1349,40 +1345,40 @@
         </is>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>2.99</v>
+        <v>2.98</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>2.98</v>
+        <v>2.975</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>3.005</v>
+        <v>3</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>3.007</v>
+        <v>3.004</v>
       </c>
       <c r="AK7" s="2" t="n">
         <v>3.018</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>3.02</v>
+        <v>3.019</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>3.044</v>
+        <v>3.043</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>-0.2745</v>
+        <v>-0.2703</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>-0.0484</v>
+        <v>-0.1326</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>-0.08359999999999999</v>
+        <v>-0.0585</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>-0.0498</v>
+        <v>-0.07439999999999999</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>-0.0199</v>
+        <v>-0.0255</v>
       </c>
     </row>
     <row r="8">
@@ -1397,10 +1393,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.515</v>
+        <v>4.417</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>10.81</v>
+        <v>9.76</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1420,32 +1416,32 @@
       <c r="R8" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S8" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>1.81</v>
+        <v>0.53</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.32</v>
+        <v>1.37</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>0.23</v>
+        <v>0.08</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>1.4</v>
+        <v>-0</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1455,40 +1451,40 @@
         </is>
       </c>
       <c r="AG8" s="2" t="n">
-        <v>4.582</v>
+        <v>4.548</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>4.564</v>
+        <v>4.548</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>4.603</v>
+        <v>4.59</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>4.632</v>
+        <v>4.621</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>4.658</v>
+        <v>4.655</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>4.777</v>
+        <v>4.772</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>4.72</v>
+        <v>4.719</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-0.2496</v>
+        <v>-0.3949</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>-0.2016</v>
+        <v>-0.2943</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>-0.2429</v>
+        <v>-0.2265</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>-0.1279</v>
+        <v>-0.16</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>0.0181</v>
+        <v>0.0053</v>
       </c>
     </row>
     <row r="9">
@@ -1503,10 +1499,10 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.65</v>
+        <v>7.44</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>28.85</v>
+        <v>52.12</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1526,30 +1522,32 @@
       <c r="R9" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>14.34</v>
+        <v>12.78</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>3</v>
+        <v>2.38</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-0.15</v>
+        <v>-1.63</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-0.77</v>
+        <v>-1.16</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>20.8</v>
+        <v>18.6</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
@@ -1559,40 +1557,40 @@
         </is>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>7.803</v>
+        <v>7.727</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>7.72</v>
+        <v>7.705</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>7.763</v>
+        <v>7.741</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>7.813</v>
+        <v>7.796</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>7.768</v>
+        <v>7.769</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>8.131</v>
+        <v>8.121</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>8.004</v>
+        <v>8.007999999999999</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>0.1749</v>
+        <v>-0.0476</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>-0.0246</v>
+        <v>-0.1752</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>-0.2717</v>
+        <v>-0.1859</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>-0.1522</v>
+        <v>-0.2024</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>0.1434</v>
+        <v>0.1278</v>
       </c>
     </row>
     <row r="10">
@@ -1607,27 +1605,17 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.357</v>
+        <v>3.342</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>114.34</v>
+        <v>100.6</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="n">
         <v>-9</v>
@@ -1639,42 +1627,36 @@
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="n">
-        <v>1</v>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>10.99</v>
+        <v>10.96</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>10.84</v>
+        <v>12.78</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>0.65</v>
+        <v>4.02</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>0.82</v>
+        <v>2.03</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>84.8</v>
+        <v>83.2</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="AB10" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
@@ -1683,40 +1665,40 @@
         </is>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>3.362</v>
+        <v>3.363</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.373</v>
+        <v>3.365</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>3.414</v>
+        <v>3.408</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>3.403</v>
+        <v>3.404</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>3.346</v>
+        <v>3.35</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>3.256</v>
+        <v>3.257</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>3.213</v>
+        <v>3.214</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>-0.6605</v>
+        <v>-0.6296</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>-0.242</v>
+        <v>-0.2962</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>0.3855</v>
+        <v>0.3574</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>0.0292</v>
+        <v>0.0301</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>0.1099</v>
+        <v>0.1096</v>
       </c>
     </row>
     <row r="11">
@@ -1731,10 +1713,10 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.501</v>
+        <v>0.49</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6.73</v>
+        <v>4.78</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1743,7 +1725,9 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M11" s="2" t="n">
         <v>9</v>
       </c>
@@ -1753,33 +1737,29 @@
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R11" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S11" s="2" t="inlineStr"/>
-      <c r="T11" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-13.66</v>
+        <v>-14.2</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-3.41</v>
+        <v>-3.32</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>1.2</v>
+        <v>1.07</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.59</v>
+        <v>0.34</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>33.5</v>
+        <v>29.5</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1787,23 +1767,23 @@
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG11" s="2" t="n">
-        <v>0.507</v>
+        <v>0.504</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>0.505</v>
+        <v>0.503</v>
       </c>
       <c r="AI11" s="2" t="n">
-        <v>0.515</v>
+        <v>0.513</v>
       </c>
       <c r="AJ11" s="2" t="n">
-        <v>0.515</v>
+        <v>0.514</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>0.52</v>
+        <v>0.519</v>
       </c>
       <c r="AL11" s="2" t="n">
         <v>0.518</v>
@@ -1812,19 +1792,19 @@
         <v>0.533</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>-0.7411</v>
+        <v>-0.6731</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>-0.2113</v>
+        <v>-0.3875</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>-0.2389</v>
+        <v>-0.2531</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>-0.0341</v>
+        <v>-0.06419999999999999</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>-0.1366</v>
+        <v>-0.142</v>
       </c>
     </row>
     <row r="12">
@@ -1839,10 +1819,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.375</v>
+        <v>0.376</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>12.91</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1861,31 +1841,29 @@
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R12" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-4.42</v>
+        <v>-3.87</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>3.45</v>
+        <v>6.14</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>1.65</v>
+        <v>5.05</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>2.85</v>
+        <v>5.74</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>65.2</v>
+        <v>64.5</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1900,7 +1878,7 @@
         <v>0.381</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>0.375</v>
+        <v>0.376</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>0.376</v>
@@ -1915,22 +1893,22 @@
         <v>0.364</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>0.372</v>
+        <v>0.371</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>0.3108</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>-0.1025</v>
+        <v>-0.0496</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>0.1507</v>
+        <v>0.1562</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0759</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>-0.0442</v>
+        <v>-0.0387</v>
       </c>
     </row>
     <row r="13">
@@ -1945,10 +1923,10 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.772</v>
+        <v>0.757</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>79.75</v>
+        <v>2.2</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1962,7 +1940,7 @@
         <v>9</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
@@ -1972,26 +1950,26 @@
       </c>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-11.82</v>
+        <v>-12.4</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-3.23</v>
+        <v>-2.89</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>0.59</v>
+        <v>0.89</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>0.66</v>
+        <v>0.96</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>55.2</v>
+        <v>48.6</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -2003,40 +1981,40 @@
         </is>
       </c>
       <c r="AG13" s="2" t="n">
-        <v>0.784</v>
+        <v>0.779</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>0.782</v>
+        <v>0.779</v>
       </c>
       <c r="AI13" s="2" t="n">
-        <v>0.796</v>
+        <v>0.793</v>
       </c>
       <c r="AJ13" s="2" t="n">
-        <v>0.793</v>
+        <v>0.792</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>0.798</v>
+        <v>0.797</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>0.79</v>
+        <v>0.789</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>0.829</v>
+        <v>0.828</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>-0.7961</v>
+        <v>-0.7272</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>-0.1788</v>
+        <v>-0.351</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>-0.0597</v>
+        <v>-0.0882</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>-0.0703</v>
+        <v>-0.1031</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>-0.1182</v>
+        <v>-0.124</v>
       </c>
     </row>
     <row r="14">
@@ -2051,7 +2029,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>3.079</v>
+        <v>2.968</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>43.79</v>
@@ -2074,26 +2052,28 @@
       <c r="R14" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>8.74</v>
+        <v>7.19</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>2.47</v>
+        <v>1.03</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>0.79</v>
+        <v>-1.67</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>2.13</v>
+        <v>0.58</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>39.5</v>
+        <v>37.6</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
@@ -2105,40 +2085,40 @@
         </is>
       </c>
       <c r="AG14" s="2" t="n">
-        <v>3.131</v>
+        <v>3.097</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>3.087</v>
+        <v>3.082</v>
       </c>
       <c r="AI14" s="2" t="n">
-        <v>3.093</v>
+        <v>3.084</v>
       </c>
       <c r="AJ14" s="2" t="n">
-        <v>3.098</v>
+        <v>3.091</v>
       </c>
       <c r="AK14" s="2" t="n">
         <v>3.042</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>3.237</v>
+        <v>3.231</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>3.216</v>
+        <v>3.215</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>0.378</v>
+        <v>0.1544</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>0.238</v>
+        <v>0.0634</v>
       </c>
       <c r="AP14" s="2" t="n">
-        <v>-0.098</v>
+        <v>-0.0147</v>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>-0.1805</v>
+        <v>-0.2309</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.07190000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -2153,7 +2133,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.341</v>
+        <v>0.34</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>40.85</v>
@@ -2175,10 +2155,8 @@
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R15" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
@@ -2186,22 +2164,22 @@
         <v>1</v>
       </c>
       <c r="V15" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.27</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>4.47</v>
+        <v>6.58</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>2.08</v>
+        <v>4.24</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>4.33</v>
+        <v>7.03</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>74.5</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
@@ -2216,7 +2194,7 @@
         <v>0.345</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>0.339</v>
+        <v>0.34</v>
       </c>
       <c r="AI15" s="2" t="n">
         <v>0.339</v>
@@ -2225,7 +2203,7 @@
         <v>0.342</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>0.338</v>
+        <v>0.339</v>
       </c>
       <c r="AL15" s="2" t="n">
         <v>0.325</v>
@@ -2234,19 +2212,19 @@
         <v>0.336</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>0.6067</v>
+        <v>0.7904</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0567</v>
       </c>
       <c r="AP15" s="2" t="n">
-        <v>0.3553</v>
+        <v>0.3489</v>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>0.07190000000000001</v>
+        <v>0.0626</v>
       </c>
       <c r="AR15" s="2" t="n">
-        <v>-0.0057</v>
+        <v>-0.0027</v>
       </c>
     </row>
     <row r="16">
@@ -2261,10 +2239,10 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.129</v>
+        <v>1.098</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>33.19</v>
+        <v>81.33</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -2288,26 +2266,26 @@
         <v>-1</v>
       </c>
       <c r="T16" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-1.46</v>
+        <v>-2.67</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-7.2</v>
+        <v>-7.69</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-1.54</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>5.23</v>
+        <v>4.12</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>44.1</v>
+        <v>41.9</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
@@ -2319,40 +2297,40 @@
         </is>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>1.157</v>
+        <v>1.144</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>1.153</v>
+        <v>1.146</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>1.152</v>
+        <v>1.151</v>
       </c>
       <c r="AJ16" s="2" t="n">
-        <v>1.142</v>
+        <v>1.14</v>
       </c>
       <c r="AK16" s="2" t="n">
         <v>1.129</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>1.213</v>
+        <v>1.209</v>
       </c>
       <c r="AM16" s="2" t="n">
         <v>1.303</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>-0.1708</v>
+        <v>-0.5344</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>0.6143</v>
+        <v>0.4352</v>
       </c>
       <c r="AP16" s="2" t="n">
-        <v>-0.1021</v>
+        <v>0.0424</v>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>-0.5041</v>
+        <v>-0.554</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>-0.0146</v>
+        <v>-0.0267</v>
       </c>
     </row>
     <row r="17">
@@ -2367,10 +2345,10 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.408</v>
+        <v>0.406</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>76.56999999999999</v>
+        <v>-1.36</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -2387,33 +2365,29 @@
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R17" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S17" s="2" t="inlineStr"/>
-      <c r="T17" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-45.99</v>
+        <v>-46.07</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-14.2</v>
+        <v>-12.51</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>1.16</v>
+        <v>2.96</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>3.76</v>
+        <v>4.56</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>52.8</v>
+        <v>51.1</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
@@ -2425,40 +2399,40 @@
         </is>
       </c>
       <c r="AG17" s="2" t="n">
-        <v>0.413</v>
+        <v>0.412</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>0.412</v>
+        <v>0.411</v>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>0.419</v>
+        <v>0.418</v>
       </c>
       <c r="AJ17" s="2" t="n">
-        <v>0.421</v>
+        <v>0.42</v>
       </c>
       <c r="AK17" s="2" t="n">
         <v>0.427</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>0.427</v>
+        <v>0.426</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>0.475</v>
+        <v>0.474</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>-0.9673</v>
+        <v>-0.7622</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>-0.2526</v>
+        <v>-0.3085</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>0.1053</v>
+        <v>0.0549</v>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>-0.4193</v>
+        <v>-0.4214</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>-0.4599</v>
+        <v>-0.4607</v>
       </c>
     </row>
     <row r="18">
@@ -2473,7 +2447,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.121</v>
+        <v>1.086</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>5.68</v>
@@ -2490,40 +2464,40 @@
         <v>9</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-6.22</v>
+        <v>-7.08</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-4.79</v>
+        <v>-5.6</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>1.17</v>
+        <v>-0.34</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>0.13</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
@@ -2533,40 +2507,40 @@
         </is>
       </c>
       <c r="AG18" s="2" t="n">
-        <v>1.139</v>
+        <v>1.129</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>1.125</v>
+        <v>1.122</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>1.146</v>
+        <v>1.141</v>
       </c>
       <c r="AJ18" s="2" t="n">
-        <v>1.156</v>
+        <v>1.151</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>1.172</v>
+        <v>1.171</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>1.215</v>
+        <v>1.211</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>1.234</v>
+        <v>1.233</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-0.18</v>
+        <v>-0.1721</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>-0.1338</v>
+        <v>-0.2658</v>
       </c>
       <c r="AP18" s="2" t="n">
-        <v>-0.4415</v>
+        <v>-0.3384</v>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>-0.3429</v>
+        <v>-0.3953</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>-0.0622</v>
+        <v>-0.0708</v>
       </c>
     </row>
     <row r="19">
@@ -2581,7 +2555,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.083</v>
+        <v>1.035</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>-3.59</v>
@@ -2598,40 +2572,40 @@
       <c r="N19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr">
+      <c r="R19" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>43.32</v>
+        <v>40.97</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>16.99</v>
+        <v>14.18</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>2.1</v>
+        <v>-3.61</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-2.84</v>
+        <v>-3.51</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>-1.9</v>
+        <v>-2.5</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
@@ -2641,58 +2615,58 @@
         </is>
       </c>
       <c r="AG19" s="2" t="n">
-        <v>1.101</v>
+        <v>1.088</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>1.068</v>
+        <v>1.07</v>
       </c>
       <c r="AI19" s="2" t="n">
-        <v>1.068</v>
+        <v>1.065</v>
       </c>
       <c r="AJ19" s="2" t="n">
-        <v>1.085</v>
+        <v>1.082</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>1.107</v>
+        <v>1.105</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>1.182</v>
+        <v>1.181</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>1.021</v>
+        <v>1.022</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>1.3991</v>
+        <v>1.138</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>0.1579</v>
+        <v>0.007</v>
       </c>
       <c r="AP19" s="2" t="n">
-        <v>-1.1787</v>
+        <v>-0.9752</v>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>0.2858</v>
+        <v>0.2121</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>0.4332</v>
+        <v>0.4097</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.839</v>
+        <v>1.018</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>99.92</v>
+        <v>-3.21</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -2701,45 +2675,45 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N20" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R20" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-0.65</v>
+        <v>-53.3</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>9.9</v>
+        <v>-16.71</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>0.8</v>
+        <v>4.09</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>7.37</v>
+        <v>2.67</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>95</v>
+        <v>34.1</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="n">
-        <v>7</v>
-      </c>
+      <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
@@ -2747,58 +2721,58 @@
         </is>
       </c>
       <c r="AG20" s="2" t="n">
-        <v>0.837</v>
+        <v>1.031</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>0.841</v>
+        <v>1.022</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>0.84</v>
+        <v>1.032</v>
       </c>
       <c r="AJ20" s="2" t="n">
-        <v>0.831</v>
+        <v>1.054</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>0.822</v>
+        <v>1.086</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>0.798</v>
+        <v>1.092</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>0.798</v>
+        <v>1.23</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>-0.1973</v>
+        <v>0.0407</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>0.2302</v>
+        <v>-0.5878</v>
       </c>
       <c r="AP20" s="2" t="n">
-        <v>0.3646</v>
+        <v>-0.3605</v>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>0.1301</v>
+        <v>-0.3969</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>-0.0065</v>
+        <v>-0.533</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.025</v>
+        <v>1.749</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-2.39</v>
+        <v>4.5</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2807,45 +2781,41 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="n">
         <v>13</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S21" s="2" t="n">
+      <c r="R21" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-53.25</v>
+        <v>-17.01</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-18.14</v>
+        <v>-3.79</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>2.82</v>
+        <v>1.4</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>1.82</v>
+        <v>-0.39</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>35.1</v>
+        <v>44.4</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2857,76 +2827,82 @@
         </is>
       </c>
       <c r="AG21" s="2" t="n">
-        <v>1.03</v>
+        <v>1.793</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>1.022</v>
+        <v>1.793</v>
       </c>
       <c r="AI21" s="2" t="n">
-        <v>1.035</v>
+        <v>1.83</v>
       </c>
       <c r="AJ21" s="2" t="n">
-        <v>1.057</v>
+        <v>1.835</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>1.087</v>
+        <v>1.838</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>1.094</v>
+        <v>1.82</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>1.233</v>
+        <v>1.889</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>-0.1876</v>
+        <v>-0.7657</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>-0.6889</v>
+        <v>-0.5553</v>
       </c>
       <c r="AP21" s="2" t="n">
-        <v>-0.3591</v>
+        <v>-0.0735</v>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>-0.3816</v>
+        <v>-0.09329999999999999</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>-0.5325</v>
+        <v>-0.1701</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.782</v>
+        <v>2.304</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>93.77</v>
+        <v>101.52</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O22" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr">
@@ -2935,27 +2911,25 @@
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-16.43</v>
+        <v>24.22</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-4.25</v>
+        <v>24.45</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>1.52</v>
+        <v>5.67</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>0.03</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>50.7</v>
+        <v>58.3</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
@@ -2963,166 +2937,178 @@
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG22" s="2" t="n">
-        <v>1.803</v>
+        <v>2.31</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>1.8</v>
+        <v>2.264</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>1.838</v>
+        <v>2.242</v>
       </c>
       <c r="AJ22" s="2" t="n">
-        <v>1.837</v>
+        <v>2.233</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>1.839</v>
+        <v>2.206</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>1.821</v>
+        <v>2.192</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>1.89</v>
+        <v>2.025</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>-0.8833</v>
+        <v>0.9967</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>-0.368</v>
+        <v>0.6111</v>
       </c>
       <c r="AP22" s="2" t="n">
-        <v>-0.0559</v>
+        <v>0.3555</v>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>-0.0613</v>
+        <v>0.3825</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>-0.1643</v>
+        <v>0.2422</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.312</v>
+        <v>1.433</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>78.59</v>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
+        <v>7.28</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N23" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S23" s="2" t="inlineStr"/>
-      <c r="T23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>24.35</v>
+        <v>-21.59</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>22.29</v>
+        <v>-14.9</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>4.72</v>
+        <v>-0.7</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>6.96</v>
+        <v>-6.2</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>54.6</v>
+        <v>3</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>68</v>
+        <v>15</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>2.303</v>
+        <v>1.485</v>
       </c>
       <c r="AH23" s="2" t="n">
-        <v>2.254</v>
+        <v>1.489</v>
       </c>
       <c r="AI23" s="2" t="n">
-        <v>2.238</v>
+        <v>1.522</v>
       </c>
       <c r="AJ23" s="2" t="n">
-        <v>2.231</v>
+        <v>1.562</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>2.202</v>
+        <v>1.585</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>2.189</v>
+        <v>1.739</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>2.023</v>
+        <v>1.814</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>0.8675</v>
+        <v>-0.7641</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>0.618</v>
+        <v>-1.1921</v>
       </c>
       <c r="AP23" s="2" t="n">
-        <v>0.3073</v>
+        <v>-0.3766</v>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>0.4008</v>
+        <v>-0.9557</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>0.2435</v>
+        <v>-0.2159</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.472</v>
+        <v>0.967</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>12.11</v>
+        <v>25.84</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -3132,107 +3118,105 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R24" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T24" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-20.35</v>
+        <v>49.3</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-14.55</v>
+        <v>14.79</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-0.1</v>
+        <v>-8.710000000000001</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-5.53</v>
+        <v>-5.66</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>4.2</v>
+        <v>22.5</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>1.499</v>
+        <v>1.047</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>1.494</v>
+        <v>1.043</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>1.532</v>
+        <v>1.037</v>
       </c>
       <c r="AJ24" s="2" t="n">
-        <v>1.57</v>
+        <v>1.038</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>1.587</v>
+        <v>1.027</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>1.747</v>
+        <v>1.125</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>1.816</v>
+        <v>0.968</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>-0.7512</v>
+        <v>0.005</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>-1.0887</v>
+        <v>0.328</v>
       </c>
       <c r="AP24" s="2" t="n">
-        <v>-0.407</v>
+        <v>-0.5839</v>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>-0.9011</v>
+        <v>0.0934</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>-0.2035</v>
+        <v>0.493</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.038</v>
+        <v>1.264</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>25.84</v>
+        <v>96.61</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -3246,103 +3230,101 @@
         <v>-13</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S25" s="2" t="inlineStr">
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="T25" s="2" t="inlineStr"/>
-      <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>53.69</v>
+        <v>20</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>20.66</v>
+        <v>15.08</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-1.36</v>
+        <v>5.08</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-1.12</v>
+        <v>-2.56</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>24.1</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG25" s="2" t="n">
-        <v>1.068</v>
+        <v>1.273</v>
       </c>
       <c r="AH25" s="2" t="n">
-        <v>1.051</v>
+        <v>1.269</v>
       </c>
       <c r="AI25" s="2" t="n">
-        <v>1.04</v>
+        <v>1.292</v>
       </c>
       <c r="AJ25" s="2" t="n">
-        <v>1.042</v>
+        <v>1.293</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>1.029</v>
+        <v>1.261</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>1.126</v>
+        <v>1.238</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>0.966</v>
+        <v>1.199</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>0.8246</v>
+        <v>-0.6389</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>0.5531</v>
+        <v>-0.4853</v>
       </c>
       <c r="AP25" s="2" t="n">
-        <v>-0.6481</v>
+        <v>0.4967</v>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>0.1638</v>
+        <v>-0.0614</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>0.5369</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.266</v>
+        <v>0.771</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>117.45</v>
+        <v>31.83</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -3352,103 +3334,103 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>19.86</v>
+        <v>-19.44</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>12.84</v>
+        <v>-15.7</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>0.79</v>
+        <v>-1.34</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-3.57</v>
+        <v>-2.46</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>65.90000000000001</v>
+        <v>8</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>1.27</v>
+        <v>0.803</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>1.272</v>
+        <v>0.8</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>1.296</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="AJ26" s="2" t="n">
-        <v>1.293</v>
+        <v>0.823</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>1.259</v>
+        <v>0.828</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>1.238</v>
+        <v>0.924</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>1.198</v>
+        <v>0.991</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>-0.721</v>
+        <v>-0.2651</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>-0.3698</v>
+        <v>-0.6647</v>
       </c>
       <c r="AP26" s="2" t="n">
-        <v>0.5013</v>
+        <v>-0.2026</v>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>-0.0664</v>
+        <v>-0.7403</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>0.1986</v>
+        <v>-0.1944</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.792</v>
+        <v>0.627</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>20.09</v>
+        <v>32.9</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -3458,9 +3440,11 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N27" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
@@ -3468,30 +3452,32 @@
       <c r="R27" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-18.31</v>
+        <v>48.11</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-15.36</v>
+        <v>12.93</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>0.45</v>
+        <v>-10.34</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-1.73</v>
+        <v>-4.73</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>9.5</v>
+        <v>26.9</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
@@ -3501,72 +3487,90 @@
         </is>
       </c>
       <c r="AG27" s="2" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="AH27" s="2" t="n">
-        <v>0.802</v>
+        <v>0.681</v>
       </c>
       <c r="AI27" s="2" t="n">
-        <v>0.8110000000000001</v>
+        <v>0.672</v>
       </c>
       <c r="AJ27" s="2" t="n">
-        <v>0.826</v>
+        <v>0.672</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>0.829</v>
+        <v>0.66</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>0.928</v>
+        <v>0.731</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>0.992</v>
+        <v>0.64</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>-0.0583</v>
+        <v>0.4234</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>-0.5426</v>
+        <v>0.5313</v>
       </c>
       <c r="AP27" s="2" t="n">
-        <v>-0.2721</v>
+        <v>-0.3788</v>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>-0.6875</v>
+        <v>0.038</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>-0.1831</v>
+        <v>0.4811</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.679</v>
+        <v>2.202</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>30.88</v>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
+        <v>3.12</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
@@ -3574,95 +3578,95 @@
       <c r="R28" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S28" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T28" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>53.08</v>
+        <v>-23.34</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>19.76</v>
+        <v>-16.79</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-1.89</v>
+        <v>-1.48</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>0.62</v>
+        <v>-4.98</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>28.5</v>
+        <v>1.1</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG28" s="2" t="n">
-        <v>0.701</v>
+        <v>2.289</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>0.6860000000000001</v>
+        <v>2.299</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>0.674</v>
+        <v>2.334</v>
       </c>
       <c r="AJ28" s="2" t="n">
-        <v>0.674</v>
+        <v>2.397</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>0.66</v>
+        <v>2.429</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>0.732</v>
+        <v>2.696</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>0.639</v>
+        <v>2.862</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>1.306</v>
+        <v>-0.6499</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>0.7986</v>
+        <v>-1.0828</v>
       </c>
       <c r="AP28" s="2" t="n">
-        <v>-0.4451</v>
+        <v>-0.3287</v>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>0.1138</v>
+        <v>-0.955</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>0.5308</v>
+        <v>-0.2334</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2.265</v>
+        <v>0.895</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>10.28</v>
+        <v>3.17</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -3674,7 +3678,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -3682,33 +3686,31 @@
       <c r="R29" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S29" s="2" t="inlineStr"/>
-      <c r="T29" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-22</v>
+        <v>-3.28</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-16.39</v>
+        <v>-6.04</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-0.54</v>
+        <v>-0.28</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-4.55</v>
+        <v>0.4</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA29" s="2" t="n">
-        <v>26</v>
-      </c>
+        <v>-1.6</v>
+      </c>
+      <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AC29" s="2" t="inlineStr"/>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
@@ -3717,58 +3719,58 @@
         </is>
       </c>
       <c r="AG29" s="2" t="n">
-        <v>2.317</v>
+        <v>0.923</v>
       </c>
       <c r="AH29" s="2" t="n">
-        <v>2.311</v>
+        <v>0.919</v>
       </c>
       <c r="AI29" s="2" t="n">
-        <v>2.349</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="AJ29" s="2" t="n">
-        <v>2.411</v>
+        <v>0.944</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>2.434</v>
+        <v>0.956</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>2.709</v>
+        <v>1.045</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>2.867</v>
+        <v>1.029</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-0.4618</v>
+        <v>-0.404</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>-0.994</v>
+        <v>-0.3708</v>
       </c>
       <c r="AP29" s="2" t="n">
-        <v>-0.3679</v>
+        <v>-0.5609</v>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>-0.9019</v>
+        <v>-0.2994</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>-0.22</v>
+        <v>-0.0328</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.919</v>
+        <v>1.643</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>3.17</v>
+        <v>-4.94</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -3780,97 +3782,103 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr">
+      <c r="R30" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S30" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-2.22</v>
+        <v>26.17</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-5.7</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>0.92</v>
+        <v>-2.97</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>0.12</v>
+        <v>-2.69</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="AA30" s="2" t="inlineStr"/>
+        <v>-2.4</v>
+      </c>
+      <c r="AA30" s="2" t="n">
+        <v>29</v>
+      </c>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG30" s="2" t="n">
-        <v>0.93</v>
+        <v>1.724</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>0.921</v>
+        <v>1.702</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>0.9360000000000001</v>
+        <v>1.698</v>
       </c>
       <c r="AJ30" s="2" t="n">
-        <v>0.948</v>
+        <v>1.721</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>0.957</v>
+        <v>1.759</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>1.047</v>
+        <v>1.856</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>1.029</v>
+        <v>1.671</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>-0.3421</v>
+        <v>0.8163</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>-0.2736</v>
+        <v>-0.0474</v>
       </c>
       <c r="AP30" s="2" t="n">
-        <v>-0.6682</v>
+        <v>-0.8075</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>-0.2482</v>
+        <v>0.0864</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>-0.0222</v>
+        <v>0.2617</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.713</v>
+        <v>0.835</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>-4.94</v>
+        <v>99.92</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -3880,87 +3888,81 @@
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R31" s="2" t="inlineStr"/>
       <c r="S31" s="2" t="inlineStr"/>
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>28.06</v>
+        <v>-0.49</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>10.99</v>
+        <v>11.83</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>1.05</v>
+        <v>4.12</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-2.13</v>
+        <v>9.02</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>-1.6</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AD31" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG31" s="2" t="n">
-        <v>1.744</v>
+        <v>0.837</v>
       </c>
       <c r="AH31" s="2" t="n">
-        <v>1.701</v>
+        <v>0.84</v>
       </c>
       <c r="AI31" s="2" t="n">
-        <v>1.704</v>
+        <v>0.841</v>
       </c>
       <c r="AJ31" s="2" t="n">
-        <v>1.727</v>
+        <v>0.833</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>1.762</v>
+        <v>0.823</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>1.857</v>
+        <v>0.799</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>1.669</v>
+        <v>0.798</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>1.0445</v>
+        <v>-0.1914</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>0.1239</v>
+        <v>0.2237</v>
       </c>
       <c r="AP31" s="2" t="n">
-        <v>-0.9776</v>
+        <v>0.336</v>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>0.1649</v>
+        <v>0.1405</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>0.2806</v>
+        <v>-0.0049</v>
       </c>
     </row>
   </sheetData>
@@ -3991,7 +3993,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-24 | 30 只</t>
+          <t>截至: 2026-09-28 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-29
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.159</v>
+        <v>3.162</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -777,29 +777,31 @@
       <c r="S2" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>11.15</v>
+        <v>9.31</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-0.88</v>
+        <v>-0.92</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-3.61</v>
+        <v>-3.68</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-3.89</v>
+        <v>-3.88</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>1</v>
+        <v>-0.5</v>
       </c>
       <c r="AA2" s="2" t="n">
         <v>15</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -809,40 +811,40 @@
         </is>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>3.342</v>
+        <v>3.29</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>3.332</v>
+        <v>3.318</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>3.351</v>
+        <v>3.336</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>3.41</v>
+        <v>3.391</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>3.454</v>
+        <v>3.448</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>3.732</v>
+        <v>3.726</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>3.525</v>
+        <v>3.526</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-0.2392</v>
+        <v>-0.466</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>-0.4133</v>
+        <v>-0.61</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>-0.5729</v>
+        <v>-0.5686</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>-0.2645</v>
+        <v>-0.3284</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.1115</v>
+        <v>0.0931</v>
       </c>
     </row>
     <row r="3">
@@ -857,7 +859,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.452</v>
+        <v>1.444</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>7.34</v>
@@ -874,38 +876,34 @@
         <v>13</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R3" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-11.42</v>
+        <v>-11.45</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>1.56</v>
+        <v>0.89</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>3.93</v>
+        <v>3.28</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>3.33</v>
+        <v>3.38</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>65.8</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -917,16 +915,16 @@
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>1.46</v>
+        <v>1.457</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>1.456</v>
+        <v>1.454</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>1.47</v>
+        <v>1.468</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>1.482</v>
+        <v>1.48</v>
       </c>
       <c r="AK3" s="2" t="n">
         <v>1.49</v>
@@ -938,19 +936,19 @@
         <v>1.517</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>-0.3039</v>
+        <v>-0.2505</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>-0.3724</v>
+        <v>-0.3996</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>0.0073</v>
+        <v>-0.0451</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>-0.1367</v>
+        <v>-0.1568</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>-0.1142</v>
+        <v>-0.1145</v>
       </c>
     </row>
     <row r="4">
@@ -965,7 +963,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.645</v>
+        <v>0.647</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>-2.04</v>
@@ -978,10 +976,8 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>+13/-13</t>
-        </is>
+      <c r="M4" s="2" t="n">
+        <v>-13</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>3</v>
@@ -994,26 +990,26 @@
       </c>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-31.04</v>
+        <v>-31.08</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-6.88</v>
+        <v>-6.58</v>
       </c>
       <c r="X4" s="2" t="n">
         <v>3.04</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>4.06</v>
+        <v>5.22</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>67.2</v>
+        <v>65.7</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
@@ -1025,40 +1021,40 @@
         </is>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>0.653</v>
+        <v>0.65</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.652</v>
+        <v>0.651</v>
       </c>
       <c r="AI4" s="2" t="n">
+        <v>0.662</v>
+      </c>
+      <c r="AJ4" s="2" t="n">
         <v>0.663</v>
-      </c>
-      <c r="AJ4" s="2" t="n">
-        <v>0.664</v>
       </c>
       <c r="AK4" s="2" t="n">
         <v>0.669</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>0.664</v>
+        <v>0.663</v>
       </c>
       <c r="AM4" s="2" t="n">
         <v>0.719</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>-0.8391999999999999</v>
+        <v>-0.7243000000000001</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>-0.2421</v>
+        <v>-0.3086</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>0.0404</v>
+        <v>-0.0466</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>-0.3439</v>
+        <v>-0.3544</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>-0.3104</v>
+        <v>-0.3108</v>
       </c>
     </row>
     <row r="5">
@@ -1073,7 +1069,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.751</v>
+        <v>1.778</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>101.26</v>
@@ -1096,41 +1092,39 @@
       </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>43.86</v>
+        <v>44.15</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>29.85</v>
+        <v>31.51</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>4.68</v>
+        <v>6.95</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>19.15</v>
+        <v>15.63</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>97</v>
+        <v>97.7</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
@@ -1139,40 +1133,40 @@
         </is>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>1.734</v>
+        <v>1.74</v>
       </c>
       <c r="AH5" s="2" t="n">
         <v>1.757</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>1.729</v>
+        <v>1.737</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>1.672</v>
+        <v>1.679</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>1.601</v>
+        <v>1.606</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>1.574</v>
+        <v>1.575</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>1.503</v>
+        <v>1.506</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>-0.124</v>
+        <v>-0.3265</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>1.4322</v>
+        <v>1.3896</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>0.8235</v>
+        <v>0.7763</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.0264</v>
+        <v>0.0701</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.4386</v>
+        <v>0.4415</v>
       </c>
     </row>
     <row r="6">
@@ -1187,7 +1181,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.845</v>
+        <v>0.844</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>4.26</v>
@@ -1214,22 +1208,22 @@
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-2.84</v>
+        <v>-2.9</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>6.83</v>
+        <v>6.64</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>5.5</v>
+        <v>1.86</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>5.63</v>
+        <v>7.35</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>57.6</v>
+        <v>57</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
@@ -1241,16 +1235,16 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>0.858</v>
+        <v>0.853</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>0.843</v>
+        <v>0.845</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>0.841</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>0.857</v>
+        <v>0.854</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>0.864</v>
@@ -1262,19 +1256,19 @@
         <v>0.833</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.884</v>
+        <v>0.7936</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>-0.09569999999999999</v>
+        <v>-0.1664</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>-0.1177</v>
+        <v>-0.174</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.0643</v>
+        <v>0.0567</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>-0.0284</v>
+        <v>-0.029</v>
       </c>
     </row>
     <row r="7">
@@ -1304,7 +1298,7 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -1315,25 +1309,27 @@
       <c r="S7" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-2.55</v>
+        <v>-3.19</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>3.21</v>
+        <v>3.1</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>2.02</v>
+        <v>1.72</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>2.33</v>
+        <v>2.41</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
@@ -1345,40 +1341,40 @@
         </is>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>2.98</v>
+        <v>2.964</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>2.975</v>
+        <v>2.969</v>
       </c>
       <c r="AI7" s="2" t="n">
+        <v>2.994</v>
+      </c>
+      <c r="AJ7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ7" s="2" t="n">
-        <v>3.004</v>
-      </c>
       <c r="AK7" s="2" t="n">
-        <v>3.018</v>
+        <v>3.016</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>3.019</v>
+        <v>3.017</v>
       </c>
       <c r="AM7" s="2" t="n">
         <v>3.043</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>-0.2703</v>
+        <v>-0.3377</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>-0.1326</v>
+        <v>-0.2555</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>-0.0585</v>
+        <v>-0.08459999999999999</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>-0.07439999999999999</v>
+        <v>-0.097</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>-0.0255</v>
+        <v>-0.0319</v>
       </c>
     </row>
     <row r="8">
@@ -1393,7 +1389,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.417</v>
+        <v>4.416</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>9.76</v>
@@ -1419,29 +1415,31 @@
       <c r="S8" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>0.53</v>
+        <v>-0.63</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.37</v>
+        <v>1.24</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>0.08</v>
+        <v>0.19</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>-0</v>
+        <v>-1.3</v>
       </c>
       <c r="AA8" s="2" t="n">
         <v>13</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1451,40 +1449,40 @@
         </is>
       </c>
       <c r="AG8" s="2" t="n">
-        <v>4.548</v>
+        <v>4.51</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>4.548</v>
+        <v>4.534</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>4.59</v>
+        <v>4.576</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>4.621</v>
+        <v>4.608</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>4.655</v>
+        <v>4.65</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>4.772</v>
+        <v>4.767</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>4.719</v>
+        <v>4.718</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-0.3949</v>
+        <v>-0.5197000000000001</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>-0.2943</v>
+        <v>-0.4348</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>-0.2265</v>
+        <v>-0.2484</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.1935</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>0.0053</v>
+        <v>-0.0063</v>
       </c>
     </row>
     <row r="9">
@@ -1499,7 +1497,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.44</v>
+        <v>7.476</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>52.12</v>
@@ -1525,29 +1523,31 @@
       <c r="S9" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>12.78</v>
+        <v>11.37</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>2.38</v>
+        <v>2.77</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-1.63</v>
+        <v>-1</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-1.16</v>
+        <v>-0.96</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>18.6</v>
+        <v>16.9</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
@@ -1557,40 +1557,40 @@
         </is>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>7.727</v>
+        <v>7.646</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>7.705</v>
+        <v>7.69</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>7.741</v>
+        <v>7.714</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>7.796</v>
+        <v>7.77</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>7.769</v>
+        <v>7.767</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>8.121</v>
+        <v>8.106999999999999</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>8.007999999999999</v>
+        <v>8.009</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>-0.0476</v>
+        <v>-0.1961</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>-0.1752</v>
+        <v>-0.3836</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>-0.1859</v>
+        <v>-0.1429</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>-0.2024</v>
+        <v>-0.2587</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>0.1278</v>
+        <v>0.1137</v>
       </c>
     </row>
     <row r="10">
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.342</v>
+        <v>3.325</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>100.6</v>
@@ -1636,27 +1636,27 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>10.96</v>
+        <v>10.35</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>12.78</v>
+        <v>12.03</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>4.02</v>
+        <v>2.6</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>2.03</v>
+        <v>0.78</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>83.2</v>
+        <v>81.2</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
@@ -1665,40 +1665,40 @@
         </is>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>3.363</v>
+        <v>3.351</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.365</v>
+        <v>3.358</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>3.408</v>
+        <v>3.4</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>3.404</v>
+        <v>3.405</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>3.35</v>
+        <v>3.352</v>
       </c>
       <c r="AL10" s="2" t="n">
         <v>3.257</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>3.214</v>
+        <v>3.215</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>-0.6296</v>
+        <v>-0.7433</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>-0.2962</v>
+        <v>-0.3793</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>0.3574</v>
+        <v>0.2831</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>0.0301</v>
+        <v>0.0307</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>0.1096</v>
+        <v>0.1035</v>
       </c>
     </row>
     <row r="11">
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.49</v>
+        <v>0.491</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>4.78</v>
@@ -1741,25 +1741,27 @@
         <v>-1</v>
       </c>
       <c r="S11" s="2" t="inlineStr"/>
-      <c r="T11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-14.2</v>
+        <v>-14.79</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-3.32</v>
+        <v>-3.15</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>1.07</v>
+        <v>0.91</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.34</v>
+        <v>0.73</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>29.5</v>
+        <v>24.7</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1771,40 +1773,40 @@
         </is>
       </c>
       <c r="AG11" s="2" t="n">
-        <v>0.504</v>
+        <v>0.501</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>0.503</v>
+        <v>0.502</v>
       </c>
       <c r="AI11" s="2" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="AJ11" s="2" t="n">
         <v>0.513</v>
       </c>
-      <c r="AJ11" s="2" t="n">
-        <v>0.514</v>
-      </c>
       <c r="AK11" s="2" t="n">
-        <v>0.519</v>
+        <v>0.518</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>0.518</v>
+        <v>0.517</v>
       </c>
       <c r="AM11" s="2" t="n">
         <v>0.533</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>-0.6731</v>
+        <v>-0.6646</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>-0.3875</v>
+        <v>-0.5737</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>-0.2531</v>
+        <v>-0.3071</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>-0.06419999999999999</v>
+        <v>-0.0883</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>-0.142</v>
+        <v>-0.1479</v>
       </c>
     </row>
     <row r="12">
@@ -1819,7 +1821,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.376</v>
+        <v>0.377</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>9.880000000000001</v>
@@ -1848,22 +1850,22 @@
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-3.87</v>
+        <v>-3.92</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>6.14</v>
+        <v>6.37</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>5.05</v>
+        <v>2.48</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>5.74</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>64.5</v>
+        <v>64</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1875,16 +1877,16 @@
         </is>
       </c>
       <c r="AG12" s="2" t="n">
-        <v>0.381</v>
+        <v>0.379</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>0.376</v>
+        <v>0.377</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>0.376</v>
       </c>
       <c r="AJ12" s="2" t="n">
-        <v>0.381</v>
+        <v>0.38</v>
       </c>
       <c r="AK12" s="2" t="n">
         <v>0.381</v>
@@ -1896,19 +1898,19 @@
         <v>0.371</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.5179</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>-0.0496</v>
+        <v>-0.1114</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>0.1562</v>
+        <v>0.0881</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>0.0759</v>
+        <v>0.0718</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>-0.0387</v>
+        <v>-0.0392</v>
       </c>
     </row>
     <row r="13">
@@ -1923,7 +1925,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.757</v>
+        <v>0.758</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>2.2</v>
@@ -1954,22 +1956,22 @@
       </c>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-12.4</v>
+        <v>-12.91</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-2.89</v>
+        <v>-2.81</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>0.89</v>
+        <v>0.73</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>0.96</v>
+        <v>1.4</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>48.6</v>
+        <v>42.3</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1981,40 +1983,40 @@
         </is>
       </c>
       <c r="AG13" s="2" t="n">
-        <v>0.779</v>
+        <v>0.773</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>0.779</v>
+        <v>0.776</v>
       </c>
       <c r="AI13" s="2" t="n">
-        <v>0.793</v>
+        <v>0.791</v>
       </c>
       <c r="AJ13" s="2" t="n">
-        <v>0.792</v>
+        <v>0.791</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>0.797</v>
+        <v>0.796</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>0.789</v>
+        <v>0.788</v>
       </c>
       <c r="AM13" s="2" t="n">
         <v>0.828</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>-0.7272</v>
+        <v>-0.7823</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>-0.351</v>
+        <v>-0.5034</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>-0.0882</v>
+        <v>-0.1663</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>-0.1031</v>
+        <v>-0.1321</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>-0.124</v>
+        <v>-0.1291</v>
       </c>
     </row>
     <row r="14">
@@ -2029,7 +2031,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.968</v>
+        <v>2.98</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>43.79</v>
@@ -2042,7 +2044,9 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
       </c>
@@ -2055,25 +2059,27 @@
       <c r="S14" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>7.19</v>
+        <v>5.8</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>1.03</v>
+        <v>1.27</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-1.67</v>
+        <v>-1.28</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>0.58</v>
+        <v>0.48</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>37.6</v>
+        <v>36.1</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
@@ -2085,40 +2091,40 @@
         </is>
       </c>
       <c r="AG14" s="2" t="n">
-        <v>3.097</v>
+        <v>3.065</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>3.082</v>
+        <v>3.078</v>
       </c>
       <c r="AI14" s="2" t="n">
+        <v>3.077</v>
+      </c>
+      <c r="AJ14" s="2" t="n">
         <v>3.084</v>
       </c>
-      <c r="AJ14" s="2" t="n">
-        <v>3.091</v>
-      </c>
       <c r="AK14" s="2" t="n">
-        <v>3.042</v>
+        <v>3.047</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>3.231</v>
+        <v>3.227</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>3.215</v>
+        <v>3.217</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>0.1544</v>
+        <v>-0.0227</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>0.0634</v>
+        <v>-0.1696</v>
       </c>
       <c r="AP14" s="2" t="n">
-        <v>-0.0147</v>
+        <v>0.044</v>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>-0.2309</v>
+        <v>-0.2916</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>0.07190000000000001</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="15">
@@ -2133,7 +2139,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.34</v>
+        <v>0.339</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>40.85</v>
@@ -2160,26 +2166,24 @@
       </c>
       <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
-      <c r="U15" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-0.27</v>
+        <v>-0.45</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>6.58</v>
+        <v>6.12</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>4.24</v>
+        <v>2.15</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>7.03</v>
+        <v>7.75</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>74.09999999999999</v>
+        <v>73.5</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
@@ -2191,16 +2195,16 @@
         </is>
       </c>
       <c r="AG15" s="2" t="n">
-        <v>0.345</v>
+        <v>0.344</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>0.34</v>
+        <v>0.341</v>
       </c>
       <c r="AI15" s="2" t="n">
         <v>0.339</v>
       </c>
       <c r="AJ15" s="2" t="n">
-        <v>0.342</v>
+        <v>0.341</v>
       </c>
       <c r="AK15" s="2" t="n">
         <v>0.339</v>
@@ -2212,19 +2216,19 @@
         <v>0.336</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>0.7904</v>
+        <v>0.6937</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>0.0567</v>
+        <v>-0.0123</v>
       </c>
       <c r="AP15" s="2" t="n">
-        <v>0.3489</v>
+        <v>0.2739</v>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>0.0626</v>
+        <v>0.0533</v>
       </c>
       <c r="AR15" s="2" t="n">
-        <v>-0.0027</v>
+        <v>-0.0045</v>
       </c>
     </row>
     <row r="16">
@@ -2239,7 +2243,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.098</v>
+        <v>1.102</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>81.33</v>
@@ -2254,14 +2258,12 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R16" s="2" t="inlineStr"/>
       <c r="S16" s="2" t="n">
         <v>-1</v>
       </c>
@@ -2270,22 +2272,22 @@
       </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-2.67</v>
+        <v>-4.33</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-7.69</v>
+        <v>-7.43</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-1.54</v>
+        <v>-1.91</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>4.12</v>
+        <v>3.13</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>41.9</v>
+        <v>40.1</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
@@ -2297,40 +2299,40 @@
         </is>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>1.144</v>
+        <v>1.129</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>1.146</v>
+        <v>1.141</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>1.151</v>
+        <v>1.149</v>
       </c>
       <c r="AJ16" s="2" t="n">
-        <v>1.14</v>
+        <v>1.138</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>1.129</v>
+        <v>1.13</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>1.209</v>
+        <v>1.205</v>
       </c>
       <c r="AM16" s="2" t="n">
         <v>1.303</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>-0.5344</v>
+        <v>-0.8558</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>0.4352</v>
+        <v>0.1475</v>
       </c>
       <c r="AP16" s="2" t="n">
-        <v>0.0424</v>
+        <v>0.1005</v>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>-0.554</v>
+        <v>-0.6303</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>-0.0267</v>
+        <v>-0.0433</v>
       </c>
     </row>
     <row r="17">
@@ -2345,7 +2347,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.406</v>
+        <v>0.405</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>-1.36</v>
@@ -2369,25 +2371,27 @@
         <v>-1</v>
       </c>
       <c r="S17" s="2" t="inlineStr"/>
-      <c r="T17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-46.07</v>
+        <v>-46.09</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-12.51</v>
+        <v>-12.7</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>2.96</v>
+        <v>2.23</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>4.56</v>
+        <v>5.32</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>51.1</v>
+        <v>49.3</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
@@ -2399,40 +2403,40 @@
         </is>
       </c>
       <c r="AG17" s="2" t="n">
-        <v>0.412</v>
+        <v>0.41</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>0.411</v>
+        <v>0.41</v>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>0.418</v>
+        <v>0.417</v>
       </c>
       <c r="AJ17" s="2" t="n">
-        <v>0.42</v>
+        <v>0.419</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>0.427</v>
+        <v>0.426</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>0.426</v>
+        <v>0.425</v>
       </c>
       <c r="AM17" s="2" t="n">
         <v>0.474</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>-0.7622</v>
+        <v>-0.6385999999999999</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>-0.3085</v>
+        <v>-0.3621</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>0.0549</v>
+        <v>-0.0667</v>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>-0.4214</v>
+        <v>-0.4279</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>-0.4607</v>
+        <v>-0.4609</v>
       </c>
     </row>
     <row r="18">
@@ -2447,7 +2451,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.086</v>
+        <v>1.091</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>5.68</v>
@@ -2475,29 +2479,31 @@
       <c r="S18" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-7.08</v>
+        <v>-7.62</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-5.6</v>
+        <v>-5.27</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-0.34</v>
+        <v>-0.04</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-2.63</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="AA18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
@@ -2507,40 +2513,40 @@
         </is>
       </c>
       <c r="AG18" s="2" t="n">
-        <v>1.129</v>
+        <v>1.119</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>1.122</v>
+        <v>1.121</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>1.141</v>
+        <v>1.136</v>
       </c>
       <c r="AJ18" s="2" t="n">
-        <v>1.151</v>
+        <v>1.147</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>1.171</v>
+        <v>1.17</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>1.211</v>
+        <v>1.209</v>
       </c>
       <c r="AM18" s="2" t="n">
         <v>1.233</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-0.1721</v>
+        <v>-0.1598</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>-0.2658</v>
+        <v>-0.5416</v>
       </c>
       <c r="AP18" s="2" t="n">
-        <v>-0.3384</v>
+        <v>-0.3133</v>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>-0.3953</v>
+        <v>-0.4623</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>-0.0708</v>
+        <v>-0.0762</v>
       </c>
     </row>
     <row r="19">
@@ -2555,7 +2561,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.035</v>
+        <v>1.042</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>-3.59</v>
@@ -2570,7 +2576,7 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
@@ -2578,34 +2584,30 @@
       <c r="R19" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S19" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>40.97</v>
+        <v>39.13</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>14.18</v>
+        <v>14.67</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-3.61</v>
+        <v>-2.3</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-3.51</v>
+        <v>-4.33</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>-2.5</v>
+        <v>-2.9</v>
       </c>
       <c r="AA19" s="2" t="n">
         <v>30</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
@@ -2615,58 +2617,58 @@
         </is>
       </c>
       <c r="AG19" s="2" t="n">
-        <v>1.088</v>
+        <v>1.076</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>1.07</v>
+        <v>1.074</v>
       </c>
       <c r="AI19" s="2" t="n">
-        <v>1.065</v>
+        <v>1.061</v>
       </c>
       <c r="AJ19" s="2" t="n">
-        <v>1.082</v>
+        <v>1.076</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>1.105</v>
+        <v>1.103</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>1.181</v>
+        <v>1.182</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>1.022</v>
+        <v>1.024</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>1.138</v>
+        <v>1.1195</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>0.007</v>
+        <v>-0.2683</v>
       </c>
       <c r="AP19" s="2" t="n">
-        <v>-0.9752</v>
+        <v>-0.8028</v>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>0.2121</v>
+        <v>0.1479</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>0.4097</v>
+        <v>0.3913</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.018</v>
+        <v>0.841</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-3.21</v>
+        <v>99.92</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -2675,45 +2677,43 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-53.3</v>
+        <v>-0.26</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-16.71</v>
+        <v>12.49</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>4.09</v>
+        <v>5.03</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>2.67</v>
+        <v>8.48</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>34.1</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
@@ -2721,58 +2721,58 @@
         </is>
       </c>
       <c r="AG20" s="2" t="n">
-        <v>1.031</v>
+        <v>0.837</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>1.022</v>
+        <v>0.838</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>1.032</v>
+        <v>0.842</v>
       </c>
       <c r="AJ20" s="2" t="n">
-        <v>1.054</v>
+        <v>0.834</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>1.086</v>
+        <v>0.824</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>1.092</v>
+        <v>0.799</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>1.23</v>
+        <v>0.798</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>0.0407</v>
+        <v>-0.3086</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>-0.5878</v>
+        <v>0.2235</v>
       </c>
       <c r="AP20" s="2" t="n">
-        <v>-0.3605</v>
+        <v>0.3012</v>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>-0.3969</v>
+        <v>0.1534</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>-0.533</v>
+        <v>-0.0026</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.749</v>
+        <v>1.007</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>4.5</v>
+        <v>-3.21</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2781,12 +2781,14 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M21" s="2" t="n">
         <v>13</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -2794,28 +2796,30 @@
       <c r="R21" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S21" s="2" t="inlineStr"/>
-      <c r="T21" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-17.01</v>
+        <v>-53.46</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-3.79</v>
+        <v>-17.54</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>1.4</v>
+        <v>2.44</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-0.39</v>
+        <v>2.21</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>44.4</v>
+        <v>32.5</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2827,109 +2831,101 @@
         </is>
       </c>
       <c r="AG21" s="2" t="n">
-        <v>1.793</v>
+        <v>1.026</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>1.793</v>
+        <v>1.022</v>
       </c>
       <c r="AI21" s="2" t="n">
-        <v>1.83</v>
+        <v>1.029</v>
       </c>
       <c r="AJ21" s="2" t="n">
-        <v>1.835</v>
+        <v>1.051</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>1.838</v>
+        <v>1.083</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>1.82</v>
+        <v>1.09</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>1.889</v>
+        <v>1.227</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>-0.7657</v>
+        <v>0.1122</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>-0.5553</v>
+        <v>-0.6637999999999999</v>
       </c>
       <c r="AP21" s="2" t="n">
-        <v>-0.0735</v>
+        <v>-0.4323</v>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>-0.09329999999999999</v>
+        <v>-0.4349</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>-0.1701</v>
+        <v>-0.5346</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2.304</v>
+        <v>1.754</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>101.52</v>
+        <v>4.5</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N22" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R22" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>24.22</v>
+        <v>-17.27</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>24.45</v>
+        <v>-3.51</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>5.67</v>
+        <v>1.74</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>8.359999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>58.3</v>
+        <v>38.3</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
@@ -2937,189 +2933,189 @@
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG22" s="2" t="n">
-        <v>2.31</v>
+        <v>1.782</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>2.264</v>
+        <v>1.788</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>2.242</v>
+        <v>1.823</v>
       </c>
       <c r="AJ22" s="2" t="n">
-        <v>2.233</v>
+        <v>1.833</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>2.206</v>
+        <v>1.836</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>2.192</v>
+        <v>1.819</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>2.025</v>
+        <v>1.887</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>0.9967</v>
+        <v>-0.7199</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>0.6111</v>
+        <v>-0.7258</v>
       </c>
       <c r="AP22" s="2" t="n">
-        <v>0.3555</v>
+        <v>-0.1266</v>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>0.3825</v>
+        <v>-0.117</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>0.2422</v>
+        <v>-0.1727</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.433</v>
+        <v>2.324</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>7.28</v>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
+        <v>101.52</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S23" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T23" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>-21.59</v>
+        <v>24.24</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>-14.9</v>
+        <v>25.22</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-0.7</v>
+        <v>6.69</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-6.2</v>
+        <v>10.22</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>3</v>
+        <v>62.5</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>1.485</v>
+        <v>2.318</v>
       </c>
       <c r="AH23" s="2" t="n">
-        <v>1.489</v>
+        <v>2.278</v>
       </c>
       <c r="AI23" s="2" t="n">
-        <v>1.522</v>
+        <v>2.247</v>
       </c>
       <c r="AJ23" s="2" t="n">
-        <v>1.562</v>
+        <v>2.234</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>1.585</v>
+        <v>2.21</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>1.739</v>
+        <v>2.194</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>1.814</v>
+        <v>2.027</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>-0.7641</v>
+        <v>1.1954</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>-1.1921</v>
+        <v>0.5908</v>
       </c>
       <c r="AP23" s="2" t="n">
-        <v>-0.3766</v>
+        <v>0.4087</v>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>-0.9557</v>
+        <v>0.3674</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>-0.2159</v>
+        <v>0.2424</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.967</v>
+        <v>1.445</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>25.84</v>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+        <v>7.28</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="n">
-        <v>-13</v>
+        <v>13</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -3133,90 +3129,92 @@
       <c r="S24" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>49.3</v>
+        <v>-22.18</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>14.79</v>
+        <v>-14.25</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-8.710000000000001</v>
+        <v>0.48</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-5.66</v>
+        <v>-4.21</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>22.5</v>
+        <v>2.4</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>1.047</v>
+        <v>1.474</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>1.043</v>
+        <v>1.482</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>1.037</v>
+        <v>1.513</v>
       </c>
       <c r="AJ24" s="2" t="n">
-        <v>1.038</v>
+        <v>1.553</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>1.027</v>
+        <v>1.583</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>1.125</v>
+        <v>1.732</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>0.968</v>
+        <v>1.813</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>0.005</v>
+        <v>-0.791</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>0.328</v>
+        <v>-1.2658</v>
       </c>
       <c r="AP24" s="2" t="n">
-        <v>-0.5839</v>
+        <v>-0.3614</v>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>0.0934</v>
+        <v>-1.0053</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>0.493</v>
+        <v>-0.2218</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.264</v>
+        <v>0.976</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>96.61</v>
+        <v>25.84</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -3230,101 +3228,103 @@
         <v>-13</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U25" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>20</v>
+        <v>45.98</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>15.08</v>
+        <v>15.56</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>5.08</v>
+        <v>-8.08</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-2.56</v>
+        <v>-5.82</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>65.90000000000001</v>
+        <v>21.3</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG25" s="2" t="n">
-        <v>1.273</v>
+        <v>1.026</v>
       </c>
       <c r="AH25" s="2" t="n">
-        <v>1.269</v>
+        <v>1.039</v>
       </c>
       <c r="AI25" s="2" t="n">
-        <v>1.292</v>
+        <v>1.033</v>
       </c>
       <c r="AJ25" s="2" t="n">
-        <v>1.293</v>
+        <v>1.033</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>1.261</v>
+        <v>1.026</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>1.238</v>
+        <v>1.124</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>1.199</v>
+        <v>0.969</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>-0.6389</v>
+        <v>-0.3531</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>-0.4853</v>
+        <v>-0.0553</v>
       </c>
       <c r="AP25" s="2" t="n">
-        <v>0.4967</v>
+        <v>-0.5486</v>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>-0.0614</v>
+        <v>0.0119</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>0.2</v>
+        <v>0.4598</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.771</v>
+        <v>1.245</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>31.83</v>
+        <v>96.61</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -3334,103 +3334,105 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S26" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-19.44</v>
+        <v>18.7</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-15.7</v>
+        <v>13.14</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-1.34</v>
+        <v>1.14</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-2.46</v>
+        <v>-6.45</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>8</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>0.803</v>
+        <v>1.266</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>0.8</v>
+        <v>1.266</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>1.285</v>
       </c>
       <c r="AJ26" s="2" t="n">
-        <v>0.823</v>
+        <v>1.292</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>0.828</v>
+        <v>1.262</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>0.924</v>
+        <v>1.238</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>0.991</v>
+        <v>1.2</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>-0.2651</v>
+        <v>-0.7992</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>-0.6647</v>
+        <v>-0.6993</v>
       </c>
       <c r="AP26" s="2" t="n">
-        <v>-0.2026</v>
+        <v>0.3878</v>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>-0.7403</v>
+        <v>-0.0549</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>-0.1944</v>
+        <v>0.187</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.627</v>
+        <v>0.772</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>32.9</v>
+        <v>31.83</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -3440,9 +3442,7 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
         <v>1</v>
       </c>
@@ -3455,29 +3455,31 @@
       <c r="S27" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>48.11</v>
+        <v>-20.37</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>12.93</v>
+        <v>-15.65</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-10.34</v>
+        <v>-1.24</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-4.73</v>
+        <v>-0.89</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>26.9</v>
+        <v>6.7</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
@@ -3487,90 +3489,72 @@
         </is>
       </c>
       <c r="AG27" s="2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.793</v>
       </c>
       <c r="AH27" s="2" t="n">
-        <v>0.681</v>
+        <v>0.798</v>
       </c>
       <c r="AI27" s="2" t="n">
-        <v>0.672</v>
+        <v>0.804</v>
       </c>
       <c r="AJ27" s="2" t="n">
-        <v>0.672</v>
+        <v>0.819</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>0.66</v>
+        <v>0.828</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>0.731</v>
+        <v>0.921</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>0.64</v>
+        <v>0.99</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>0.4234</v>
+        <v>-0.4138</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>0.5313</v>
+        <v>-0.793</v>
       </c>
       <c r="AP27" s="2" t="n">
-        <v>-0.3788</v>
+        <v>-0.1827</v>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>0.038</v>
+        <v>-0.7998</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>0.4811</v>
+        <v>-0.2037</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2.202</v>
+        <v>0.629</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>32.9</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="n">
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="N28" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
@@ -3586,99 +3570,121 @@
       </c>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-23.34</v>
+        <v>44.06</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-16.79</v>
+        <v>13</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-1.48</v>
+        <v>-10.54</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-4.98</v>
+        <v>-4.7</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>1.1</v>
+        <v>25.5</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG28" s="2" t="n">
-        <v>2.289</v>
+        <v>0.669</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>2.299</v>
+        <v>0.678</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>2.334</v>
+        <v>0.67</v>
       </c>
       <c r="AJ28" s="2" t="n">
-        <v>2.397</v>
+        <v>0.669</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>2.429</v>
+        <v>0.659</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>2.696</v>
+        <v>0.731</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>2.862</v>
+        <v>0.641</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>-0.6499</v>
+        <v>-0.0613</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>-1.0828</v>
+        <v>0.1128</v>
       </c>
       <c r="AP28" s="2" t="n">
-        <v>-0.3287</v>
+        <v>-0.3635</v>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>-0.955</v>
+        <v>-0.0577</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>-0.2334</v>
+        <v>0.4406</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.895</v>
+        <v>2.224</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
+        <v>3.12</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -3686,31 +3692,35 @@
       <c r="R29" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S29" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T29" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-3.28</v>
+        <v>-24.15</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-6.04</v>
+        <v>-16.11</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.35</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>0.4</v>
+        <v>-2.96</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="AA29" s="2" t="inlineStr"/>
+        <v>0.6</v>
+      </c>
+      <c r="AA29" s="2" t="n">
+        <v>17</v>
+      </c>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
@@ -3719,58 +3729,58 @@
         </is>
       </c>
       <c r="AG29" s="2" t="n">
-        <v>0.923</v>
+        <v>2.269</v>
       </c>
       <c r="AH29" s="2" t="n">
-        <v>0.919</v>
+        <v>2.292</v>
       </c>
       <c r="AI29" s="2" t="n">
-        <v>0.9330000000000001</v>
+        <v>2.325</v>
       </c>
       <c r="AJ29" s="2" t="n">
-        <v>0.944</v>
+        <v>2.386</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>0.956</v>
+        <v>2.43</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>1.045</v>
+        <v>2.688</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>1.029</v>
+        <v>2.862</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-0.404</v>
+        <v>-0.7955</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>-0.3708</v>
+        <v>-1.1504</v>
       </c>
       <c r="AP29" s="2" t="n">
-        <v>-0.5609</v>
+        <v>-0.3139</v>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>-0.2994</v>
+        <v>-1.004</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>-0.0328</v>
+        <v>-0.2415</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.643</v>
+        <v>0.9</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-4.94</v>
+        <v>3.17</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -3780,9 +3790,11 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -3790,95 +3802,91 @@
       <c r="R30" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S30" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>26.17</v>
+        <v>-4.09</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>8.779999999999999</v>
+        <v>-5.57</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-2.97</v>
+        <v>0.63</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-2.69</v>
+        <v>-0.7</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-2.4</v>
-      </c>
-      <c r="AA30" s="2" t="n">
-        <v>29</v>
-      </c>
+        <v>-2.3</v>
+      </c>
+      <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG30" s="2" t="n">
-        <v>1.724</v>
+        <v>0.915</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>1.702</v>
+        <v>0.918</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>1.698</v>
+        <v>0.929</v>
       </c>
       <c r="AJ30" s="2" t="n">
-        <v>1.721</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>1.759</v>
+        <v>0.955</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>1.856</v>
+        <v>1.042</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>1.671</v>
+        <v>1.029</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>0.8163</v>
+        <v>-0.3711</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>-0.0474</v>
+        <v>-0.5838</v>
       </c>
       <c r="AP30" s="2" t="n">
-        <v>-0.8075</v>
+        <v>-0.4844</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>0.0864</v>
+        <v>-0.372</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>0.2617</v>
+        <v>-0.0409</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.835</v>
+        <v>1.657</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>99.92</v>
+        <v>-4.94</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -3890,79 +3898,83 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S31" s="2" t="inlineStr"/>
-      <c r="T31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-0.49</v>
+        <v>24.81</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>11.83</v>
+        <v>9.5</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>4.12</v>
+        <v>-1.66</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>9.02</v>
+        <v>-2.76</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>94.09999999999999</v>
+        <v>-2.8</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="inlineStr"/>
-      <c r="AD31" s="2" t="n">
-        <v>8</v>
-      </c>
+      <c r="AC31" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG31" s="2" t="n">
-        <v>0.837</v>
+        <v>1.705</v>
       </c>
       <c r="AH31" s="2" t="n">
-        <v>0.84</v>
+        <v>1.706</v>
       </c>
       <c r="AI31" s="2" t="n">
-        <v>0.841</v>
+        <v>1.692</v>
       </c>
       <c r="AJ31" s="2" t="n">
-        <v>0.833</v>
+        <v>1.714</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>0.823</v>
+        <v>1.756</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>0.799</v>
+        <v>1.855</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>0.798</v>
+        <v>1.672</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>-0.1914</v>
+        <v>0.8141</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>0.2237</v>
+        <v>-0.3191</v>
       </c>
       <c r="AP31" s="2" t="n">
-        <v>0.336</v>
+        <v>-0.6979</v>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>0.1405</v>
+        <v>0.016</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>-0.0049</v>
+        <v>0.2481</v>
       </c>
     </row>
   </sheetData>
@@ -3993,7 +4005,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-28 | 30 只</t>
+          <t>截至: 2026-09-29 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-30
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.162</v>
+        <v>3.154</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -771,9 +771,7 @@
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R2" s="2" t="inlineStr"/>
       <c r="S2" s="2" t="n">
         <v>-1</v>
       </c>
@@ -782,26 +780,26 @@
       </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>9.31</v>
+        <v>7.06</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-0.92</v>
+        <v>-1.48</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-3.68</v>
+        <v>-4.13</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-3.88</v>
+        <v>-3.35</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>-0.5</v>
+        <v>-1.9</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -811,40 +809,40 @@
         </is>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>3.29</v>
+        <v>3.237</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>3.318</v>
+        <v>3.306</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>3.336</v>
+        <v>3.323</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>3.391</v>
+        <v>3.372</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>3.448</v>
+        <v>3.437</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>3.726</v>
+        <v>3.718</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>3.526</v>
+        <v>3.527</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-0.466</v>
+        <v>-0.7105</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>-0.61</v>
+        <v>-0.8094</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>-0.5686</v>
+        <v>-0.6024</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>-0.3284</v>
+        <v>-0.4007</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.0931</v>
+        <v>0.0706</v>
       </c>
     </row>
     <row r="3">
@@ -859,7 +857,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.444</v>
+        <v>1.445</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>7.34</v>
@@ -876,7 +874,7 @@
         <v>13</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -885,25 +883,27 @@
         <v>-1</v>
       </c>
       <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-11.45</v>
+        <v>-11.91</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>0.89</v>
+        <v>0.77</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>3.28</v>
+        <v>2.48</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>3.38</v>
+        <v>3.35</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>64.09999999999999</v>
+        <v>62.6</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -915,40 +915,40 @@
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>1.457</v>
+        <v>1.45</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>1.454</v>
+        <v>1.453</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>1.468</v>
+        <v>1.465</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>1.48</v>
+        <v>1.477</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>1.49</v>
+        <v>1.488</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>1.472</v>
+        <v>1.47</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>1.517</v>
+        <v>1.515</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>-0.2505</v>
+        <v>-0.227</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>-0.3996</v>
+        <v>-0.4334</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>-0.0451</v>
+        <v>-0.09279999999999999</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>-0.1568</v>
+        <v>-0.1726</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>-0.1145</v>
+        <v>-0.1191</v>
       </c>
     </row>
     <row r="4">
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.647</v>
+        <v>0.658</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>-2.04</v>
@@ -980,36 +980,40 @@
         <v>-13</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S4" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T4" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-31.08</v>
+        <v>-30.46</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-6.58</v>
+        <v>-5.16</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>3.04</v>
+        <v>4.45</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>5.22</v>
+        <v>5.21</v>
       </c>
       <c r="Z4" s="2" t="n">
         <v>65.7</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
@@ -1024,37 +1028,37 @@
         <v>0.65</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.651</v>
+        <v>0.652</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>0.662</v>
+        <v>0.661</v>
       </c>
       <c r="AJ4" s="2" t="n">
         <v>0.663</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>0.669</v>
+        <v>0.668</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>0.663</v>
+        <v>0.662</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>0.719</v>
+        <v>0.718</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>-0.7243000000000001</v>
+        <v>-0.4979</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>-0.3086</v>
+        <v>-0.3478</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>-0.0466</v>
+        <v>-0.104</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>-0.3544</v>
+        <v>-0.3478</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>-0.3108</v>
+        <v>-0.3046</v>
       </c>
     </row>
     <row r="5">
@@ -1069,7 +1073,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.778</v>
+        <v>1.772</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>101.26</v>
@@ -1104,27 +1108,27 @@
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>44.15</v>
+        <v>44.4</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>31.51</v>
+        <v>30.49</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>6.95</v>
+        <v>6.57</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>15.63</v>
+        <v>12.78</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>97.7</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
@@ -1133,40 +1137,40 @@
         </is>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>1.74</v>
+        <v>1.746</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>1.757</v>
+        <v>1.755</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>1.737</v>
+        <v>1.743</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>1.679</v>
+        <v>1.686</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>1.606</v>
+        <v>1.611</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>1.575</v>
+        <v>1.576</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>1.506</v>
+        <v>1.509</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>-0.3265</v>
+        <v>-0.356</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>1.3896</v>
+        <v>1.3265</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>0.7763</v>
+        <v>0.7924</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.0701</v>
+        <v>0.0992</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.4415</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="6">
@@ -1181,7 +1185,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.844</v>
+        <v>0.872</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>4.26</v>
@@ -1202,28 +1206,28 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-2.9</v>
+        <v>-2.47</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>6.64</v>
+        <v>9.91</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>1.86</v>
+        <v>5.4</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>7.35</v>
+        <v>10.13</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>57</v>
+        <v>58.1</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
@@ -1235,40 +1239,40 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="AH6" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AI6" s="2" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="AJ6" s="2" t="n">
         <v>0.853</v>
       </c>
-      <c r="AH6" s="2" t="n">
-        <v>0.845</v>
-      </c>
-      <c r="AI6" s="2" t="n">
-        <v>0.841</v>
-      </c>
-      <c r="AJ6" s="2" t="n">
-        <v>0.854</v>
-      </c>
       <c r="AK6" s="2" t="n">
-        <v>0.864</v>
+        <v>0.863</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>0.826</v>
+        <v>0.827</v>
       </c>
       <c r="AM6" s="2" t="n">
         <v>0.833</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.7936</v>
+        <v>0.9913999999999999</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>-0.1664</v>
+        <v>-0.0925</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>-0.174</v>
+        <v>-0.1693</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.0567</v>
+        <v>0.0542</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>-0.029</v>
+        <v>-0.0247</v>
       </c>
     </row>
     <row r="7">
@@ -1283,7 +1287,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.922</v>
+        <v>2.938</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>2.95</v>
@@ -1306,30 +1310,28 @@
       <c r="R7" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S7" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S7" s="2" t="inlineStr"/>
       <c r="T7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-3.19</v>
+        <v>-3.88</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>3.1</v>
+        <v>3.39</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>1.72</v>
+        <v>1.67</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>2.41</v>
+        <v>1.93</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>30</v>
+        <v>26.6</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
@@ -1341,40 +1343,40 @@
         </is>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>2.964</v>
+        <v>2.948</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>2.969</v>
+        <v>2.967</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>2.994</v>
+        <v>2.987</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>3</v>
+        <v>2.996</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>3.016</v>
+        <v>3.013</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>3.017</v>
+        <v>3.015</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>3.043</v>
+        <v>3.042</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>-0.3377</v>
+        <v>-0.3678</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>-0.2555</v>
+        <v>-0.3849</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>-0.08459999999999999</v>
+        <v>-0.1184</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>-0.097</v>
+        <v>-0.123</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>-0.0319</v>
+        <v>-0.0388</v>
       </c>
     </row>
     <row r="8">
@@ -1389,7 +1391,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.416</v>
+        <v>4.432</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>9.76</v>
@@ -1409,9 +1411,7 @@
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
       <c r="S8" s="2" t="n">
         <v>-1</v>
       </c>
@@ -1420,26 +1420,26 @@
       </c>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>-0.63</v>
+        <v>-1.82</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.24</v>
+        <v>1.3</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.08</v>
+        <v>0.17</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>0.19</v>
+        <v>-0.02</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>-1.3</v>
+        <v>-2.1</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
@@ -1449,40 +1449,40 @@
         </is>
       </c>
       <c r="AG8" s="2" t="n">
-        <v>4.51</v>
+        <v>4.474</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>4.534</v>
+        <v>4.525</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>4.576</v>
+        <v>4.564</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>4.608</v>
+        <v>4.597</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>4.65</v>
+        <v>4.643</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>4.767</v>
+        <v>4.762</v>
       </c>
       <c r="AM8" s="2" t="n">
         <v>4.718</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-0.5197000000000001</v>
+        <v>-0.6103</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>-0.4348</v>
+        <v>-0.5749</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>-0.2484</v>
+        <v>-0.2778</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>-0.1935</v>
+        <v>-0.2289</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>-0.0063</v>
+        <v>-0.0182</v>
       </c>
     </row>
     <row r="9">
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.476</v>
+        <v>7.472</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>52.12</v>
@@ -1517,9 +1517,7 @@
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R9" s="2" t="inlineStr"/>
       <c r="S9" s="2" t="n">
         <v>-1</v>
       </c>
@@ -1528,26 +1526,26 @@
       </c>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>11.37</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>2.77</v>
+        <v>2.35</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-1</v>
+        <v>-0.98</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-0.96</v>
+        <v>-0.48</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>16.9</v>
+        <v>15.4</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
@@ -1557,40 +1555,40 @@
         </is>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>7.646</v>
+        <v>7.572</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>7.69</v>
+        <v>7.68</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>7.714</v>
+        <v>7.695</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>7.77</v>
+        <v>7.748</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>7.767</v>
+        <v>7.763</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>8.106999999999999</v>
+        <v>8.096</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>8.009</v>
+        <v>8.013</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>-0.1961</v>
+        <v>-0.3166</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>-0.3836</v>
+        <v>-0.5612</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>-0.1429</v>
+        <v>-0.1305</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>-0.2587</v>
+        <v>-0.3137</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>0.1137</v>
+        <v>0.0989</v>
       </c>
     </row>
     <row r="10">
@@ -1605,7 +1603,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.325</v>
+        <v>3.368</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>100.6</v>
@@ -1622,41 +1620,41 @@
       </c>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="V10" s="2" t="n">
-        <v>10.35</v>
+        <v>10.27</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>12.03</v>
+        <v>13.08</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>2.6</v>
+        <v>3.98</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>0.78</v>
+        <v>1.75</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>81.2</v>
+        <v>80.5</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
@@ -1665,40 +1663,40 @@
         </is>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>3.351</v>
+        <v>3.348</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.358</v>
+        <v>3.356</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>3.4</v>
+        <v>3.394</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>3.405</v>
+        <v>3.406</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>3.352</v>
+        <v>3.355</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>3.257</v>
+        <v>3.258</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>3.215</v>
+        <v>3.216</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>-0.7433</v>
+        <v>-0.6655</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>-0.3793</v>
+        <v>-0.444</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>0.2831</v>
+        <v>0.258</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>0.0307</v>
+        <v>0.0422</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>0.1035</v>
+        <v>0.1027</v>
       </c>
     </row>
     <row r="11">
@@ -1713,7 +1711,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.491</v>
+        <v>0.492</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>4.78</v>
@@ -1746,22 +1744,22 @@
       </c>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-14.79</v>
+        <v>-15.48</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-3.15</v>
+        <v>-3.16</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.91</v>
+        <v>0.74</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.73</v>
+        <v>-0.4</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>24.7</v>
+        <v>20.5</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1773,16 +1771,16 @@
         </is>
       </c>
       <c r="AG11" s="2" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="AH11" s="2" t="n">
         <v>0.501</v>
       </c>
-      <c r="AH11" s="2" t="n">
-        <v>0.502</v>
-      </c>
       <c r="AI11" s="2" t="n">
-        <v>0.511</v>
+        <v>0.509</v>
       </c>
       <c r="AJ11" s="2" t="n">
-        <v>0.513</v>
+        <v>0.512</v>
       </c>
       <c r="AK11" s="2" t="n">
         <v>0.518</v>
@@ -1791,22 +1789,22 @@
         <v>0.517</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>0.533</v>
+        <v>0.532</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>-0.6646</v>
+        <v>-0.6657</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>-0.5737</v>
+        <v>-0.7849</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>-0.3071</v>
+        <v>-0.3612</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>-0.0883</v>
+        <v>-0.1184</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>-0.1479</v>
+        <v>-0.1548</v>
       </c>
     </row>
     <row r="12">
@@ -1821,7 +1819,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.377</v>
+        <v>0.388</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>9.880000000000001</v>
@@ -1838,34 +1836,38 @@
       </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
-      <c r="U12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="V12" s="2" t="n">
-        <v>-3.92</v>
+        <v>-3.3</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>6.37</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>2.48</v>
+        <v>5.83</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>8.109999999999999</v>
+        <v>10.04</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>64</v>
+        <v>65.2</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1877,19 +1879,19 @@
         </is>
       </c>
       <c r="AG12" s="2" t="n">
-        <v>0.379</v>
+        <v>0.38</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>0.377</v>
+        <v>0.378</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>0.376</v>
       </c>
       <c r="AJ12" s="2" t="n">
-        <v>0.38</v>
+        <v>0.379</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>0.381</v>
+        <v>0.382</v>
       </c>
       <c r="AL12" s="2" t="n">
         <v>0.364</v>
@@ -1898,19 +1900,19 @@
         <v>0.371</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>0.5179</v>
+        <v>0.7098</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>-0.1114</v>
+        <v>-0.0495</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>0.0881</v>
+        <v>0.0741</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>0.0718</v>
+        <v>0.0828</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>-0.0392</v>
+        <v>-0.033</v>
       </c>
     </row>
     <row r="13">
@@ -1925,7 +1927,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.758</v>
+        <v>0.764</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>2.2</v>
@@ -1942,36 +1944,36 @@
         <v>9</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="n">
-        <v>-1</v>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S13" s="2" t="inlineStr"/>
-      <c r="T13" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-12.91</v>
+        <v>-13.54</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-2.81</v>
+        <v>-2.28</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>0.73</v>
+        <v>0.95</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>1.4</v>
+        <v>0.12</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>42.3</v>
+        <v>37.7</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1983,40 +1985,40 @@
         </is>
       </c>
       <c r="AG13" s="2" t="n">
-        <v>0.773</v>
+        <v>0.767</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>0.776</v>
+        <v>0.775</v>
       </c>
       <c r="AI13" s="2" t="n">
-        <v>0.791</v>
+        <v>0.788</v>
       </c>
       <c r="AJ13" s="2" t="n">
-        <v>0.791</v>
+        <v>0.79</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>0.796</v>
+        <v>0.795</v>
       </c>
       <c r="AL13" s="2" t="n">
         <v>0.788</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>0.828</v>
+        <v>0.827</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>-0.7823</v>
+        <v>-0.8166</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>-0.5034</v>
+        <v>-0.6854</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>-0.1663</v>
+        <v>-0.2365</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>-0.1321</v>
+        <v>-0.1572</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>-0.1291</v>
+        <v>-0.1354</v>
       </c>
     </row>
     <row r="14">
@@ -2031,7 +2033,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.98</v>
+        <v>2.971</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>43.79</v>
@@ -2053,9 +2055,7 @@
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R14" s="2" t="inlineStr"/>
       <c r="S14" s="2" t="n">
         <v>-1</v>
       </c>
@@ -2064,22 +2064,22 @@
       </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>5.8</v>
+        <v>4.34</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>1.27</v>
+        <v>0.7</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-1.28</v>
+        <v>-1.72</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>36.1</v>
+        <v>34.6</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
@@ -2091,40 +2091,40 @@
         </is>
       </c>
       <c r="AG14" s="2" t="n">
-        <v>3.065</v>
+        <v>3.028</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>3.078</v>
+        <v>3.071</v>
       </c>
       <c r="AI14" s="2" t="n">
-        <v>3.077</v>
+        <v>3.069</v>
       </c>
       <c r="AJ14" s="2" t="n">
-        <v>3.084</v>
+        <v>3.075</v>
       </c>
       <c r="AK14" s="2" t="n">
         <v>3.047</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>3.227</v>
+        <v>3.22</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>3.217</v>
+        <v>3.216</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>-0.0227</v>
+        <v>-0.1856</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>-0.1696</v>
+        <v>-0.3792</v>
       </c>
       <c r="AP14" s="2" t="n">
-        <v>0.044</v>
+        <v>0.0762</v>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>-0.2916</v>
+        <v>-0.3534</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>0.058</v>
+        <v>0.0434</v>
       </c>
     </row>
     <row r="15">
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.339</v>
+        <v>0.349</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>40.85</v>
@@ -2156,34 +2156,34 @@
       </c>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-0.45</v>
+        <v>-0.05</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>6.12</v>
+        <v>9.06</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>2.15</v>
+        <v>5.13</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>7.75</v>
+        <v>9.67</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>73.5</v>
+        <v>74.8</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
@@ -2198,7 +2198,7 @@
         <v>0.344</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>0.341</v>
+        <v>0.342</v>
       </c>
       <c r="AI15" s="2" t="n">
         <v>0.339</v>
@@ -2216,37 +2216,37 @@
         <v>0.336</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>0.6937</v>
+        <v>0.8506</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>-0.0123</v>
+        <v>0.0418</v>
       </c>
       <c r="AP15" s="2" t="n">
-        <v>0.2739</v>
+        <v>0.2498</v>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>0.0533</v>
+        <v>0.0518</v>
       </c>
       <c r="AR15" s="2" t="n">
-        <v>-0.0045</v>
+        <v>-0.0005</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.102</v>
+        <v>0.417</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>81.33</v>
+        <v>-1.36</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -2258,36 +2258,36 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr"/>
-      <c r="S16" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-4.33</v>
+        <v>-44.86</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-7.43</v>
+        <v>-10.23</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-1.91</v>
+        <v>4.8</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>3.13</v>
+        <v>5.42</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>40.1</v>
+        <v>49.9</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
@@ -2295,62 +2295,62 @@
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>1.129</v>
+        <v>0.41</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>1.141</v>
+        <v>0.411</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>1.149</v>
+        <v>0.417</v>
       </c>
       <c r="AJ16" s="2" t="n">
-        <v>1.138</v>
+        <v>0.419</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>1.13</v>
+        <v>0.426</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>1.205</v>
+        <v>0.425</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>1.303</v>
+        <v>0.473</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>-0.8558</v>
+        <v>-0.3394</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>0.1475</v>
+        <v>-0.3949</v>
       </c>
       <c r="AP16" s="2" t="n">
-        <v>0.1005</v>
+        <v>-0.1324</v>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>-0.6303</v>
+        <v>-0.4118</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>-0.0433</v>
+        <v>-0.4486</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.405</v>
+        <v>1.082</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-1.36</v>
+        <v>5.68</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -2362,7 +2362,7 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
@@ -2370,91 +2370,95 @@
       <c r="R17" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T17" s="2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-46.09</v>
+        <v>-8.94</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-12.7</v>
+        <v>-6.28</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>2.23</v>
+        <v>-2.11</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>5.32</v>
+        <v>-3.45</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>49.3</v>
+        <v>3.8</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
-      <c r="AC17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="AD17" s="2" t="inlineStr"/>
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG17" s="2" t="n">
-        <v>0.41</v>
+        <v>1.105</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>0.41</v>
+        <v>1.119</v>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>0.417</v>
+        <v>1.13</v>
       </c>
       <c r="AJ17" s="2" t="n">
-        <v>0.419</v>
+        <v>1.142</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>0.426</v>
+        <v>1.167</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>0.425</v>
+        <v>1.206</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>0.474</v>
+        <v>1.232</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>-0.6385999999999999</v>
+        <v>-0.3151</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>-0.3621</v>
+        <v>-0.8376</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>-0.0667</v>
+        <v>-0.3717</v>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>-0.4279</v>
+        <v>-0.54</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>-0.4609</v>
+        <v>-0.08939999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.091</v>
+        <v>1.012</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>5.68</v>
+        <v>-3.59</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -2464,11 +2468,9 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -2476,95 +2478,97 @@
       <c r="R18" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S18" s="2" t="n">
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="n">
         <v>-1</v>
-      </c>
-      <c r="T18" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-7.62</v>
+        <v>35.94</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-5.27</v>
+        <v>10.91</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-0.04</v>
+        <v>-6.8</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-2.63</v>
+        <v>-5.25</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>5.5</v>
+        <v>-3.8</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG18" s="2" t="n">
-        <v>1.119</v>
+        <v>1.056</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>1.121</v>
+        <v>1.072</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>1.136</v>
+        <v>1.057</v>
       </c>
       <c r="AJ18" s="2" t="n">
-        <v>1.147</v>
+        <v>1.07</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>1.17</v>
+        <v>1.098</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>1.209</v>
+        <v>1.181</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>1.233</v>
+        <v>1.025</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-0.1598</v>
+        <v>0.7383</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>-0.5416</v>
+        <v>-0.5714</v>
       </c>
       <c r="AP18" s="2" t="n">
-        <v>-0.3133</v>
+        <v>-0.7566000000000001</v>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>-0.4623</v>
+        <v>0.0366</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>-0.0762</v>
+        <v>0.3594</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.042</v>
+        <v>0.853</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>-3.59</v>
+        <v>99.92</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -2576,99 +2580,105 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>39.13</v>
+        <v>0.55</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>14.67</v>
+        <v>13.73</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-2.3</v>
+        <v>6.39</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-4.33</v>
+        <v>7.23</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>-2.9</v>
+        <v>95</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>30</v>
+        <v>72</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
-      <c r="AC19" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AD19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AD19" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG19" s="2" t="n">
-        <v>1.076</v>
+        <v>0.84</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>1.074</v>
+        <v>0.839</v>
       </c>
       <c r="AI19" s="2" t="n">
-        <v>1.061</v>
+        <v>0.842</v>
       </c>
       <c r="AJ19" s="2" t="n">
-        <v>1.076</v>
+        <v>0.836</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>1.103</v>
+        <v>0.825</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>1.182</v>
+        <v>0.8</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>1.024</v>
+        <v>0.798</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>1.1195</v>
+        <v>-0.2469</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>-0.2683</v>
+        <v>0.1892</v>
       </c>
       <c r="AP19" s="2" t="n">
-        <v>-0.8028</v>
+        <v>0.3071</v>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>0.1479</v>
+        <v>0.1723</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>0.3913</v>
+        <v>0.0055</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.841</v>
+        <v>1.006</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>99.92</v>
+        <v>-3.21</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -2677,8 +2687,12 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N20" s="2" t="n">
         <v>3</v>
       </c>
@@ -2686,34 +2700,34 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-0.26</v>
+        <v>-54.55</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>12.49</v>
+        <v>-17.7</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>5.03</v>
+        <v>0.68</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>8.48</v>
+        <v>3.1</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>93.90000000000001</v>
+        <v>31.1</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
@@ -2721,58 +2735,58 @@
         </is>
       </c>
       <c r="AG20" s="2" t="n">
-        <v>0.837</v>
+        <v>1.017</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>0.838</v>
+        <v>1.02</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>0.842</v>
+        <v>1.026</v>
       </c>
       <c r="AJ20" s="2" t="n">
-        <v>0.834</v>
+        <v>1.047</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>0.824</v>
+        <v>1.081</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>0.799</v>
+        <v>1.088</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>0.798</v>
+        <v>1.225</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>-0.3086</v>
+        <v>-0.0153</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>0.2235</v>
+        <v>-0.7419</v>
       </c>
       <c r="AP20" s="2" t="n">
-        <v>0.3012</v>
+        <v>-0.5193</v>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>0.1534</v>
+        <v>-0.4658</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>-0.0026</v>
+        <v>-0.5455</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.007</v>
+        <v>1.762</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-3.21</v>
+        <v>4.5</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2781,14 +2795,12 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="n">
         <v>13</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -2796,30 +2808,28 @@
       <c r="R21" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-53.46</v>
+        <v>-17.61</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-17.54</v>
+        <v>-3.26</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>2.44</v>
+        <v>1.75</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>2.21</v>
+        <v>0.24</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>32.5</v>
+        <v>33.3</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2831,69 +2841,79 @@
         </is>
       </c>
       <c r="AG21" s="2" t="n">
-        <v>1.026</v>
+        <v>1.772</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>1.022</v>
+        <v>1.785</v>
       </c>
       <c r="AI21" s="2" t="n">
-        <v>1.029</v>
+        <v>1.816</v>
       </c>
       <c r="AJ21" s="2" t="n">
-        <v>1.051</v>
+        <v>1.831</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>1.083</v>
+        <v>1.834</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>1.09</v>
+        <v>1.817</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>1.227</v>
+        <v>1.886</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>0.1122</v>
+        <v>-0.7183</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>-0.6637999999999999</v>
+        <v>-0.9075</v>
       </c>
       <c r="AP21" s="2" t="n">
-        <v>-0.4323</v>
+        <v>-0.1909</v>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>-0.4349</v>
+        <v>-0.1364</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>-0.5346</v>
+        <v>-0.1761</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.754</v>
+        <v>2.352</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>4.5</v>
+        <v>101.52</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="n">
-        <v>13</v>
+        <v>-9</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>1</v>
@@ -2901,31 +2921,27 @@
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-17.27</v>
+        <v>24.16</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-3.51</v>
+        <v>26.19</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>1.74</v>
+        <v>6.23</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>0.88</v>
+        <v>10.43</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>38.3</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
@@ -2933,189 +2949,189 @@
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG22" s="2" t="n">
-        <v>1.782</v>
+        <v>2.325</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>1.788</v>
+        <v>2.293</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>1.823</v>
+        <v>2.253</v>
       </c>
       <c r="AJ22" s="2" t="n">
-        <v>1.833</v>
+        <v>2.238</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>1.836</v>
+        <v>2.214</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>1.819</v>
+        <v>2.197</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>1.887</v>
+        <v>2.028</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>-0.7199</v>
+        <v>1.3612</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>-0.7258</v>
+        <v>0.5871</v>
       </c>
       <c r="AP22" s="2" t="n">
-        <v>-0.1266</v>
+        <v>0.4442</v>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>-0.117</v>
+        <v>0.3406</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>-0.1727</v>
+        <v>0.2416</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.324</v>
+        <v>1.456</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>101.52</v>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+        <v>7.28</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>24.24</v>
+        <v>-22.98</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>25.22</v>
+        <v>-13.81</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>6.69</v>
+        <v>0.41</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>10.22</v>
+        <v>-2.91</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>62.5</v>
+        <v>2.1</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>2.318</v>
+        <v>1.462</v>
       </c>
       <c r="AH23" s="2" t="n">
-        <v>2.278</v>
+        <v>1.48</v>
       </c>
       <c r="AI23" s="2" t="n">
-        <v>2.247</v>
+        <v>1.506</v>
       </c>
       <c r="AJ23" s="2" t="n">
-        <v>2.234</v>
+        <v>1.546</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>2.21</v>
+        <v>1.581</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>2.194</v>
+        <v>1.725</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>2.027</v>
+        <v>1.811</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>1.1954</v>
+        <v>-0.789</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>0.5908</v>
+        <v>-1.3404</v>
       </c>
       <c r="AP23" s="2" t="n">
-        <v>0.4087</v>
+        <v>-0.3665</v>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>0.3674</v>
+        <v>-1.0275</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>0.2424</v>
+        <v>-0.2298</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.445</v>
+        <v>0.965</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>7.28</v>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>25.84</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="n">
-        <v>13</v>
+        <v>-13</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -3123,98 +3139,96 @@
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R24" s="2" t="inlineStr"/>
       <c r="S24" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-22.18</v>
+        <v>42.28</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-14.25</v>
+        <v>13.76</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>0.48</v>
+        <v>-9.26</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-4.21</v>
+        <v>-5.18</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>2.4</v>
+        <v>19.9</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>1.474</v>
+        <v>1.003</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>1.482</v>
+        <v>1.034</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>1.513</v>
+        <v>1.03</v>
       </c>
       <c r="AJ24" s="2" t="n">
-        <v>1.553</v>
+        <v>1.029</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>1.583</v>
+        <v>1.023</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>1.732</v>
+        <v>1.123</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>1.813</v>
+        <v>0.97</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>-0.791</v>
+        <v>-0.7631</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>-1.2658</v>
+        <v>-0.3958</v>
       </c>
       <c r="AP24" s="2" t="n">
-        <v>-0.3614</v>
+        <v>-0.5372</v>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>-1.0053</v>
+        <v>-0.0912</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>-0.2218</v>
+        <v>0.4228</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.976</v>
+        <v>1.256</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>25.84</v>
+        <v>96.61</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -3228,103 +3242,97 @@
         <v>-13</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="n">
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="n">
         <v>-1</v>
-      </c>
-      <c r="S25" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T25" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>45.98</v>
+        <v>17.78</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>15.56</v>
+        <v>13.72</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-8.08</v>
+        <v>1.04</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-5.82</v>
+        <v>-3.02</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>21.3</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="n">
-        <v>8</v>
-      </c>
+      <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG25" s="2" t="n">
-        <v>1.026</v>
+        <v>1.258</v>
       </c>
       <c r="AH25" s="2" t="n">
-        <v>1.039</v>
+        <v>1.264</v>
       </c>
       <c r="AI25" s="2" t="n">
-        <v>1.033</v>
+        <v>1.28</v>
       </c>
       <c r="AJ25" s="2" t="n">
-        <v>1.033</v>
+        <v>1.292</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>1.026</v>
+        <v>1.263</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>1.124</v>
+        <v>1.238</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>0.969</v>
+        <v>1.201</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>-0.3531</v>
+        <v>-0.8154</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>-0.0553</v>
+        <v>-0.8499</v>
       </c>
       <c r="AP25" s="2" t="n">
-        <v>-0.5486</v>
+        <v>0.3363</v>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>0.0119</v>
+        <v>-0.0415</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>0.4598</v>
+        <v>0.1778</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.245</v>
+        <v>0.776</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>96.61</v>
+        <v>31.83</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -3334,105 +3342,103 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T26" s="2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>18.7</v>
+        <v>-21.17</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>13.14</v>
+        <v>-15.42</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>1.14</v>
+        <v>-0.65</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-6.45</v>
+        <v>-0.11</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>65.09999999999999</v>
+        <v>5.7</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>1.266</v>
+        <v>0.785</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>1.266</v>
+        <v>0.797</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>1.285</v>
+        <v>0.801</v>
       </c>
       <c r="AJ26" s="2" t="n">
-        <v>1.292</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>1.262</v>
+        <v>0.827</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>1.238</v>
+        <v>0.918</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>1.2</v>
+        <v>0.99</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>-0.7992</v>
+        <v>-0.4721</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>-0.6993</v>
+        <v>-0.8865</v>
       </c>
       <c r="AP26" s="2" t="n">
-        <v>0.3878</v>
+        <v>-0.1854</v>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>-0.0549</v>
+        <v>-0.8604000000000001</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>0.187</v>
+        <v>-0.2117</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.772</v>
+        <v>0.626</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>31.83</v>
+        <v>32.9</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -3444,14 +3450,12 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R27" s="2" t="inlineStr"/>
       <c r="S27" s="2" t="n">
         <v>-1</v>
       </c>
@@ -3460,26 +3464,26 @@
       </c>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-20.37</v>
+        <v>40.03</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-15.65</v>
+        <v>11.98</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-1.24</v>
+        <v>-10.31</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-0.89</v>
+        <v>-4.08</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>6.7</v>
+        <v>24.2</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
@@ -3489,202 +3493,202 @@
         </is>
       </c>
       <c r="AG27" s="2" t="n">
-        <v>0.793</v>
+        <v>0.652</v>
       </c>
       <c r="AH27" s="2" t="n">
-        <v>0.798</v>
+        <v>0.676</v>
       </c>
       <c r="AI27" s="2" t="n">
-        <v>0.804</v>
+        <v>0.669</v>
       </c>
       <c r="AJ27" s="2" t="n">
-        <v>0.819</v>
+        <v>0.666</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>0.828</v>
+        <v>0.658</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>0.921</v>
+        <v>0.729</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>0.99</v>
+        <v>0.642</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>-0.4138</v>
+        <v>-0.5409</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>-0.793</v>
+        <v>-0.2555</v>
       </c>
       <c r="AP27" s="2" t="n">
-        <v>-0.1827</v>
+        <v>-0.3674</v>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>-0.7998</v>
+        <v>-0.1703</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>-0.2037</v>
+        <v>0.4003</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.629</v>
+        <v>2.24</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
+        <v>3.12</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="n">
-        <v>-13</v>
+        <v>13</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="n">
-        <v>-1</v>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S28" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T28" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>44.06</v>
+        <v>-24.84</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>13</v>
+        <v>-15.71</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-10.54</v>
+        <v>0.22</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-4.7</v>
+        <v>-1.54</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>25.5</v>
+        <v>0.4</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG28" s="2" t="n">
-        <v>0.669</v>
+        <v>2.25</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>0.678</v>
+        <v>2.286</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>0.67</v>
+        <v>2.316</v>
       </c>
       <c r="AJ28" s="2" t="n">
-        <v>0.669</v>
+        <v>2.373</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>0.659</v>
+        <v>2.427</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>0.731</v>
+        <v>2.677</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>0.641</v>
+        <v>2.86</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>-0.0613</v>
+        <v>-0.869</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>0.1128</v>
+        <v>-1.2034</v>
       </c>
       <c r="AP28" s="2" t="n">
-        <v>-0.3635</v>
+        <v>-0.313</v>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>-0.0577</v>
+        <v>-1.0341</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>0.4406</v>
+        <v>-0.2484</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2.224</v>
+        <v>0.897</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>3.17</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="n">
         <v>13</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -3696,31 +3700,27 @@
         <v>-1</v>
       </c>
       <c r="T29" s="2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-24.15</v>
+        <v>-5.4</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-16.11</v>
+        <v>-6.12</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-0.35</v>
+        <v>0.35</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-2.96</v>
+        <v>-0.68</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AA29" s="2" t="n">
-        <v>17</v>
-      </c>
+        <v>-3</v>
+      </c>
+      <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="AC29" s="2" t="inlineStr"/>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
@@ -3729,58 +3729,58 @@
         </is>
       </c>
       <c r="AG29" s="2" t="n">
-        <v>2.269</v>
+        <v>0.908</v>
       </c>
       <c r="AH29" s="2" t="n">
-        <v>2.292</v>
+        <v>0.917</v>
       </c>
       <c r="AI29" s="2" t="n">
-        <v>2.325</v>
+        <v>0.926</v>
       </c>
       <c r="AJ29" s="2" t="n">
-        <v>2.386</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>2.43</v>
+        <v>0.953</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>2.688</v>
+        <v>1.04</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>2.862</v>
+        <v>1.028</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-0.7955</v>
+        <v>-0.3268</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>-1.1504</v>
+        <v>-0.7282999999999999</v>
       </c>
       <c r="AP29" s="2" t="n">
-        <v>-0.3139</v>
+        <v>-0.4477</v>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>-1.004</v>
+        <v>-0.4501</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>-0.2415</v>
+        <v>-0.054</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.9</v>
+        <v>1.616</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>3.17</v>
+        <v>-4.94</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -3790,11 +3790,9 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -3810,83 +3808,87 @@
       </c>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-4.09</v>
+        <v>22.33</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-5.57</v>
+        <v>6.42</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>0.63</v>
+        <v>-5.08</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-0.7</v>
+        <v>-3.71</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-2.3</v>
-      </c>
-      <c r="AA30" s="2" t="inlineStr"/>
+        <v>-3.9</v>
+      </c>
+      <c r="AA30" s="2" t="n">
+        <v>17</v>
+      </c>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG30" s="2" t="n">
-        <v>0.915</v>
+        <v>1.677</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>0.918</v>
+        <v>1.704</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>0.929</v>
+        <v>1.686</v>
       </c>
       <c r="AJ30" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.705</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>0.955</v>
+        <v>1.748</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>1.042</v>
+        <v>1.853</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>1.029</v>
+        <v>1.673</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>-0.3711</v>
+        <v>0.5054</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>-0.5838</v>
+        <v>-0.6065</v>
       </c>
       <c r="AP30" s="2" t="n">
-        <v>-0.4844</v>
+        <v>-0.7201</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>-0.372</v>
+        <v>-0.08989999999999999</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>-0.0409</v>
+        <v>0.2233</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.657</v>
+        <v>1.101</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>-4.94</v>
+        <v>81.33</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -3898,83 +3900,77 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R31" s="2" t="inlineStr"/>
       <c r="S31" s="2" t="inlineStr"/>
-      <c r="T31" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>24.81</v>
+        <v>-6.02</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>9.5</v>
+        <v>-7.77</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-1.66</v>
+        <v>-1.52</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-2.76</v>
+        <v>2.54</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>-2.8</v>
+        <v>38.4</v>
       </c>
       <c r="AA31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="n">
-        <v>7</v>
-      </c>
+      <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG31" s="2" t="n">
-        <v>1.705</v>
+        <v>1.116</v>
       </c>
       <c r="AH31" s="2" t="n">
-        <v>1.706</v>
+        <v>1.138</v>
       </c>
       <c r="AI31" s="2" t="n">
-        <v>1.692</v>
+        <v>1.147</v>
       </c>
       <c r="AJ31" s="2" t="n">
-        <v>1.714</v>
+        <v>1.135</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>1.756</v>
+        <v>1.13</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>1.855</v>
+        <v>1.202</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>1.672</v>
+        <v>1.302</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>0.8141</v>
+        <v>-1.0525</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>-0.3191</v>
+        <v>-0.1086</v>
       </c>
       <c r="AP31" s="2" t="n">
-        <v>-0.6979</v>
+        <v>0.1014</v>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>0.016</v>
+        <v>-0.7053</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>0.2481</v>
+        <v>-0.0602</v>
       </c>
     </row>
   </sheetData>
@@ -4005,7 +4001,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-29 | 30 只</t>
+          <t>截至: 2026-09-30 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-03
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -4195,14 +4195,14 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置(位置门前): {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。位置门 = A OR B。A: 200日pos&lt;=0.80(200日数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5% 且距250日收盘高点回落≥5%(创新高处的平台突破归新高, 不算SOS)。仙股过滤: 信号K线收盘&lt;0.5(本币)不触发。强度: 放量+RS超额+阳线。捕获纠缠平台突破、次新股底部反强</t>
+          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置: {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。强度路径: 放量+RS超额+阳线。无位置门(2026-10-02取消: 原A门200日pos&lt;=0.80/B门均线纠缠+距250日高点回落≥5%/门E Stage 1B-2B 全部移除, 高位/新高处的放量突破同样算SOS)。仙股过滤: 信号K线收盘&lt;0.5(本币)不触发</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=2x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
+          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=2x 20日均量; 海外大盘股池放宽至1.5x) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-08
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -742,19 +742,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.154</v>
+        <v>1.403</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>12.25</v>
+        <v>-1.36</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -764,103 +764,103 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="n">
+      <c r="R2" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>7.06</v>
+        <v>-13.19</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-1.48</v>
+        <v>-1.1</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-4.13</v>
+        <v>0.87</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-3.35</v>
+        <v>0.52</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>-1.9</v>
+        <v>58.5</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="AC2" s="2" t="inlineStr"/>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>3.237</v>
+        <v>1.44</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>3.306</v>
+        <v>1.449</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>3.323</v>
+        <v>1.462</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>3.372</v>
+        <v>1.475</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>3.437</v>
+        <v>1.488</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>3.718</v>
+        <v>1.469</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>3.527</v>
+        <v>1.515</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-0.7105</v>
+        <v>-0.3257</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>-0.8094</v>
+        <v>-0.4861</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>-0.6024</v>
+        <v>-0.1366</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>-0.4007</v>
+        <v>-0.2006</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.0706</v>
+        <v>-0.1319</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.445</v>
+        <v>0.653</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>7.34</v>
+        <v>-2.04</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -871,7 +871,7 @@
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="n">
-        <v>13</v>
+        <v>-13</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>2</v>
@@ -880,30 +880,28 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-11.91</v>
+        <v>-29.89</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>0.77</v>
+        <v>-4.75</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>2.48</v>
+        <v>4.47</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>3.35</v>
+        <v>5.07</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>62.6</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -915,72 +913,78 @@
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>1.45</v>
+        <v>0.65</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>1.453</v>
+        <v>0.652</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>1.465</v>
+        <v>0.66</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>1.477</v>
+        <v>0.662</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>1.488</v>
+        <v>0.668</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>1.47</v>
+        <v>0.662</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>1.515</v>
+        <v>0.717</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>-0.227</v>
+        <v>-0.2776</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>-0.4334</v>
+        <v>-0.3715</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>-0.09279999999999999</v>
+        <v>-0.1351</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>-0.1726</v>
+        <v>-0.3334</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>-0.1191</v>
+        <v>-0.2989</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.658</v>
+        <v>1.937</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-2.04</v>
+        <v>100.48</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="L4" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
@@ -988,36 +992,36 @@
       <c r="R4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="S4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-30.46</v>
+        <v>49.14</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-5.16</v>
+        <v>43.92</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>4.45</v>
+        <v>24.02</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>5.21</v>
+        <v>22.12</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>65.7</v>
+        <v>100.3</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
@@ -1025,111 +1029,103 @@
         </is>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>0.65</v>
+        <v>1.797</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.652</v>
+        <v>1.767</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>0.661</v>
+        <v>1.755</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>0.662</v>
+        <v>1.699</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>0.668</v>
+        <v>1.619</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>0.662</v>
+        <v>1.579</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>0.718</v>
+        <v>1.512</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>-0.4979</v>
+        <v>0.2157</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>-0.3478</v>
+        <v>1.4417</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>-0.104</v>
+        <v>0.9384</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>-0.3478</v>
+        <v>0.204</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>-0.3046</v>
+        <v>0.4914</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.772</v>
+        <v>0.839</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>101.26</v>
+        <v>4.26</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S5" s="2" t="inlineStr"/>
-      <c r="T5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>44.4</v>
+        <v>-3.21</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>30.49</v>
+        <v>6.96</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>6.57</v>
+        <v>1.39</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>12.78</v>
+        <v>6.43</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>98.09999999999999</v>
+        <v>57.2</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
         <is>
@@ -1137,160 +1133,166 @@
         </is>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>1.746</v>
+        <v>0.848</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>1.755</v>
+        <v>0.851</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>1.743</v>
+        <v>0.842</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>1.686</v>
+        <v>0.851</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>1.611</v>
+        <v>0.863</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>1.576</v>
+        <v>0.827</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>1.509</v>
+        <v>0.833</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>-0.356</v>
+        <v>0.8633</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>1.3265</v>
+        <v>-0.1109</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>0.7924</v>
+        <v>-0.1682</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.0992</v>
+        <v>0.0315</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.444</v>
+        <v>-0.0321</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.872</v>
+        <v>4.389</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+        <v>4.59</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R6" s="2" t="inlineStr"/>
       <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-2.47</v>
+        <v>-3.27</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>9.91</v>
+        <v>1.4</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>5.4</v>
+        <v>0.17</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>10.13</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>58.1</v>
+        <v>-2.9</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>77</v>
+        <v>19</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
-      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>0.854</v>
+        <v>4.434</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>0.85</v>
+        <v>4.51</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>0.842</v>
+        <v>4.553</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>0.853</v>
+        <v>4.588</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>0.863</v>
+        <v>4.636</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>0.827</v>
+        <v>4.757</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>0.833</v>
+        <v>4.717</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>-0.7401</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>-0.0925</v>
+        <v>-0.6705</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>-0.1693</v>
+        <v>-0.3068</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.0542</v>
+        <v>-0.266</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>-0.0247</v>
+        <v>-0.0327</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.938</v>
+        <v>3.416</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2.95</v>
+        <v>88.95</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -1299,102 +1301,108 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-3.88</v>
+        <v>10.83</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>3.39</v>
+        <v>15.86</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>1.67</v>
+        <v>7.11</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>1.93</v>
+        <v>4.75</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>26.6</v>
+        <v>80.8</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>2.948</v>
+        <v>3.362</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>2.967</v>
+        <v>3.361</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>2.987</v>
+        <v>3.393</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>2.996</v>
+        <v>3.408</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>3.013</v>
+        <v>3.358</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>3.015</v>
+        <v>3.26</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>3.042</v>
+        <v>3.218</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>-0.3678</v>
+        <v>-0.366</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>-0.3849</v>
+        <v>-0.3854</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>-0.1184</v>
+        <v>0.2569</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>-0.123</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>-0.0388</v>
+        <v>0.1083</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.432</v>
+        <v>0.484</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>9.76</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1403,44 +1411,40 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T8" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>-1.82</v>
+        <v>-17.1</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.3</v>
+        <v>-3.62</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-0.02</v>
+        <v>-0.28</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>-2.1</v>
+        <v>16.6</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
-      <c r="AC8" s="2" t="n">
-        <v>7</v>
-      </c>
+      <c r="AC8" s="2" t="inlineStr"/>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
       <c r="AF8" s="2" t="inlineStr">
@@ -1449,58 +1453,58 @@
         </is>
       </c>
       <c r="AG8" s="2" t="n">
-        <v>4.474</v>
+        <v>0.492</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>4.525</v>
+        <v>0.499</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>4.564</v>
+        <v>0.507</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>4.597</v>
+        <v>0.511</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>4.643</v>
+        <v>0.517</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>4.762</v>
+        <v>0.517</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>4.718</v>
+        <v>0.532</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-0.6103</v>
+        <v>-0.7796</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>-0.5749</v>
+        <v>-0.9068000000000001</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>-0.2778</v>
+        <v>-0.3975</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>-0.2289</v>
+        <v>-0.1556</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>-0.0182</v>
+        <v>-0.171</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.472</v>
+        <v>0.382</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>52.12</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1512,101 +1516,105 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="n">
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="V9" s="2" t="n">
-        <v>9.890000000000001</v>
+        <v>-3.15</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>2.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-0.98</v>
+        <v>4.7</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-0.48</v>
+        <v>8.43</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>15.4</v>
+        <v>65.5</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
-      <c r="AC9" s="2" t="n">
-        <v>7</v>
-      </c>
+      <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>7.572</v>
+        <v>0.379</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>7.68</v>
+        <v>0.38</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>7.695</v>
+        <v>0.376</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>7.748</v>
+        <v>0.379</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>7.763</v>
+        <v>0.382</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>8.096</v>
+        <v>0.364</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>8.013</v>
+        <v>0.371</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>-0.3166</v>
+        <v>0.747</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>-0.5612</v>
+        <v>-0.0141</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>-0.1305</v>
+        <v>0.0741</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>-0.3137</v>
+        <v>0.0769</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>0.0989</v>
+        <v>-0.0315</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.368</v>
+        <v>2.904</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>100.6</v>
+        <v>77.83</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1615,12 +1623,12 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
@@ -1628,93 +1636,87 @@
       <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>10.27</v>
+        <v>2.3</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>13.08</v>
+        <v>-0.5</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>3.98</v>
+        <v>-3.43</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>1.75</v>
+        <v>-0.74</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>80.5</v>
+        <v>32.2</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="n">
-        <v>3</v>
-      </c>
+      <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>3.348</v>
+        <v>2.98</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.356</v>
+        <v>3.054</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>3.394</v>
+        <v>3.06</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>3.406</v>
+        <v>3.071</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>3.355</v>
+        <v>3.047</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>3.258</v>
+        <v>3.214</v>
       </c>
       <c r="AM10" s="2" t="n">
         <v>3.216</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>-0.6655</v>
+        <v>-0.5606</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>-0.444</v>
+        <v>-0.5973000000000001</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>0.258</v>
+        <v>0.089</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>0.0422</v>
+        <v>-0.4208</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>0.1027</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.492</v>
+        <v>0.339</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>4.78</v>
+        <v>40.85</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1723,14 +1725,10 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
@@ -1744,22 +1742,22 @@
       </c>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-15.48</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-3.16</v>
+        <v>7.07</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.74</v>
+        <v>2.07</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>-0.4</v>
+        <v>7.16</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>20.5</v>
+        <v>74</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1767,62 +1765,62 @@
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG11" s="2" t="n">
-        <v>0.497</v>
+        <v>0.342</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>0.501</v>
+        <v>0.343</v>
       </c>
       <c r="AI11" s="2" t="n">
-        <v>0.509</v>
+        <v>0.339</v>
       </c>
       <c r="AJ11" s="2" t="n">
-        <v>0.512</v>
+        <v>0.341</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>0.518</v>
+        <v>0.34</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>0.517</v>
+        <v>0.326</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>0.532</v>
+        <v>0.336</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>-0.6657</v>
+        <v>0.7194</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>-0.7849</v>
+        <v>0.0172</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>-0.3612</v>
+        <v>0.2337</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>-0.1184</v>
+        <v>0.0338</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>-0.1548</v>
+        <v>-0.0069</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.388</v>
+        <v>0.417</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>9.880000000000001</v>
+        <v>-1.36</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1831,9 +1829,7 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
         <v>2</v>
@@ -1844,30 +1840,28 @@
       <c r="R12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T12" s="2" t="inlineStr"/>
-      <c r="U12" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-3.3</v>
+        <v>-43.76</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>9.210000000000001</v>
+        <v>-9.109999999999999</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>5.83</v>
+        <v>5.25</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>10.04</v>
+        <v>6.42</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>65.2</v>
+        <v>50.4</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1879,58 +1873,58 @@
         </is>
       </c>
       <c r="AG12" s="2" t="n">
-        <v>0.38</v>
+        <v>0.411</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>0.378</v>
+        <v>0.412</v>
       </c>
       <c r="AI12" s="2" t="n">
-        <v>0.376</v>
+        <v>0.416</v>
       </c>
       <c r="AJ12" s="2" t="n">
-        <v>0.379</v>
+        <v>0.418</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>0.382</v>
+        <v>0.426</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>0.364</v>
+        <v>0.424</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>0.371</v>
+        <v>0.472</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>0.7098</v>
+        <v>-0.0898</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>-0.0495</v>
+        <v>-0.3837</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>0.0741</v>
+        <v>-0.1625</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>0.0828</v>
+        <v>-0.3919</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>-0.033</v>
+        <v>-0.4376</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.764</v>
+        <v>0.971</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2.2</v>
+        <v>-3.59</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1940,103 +1934,103 @@
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S13" s="2" t="inlineStr"/>
-      <c r="T13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-13.54</v>
+        <v>32.13</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-2.28</v>
+        <v>7.5</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>0.95</v>
+        <v>-10.32</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>0.12</v>
+        <v>-8.16</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>37.7</v>
+        <v>-4.9</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
-      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="AD13" s="2" t="inlineStr"/>
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG13" s="2" t="n">
-        <v>0.767</v>
+        <v>1.029</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>0.775</v>
+        <v>1.062</v>
       </c>
       <c r="AI13" s="2" t="n">
-        <v>0.788</v>
+        <v>1.052</v>
       </c>
       <c r="AJ13" s="2" t="n">
-        <v>0.79</v>
+        <v>1.065</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>0.795</v>
+        <v>1.093</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>0.788</v>
+        <v>1.179</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>0.827</v>
+        <v>1.026</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>-0.8166</v>
+        <v>-0.063</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>-0.6854</v>
+        <v>-0.8867</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>-0.2365</v>
+        <v>-0.8214</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>-0.1572</v>
+        <v>-0.07389999999999999</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>-0.1354</v>
+        <v>0.3213</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.971</v>
+        <v>0.859</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>43.79</v>
+        <v>99.92</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -2046,103 +2040,105 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S14" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>4.34</v>
+        <v>1.7</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>0.7</v>
+        <v>15.73</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-1.72</v>
+        <v>8.51</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>0.47</v>
+        <v>7.96</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>34.6</v>
+        <v>96.5</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>22</v>
+        <v>84</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
-      <c r="AD14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG14" s="2" t="n">
-        <v>3.028</v>
+        <v>0.845</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>3.071</v>
+        <v>0.841</v>
       </c>
       <c r="AI14" s="2" t="n">
-        <v>3.069</v>
+        <v>0.843</v>
       </c>
       <c r="AJ14" s="2" t="n">
-        <v>3.075</v>
+        <v>0.837</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>3.047</v>
+        <v>0.826</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>3.22</v>
+        <v>0.801</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>3.216</v>
+        <v>0.798</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>-0.1856</v>
+        <v>-0.068</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>-0.3792</v>
+        <v>0.2233</v>
       </c>
       <c r="AP14" s="2" t="n">
-        <v>0.0762</v>
+        <v>0.3283</v>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>-0.3534</v>
+        <v>0.1977</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>0.0434</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.349</v>
+        <v>0.981</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>40.85</v>
+        <v>-8.65</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -2152,38 +2148,42 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M15" s="2" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N15" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S15" s="2" t="inlineStr"/>
-      <c r="T15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-0.05</v>
+        <v>-55.92</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>9.06</v>
+        <v>-18.7</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>5.13</v>
+        <v>0.6</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>9.67</v>
+        <v>1.54</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>74.8</v>
+        <v>28.4</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
@@ -2195,58 +2195,58 @@
         </is>
       </c>
       <c r="AG15" s="2" t="n">
-        <v>0.344</v>
+        <v>1.007</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>0.342</v>
+        <v>1.016</v>
       </c>
       <c r="AI15" s="2" t="n">
-        <v>0.339</v>
+        <v>1.022</v>
       </c>
       <c r="AJ15" s="2" t="n">
-        <v>0.341</v>
+        <v>1.043</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>0.339</v>
+        <v>1.079</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>0.325</v>
+        <v>1.085</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>0.336</v>
+        <v>1.222</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>0.8506</v>
+        <v>-0.1937</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>0.0418</v>
+        <v>-0.779</v>
       </c>
       <c r="AP15" s="2" t="n">
-        <v>0.2498</v>
+        <v>-0.5306</v>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>0.0518</v>
+        <v>-0.5001</v>
       </c>
       <c r="AR15" s="2" t="n">
-        <v>-0.0005</v>
+        <v>-0.5592</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.417</v>
+        <v>1.721</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>-1.36</v>
+        <v>-4.21</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -2256,38 +2256,36 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R16" s="2" t="inlineStr"/>
       <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-44.86</v>
+        <v>-19.2</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-10.23</v>
+        <v>-4.37</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>4.8</v>
+        <v>0.01</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>5.42</v>
+        <v>0.24</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>49.9</v>
+        <v>27.9</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>72</v>
+        <v>22</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
@@ -2299,58 +2297,58 @@
         </is>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>0.41</v>
+        <v>1.754</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>0.411</v>
+        <v>1.777</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>0.417</v>
+        <v>1.809</v>
       </c>
       <c r="AJ16" s="2" t="n">
-        <v>0.419</v>
+        <v>1.828</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>0.426</v>
+        <v>1.832</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>0.425</v>
+        <v>1.816</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>0.473</v>
+        <v>1.884</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>-0.3394</v>
+        <v>-0.8405</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>-0.3949</v>
+        <v>-0.98</v>
       </c>
       <c r="AP16" s="2" t="n">
-        <v>-0.1324</v>
+        <v>-0.2441</v>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>-0.4118</v>
+        <v>-0.1704</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>-0.4486</v>
+        <v>-0.192</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.082</v>
+        <v>2.374</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>5.68</v>
+        <v>109.67</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -2359,216 +2357,216 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N17" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S17" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T17" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-8.94</v>
+        <v>24.4</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-6.28</v>
+        <v>28.57</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-2.11</v>
+        <v>7.1</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-3.45</v>
+        <v>13.27</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>3.8</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>19</v>
+        <v>86</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
-      <c r="AC17" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AC17" s="2" t="inlineStr"/>
       <c r="AD17" s="2" t="inlineStr"/>
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG17" s="2" t="n">
-        <v>1.105</v>
+        <v>2.333</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>1.119</v>
+        <v>2.309</v>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>1.13</v>
+        <v>2.262</v>
       </c>
       <c r="AJ17" s="2" t="n">
-        <v>1.142</v>
+        <v>2.244</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>1.167</v>
+        <v>2.219</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>1.206</v>
+        <v>2.2</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>1.232</v>
+        <v>2.03</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>-0.3151</v>
+        <v>1.4853</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>-0.8376</v>
+        <v>0.6415</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>-0.3717</v>
+        <v>0.4901</v>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>-0.54</v>
+        <v>0.3206</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>-0.08939999999999999</v>
+        <v>0.244</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.012</v>
+        <v>1.448</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>-3.59</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
+        <v>6.69</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N18" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S18" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T18" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>35.94</v>
+        <v>-23.49</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>10.91</v>
+        <v>-13.3</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-6.8</v>
+        <v>0.93</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-5.25</v>
+        <v>-1.48</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>-3.8</v>
+        <v>1.6</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG18" s="2" t="n">
-        <v>1.056</v>
+        <v>1.451</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>1.072</v>
+        <v>1.476</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>1.057</v>
+        <v>1.501</v>
       </c>
       <c r="AJ18" s="2" t="n">
-        <v>1.07</v>
+        <v>1.539</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>1.098</v>
+        <v>1.579</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>1.181</v>
+        <v>1.719</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>1.025</v>
+        <v>1.809</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>0.7383</v>
+        <v>-0.7841</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>-0.5714</v>
+        <v>-1.3172</v>
       </c>
       <c r="AP18" s="2" t="n">
-        <v>-0.7566000000000001</v>
+        <v>-0.3585</v>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>0.0366</v>
+        <v>-1.0389</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>0.3594</v>
+        <v>-0.2349</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.853</v>
+        <v>1.279</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>99.92</v>
+        <v>81.22</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -2578,48 +2576,44 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="T19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>0.55</v>
+        <v>18.09</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>13.73</v>
+        <v>16.92</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>6.39</v>
+        <v>6.27</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>7.23</v>
+        <v>2.09</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>95</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
-      <c r="AD19" s="2" t="n">
-        <v>10</v>
-      </c>
+      <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
@@ -2627,174 +2621,198 @@
         </is>
       </c>
       <c r="AG19" s="2" t="n">
-        <v>0.84</v>
+        <v>1.262</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>0.839</v>
+        <v>1.265</v>
       </c>
       <c r="AI19" s="2" t="n">
-        <v>0.842</v>
+        <v>1.28</v>
       </c>
       <c r="AJ19" s="2" t="n">
-        <v>0.836</v>
+        <v>1.292</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>0.825</v>
+        <v>1.264</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>0.8</v>
+        <v>1.239</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>0.798</v>
+        <v>1.202</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>-0.2469</v>
+        <v>-0.472</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>0.1892</v>
+        <v>-0.8077</v>
       </c>
       <c r="AP19" s="2" t="n">
-        <v>0.3071</v>
+        <v>0.3182</v>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>0.1723</v>
+        <v>-0.0025</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>0.0055</v>
+        <v>0.1809</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.006</v>
+        <v>0.763</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-3.21</v>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+        <v>7.96</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-54.55</v>
+        <v>-22.39</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-17.7</v>
+        <v>-15.89</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>0.68</v>
+        <v>-1.35</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>3.1</v>
+        <v>-0.21</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>31.1</v>
+        <v>4.6</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG20" s="2" t="n">
-        <v>1.017</v>
+        <v>0.775</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>1.02</v>
+        <v>0.793</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>1.026</v>
+        <v>0.799</v>
       </c>
       <c r="AJ20" s="2" t="n">
-        <v>1.047</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>1.081</v>
+        <v>0.826</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>1.088</v>
+        <v>0.914</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>1.225</v>
+        <v>0.989</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>-0.0153</v>
+        <v>-0.6793</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>-0.7419</v>
+        <v>-0.9237</v>
       </c>
       <c r="AP20" s="2" t="n">
-        <v>-0.5193</v>
+        <v>-0.2119</v>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>-0.4658</v>
+        <v>-0.9242</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>-0.5455</v>
+        <v>-0.2239</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.762</v>
+        <v>2.234</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
+        <v>3.12</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="n">
         <v>13</v>
@@ -2805,322 +2823,304 @@
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R21" s="2" t="inlineStr"/>
       <c r="S21" s="2" t="inlineStr"/>
-      <c r="T21" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-17.61</v>
+        <v>-25.3</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-3.26</v>
+        <v>-15.01</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>1.75</v>
+        <v>0.98</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>0.24</v>
+        <v>-0.16</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>33.3</v>
+        <v>0.1</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
-      <c r="AC21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="inlineStr"/>
       <c r="AF21" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG21" s="2" t="n">
-        <v>1.772</v>
+        <v>2.234</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>1.785</v>
+        <v>2.279</v>
       </c>
       <c r="AI21" s="2" t="n">
-        <v>1.816</v>
+        <v>2.31</v>
       </c>
       <c r="AJ21" s="2" t="n">
-        <v>1.831</v>
+        <v>2.364</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>1.834</v>
+        <v>2.424</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>1.817</v>
+        <v>2.667</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>1.886</v>
+        <v>2.857</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>-0.7183</v>
+        <v>-0.9287</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>-0.9075</v>
+        <v>-1.151</v>
       </c>
       <c r="AP21" s="2" t="n">
-        <v>-0.1909</v>
+        <v>-0.3051</v>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>-0.1364</v>
+        <v>-1.0557</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>-0.1761</v>
+        <v>-0.253</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2.352</v>
+        <v>0.862</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>101.52</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+        <v>3.17</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="n">
-        <v>-9</v>
+        <v>13</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>24.16</v>
+        <v>-7.63</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>26.19</v>
+        <v>-8.73</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>6.23</v>
+        <v>-2.36</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>10.43</v>
+        <v>-2.96</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>67.40000000000001</v>
-      </c>
-      <c r="AA22" s="2" t="n">
-        <v>82</v>
-      </c>
+        <v>-3.8</v>
+      </c>
+      <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG22" s="2" t="n">
-        <v>2.325</v>
+        <v>0.895</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>2.293</v>
+        <v>0.912</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>2.253</v>
+        <v>0.922</v>
       </c>
       <c r="AJ22" s="2" t="n">
-        <v>2.238</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>2.214</v>
+        <v>0.951</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>2.197</v>
+        <v>1.037</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>2.028</v>
+        <v>1.028</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>1.3612</v>
+        <v>-0.536</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>0.5871</v>
+        <v>-0.9147</v>
       </c>
       <c r="AP22" s="2" t="n">
-        <v>0.4442</v>
+        <v>-0.4293</v>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>0.3406</v>
+        <v>-0.5324</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>0.2416</v>
+        <v>-0.07630000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.456</v>
+        <v>1.537</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>7.28</v>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>-4.94</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R23" s="2" t="inlineStr"/>
       <c r="S23" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>-22.98</v>
+        <v>18.89</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>-13.81</v>
+        <v>2.28</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>0.41</v>
+        <v>-9.58</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-2.91</v>
+        <v>-7.21</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>2.1</v>
+        <v>-4.9</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>1.462</v>
+        <v>1.633</v>
       </c>
       <c r="AH23" s="2" t="n">
-        <v>1.48</v>
+        <v>1.687</v>
       </c>
       <c r="AI23" s="2" t="n">
-        <v>1.506</v>
+        <v>1.678</v>
       </c>
       <c r="AJ23" s="2" t="n">
-        <v>1.546</v>
+        <v>1.697</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>1.581</v>
+        <v>1.739</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>1.725</v>
+        <v>1.85</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>1.811</v>
+        <v>1.674</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>-0.789</v>
+        <v>-0.279</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>-1.3404</v>
+        <v>-0.918</v>
       </c>
       <c r="AP23" s="2" t="n">
-        <v>-0.3665</v>
+        <v>-0.8077</v>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>-1.0275</v>
+        <v>-0.1962</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>-0.2298</v>
+        <v>0.1889</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.965</v>
+        <v>3.053</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>25.84</v>
+        <v>6.32</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -3130,9 +3130,7 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
         <v>0</v>
       </c>
@@ -3140,34 +3138,30 @@
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T24" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>42.28</v>
+        <v>4.1</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>13.76</v>
+        <v>-3.61</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-9.26</v>
+        <v>-6.18</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-5.18</v>
+        <v>-4.5</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>19.9</v>
+        <v>-3.1</v>
       </c>
       <c r="AA24" s="2" t="n">
         <v>15</v>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
@@ -3177,58 +3171,58 @@
         </is>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>1.003</v>
+        <v>3.168</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>1.034</v>
+        <v>3.279</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>1.03</v>
+        <v>3.309</v>
       </c>
       <c r="AJ24" s="2" t="n">
-        <v>1.029</v>
+        <v>3.357</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>1.023</v>
+        <v>3.426</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>1.123</v>
+        <v>3.709</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>0.97</v>
+        <v>3.526</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>-0.7631</v>
+        <v>-1.1796</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>-0.3958</v>
+        <v>-1.0017</v>
       </c>
       <c r="AP24" s="2" t="n">
-        <v>-0.5372</v>
+        <v>-0.635</v>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>-0.0912</v>
+        <v>-0.4839</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>0.4228</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.256</v>
+        <v>2.918</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>96.61</v>
+        <v>2.95</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -3238,9 +3232,7 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
         <v>1</v>
       </c>
@@ -3249,27 +3241,25 @@
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr"/>
-      <c r="T25" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>17.78</v>
+        <v>-4.84</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>13.72</v>
+        <v>3.8</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>1.04</v>
+        <v>1.98</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-3.02</v>
+        <v>1.94</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>64.90000000000001</v>
+        <v>22.3</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="inlineStr"/>
@@ -3277,62 +3267,62 @@
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG25" s="2" t="n">
-        <v>1.258</v>
+        <v>2.932</v>
       </c>
       <c r="AH25" s="2" t="n">
-        <v>1.264</v>
+        <v>2.961</v>
       </c>
       <c r="AI25" s="2" t="n">
-        <v>1.28</v>
+        <v>2.982</v>
       </c>
       <c r="AJ25" s="2" t="n">
-        <v>1.292</v>
+        <v>2.993</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>1.263</v>
+        <v>3.01</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>1.238</v>
+        <v>3.013</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>1.201</v>
+        <v>3.041</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>-0.8154</v>
+        <v>-0.4378</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>-0.8499</v>
+        <v>-0.4655</v>
       </c>
       <c r="AP25" s="2" t="n">
-        <v>0.3363</v>
+        <v>-0.1542</v>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>-0.0415</v>
+        <v>-0.1469</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>0.1778</v>
+        <v>-0.0484</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.776</v>
+        <v>7.279</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>31.83</v>
+        <v>52.12</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -3344,40 +3334,36 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T26" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-21.17</v>
+        <v>7.88</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-15.42</v>
+        <v>0.8</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-0.65</v>
+        <v>-2.68</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-0.11</v>
+        <v>-1.72</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>5.7</v>
+        <v>12.5</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
@@ -3387,58 +3373,58 @@
         </is>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>0.785</v>
+        <v>7.462</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>0.797</v>
+        <v>7.636</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>0.801</v>
+        <v>7.67</v>
       </c>
       <c r="AJ26" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>7.729</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>0.827</v>
+        <v>7.752</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>0.918</v>
+        <v>8.08</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>0.99</v>
+        <v>8.012</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>-0.4721</v>
+        <v>-0.627</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>-0.8865</v>
+        <v>-0.7281</v>
       </c>
       <c r="AP26" s="2" t="n">
-        <v>-0.1854</v>
+        <v>-0.1475</v>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>-0.8604000000000001</v>
+        <v>-0.3755</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>-0.2117</v>
+        <v>0.0788</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.626</v>
+        <v>0.752</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>32.9</v>
+        <v>-4.85</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -3450,171 +3436,135 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T27" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>40.03</v>
+        <v>-15.29</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>11.98</v>
+        <v>-2.73</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-10.31</v>
+        <v>0.48</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-4.08</v>
+        <v>-0.18</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>24.2</v>
+        <v>31.8</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="AC27" s="2" t="inlineStr"/>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG27" s="2" t="n">
-        <v>0.652</v>
+        <v>0.761</v>
       </c>
       <c r="AH27" s="2" t="n">
-        <v>0.676</v>
+        <v>0.772</v>
       </c>
       <c r="AI27" s="2" t="n">
-        <v>0.669</v>
+        <v>0.786</v>
       </c>
       <c r="AJ27" s="2" t="n">
-        <v>0.666</v>
+        <v>0.79</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>0.658</v>
+        <v>0.794</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>0.729</v>
+        <v>0.787</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>0.642</v>
+        <v>0.827</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>-0.5409</v>
+        <v>-0.8985</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>-0.2555</v>
+        <v>-0.7939000000000001</v>
       </c>
       <c r="AP27" s="2" t="n">
-        <v>-0.3674</v>
+        <v>-0.2915</v>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>-0.1703</v>
+        <v>-0.1857</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>0.4003</v>
+        <v>-0.1529</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2.24</v>
+        <v>1.095</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>81.33</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S28" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-24.84</v>
+        <v>-7.76</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-15.71</v>
+        <v>-7.25</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>0.22</v>
+        <v>-0.13</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-1.54</v>
+        <v>1.67</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>0.4</v>
+        <v>36.5</v>
       </c>
       <c r="AA28" s="2" t="n">
         <v>33</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="n">
-        <v>7</v>
-      </c>
+      <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
@@ -3623,58 +3573,58 @@
         </is>
       </c>
       <c r="AG28" s="2" t="n">
-        <v>2.25</v>
+        <v>1.105</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>2.286</v>
+        <v>1.132</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>2.316</v>
+        <v>1.144</v>
       </c>
       <c r="AJ28" s="2" t="n">
-        <v>2.373</v>
+        <v>1.135</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>2.427</v>
+        <v>1.131</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>2.677</v>
+        <v>1.198</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>2.86</v>
+        <v>1.302</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>-0.869</v>
+        <v>-1.1674</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>-1.2034</v>
+        <v>-0.3251</v>
       </c>
       <c r="AP28" s="2" t="n">
-        <v>-0.313</v>
+        <v>0.106</v>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>-1.0341</v>
+        <v>-0.7602</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>-0.2484</v>
+        <v>-0.0776</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.897</v>
+        <v>1.057</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>3.17</v>
+        <v>-0.29</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -3684,43 +3634,39 @@
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S29" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T29" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-5.4</v>
+        <v>-10.61</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-6.12</v>
+        <v>-7.35</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>0.35</v>
+        <v>-2.64</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-0.68</v>
+        <v>-4.27</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>-3</v>
-      </c>
-      <c r="AA29" s="2" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="AA29" s="2" t="n">
+        <v>17</v>
+      </c>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr">
@@ -3729,58 +3675,58 @@
         </is>
       </c>
       <c r="AG29" s="2" t="n">
-        <v>0.908</v>
+        <v>1.087</v>
       </c>
       <c r="AH29" s="2" t="n">
-        <v>0.917</v>
+        <v>1.112</v>
       </c>
       <c r="AI29" s="2" t="n">
-        <v>0.926</v>
+        <v>1.124</v>
       </c>
       <c r="AJ29" s="2" t="n">
-        <v>0.9360000000000001</v>
+        <v>1.138</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>0.953</v>
+        <v>1.163</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>1.04</v>
+        <v>1.203</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>1.028</v>
+        <v>1.231</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-0.3268</v>
+        <v>-0.6256</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>-0.7282999999999999</v>
+        <v>-1.1093</v>
       </c>
       <c r="AP29" s="2" t="n">
-        <v>-0.4477</v>
+        <v>-0.4735</v>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>-0.4501</v>
+        <v>-0.6036</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>-0.054</v>
+        <v>-0.1061</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.616</v>
+        <v>0.916</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-4.94</v>
+        <v>79.97</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -3797,37 +3743,31 @@
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S30" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T30" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>22.33</v>
+        <v>37.48</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>6.42</v>
+        <v>9.02</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-5.08</v>
+        <v>-13.44</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-3.71</v>
+        <v>-9.1</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-3.9</v>
+        <v>17.4</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
@@ -3837,58 +3777,58 @@
         </is>
       </c>
       <c r="AG30" s="2" t="n">
-        <v>1.677</v>
+        <v>0.972</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>1.704</v>
+        <v>1.021</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>1.686</v>
+        <v>1.025</v>
       </c>
       <c r="AJ30" s="2" t="n">
-        <v>1.705</v>
+        <v>1.026</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>1.748</v>
+        <v>1.02</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>1.853</v>
+        <v>1.121</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>1.673</v>
+        <v>0.971</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>0.5054</v>
+        <v>-1.5137</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>-0.6065</v>
+        <v>-0.7768</v>
       </c>
       <c r="AP30" s="2" t="n">
-        <v>-0.7201</v>
+        <v>-0.5547</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>-0.08989999999999999</v>
+        <v>-0.2181</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>0.2233</v>
+        <v>0.3748</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.101</v>
+        <v>0.594</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>81.33</v>
+        <v>89.25</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -3910,67 +3850,69 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-6.02</v>
+        <v>34.83</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-7.77</v>
+        <v>7.28</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-1.52</v>
+        <v>-14.45</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>2.54</v>
+        <v>-7.69</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>38.4</v>
+        <v>21.9</v>
       </c>
       <c r="AA31" s="2" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG31" s="2" t="n">
-        <v>1.116</v>
+        <v>0.631</v>
       </c>
       <c r="AH31" s="2" t="n">
-        <v>1.138</v>
+        <v>0.667</v>
       </c>
       <c r="AI31" s="2" t="n">
-        <v>1.147</v>
+        <v>0.666</v>
       </c>
       <c r="AJ31" s="2" t="n">
-        <v>1.135</v>
+        <v>0.664</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>1.13</v>
+        <v>0.656</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>1.202</v>
+        <v>0.728</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>1.302</v>
+        <v>0.643</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>-1.0525</v>
+        <v>-1.4121</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>-0.1086</v>
+        <v>-0.6671</v>
       </c>
       <c r="AP31" s="2" t="n">
-        <v>0.1014</v>
+        <v>-0.3979</v>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>-0.7053</v>
+        <v>-0.3102</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>-0.0602</v>
+        <v>0.3483</v>
       </c>
     </row>
   </sheetData>
@@ -4001,7 +3943,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-30 | 30 只</t>
+          <t>截至: 2026-10-08 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-09
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -742,19 +742,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.403</v>
+        <v>3.064</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-1.36</v>
+        <v>6.32</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -764,103 +764,103 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="n">
-        <v>-1</v>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>-13.19</v>
+        <v>1.55</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-1.1</v>
+        <v>-3.43</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>0.87</v>
+        <v>-5.08</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>0.52</v>
+        <v>-4</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>58.5</v>
+        <v>-3.3</v>
       </c>
       <c r="AA2" s="2" t="n">
         <v>15</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>1.44</v>
+        <v>3.118</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>1.449</v>
+        <v>3.253</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>1.462</v>
+        <v>3.296</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>1.475</v>
+        <v>3.342</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>1.488</v>
+        <v>3.416</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>1.469</v>
+        <v>3.699</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>1.515</v>
+        <v>3.526</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-0.3257</v>
+        <v>-1.5056</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>-0.4861</v>
+        <v>-1.0693</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>-0.1366</v>
+        <v>-0.6732</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>-0.2006</v>
+        <v>-0.5555</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>-0.1319</v>
+        <v>0.0155</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.653</v>
+        <v>1.421</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-2.04</v>
+        <v>-2.87</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -871,37 +871,35 @@
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="n">
-        <v>-13</v>
+        <v>13</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-29.89</v>
+        <v>-13.59</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-4.75</v>
+        <v>0.06</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>4.47</v>
+        <v>0.71</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>5.07</v>
+        <v>1.85</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>65.09999999999999</v>
+        <v>55.9</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -913,78 +911,72 @@
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0.65</v>
+        <v>1.433</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>0.652</v>
+        <v>1.447</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>0.66</v>
+        <v>1.458</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>0.662</v>
+        <v>1.472</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>0.668</v>
+        <v>1.486</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>0.662</v>
+        <v>1.468</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>0.717</v>
+        <v>1.514</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>-0.2776</v>
+        <v>-0.3498</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>-0.3715</v>
+        <v>-0.5054</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>-0.1351</v>
+        <v>-0.1659</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>-0.3334</v>
+        <v>-0.2134</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>-0.2989</v>
+        <v>-0.1359</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.937</v>
+        <v>0.661</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>100.48</v>
+        <v>-2.04</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
@@ -995,33 +987,29 @@
       <c r="S4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T4" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>49.14</v>
+        <v>-28.48</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>43.92</v>
+        <v>-3.64</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>24.02</v>
+        <v>5.27</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>22.12</v>
+        <v>6.56</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>100.3</v>
+        <v>65.5</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
@@ -1029,103 +1017,113 @@
         </is>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>1.797</v>
+        <v>0.653</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>1.767</v>
+        <v>0.653</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>1.755</v>
+        <v>0.66</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>1.699</v>
+        <v>0.662</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>1.619</v>
+        <v>0.668</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>1.579</v>
+        <v>0.661</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>1.512</v>
+        <v>0.716</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.2157</v>
+        <v>-0.0159</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>1.4417</v>
+        <v>-0.3133</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>0.9384</v>
+        <v>-0.1196</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.204</v>
+        <v>-0.3042</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.4914</v>
+        <v>-0.2848</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.839</v>
+        <v>1.928</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4.26</v>
+        <v>95.31</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T5" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-3.21</v>
+        <v>52.63</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>6.96</v>
+        <v>42.73</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>1.39</v>
+        <v>15.72</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>6.43</v>
+        <v>22.81</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>57.2</v>
+        <v>101.4</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>48</v>
+        <v>89</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
         <is>
@@ -1133,166 +1131,162 @@
         </is>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>0.848</v>
+        <v>1.833</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>0.851</v>
+        <v>1.783</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>0.842</v>
+        <v>1.768</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>0.851</v>
+        <v>1.711</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>0.863</v>
+        <v>1.627</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>0.827</v>
+        <v>1.582</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>0.833</v>
+        <v>1.516</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.8633</v>
+        <v>0.7366</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>-0.1109</v>
+        <v>1.4851</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>-0.1682</v>
+        <v>1.0148</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.0315</v>
+        <v>0.2936</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>-0.0321</v>
+        <v>0.5263</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4.389</v>
+        <v>0.843</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4.59</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>4.98</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-3.27</v>
+        <v>-2.87</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.4</v>
+        <v>7.35</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>0.17</v>
+        <v>3.43</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>5.89</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>-2.9</v>
+        <v>56.6</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
-      <c r="AC6" s="2" t="n">
-        <v>8</v>
-      </c>
+      <c r="AC6" s="2" t="inlineStr"/>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>4.434</v>
+        <v>0.849</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>4.51</v>
+        <v>0.853</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>4.553</v>
+        <v>0.841</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>4.588</v>
+        <v>0.848</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>4.636</v>
+        <v>0.862</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>4.757</v>
+        <v>0.827</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>4.717</v>
+        <v>0.833</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>-0.7401</v>
+        <v>0.8178</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>-0.6705</v>
+        <v>-0.0309</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>-0.3068</v>
+        <v>-0.1276</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>-0.266</v>
+        <v>0.0378</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>-0.0327</v>
+        <v>-0.0287</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3.416</v>
+        <v>2.919</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>88.95</v>
+        <v>2.95</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -1301,9 +1295,7 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1311,200 +1303,208 @@
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="T7" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>10.83</v>
+        <v>-5.4</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>15.86</v>
+        <v>3.65</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>7.11</v>
+        <v>1.43</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>4.75</v>
+        <v>1.68</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>80.8</v>
+        <v>19.6</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="n">
-        <v>4</v>
-      </c>
+      <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>3.362</v>
+        <v>2.924</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>3.361</v>
+        <v>2.957</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>3.393</v>
+        <v>2.977</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>3.408</v>
+        <v>2.991</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>3.358</v>
+        <v>3.007</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>3.26</v>
+        <v>3.011</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>3.218</v>
+        <v>3.041</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>-0.366</v>
+        <v>-0.4073</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>-0.3854</v>
+        <v>-0.493</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>0.2569</v>
+        <v>-0.1957</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>0.06610000000000001</v>
+        <v>-0.1578</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>0.1083</v>
+        <v>-0.054</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.484</v>
+        <v>4.385</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>-0.8100000000000001</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+        <v>4.59</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="n">
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>-17.1</v>
+        <v>-4.23</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>-3.62</v>
+        <v>1.14</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-0.18</v>
+        <v>-0.19</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.1</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>16.6</v>
+        <v>-2.8</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
-      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
       <c r="AF8" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG8" s="2" t="n">
-        <v>0.492</v>
+        <v>4.408</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>0.499</v>
+        <v>4.495</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>0.507</v>
+        <v>4.541</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>0.511</v>
+        <v>4.579</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>0.517</v>
+        <v>4.628</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>0.517</v>
+        <v>4.751</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>0.532</v>
+        <v>4.716</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-0.7796</v>
+        <v>-0.7939000000000001</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>-0.9068000000000001</v>
+        <v>-0.7057</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>-0.3975</v>
+        <v>-0.3438</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>-0.1556</v>
+        <v>-0.2944</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>-0.171</v>
+        <v>-0.0423</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.382</v>
+        <v>7.282</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>9.880000000000001</v>
+        <v>14.72</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1516,105 +1516,101 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
+          <t>预1</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr"/>
-      <c r="T9" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="U9" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="T9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>-3.15</v>
+        <v>6.45</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>8.779999999999999</v>
+        <v>0.65</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>4.7</v>
+        <v>-2.35</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>8.43</v>
+        <v>-2.12</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>65.5</v>
+        <v>11</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
-      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>0.379</v>
+        <v>7.389</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>0.38</v>
+        <v>7.596</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>0.376</v>
+        <v>7.645</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>0.379</v>
+        <v>7.709</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>0.382</v>
+        <v>7.743</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>0.364</v>
+        <v>8.064</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>0.371</v>
+        <v>8.013</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>0.747</v>
+        <v>-0.8337</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>-0.0141</v>
+        <v>-0.7877</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>0.0741</v>
+        <v>-0.1673</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>0.0769</v>
+        <v>-0.4214</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>-0.0315</v>
+        <v>0.0645</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2.904</v>
+        <v>3.431</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>77.83</v>
+        <v>41.01</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1623,10 +1619,10 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L10" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
         <v>0</v>
       </c>
@@ -1635,88 +1631,92 @@
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>2.3</v>
+        <v>11.7</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-0.5</v>
+        <v>16.11</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-3.43</v>
+        <v>5.27</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>-0.74</v>
+        <v>4.86</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>32.2</v>
+        <v>81.5</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>2.98</v>
+        <v>3.376</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.054</v>
+        <v>3.369</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>3.06</v>
+        <v>3.393</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>3.071</v>
+        <v>3.409</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>3.047</v>
+        <v>3.361</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>3.214</v>
+        <v>3.261</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>3.216</v>
+        <v>3.219</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>-0.5606</v>
+        <v>-0.0578</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>-0.5973000000000001</v>
+        <v>-0.3158</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>0.089</v>
+        <v>0.238</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>-0.4208</v>
+        <v>0.0934</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>0.023</v>
+        <v>0.117</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.339</v>
+        <v>0.495</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>40.85</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1725,39 +1725,39 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S11" s="2" t="inlineStr"/>
-      <c r="T11" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-18.23</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>7.07</v>
+        <v>-1.53</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>2.07</v>
+        <v>1.88</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>7.16</v>
+        <v>0.88</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>74</v>
+        <v>14.8</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1765,62 +1765,62 @@
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG11" s="2" t="n">
-        <v>0.342</v>
+        <v>0.49</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>0.343</v>
+        <v>0.499</v>
       </c>
       <c r="AI11" s="2" t="n">
-        <v>0.339</v>
+        <v>0.506</v>
       </c>
       <c r="AJ11" s="2" t="n">
-        <v>0.341</v>
+        <v>0.511</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>0.34</v>
+        <v>0.516</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>0.326</v>
+        <v>0.516</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>0.336</v>
+        <v>0.532</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>0.7194</v>
+        <v>-0.6179</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>0.0172</v>
+        <v>-0.9244</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>0.2337</v>
+        <v>-0.424</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>0.0338</v>
+        <v>-0.1617</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>-0.0069</v>
+        <v>-0.1823</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.417</v>
+        <v>0.38</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-1.36</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1838,30 +1838,30 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-43.76</v>
+        <v>-2.65</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-9.109999999999999</v>
+        <v>8.08</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>5.25</v>
+        <v>4.63</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>6.42</v>
+        <v>7.21</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>50.4</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1873,58 +1873,58 @@
         </is>
       </c>
       <c r="AG12" s="2" t="n">
-        <v>0.411</v>
+        <v>0.381</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>0.412</v>
+        <v>0.38</v>
       </c>
       <c r="AI12" s="2" t="n">
-        <v>0.416</v>
+        <v>0.377</v>
       </c>
       <c r="AJ12" s="2" t="n">
-        <v>0.418</v>
+        <v>0.378</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>0.426</v>
+        <v>0.382</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>0.424</v>
+        <v>0.364</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>0.472</v>
+        <v>0.371</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>-0.0898</v>
+        <v>0.7743</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>-0.3837</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>-0.1625</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>-0.3919</v>
+        <v>0.0813</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>-0.4376</v>
+        <v>-0.0265</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.971</v>
+        <v>0.764</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>-3.59</v>
+        <v>-4.85</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1936,101 +1936,97 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T13" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>32.13</v>
+        <v>-16.83</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>7.5</v>
+        <v>-1.28</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-10.32</v>
+        <v>1.95</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>-8.16</v>
+        <v>-0.31</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>-4.9</v>
+        <v>28.5</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
-      <c r="AC13" s="2" t="n">
-        <v>10</v>
-      </c>
+      <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG13" s="2" t="n">
-        <v>1.029</v>
+        <v>0.759</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>1.062</v>
+        <v>0.771</v>
       </c>
       <c r="AI13" s="2" t="n">
-        <v>1.052</v>
+        <v>0.783</v>
       </c>
       <c r="AJ13" s="2" t="n">
-        <v>1.065</v>
+        <v>0.789</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>1.093</v>
+        <v>0.792</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>1.179</v>
+        <v>0.786</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>1.026</v>
+        <v>0.826</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>-0.063</v>
+        <v>-0.7279</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>-0.8867</v>
+        <v>-0.8443000000000001</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>-0.8214</v>
+        <v>-0.3374</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>-0.07389999999999999</v>
+        <v>-0.1842</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>0.3213</v>
+        <v>-0.1683</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.859</v>
+        <v>2.909</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>99.92</v>
+        <v>77.83</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -2040,105 +2036,103 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N14" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T14" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>15.73</v>
+        <v>-0.49</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>8.51</v>
+        <v>-2.96</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>7.96</v>
+        <v>-0.89</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>96.5</v>
+        <v>30.1</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>84</v>
+        <v>19</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
-      <c r="AD14" s="2" t="n">
-        <v>11</v>
-      </c>
+      <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG14" s="2" t="n">
-        <v>0.845</v>
+        <v>2.946</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>0.841</v>
+        <v>3.038</v>
       </c>
       <c r="AI14" s="2" t="n">
-        <v>0.843</v>
+        <v>3.051</v>
       </c>
       <c r="AJ14" s="2" t="n">
-        <v>0.837</v>
+        <v>3.065</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>0.826</v>
+        <v>3.047</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>0.801</v>
+        <v>3.207</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>0.798</v>
+        <v>3.215</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>-0.068</v>
+        <v>-0.8184</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>0.2233</v>
+        <v>-0.6972</v>
       </c>
       <c r="AP14" s="2" t="n">
-        <v>0.3283</v>
+        <v>0.09180000000000001</v>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>0.1977</v>
+        <v>-0.4747</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>0.017</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.981</v>
+        <v>0.341</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>-8.65</v>
+        <v>52.3</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -2147,43 +2141,41 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="n">
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="n">
         <v>-1</v>
-      </c>
-      <c r="T15" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-55.92</v>
+        <v>-0.47</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-18.7</v>
+        <v>7.66</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>0.6</v>
+        <v>3.19</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>1.54</v>
+        <v>7.48</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>28.4</v>
+        <v>73.8</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
@@ -2195,58 +2187,58 @@
         </is>
       </c>
       <c r="AG15" s="2" t="n">
-        <v>1.007</v>
+        <v>0.342</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>1.016</v>
+        <v>0.343</v>
       </c>
       <c r="AI15" s="2" t="n">
-        <v>1.022</v>
+        <v>0.339</v>
       </c>
       <c r="AJ15" s="2" t="n">
-        <v>1.043</v>
+        <v>0.34</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>1.079</v>
+        <v>0.34</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>1.085</v>
+        <v>0.325</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>1.222</v>
+        <v>0.336</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>-0.1937</v>
+        <v>0.6587</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>-0.779</v>
+        <v>0.0713</v>
       </c>
       <c r="AP15" s="2" t="n">
-        <v>-0.5306</v>
+        <v>0.2583</v>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>-0.5001</v>
+        <v>0.0323</v>
       </c>
       <c r="AR15" s="2" t="n">
-        <v>-0.5592</v>
+        <v>-0.0047</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.721</v>
+        <v>1.082</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>-4.21</v>
+        <v>81.33</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -2256,36 +2248,38 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-19.2</v>
+        <v>-9.34</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-4.37</v>
+        <v>-8.48</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>0.01</v>
+        <v>-1.28</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>0.24</v>
+        <v>0.63</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>27.9</v>
+        <v>34.2</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
@@ -2293,62 +2287,62 @@
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>1.754</v>
+        <v>1.096</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>1.777</v>
+        <v>1.126</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>1.809</v>
+        <v>1.141</v>
       </c>
       <c r="AJ16" s="2" t="n">
-        <v>1.828</v>
+        <v>1.134</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>1.832</v>
+        <v>1.13</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>1.816</v>
+        <v>1.194</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>1.884</v>
+        <v>1.301</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>-0.8405</v>
+        <v>-1.2132</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.474</v>
       </c>
       <c r="AP16" s="2" t="n">
-        <v>-0.2441</v>
+        <v>0.08019999999999999</v>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>-0.1704</v>
+        <v>-0.8071</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>-0.192</v>
+        <v>-0.0934</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>2.374</v>
+        <v>0.419</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>109.67</v>
+        <v>-1.36</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -2357,43 +2351,41 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="n">
-        <v>-13</v>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>24.4</v>
+        <v>-41.83</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>28.57</v>
+        <v>-8.720000000000001</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>7.1</v>
+        <v>5.48</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>13.27</v>
+        <v>7.12</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>72.09999999999999</v>
+        <v>51.3</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
@@ -2405,107 +2397,103 @@
         </is>
       </c>
       <c r="AG17" s="2" t="n">
-        <v>2.333</v>
+        <v>0.413</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>2.309</v>
+        <v>0.413</v>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>2.262</v>
+        <v>0.416</v>
       </c>
       <c r="AJ17" s="2" t="n">
-        <v>2.244</v>
+        <v>0.418</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>2.219</v>
+        <v>0.426</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>2.2</v>
+        <v>0.424</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>2.03</v>
+        <v>0.472</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>1.4853</v>
+        <v>0.1753</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>0.6415</v>
+        <v>-0.3167</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>0.4901</v>
+        <v>-0.148</v>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>0.3206</v>
+        <v>-0.361</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>0.244</v>
+        <v>-0.4183</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.448</v>
+        <v>1.07</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>6.69</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>-0.29</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-23.49</v>
+        <v>-11.51</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-13.3</v>
+        <v>-6.34</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>0.93</v>
+        <v>-1.55</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-1.48</v>
+        <v>-3.34</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>1.6</v>
+        <v>2.9</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
@@ -2515,58 +2503,58 @@
         </is>
       </c>
       <c r="AG18" s="2" t="n">
-        <v>1.451</v>
+        <v>1.077</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>1.476</v>
+        <v>1.108</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>1.501</v>
+        <v>1.119</v>
       </c>
       <c r="AJ18" s="2" t="n">
-        <v>1.539</v>
+        <v>1.135</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>1.579</v>
+        <v>1.16</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>1.719</v>
+        <v>1.199</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>1.809</v>
+        <v>1.231</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-0.7841</v>
+        <v>-0.7941</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>-1.3172</v>
+        <v>-1.2317</v>
       </c>
       <c r="AP18" s="2" t="n">
-        <v>-0.3585</v>
+        <v>-0.5178</v>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>-1.0389</v>
+        <v>-0.6496</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>-0.2349</v>
+        <v>-0.1151</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.279</v>
+        <v>0.97</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>81.22</v>
+        <v>14.64</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -2576,120 +2564,112 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr"/>
-      <c r="S19" s="2" t="inlineStr">
+      <c r="R19" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>18.09</v>
+        <v>28.83</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>16.92</v>
+        <v>7.09</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>6.27</v>
+        <v>-9.9</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>2.09</v>
+        <v>-7.53</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>65.59999999999999</v>
+        <v>-5</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
-      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG19" s="2" t="n">
-        <v>1.262</v>
+        <v>1.006</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>1.265</v>
+        <v>1.054</v>
       </c>
       <c r="AI19" s="2" t="n">
-        <v>1.28</v>
+        <v>1.047</v>
       </c>
       <c r="AJ19" s="2" t="n">
-        <v>1.292</v>
+        <v>1.061</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>1.264</v>
+        <v>1.088</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>1.239</v>
+        <v>1.178</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>1.202</v>
+        <v>1.027</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>-0.472</v>
+        <v>-0.7294</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>-0.8077</v>
+        <v>-1.0226</v>
       </c>
       <c r="AP19" s="2" t="n">
-        <v>0.3182</v>
+        <v>-0.8897</v>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>-0.0025</v>
+        <v>-0.161</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>0.1809</v>
+        <v>0.2883</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.763</v>
+        <v>0.85</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>7.96</v>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>85.37</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
@@ -2699,121 +2679,109 @@
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-22.39</v>
+        <v>2.54</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-15.89</v>
+        <v>14.28</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-1.35</v>
+        <v>4.38</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-0.21</v>
+        <v>7.1</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>4.6</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG20" s="2" t="n">
-        <v>0.775</v>
+        <v>0.848</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>0.793</v>
+        <v>0.842</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>0.799</v>
+        <v>0.843</v>
       </c>
       <c r="AJ20" s="2" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.838</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>0.826</v>
+        <v>0.827</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>0.914</v>
+        <v>0.801</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>0.989</v>
+        <v>0.798</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>-0.6793</v>
+        <v>0.099</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>-0.9237</v>
+        <v>0.192</v>
       </c>
       <c r="AP20" s="2" t="n">
-        <v>-0.2119</v>
+        <v>0.3152</v>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>-0.9242</v>
+        <v>0.2099</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>-0.2239</v>
+        <v>0.0254</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.234</v>
+        <v>1.002</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>-8.65</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M21" s="2" t="n">
         <v>13</v>
       </c>
@@ -2823,200 +2791,202 @@
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr"/>
-      <c r="S21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-25.3</v>
+        <v>-56.38</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-15.01</v>
+        <v>-16.93</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>0.98</v>
+        <v>1.21</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-0.16</v>
+        <v>4.41</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>0.1</v>
+        <v>27.2</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
-      <c r="AC21" s="2" t="n">
-        <v>8</v>
-      </c>
+      <c r="AC21" s="2" t="inlineStr"/>
       <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="inlineStr"/>
       <c r="AF21" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG21" s="2" t="n">
-        <v>2.234</v>
+        <v>1.003</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>2.279</v>
+        <v>1.016</v>
       </c>
       <c r="AI21" s="2" t="n">
-        <v>2.31</v>
+        <v>1.021</v>
       </c>
       <c r="AJ21" s="2" t="n">
-        <v>2.364</v>
+        <v>1.038</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>2.424</v>
+        <v>1.077</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>2.667</v>
+        <v>1.083</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>2.857</v>
+        <v>1.219</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>-0.9287</v>
+        <v>-0.2748</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>-1.151</v>
+        <v>-0.7258</v>
       </c>
       <c r="AP21" s="2" t="n">
-        <v>-0.3051</v>
+        <v>-0.506</v>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>-1.0557</v>
+        <v>-0.5147</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>-0.253</v>
+        <v>-0.5638</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.862</v>
+        <v>1.732</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>-5.36</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="n">
         <v>13</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-7.63</v>
+        <v>-20.66</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-8.73</v>
+        <v>-3.82</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-2.36</v>
+        <v>0.43</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-2.96</v>
+        <v>-0.22</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>-3.8</v>
-      </c>
-      <c r="AA22" s="2" t="inlineStr"/>
+        <v>24</v>
+      </c>
+      <c r="AA22" s="2" t="n">
+        <v>32</v>
+      </c>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG22" s="2" t="n">
-        <v>0.895</v>
+        <v>1.744</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>0.912</v>
+        <v>1.773</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>0.922</v>
+        <v>1.802</v>
       </c>
       <c r="AJ22" s="2" t="n">
-        <v>0.9320000000000001</v>
+        <v>1.825</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>0.951</v>
+        <v>1.828</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>1.037</v>
+        <v>1.815</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>1.028</v>
+        <v>1.883</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>-0.536</v>
+        <v>-0.7599</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>-0.9147</v>
+        <v>-1.0073</v>
       </c>
       <c r="AP22" s="2" t="n">
-        <v>-0.4293</v>
+        <v>-0.2969</v>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>-0.5324</v>
+        <v>-0.1816</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>-0.07630000000000001</v>
+        <v>-0.2066</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.537</v>
+        <v>2.398</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>-4.94</v>
+        <v>110.91</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -3025,8 +2995,12 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
       </c>
@@ -3034,195 +3008,207 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>18.89</v>
+        <v>25.28</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>2.28</v>
+        <v>29.45</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-9.58</v>
+        <v>7.16</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-7.21</v>
+        <v>14.31</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>-4.9</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>12</v>
+        <v>87</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>1.633</v>
+        <v>2.35</v>
       </c>
       <c r="AH23" s="2" t="n">
-        <v>1.687</v>
+        <v>2.326</v>
       </c>
       <c r="AI23" s="2" t="n">
-        <v>1.678</v>
+        <v>2.272</v>
       </c>
       <c r="AJ23" s="2" t="n">
-        <v>1.697</v>
+        <v>2.25</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>1.739</v>
+        <v>2.225</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>1.85</v>
+        <v>2.203</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>1.674</v>
+        <v>2.033</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>-0.279</v>
+        <v>1.6757</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>-0.918</v>
+        <v>0.7786999999999999</v>
       </c>
       <c r="AP23" s="2" t="n">
-        <v>-0.8077</v>
+        <v>0.5471</v>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>-0.1962</v>
+        <v>0.3209</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>0.1889</v>
+        <v>0.2528</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>3.053</v>
+        <v>1.475</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>6.32</v>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+        <v>6.69</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N24" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>4.1</v>
+        <v>-23.54</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-3.61</v>
+        <v>-11.79</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-6.18</v>
+        <v>2.76</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-4.5</v>
+        <v>-0.83</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>-3.1</v>
+        <v>1.9</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="AB24" s="2" t="inlineStr"/>
+        <v>59</v>
+      </c>
+      <c r="AB24" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="AC24" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>3.168</v>
+        <v>1.451</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>3.279</v>
+        <v>1.475</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>3.309</v>
+        <v>1.496</v>
       </c>
       <c r="AJ24" s="2" t="n">
-        <v>3.357</v>
+        <v>1.535</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>3.426</v>
+        <v>1.576</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>3.709</v>
+        <v>1.713</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>3.526</v>
+        <v>1.808</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>-1.1796</v>
+        <v>-0.6474</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>-1.0017</v>
+        <v>-1.2172</v>
       </c>
       <c r="AP24" s="2" t="n">
-        <v>-0.635</v>
+        <v>-0.3617</v>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>-0.4839</v>
+        <v>-1.0128</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>0.041</v>
+        <v>-0.2354</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2.918</v>
+        <v>0.905</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>2.95</v>
+        <v>79.97</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -3239,30 +3225,36 @@
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>-4.84</v>
+        <v>32.89</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>3.8</v>
+        <v>7.41</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>1.98</v>
+        <v>-13.26</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>1.94</v>
+        <v>-9.779999999999999</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>22.3</v>
+        <v>15</v>
       </c>
       <c r="AA25" s="2" t="n">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
@@ -3271,58 +3263,58 @@
         </is>
       </c>
       <c r="AG25" s="2" t="n">
-        <v>2.932</v>
+        <v>0.946</v>
       </c>
       <c r="AH25" s="2" t="n">
-        <v>2.961</v>
+        <v>1.007</v>
       </c>
       <c r="AI25" s="2" t="n">
-        <v>2.982</v>
+        <v>1.02</v>
       </c>
       <c r="AJ25" s="2" t="n">
-        <v>2.993</v>
+        <v>1.022</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>3.01</v>
+        <v>1.017</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>3.013</v>
+        <v>1.119</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>3.041</v>
+        <v>0.972</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>-0.4378</v>
+        <v>-2.1729</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>-0.4655</v>
+        <v>-0.9947</v>
       </c>
       <c r="AP25" s="2" t="n">
-        <v>-0.1542</v>
+        <v>-0.5753</v>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>-0.1469</v>
+        <v>-0.346</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>-0.0484</v>
+        <v>0.3289</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>7.279</v>
+        <v>1.298</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>52.12</v>
+        <v>55.37</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -3332,7 +3324,9 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
       </c>
@@ -3340,191 +3334,209 @@
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>7.88</v>
+        <v>19.32</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>0.8</v>
+        <v>18.37</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-2.68</v>
+        <v>5.52</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-1.72</v>
+        <v>3.99</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>12.5</v>
+        <v>67</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>16</v>
+        <v>77</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="n">
-        <v>8</v>
-      </c>
+      <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>7.462</v>
+        <v>1.268</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>7.636</v>
+        <v>1.269</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>7.67</v>
+        <v>1.279</v>
       </c>
       <c r="AJ26" s="2" t="n">
-        <v>7.729</v>
+        <v>1.293</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>7.752</v>
+        <v>1.265</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>8.08</v>
+        <v>1.239</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>8.012</v>
+        <v>1.203</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>-0.627</v>
+        <v>-0.0927</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>-0.7281</v>
+        <v>-0.6633</v>
       </c>
       <c r="AP26" s="2" t="n">
-        <v>-0.1475</v>
+        <v>0.2788</v>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>-0.3755</v>
+        <v>0.0505</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>0.0788</v>
+        <v>0.1932</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.752</v>
+        <v>0.765</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>-4.85</v>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
+        <v>7.96</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-15.29</v>
+        <v>-23.3</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-2.73</v>
+        <v>-15.77</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>0.48</v>
+        <v>-0.41</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-0.18</v>
+        <v>0.09</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>31.8</v>
+        <v>4.4</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG27" s="2" t="n">
-        <v>0.761</v>
+        <v>0.769</v>
       </c>
       <c r="AH27" s="2" t="n">
-        <v>0.772</v>
+        <v>0.79</v>
       </c>
       <c r="AI27" s="2" t="n">
-        <v>0.786</v>
+        <v>0.797</v>
       </c>
       <c r="AJ27" s="2" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>0.794</v>
+        <v>0.825</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>0.787</v>
+        <v>0.91</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>0.827</v>
+        <v>0.988</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>-0.8985</v>
+        <v>-0.7584</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>-0.7939000000000001</v>
+        <v>-0.8979</v>
       </c>
       <c r="AP27" s="2" t="n">
-        <v>-0.2915</v>
+        <v>-0.2623</v>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>-0.1857</v>
+        <v>-0.9759</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>-0.1529</v>
+        <v>-0.233</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.095</v>
+        <v>0.592</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>81.33</v>
+        <v>89.25</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -3534,138 +3546,176 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N28" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-7.76</v>
+        <v>29.94</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-7.25</v>
+        <v>6.61</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-0.13</v>
+        <v>-13.15</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>1.67</v>
+        <v>-7.67</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>36.5</v>
+        <v>19.7</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG28" s="2" t="n">
-        <v>1.105</v>
+        <v>0.614</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>1.132</v>
+        <v>0.657</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>1.144</v>
+        <v>0.663</v>
       </c>
       <c r="AJ28" s="2" t="n">
-        <v>1.135</v>
+        <v>0.662</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>1.131</v>
+        <v>0.655</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>1.198</v>
+        <v>0.726</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>1.302</v>
+        <v>0.643</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>-1.1674</v>
+        <v>-2.1839</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>-0.3251</v>
+        <v>-0.8791</v>
       </c>
       <c r="AP28" s="2" t="n">
-        <v>0.106</v>
+        <v>-0.4395</v>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>-0.7602</v>
+        <v>-0.4448</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>-0.0776</v>
+        <v>0.2994</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.057</v>
+        <v>2.249</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>-0.29</v>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
+        <v>3.12</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
-      <c r="S29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-10.61</v>
+        <v>-25.56</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-7.35</v>
+        <v>-14.5</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-2.64</v>
+        <v>1.89</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-4.27</v>
+        <v>0.21</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>2.5</v>
+        <v>0.1</v>
       </c>
       <c r="AA29" s="2" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
@@ -3675,58 +3725,58 @@
         </is>
       </c>
       <c r="AG29" s="2" t="n">
-        <v>1.087</v>
+        <v>2.23</v>
       </c>
       <c r="AH29" s="2" t="n">
-        <v>1.112</v>
+        <v>2.273</v>
       </c>
       <c r="AI29" s="2" t="n">
-        <v>1.124</v>
+        <v>2.303</v>
       </c>
       <c r="AJ29" s="2" t="n">
-        <v>1.138</v>
+        <v>2.355</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>1.163</v>
+        <v>2.418</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>1.203</v>
+        <v>2.655</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>1.231</v>
+        <v>2.853</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-0.6256</v>
+        <v>-0.8519</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>-1.1093</v>
+        <v>-1.042</v>
       </c>
       <c r="AP29" s="2" t="n">
-        <v>-0.4735</v>
+        <v>-0.3373</v>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>-0.6036</v>
+        <v>-1.0526</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>-0.1061</v>
+        <v>-0.2556</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.916</v>
+        <v>0.863</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>79.97</v>
+        <v>7.5</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -3736,99 +3786,101 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N30" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>37.48</v>
+        <v>-9.57</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>9.02</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-13.44</v>
+        <v>-3</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-9.1</v>
+        <v>-3.58</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="AA30" s="2" t="n">
-        <v>12</v>
-      </c>
+        <v>-3.5</v>
+      </c>
+      <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="n">
-        <v>10</v>
-      </c>
+      <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG30" s="2" t="n">
-        <v>0.972</v>
+        <v>0.883</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>1.021</v>
+        <v>0.907</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>1.025</v>
+        <v>0.917</v>
       </c>
       <c r="AJ30" s="2" t="n">
-        <v>1.026</v>
+        <v>0.929</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>1.02</v>
+        <v>0.95</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>1.121</v>
+        <v>1.034</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>0.971</v>
+        <v>1.027</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>-1.5137</v>
+        <v>-0.7961</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>-0.7768</v>
+        <v>-1.0419</v>
       </c>
       <c r="AP30" s="2" t="n">
-        <v>-0.5547</v>
+        <v>-0.4096</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>-0.2181</v>
+        <v>-0.6106</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>0.3748</v>
+        <v>-0.09569999999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.594</v>
+        <v>1.541</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>89.25</v>
+        <v>12.87</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -3840,29 +3892,35 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
-      <c r="S31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>34.83</v>
+        <v>15.95</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>7.28</v>
+        <v>2.33</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-14.45</v>
+        <v>-8.66</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-7.69</v>
+        <v>-6.61</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>21.9</v>
+        <v>-4.9</v>
       </c>
       <c r="AA31" s="2" t="n">
         <v>12</v>
@@ -3879,40 +3937,40 @@
         </is>
       </c>
       <c r="AG31" s="2" t="n">
-        <v>0.631</v>
+        <v>1.599</v>
       </c>
       <c r="AH31" s="2" t="n">
-        <v>0.667</v>
+        <v>1.671</v>
       </c>
       <c r="AI31" s="2" t="n">
-        <v>0.666</v>
+        <v>1.67</v>
       </c>
       <c r="AJ31" s="2" t="n">
-        <v>0.664</v>
+        <v>1.69</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>0.656</v>
+        <v>1.732</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>0.728</v>
+        <v>1.847</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>0.643</v>
+        <v>1.674</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>-1.4121</v>
+        <v>-0.9169</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>-0.6671</v>
+        <v>-1.0528</v>
       </c>
       <c r="AP31" s="2" t="n">
-        <v>-0.3979</v>
+        <v>-0.8777</v>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>-0.3102</v>
+        <v>-0.2783</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>0.3483</v>
+        <v>0.1595</v>
       </c>
     </row>
   </sheetData>
@@ -3943,7 +4001,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-08 | 30 只</t>
+          <t>截至: 2026-10-09 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-12
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -742,19 +742,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.064</v>
+        <v>1.426</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>6.32</v>
+        <v>-2.87</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -764,9 +764,11 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
@@ -780,27 +782,25 @@
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>1.55</v>
+        <v>-13.46</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-3.43</v>
+        <v>1.18</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-5.08</v>
+        <v>-0.38</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-4</v>
+        <v>0.95</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>-3.3</v>
+        <v>53.9</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="n">
-        <v>8</v>
-      </c>
+      <c r="AC2" s="2" t="inlineStr"/>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr">
@@ -809,58 +809,58 @@
         </is>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>3.118</v>
+        <v>1.427</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>3.253</v>
+        <v>1.443</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>3.296</v>
+        <v>1.454</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>3.342</v>
+        <v>1.468</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>3.416</v>
+        <v>1.484</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>3.699</v>
+        <v>1.466</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>3.526</v>
+        <v>1.513</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-1.5056</v>
+        <v>-0.4246</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>-1.0693</v>
+        <v>-0.5635</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>-0.6732</v>
+        <v>-0.1951</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>-0.5555</v>
+        <v>-0.2166</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.0155</v>
+        <v>-0.1346</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.421</v>
+        <v>0.666</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-2.87</v>
+        <v>-2.04</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -871,35 +871,39 @@
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="n">
-        <v>13</v>
+        <v>-13</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-13.59</v>
+        <v>-26.75</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>0.06</v>
+        <v>-2.16</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>0.71</v>
+        <v>4.72</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>1.85</v>
+        <v>4.87</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>55.9</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
@@ -911,78 +915,86 @@
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>1.433</v>
+        <v>0.657</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>1.447</v>
+        <v>0.655</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>1.458</v>
+        <v>0.659</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>1.472</v>
+        <v>0.662</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>1.486</v>
+        <v>0.668</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>1.468</v>
+        <v>0.661</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>1.514</v>
+        <v>0.716</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>-0.3498</v>
+        <v>0.1993</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>-0.5054</v>
+        <v>-0.2943</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>-0.1659</v>
+        <v>-0.0917</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>-0.2134</v>
+        <v>-0.2733</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>-0.1359</v>
+        <v>-0.2675</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.661</v>
+        <v>1.874</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-2.04</v>
+        <v>95.31</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="L4" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="n">
-        <v>1</v>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S4" s="2" t="n">
         <v>1</v>
@@ -990,26 +1002,28 @@
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-28.48</v>
+        <v>55.36</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-3.64</v>
+        <v>39.41</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>5.27</v>
+        <v>9.57</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>6.56</v>
+        <v>18.89</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>65.5</v>
+        <v>101</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
@@ -1017,113 +1031,105 @@
         </is>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>0.653</v>
+        <v>1.858</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.653</v>
+        <v>1.796</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>0.66</v>
+        <v>1.778</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>0.662</v>
+        <v>1.721</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>0.668</v>
+        <v>1.634</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>0.661</v>
+        <v>1.584</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>0.716</v>
+        <v>1.519</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>-0.0159</v>
+        <v>1.1513</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>-0.3133</v>
+        <v>1.4795</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>-0.1196</v>
+        <v>1.0568</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>-0.3042</v>
+        <v>0.3456</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>-0.2848</v>
+        <v>0.5536</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.928</v>
+        <v>0.83</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>95.31</v>
+        <v>4.98</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T5" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R5" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>52.63</v>
+        <v>-3.43</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>42.73</v>
+        <v>6.47</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>15.72</v>
+        <v>-0.35</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>22.81</v>
+        <v>5.56</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>101.4</v>
+        <v>55.2</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="inlineStr">
         <is>
@@ -1131,58 +1137,58 @@
         </is>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>1.833</v>
+        <v>0.846</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>1.783</v>
+        <v>0.852</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>1.768</v>
+        <v>0.841</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>1.711</v>
+        <v>0.846</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>1.627</v>
+        <v>0.862</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>1.582</v>
+        <v>0.827</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>1.516</v>
+        <v>0.832</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.7366</v>
+        <v>0.524</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>1.4851</v>
+        <v>-0.0247</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>1.0148</v>
+        <v>-0.1408</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.2936</v>
+        <v>0.0522</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.5263</v>
+        <v>-0.0343</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.843</v>
+        <v>2.932</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4.98</v>
+        <v>2.95</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -1194,36 +1200,36 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="n">
-        <v>-1</v>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-2.87</v>
+        <v>-5.49</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>7.35</v>
+        <v>4.81</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>3.43</v>
+        <v>1.6</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>5.89</v>
+        <v>2.52</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>56.6</v>
+        <v>18.1</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
@@ -1231,280 +1237,278 @@
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>0.849</v>
+        <v>2.926</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>0.853</v>
+        <v>2.953</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>0.841</v>
+        <v>2.971</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>0.848</v>
+        <v>2.989</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>0.862</v>
+        <v>3.004</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>0.827</v>
+        <v>3.01</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>0.833</v>
+        <v>3.04</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.8178</v>
+        <v>-0.3792</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>-0.0309</v>
+        <v>-0.485</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>-0.1276</v>
+        <v>-0.2333</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.0378</v>
+        <v>-0.1511</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>-0.0287</v>
+        <v>-0.0549</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.919</v>
+        <v>4.36</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+        <v>4.59</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R7" s="2" t="inlineStr"/>
       <c r="S7" s="2" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-5.4</v>
+        <v>-4.77</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>3.65</v>
+        <v>1.25</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>1.43</v>
+        <v>-0.11</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>1.68</v>
+        <v>0.03</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>19.6</v>
+        <v>-3.1</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>2.924</v>
+        <v>4.396</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>2.957</v>
+        <v>4.472</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>2.977</v>
+        <v>4.527</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>2.991</v>
+        <v>4.568</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>3.007</v>
+        <v>4.62</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>3.011</v>
+        <v>4.744</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>3.041</v>
+        <v>4.714</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>-0.4073</v>
+        <v>-0.8653</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>-0.493</v>
+        <v>-0.7040999999999999</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>-0.1957</v>
+        <v>-0.3818</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>-0.1578</v>
+        <v>-0.3041</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>-0.054</v>
+        <v>-0.0477</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.385</v>
+        <v>3.447</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>4.59</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>41.01</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>-4.23</v>
+        <v>13.05</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.14</v>
+        <v>17.35</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-0.19</v>
+        <v>4.56</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-0.1</v>
+        <v>5.95</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>-2.8</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>19</v>
+        <v>82</v>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
-      <c r="AC8" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="AE8" s="2" t="inlineStr"/>
       <c r="AF8" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG8" s="2" t="n">
-        <v>4.408</v>
+        <v>3.397</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>4.495</v>
+        <v>3.38</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>4.541</v>
+        <v>3.393</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>4.579</v>
+        <v>3.411</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>4.628</v>
+        <v>3.366</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>4.751</v>
+        <v>3.264</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>4.716</v>
+        <v>3.221</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-0.7939000000000001</v>
+        <v>0.2283</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>-0.7057</v>
+        <v>-0.2183</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>-0.3438</v>
+        <v>0.2432</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>-0.2944</v>
+        <v>0.1181</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>-0.0423</v>
+        <v>0.1305</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.282</v>
+        <v>0.495</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>14.72</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1513,43 +1517,47 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R9" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>6.45</v>
+        <v>-18.68</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>0.65</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-2.35</v>
+        <v>2.51</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-2.12</v>
+        <v>1.05</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>11</v>
+        <v>13.3</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="AB9" s="2" t="inlineStr"/>
+        <v>54</v>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="AC9" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
@@ -1559,58 +1567,58 @@
         </is>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>7.389</v>
+        <v>0.491</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>7.596</v>
+        <v>0.498</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>7.645</v>
+        <v>0.504</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>7.709</v>
+        <v>0.51</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>7.743</v>
+        <v>0.515</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>8.064</v>
+        <v>0.516</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>8.013</v>
+        <v>0.531</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>-0.8337</v>
+        <v>-0.5579</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>-0.7877</v>
+        <v>-0.9025</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>-0.1673</v>
+        <v>-0.4185</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>-0.4214</v>
+        <v>-0.1477</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>0.0645</v>
+        <v>-0.1868</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.431</v>
+        <v>0.379</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>41.01</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1619,45 +1627,47 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>11.7</v>
+        <v>-2.65</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>16.11</v>
+        <v>8.58</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>5.27</v>
+        <v>2.44</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>4.86</v>
+        <v>7.27</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>81.5</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr">
         <is>
@@ -1665,58 +1675,58 @@
         </is>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>3.376</v>
+        <v>0.381</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.369</v>
+        <v>0.381</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>3.393</v>
+        <v>0.377</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>3.409</v>
+        <v>0.378</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>3.361</v>
+        <v>0.382</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>3.261</v>
+        <v>0.365</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>3.219</v>
+        <v>0.371</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>-0.0578</v>
+        <v>0.7012</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>-0.3158</v>
+        <v>0.1116</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>0.238</v>
+        <v>0.0964</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>0.0934</v>
+        <v>0.097</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>0.117</v>
+        <v>-0.0265</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.495</v>
+        <v>0.767</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-4.85</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1725,9 +1735,7 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
         <v>2</v>
@@ -1738,26 +1746,30 @@
       <c r="R11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-18.23</v>
+        <v>-17.61</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-1.53</v>
+        <v>-0.24</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>1.88</v>
+        <v>2.65</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.88</v>
+        <v>-0.04</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>14.8</v>
+        <v>26.1</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
@@ -1769,58 +1781,58 @@
         </is>
       </c>
       <c r="AG11" s="2" t="n">
-        <v>0.49</v>
+        <v>0.761</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>0.499</v>
+        <v>0.77</v>
       </c>
       <c r="AI11" s="2" t="n">
-        <v>0.506</v>
+        <v>0.78</v>
       </c>
       <c r="AJ11" s="2" t="n">
-        <v>0.511</v>
+        <v>0.789</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>0.516</v>
+        <v>0.792</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>0.516</v>
+        <v>0.787</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>0.532</v>
+        <v>0.826</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>-0.6179</v>
+        <v>-0.6183</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>-0.9244</v>
+        <v>-0.8679</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>-0.424</v>
+        <v>-0.3469</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>-0.1617</v>
+        <v>-0.1601</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>-0.1823</v>
+        <v>-0.1761</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.38</v>
+        <v>2.856</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>9.880000000000001</v>
+        <v>77.83</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1830,38 +1842,36 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N12" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R12" s="2" t="inlineStr"/>
       <c r="S12" s="2" t="inlineStr"/>
-      <c r="T12" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-2.65</v>
+        <v>-0.3</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>8.08</v>
+        <v>-1.66</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>4.63</v>
+        <v>-2.69</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>7.21</v>
+        <v>-0.76</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>65.40000000000001</v>
+        <v>27.3</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
@@ -1869,62 +1879,62 @@
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG12" s="2" t="n">
-        <v>0.381</v>
+        <v>2.924</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>0.38</v>
+        <v>3.011</v>
       </c>
       <c r="AI12" s="2" t="n">
-        <v>0.377</v>
+        <v>3.042</v>
       </c>
       <c r="AJ12" s="2" t="n">
-        <v>0.378</v>
+        <v>3.058</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>0.382</v>
+        <v>3.048</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>0.364</v>
+        <v>3.201</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>0.371</v>
+        <v>3.216</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>0.7743</v>
+        <v>-1.2045</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>0.06900000000000001</v>
+        <v>-0.7239</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.0789</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>0.0813</v>
+        <v>-0.4997</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>-0.0265</v>
+        <v>-0.003</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.764</v>
+        <v>0.34</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>-4.85</v>
+        <v>52.3</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1942,28 +1952,30 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
       <c r="R13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="2" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-16.83</v>
+        <v>-0.47</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-1.28</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>1.95</v>
+        <v>1.55</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>-0.31</v>
+        <v>7.78</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>28.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="AA13" s="2" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -1975,58 +1987,58 @@
         </is>
       </c>
       <c r="AG13" s="2" t="n">
-        <v>0.759</v>
+        <v>0.341</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>0.771</v>
+        <v>0.343</v>
       </c>
       <c r="AI13" s="2" t="n">
-        <v>0.783</v>
+        <v>0.339</v>
       </c>
       <c r="AJ13" s="2" t="n">
-        <v>0.789</v>
+        <v>0.34</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>0.792</v>
+        <v>0.34</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>0.786</v>
+        <v>0.325</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>0.826</v>
+        <v>0.336</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>-0.7279</v>
+        <v>0.4554</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>-0.8443000000000001</v>
+        <v>0.096</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>-0.3374</v>
+        <v>0.2668</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>-0.1842</v>
+        <v>0.0466</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>-0.1683</v>
+        <v>-0.0047</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.909</v>
+        <v>0.419</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>77.83</v>
+        <v>-1.36</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -2036,40 +2048,40 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S14" s="2" t="inlineStr"/>
-      <c r="T14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>0.8</v>
+        <v>-39.66</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-0.49</v>
+        <v>-7.97</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-2.96</v>
+        <v>4.54</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>-0.89</v>
+        <v>5.09</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>30.1</v>
+        <v>52</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>19</v>
+        <v>73</v>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
@@ -2077,62 +2089,62 @@
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG14" s="2" t="n">
-        <v>2.946</v>
+        <v>0.415</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>3.038</v>
+        <v>0.414</v>
       </c>
       <c r="AI14" s="2" t="n">
-        <v>3.051</v>
+        <v>0.415</v>
       </c>
       <c r="AJ14" s="2" t="n">
-        <v>3.065</v>
+        <v>0.418</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>3.047</v>
+        <v>0.426</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>3.207</v>
+        <v>0.423</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>3.215</v>
+        <v>0.471</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>-0.8184</v>
+        <v>0.3512</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>-0.6972</v>
+        <v>-0.3057</v>
       </c>
       <c r="AP14" s="2" t="n">
-        <v>0.09180000000000001</v>
+        <v>-0.1243</v>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>-0.4747</v>
+        <v>-0.3314</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>0.008</v>
+        <v>-0.3966</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.341</v>
+        <v>0.946</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>52.3</v>
+        <v>14.64</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -2149,96 +2161,94 @@
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S15" s="2" t="inlineStr"/>
-      <c r="T15" s="2" t="n">
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-0.47</v>
+        <v>25.94</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>7.66</v>
+        <v>5.08</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>3.19</v>
+        <v>-9.1</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>7.48</v>
+        <v>-6.26</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>73.8</v>
+        <v>-5.5</v>
       </c>
       <c r="AA15" s="2" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
-      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG15" s="2" t="n">
-        <v>0.342</v>
+        <v>0.988</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>0.343</v>
+        <v>1.038</v>
       </c>
       <c r="AI15" s="2" t="n">
-        <v>0.339</v>
+        <v>1.042</v>
       </c>
       <c r="AJ15" s="2" t="n">
-        <v>0.34</v>
+        <v>1.056</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>0.34</v>
+        <v>1.083</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>0.325</v>
+        <v>1.176</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>0.336</v>
+        <v>1.027</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>0.6587</v>
+        <v>-1.5406</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>0.0713</v>
+        <v>-1.0846</v>
       </c>
       <c r="AP15" s="2" t="n">
-        <v>0.2583</v>
+        <v>-1.0274</v>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>0.0323</v>
+        <v>-0.2205</v>
       </c>
       <c r="AR15" s="2" t="n">
-        <v>-0.0047</v>
+        <v>0.2594</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.082</v>
+        <v>0.868</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>81.33</v>
+        <v>85.37</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -2250,99 +2260,99 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-9.34</v>
+        <v>4.11</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-8.48</v>
+        <v>17.43</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-1.28</v>
+        <v>5.6</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>0.63</v>
+        <v>9.08</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>34.2</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
-      <c r="AD16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>1.096</v>
+        <v>0.854</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>1.126</v>
+        <v>0.846</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>1.141</v>
+        <v>0.844</v>
       </c>
       <c r="AJ16" s="2" t="n">
-        <v>1.134</v>
+        <v>0.84</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>1.13</v>
+        <v>0.828</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>1.194</v>
+        <v>0.802</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>1.301</v>
+        <v>0.799</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>-1.2132</v>
+        <v>0.3781</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>-0.474</v>
+        <v>0.198</v>
       </c>
       <c r="AP16" s="2" t="n">
-        <v>0.08019999999999999</v>
+        <v>0.3376</v>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>-0.8071</v>
+        <v>0.2313</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>-0.0934</v>
+        <v>0.0411</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.419</v>
+        <v>1.008</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-1.36</v>
+        <v>-8.65</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -2351,18 +2361,22 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N17" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O17" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="n">
-        <v>1</v>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S17" s="2" t="n">
         <v>1</v>
@@ -2370,22 +2384,22 @@
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-41.83</v>
+        <v>-56.16</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-8.720000000000001</v>
+        <v>-15.69</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>5.48</v>
+        <v>1.02</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>7.12</v>
+        <v>3.85</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>51.3</v>
+        <v>26.4</v>
       </c>
       <c r="AA17" s="2" t="n">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
@@ -2397,58 +2411,58 @@
         </is>
       </c>
       <c r="AG17" s="2" t="n">
-        <v>0.413</v>
+        <v>1.001</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>0.413</v>
+        <v>1.016</v>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>0.416</v>
+        <v>1.018</v>
       </c>
       <c r="AJ17" s="2" t="n">
-        <v>0.418</v>
+        <v>1.035</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>0.426</v>
+        <v>1.076</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>0.424</v>
+        <v>1.081</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>0.472</v>
+        <v>1.217</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>0.1753</v>
+        <v>-0.3205</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>-0.3167</v>
+        <v>-0.6902</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>-0.148</v>
+        <v>-0.4837</v>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>-0.361</v>
+        <v>-0.5124</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>-0.4183</v>
+        <v>-0.5616</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.07</v>
+        <v>1.739</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>-0.29</v>
+        <v>-5.36</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -2458,7 +2472,9 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N18" s="2" t="n">
         <v>1</v>
       </c>
@@ -2474,87 +2490,85 @@
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-11.51</v>
+        <v>-21.03</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-6.34</v>
+        <v>-2.68</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-1.55</v>
+        <v>1.11</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-3.34</v>
+        <v>-1.17</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>2.9</v>
+        <v>21</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
-      <c r="AC18" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG18" s="2" t="n">
-        <v>1.077</v>
+        <v>1.742</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>1.108</v>
+        <v>1.768</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>1.119</v>
+        <v>1.794</v>
       </c>
       <c r="AJ18" s="2" t="n">
-        <v>1.135</v>
+        <v>1.822</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>1.16</v>
+        <v>1.826</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>1.199</v>
+        <v>1.814</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>1.231</v>
+        <v>1.881</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-0.7941</v>
+        <v>-0.7481</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>-1.2317</v>
+        <v>-1.0217</v>
       </c>
       <c r="AP18" s="2" t="n">
-        <v>-0.5178</v>
+        <v>-0.3311</v>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>-0.6496</v>
+        <v>-0.1706</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>-0.1151</v>
+        <v>-0.2103</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.97</v>
+        <v>2.4</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>14.64</v>
+        <v>110.91</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -2563,126 +2577,130 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S19" s="2" t="n">
+      <c r="R19" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>28.83</v>
+        <v>26.65</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>7.09</v>
+        <v>30.24</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-9.9</v>
+        <v>5.79</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-7.53</v>
+        <v>13.72</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>-5</v>
+        <v>80.5</v>
       </c>
       <c r="AA19" s="2" t="n">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
-      <c r="AC19" s="2" t="n">
-        <v>11</v>
-      </c>
+      <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AG19" s="2" t="n">
-        <v>1.006</v>
+        <v>2.37</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>1.054</v>
+        <v>2.34</v>
       </c>
       <c r="AI19" s="2" t="n">
-        <v>1.047</v>
+        <v>2.281</v>
       </c>
       <c r="AJ19" s="2" t="n">
-        <v>1.061</v>
+        <v>2.257</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>1.088</v>
+        <v>2.231</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>1.178</v>
+        <v>2.206</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>1.027</v>
+        <v>2.035</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>-0.7294</v>
+        <v>1.7328</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>-1.0226</v>
+        <v>0.9041</v>
       </c>
       <c r="AP19" s="2" t="n">
-        <v>-0.8897</v>
+        <v>0.5929</v>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>-0.161</v>
+        <v>0.3313</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>0.2883</v>
+        <v>0.2665</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.85</v>
+        <v>1.444</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>85.37</v>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+        <v>6.69</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R20" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>1</v>
@@ -2690,87 +2708,87 @@
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>2.54</v>
+        <v>-23.53</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>14.28</v>
+        <v>-13.02</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>4.38</v>
+        <v>1.88</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>7.1</v>
+        <v>-1</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>96.59999999999999</v>
+        <v>1.4</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="AC20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG20" s="2" t="n">
-        <v>0.848</v>
+        <v>1.454</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>0.842</v>
+        <v>1.47</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>0.843</v>
+        <v>1.49</v>
       </c>
       <c r="AJ20" s="2" t="n">
-        <v>0.838</v>
+        <v>1.528</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>0.827</v>
+        <v>1.574</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>0.801</v>
+        <v>1.707</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>0.798</v>
+        <v>1.806</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>0.099</v>
+        <v>-0.6672</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>0.192</v>
+        <v>-1.0714</v>
       </c>
       <c r="AP20" s="2" t="n">
-        <v>0.3152</v>
+        <v>-0.3609</v>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>0.2099</v>
+        <v>-0.9706</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>0.0254</v>
+        <v>-0.2353</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.002</v>
+        <v>1.274</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-8.65</v>
+        <v>55.37</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -2779,45 +2797,39 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S21" s="2" t="n">
-        <v>-1</v>
-      </c>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-56.38</v>
+        <v>20.38</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-16.93</v>
+        <v>16.85</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>1.21</v>
+        <v>1.77</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>4.41</v>
+        <v>2.58</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>27.2</v>
+        <v>67.3</v>
       </c>
       <c r="AA21" s="2" t="n">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
@@ -2829,164 +2841,170 @@
         </is>
       </c>
       <c r="AG21" s="2" t="n">
-        <v>1.003</v>
+        <v>1.27</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>1.016</v>
+        <v>1.272</v>
       </c>
       <c r="AI21" s="2" t="n">
-        <v>1.021</v>
+        <v>1.278</v>
       </c>
       <c r="AJ21" s="2" t="n">
-        <v>1.038</v>
+        <v>1.293</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>1.077</v>
+        <v>1.267</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>1.083</v>
+        <v>1.24</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>1.219</v>
+        <v>1.204</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>-0.2748</v>
+        <v>0.1262</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>-0.7258</v>
+        <v>-0.5407</v>
       </c>
       <c r="AP21" s="2" t="n">
-        <v>-0.506</v>
+        <v>0.249</v>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>-0.5147</v>
+        <v>0.0737</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>-0.5638</v>
+        <v>0.2038</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.732</v>
+        <v>0.76</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>-5.36</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
+        <v>7.96</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-20.66</v>
+        <v>-24.32</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-3.82</v>
+        <v>-15.72</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>0.43</v>
+        <v>-0.01</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-0.22</v>
+        <v>0.57</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG22" s="2" t="n">
-        <v>1.744</v>
+        <v>0.767</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>1.773</v>
+        <v>0.785</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>1.802</v>
+        <v>0.795</v>
       </c>
       <c r="AJ22" s="2" t="n">
-        <v>1.825</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>1.828</v>
+        <v>0.824</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>1.815</v>
+        <v>0.907</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>1.883</v>
+        <v>0.987</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>-0.7599</v>
+        <v>-0.975</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>-1.0073</v>
+        <v>-0.8054</v>
       </c>
       <c r="AP22" s="2" t="n">
-        <v>-0.2969</v>
+        <v>-0.2938</v>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>-0.1816</v>
+        <v>-1.0007</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>-0.2066</v>
+        <v>-0.2432</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.398</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>110.91</v>
+        <v>89.25</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -2995,14 +3013,12 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="n">
-        <v>-9</v>
+        <v>13</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -3012,85 +3028,87 @@
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>25.28</v>
+        <v>25.43</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>29.45</v>
+        <v>1.79</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>7.16</v>
+        <v>-11.14</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>14.31</v>
+        <v>-11.15</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>77.09999999999999</v>
+        <v>16.7</v>
       </c>
       <c r="AA23" s="2" t="n">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>2.35</v>
+        <v>0.601</v>
       </c>
       <c r="AH23" s="2" t="n">
-        <v>2.326</v>
+        <v>0.643</v>
       </c>
       <c r="AI23" s="2" t="n">
-        <v>2.272</v>
+        <v>0.659</v>
       </c>
       <c r="AJ23" s="2" t="n">
-        <v>2.25</v>
+        <v>0.658</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>2.225</v>
+        <v>0.653</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>2.203</v>
+        <v>0.724</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>2.033</v>
+        <v>0.643</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>1.6757</v>
+        <v>-2.9172</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>0.7786999999999999</v>
+        <v>-1.021</v>
       </c>
       <c r="AP23" s="2" t="n">
-        <v>0.5471</v>
+        <v>-0.522</v>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>0.3209</v>
+        <v>-0.5377</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>0.2528</v>
+        <v>0.2543</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.475</v>
+        <v>2.218</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>6.69</v>
+        <v>3.12</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
@@ -3098,56 +3116,62 @@
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="n">
         <v>13</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S24" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-23.54</v>
+        <v>-25.73</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-11.79</v>
+        <v>-15</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>2.76</v>
+        <v>1.78</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-0.83</v>
+        <v>0.44</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>1.9</v>
+        <v>-0.3</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="AB24" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
@@ -3157,58 +3181,58 @@
         </is>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>1.451</v>
+        <v>2.231</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>1.475</v>
+        <v>2.26</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>1.496</v>
+        <v>2.294</v>
       </c>
       <c r="AJ24" s="2" t="n">
-        <v>1.535</v>
+        <v>2.342</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>1.576</v>
+        <v>2.413</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>1.713</v>
+        <v>2.643</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>1.808</v>
+        <v>2.847</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>-0.6474</v>
+        <v>-0.8848</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>-1.2172</v>
+        <v>-0.8825</v>
       </c>
       <c r="AP24" s="2" t="n">
-        <v>-0.3617</v>
+        <v>-0.3571</v>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>-1.0128</v>
+        <v>-1.0278</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>-0.2354</v>
+        <v>-0.2573</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.905</v>
+        <v>0.841</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>79.97</v>
+        <v>7.5</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -3218,103 +3242,97 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>32.89</v>
+        <v>-11.47</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>7.41</v>
+        <v>-10.34</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-13.26</v>
+        <v>-4.3</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-9.779999999999999</v>
+        <v>-3.76</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="AA25" s="2" t="n">
-        <v>11</v>
-      </c>
+        <v>-4</v>
+      </c>
+      <c r="AA25" s="2" t="inlineStr"/>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="n">
-        <v>11</v>
-      </c>
+      <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG25" s="2" t="n">
-        <v>0.946</v>
+        <v>0.873</v>
       </c>
       <c r="AH25" s="2" t="n">
-        <v>1.007</v>
+        <v>0.898</v>
       </c>
       <c r="AI25" s="2" t="n">
-        <v>1.02</v>
+        <v>0.912</v>
       </c>
       <c r="AJ25" s="2" t="n">
-        <v>1.022</v>
+        <v>0.926</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>1.017</v>
+        <v>0.948</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>1.119</v>
+        <v>1.031</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>0.972</v>
+        <v>1.027</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>-2.1729</v>
+        <v>-1.2385</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>-0.9947</v>
+        <v>-1.1512</v>
       </c>
       <c r="AP25" s="2" t="n">
-        <v>-0.5753</v>
+        <v>-0.4222</v>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>-0.346</v>
+        <v>-0.6541</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>0.3289</v>
+        <v>-0.1147</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.298</v>
+        <v>2.983</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>55.37</v>
+        <v>6.32</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -3324,9 +3342,7 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
         <v>0</v>
       </c>
@@ -3334,148 +3350,132 @@
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>19.32</v>
+        <v>-0.75</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>18.37</v>
+        <v>-5.35</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>5.52</v>
+        <v>-4.47</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>3.99</v>
+        <v>-5.19</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>67</v>
+        <v>-4.2</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>77</v>
+        <v>13</v>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>1.268</v>
+        <v>3.083</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>1.269</v>
+        <v>3.212</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>1.279</v>
+        <v>3.28</v>
       </c>
       <c r="AJ26" s="2" t="n">
-        <v>1.293</v>
+        <v>3.323</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>1.265</v>
+        <v>3.405</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>1.239</v>
+        <v>3.689</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>1.203</v>
+        <v>3.525</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>-0.0927</v>
+        <v>-1.8665</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>-0.6633</v>
+        <v>-1.1033</v>
       </c>
       <c r="AP26" s="2" t="n">
-        <v>0.2788</v>
+        <v>-0.7409</v>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>0.0505</v>
+        <v>-0.5972</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>0.1932</v>
+        <v>-0.0075</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.765</v>
+        <v>7.125</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>7.96</v>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>14.72</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R27" s="2" t="inlineStr"/>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-23.3</v>
+        <v>5.17</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-15.77</v>
+        <v>-0.89</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.41</v>
+        <v>-3.27</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>0.09</v>
+        <v>-2.33</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>4.4</v>
+        <v>8.6</v>
       </c>
       <c r="AA27" s="2" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
@@ -3485,58 +3485,58 @@
         </is>
       </c>
       <c r="AG27" s="2" t="n">
-        <v>0.769</v>
+        <v>7.328</v>
       </c>
       <c r="AH27" s="2" t="n">
-        <v>0.79</v>
+        <v>7.527</v>
       </c>
       <c r="AI27" s="2" t="n">
-        <v>0.797</v>
+        <v>7.619</v>
       </c>
       <c r="AJ27" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>7.687</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>0.825</v>
+        <v>7.736</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>0.91</v>
+        <v>8.051</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>0.988</v>
+        <v>8.016</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>-0.7584</v>
+        <v>-1.1948</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>-0.8979</v>
+        <v>-0.8119</v>
       </c>
       <c r="AP27" s="2" t="n">
-        <v>-0.2623</v>
+        <v>-0.2146</v>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>-0.9759</v>
+        <v>-0.4423</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>-0.233</v>
+        <v>0.0517</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.592</v>
+        <v>1.058</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>89.25</v>
+        <v>81.33</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -3546,45 +3546,37 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R28" s="2" t="inlineStr"/>
       <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>29.94</v>
+        <v>-10.81</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>6.61</v>
+        <v>-9.880000000000001</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-13.15</v>
+        <v>-2.19</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-7.67</v>
+        <v>-1.55</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>19.7</v>
+        <v>30.8</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="n">
-        <v>11</v>
-      </c>
+      <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr">
@@ -3593,129 +3585,99 @@
         </is>
       </c>
       <c r="AG28" s="2" t="n">
-        <v>0.614</v>
+        <v>1.088</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>0.657</v>
+        <v>1.116</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>0.663</v>
+        <v>1.137</v>
       </c>
       <c r="AJ28" s="2" t="n">
-        <v>0.662</v>
+        <v>1.133</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>0.655</v>
+        <v>1.13</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>0.726</v>
+        <v>1.19</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>0.643</v>
+        <v>1.3</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>-2.1839</v>
+        <v>-1.3702</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>-0.8791</v>
+        <v>-0.6214</v>
       </c>
       <c r="AP28" s="2" t="n">
-        <v>-0.4395</v>
+        <v>0.0295</v>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>-0.4448</v>
+        <v>-0.8149999999999999</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>0.2994</v>
+        <v>-0.1081</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2.249</v>
+        <v>1.053</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>-0.29</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S29" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-25.56</v>
+        <v>-12.23</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-14.5</v>
+        <v>-7.17</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>1.89</v>
+        <v>-1.57</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>0.21</v>
+        <v>-2.74</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>0.1</v>
+        <v>2.6</v>
       </c>
       <c r="AA29" s="2" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
@@ -3725,58 +3687,58 @@
         </is>
       </c>
       <c r="AG29" s="2" t="n">
-        <v>2.23</v>
+        <v>1.071</v>
       </c>
       <c r="AH29" s="2" t="n">
-        <v>2.273</v>
+        <v>1.1</v>
       </c>
       <c r="AI29" s="2" t="n">
-        <v>2.303</v>
+        <v>1.113</v>
       </c>
       <c r="AJ29" s="2" t="n">
-        <v>2.355</v>
+        <v>1.132</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>2.418</v>
+        <v>1.158</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>2.655</v>
+        <v>1.197</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>2.853</v>
+        <v>1.231</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-0.8519</v>
+        <v>-1.0568</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>-1.042</v>
+        <v>-1.286</v>
       </c>
       <c r="AP29" s="2" t="n">
-        <v>-0.3373</v>
+        <v>-0.5828</v>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>-1.0526</v>
+        <v>-0.6573</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>-0.2556</v>
+        <v>-0.1223</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v>0.863</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>7.5</v>
+        <v>79.97</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -3786,83 +3748,81 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R30" s="2" t="inlineStr"/>
       <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-9.57</v>
+        <v>28.66</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-8.699999999999999</v>
+        <v>3.02</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-3</v>
+        <v>-11.77</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-3.58</v>
+        <v>-12.08</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="AA30" s="2" t="inlineStr"/>
+        <v>11.7</v>
+      </c>
+      <c r="AA30" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AG30" s="2" t="n">
-        <v>0.883</v>
+        <v>0.925</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>0.907</v>
+        <v>0.986</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>0.917</v>
+        <v>1.014</v>
       </c>
       <c r="AJ30" s="2" t="n">
-        <v>0.929</v>
+        <v>1.016</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>0.95</v>
+        <v>1.014</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>1.034</v>
+        <v>1.116</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>1.027</v>
+        <v>0.973</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>-0.7961</v>
+        <v>-2.8229</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>-1.0419</v>
+        <v>-1.1359</v>
       </c>
       <c r="AP30" s="2" t="n">
-        <v>-0.4096</v>
+        <v>-0.6543</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>-0.6106</v>
+        <v>-0.4305</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>-0.09569999999999999</v>
+        <v>0.2866</v>
       </c>
     </row>
     <row r="31">
@@ -3877,7 +3837,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.541</v>
+        <v>1.506</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>12.87</v>
@@ -3897,37 +3857,31 @@
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S31" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr"/>
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>15.95</v>
+        <v>13.38</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>2.33</v>
+        <v>0.66</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-8.66</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-6.61</v>
+        <v>-6.05</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>-4.9</v>
+        <v>-5.3</v>
       </c>
       <c r="AA31" s="2" t="n">
         <v>12</v>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
@@ -3937,40 +3891,40 @@
         </is>
       </c>
       <c r="AG31" s="2" t="n">
-        <v>1.599</v>
+        <v>1.571</v>
       </c>
       <c r="AH31" s="2" t="n">
-        <v>1.671</v>
+        <v>1.648</v>
       </c>
       <c r="AI31" s="2" t="n">
-        <v>1.67</v>
+        <v>1.661</v>
       </c>
       <c r="AJ31" s="2" t="n">
-        <v>1.69</v>
+        <v>1.682</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>1.732</v>
+        <v>1.725</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>1.847</v>
+        <v>1.844</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>1.674</v>
+        <v>1.675</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>-0.9169</v>
+        <v>-1.6562</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>-1.0528</v>
+        <v>-1.1313</v>
       </c>
       <c r="AP31" s="2" t="n">
-        <v>-0.8777</v>
+        <v>-1.0065</v>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>-0.2783</v>
+        <v>-0.3298</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>0.1595</v>
+        <v>0.1338</v>
       </c>
     </row>
   </sheetData>
@@ -4001,7 +3955,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-09 | 30 只</t>
+          <t>截至: 2026-10-12 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-13
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$AV$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$AZ$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV31"/>
+  <dimension ref="A1:AZ31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -519,6 +519,10 @@
     <col width="11" customWidth="1" min="46" max="46"/>
     <col width="11" customWidth="1" min="47" max="47"/>
     <col width="11" customWidth="1" min="48" max="48"/>
+    <col width="11" customWidth="1" min="49" max="49"/>
+    <col width="11" customWidth="1" min="50" max="50"/>
+    <col width="11" customWidth="1" min="51" max="51"/>
+    <col width="11" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,135 +633,155 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Stage持续</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>1→2</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>3→4</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>KDJ Cross</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>日MACD Cross</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>5_10 Cross</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>10_50 Cross</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>年线斜率</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300_1W</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300_4W</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>风险度</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>动量</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>DS信号</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>B距今</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>S距今</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>急杀</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>周线档</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>5D MV</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>10D MV</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>20D MV</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>30D MV</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>50D MV</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>100D MV</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>200D MV</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>10D斜率</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>20D斜率</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>50D斜率</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>100D斜率</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>200D斜率</t>
         </is>
@@ -813,75 +837,85 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="W2" s="2" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="n">
+        <v>24</v>
+      </c>
       <c r="X2" s="2" t="inlineStr"/>
       <c r="Y2" s="2" t="inlineStr"/>
-      <c r="Z2" s="2" t="n">
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="n">
         <v>-3.41</v>
       </c>
-      <c r="AA2" s="2" t="n">
+      <c r="AE2" s="2" t="n">
         <v>-5.35</v>
       </c>
-      <c r="AB2" s="2" t="n">
+      <c r="AF2" s="2" t="n">
         <v>-4.47</v>
       </c>
-      <c r="AC2" s="2" t="n">
+      <c r="AG2" s="2" t="n">
         <v>-5.19</v>
       </c>
-      <c r="AD2" s="2" t="n">
+      <c r="AH2" s="2" t="n">
         <v>-4.2</v>
       </c>
-      <c r="AE2" s="2" t="n">
+      <c r="AI2" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AF2" s="2" t="inlineStr"/>
-      <c r="AG2" s="2" t="n">
+      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AK2" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="AH2" s="2" t="inlineStr"/>
-      <c r="AI2" s="2" t="inlineStr"/>
-      <c r="AJ2" s="2" t="inlineStr">
+      <c r="AL2" s="2" t="inlineStr"/>
+      <c r="AM2" s="2" t="inlineStr"/>
+      <c r="AN2" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="n">
+      <c r="AO2" s="2" t="n">
         <v>3.046</v>
       </c>
-      <c r="AL2" s="2" t="n">
+      <c r="AP2" s="2" t="n">
         <v>3.168</v>
       </c>
-      <c r="AM2" s="2" t="n">
+      <c r="AQ2" s="2" t="n">
         <v>3.258</v>
       </c>
-      <c r="AN2" s="2" t="n">
+      <c r="AR2" s="2" t="n">
         <v>3.307</v>
       </c>
-      <c r="AO2" s="2" t="n">
+      <c r="AS2" s="2" t="n">
         <v>3.392</v>
       </c>
-      <c r="AP2" s="2" t="n">
+      <c r="AT2" s="2" t="n">
         <v>3.679</v>
       </c>
-      <c r="AQ2" s="2" t="n">
+      <c r="AU2" s="2" t="n">
         <v>3.524</v>
       </c>
-      <c r="AR2" s="2" t="n">
+      <c r="AV2" s="2" t="n">
         <v>-2.3478</v>
       </c>
-      <c r="AS2" s="2" t="n">
+      <c r="AW2" s="2" t="n">
         <v>-1.222</v>
       </c>
-      <c r="AT2" s="2" t="n">
+      <c r="AX2" s="2" t="n">
         <v>-0.8397</v>
       </c>
-      <c r="AU2" s="2" t="n">
+      <c r="AY2" s="2" t="n">
         <v>-0.6473</v>
       </c>
-      <c r="AV2" s="2" t="n">
+      <c r="AZ2" s="2" t="n">
         <v>-0.0341</v>
       </c>
     </row>
@@ -914,7 +948,7 @@
         <v>13</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -935,71 +969,81 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V3" s="2" t="inlineStr"/>
-      <c r="W3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="X3" s="2" t="inlineStr"/>
       <c r="Y3" s="2" t="inlineStr"/>
-      <c r="Z3" s="2" t="n">
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="n">
         <v>-14.69</v>
       </c>
-      <c r="AA3" s="2" t="n">
+      <c r="AE3" s="2" t="n">
         <v>1.18</v>
       </c>
-      <c r="AB3" s="2" t="n">
+      <c r="AF3" s="2" t="n">
         <v>-0.38</v>
       </c>
-      <c r="AC3" s="2" t="n">
+      <c r="AG3" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AD3" s="2" t="n">
+      <c r="AH3" s="2" t="n">
         <v>53.9</v>
       </c>
-      <c r="AE3" s="2" t="n">
+      <c r="AI3" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="AF3" s="2" t="inlineStr"/>
-      <c r="AG3" s="2" t="inlineStr"/>
-      <c r="AH3" s="2" t="inlineStr"/>
-      <c r="AI3" s="2" t="inlineStr"/>
-      <c r="AJ3" s="2" t="inlineStr">
+      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AK3" s="2" t="inlineStr"/>
+      <c r="AL3" s="2" t="inlineStr"/>
+      <c r="AM3" s="2" t="inlineStr"/>
+      <c r="AN3" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK3" s="2" t="n">
+      <c r="AO3" s="2" t="n">
         <v>1.483</v>
       </c>
-      <c r="AL3" s="2" t="n">
+      <c r="AP3" s="2" t="n">
         <v>1.507</v>
       </c>
-      <c r="AM3" s="2" t="n">
+      <c r="AQ3" s="2" t="n">
         <v>1.522</v>
       </c>
-      <c r="AN3" s="2" t="n">
+      <c r="AR3" s="2" t="n">
         <v>1.539</v>
       </c>
-      <c r="AO3" s="2" t="n">
+      <c r="AS3" s="2" t="n">
         <v>1.559</v>
       </c>
-      <c r="AP3" s="2" t="n">
+      <c r="AT3" s="2" t="n">
         <v>1.54</v>
       </c>
-      <c r="AQ3" s="2" t="n">
+      <c r="AU3" s="2" t="n">
         <v>1.59</v>
       </c>
-      <c r="AR3" s="2" t="n">
+      <c r="AV3" s="2" t="n">
         <v>-0.738</v>
       </c>
-      <c r="AS3" s="2" t="n">
+      <c r="AW3" s="2" t="n">
         <v>-0.7178</v>
       </c>
-      <c r="AT3" s="2" t="n">
+      <c r="AX3" s="2" t="n">
         <v>-0.2576</v>
       </c>
-      <c r="AU3" s="2" t="n">
+      <c r="AY3" s="2" t="n">
         <v>-0.2383</v>
       </c>
-      <c r="AV3" s="2" t="n">
+      <c r="AZ3" s="2" t="n">
         <v>-0.1469</v>
       </c>
     </row>
@@ -1051,77 +1095,87 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V4" s="2" t="n">
-        <v>-1</v>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="X4" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="X4" s="2" t="inlineStr"/>
       <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA4" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="n">
         <v>-43.55</v>
       </c>
-      <c r="AA4" s="2" t="n">
+      <c r="AE4" s="2" t="n">
         <v>-2.16</v>
       </c>
-      <c r="AB4" s="2" t="n">
+      <c r="AF4" s="2" t="n">
         <v>4.72</v>
       </c>
-      <c r="AC4" s="2" t="n">
+      <c r="AG4" s="2" t="n">
         <v>4.87</v>
       </c>
-      <c r="AD4" s="2" t="n">
+      <c r="AH4" s="2" t="n">
         <v>66.59999999999999</v>
       </c>
-      <c r="AE4" s="2" t="n">
+      <c r="AI4" s="2" t="n">
         <v>76</v>
       </c>
-      <c r="AF4" s="2" t="inlineStr"/>
-      <c r="AG4" s="2" t="inlineStr"/>
-      <c r="AH4" s="2" t="inlineStr"/>
-      <c r="AI4" s="2" t="inlineStr"/>
-      <c r="AJ4" s="2" t="inlineStr">
+      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AK4" s="2" t="inlineStr"/>
+      <c r="AL4" s="2" t="inlineStr"/>
+      <c r="AM4" s="2" t="inlineStr"/>
+      <c r="AN4" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK4" s="2" t="n">
+      <c r="AO4" s="2" t="n">
         <v>2.242</v>
       </c>
-      <c r="AL4" s="2" t="n">
+      <c r="AP4" s="2" t="n">
         <v>2.422</v>
       </c>
-      <c r="AM4" s="2" t="n">
+      <c r="AQ4" s="2" t="n">
         <v>2.532</v>
       </c>
-      <c r="AN4" s="2" t="n">
+      <c r="AR4" s="2" t="n">
         <v>2.582</v>
       </c>
-      <c r="AO4" s="2" t="n">
+      <c r="AS4" s="2" t="n">
         <v>2.632</v>
       </c>
-      <c r="AP4" s="2" t="n">
+      <c r="AT4" s="2" t="n">
         <v>2.62</v>
       </c>
-      <c r="AQ4" s="2" t="n">
+      <c r="AU4" s="2" t="n">
         <v>2.85</v>
       </c>
-      <c r="AR4" s="2" t="n">
+      <c r="AV4" s="2" t="n">
         <v>-3.6607</v>
       </c>
-      <c r="AS4" s="2" t="n">
+      <c r="AW4" s="2" t="n">
         <v>-2.2574</v>
       </c>
-      <c r="AT4" s="2" t="n">
+      <c r="AX4" s="2" t="n">
         <v>-0.8221000000000001</v>
       </c>
-      <c r="AU4" s="2" t="n">
+      <c r="AY4" s="2" t="n">
         <v>-0.6316000000000001</v>
       </c>
-      <c r="AV4" s="2" t="n">
+      <c r="AZ4" s="2" t="n">
         <v>-0.4355</v>
       </c>
     </row>
@@ -1160,7 +1214,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -1183,75 +1237,85 @@
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="W5" s="2" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>27</v>
+      </c>
       <c r="X5" s="2" t="inlineStr"/>
       <c r="Y5" s="2" t="inlineStr"/>
-      <c r="Z5" s="2" t="n">
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="n">
         <v>57.45</v>
       </c>
-      <c r="AA5" s="2" t="n">
+      <c r="AE5" s="2" t="n">
         <v>39.41</v>
       </c>
-      <c r="AB5" s="2" t="n">
+      <c r="AF5" s="2" t="n">
         <v>9.57</v>
       </c>
-      <c r="AC5" s="2" t="n">
+      <c r="AG5" s="2" t="n">
         <v>18.89</v>
       </c>
-      <c r="AD5" s="2" t="n">
+      <c r="AH5" s="2" t="n">
         <v>101</v>
       </c>
-      <c r="AE5" s="2" t="n">
+      <c r="AI5" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="AF5" s="2" t="inlineStr"/>
-      <c r="AG5" s="2" t="inlineStr"/>
-      <c r="AH5" s="2" t="n">
+      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AK5" s="2" t="inlineStr"/>
+      <c r="AL5" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="AI5" s="2" t="inlineStr"/>
-      <c r="AJ5" s="2" t="inlineStr">
+      <c r="AM5" s="2" t="inlineStr"/>
+      <c r="AN5" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK5" s="2" t="n">
+      <c r="AO5" s="2" t="n">
         <v>1.876</v>
       </c>
-      <c r="AL5" s="2" t="n">
+      <c r="AP5" s="2" t="n">
         <v>1.808</v>
       </c>
-      <c r="AM5" s="2" t="n">
+      <c r="AQ5" s="2" t="n">
         <v>1.788</v>
       </c>
-      <c r="AN5" s="2" t="n">
+      <c r="AR5" s="2" t="n">
         <v>1.73</v>
       </c>
-      <c r="AO5" s="2" t="n">
+      <c r="AS5" s="2" t="n">
         <v>1.642</v>
       </c>
-      <c r="AP5" s="2" t="n">
+      <c r="AT5" s="2" t="n">
         <v>1.586</v>
       </c>
-      <c r="AQ5" s="2" t="n">
+      <c r="AU5" s="2" t="n">
         <v>1.523</v>
       </c>
-      <c r="AR5" s="2" t="n">
+      <c r="AV5" s="2" t="n">
         <v>1.5095</v>
       </c>
-      <c r="AS5" s="2" t="n">
+      <c r="AW5" s="2" t="n">
         <v>1.5361</v>
       </c>
-      <c r="AT5" s="2" t="n">
+      <c r="AX5" s="2" t="n">
         <v>1.1671</v>
       </c>
-      <c r="AU5" s="2" t="n">
+      <c r="AY5" s="2" t="n">
         <v>0.3711</v>
       </c>
-      <c r="AV5" s="2" t="n">
+      <c r="AZ5" s="2" t="n">
         <v>0.5745</v>
       </c>
     </row>
@@ -1282,7 +1346,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
@@ -1303,73 +1367,83 @@
           <t>0010011000</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W6" s="2" t="n">
-        <v>-1</v>
+        <v>12</v>
       </c>
       <c r="X6" s="2" t="inlineStr"/>
       <c r="Y6" s="2" t="inlineStr"/>
-      <c r="Z6" s="2" t="n">
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="n">
         <v>-4.46</v>
       </c>
-      <c r="AA6" s="2" t="n">
+      <c r="AE6" s="2" t="n">
         <v>6.47</v>
       </c>
-      <c r="AB6" s="2" t="n">
+      <c r="AF6" s="2" t="n">
         <v>-0.35</v>
       </c>
-      <c r="AC6" s="2" t="n">
+      <c r="AG6" s="2" t="n">
         <v>5.56</v>
       </c>
-      <c r="AD6" s="2" t="n">
+      <c r="AH6" s="2" t="n">
         <v>55.2</v>
       </c>
-      <c r="AE6" s="2" t="n">
+      <c r="AI6" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="AF6" s="2" t="inlineStr"/>
-      <c r="AG6" s="2" t="inlineStr"/>
-      <c r="AH6" s="2" t="inlineStr"/>
-      <c r="AI6" s="2" t="inlineStr"/>
-      <c r="AJ6" s="2" t="inlineStr">
+      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AK6" s="2" t="inlineStr"/>
+      <c r="AL6" s="2" t="inlineStr"/>
+      <c r="AM6" s="2" t="inlineStr"/>
+      <c r="AN6" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK6" s="2" t="n">
+      <c r="AO6" s="2" t="n">
         <v>0.841</v>
       </c>
-      <c r="AL6" s="2" t="n">
+      <c r="AP6" s="2" t="n">
         <v>0.847</v>
       </c>
-      <c r="AM6" s="2" t="n">
+      <c r="AQ6" s="2" t="n">
         <v>0.84</v>
       </c>
-      <c r="AN6" s="2" t="n">
+      <c r="AR6" s="2" t="n">
         <v>0.845</v>
       </c>
-      <c r="AO6" s="2" t="n">
+      <c r="AS6" s="2" t="n">
         <v>0.861</v>
       </c>
-      <c r="AP6" s="2" t="n">
+      <c r="AT6" s="2" t="n">
         <v>0.827</v>
       </c>
-      <c r="AQ6" s="2" t="n">
+      <c r="AU6" s="2" t="n">
         <v>0.832</v>
       </c>
-      <c r="AR6" s="2" t="n">
+      <c r="AV6" s="2" t="n">
         <v>0.1354</v>
       </c>
-      <c r="AS6" s="2" t="n">
+      <c r="AW6" s="2" t="n">
         <v>-0.07729999999999999</v>
       </c>
-      <c r="AT6" s="2" t="n">
+      <c r="AX6" s="2" t="n">
         <v>-0.1566</v>
       </c>
-      <c r="AU6" s="2" t="n">
+      <c r="AY6" s="2" t="n">
         <v>0.0541</v>
       </c>
-      <c r="AV6" s="2" t="n">
+      <c r="AZ6" s="2" t="n">
         <v>-0.0446</v>
       </c>
     </row>
@@ -1423,71 +1497,81 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>16</v>
+      </c>
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="2" t="inlineStr"/>
-      <c r="Z7" s="2" t="n">
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="n">
         <v>-13.44</v>
       </c>
-      <c r="AA7" s="2" t="n">
+      <c r="AE7" s="2" t="n">
         <v>4.81</v>
       </c>
-      <c r="AB7" s="2" t="n">
+      <c r="AF7" s="2" t="n">
         <v>1.6</v>
       </c>
-      <c r="AC7" s="2" t="n">
+      <c r="AG7" s="2" t="n">
         <v>2.52</v>
       </c>
-      <c r="AD7" s="2" t="n">
+      <c r="AH7" s="2" t="n">
         <v>18.1</v>
       </c>
-      <c r="AE7" s="2" t="n">
+      <c r="AI7" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="AF7" s="2" t="inlineStr"/>
-      <c r="AG7" s="2" t="inlineStr"/>
-      <c r="AH7" s="2" t="inlineStr"/>
-      <c r="AI7" s="2" t="inlineStr"/>
-      <c r="AJ7" s="2" t="inlineStr">
+      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AK7" s="2" t="inlineStr"/>
+      <c r="AL7" s="2" t="inlineStr"/>
+      <c r="AM7" s="2" t="inlineStr"/>
+      <c r="AN7" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK7" s="2" t="n">
+      <c r="AO7" s="2" t="n">
         <v>3.973</v>
       </c>
-      <c r="AL7" s="2" t="n">
+      <c r="AP7" s="2" t="n">
         <v>4.132</v>
       </c>
-      <c r="AM7" s="2" t="n">
+      <c r="AQ7" s="2" t="n">
         <v>4.229</v>
       </c>
-      <c r="AN7" s="2" t="n">
+      <c r="AR7" s="2" t="n">
         <v>4.281</v>
       </c>
-      <c r="AO7" s="2" t="n">
+      <c r="AS7" s="2" t="n">
         <v>4.319</v>
       </c>
-      <c r="AP7" s="2" t="n">
+      <c r="AT7" s="2" t="n">
         <v>4.343</v>
       </c>
-      <c r="AQ7" s="2" t="n">
+      <c r="AU7" s="2" t="n">
         <v>4.394</v>
       </c>
-      <c r="AR7" s="2" t="n">
+      <c r="AV7" s="2" t="n">
         <v>-2.0131</v>
       </c>
-      <c r="AS7" s="2" t="n">
+      <c r="AW7" s="2" t="n">
         <v>-1.2533</v>
       </c>
-      <c r="AT7" s="2" t="n">
+      <c r="AX7" s="2" t="n">
         <v>-0.5623</v>
       </c>
-      <c r="AU7" s="2" t="n">
+      <c r="AY7" s="2" t="n">
         <v>-0.3006</v>
       </c>
-      <c r="AV7" s="2" t="n">
+      <c r="AZ7" s="2" t="n">
         <v>-0.1344</v>
       </c>
     </row>
@@ -1547,73 +1631,83 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr"/>
-      <c r="W8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="n">
+        <v>15</v>
+      </c>
       <c r="X8" s="2" t="inlineStr"/>
       <c r="Y8" s="2" t="inlineStr"/>
-      <c r="Z8" s="2" t="n">
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="n">
         <v>-10.51</v>
       </c>
-      <c r="AA8" s="2" t="n">
+      <c r="AE8" s="2" t="n">
         <v>1.25</v>
       </c>
-      <c r="AB8" s="2" t="n">
+      <c r="AF8" s="2" t="n">
         <v>-0.11</v>
       </c>
-      <c r="AC8" s="2" t="n">
+      <c r="AG8" s="2" t="n">
         <v>0.03</v>
       </c>
-      <c r="AD8" s="2" t="n">
+      <c r="AH8" s="2" t="n">
         <v>-3.1</v>
       </c>
-      <c r="AE8" s="2" t="n">
+      <c r="AI8" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="AF8" s="2" t="inlineStr"/>
-      <c r="AG8" s="2" t="n">
+      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AK8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="AH8" s="2" t="inlineStr"/>
-      <c r="AI8" s="2" t="inlineStr"/>
-      <c r="AJ8" s="2" t="inlineStr">
+      <c r="AL8" s="2" t="inlineStr"/>
+      <c r="AM8" s="2" t="inlineStr"/>
+      <c r="AN8" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AK8" s="2" t="n">
+      <c r="AO8" s="2" t="n">
         <v>5.321</v>
       </c>
-      <c r="AL8" s="2" t="n">
+      <c r="AP8" s="2" t="n">
         <v>5.518</v>
       </c>
-      <c r="AM8" s="2" t="n">
+      <c r="AQ8" s="2" t="n">
         <v>5.661</v>
       </c>
-      <c r="AN8" s="2" t="n">
+      <c r="AR8" s="2" t="n">
         <v>5.738</v>
       </c>
-      <c r="AO8" s="2" t="n">
+      <c r="AS8" s="2" t="n">
         <v>5.821</v>
       </c>
-      <c r="AP8" s="2" t="n">
+      <c r="AT8" s="2" t="n">
         <v>5.993</v>
       </c>
-      <c r="AQ8" s="2" t="n">
+      <c r="AU8" s="2" t="n">
         <v>5.967</v>
       </c>
-      <c r="AR8" s="2" t="n">
+      <c r="AV8" s="2" t="n">
         <v>-2.0643</v>
       </c>
-      <c r="AS8" s="2" t="n">
+      <c r="AW8" s="2" t="n">
         <v>-1.2384</v>
       </c>
-      <c r="AT8" s="2" t="n">
+      <c r="AX8" s="2" t="n">
         <v>-0.6261</v>
       </c>
-      <c r="AU8" s="2" t="n">
+      <c r="AY8" s="2" t="n">
         <v>-0.4112</v>
       </c>
-      <c r="AV8" s="2" t="n">
+      <c r="AZ8" s="2" t="n">
         <v>-0.1051</v>
       </c>
     </row>
@@ -1665,81 +1759,95 @@
           <t>1111111101</t>
         </is>
       </c>
-      <c r="V9" s="2" t="n">
-        <v>1</v>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="W9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="X9" s="2" t="n">
+      <c r="X9" s="2" t="inlineStr"/>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>4d</t>
+        </is>
+      </c>
+      <c r="Z9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="Y9" s="2" t="n">
+      <c r="AC9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Z9" s="2" t="n">
+      <c r="AD9" s="2" t="n">
         <v>48.24</v>
       </c>
-      <c r="AA9" s="2" t="n">
+      <c r="AE9" s="2" t="n">
         <v>-0.89</v>
       </c>
-      <c r="AB9" s="2" t="n">
+      <c r="AF9" s="2" t="n">
         <v>-3.27</v>
       </c>
-      <c r="AC9" s="2" t="n">
+      <c r="AG9" s="2" t="n">
         <v>-2.33</v>
       </c>
-      <c r="AD9" s="2" t="n">
+      <c r="AH9" s="2" t="n">
         <v>8.6</v>
       </c>
-      <c r="AE9" s="2" t="n">
+      <c r="AI9" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AF9" s="2" t="inlineStr"/>
-      <c r="AG9" s="2" t="n">
+      <c r="AJ9" s="2" t="inlineStr"/>
+      <c r="AK9" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="AH9" s="2" t="inlineStr"/>
-      <c r="AI9" s="2" t="inlineStr"/>
-      <c r="AJ9" s="2" t="inlineStr">
+      <c r="AL9" s="2" t="inlineStr"/>
+      <c r="AM9" s="2" t="inlineStr"/>
+      <c r="AN9" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AK9" s="2" t="n">
+      <c r="AO9" s="2" t="n">
         <v>3.405</v>
       </c>
-      <c r="AL9" s="2" t="n">
+      <c r="AP9" s="2" t="n">
         <v>3.003</v>
       </c>
-      <c r="AM9" s="2" t="n">
+      <c r="AQ9" s="2" t="n">
         <v>2.814</v>
       </c>
-      <c r="AN9" s="2" t="n">
+      <c r="AR9" s="2" t="n">
         <v>2.763</v>
       </c>
-      <c r="AO9" s="2" t="n">
+      <c r="AS9" s="2" t="n">
         <v>2.72</v>
       </c>
-      <c r="AP9" s="2" t="n">
+      <c r="AT9" s="2" t="n">
         <v>2.78</v>
       </c>
-      <c r="AQ9" s="2" t="n">
+      <c r="AU9" s="2" t="n">
         <v>2.749</v>
       </c>
-      <c r="AR9" s="2" t="n">
+      <c r="AV9" s="2" t="n">
         <v>7.6949</v>
       </c>
-      <c r="AS9" s="2" t="n">
+      <c r="AW9" s="2" t="n">
         <v>3.7764</v>
       </c>
-      <c r="AT9" s="2" t="n">
+      <c r="AX9" s="2" t="n">
         <v>1.5426</v>
       </c>
-      <c r="AU9" s="2" t="n">
+      <c r="AY9" s="2" t="n">
         <v>0.4281</v>
       </c>
-      <c r="AV9" s="2" t="n">
+      <c r="AZ9" s="2" t="n">
         <v>0.4824</v>
       </c>
     </row>
@@ -1793,79 +1901,89 @@
           <t>0000001000</t>
         </is>
       </c>
-      <c r="V10" s="2" t="n">
-        <v>-1</v>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="X10" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="X10" s="2" t="inlineStr"/>
       <c r="Y10" s="2" t="inlineStr"/>
       <c r="Z10" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA10" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="n">
         <v>2.19</v>
       </c>
-      <c r="AA10" s="2" t="n">
+      <c r="AE10" s="2" t="n">
         <v>17.35</v>
       </c>
-      <c r="AB10" s="2" t="n">
+      <c r="AF10" s="2" t="n">
         <v>4.56</v>
       </c>
-      <c r="AC10" s="2" t="n">
+      <c r="AG10" s="2" t="n">
         <v>5.95</v>
       </c>
-      <c r="AD10" s="2" t="n">
+      <c r="AH10" s="2" t="n">
         <v>82.40000000000001</v>
       </c>
-      <c r="AE10" s="2" t="n">
+      <c r="AI10" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="AF10" s="2" t="inlineStr"/>
-      <c r="AG10" s="2" t="inlineStr"/>
-      <c r="AH10" s="2" t="n">
+      <c r="AJ10" s="2" t="inlineStr"/>
+      <c r="AK10" s="2" t="inlineStr"/>
+      <c r="AL10" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="AI10" s="2" t="inlineStr"/>
-      <c r="AJ10" s="2" t="inlineStr">
+      <c r="AM10" s="2" t="inlineStr"/>
+      <c r="AN10" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK10" s="2" t="n">
+      <c r="AO10" s="2" t="n">
         <v>5.65</v>
       </c>
-      <c r="AL10" s="2" t="n">
+      <c r="AP10" s="2" t="n">
         <v>5.864</v>
       </c>
-      <c r="AM10" s="2" t="n">
+      <c r="AQ10" s="2" t="n">
         <v>6.02</v>
       </c>
-      <c r="AN10" s="2" t="n">
+      <c r="AR10" s="2" t="n">
         <v>6.095</v>
       </c>
-      <c r="AO10" s="2" t="n">
+      <c r="AS10" s="2" t="n">
         <v>6.057</v>
       </c>
-      <c r="AP10" s="2" t="n">
+      <c r="AT10" s="2" t="n">
         <v>5.896</v>
       </c>
-      <c r="AQ10" s="2" t="n">
+      <c r="AU10" s="2" t="n">
         <v>5.833</v>
       </c>
-      <c r="AR10" s="2" t="n">
+      <c r="AV10" s="2" t="n">
         <v>-1.9249</v>
       </c>
-      <c r="AS10" s="2" t="n">
+      <c r="AW10" s="2" t="n">
         <v>-1.2213</v>
       </c>
-      <c r="AT10" s="2" t="n">
+      <c r="AX10" s="2" t="n">
         <v>-0.1913</v>
       </c>
-      <c r="AU10" s="2" t="n">
+      <c r="AY10" s="2" t="n">
         <v>-0.101</v>
       </c>
-      <c r="AV10" s="2" t="n">
+      <c r="AZ10" s="2" t="n">
         <v>0.0219</v>
       </c>
     </row>
@@ -1919,79 +2037,89 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V11" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="W11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="X11" s="2" t="inlineStr"/>
       <c r="Y11" s="2" t="inlineStr"/>
       <c r="Z11" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA11" s="2" t="inlineStr"/>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="n">
         <v>-31.6</v>
       </c>
-      <c r="AA11" s="2" t="n">
+      <c r="AE11" s="2" t="n">
         <v>-0.8100000000000001</v>
       </c>
-      <c r="AB11" s="2" t="n">
+      <c r="AF11" s="2" t="n">
         <v>2.51</v>
       </c>
-      <c r="AC11" s="2" t="n">
+      <c r="AG11" s="2" t="n">
         <v>1.05</v>
       </c>
-      <c r="AD11" s="2" t="n">
+      <c r="AH11" s="2" t="n">
         <v>13.3</v>
       </c>
-      <c r="AE11" s="2" t="n">
+      <c r="AI11" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="AF11" s="2" t="inlineStr">
+      <c r="AJ11" s="2" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="AG11" s="2" t="n">
+      <c r="AK11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH11" s="2" t="inlineStr"/>
-      <c r="AI11" s="2" t="inlineStr"/>
-      <c r="AJ11" s="2" t="inlineStr">
+      <c r="AL11" s="2" t="inlineStr"/>
+      <c r="AM11" s="2" t="inlineStr"/>
+      <c r="AN11" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK11" s="2" t="n">
+      <c r="AO11" s="2" t="n">
         <v>0.885</v>
       </c>
-      <c r="AL11" s="2" t="n">
+      <c r="AP11" s="2" t="n">
         <v>0.9429999999999999</v>
       </c>
-      <c r="AM11" s="2" t="n">
+      <c r="AQ11" s="2" t="n">
         <v>0.98</v>
       </c>
-      <c r="AN11" s="2" t="n">
+      <c r="AR11" s="2" t="n">
         <v>1.003</v>
       </c>
-      <c r="AO11" s="2" t="n">
+      <c r="AS11" s="2" t="n">
         <v>1.019</v>
       </c>
-      <c r="AP11" s="2" t="n">
+      <c r="AT11" s="2" t="n">
         <v>1.027</v>
       </c>
-      <c r="AQ11" s="2" t="n">
+      <c r="AU11" s="2" t="n">
         <v>1.059</v>
       </c>
-      <c r="AR11" s="2" t="n">
+      <c r="AV11" s="2" t="n">
         <v>-3.1536</v>
       </c>
-      <c r="AS11" s="2" t="n">
+      <c r="AW11" s="2" t="n">
         <v>-2.1194</v>
       </c>
-      <c r="AT11" s="2" t="n">
+      <c r="AX11" s="2" t="n">
         <v>-0.8976</v>
       </c>
-      <c r="AU11" s="2" t="n">
+      <c r="AY11" s="2" t="n">
         <v>-0.3764</v>
       </c>
-      <c r="AV11" s="2" t="n">
+      <c r="AZ11" s="2" t="n">
         <v>-0.316</v>
       </c>
     </row>
@@ -2043,77 +2171,87 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V12" s="2" t="n">
-        <v>-1</v>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="X12" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="inlineStr"/>
       <c r="Z12" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA12" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB12" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="n">
         <v>-22.74</v>
       </c>
-      <c r="AA12" s="2" t="n">
+      <c r="AE12" s="2" t="n">
         <v>8.58</v>
       </c>
-      <c r="AB12" s="2" t="n">
+      <c r="AF12" s="2" t="n">
         <v>2.44</v>
       </c>
-      <c r="AC12" s="2" t="n">
+      <c r="AG12" s="2" t="n">
         <v>7.27</v>
       </c>
-      <c r="AD12" s="2" t="n">
+      <c r="AH12" s="2" t="n">
         <v>65.09999999999999</v>
       </c>
-      <c r="AE12" s="2" t="n">
+      <c r="AI12" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="AF12" s="2" t="inlineStr"/>
-      <c r="AG12" s="2" t="inlineStr"/>
-      <c r="AH12" s="2" t="inlineStr"/>
-      <c r="AI12" s="2" t="inlineStr"/>
-      <c r="AJ12" s="2" t="inlineStr">
+      <c r="AJ12" s="2" t="inlineStr"/>
+      <c r="AK12" s="2" t="inlineStr"/>
+      <c r="AL12" s="2" t="inlineStr"/>
+      <c r="AM12" s="2" t="inlineStr"/>
+      <c r="AN12" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK12" s="2" t="n">
+      <c r="AO12" s="2" t="n">
         <v>1.269</v>
       </c>
-      <c r="AL12" s="2" t="n">
+      <c r="AP12" s="2" t="n">
         <v>1.375</v>
       </c>
-      <c r="AM12" s="2" t="n">
+      <c r="AQ12" s="2" t="n">
         <v>1.415</v>
       </c>
-      <c r="AN12" s="2" t="n">
+      <c r="AR12" s="2" t="n">
         <v>1.439</v>
       </c>
-      <c r="AO12" s="2" t="n">
+      <c r="AS12" s="2" t="n">
         <v>1.471</v>
       </c>
-      <c r="AP12" s="2" t="n">
+      <c r="AT12" s="2" t="n">
         <v>1.414</v>
       </c>
-      <c r="AQ12" s="2" t="n">
+      <c r="AU12" s="2" t="n">
         <v>1.444</v>
       </c>
-      <c r="AR12" s="2" t="n">
+      <c r="AV12" s="2" t="n">
         <v>-3.3669</v>
       </c>
-      <c r="AS12" s="2" t="n">
+      <c r="AW12" s="2" t="n">
         <v>-1.8444</v>
       </c>
-      <c r="AT12" s="2" t="n">
+      <c r="AX12" s="2" t="n">
         <v>-0.6474</v>
       </c>
-      <c r="AU12" s="2" t="n">
+      <c r="AY12" s="2" t="n">
         <v>-0.2897</v>
       </c>
-      <c r="AV12" s="2" t="n">
+      <c r="AZ12" s="2" t="n">
         <v>-0.2274</v>
       </c>
     </row>
@@ -2165,73 +2303,83 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V13" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="W13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="X13" s="2" t="inlineStr"/>
       <c r="Y13" s="2" t="inlineStr"/>
       <c r="Z13" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA13" s="2" t="inlineStr"/>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AD13" s="2" t="n">
         <v>-34.81</v>
       </c>
-      <c r="AA13" s="2" t="n">
+      <c r="AE13" s="2" t="n">
         <v>-0.24</v>
       </c>
-      <c r="AB13" s="2" t="n">
+      <c r="AF13" s="2" t="n">
         <v>2.65</v>
       </c>
-      <c r="AC13" s="2" t="n">
+      <c r="AG13" s="2" t="n">
         <v>-0.04</v>
       </c>
-      <c r="AD13" s="2" t="n">
+      <c r="AH13" s="2" t="n">
         <v>26.1</v>
       </c>
-      <c r="AE13" s="2" t="n">
+      <c r="AI13" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="AF13" s="2" t="inlineStr"/>
-      <c r="AG13" s="2" t="inlineStr"/>
-      <c r="AH13" s="2" t="inlineStr"/>
-      <c r="AI13" s="2" t="inlineStr"/>
-      <c r="AJ13" s="2" t="inlineStr">
+      <c r="AJ13" s="2" t="inlineStr"/>
+      <c r="AK13" s="2" t="inlineStr"/>
+      <c r="AL13" s="2" t="inlineStr"/>
+      <c r="AM13" s="2" t="inlineStr"/>
+      <c r="AN13" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK13" s="2" t="n">
+      <c r="AO13" s="2" t="n">
         <v>1.96</v>
       </c>
-      <c r="AL13" s="2" t="n">
+      <c r="AP13" s="2" t="n">
         <v>2.127</v>
       </c>
-      <c r="AM13" s="2" t="n">
+      <c r="AQ13" s="2" t="n">
         <v>2.234</v>
       </c>
-      <c r="AN13" s="2" t="n">
+      <c r="AR13" s="2" t="n">
         <v>2.289</v>
       </c>
-      <c r="AO13" s="2" t="n">
+      <c r="AS13" s="2" t="n">
         <v>2.317</v>
       </c>
-      <c r="AP13" s="2" t="n">
+      <c r="AT13" s="2" t="n">
         <v>2.319</v>
       </c>
-      <c r="AQ13" s="2" t="n">
+      <c r="AU13" s="2" t="n">
         <v>2.441</v>
       </c>
-      <c r="AR13" s="2" t="n">
+      <c r="AV13" s="2" t="n">
         <v>-4.0071</v>
       </c>
-      <c r="AS13" s="2" t="n">
+      <c r="AW13" s="2" t="n">
         <v>-2.5263</v>
       </c>
-      <c r="AT13" s="2" t="n">
+      <c r="AX13" s="2" t="n">
         <v>-0.9963</v>
       </c>
-      <c r="AU13" s="2" t="n">
+      <c r="AY13" s="2" t="n">
         <v>-0.4661</v>
       </c>
-      <c r="AV13" s="2" t="n">
+      <c r="AZ13" s="2" t="n">
         <v>-0.3481</v>
       </c>
     </row>
@@ -2285,79 +2433,89 @@
           <t>1111111101</t>
         </is>
       </c>
-      <c r="V14" s="2" t="n">
-        <v>1</v>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="W14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="X14" s="2" t="n">
+      <c r="X14" s="2" t="inlineStr"/>
+      <c r="Y14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="Y14" s="2" t="n">
+      <c r="AC14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Z14" s="2" t="n">
+      <c r="AD14" s="2" t="n">
         <v>36.98</v>
       </c>
-      <c r="AA14" s="2" t="n">
+      <c r="AE14" s="2" t="n">
         <v>-1.66</v>
       </c>
-      <c r="AB14" s="2" t="n">
+      <c r="AF14" s="2" t="n">
         <v>-2.69</v>
       </c>
-      <c r="AC14" s="2" t="n">
+      <c r="AG14" s="2" t="n">
         <v>-0.76</v>
       </c>
-      <c r="AD14" s="2" t="n">
+      <c r="AH14" s="2" t="n">
         <v>27.3</v>
       </c>
-      <c r="AE14" s="2" t="n">
+      <c r="AI14" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="AF14" s="2" t="inlineStr"/>
-      <c r="AG14" s="2" t="inlineStr"/>
-      <c r="AH14" s="2" t="inlineStr"/>
-      <c r="AI14" s="2" t="inlineStr"/>
-      <c r="AJ14" s="2" t="inlineStr">
+      <c r="AJ14" s="2" t="inlineStr"/>
+      <c r="AK14" s="2" t="inlineStr"/>
+      <c r="AL14" s="2" t="inlineStr"/>
+      <c r="AM14" s="2" t="inlineStr"/>
+      <c r="AN14" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK14" s="2" t="n">
+      <c r="AO14" s="2" t="n">
         <v>1.438</v>
       </c>
-      <c r="AL14" s="2" t="n">
+      <c r="AP14" s="2" t="n">
         <v>1.29</v>
       </c>
-      <c r="AM14" s="2" t="n">
+      <c r="AQ14" s="2" t="n">
         <v>1.218</v>
       </c>
-      <c r="AN14" s="2" t="n">
+      <c r="AR14" s="2" t="n">
         <v>1.197</v>
       </c>
-      <c r="AO14" s="2" t="n">
+      <c r="AS14" s="2" t="n">
         <v>1.171</v>
       </c>
-      <c r="AP14" s="2" t="n">
+      <c r="AT14" s="2" t="n">
         <v>1.208</v>
       </c>
-      <c r="AQ14" s="2" t="n">
+      <c r="AU14" s="2" t="n">
         <v>1.207</v>
       </c>
-      <c r="AR14" s="2" t="n">
+      <c r="AV14" s="2" t="n">
         <v>6.5</v>
       </c>
-      <c r="AS14" s="2" t="n">
+      <c r="AW14" s="2" t="n">
         <v>3.2686</v>
       </c>
-      <c r="AT14" s="2" t="n">
+      <c r="AX14" s="2" t="n">
         <v>1.6367</v>
       </c>
-      <c r="AU14" s="2" t="n">
+      <c r="AY14" s="2" t="n">
         <v>0.2557</v>
       </c>
-      <c r="AV14" s="2" t="n">
+      <c r="AZ14" s="2" t="n">
         <v>0.3698</v>
       </c>
     </row>
@@ -2409,73 +2567,83 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="W15" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="2" t="inlineStr"/>
-      <c r="Z15" s="2" t="n">
+      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AA15" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="n">
         <v>-18.54</v>
       </c>
-      <c r="AA15" s="2" t="n">
+      <c r="AE15" s="2" t="n">
         <v>8.130000000000001</v>
       </c>
-      <c r="AB15" s="2" t="n">
+      <c r="AF15" s="2" t="n">
         <v>1.55</v>
       </c>
-      <c r="AC15" s="2" t="n">
+      <c r="AG15" s="2" t="n">
         <v>7.78</v>
       </c>
-      <c r="AD15" s="2" t="n">
+      <c r="AH15" s="2" t="n">
         <v>73.40000000000001</v>
       </c>
-      <c r="AE15" s="2" t="n">
+      <c r="AI15" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="AF15" s="2" t="inlineStr"/>
-      <c r="AG15" s="2" t="inlineStr"/>
-      <c r="AH15" s="2" t="inlineStr"/>
-      <c r="AI15" s="2" t="inlineStr"/>
-      <c r="AJ15" s="2" t="inlineStr">
+      <c r="AJ15" s="2" t="inlineStr"/>
+      <c r="AK15" s="2" t="inlineStr"/>
+      <c r="AL15" s="2" t="inlineStr"/>
+      <c r="AM15" s="2" t="inlineStr"/>
+      <c r="AN15" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK15" s="2" t="n">
+      <c r="AO15" s="2" t="n">
         <v>0.921</v>
       </c>
-      <c r="AL15" s="2" t="n">
+      <c r="AP15" s="2" t="n">
         <v>0.996</v>
       </c>
-      <c r="AM15" s="2" t="n">
+      <c r="AQ15" s="2" t="n">
         <v>1.023</v>
       </c>
-      <c r="AN15" s="2" t="n">
+      <c r="AR15" s="2" t="n">
         <v>1.037</v>
       </c>
-      <c r="AO15" s="2" t="n">
+      <c r="AS15" s="2" t="n">
         <v>1.048</v>
       </c>
-      <c r="AP15" s="2" t="n">
+      <c r="AT15" s="2" t="n">
         <v>1.009</v>
       </c>
-      <c r="AQ15" s="2" t="n">
+      <c r="AU15" s="2" t="n">
         <v>1.044</v>
       </c>
-      <c r="AR15" s="2" t="n">
+      <c r="AV15" s="2" t="n">
         <v>-3.2861</v>
       </c>
-      <c r="AS15" s="2" t="n">
+      <c r="AW15" s="2" t="n">
         <v>-1.6658</v>
       </c>
-      <c r="AT15" s="2" t="n">
+      <c r="AX15" s="2" t="n">
         <v>-0.4348</v>
       </c>
-      <c r="AU15" s="2" t="n">
+      <c r="AY15" s="2" t="n">
         <v>-0.3075</v>
       </c>
-      <c r="AV15" s="2" t="n">
+      <c r="AZ15" s="2" t="n">
         <v>-0.1854</v>
       </c>
     </row>
@@ -2527,73 +2695,83 @@
           <t>0000000100</t>
         </is>
       </c>
-      <c r="V16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="W16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="n">
+        <v>42</v>
+      </c>
       <c r="X16" s="2" t="inlineStr"/>
       <c r="Y16" s="2" t="inlineStr"/>
       <c r="Z16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA16" s="2" t="inlineStr"/>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="n">
         <v>-12.33</v>
       </c>
-      <c r="AA16" s="2" t="n">
+      <c r="AE16" s="2" t="n">
         <v>-9.880000000000001</v>
       </c>
-      <c r="AB16" s="2" t="n">
+      <c r="AF16" s="2" t="n">
         <v>-2.19</v>
       </c>
-      <c r="AC16" s="2" t="n">
+      <c r="AG16" s="2" t="n">
         <v>-1.55</v>
       </c>
-      <c r="AD16" s="2" t="n">
+      <c r="AH16" s="2" t="n">
         <v>30.8</v>
       </c>
-      <c r="AE16" s="2" t="n">
+      <c r="AI16" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="AF16" s="2" t="inlineStr"/>
-      <c r="AG16" s="2" t="inlineStr"/>
-      <c r="AH16" s="2" t="inlineStr"/>
-      <c r="AI16" s="2" t="inlineStr"/>
-      <c r="AJ16" s="2" t="inlineStr">
+      <c r="AJ16" s="2" t="inlineStr"/>
+      <c r="AK16" s="2" t="inlineStr"/>
+      <c r="AL16" s="2" t="inlineStr"/>
+      <c r="AM16" s="2" t="inlineStr"/>
+      <c r="AN16" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK16" s="2" t="n">
+      <c r="AO16" s="2" t="n">
         <v>1.084</v>
       </c>
-      <c r="AL16" s="2" t="n">
+      <c r="AP16" s="2" t="n">
         <v>1.107</v>
       </c>
-      <c r="AM16" s="2" t="n">
-        <v>1.134</v>
-      </c>
-      <c r="AN16" s="2" t="n">
+      <c r="AQ16" s="2" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="AR16" s="2" t="n">
         <v>1.132</v>
       </c>
-      <c r="AO16" s="2" t="n">
+      <c r="AS16" s="2" t="n">
         <v>1.129</v>
       </c>
-      <c r="AP16" s="2" t="n">
+      <c r="AT16" s="2" t="n">
         <v>1.187</v>
       </c>
-      <c r="AQ16" s="2" t="n">
+      <c r="AU16" s="2" t="n">
         <v>1.3</v>
       </c>
-      <c r="AR16" s="2" t="n">
+      <c r="AV16" s="2" t="n">
         <v>-1.59</v>
       </c>
-      <c r="AS16" s="2" t="n">
+      <c r="AW16" s="2" t="n">
         <v>-0.6881</v>
       </c>
-      <c r="AT16" s="2" t="n">
+      <c r="AX16" s="2" t="n">
         <v>-0.034</v>
       </c>
-      <c r="AU16" s="2" t="n">
+      <c r="AY16" s="2" t="n">
         <v>-0.7877</v>
       </c>
-      <c r="AV16" s="2" t="n">
+      <c r="AZ16" s="2" t="n">
         <v>-0.1233</v>
       </c>
     </row>
@@ -2647,77 +2825,87 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V17" s="2" t="n">
-        <v>-1</v>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="X17" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="X17" s="2" t="inlineStr"/>
       <c r="Y17" s="2" t="inlineStr"/>
       <c r="Z17" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA17" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="2" t="inlineStr"/>
+      <c r="AD17" s="2" t="n">
         <v>-52.49</v>
       </c>
-      <c r="AA17" s="2" t="n">
+      <c r="AE17" s="2" t="n">
         <v>-7.97</v>
       </c>
-      <c r="AB17" s="2" t="n">
+      <c r="AF17" s="2" t="n">
         <v>4.54</v>
       </c>
-      <c r="AC17" s="2" t="n">
+      <c r="AG17" s="2" t="n">
         <v>5.09</v>
       </c>
-      <c r="AD17" s="2" t="n">
+      <c r="AH17" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="AE17" s="2" t="n">
+      <c r="AI17" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="AF17" s="2" t="inlineStr"/>
-      <c r="AG17" s="2" t="inlineStr"/>
-      <c r="AH17" s="2" t="inlineStr"/>
-      <c r="AI17" s="2" t="inlineStr"/>
-      <c r="AJ17" s="2" t="inlineStr">
+      <c r="AJ17" s="2" t="inlineStr"/>
+      <c r="AK17" s="2" t="inlineStr"/>
+      <c r="AL17" s="2" t="inlineStr"/>
+      <c r="AM17" s="2" t="inlineStr"/>
+      <c r="AN17" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK17" s="2" t="n">
+      <c r="AO17" s="2" t="n">
         <v>0.975</v>
       </c>
-      <c r="AL17" s="2" t="n">
+      <c r="AP17" s="2" t="n">
         <v>1.034</v>
       </c>
-      <c r="AM17" s="2" t="n">
+      <c r="AQ17" s="2" t="n">
         <v>1.071</v>
       </c>
-      <c r="AN17" s="2" t="n">
+      <c r="AR17" s="2" t="n">
         <v>1.091</v>
       </c>
-      <c r="AO17" s="2" t="n">
+      <c r="AS17" s="2" t="n">
         <v>1.121</v>
       </c>
-      <c r="AP17" s="2" t="n">
+      <c r="AT17" s="2" t="n">
         <v>1.121</v>
       </c>
-      <c r="AQ17" s="2" t="n">
+      <c r="AU17" s="2" t="n">
         <v>1.25</v>
       </c>
-      <c r="AR17" s="2" t="n">
+      <c r="AV17" s="2" t="n">
         <v>-2.8569</v>
       </c>
-      <c r="AS17" s="2" t="n">
+      <c r="AW17" s="2" t="n">
         <v>-1.9494</v>
       </c>
-      <c r="AT17" s="2" t="n">
+      <c r="AX17" s="2" t="n">
         <v>-0.7037</v>
       </c>
-      <c r="AU17" s="2" t="n">
+      <c r="AY17" s="2" t="n">
         <v>-0.6112</v>
       </c>
-      <c r="AV17" s="2" t="n">
+      <c r="AZ17" s="2" t="n">
         <v>-0.5249</v>
       </c>
     </row>
@@ -2769,79 +2957,89 @@
           <t>0000001000</t>
         </is>
       </c>
-      <c r="V18" s="2" t="n">
-        <v>-1</v>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="X18" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="X18" s="2" t="inlineStr"/>
       <c r="Y18" s="2" t="inlineStr"/>
       <c r="Z18" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA18" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AD18" s="2" t="n">
         <v>-8.56</v>
       </c>
-      <c r="AA18" s="2" t="n">
+      <c r="AE18" s="2" t="n">
         <v>17.43</v>
       </c>
-      <c r="AB18" s="2" t="n">
+      <c r="AF18" s="2" t="n">
         <v>5.6</v>
       </c>
-      <c r="AC18" s="2" t="n">
+      <c r="AG18" s="2" t="n">
         <v>9.08</v>
       </c>
-      <c r="AD18" s="2" t="n">
+      <c r="AH18" s="2" t="n">
         <v>97.90000000000001</v>
       </c>
-      <c r="AE18" s="2" t="n">
+      <c r="AI18" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="AF18" s="2" t="inlineStr"/>
-      <c r="AG18" s="2" t="inlineStr"/>
-      <c r="AH18" s="2" t="n">
+      <c r="AJ18" s="2" t="inlineStr"/>
+      <c r="AK18" s="2" t="inlineStr"/>
+      <c r="AL18" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AI18" s="2" t="inlineStr"/>
-      <c r="AJ18" s="2" t="inlineStr">
+      <c r="AM18" s="2" t="inlineStr"/>
+      <c r="AN18" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK18" s="2" t="n">
+      <c r="AO18" s="2" t="n">
         <v>1.544</v>
       </c>
-      <c r="AL18" s="2" t="n">
+      <c r="AP18" s="2" t="n">
         <v>1.609</v>
       </c>
-      <c r="AM18" s="2" t="n">
+      <c r="AQ18" s="2" t="n">
         <v>1.647</v>
       </c>
-      <c r="AN18" s="2" t="n">
+      <c r="AR18" s="2" t="n">
         <v>1.653</v>
       </c>
-      <c r="AO18" s="2" t="n">
+      <c r="AS18" s="2" t="n">
         <v>1.641</v>
       </c>
-      <c r="AP18" s="2" t="n">
+      <c r="AT18" s="2" t="n">
         <v>1.596</v>
       </c>
-      <c r="AQ18" s="2" t="n">
+      <c r="AU18" s="2" t="n">
         <v>1.593</v>
       </c>
-      <c r="AR18" s="2" t="n">
+      <c r="AV18" s="2" t="n">
         <v>-2.0521</v>
       </c>
-      <c r="AS18" s="2" t="n">
+      <c r="AW18" s="2" t="n">
         <v>-1.0836</v>
       </c>
-      <c r="AT18" s="2" t="n">
+      <c r="AX18" s="2" t="n">
         <v>-0.175</v>
       </c>
-      <c r="AU18" s="2" t="n">
+      <c r="AY18" s="2" t="n">
         <v>-0.0309</v>
       </c>
-      <c r="AV18" s="2" t="n">
+      <c r="AZ18" s="2" t="n">
         <v>-0.0856</v>
       </c>
     </row>
@@ -2897,75 +3095,85 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V19" s="2" t="n">
-        <v>1</v>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="W19" s="2" t="n">
-        <v>1</v>
+        <v>138</v>
       </c>
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="2" t="inlineStr"/>
       <c r="Z19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AD19" s="2" t="n">
         <v>-56.32</v>
       </c>
-      <c r="AA19" s="2" t="n">
+      <c r="AE19" s="2" t="n">
         <v>-15.69</v>
       </c>
-      <c r="AB19" s="2" t="n">
+      <c r="AF19" s="2" t="n">
         <v>1.02</v>
       </c>
-      <c r="AC19" s="2" t="n">
+      <c r="AG19" s="2" t="n">
         <v>3.85</v>
       </c>
-      <c r="AD19" s="2" t="n">
+      <c r="AH19" s="2" t="n">
         <v>26.4</v>
       </c>
-      <c r="AE19" s="2" t="n">
+      <c r="AI19" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="AF19" s="2" t="inlineStr"/>
-      <c r="AG19" s="2" t="inlineStr"/>
-      <c r="AH19" s="2" t="inlineStr"/>
-      <c r="AI19" s="2" t="inlineStr"/>
-      <c r="AJ19" s="2" t="inlineStr">
+      <c r="AJ19" s="2" t="inlineStr"/>
+      <c r="AK19" s="2" t="inlineStr"/>
+      <c r="AL19" s="2" t="inlineStr"/>
+      <c r="AM19" s="2" t="inlineStr"/>
+      <c r="AN19" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK19" s="2" t="n">
+      <c r="AO19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AL19" s="2" t="n">
+      <c r="AP19" s="2" t="n">
         <v>1.013</v>
       </c>
-      <c r="AM19" s="2" t="n">
+      <c r="AQ19" s="2" t="n">
         <v>1.016</v>
       </c>
-      <c r="AN19" s="2" t="n">
+      <c r="AR19" s="2" t="n">
         <v>1.032</v>
       </c>
-      <c r="AO19" s="2" t="n">
+      <c r="AS19" s="2" t="n">
         <v>1.074</v>
       </c>
-      <c r="AP19" s="2" t="n">
+      <c r="AT19" s="2" t="n">
         <v>1.079</v>
       </c>
-      <c r="AQ19" s="2" t="n">
+      <c r="AU19" s="2" t="n">
         <v>1.214</v>
       </c>
-      <c r="AR19" s="2" t="n">
+      <c r="AV19" s="2" t="n">
         <v>-0.4378</v>
       </c>
-      <c r="AS19" s="2" t="n">
+      <c r="AW19" s="2" t="n">
         <v>-0.6319</v>
       </c>
-      <c r="AT19" s="2" t="n">
+      <c r="AX19" s="2" t="n">
         <v>-0.4446</v>
       </c>
-      <c r="AU19" s="2" t="n">
+      <c r="AY19" s="2" t="n">
         <v>-0.4934</v>
       </c>
-      <c r="AV19" s="2" t="n">
+      <c r="AZ19" s="2" t="n">
         <v>-0.5632</v>
       </c>
     </row>
@@ -3021,73 +3229,83 @@
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="W20" s="2" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="n">
+        <v>17</v>
+      </c>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
-      <c r="Z20" s="2" t="n">
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr"/>
+      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="n">
         <v>-21.72</v>
       </c>
-      <c r="AA20" s="2" t="n">
+      <c r="AE20" s="2" t="n">
         <v>-2.68</v>
       </c>
-      <c r="AB20" s="2" t="n">
+      <c r="AF20" s="2" t="n">
         <v>1.11</v>
       </c>
-      <c r="AC20" s="2" t="n">
+      <c r="AG20" s="2" t="n">
         <v>-1.17</v>
       </c>
-      <c r="AD20" s="2" t="n">
+      <c r="AH20" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="AE20" s="2" t="n">
+      <c r="AI20" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="AF20" s="2" t="inlineStr"/>
-      <c r="AG20" s="2" t="inlineStr"/>
-      <c r="AH20" s="2" t="inlineStr"/>
-      <c r="AI20" s="2" t="inlineStr"/>
-      <c r="AJ20" s="2" t="inlineStr">
+      <c r="AJ20" s="2" t="inlineStr"/>
+      <c r="AK20" s="2" t="inlineStr"/>
+      <c r="AL20" s="2" t="inlineStr"/>
+      <c r="AM20" s="2" t="inlineStr"/>
+      <c r="AN20" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK20" s="2" t="n">
+      <c r="AO20" s="2" t="n">
         <v>1.738</v>
       </c>
-      <c r="AL20" s="2" t="n">
+      <c r="AP20" s="2" t="n">
         <v>1.76</v>
       </c>
-      <c r="AM20" s="2" t="n">
+      <c r="AQ20" s="2" t="n">
         <v>1.787</v>
       </c>
-      <c r="AN20" s="2" t="n">
+      <c r="AR20" s="2" t="n">
         <v>1.819</v>
       </c>
-      <c r="AO20" s="2" t="n">
+      <c r="AS20" s="2" t="n">
         <v>1.823</v>
       </c>
-      <c r="AP20" s="2" t="n">
+      <c r="AT20" s="2" t="n">
         <v>1.813</v>
       </c>
-      <c r="AQ20" s="2" t="n">
+      <c r="AU20" s="2" t="n">
         <v>1.88</v>
       </c>
-      <c r="AR20" s="2" t="n">
+      <c r="AV20" s="2" t="n">
         <v>-0.8143</v>
       </c>
-      <c r="AS20" s="2" t="n">
+      <c r="AW20" s="2" t="n">
         <v>-1.0327</v>
       </c>
-      <c r="AT20" s="2" t="n">
+      <c r="AX20" s="2" t="n">
         <v>-0.3636</v>
       </c>
-      <c r="AU20" s="2" t="n">
+      <c r="AY20" s="2" t="n">
         <v>-0.159</v>
       </c>
-      <c r="AV20" s="2" t="n">
+      <c r="AZ20" s="2" t="n">
         <v>-0.2172</v>
       </c>
     </row>
@@ -3143,77 +3361,87 @@
           <t>0000001000</t>
         </is>
       </c>
-      <c r="V21" s="2" t="n">
-        <v>-1</v>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="X21" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="X21" s="2" t="inlineStr"/>
       <c r="Y21" s="2" t="inlineStr"/>
       <c r="Z21" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA21" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB21" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC21" s="2" t="inlineStr"/>
+      <c r="AD21" s="2" t="n">
         <v>3.17</v>
       </c>
-      <c r="AA21" s="2" t="n">
+      <c r="AE21" s="2" t="n">
         <v>30.24</v>
       </c>
-      <c r="AB21" s="2" t="n">
+      <c r="AF21" s="2" t="n">
         <v>5.79</v>
       </c>
-      <c r="AC21" s="2" t="n">
+      <c r="AG21" s="2" t="n">
         <v>13.72</v>
       </c>
-      <c r="AD21" s="2" t="n">
+      <c r="AH21" s="2" t="n">
         <v>80.5</v>
       </c>
-      <c r="AE21" s="2" t="n">
+      <c r="AI21" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="AF21" s="2" t="inlineStr"/>
-      <c r="AG21" s="2" t="inlineStr"/>
-      <c r="AH21" s="2" t="inlineStr"/>
-      <c r="AI21" s="2" t="inlineStr"/>
-      <c r="AJ21" s="2" t="inlineStr">
+      <c r="AJ21" s="2" t="inlineStr"/>
+      <c r="AK21" s="2" t="inlineStr"/>
+      <c r="AL21" s="2" t="inlineStr"/>
+      <c r="AM21" s="2" t="inlineStr"/>
+      <c r="AN21" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK21" s="2" t="n">
+      <c r="AO21" s="2" t="n">
         <v>10.003</v>
       </c>
-      <c r="AL21" s="2" t="n">
+      <c r="AP21" s="2" t="n">
         <v>10.799</v>
       </c>
-      <c r="AM21" s="2" t="n">
+      <c r="AQ21" s="2" t="n">
         <v>10.967</v>
       </c>
-      <c r="AN21" s="2" t="n">
+      <c r="AR21" s="2" t="n">
         <v>11.007</v>
       </c>
-      <c r="AO21" s="2" t="n">
+      <c r="AS21" s="2" t="n">
         <v>10.993</v>
       </c>
-      <c r="AP21" s="2" t="n">
+      <c r="AT21" s="2" t="n">
         <v>10.951</v>
       </c>
-      <c r="AQ21" s="2" t="n">
+      <c r="AU21" s="2" t="n">
         <v>10.142</v>
       </c>
-      <c r="AR21" s="2" t="n">
+      <c r="AV21" s="2" t="n">
         <v>-2.7091</v>
       </c>
-      <c r="AS21" s="2" t="n">
+      <c r="AW21" s="2" t="n">
         <v>-1.2528</v>
       </c>
-      <c r="AT21" s="2" t="n">
+      <c r="AX21" s="2" t="n">
         <v>-0.2888</v>
       </c>
-      <c r="AU21" s="2" t="n">
+      <c r="AY21" s="2" t="n">
         <v>-0.1156</v>
       </c>
-      <c r="AV21" s="2" t="n">
+      <c r="AZ21" s="2" t="n">
         <v>0.0317</v>
       </c>
     </row>
@@ -3273,77 +3501,87 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V22" s="2" t="n">
-        <v>-1</v>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-1</v>
+        <v>50</v>
       </c>
       <c r="X22" s="2" t="inlineStr"/>
       <c r="Y22" s="2" t="inlineStr"/>
       <c r="Z22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AD22" s="2" t="n">
         <v>-24.86</v>
       </c>
-      <c r="AA22" s="2" t="n">
+      <c r="AE22" s="2" t="n">
         <v>-13.02</v>
       </c>
-      <c r="AB22" s="2" t="n">
+      <c r="AF22" s="2" t="n">
         <v>1.88</v>
       </c>
-      <c r="AC22" s="2" t="n">
+      <c r="AG22" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD22" s="2" t="n">
+      <c r="AH22" s="2" t="n">
         <v>1.4</v>
       </c>
-      <c r="AE22" s="2" t="n">
+      <c r="AI22" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="AF22" s="2" t="inlineStr"/>
-      <c r="AG22" s="2" t="n">
+      <c r="AJ22" s="2" t="inlineStr"/>
+      <c r="AK22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AH22" s="2" t="inlineStr"/>
-      <c r="AI22" s="2" t="inlineStr"/>
-      <c r="AJ22" s="2" t="inlineStr">
+      <c r="AL22" s="2" t="inlineStr"/>
+      <c r="AM22" s="2" t="inlineStr"/>
+      <c r="AN22" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AK22" s="2" t="n">
+      <c r="AO22" s="2" t="n">
         <v>1.446</v>
       </c>
-      <c r="AL22" s="2" t="n">
+      <c r="AP22" s="2" t="n">
         <v>1.46</v>
       </c>
-      <c r="AM22" s="2" t="n">
+      <c r="AQ22" s="2" t="n">
         <v>1.482</v>
       </c>
-      <c r="AN22" s="2" t="n">
+      <c r="AR22" s="2" t="n">
         <v>1.52</v>
       </c>
-      <c r="AO22" s="2" t="n">
+      <c r="AS22" s="2" t="n">
         <v>1.57</v>
       </c>
-      <c r="AP22" s="2" t="n">
+      <c r="AT22" s="2" t="n">
         <v>1.7</v>
       </c>
-      <c r="AQ22" s="2" t="n">
+      <c r="AU22" s="2" t="n">
         <v>1.804</v>
       </c>
-      <c r="AR22" s="2" t="n">
+      <c r="AV22" s="2" t="n">
         <v>-0.8032</v>
       </c>
-      <c r="AS22" s="2" t="n">
+      <c r="AW22" s="2" t="n">
         <v>-1.0482</v>
       </c>
-      <c r="AT22" s="2" t="n">
+      <c r="AX22" s="2" t="n">
         <v>-0.446</v>
       </c>
-      <c r="AU22" s="2" t="n">
+      <c r="AY22" s="2" t="n">
         <v>-0.957</v>
       </c>
-      <c r="AV22" s="2" t="n">
+      <c r="AZ22" s="2" t="n">
         <v>-0.2486</v>
       </c>
     </row>
@@ -3395,73 +3633,83 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V23" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="W23" s="2" t="inlineStr"/>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="2" t="inlineStr"/>
       <c r="Z23" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA23" s="2" t="inlineStr"/>
+      <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="inlineStr"/>
+      <c r="AD23" s="2" t="n">
         <v>6.3</v>
       </c>
-      <c r="AA23" s="2" t="n">
+      <c r="AE23" s="2" t="n">
         <v>16.85</v>
       </c>
-      <c r="AB23" s="2" t="n">
+      <c r="AF23" s="2" t="n">
         <v>1.77</v>
       </c>
-      <c r="AC23" s="2" t="n">
+      <c r="AG23" s="2" t="n">
         <v>2.58</v>
       </c>
-      <c r="AD23" s="2" t="n">
+      <c r="AH23" s="2" t="n">
         <v>67.3</v>
       </c>
-      <c r="AE23" s="2" t="n">
+      <c r="AI23" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="AF23" s="2" t="inlineStr"/>
-      <c r="AG23" s="2" t="inlineStr"/>
-      <c r="AH23" s="2" t="inlineStr"/>
-      <c r="AI23" s="2" t="inlineStr"/>
-      <c r="AJ23" s="2" t="inlineStr">
+      <c r="AJ23" s="2" t="inlineStr"/>
+      <c r="AK23" s="2" t="inlineStr"/>
+      <c r="AL23" s="2" t="inlineStr"/>
+      <c r="AM23" s="2" t="inlineStr"/>
+      <c r="AN23" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AK23" s="2" t="n">
+      <c r="AO23" s="2" t="n">
         <v>2.647</v>
       </c>
-      <c r="AL23" s="2" t="n">
+      <c r="AP23" s="2" t="n">
         <v>2.803</v>
       </c>
-      <c r="AM23" s="2" t="n">
+      <c r="AQ23" s="2" t="n">
         <v>2.905</v>
       </c>
-      <c r="AN23" s="2" t="n">
+      <c r="AR23" s="2" t="n">
         <v>2.965</v>
       </c>
-      <c r="AO23" s="2" t="n">
+      <c r="AS23" s="2" t="n">
         <v>2.933</v>
       </c>
-      <c r="AP23" s="2" t="n">
+      <c r="AT23" s="2" t="n">
         <v>2.883</v>
       </c>
-      <c r="AQ23" s="2" t="n">
+      <c r="AU23" s="2" t="n">
         <v>2.809</v>
       </c>
-      <c r="AR23" s="2" t="n">
+      <c r="AV23" s="2" t="n">
         <v>-2.7547</v>
       </c>
-      <c r="AS23" s="2" t="n">
+      <c r="AW23" s="2" t="n">
         <v>-1.7257</v>
       </c>
-      <c r="AT23" s="2" t="n">
+      <c r="AX23" s="2" t="n">
         <v>-0.3003</v>
       </c>
-      <c r="AU23" s="2" t="n">
+      <c r="AY23" s="2" t="n">
         <v>-0.2109</v>
       </c>
-      <c r="AV23" s="2" t="n">
+      <c r="AZ23" s="2" t="n">
         <v>0.063</v>
       </c>
     </row>
@@ -3525,75 +3773,85 @@
       </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="W24" s="2" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="n">
+        <v>52</v>
+      </c>
       <c r="X24" s="2" t="inlineStr"/>
       <c r="Y24" s="2" t="inlineStr"/>
-      <c r="Z24" s="2" t="n">
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AA24" s="2" t="inlineStr"/>
+      <c r="AB24" s="2" t="inlineStr"/>
+      <c r="AC24" s="2" t="inlineStr"/>
+      <c r="AD24" s="2" t="n">
         <v>-25.36</v>
       </c>
-      <c r="AA24" s="2" t="n">
+      <c r="AE24" s="2" t="n">
         <v>-15.72</v>
       </c>
-      <c r="AB24" s="2" t="n">
+      <c r="AF24" s="2" t="n">
         <v>-0.01</v>
       </c>
-      <c r="AC24" s="2" t="n">
+      <c r="AG24" s="2" t="n">
         <v>0.57</v>
       </c>
-      <c r="AD24" s="2" t="n">
+      <c r="AH24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AE24" s="2" t="n">
+      <c r="AI24" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="AF24" s="2" t="inlineStr"/>
-      <c r="AG24" s="2" t="n">
+      <c r="AJ24" s="2" t="inlineStr"/>
+      <c r="AK24" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="AH24" s="2" t="inlineStr"/>
-      <c r="AI24" s="2" t="inlineStr"/>
-      <c r="AJ24" s="2" t="inlineStr">
+      <c r="AL24" s="2" t="inlineStr"/>
+      <c r="AM24" s="2" t="inlineStr"/>
+      <c r="AN24" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AK24" s="2" t="n">
+      <c r="AO24" s="2" t="n">
         <v>0.763</v>
       </c>
-      <c r="AL24" s="2" t="n">
+      <c r="AP24" s="2" t="n">
         <v>0.778</v>
       </c>
-      <c r="AM24" s="2" t="n">
+      <c r="AQ24" s="2" t="n">
         <v>0.791</v>
       </c>
-      <c r="AN24" s="2" t="n">
+      <c r="AR24" s="2" t="n">
         <v>0.804</v>
       </c>
-      <c r="AO24" s="2" t="n">
+      <c r="AS24" s="2" t="n">
         <v>0.822</v>
       </c>
-      <c r="AP24" s="2" t="n">
+      <c r="AT24" s="2" t="n">
         <v>0.903</v>
       </c>
-      <c r="AQ24" s="2" t="n">
+      <c r="AU24" s="2" t="n">
         <v>0.986</v>
       </c>
-      <c r="AR24" s="2" t="n">
+      <c r="AV24" s="2" t="n">
         <v>-1.2839</v>
       </c>
-      <c r="AS24" s="2" t="n">
+      <c r="AW24" s="2" t="n">
         <v>-0.8214</v>
       </c>
-      <c r="AT24" s="2" t="n">
+      <c r="AX24" s="2" t="n">
         <v>-0.3755</v>
       </c>
-      <c r="AU24" s="2" t="n">
+      <c r="AY24" s="2" t="n">
         <v>-1.0223</v>
       </c>
-      <c r="AV24" s="2" t="n">
+      <c r="AZ24" s="2" t="n">
         <v>-0.2536</v>
       </c>
     </row>
@@ -3647,73 +3905,83 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V25" s="2" t="inlineStr"/>
-      <c r="W25" s="2" t="inlineStr"/>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="2" t="inlineStr"/>
-      <c r="Z25" s="2" t="n">
+      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="AA25" s="2" t="inlineStr"/>
+      <c r="AB25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AD25" s="2" t="n">
         <v>1.58</v>
       </c>
-      <c r="AA25" s="2" t="n">
+      <c r="AE25" s="2" t="n">
         <v>1.79</v>
       </c>
-      <c r="AB25" s="2" t="n">
+      <c r="AF25" s="2" t="n">
         <v>-11.14</v>
       </c>
-      <c r="AC25" s="2" t="n">
+      <c r="AG25" s="2" t="n">
         <v>-11.15</v>
       </c>
-      <c r="AD25" s="2" t="n">
+      <c r="AH25" s="2" t="n">
         <v>16.7</v>
       </c>
-      <c r="AE25" s="2" t="n">
+      <c r="AI25" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AF25" s="2" t="inlineStr"/>
-      <c r="AG25" s="2" t="n">
+      <c r="AJ25" s="2" t="inlineStr"/>
+      <c r="AK25" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AH25" s="2" t="inlineStr"/>
-      <c r="AI25" s="2" t="inlineStr"/>
-      <c r="AJ25" s="2" t="inlineStr">
+      <c r="AL25" s="2" t="inlineStr"/>
+      <c r="AM25" s="2" t="inlineStr"/>
+      <c r="AN25" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK25" s="2" t="n">
+      <c r="AO25" s="2" t="n">
         <v>2.962</v>
       </c>
-      <c r="AL25" s="2" t="n">
+      <c r="AP25" s="2" t="n">
         <v>3.487</v>
       </c>
-      <c r="AM25" s="2" t="n">
+      <c r="AQ25" s="2" t="n">
         <v>3.78</v>
       </c>
-      <c r="AN25" s="2" t="n">
+      <c r="AR25" s="2" t="n">
         <v>3.837</v>
       </c>
-      <c r="AO25" s="2" t="n">
+      <c r="AS25" s="2" t="n">
         <v>3.849</v>
       </c>
-      <c r="AP25" s="2" t="n">
+      <c r="AT25" s="2" t="n">
         <v>4.303</v>
       </c>
-      <c r="AQ25" s="2" t="n">
+      <c r="AU25" s="2" t="n">
         <v>3.846</v>
       </c>
-      <c r="AR25" s="2" t="n">
+      <c r="AV25" s="2" t="n">
         <v>-7.4419</v>
       </c>
-      <c r="AS25" s="2" t="n">
+      <c r="AW25" s="2" t="n">
         <v>-3.1136</v>
       </c>
-      <c r="AT25" s="2" t="n">
+      <c r="AX25" s="2" t="n">
         <v>-1.3986</v>
       </c>
-      <c r="AU25" s="2" t="n">
+      <c r="AY25" s="2" t="n">
         <v>-0.9429999999999999</v>
       </c>
-      <c r="AV25" s="2" t="n">
+      <c r="AZ25" s="2" t="n">
         <v>0.0158</v>
       </c>
     </row>
@@ -3777,81 +4045,91 @@
           <t>1111110101</t>
         </is>
       </c>
-      <c r="V26" s="2" t="n">
-        <v>1</v>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="W26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="X26" s="2" t="n">
+      <c r="X26" s="2" t="inlineStr"/>
+      <c r="Y26" s="2" t="inlineStr"/>
+      <c r="Z26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="Y26" s="2" t="n">
+      <c r="AC26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Z26" s="2" t="n">
+      <c r="AD26" s="2" t="n">
         <v>17.47</v>
       </c>
-      <c r="AA26" s="2" t="n">
+      <c r="AE26" s="2" t="n">
         <v>-15</v>
       </c>
-      <c r="AB26" s="2" t="n">
+      <c r="AF26" s="2" t="n">
         <v>1.78</v>
       </c>
-      <c r="AC26" s="2" t="n">
+      <c r="AG26" s="2" t="n">
         <v>0.44</v>
       </c>
-      <c r="AD26" s="2" t="n">
+      <c r="AH26" s="2" t="n">
         <v>-0.3</v>
       </c>
-      <c r="AE26" s="2" t="n">
+      <c r="AI26" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="AF26" s="2" t="inlineStr"/>
-      <c r="AG26" s="2" t="n">
+      <c r="AJ26" s="2" t="inlineStr"/>
+      <c r="AK26" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="AH26" s="2" t="inlineStr"/>
-      <c r="AI26" s="2" t="inlineStr"/>
-      <c r="AJ26" s="2" t="inlineStr">
+      <c r="AL26" s="2" t="inlineStr"/>
+      <c r="AM26" s="2" t="inlineStr"/>
+      <c r="AN26" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AK26" s="2" t="n">
+      <c r="AO26" s="2" t="n">
         <v>0.987</v>
       </c>
-      <c r="AL26" s="2" t="n">
+      <c r="AP26" s="2" t="n">
         <v>0.844</v>
       </c>
-      <c r="AM26" s="2" t="n">
+      <c r="AQ26" s="2" t="n">
         <v>0.781</v>
       </c>
-      <c r="AN26" s="2" t="n">
+      <c r="AR26" s="2" t="n">
         <v>0.771</v>
       </c>
-      <c r="AO26" s="2" t="n">
+      <c r="AS26" s="2" t="n">
         <v>0.774</v>
       </c>
-      <c r="AP26" s="2" t="n">
+      <c r="AT26" s="2" t="n">
         <v>0.829</v>
       </c>
-      <c r="AQ26" s="2" t="n">
+      <c r="AU26" s="2" t="n">
         <v>0.887</v>
       </c>
-      <c r="AR26" s="2" t="n">
+      <c r="AV26" s="2" t="n">
         <v>9.9887</v>
       </c>
-      <c r="AS26" s="2" t="n">
+      <c r="AW26" s="2" t="n">
         <v>4.5792</v>
       </c>
-      <c r="AT26" s="2" t="n">
+      <c r="AX26" s="2" t="n">
         <v>1.6276</v>
       </c>
-      <c r="AU26" s="2" t="n">
+      <c r="AY26" s="2" t="n">
         <v>-0.0827</v>
       </c>
-      <c r="AV26" s="2" t="n">
+      <c r="AZ26" s="2" t="n">
         <v>0.1747</v>
       </c>
     </row>
@@ -3905,69 +4183,79 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V27" s="2" t="inlineStr"/>
-      <c r="W27" s="2" t="inlineStr"/>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="X27" s="2" t="inlineStr"/>
       <c r="Y27" s="2" t="inlineStr"/>
-      <c r="Z27" s="2" t="n">
+      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AA27" s="2" t="inlineStr"/>
+      <c r="AB27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="inlineStr"/>
+      <c r="AD27" s="2" t="n">
         <v>-13.95</v>
       </c>
-      <c r="AA27" s="2" t="n">
+      <c r="AE27" s="2" t="n">
         <v>-10.34</v>
       </c>
-      <c r="AB27" s="2" t="n">
+      <c r="AF27" s="2" t="n">
         <v>-4.3</v>
       </c>
-      <c r="AC27" s="2" t="n">
+      <c r="AG27" s="2" t="n">
         <v>-3.76</v>
       </c>
-      <c r="AD27" s="2" t="n">
+      <c r="AH27" s="2" t="n">
         <v>-4</v>
       </c>
-      <c r="AE27" s="2" t="inlineStr"/>
-      <c r="AF27" s="2" t="inlineStr"/>
-      <c r="AG27" s="2" t="inlineStr"/>
-      <c r="AH27" s="2" t="inlineStr"/>
       <c r="AI27" s="2" t="inlineStr"/>
-      <c r="AJ27" s="2" t="inlineStr">
+      <c r="AJ27" s="2" t="inlineStr"/>
+      <c r="AK27" s="2" t="inlineStr"/>
+      <c r="AL27" s="2" t="inlineStr"/>
+      <c r="AM27" s="2" t="inlineStr"/>
+      <c r="AN27" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AK27" s="2" t="n">
+      <c r="AO27" s="2" t="n">
         <v>0.86</v>
       </c>
-      <c r="AL27" s="2" t="n">
+      <c r="AP27" s="2" t="n">
         <v>0.888</v>
       </c>
-      <c r="AM27" s="2" t="n">
+      <c r="AQ27" s="2" t="n">
         <v>0.906</v>
       </c>
-      <c r="AN27" s="2" t="n">
+      <c r="AR27" s="2" t="n">
         <v>0.922</v>
       </c>
-      <c r="AO27" s="2" t="n">
+      <c r="AS27" s="2" t="n">
         <v>0.946</v>
       </c>
-      <c r="AP27" s="2" t="n">
+      <c r="AT27" s="2" t="n">
         <v>1.028</v>
       </c>
-      <c r="AQ27" s="2" t="n">
+      <c r="AU27" s="2" t="n">
         <v>1.026</v>
       </c>
-      <c r="AR27" s="2" t="n">
+      <c r="AV27" s="2" t="n">
         <v>-1.7218</v>
       </c>
-      <c r="AS27" s="2" t="n">
+      <c r="AW27" s="2" t="n">
         <v>-1.2844</v>
       </c>
-      <c r="AT27" s="2" t="n">
+      <c r="AX27" s="2" t="n">
         <v>-0.5042</v>
       </c>
-      <c r="AU27" s="2" t="n">
+      <c r="AY27" s="2" t="n">
         <v>-0.7079</v>
       </c>
-      <c r="AV27" s="2" t="n">
+      <c r="AZ27" s="2" t="n">
         <v>-0.1395</v>
       </c>
     </row>
@@ -4021,75 +4309,85 @@
       </c>
       <c r="V28" s="2" t="inlineStr">
         <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="W28" s="2" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="inlineStr"/>
-      <c r="Z28" s="2" t="n">
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr"/>
+      <c r="AB28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="inlineStr"/>
+      <c r="AD28" s="2" t="n">
         <v>10.42</v>
       </c>
-      <c r="AA28" s="2" t="n">
+      <c r="AE28" s="2" t="n">
         <v>0.66</v>
       </c>
-      <c r="AB28" s="2" t="n">
+      <c r="AF28" s="2" t="n">
         <v>-8.119999999999999</v>
       </c>
-      <c r="AC28" s="2" t="n">
+      <c r="AG28" s="2" t="n">
         <v>-6.05</v>
       </c>
-      <c r="AD28" s="2" t="n">
+      <c r="AH28" s="2" t="n">
         <v>-5.3</v>
       </c>
-      <c r="AE28" s="2" t="n">
+      <c r="AI28" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AF28" s="2" t="inlineStr"/>
-      <c r="AG28" s="2" t="n">
+      <c r="AJ28" s="2" t="inlineStr"/>
+      <c r="AK28" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AH28" s="2" t="inlineStr"/>
-      <c r="AI28" s="2" t="inlineStr"/>
-      <c r="AJ28" s="2" t="inlineStr">
+      <c r="AL28" s="2" t="inlineStr"/>
+      <c r="AM28" s="2" t="inlineStr"/>
+      <c r="AN28" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK28" s="2" t="n">
+      <c r="AO28" s="2" t="n">
         <v>1.541</v>
       </c>
-      <c r="AL28" s="2" t="n">
+      <c r="AP28" s="2" t="n">
         <v>1.623</v>
       </c>
-      <c r="AM28" s="2" t="n">
+      <c r="AQ28" s="2" t="n">
         <v>1.652</v>
       </c>
-      <c r="AN28" s="2" t="n">
+      <c r="AR28" s="2" t="n">
         <v>1.676</v>
       </c>
-      <c r="AO28" s="2" t="n">
+      <c r="AS28" s="2" t="n">
         <v>1.717</v>
       </c>
-      <c r="AP28" s="2" t="n">
+      <c r="AT28" s="2" t="n">
         <v>1.841</v>
       </c>
-      <c r="AQ28" s="2" t="n">
+      <c r="AU28" s="2" t="n">
         <v>1.675</v>
       </c>
-      <c r="AR28" s="2" t="n">
+      <c r="AV28" s="2" t="n">
         <v>-2.5237</v>
       </c>
-      <c r="AS28" s="2" t="n">
+      <c r="AW28" s="2" t="n">
         <v>-1.2551</v>
       </c>
-      <c r="AT28" s="2" t="n">
+      <c r="AX28" s="2" t="n">
         <v>-1.154</v>
       </c>
-      <c r="AU28" s="2" t="n">
+      <c r="AY28" s="2" t="n">
         <v>-0.3888</v>
       </c>
-      <c r="AV28" s="2" t="n">
+      <c r="AZ28" s="2" t="n">
         <v>0.1042</v>
       </c>
     </row>
@@ -4120,7 +4418,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -4141,73 +4439,83 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V29" s="2" t="inlineStr"/>
-      <c r="W29" s="2" t="inlineStr"/>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="n">
+        <v>24</v>
+      </c>
       <c r="X29" s="2" t="inlineStr"/>
       <c r="Y29" s="2" t="inlineStr"/>
-      <c r="Z29" s="2" t="n">
+      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="AA29" s="2" t="inlineStr"/>
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="inlineStr"/>
+      <c r="AD29" s="2" t="n">
         <v>-15.22</v>
       </c>
-      <c r="AA29" s="2" t="n">
+      <c r="AE29" s="2" t="n">
         <v>-7.17</v>
       </c>
-      <c r="AB29" s="2" t="n">
+      <c r="AF29" s="2" t="n">
         <v>-1.57</v>
       </c>
-      <c r="AC29" s="2" t="n">
+      <c r="AG29" s="2" t="n">
         <v>-2.74</v>
       </c>
-      <c r="AD29" s="2" t="n">
+      <c r="AH29" s="2" t="n">
         <v>2.6</v>
       </c>
-      <c r="AE29" s="2" t="n">
+      <c r="AI29" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="AF29" s="2" t="inlineStr"/>
-      <c r="AG29" s="2" t="n">
+      <c r="AJ29" s="2" t="inlineStr"/>
+      <c r="AK29" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="AH29" s="2" t="inlineStr"/>
-      <c r="AI29" s="2" t="inlineStr"/>
-      <c r="AJ29" s="2" t="inlineStr">
+      <c r="AL29" s="2" t="inlineStr"/>
+      <c r="AM29" s="2" t="inlineStr"/>
+      <c r="AN29" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AK29" s="2" t="n">
+      <c r="AO29" s="2" t="n">
         <v>1.148</v>
       </c>
-      <c r="AL29" s="2" t="n">
+      <c r="AP29" s="2" t="n">
         <v>1.19</v>
       </c>
-      <c r="AM29" s="2" t="n">
+      <c r="AQ29" s="2" t="n">
         <v>1.213</v>
       </c>
-      <c r="AN29" s="2" t="n">
+      <c r="AR29" s="2" t="n">
         <v>1.238</v>
       </c>
-      <c r="AO29" s="2" t="n">
+      <c r="AS29" s="2" t="n">
         <v>1.269</v>
       </c>
-      <c r="AP29" s="2" t="n">
+      <c r="AT29" s="2" t="n">
         <v>1.312</v>
       </c>
-      <c r="AQ29" s="2" t="n">
+      <c r="AU29" s="2" t="n">
         <v>1.352</v>
       </c>
-      <c r="AR29" s="2" t="n">
+      <c r="AV29" s="2" t="n">
         <v>-1.8305</v>
       </c>
-      <c r="AS29" s="2" t="n">
+      <c r="AW29" s="2" t="n">
         <v>-1.5088</v>
       </c>
-      <c r="AT29" s="2" t="n">
+      <c r="AX29" s="2" t="n">
         <v>-0.7282999999999999</v>
       </c>
-      <c r="AU29" s="2" t="n">
+      <c r="AY29" s="2" t="n">
         <v>-0.6964</v>
       </c>
-      <c r="AV29" s="2" t="n">
+      <c r="AZ29" s="2" t="n">
         <v>-0.1522</v>
       </c>
     </row>
@@ -4259,73 +4567,83 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V30" s="2" t="inlineStr"/>
-      <c r="W30" s="2" t="inlineStr"/>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="X30" s="2" t="inlineStr"/>
       <c r="Y30" s="2" t="inlineStr"/>
-      <c r="Z30" s="2" t="n">
+      <c r="Z30" s="2" t="inlineStr"/>
+      <c r="AA30" s="2" t="inlineStr"/>
+      <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AD30" s="2" t="n">
         <v>4.43</v>
       </c>
-      <c r="AA30" s="2" t="n">
+      <c r="AE30" s="2" t="n">
         <v>5.08</v>
       </c>
-      <c r="AB30" s="2" t="n">
+      <c r="AF30" s="2" t="n">
         <v>-9.1</v>
       </c>
-      <c r="AC30" s="2" t="n">
+      <c r="AG30" s="2" t="n">
         <v>-6.26</v>
       </c>
-      <c r="AD30" s="2" t="n">
+      <c r="AH30" s="2" t="n">
         <v>-5.5</v>
       </c>
-      <c r="AE30" s="2" t="n">
+      <c r="AI30" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AF30" s="2" t="inlineStr"/>
-      <c r="AG30" s="2" t="n">
+      <c r="AJ30" s="2" t="inlineStr"/>
+      <c r="AK30" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AH30" s="2" t="inlineStr"/>
-      <c r="AI30" s="2" t="inlineStr"/>
-      <c r="AJ30" s="2" t="inlineStr">
+      <c r="AL30" s="2" t="inlineStr"/>
+      <c r="AM30" s="2" t="inlineStr"/>
+      <c r="AN30" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK30" s="2" t="n">
+      <c r="AO30" s="2" t="n">
         <v>3.456</v>
       </c>
-      <c r="AL30" s="2" t="n">
-        <v>3.982</v>
-      </c>
-      <c r="AM30" s="2" t="n">
+      <c r="AP30" s="2" t="n">
+        <v>3.983</v>
+      </c>
+      <c r="AQ30" s="2" t="n">
         <v>4.193</v>
       </c>
-      <c r="AN30" s="2" t="n">
+      <c r="AR30" s="2" t="n">
         <v>4.306</v>
       </c>
-      <c r="AO30" s="2" t="n">
+      <c r="AS30" s="2" t="n">
         <v>4.454</v>
       </c>
-      <c r="AP30" s="2" t="n">
+      <c r="AT30" s="2" t="n">
         <v>4.893</v>
       </c>
-      <c r="AQ30" s="2" t="n">
+      <c r="AU30" s="2" t="n">
         <v>4.293</v>
       </c>
-      <c r="AR30" s="2" t="n">
+      <c r="AV30" s="2" t="n">
         <v>-5.9595</v>
       </c>
-      <c r="AS30" s="2" t="n">
+      <c r="AW30" s="2" t="n">
         <v>-2.9498</v>
       </c>
-      <c r="AT30" s="2" t="n">
+      <c r="AX30" s="2" t="n">
         <v>-1.8791</v>
       </c>
-      <c r="AU30" s="2" t="n">
+      <c r="AY30" s="2" t="n">
         <v>-0.6089</v>
       </c>
-      <c r="AV30" s="2" t="n">
+      <c r="AZ30" s="2" t="n">
         <v>0.0443</v>
       </c>
     </row>
@@ -4377,78 +4695,88 @@
           <t>0000000000</t>
         </is>
       </c>
-      <c r="V31" s="2" t="inlineStr"/>
-      <c r="W31" s="2" t="inlineStr"/>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="X31" s="2" t="inlineStr"/>
       <c r="Y31" s="2" t="inlineStr"/>
-      <c r="Z31" s="2" t="n">
+      <c r="Z31" s="2" t="inlineStr"/>
+      <c r="AA31" s="2" t="inlineStr"/>
+      <c r="AB31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AD31" s="2" t="n">
         <v>8.619999999999999</v>
       </c>
-      <c r="AA31" s="2" t="n">
+      <c r="AE31" s="2" t="n">
         <v>3.02</v>
       </c>
-      <c r="AB31" s="2" t="n">
+      <c r="AF31" s="2" t="n">
         <v>-11.77</v>
       </c>
-      <c r="AC31" s="2" t="n">
+      <c r="AG31" s="2" t="n">
         <v>-12.08</v>
       </c>
-      <c r="AD31" s="2" t="n">
+      <c r="AH31" s="2" t="n">
         <v>11.7</v>
       </c>
-      <c r="AE31" s="2" t="n">
+      <c r="AI31" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AF31" s="2" t="inlineStr"/>
-      <c r="AG31" s="2" t="n">
+      <c r="AJ31" s="2" t="inlineStr"/>
+      <c r="AK31" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AH31" s="2" t="inlineStr"/>
-      <c r="AI31" s="2" t="inlineStr"/>
-      <c r="AJ31" s="2" t="inlineStr">
+      <c r="AL31" s="2" t="inlineStr"/>
+      <c r="AM31" s="2" t="inlineStr"/>
+      <c r="AN31" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AK31" s="2" t="n">
+      <c r="AO31" s="2" t="n">
         <v>2.365</v>
       </c>
-      <c r="AL31" s="2" t="n">
-        <v>2.722</v>
-      </c>
-      <c r="AM31" s="2" t="n">
+      <c r="AP31" s="2" t="n">
+        <v>2.721</v>
+      </c>
+      <c r="AQ31" s="2" t="n">
         <v>2.929</v>
       </c>
-      <c r="AN31" s="2" t="n">
+      <c r="AR31" s="2" t="n">
         <v>2.976</v>
       </c>
-      <c r="AO31" s="2" t="n">
+      <c r="AS31" s="2" t="n">
         <v>2.996</v>
       </c>
-      <c r="AP31" s="2" t="n">
+      <c r="AT31" s="2" t="n">
         <v>3.324</v>
       </c>
-      <c r="AQ31" s="2" t="n">
+      <c r="AU31" s="2" t="n">
         <v>2.912</v>
       </c>
-      <c r="AR31" s="2" t="n">
+      <c r="AV31" s="2" t="n">
         <v>-6.5805</v>
       </c>
-      <c r="AS31" s="2" t="n">
+      <c r="AW31" s="2" t="n">
         <v>-2.857</v>
       </c>
-      <c r="AT31" s="2" t="n">
+      <c r="AX31" s="2" t="n">
         <v>-1.3881</v>
       </c>
-      <c r="AU31" s="2" t="n">
+      <c r="AY31" s="2" t="n">
         <v>-0.7699</v>
       </c>
-      <c r="AV31" s="2" t="n">
+      <c r="AZ31" s="2" t="n">
         <v>0.0862</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AV1"/>
+  <autoFilter ref="A1:AZ1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4459,7 +4787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -4709,121 +5037,142 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr"/>
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stage (Weinstein 大阶段, MA150=30周线为锚, 内部11子档判定后归并为大阶段): 1=筑底 2=上行 3=做顶 4=下行; NA=历史不足(&lt;218日)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>【④ 企稳上行 — Cross】</t>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stage持续: 处于当前大阶段的天数 (距最近一次大阶段变化)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
+          <t xml:space="preserve">  1→2 / 3→4: 大阶段转换信号, 显示'Nd'=N个交易日前触发 (如'3d'=3天前刚完成1→2, 进场关注; 3→4=离场/回避)。触发后≤10个交易日持续显示(追溯保留, 同东吴B/S≤10天口径), 更早的转换不显示但Stage持续列可推</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
-        </is>
-      </c>
+      <c r="A41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>【④ 企稳上行 — Cross】</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
+          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
+          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    有过零但不稳定(whipsaw/暴涨驱动等脏交叉) → 0; 无过零但两线持续重叠(近5日rel&lt;0.2%) → 0; 其余空</t>
+          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr"/>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>【⑦ 均线 MV 与年化斜率】(最右 12 列)</t>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    有过零但不稳定(whipsaw/暴涨驱动等脏交叉) → 0; 无过零但两线持续重叠(近5日rel&lt;0.2%) → 0; 其余空</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>【⑦ 均线 MV 与年化斜率】(最右 12 列)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  ND MV: N日收盘均线(前复权)最新值, N=5/10/20/30/50/100/200。历史不足N个交易日留空</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  ND斜率: (N日均线最新 ÷ 5个交易日前的N日均线 - 1) ×52, 年化小数(0.1=10%)。N=10/20/50/100/200, 正值=均线上行</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">           (与【⑤】年线斜率列的×100百分比口径不同, 本列为原始×52; 不足N+5个交易日留空)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>【⑤ ETF 专属 — 趋势/Mansfield RS】</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">           (与【⑤】年线斜率列的×100百分比口径不同, 本列为原始×52; 不足N+5个交易日留空)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>【⑤ ETF 专属 — 趋势/Mansfield RS】</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  MRS_沪深300_1W / MRS_沪深300_4W: MRS_沪深300 分数的 5日 / 20日 变化</t>
         </is>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-14
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.947</v>
+        <v>2.896</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>6.32</v>
@@ -859,7 +859,7 @@
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>3B·25d</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr"/>
@@ -870,7 +870,7 @@
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="n">
-        <v>-5.64</v>
+        <v>-6.02</v>
       </c>
       <c r="AG2" s="2" t="n">
         <v>-5.37</v>
@@ -899,40 +899,40 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>3.004</v>
+        <v>2.994</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>3.121</v>
+        <v>3.116</v>
       </c>
       <c r="AS2" s="2" t="n">
-        <v>3.236</v>
+        <v>3.234</v>
       </c>
       <c r="AT2" s="2" t="n">
-        <v>3.291</v>
+        <v>3.289</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>3.384</v>
+        <v>3.383</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>3.67</v>
+        <v>3.669</v>
       </c>
       <c r="AW2" s="2" t="n">
         <v>3.523</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>-2.9205</v>
+        <v>-3.0007</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>-1.3605</v>
+        <v>-1.4004</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>-0.7979000000000001</v>
+        <v>-0.8134</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>-0.6743</v>
+        <v>-0.6814</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>-0.0564</v>
+        <v>-0.0602</v>
       </c>
     </row>
     <row r="3">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.433</v>
+        <v>1.432</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>-2.87</v>
@@ -995,7 +995,7 @@
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>4B·22d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr"/>
@@ -1006,7 +1006,7 @@
       <c r="AD3" s="2" t="inlineStr"/>
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="n">
-        <v>-14.52</v>
+        <v>-14.53</v>
       </c>
       <c r="AG3" s="2" t="n">
         <v>1.51</v>
@@ -1054,19 +1054,19 @@
         <v>1.589</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>-0.8575</v>
+        <v>-0.8609</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>-0.7357</v>
+        <v>-0.7374000000000001</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>-0.2691</v>
+        <v>-0.2697</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>-0.2274</v>
+        <v>-0.2277</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>-0.1452</v>
+        <v>-0.1453</v>
       </c>
     </row>
     <row r="4">
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.663</v>
+        <v>0.661</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>-2.04</v>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>4B·149d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr"/>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="n">
-        <v>-42.97</v>
+        <v>-42.99</v>
       </c>
       <c r="AG4" s="2" t="n">
         <v>-2.97</v>
@@ -1192,19 +1192,19 @@
         <v>2.847</v>
       </c>
       <c r="AX4" s="2" t="n">
-        <v>-3.6804</v>
+        <v>-3.6844</v>
       </c>
       <c r="AY4" s="2" t="n">
-        <v>-2.2906</v>
+        <v>-2.2926</v>
       </c>
       <c r="AZ4" s="2" t="n">
-        <v>-0.8267</v>
+        <v>-0.8274</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>-0.6031</v>
+        <v>-0.6035</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>-0.4297</v>
+        <v>-0.4299</v>
       </c>
     </row>
     <row r="5">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.884</v>
+        <v>1.877</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>95.31</v>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>2B·28d</t>
+          <t>2B</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr"/>
@@ -1288,7 +1288,7 @@
       <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="n">
-        <v>59.93</v>
+        <v>59.81</v>
       </c>
       <c r="AG5" s="2" t="n">
         <v>39.18</v>
@@ -1321,13 +1321,13 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>1.898</v>
+        <v>1.897</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>1.822</v>
+        <v>1.821</v>
       </c>
       <c r="AS5" s="2" t="n">
-        <v>1.795</v>
+        <v>1.794</v>
       </c>
       <c r="AT5" s="2" t="n">
         <v>1.74</v>
@@ -1342,19 +1342,19 @@
         <v>1.526</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>1.9729</v>
+        <v>1.9521</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>1.5546</v>
+        <v>1.5442</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>1.2679</v>
+        <v>1.2634</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>0.4005</v>
+        <v>0.3982</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>0.5993000000000001</v>
+        <v>0.5981</v>
       </c>
     </row>
     <row r="6">
@@ -1369,7 +1369,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.821</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>4.98</v>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>1·2d</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1432,7 +1432,7 @@
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="n">
-        <v>-6.03</v>
+        <v>-6.31</v>
       </c>
       <c r="AG6" s="2" t="n">
         <v>5.54</v>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.831</v>
+        <v>0.829</v>
       </c>
       <c r="AR6" s="2" t="n">
         <v>0.842</v>
@@ -1471,7 +1471,7 @@
         <v>0.843</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>0.861</v>
+        <v>0.86</v>
       </c>
       <c r="AV6" s="2" t="n">
         <v>0.828</v>
@@ -1480,19 +1480,19 @@
         <v>0.832</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>-0.4528</v>
+        <v>-0.5078</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>-0.2347</v>
+        <v>-0.2625</v>
       </c>
       <c r="AZ6" s="2" t="n">
-        <v>-0.1698</v>
+        <v>-0.1807</v>
       </c>
       <c r="BA6" s="2" t="n">
-        <v>0.0616</v>
+        <v>0.056</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>-0.0603</v>
+        <v>-0.0631</v>
       </c>
     </row>
     <row r="7">
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.915</v>
+        <v>2.891</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>2.95</v>
@@ -1524,7 +1524,7 @@
         <v>13</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>4B·17d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -1570,7 +1570,7 @@
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="n">
-        <v>-13.67</v>
+        <v>-13.81</v>
       </c>
       <c r="AG7" s="2" t="n">
         <v>4.55</v>
@@ -1597,13 +1597,13 @@
         </is>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>3.967</v>
+        <v>3.962</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>4.117</v>
+        <v>4.115</v>
       </c>
       <c r="AS7" s="2" t="n">
-        <v>4.222</v>
+        <v>4.221</v>
       </c>
       <c r="AT7" s="2" t="n">
         <v>4.277</v>
@@ -1618,19 +1618,19 @@
         <v>4.393</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>-2.1548</v>
+        <v>-2.1839</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>-1.2425</v>
+        <v>-1.257</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>-0.5508999999999999</v>
+        <v>-0.5566</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>-0.2861</v>
+        <v>-0.289</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>-0.1367</v>
+        <v>-0.1381</v>
       </c>
     </row>
     <row r="8">
@@ -1645,7 +1645,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.337</v>
+        <v>4.296</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>4.59</v>
@@ -1668,7 +1668,7 @@
         <v>13</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>1A·16d</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
@@ -1714,7 +1714,7 @@
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
       <c r="AF8" s="2" t="n">
-        <v>-11.08</v>
+        <v>-11.26</v>
       </c>
       <c r="AG8" s="2" t="n">
         <v>1.19</v>
@@ -1743,40 +1743,40 @@
         </is>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>5.297</v>
+        <v>5.289</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>5.483</v>
+        <v>5.479</v>
       </c>
       <c r="AS8" s="2" t="n">
-        <v>5.643</v>
+        <v>5.641</v>
       </c>
       <c r="AT8" s="2" t="n">
-        <v>5.726</v>
+        <v>5.725</v>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>5.814</v>
+        <v>5.813</v>
       </c>
       <c r="AV8" s="2" t="n">
         <v>5.987</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>5.966</v>
+        <v>5.965</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>-2.2788</v>
+        <v>-2.316</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>-1.2607</v>
+        <v>-1.2791</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>-0.612</v>
+        <v>-0.6192</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>-0.4094</v>
+        <v>-0.4129</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>-0.1108</v>
+        <v>-0.1126</v>
       </c>
     </row>
     <row r="9">
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.112</v>
+        <v>7.015</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>14.72</v>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>2A·1d</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
         <v>1</v>
       </c>
       <c r="AF9" s="2" t="n">
-        <v>46.84</v>
+        <v>45.91</v>
       </c>
       <c r="AG9" s="2" t="n">
         <v>-0.83</v>
@@ -1893,40 +1893,40 @@
         </is>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>3.381</v>
+        <v>3.362</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>2.978</v>
+        <v>2.968</v>
       </c>
       <c r="AS9" s="2" t="n">
-        <v>2.803</v>
+        <v>2.798</v>
       </c>
       <c r="AT9" s="2" t="n">
-        <v>2.756</v>
+        <v>2.753</v>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>2.718</v>
+        <v>2.716</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>2.776</v>
+        <v>2.775</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>2.75</v>
+        <v>2.749</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>7.2906</v>
+        <v>7.0975</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>3.698</v>
+        <v>3.6016</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>1.5408</v>
+        <v>1.5026</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>0.4238</v>
+        <v>0.4055</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>0.4684</v>
+        <v>0.4591</v>
       </c>
     </row>
     <row r="10">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.516</v>
+        <v>3.498</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>41.01</v>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>3B·1d</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="Y10" s="2" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="n">
-        <v>3.79</v>
+        <v>3.71</v>
       </c>
       <c r="AG10" s="2" t="n">
         <v>18.46</v>
@@ -2039,13 +2039,13 @@
         </is>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>5.697</v>
+        <v>5.693</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>5.885</v>
+        <v>5.883</v>
       </c>
       <c r="AS10" s="2" t="n">
-        <v>6.025</v>
+        <v>6.024</v>
       </c>
       <c r="AT10" s="2" t="n">
         <v>6.1</v>
@@ -2060,19 +2060,19 @@
         <v>5.837</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>-1.7224</v>
+        <v>-1.7378</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>-1.097</v>
+        <v>-1.1046</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>-0.1595</v>
+        <v>-0.1625</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>-0.073</v>
+        <v>-0.0745</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.0379</v>
+        <v>0.0371</v>
       </c>
     </row>
     <row r="11">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.497</v>
+        <v>0.493</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>-0.8100000000000001</v>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>4B·22d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr"/>
@@ -2148,7 +2148,7 @@
       <c r="AD11" s="2" t="inlineStr"/>
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="n">
-        <v>-32.01</v>
+        <v>-32.11</v>
       </c>
       <c r="AG11" s="2" t="n">
         <v>-0.47</v>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>0.887</v>
+        <v>0.886</v>
       </c>
       <c r="AR11" s="2" t="n">
         <v>0.9399999999999999</v>
@@ -2198,19 +2198,19 @@
         <v>1.058</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>-3.2215</v>
+        <v>-3.2422</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>-2.046</v>
+        <v>-2.0562</v>
       </c>
       <c r="AZ11" s="2" t="n">
-        <v>-0.857</v>
+        <v>-0.861</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>-0.3475</v>
+        <v>-0.3495</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>-0.3201</v>
+        <v>-0.3211</v>
       </c>
     </row>
     <row r="12">
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.376</v>
+        <v>0.373</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>9.880000000000001</v>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>4B·1d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="n">
-        <v>-23.8</v>
+        <v>-23.85</v>
       </c>
       <c r="AG12" s="2" t="n">
         <v>8.06</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>1.26</v>
+        <v>1.259</v>
       </c>
       <c r="AR12" s="2" t="n">
         <v>1.372</v>
@@ -2338,19 +2338,19 @@
         <v>1.443</v>
       </c>
       <c r="AX12" s="2" t="n">
-        <v>-3.7231</v>
+        <v>-3.7336</v>
       </c>
       <c r="AY12" s="2" t="n">
-        <v>-1.9322</v>
+        <v>-1.9375</v>
       </c>
       <c r="AZ12" s="2" t="n">
-        <v>-0.6525</v>
+        <v>-0.6546</v>
       </c>
       <c r="BA12" s="2" t="n">
-        <v>-0.2768</v>
+        <v>-0.2779</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>-0.238</v>
+        <v>-0.2385</v>
       </c>
     </row>
     <row r="13">
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.758</v>
+        <v>0.752</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>-4.85</v>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>4B·22d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
       <c r="AD13" s="2" t="inlineStr"/>
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="n">
-        <v>-36.09</v>
+        <v>-36.15</v>
       </c>
       <c r="AG13" s="2" t="n">
         <v>-1.07</v>
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>1.957</v>
+        <v>1.956</v>
       </c>
       <c r="AR13" s="2" t="n">
         <v>2.117</v>
@@ -2472,19 +2472,19 @@
         <v>2.439</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>-4.1369</v>
+        <v>-4.1504</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>-2.4983</v>
+        <v>-2.5049</v>
       </c>
       <c r="AZ13" s="2" t="n">
-        <v>-0.9896</v>
+        <v>-0.9922</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>-0.4359</v>
+        <v>-0.4373</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>-0.3609</v>
+        <v>-0.3615</v>
       </c>
     </row>
     <row r="14">
@@ -2499,7 +2499,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.846</v>
+        <v>2.807</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>77.83</v>
@@ -2516,20 +2516,20 @@
         <v>13</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>10</v>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>1111110101</t>
+          <t>1111110111</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>2A·1d</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="Y14" s="2" t="inlineStr">
@@ -2570,7 +2570,7 @@
         <v>1</v>
       </c>
       <c r="AF14" s="2" t="n">
-        <v>35.65</v>
+        <v>34.8</v>
       </c>
       <c r="AG14" s="2" t="n">
         <v>-1.47</v>
@@ -2597,40 +2597,40 @@
         </is>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>1.428</v>
+        <v>1.42</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>1.278</v>
+        <v>1.274</v>
       </c>
       <c r="AS14" s="2" t="n">
-        <v>1.213</v>
+        <v>1.211</v>
       </c>
       <c r="AT14" s="2" t="n">
-        <v>1.194</v>
+        <v>1.193</v>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>1.171</v>
+        <v>1.17</v>
       </c>
       <c r="AV14" s="2" t="n">
+        <v>1.205</v>
+      </c>
+      <c r="AW14" s="2" t="n">
         <v>1.206</v>
       </c>
-      <c r="AW14" s="2" t="n">
-        <v>1.207</v>
-      </c>
       <c r="AX14" s="2" t="n">
-        <v>6.0751</v>
+        <v>5.8979</v>
       </c>
       <c r="AY14" s="2" t="n">
-        <v>3.1765</v>
+        <v>3.0878</v>
       </c>
       <c r="AZ14" s="2" t="n">
-        <v>1.6198</v>
+        <v>1.584</v>
       </c>
       <c r="BA14" s="2" t="n">
-        <v>0.2427</v>
+        <v>0.2258</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>0.3565</v>
+        <v>0.348</v>
       </c>
     </row>
     <row r="15">
@@ -2645,7 +2645,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.336</v>
+        <v>0.332</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>52.3</v>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>4B·1d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y15" s="2" t="inlineStr">
@@ -2708,7 +2708,7 @@
       <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="n">
-        <v>-19.53</v>
+        <v>-19.63</v>
       </c>
       <c r="AG15" s="2" t="n">
         <v>6.85</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>0.913</v>
+        <v>0.912</v>
       </c>
       <c r="AR15" s="2" t="n">
         <v>0.992</v>
@@ -2756,19 +2756,19 @@
         <v>1.044</v>
       </c>
       <c r="AX15" s="2" t="n">
-        <v>-3.7174</v>
+        <v>-3.7369</v>
       </c>
       <c r="AY15" s="2" t="n">
-        <v>-1.7695</v>
+        <v>-1.7794</v>
       </c>
       <c r="AZ15" s="2" t="n">
-        <v>-0.452</v>
+        <v>-0.4559</v>
       </c>
       <c r="BA15" s="2" t="n">
-        <v>-0.3002</v>
+        <v>-0.3023</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>-0.1953</v>
+        <v>-0.1963</v>
       </c>
     </row>
     <row r="16">
@@ -2783,7 +2783,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.087</v>
+        <v>1.071</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>81.33</v>
@@ -2800,25 +2800,25 @@
         <v>9</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t>0100000100</t>
+          <t>0000000100</t>
         </is>
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V16" s="2" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
-          <t>4B·33d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y16" s="2" t="inlineStr"/>
@@ -2844,7 +2844,7 @@
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="n">
-        <v>-13.5</v>
+        <v>-13.82</v>
       </c>
       <c r="AG16" s="2" t="n">
         <v>-7.56</v>
@@ -2871,19 +2871,19 @@
         </is>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>1.081</v>
+        <v>1.078</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>1.098</v>
+        <v>1.097</v>
       </c>
       <c r="AS16" s="2" t="n">
-        <v>1.13</v>
+        <v>1.129</v>
       </c>
       <c r="AT16" s="2" t="n">
         <v>1.132</v>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>1.13</v>
+        <v>1.129</v>
       </c>
       <c r="AV16" s="2" t="n">
         <v>1.184</v>
@@ -2892,19 +2892,19 @@
         <v>1.299</v>
       </c>
       <c r="AX16" s="2" t="n">
-        <v>-1.7918</v>
+        <v>-1.865</v>
       </c>
       <c r="AY16" s="2" t="n">
-        <v>-0.7685999999999999</v>
+        <v>-0.8048999999999999</v>
       </c>
       <c r="AZ16" s="2" t="n">
-        <v>-0.035</v>
+        <v>-0.0497</v>
       </c>
       <c r="BA16" s="2" t="n">
-        <v>-0.7496</v>
+        <v>-0.7565</v>
       </c>
       <c r="BB16" s="2" t="n">
-        <v>-0.135</v>
+        <v>-0.1382</v>
       </c>
     </row>
     <row r="17">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.415</v>
+        <v>0.414</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>-1.36</v>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>4B·201d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr"/>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="n">
-        <v>-52.08</v>
+        <v>-52.1</v>
       </c>
       <c r="AG17" s="2" t="n">
         <v>-8.41</v>
@@ -3011,7 +3011,7 @@
         </is>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>0.974</v>
+        <v>0.973</v>
       </c>
       <c r="AR17" s="2" t="n">
         <v>1.034</v>
@@ -3032,19 +3032,19 @@
         <v>1.248</v>
       </c>
       <c r="AX17" s="2" t="n">
-        <v>-2.9421</v>
+        <v>-2.9469</v>
       </c>
       <c r="AY17" s="2" t="n">
-        <v>-1.9826</v>
+        <v>-1.985</v>
       </c>
       <c r="AZ17" s="2" t="n">
-        <v>-0.7214</v>
+        <v>-0.7223000000000001</v>
       </c>
       <c r="BA17" s="2" t="n">
-        <v>-0.585</v>
+        <v>-0.5854</v>
       </c>
       <c r="BB17" s="2" t="n">
-        <v>-0.5208</v>
+        <v>-0.521</v>
       </c>
     </row>
     <row r="18">
@@ -3059,7 +3059,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.045</v>
+        <v>1.034</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>-0.29</v>
@@ -3076,7 +3076,7 @@
         <v>9</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>4B·25d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y18" s="2" t="inlineStr"/>
@@ -3118,7 +3118,7 @@
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="n">
-        <v>-15.65</v>
+        <v>-15.86</v>
       </c>
       <c r="AG18" s="2" t="n">
         <v>-6.93</v>
@@ -3147,16 +3147,16 @@
         </is>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>1.14</v>
+        <v>1.138</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>1.177</v>
+        <v>1.176</v>
       </c>
       <c r="AS18" s="2" t="n">
-        <v>1.208</v>
+        <v>1.207</v>
       </c>
       <c r="AT18" s="2" t="n">
-        <v>1.235</v>
+        <v>1.234</v>
       </c>
       <c r="AU18" s="2" t="n">
         <v>1.266</v>
@@ -3168,19 +3168,19 @@
         <v>1.351</v>
       </c>
       <c r="AX18" s="2" t="n">
-        <v>-2.2359</v>
+        <v>-2.2824</v>
       </c>
       <c r="AY18" s="2" t="n">
-        <v>-1.4809</v>
+        <v>-1.5039</v>
       </c>
       <c r="AZ18" s="2" t="n">
-        <v>-0.7065</v>
+        <v>-0.7154</v>
       </c>
       <c r="BA18" s="2" t="n">
-        <v>-0.6919</v>
+        <v>-0.6962</v>
       </c>
       <c r="BB18" s="2" t="n">
-        <v>-0.1565</v>
+        <v>-0.1586</v>
       </c>
     </row>
     <row r="19">
@@ -3195,7 +3195,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.921</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>14.64</v>
@@ -3212,7 +3212,7 @@
         <v>9</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>1·8d</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
@@ -3258,7 +3258,7 @@
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="n">
-        <v>2.63</v>
+        <v>2.54</v>
       </c>
       <c r="AG19" s="2" t="n">
         <v>5.18</v>
@@ -3287,13 +3287,13 @@
         </is>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>3.399</v>
+        <v>3.396</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>3.912</v>
+        <v>3.91</v>
       </c>
       <c r="AS19" s="2" t="n">
-        <v>4.171</v>
+        <v>4.17</v>
       </c>
       <c r="AT19" s="2" t="n">
         <v>4.289</v>
@@ -3308,19 +3308,19 @@
         <v>4.296</v>
       </c>
       <c r="AX19" s="2" t="n">
-        <v>-6.7255</v>
+        <v>-6.7441</v>
       </c>
       <c r="AY19" s="2" t="n">
-        <v>-3.0242</v>
+        <v>-3.0336</v>
       </c>
       <c r="AZ19" s="2" t="n">
-        <v>-1.8452</v>
+        <v>-1.8488</v>
       </c>
       <c r="BA19" s="2" t="n">
-        <v>-0.6461</v>
+        <v>-0.6478</v>
       </c>
       <c r="BB19" s="2" t="n">
-        <v>0.0263</v>
+        <v>0.0254</v>
       </c>
     </row>
     <row r="20">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.869</v>
+        <v>0.863</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>85.37</v>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>1A·1d</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="n">
-        <v>-7.59</v>
+        <v>-7.69</v>
       </c>
       <c r="AG20" s="2" t="n">
         <v>17.15</v>
@@ -3431,13 +3431,13 @@
         </is>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>1.549</v>
+        <v>1.548</v>
       </c>
       <c r="AR20" s="2" t="n">
         <v>1.614</v>
       </c>
       <c r="AS20" s="2" t="n">
-        <v>1.65</v>
+        <v>1.649</v>
       </c>
       <c r="AT20" s="2" t="n">
         <v>1.656</v>
@@ -3452,19 +3452,19 @@
         <v>1.593</v>
       </c>
       <c r="AX20" s="2" t="n">
-        <v>-1.9411</v>
+        <v>-1.9597</v>
       </c>
       <c r="AY20" s="2" t="n">
-        <v>-1.0198</v>
+        <v>-1.0291</v>
       </c>
       <c r="AZ20" s="2" t="n">
-        <v>-0.193</v>
+        <v>-0.1968</v>
       </c>
       <c r="BA20" s="2" t="n">
-        <v>-0.013</v>
+        <v>-0.015</v>
       </c>
       <c r="BB20" s="2" t="n">
-        <v>-0.0759</v>
+        <v>-0.0769</v>
       </c>
     </row>
     <row r="21">
@@ -3479,7 +3479,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.02</v>
+        <v>1.024</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>-8.65</v>
@@ -3504,19 +3504,19 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000000100</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000000010</t>
         </is>
       </c>
       <c r="V21" s="2" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>4B·126d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr"/>
@@ -3544,7 +3544,7 @@
       <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="inlineStr"/>
       <c r="AF21" s="2" t="n">
-        <v>-55.7</v>
+        <v>-55.62</v>
       </c>
       <c r="AG21" s="2" t="n">
         <v>-15.78</v>
@@ -3580,7 +3580,7 @@
         <v>1.015</v>
       </c>
       <c r="AT21" s="2" t="n">
-        <v>1.03</v>
+        <v>1.031</v>
       </c>
       <c r="AU21" s="2" t="n">
         <v>1.072</v>
@@ -3592,19 +3592,19 @@
         <v>1.212</v>
       </c>
       <c r="AX21" s="2" t="n">
-        <v>-0.5048</v>
+        <v>-0.4844</v>
       </c>
       <c r="AY21" s="2" t="n">
-        <v>-0.555</v>
+        <v>-0.5449000000000001</v>
       </c>
       <c r="AZ21" s="2" t="n">
-        <v>-0.3994</v>
+        <v>-0.3956</v>
       </c>
       <c r="BA21" s="2" t="n">
-        <v>-0.4709</v>
+        <v>-0.469</v>
       </c>
       <c r="BB21" s="2" t="n">
-        <v>-0.5570000000000001</v>
+        <v>-0.5562</v>
       </c>
     </row>
     <row r="22">
@@ -3619,7 +3619,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.736</v>
+        <v>1.73</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>-5.36</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>4B·18d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y22" s="2" t="inlineStr">
@@ -3684,7 +3684,7 @@
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="n">
-        <v>-22.18</v>
+        <v>-22.26</v>
       </c>
       <c r="AG22" s="2" t="n">
         <v>-2.6</v>
@@ -3711,7 +3711,7 @@
         </is>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>1.732</v>
+        <v>1.731</v>
       </c>
       <c r="AR22" s="2" t="n">
         <v>1.752</v>
@@ -3732,19 +3732,19 @@
         <v>1.878</v>
       </c>
       <c r="AX22" s="2" t="n">
-        <v>-0.9527</v>
+        <v>-0.9701</v>
       </c>
       <c r="AY22" s="2" t="n">
-        <v>-0.9923</v>
+        <v>-1.0009</v>
       </c>
       <c r="AZ22" s="2" t="n">
-        <v>-0.3611</v>
+        <v>-0.3645</v>
       </c>
       <c r="BA22" s="2" t="n">
-        <v>-0.1379</v>
+        <v>-0.1396</v>
       </c>
       <c r="BB22" s="2" t="n">
-        <v>-0.2218</v>
+        <v>-0.2226</v>
       </c>
     </row>
     <row r="23">
@@ -3759,7 +3759,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.397</v>
+        <v>2.382</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>110.91</v>
@@ -3778,7 +3778,7 @@
         <v>-9</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>1·1d</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y23" s="2" t="inlineStr">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="n">
-        <v>4.12</v>
+        <v>4.08</v>
       </c>
       <c r="AG23" s="2" t="n">
         <v>29.05</v>
@@ -3857,13 +3857,13 @@
         </is>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>10.03</v>
+        <v>10.027</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>10.83</v>
+        <v>10.829</v>
       </c>
       <c r="AS23" s="2" t="n">
-        <v>11.004</v>
+        <v>11.003</v>
       </c>
       <c r="AT23" s="2" t="n">
         <v>11.038</v>
@@ -3878,19 +3878,19 @@
         <v>10.154</v>
       </c>
       <c r="AX23" s="2" t="n">
-        <v>-2.9006</v>
+        <v>-2.9074</v>
       </c>
       <c r="AY23" s="2" t="n">
-        <v>-1.2179</v>
+        <v>-1.2213</v>
       </c>
       <c r="AZ23" s="2" t="n">
-        <v>-0.2463</v>
+        <v>-0.2477</v>
       </c>
       <c r="BA23" s="2" t="n">
-        <v>-0.09909999999999999</v>
+        <v>-0.0998</v>
       </c>
       <c r="BB23" s="2" t="n">
-        <v>0.0412</v>
+        <v>0.0408</v>
       </c>
     </row>
     <row r="24">
@@ -3905,7 +3905,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.388</v>
+        <v>1.369</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>6.69</v>
@@ -3928,7 +3928,7 @@
         <v>13</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>4B·36d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr"/>
@@ -3974,7 +3974,7 @@
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="n">
-        <v>-26.17</v>
+        <v>-26.44</v>
       </c>
       <c r="AG24" s="2" t="n">
         <v>-15.08</v>
@@ -4003,16 +4003,16 @@
         </is>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>1.432</v>
+        <v>1.428</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>1.447</v>
+        <v>1.445</v>
       </c>
       <c r="AS24" s="2" t="n">
-        <v>1.475</v>
+        <v>1.474</v>
       </c>
       <c r="AT24" s="2" t="n">
-        <v>1.513</v>
+        <v>1.512</v>
       </c>
       <c r="AU24" s="2" t="n">
         <v>1.566</v>
@@ -4024,19 +4024,19 @@
         <v>1.802</v>
       </c>
       <c r="AX24" s="2" t="n">
-        <v>-1.1526</v>
+        <v>-1.2194</v>
       </c>
       <c r="AY24" s="2" t="n">
-        <v>-1.079</v>
+        <v>-1.1118</v>
       </c>
       <c r="AZ24" s="2" t="n">
-        <v>-0.4908</v>
+        <v>-0.5033</v>
       </c>
       <c r="BA24" s="2" t="n">
-        <v>-0.949</v>
+        <v>-0.9548</v>
       </c>
       <c r="BB24" s="2" t="n">
-        <v>-0.2617</v>
+        <v>-0.2644</v>
       </c>
     </row>
     <row r="25">
@@ -4051,7 +4051,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.866</v>
+        <v>0.848</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>79.97</v>
@@ -4068,7 +4068,7 @@
         <v>9</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>1·8d</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y25" s="2" t="inlineStr">
@@ -4114,7 +4114,7 @@
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="n">
-        <v>5.25</v>
+        <v>5.09</v>
       </c>
       <c r="AG25" s="2" t="n">
         <v>5</v>
@@ -4143,19 +4143,19 @@
         </is>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>2.31</v>
+        <v>2.307</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>2.66</v>
+        <v>2.658</v>
       </c>
       <c r="AS25" s="2" t="n">
-        <v>2.904</v>
+        <v>2.903</v>
       </c>
       <c r="AT25" s="2" t="n">
-        <v>2.963</v>
+        <v>2.962</v>
       </c>
       <c r="AU25" s="2" t="n">
-        <v>2.991</v>
+        <v>2.99</v>
       </c>
       <c r="AV25" s="2" t="n">
         <v>3.316</v>
@@ -4164,19 +4164,19 @@
         <v>2.914</v>
       </c>
       <c r="AX25" s="2" t="n">
-        <v>-7.4094</v>
+        <v>-7.4396</v>
       </c>
       <c r="AY25" s="2" t="n">
-        <v>-3.1308</v>
+        <v>-3.1459</v>
       </c>
       <c r="AZ25" s="2" t="n">
-        <v>-1.3289</v>
+        <v>-1.335</v>
       </c>
       <c r="BA25" s="2" t="n">
-        <v>-0.8260999999999999</v>
+        <v>-0.8289</v>
       </c>
       <c r="BB25" s="2" t="n">
-        <v>0.0525</v>
+        <v>0.0509</v>
       </c>
     </row>
     <row r="26">
@@ -4191,7 +4191,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.309</v>
+        <v>1.299</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>55.37</v>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>3B·1d</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="Y26" s="2" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="AG26" s="2" t="n">
         <v>18.72</v>
@@ -4285,10 +4285,10 @@
         </is>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>2.667</v>
+        <v>2.665</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>2.805</v>
+        <v>2.804</v>
       </c>
       <c r="AS26" s="2" t="n">
         <v>2.904</v>
@@ -4306,19 +4306,19 @@
         <v>2.812</v>
       </c>
       <c r="AX26" s="2" t="n">
-        <v>-2.6715</v>
+        <v>-2.6891</v>
       </c>
       <c r="AY26" s="2" t="n">
-        <v>-1.5621</v>
+        <v>-1.5708</v>
       </c>
       <c r="AZ26" s="2" t="n">
-        <v>-0.2504</v>
+        <v>-0.2539</v>
       </c>
       <c r="BA26" s="2" t="n">
-        <v>-0.1928</v>
+        <v>-0.1946</v>
       </c>
       <c r="BB26" s="2" t="n">
-        <v>0.082</v>
+        <v>0.081</v>
       </c>
     </row>
     <row r="27">
@@ -4333,7 +4333,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.75</v>
+        <v>0.741</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>7.96</v>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>4B·36d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y27" s="2" t="inlineStr"/>
@@ -4402,7 +4402,7 @@
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="n">
-        <v>-26.38</v>
+        <v>-26.62</v>
       </c>
       <c r="AG27" s="2" t="n">
         <v>-16.33</v>
@@ -4431,40 +4431,40 @@
         </is>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>0.758</v>
+        <v>0.756</v>
       </c>
       <c r="AR27" s="2" t="n">
         <v>0.771</v>
       </c>
       <c r="AS27" s="2" t="n">
-        <v>0.788</v>
+        <v>0.787</v>
       </c>
       <c r="AT27" s="2" t="n">
-        <v>0.801</v>
+        <v>0.8</v>
       </c>
       <c r="AU27" s="2" t="n">
         <v>0.821</v>
       </c>
       <c r="AV27" s="2" t="n">
-        <v>0.9</v>
+        <v>0.899</v>
       </c>
       <c r="AW27" s="2" t="n">
         <v>0.985</v>
       </c>
       <c r="AX27" s="2" t="n">
-        <v>-1.6511</v>
+        <v>-1.7098</v>
       </c>
       <c r="AY27" s="2" t="n">
-        <v>-0.8856000000000001</v>
+        <v>-0.9147999999999999</v>
       </c>
       <c r="AZ27" s="2" t="n">
-        <v>-0.4061</v>
+        <v>-0.4174</v>
       </c>
       <c r="BA27" s="2" t="n">
-        <v>-1.0284</v>
+        <v>-1.0335</v>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>-0.2638</v>
+        <v>-0.2662</v>
       </c>
     </row>
     <row r="28">
@@ -4479,7 +4479,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.549</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>89.25</v>
@@ -4496,7 +4496,7 @@
         <v>13</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>1·9d</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y28" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="n">
-        <v>-1.89</v>
+        <v>-1.99</v>
       </c>
       <c r="AG28" s="2" t="n">
         <v>3.79</v>
@@ -4571,13 +4571,13 @@
         </is>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>2.896</v>
+        <v>2.893</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>3.405</v>
+        <v>3.403</v>
       </c>
       <c r="AS28" s="2" t="n">
-        <v>3.75</v>
+        <v>3.749</v>
       </c>
       <c r="AT28" s="2" t="n">
         <v>3.821</v>
@@ -4592,19 +4592,19 @@
         <v>3.849</v>
       </c>
       <c r="AX28" s="2" t="n">
-        <v>-8.3147</v>
+        <v>-8.332599999999999</v>
       </c>
       <c r="AY28" s="2" t="n">
-        <v>-3.3729</v>
+        <v>-3.3819</v>
       </c>
       <c r="AZ28" s="2" t="n">
-        <v>-1.3299</v>
+        <v>-1.3335</v>
       </c>
       <c r="BA28" s="2" t="n">
-        <v>-0.9962</v>
+        <v>-0.9979</v>
       </c>
       <c r="BB28" s="2" t="n">
-        <v>-0.0189</v>
+        <v>-0.0199</v>
       </c>
     </row>
     <row r="29">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2.155</v>
+        <v>2.125</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>3.12</v>
@@ -4677,7 +4677,7 @@
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>1·1d</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y29" s="2" t="inlineStr">
@@ -4700,7 +4700,7 @@
         <v>1</v>
       </c>
       <c r="AF29" s="2" t="n">
-        <v>15.98</v>
+        <v>15.1</v>
       </c>
       <c r="AG29" s="2" t="n">
         <v>-16.59</v>
@@ -4729,16 +4729,16 @@
         </is>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>0.979</v>
+        <v>0.973</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>0.837</v>
+        <v>0.834</v>
       </c>
       <c r="AS29" s="2" t="n">
-        <v>0.778</v>
+        <v>0.776</v>
       </c>
       <c r="AT29" s="2" t="n">
-        <v>0.767</v>
+        <v>0.766</v>
       </c>
       <c r="AU29" s="2" t="n">
         <v>0.772</v>
@@ -4750,19 +4750,19 @@
         <v>0.886</v>
       </c>
       <c r="AX29" s="2" t="n">
-        <v>9.662100000000001</v>
+        <v>9.4412</v>
       </c>
       <c r="AY29" s="2" t="n">
-        <v>4.5205</v>
+        <v>4.4115</v>
       </c>
       <c r="AZ29" s="2" t="n">
-        <v>1.573</v>
+        <v>1.5314</v>
       </c>
       <c r="BA29" s="2" t="n">
-        <v>-0.078</v>
+        <v>-0.0968</v>
       </c>
       <c r="BB29" s="2" t="n">
-        <v>0.1598</v>
+        <v>0.151</v>
       </c>
     </row>
     <row r="30">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.826</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>7.5</v>
@@ -4794,7 +4794,7 @@
         <v>13</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>4B·8d</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="Y30" s="2" t="inlineStr">
@@ -4840,7 +4840,7 @@
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="n">
-        <v>-15.67</v>
+        <v>-15.95</v>
       </c>
       <c r="AG30" s="2" t="n">
         <v>-10.44</v>
@@ -4865,13 +4865,13 @@
         </is>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>0.846</v>
+        <v>0.844</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>0.877</v>
+        <v>0.876</v>
       </c>
       <c r="AS30" s="2" t="n">
-        <v>0.9</v>
+        <v>0.899</v>
       </c>
       <c r="AT30" s="2" t="n">
         <v>0.918</v>
@@ -4880,25 +4880,25 @@
         <v>0.944</v>
       </c>
       <c r="AV30" s="2" t="n">
-        <v>1.025</v>
+        <v>1.024</v>
       </c>
       <c r="AW30" s="2" t="n">
         <v>1.025</v>
       </c>
       <c r="AX30" s="2" t="n">
-        <v>-2.2848</v>
+        <v>-2.3471</v>
       </c>
       <c r="AY30" s="2" t="n">
-        <v>-1.4519</v>
+        <v>-1.4828</v>
       </c>
       <c r="AZ30" s="2" t="n">
-        <v>-0.5225</v>
+        <v>-0.5345</v>
       </c>
       <c r="BA30" s="2" t="n">
-        <v>-0.7661</v>
+        <v>-0.7716</v>
       </c>
       <c r="BB30" s="2" t="n">
-        <v>-0.1567</v>
+        <v>-0.1595</v>
       </c>
     </row>
     <row r="31">
@@ -4913,7 +4913,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.494</v>
+        <v>1.467</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>12.87</v>
@@ -4930,7 +4930,7 @@
         <v>9</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>3B·8d</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="Y31" s="2" t="inlineStr">
@@ -4976,7 +4976,7 @@
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="n">
-        <v>8.550000000000001</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="AG31" s="2" t="n">
         <v>0.97</v>
@@ -5005,19 +5005,19 @@
         </is>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>1.517</v>
+        <v>1.512</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>1.597</v>
+        <v>1.594</v>
       </c>
       <c r="AS31" s="2" t="n">
-        <v>1.642</v>
+        <v>1.641</v>
       </c>
       <c r="AT31" s="2" t="n">
-        <v>1.67</v>
+        <v>1.669</v>
       </c>
       <c r="AU31" s="2" t="n">
-        <v>1.711</v>
+        <v>1.71</v>
       </c>
       <c r="AV31" s="2" t="n">
         <v>1.838</v>
@@ -5026,19 +5026,19 @@
         <v>1.676</v>
       </c>
       <c r="AX31" s="2" t="n">
-        <v>-3.2654</v>
+        <v>-3.3478</v>
       </c>
       <c r="AY31" s="2" t="n">
-        <v>-1.3569</v>
+        <v>-1.3985</v>
       </c>
       <c r="AZ31" s="2" t="n">
-        <v>-1.0945</v>
+        <v>-1.1105</v>
       </c>
       <c r="BA31" s="2" t="n">
-        <v>-0.4212</v>
+        <v>-0.4287</v>
       </c>
       <c r="BB31" s="2" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.0813</v>
       </c>
     </row>
   </sheetData>
@@ -5326,7 +5326,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  子档: 当前11子档及持续 (如 2A·6d)。11子档: 1A卖压衰竭(均线下·走平·52周低位) 1筑底未定型 1B筑底后期(站上走平均线) 1C突破前夜(距60日收盘高点≤5%) 2A刚突破60日新高(均线未上弯·最佳买点) 2B趋势运行(均线上行·距均线≤30%) 2C趋势晚期(距均线&gt;30%忌追高) 3A做顶早期(均线上·走平·前期上行) 3B做顶后期(跌回均线下) 4A下行初段 4B下行确立</t>
+          <t xml:space="preserve">  子档: 当前11子档 (如 2A)。11子档: 1A卖压衰竭(均线下·走平·52周低位) 1筑底未定型 1B筑底后期(站上走平均线) 1C突破前夜(距60日收盘高点≤5%) 2A刚突破60日新高(均线未上弯·最佳买点) 2B趋势运行(均线上行·距均线≤30%) 2C趋势晚期(距均线&gt;30%忌追高) 3A做顶早期(均线上·走平·前期上行) 3B做顶后期(跌回均线下) 4A下行初段 4B下行确立</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-15
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.785</v>
+        <v>2.806</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>6.32</v>
@@ -828,7 +828,7 @@
         <v>9</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
@@ -864,7 +864,7 @@
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>1A→4·4d ← 1B→1A·17d</t>
+          <t>1→4·4d</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr"/>
@@ -874,26 +874,26 @@
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="n">
-        <v>-8.66</v>
+        <v>-8.5</v>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>-6.75</v>
+        <v>-8.359999999999999</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>-5.26</v>
+        <v>-4.75</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>-8.35</v>
+        <v>-9.5</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>-5.3</v>
+        <v>-5.9</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AL2" s="2" t="inlineStr"/>
       <c r="AM2" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AN2" s="2" t="inlineStr"/>
       <c r="AO2" s="2" t="inlineStr"/>
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>2.939</v>
+        <v>2.944</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>3.054</v>
+        <v>3.056</v>
       </c>
       <c r="AS2" s="2" t="n">
-        <v>3.204</v>
+        <v>3.205</v>
       </c>
       <c r="AT2" s="2" t="n">
-        <v>3.267</v>
+        <v>3.268</v>
       </c>
       <c r="AU2" s="2" t="n">
         <v>3.371</v>
@@ -924,19 +924,19 @@
         <v>3.521</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>-3.5685</v>
+        <v>-3.5352</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>-1.6507</v>
+        <v>-1.6342</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>-0.8429</v>
+        <v>-0.8365</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>-0.7188</v>
+        <v>-0.7159</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>-0.0866</v>
+        <v>-0.08500000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.407</v>
+        <v>1.41</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>-2.87</v>
@@ -974,19 +974,19 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
@@ -999,12 +999,12 @@
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>4→1A·8d ← 1A→4·9d</t>
+          <t>4+→1·8d ← 1→4+·9d</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr"/>
@@ -1016,22 +1016,22 @@
       <c r="AD3" s="2" t="inlineStr"/>
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="n">
-        <v>-14.15</v>
+        <v>-12.91</v>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>3.41</v>
+        <v>3.05</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>2.64</v>
+        <v>4.14</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>4.85</v>
+        <v>5.13</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>51</v>
+        <v>48.5</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="AL3" s="2" t="inlineStr"/>
       <c r="AM3" s="2" t="inlineStr"/>
@@ -1043,40 +1043,40 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>1.482</v>
+        <v>1.423</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>1.498</v>
+        <v>1.431</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>1.515</v>
+        <v>1.444</v>
       </c>
       <c r="AT3" s="2" t="n">
-        <v>1.533</v>
+        <v>1.46</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>1.555</v>
+        <v>1.48</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>1.538</v>
+        <v>1.463</v>
       </c>
       <c r="AW3" s="2" t="n">
-        <v>1.588</v>
+        <v>1.511</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>-0.8706</v>
+        <v>-0.6111</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>-0.7242</v>
+        <v>-0.5956</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>-0.3026</v>
+        <v>-0.252</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>-0.2151</v>
+        <v>-0.1896</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>-0.1415</v>
+        <v>-0.1291</v>
       </c>
     </row>
     <row r="4">
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.652</v>
+        <v>0.66</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>-2.04</v>
@@ -1106,25 +1106,25 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010100</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010110</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
@@ -1137,39 +1137,41 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y4" s="2" t="inlineStr"/>
+          <t>4+(底背离·日线纠缠)</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>4→4+·3d ← 4+→4·4d ← 4→4+·20d</t>
+        </is>
+      </c>
       <c r="Z4" s="2" t="inlineStr"/>
       <c r="AA4" s="2" t="inlineStr"/>
-      <c r="AB4" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC4" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AD4" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="n">
-        <v>-42.32</v>
+        <v>-24.3</v>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>-0.96</v>
+        <v>0.03</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>4.2</v>
+        <v>4.78</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>6.62</v>
+        <v>8.33</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>66.90000000000001</v>
+        <v>67</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="AL4" s="2" t="inlineStr"/>
       <c r="AM4" s="2" t="inlineStr"/>
@@ -1181,40 +1183,40 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>2.248</v>
+        <v>0.661</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>2.424</v>
+        <v>0.656</v>
       </c>
       <c r="AS4" s="2" t="n">
-        <v>2.523</v>
+        <v>0.656</v>
       </c>
       <c r="AT4" s="2" t="n">
-        <v>2.581</v>
+        <v>0.662</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>2.629</v>
+        <v>0.667</v>
       </c>
       <c r="AV4" s="2" t="n">
-        <v>2.617</v>
+        <v>0.659</v>
       </c>
       <c r="AW4" s="2" t="n">
-        <v>2.845</v>
+        <v>0.714</v>
       </c>
       <c r="AX4" s="2" t="n">
-        <v>-3.6915</v>
+        <v>0.2711</v>
       </c>
       <c r="AY4" s="2" t="n">
-        <v>-2.3119</v>
+        <v>-0.3545</v>
       </c>
       <c r="AZ4" s="2" t="n">
-        <v>-0.8268</v>
+        <v>-0.0529</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>-0.5792</v>
+        <v>-0.1886</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>-0.4232</v>
+        <v>-0.243</v>
       </c>
     </row>
     <row r="5">
@@ -1229,7 +1231,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.84</v>
+        <v>1.831</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>95.31</v>
@@ -1304,27 +1306,27 @@
       <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="n">
-        <v>58.52</v>
+        <v>58.36</v>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>40.81</v>
+        <v>39.38</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>10.31</v>
+        <v>-4.54</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>15.34</v>
+        <v>13.86</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>100</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="AL5" s="2" t="inlineStr"/>
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1333,16 +1335,16 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>1.876</v>
+        <v>1.874</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>1.837</v>
+        <v>1.836</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>1.798</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>1.751</v>
+        <v>1.75</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>1.657</v>
@@ -1354,19 +1356,19 @@
         <v>1.529</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>2.0512</v>
+        <v>2.0247</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>1.2754</v>
+        <v>1.2621</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>1.2224</v>
+        <v>1.2166</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>0.3639</v>
+        <v>0.361</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5836</v>
       </c>
     </row>
     <row r="6">
@@ -1381,7 +1383,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>4.98</v>
@@ -1396,7 +1398,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
@@ -1427,12 +1429,12 @@
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>1B(纠缠)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>3→1B·3d ← 1B→3·12d ← 2A→1B·17d</t>
+          <t>3→1·3d ← 1B→3·12d ← 1→1B·13d</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr"/>
@@ -1444,22 +1446,22 @@
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="n">
-        <v>-7.28</v>
+        <v>-7.18</v>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>5.74</v>
+        <v>7.08</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>-4.17</v>
+        <v>0.12</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>4.45</v>
+        <v>7.47</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>48.9</v>
+        <v>45.7</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AL6" s="2" t="inlineStr"/>
       <c r="AM6" s="2" t="inlineStr"/>
@@ -1471,7 +1473,7 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.822</v>
+        <v>0.823</v>
       </c>
       <c r="AR6" s="2" t="n">
         <v>0.835</v>
@@ -1492,19 +1494,19 @@
         <v>0.832</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>-0.9836</v>
+        <v>-0.9651999999999999</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>-0.349</v>
+        <v>-0.3397</v>
       </c>
       <c r="AZ6" s="2" t="n">
-        <v>-0.1857</v>
+        <v>-0.1821</v>
       </c>
       <c r="BA6" s="2" t="n">
-        <v>0.0698</v>
+        <v>0.0717</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>-0.0728</v>
+        <v>-0.0718</v>
       </c>
     </row>
     <row r="7">
@@ -1519,7 +1521,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.84</v>
+        <v>2.875</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>2.95</v>
@@ -1542,19 +1544,19 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
@@ -1567,37 +1569,41 @@
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>1B→1A·11d ← 1A→1B·12d ← 1B→1A·16d</t>
+          <t>1A→1·11d ← 1→1A·12d</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr"/>
       <c r="AA7" s="2" t="inlineStr"/>
-      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="n">
-        <v>-14.25</v>
+        <v>-6.44</v>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>5.07</v>
+        <v>5.72</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>1.68</v>
+        <v>1.91</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>3.67</v>
+        <v>4.47</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>12.3</v>
+        <v>10.5</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="AL7" s="2" t="inlineStr"/>
       <c r="AM7" s="2" t="inlineStr"/>
@@ -1609,40 +1615,40 @@
         </is>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>3.944</v>
+        <v>2.907</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>4.094</v>
+        <v>2.92</v>
       </c>
       <c r="AS7" s="2" t="n">
-        <v>4.209</v>
+        <v>2.953</v>
       </c>
       <c r="AT7" s="2" t="n">
-        <v>4.269</v>
+        <v>2.979</v>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>4.311</v>
+        <v>2.996</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>4.339</v>
+        <v>3.006</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>4.391</v>
+        <v>3.038</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>-2.3315</v>
+        <v>-0.7278</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>-1.3098</v>
+        <v>-0.5137</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>-0.5568</v>
+        <v>-0.2413</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>-0.2837</v>
+        <v>-0.1261</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>-0.1425</v>
+        <v>-0.0644</v>
       </c>
     </row>
     <row r="8">
@@ -1657,7 +1663,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.196</v>
+        <v>4.242</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>4.59</v>
@@ -1680,25 +1686,25 @@
         <v>13</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
@@ -1711,41 +1717,41 @@
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y8" s="2" t="inlineStr">
-        <is>
-          <t>1A→4·1d ← 1B→1A·19d</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr"/>
       <c r="Z8" s="2" t="inlineStr"/>
       <c r="AA8" s="2" t="inlineStr"/>
-      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AC8" s="2" t="inlineStr"/>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
       <c r="AF8" s="2" t="n">
-        <v>-12.2</v>
+        <v>-7.07</v>
       </c>
       <c r="AG8" s="2" t="n">
         <v>1.36</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>0.06</v>
+        <v>-0.04</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>-4.1</v>
+        <v>-4.2</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="AL8" s="2" t="inlineStr"/>
       <c r="AM8" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AN8" s="2" t="inlineStr"/>
       <c r="AO8" s="2" t="inlineStr"/>
@@ -1755,40 +1761,40 @@
         </is>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>5.245</v>
+        <v>4.325</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>5.432</v>
+        <v>4.38</v>
       </c>
       <c r="AS8" s="2" t="n">
-        <v>5.614</v>
+        <v>4.477</v>
       </c>
       <c r="AT8" s="2" t="n">
-        <v>5.706</v>
+        <v>4.534</v>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>5.802</v>
+        <v>4.598</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>5.978</v>
+        <v>4.727</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>5.963</v>
+        <v>4.711</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>-2.5709</v>
+        <v>-1.4979</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>-1.3914</v>
+        <v>-0.86</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>-0.6349</v>
+        <v>-0.4262</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>-0.4221</v>
+        <v>-0.3204</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>-0.122</v>
+        <v>-0.0707</v>
       </c>
     </row>
     <row r="9">
@@ -1803,7 +1809,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6.789</v>
+        <v>6.802</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>14.72</v>
@@ -1826,19 +1832,19 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>1111110111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>1111111111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -1847,53 +1853,45 @@
         </is>
       </c>
       <c r="W9" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>4→3·1d ← 1A→4·4d ← 1B→1A·19d</t>
+          <t>1→4·5d</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr"/>
       <c r="AA9" s="2" t="inlineStr"/>
-      <c r="AB9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="n">
-        <v>42.7</v>
+        <v>-0</v>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-2.67</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>-3.04</v>
+        <v>-3.47</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>-3.32</v>
+        <v>-4.92</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>5.4</v>
+        <v>3.5</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AL9" s="2" t="inlineStr"/>
       <c r="AM9" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AN9" s="2" t="inlineStr"/>
       <c r="AO9" s="2" t="inlineStr"/>
@@ -1903,40 +1901,40 @@
         </is>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>3.299</v>
+        <v>7.07</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>2.919</v>
+        <v>7.267</v>
       </c>
       <c r="AS9" s="2" t="n">
-        <v>2.774</v>
+        <v>7.499</v>
       </c>
       <c r="AT9" s="2" t="n">
-        <v>2.737</v>
+        <v>7.61</v>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>2.708</v>
+        <v>7.701</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>2.767</v>
+        <v>8.006</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>2.748</v>
+        <v>8.015000000000001</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>6.4367</v>
+        <v>-2.5246</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>3.2887</v>
+        <v>-1.172</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>1.4077</v>
+        <v>-0.3577</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>0.357</v>
+        <v>-0.4898</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>0.427</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="10">
@@ -1951,7 +1949,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.393</v>
+        <v>3.406</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>41.01</v>
@@ -1974,19 +1972,19 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0111111101</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -1995,52 +1993,54 @@
         </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>1B(纠缠)</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>2A→1B·1d ← 3→2A·11d</t>
+          <t>3→2A·11d ← 2B→3·13d</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr"/>
       <c r="AA10" s="2" t="inlineStr"/>
-      <c r="AB10" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC10" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AD10" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="AC10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="n">
-        <v>4.56</v>
+        <v>16.97</v>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>20.87</v>
+        <v>19</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>7.79</v>
+        <v>3.13</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>9.52</v>
+        <v>6.36</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>85.8</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="AL10" s="2" t="inlineStr"/>
+        <v>33</v>
+      </c>
+      <c r="AL10" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AO10" s="2" t="inlineStr"/>
       <c r="AP10" s="2" t="inlineStr">
@@ -2049,40 +2049,40 @@
         </is>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>5.703</v>
+        <v>3.451</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>5.899</v>
+        <v>3.406</v>
       </c>
       <c r="AS10" s="2" t="n">
-        <v>6.019</v>
+        <v>3.396</v>
       </c>
       <c r="AT10" s="2" t="n">
-        <v>6.1</v>
+        <v>3.415</v>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>6.072</v>
+        <v>3.379</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>5.905</v>
+        <v>3.271</v>
       </c>
       <c r="AW10" s="2" t="n">
-        <v>5.841</v>
+        <v>3.228</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>-1.6704</v>
+        <v>0.7047</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>-1.1391</v>
+        <v>0.0372</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>-0.1607</v>
+        <v>0.3147</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>-0.0648</v>
+        <v>0.18</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.0456</v>
+        <v>0.1697</v>
       </c>
     </row>
     <row r="11">
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.493</v>
+        <v>0.497</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>-0.8100000000000001</v>
@@ -2120,19 +2120,19 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V11" s="2" t="inlineStr">
@@ -2145,43 +2145,49 @@
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4+(周J超卖·日线纠缠)</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>1A→4·5d</t>
+          <t>4→4+·4d ← 1→4·5d</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr"/>
       <c r="AA11" s="2" t="inlineStr"/>
-      <c r="AB11" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC11" s="2" t="inlineStr"/>
-      <c r="AD11" s="2" t="inlineStr"/>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD11" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="n">
-        <v>-31.64</v>
+        <v>-19.4</v>
       </c>
       <c r="AG11" s="2" t="n">
-        <v>0.74</v>
+        <v>2.64</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>3.9</v>
+        <v>6.26</v>
       </c>
       <c r="AI11" s="2" t="n">
-        <v>4.1</v>
+        <v>6.57</v>
       </c>
       <c r="AJ11" s="2" t="n">
-        <v>10.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="AL11" s="2" t="inlineStr"/>
+        <v>57</v>
+      </c>
+      <c r="AL11" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="AM11" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AN11" s="2" t="inlineStr"/>
       <c r="AO11" s="2" t="inlineStr"/>
@@ -2191,40 +2197,40 @@
         </is>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>0.89</v>
+        <v>0.495</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.493</v>
       </c>
       <c r="AS11" s="2" t="n">
-        <v>0.975</v>
+        <v>0.5</v>
       </c>
       <c r="AT11" s="2" t="n">
-        <v>1</v>
+        <v>0.509</v>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>1.017</v>
+        <v>0.513</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>1.027</v>
+        <v>0.516</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>1.058</v>
+        <v>0.53</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>-3.2233</v>
+        <v>-0.6145</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>-1.997</v>
+        <v>-0.7127</v>
       </c>
       <c r="AZ11" s="2" t="n">
-        <v>-0.8364</v>
+        <v>-0.3321</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>-0.3176</v>
+        <v>-0.0654</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>-0.3164</v>
+        <v>-0.194</v>
       </c>
     </row>
     <row r="12">
@@ -2239,7 +2245,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.373</v>
+        <v>0.377</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>9.880000000000001</v>
@@ -2260,19 +2266,19 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0110111010</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010111010</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
@@ -2285,12 +2291,12 @@
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>1B→1A·1d</t>
+          <t>1A→1·3d ← 1B→1A·6d ← 1A→1B·7d</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr"/>
@@ -2304,22 +2310,22 @@
       </c>
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="n">
-        <v>-24.57</v>
+        <v>-4.86</v>
       </c>
       <c r="AG12" s="2" t="n">
-        <v>8.99</v>
+        <v>11.28</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>-0.22</v>
+        <v>2.49</v>
       </c>
       <c r="AI12" s="2" t="n">
-        <v>8.050000000000001</v>
+        <v>11.94</v>
       </c>
       <c r="AJ12" s="2" t="n">
-        <v>62.1</v>
+        <v>61.1</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="AL12" s="2" t="inlineStr"/>
       <c r="AM12" s="2" t="inlineStr"/>
@@ -2331,40 +2337,40 @@
         </is>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>1.253</v>
+        <v>0.377</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>1.368</v>
+        <v>0.378</v>
       </c>
       <c r="AS12" s="2" t="n">
-        <v>1.415</v>
+        <v>0.376</v>
       </c>
       <c r="AT12" s="2" t="n">
-        <v>1.436</v>
+        <v>0.377</v>
       </c>
       <c r="AU12" s="2" t="n">
-        <v>1.471</v>
+        <v>0.383</v>
       </c>
       <c r="AV12" s="2" t="n">
-        <v>1.416</v>
+        <v>0.365</v>
       </c>
       <c r="AW12" s="2" t="n">
-        <v>1.443</v>
+        <v>0.371</v>
       </c>
       <c r="AX12" s="2" t="n">
-        <v>-4.0399</v>
+        <v>-0.1859</v>
       </c>
       <c r="AY12" s="2" t="n">
-        <v>-1.9715</v>
+        <v>-0.0283</v>
       </c>
       <c r="AZ12" s="2" t="n">
-        <v>-0.6663</v>
+        <v>0.1005</v>
       </c>
       <c r="BA12" s="2" t="n">
-        <v>-0.2566</v>
+        <v>0.1451</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>-0.2457</v>
+        <v>-0.0486</v>
       </c>
     </row>
     <row r="13">
@@ -2379,7 +2385,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.751</v>
+        <v>0.758</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>-4.85</v>
@@ -2394,25 +2400,25 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
       <c r="R13" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V13" s="2" t="inlineStr">
@@ -2425,39 +2431,39 @@
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4+(周J超卖·日线纠缠)</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>1A→4·9d ← 1B→1A·19d ← 4→1B·20d</t>
+          <t>4→4+·4d ← 4+→4·6d ← 1→4+·9d</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr"/>
       <c r="AA13" s="2" t="inlineStr"/>
       <c r="AB13" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="n">
-        <v>-36.53</v>
+        <v>-20.65</v>
       </c>
       <c r="AG13" s="2" t="n">
-        <v>-0.35</v>
+        <v>1.57</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>1.92</v>
+        <v>4.3</v>
       </c>
       <c r="AI13" s="2" t="n">
-        <v>2.61</v>
+        <v>4.63</v>
       </c>
       <c r="AJ13" s="2" t="n">
-        <v>18.1</v>
+        <v>15.8</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="AL13" s="2" t="inlineStr"/>
       <c r="AM13" s="2" t="inlineStr"/>
@@ -2469,40 +2475,40 @@
         </is>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>1.956</v>
+        <v>0.76</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>2.107</v>
+        <v>0.76</v>
       </c>
       <c r="AS13" s="2" t="n">
-        <v>2.22</v>
+        <v>0.773</v>
       </c>
       <c r="AT13" s="2" t="n">
-        <v>2.281</v>
+        <v>0.785</v>
       </c>
       <c r="AU13" s="2" t="n">
-        <v>2.311</v>
+        <v>0.789</v>
       </c>
       <c r="AV13" s="2" t="n">
-        <v>2.318</v>
+        <v>0.786</v>
       </c>
       <c r="AW13" s="2" t="n">
-        <v>2.437</v>
+        <v>0.824</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>-4.2017</v>
+        <v>-0.8008999999999999</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>-2.5011</v>
+        <v>-0.8296</v>
       </c>
       <c r="AZ13" s="2" t="n">
-        <v>-0.9863</v>
+        <v>-0.3245</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>-0.406</v>
+        <v>-0.0723</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>-0.3653</v>
+        <v>-0.2065</v>
       </c>
     </row>
     <row r="14">
@@ -2517,7 +2523,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.717</v>
+        <v>2.705</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>77.83</v>
@@ -2540,19 +2546,19 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>1111110111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>1111111111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V14" s="2" t="inlineStr">
@@ -2565,45 +2571,37 @@
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>4→3·1d ← 1A→4·15d</t>
+          <t>1→4·15d</t>
         </is>
       </c>
       <c r="Z14" s="2" t="inlineStr"/>
       <c r="AA14" s="2" t="inlineStr"/>
-      <c r="AB14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE14" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="inlineStr"/>
+      <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="n">
-        <v>32</v>
+        <v>-5.08</v>
       </c>
       <c r="AG14" s="2" t="n">
-        <v>-1.62</v>
+        <v>-4.11</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>-2.32</v>
+        <v>-3.61</v>
       </c>
       <c r="AI14" s="2" t="n">
-        <v>-2.49</v>
+        <v>-4.49</v>
       </c>
       <c r="AJ14" s="2" t="n">
-        <v>21.9</v>
+        <v>17.8</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="AL14" s="2" t="inlineStr"/>
       <c r="AM14" s="2" t="inlineStr"/>
@@ -2615,40 +2613,40 @@
         </is>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>1.395</v>
+        <v>2.826</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>1.253</v>
+        <v>2.903</v>
       </c>
       <c r="AS14" s="2" t="n">
-        <v>1.201</v>
+        <v>2.995</v>
       </c>
       <c r="AT14" s="2" t="n">
-        <v>1.187</v>
+        <v>3.031</v>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>1.167</v>
+        <v>3.041</v>
       </c>
       <c r="AV14" s="2" t="n">
-        <v>1.202</v>
+        <v>3.178</v>
       </c>
       <c r="AW14" s="2" t="n">
-        <v>1.206</v>
+        <v>3.212</v>
       </c>
       <c r="AX14" s="2" t="n">
-        <v>5.2512</v>
+        <v>-2.5593</v>
       </c>
       <c r="AY14" s="2" t="n">
-        <v>2.7934</v>
+        <v>-1.1037</v>
       </c>
       <c r="AZ14" s="2" t="n">
-        <v>1.474</v>
+        <v>-0.0916</v>
       </c>
       <c r="BA14" s="2" t="n">
-        <v>0.1715</v>
+        <v>-0.5706</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>0.32</v>
+        <v>-0.0508</v>
       </c>
     </row>
     <row r="15">
@@ -2663,7 +2661,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.028</v>
+        <v>1.031</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>81.33</v>
@@ -2707,14 +2705,18 @@
         </is>
       </c>
       <c r="W15" s="2" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="Y15" s="2" t="inlineStr"/>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>4+→4·6d ← 4→4+·11d ← 4+→4·14d</t>
+        </is>
+      </c>
       <c r="Z15" s="2" t="inlineStr"/>
       <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="n">
@@ -2724,22 +2726,22 @@
       <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="n">
-        <v>-15.68</v>
+        <v>-15.62</v>
       </c>
       <c r="AG15" s="2" t="n">
-        <v>-6.96</v>
+        <v>-9.56</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>0.8</v>
+        <v>-2.31</v>
       </c>
       <c r="AI15" s="2" t="n">
-        <v>0.37</v>
+        <v>-3.42</v>
       </c>
       <c r="AJ15" s="2" t="n">
-        <v>26.9</v>
+        <v>23.4</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="AL15" s="2" t="inlineStr"/>
       <c r="AM15" s="2" t="inlineStr"/>
@@ -2757,7 +2759,7 @@
         <v>1.085</v>
       </c>
       <c r="AS15" s="2" t="n">
-        <v>1.121</v>
+        <v>1.122</v>
       </c>
       <c r="AT15" s="2" t="n">
         <v>1.129</v>
@@ -2772,37 +2774,37 @@
         <v>1.298</v>
       </c>
       <c r="AX15" s="2" t="n">
-        <v>-2.168</v>
+        <v>-2.1542</v>
       </c>
       <c r="AY15" s="2" t="n">
-        <v>-1.0383</v>
+        <v>-1.0315</v>
       </c>
       <c r="AZ15" s="2" t="n">
-        <v>-0.1187</v>
+        <v>-0.1159</v>
       </c>
       <c r="BA15" s="2" t="n">
-        <v>-0.7467</v>
+        <v>-0.7454</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>-0.1568</v>
+        <v>-0.1562</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.414</v>
+        <v>1.006</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>-1.36</v>
+        <v>-0.29</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -2813,7 +2815,7 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>2</v>
@@ -2843,106 +2845,106 @@
         </is>
       </c>
       <c r="W16" s="2" t="n">
-        <v>192</v>
+        <v>58</v>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="Y16" s="2" t="inlineStr"/>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>4+→4·6d ← 4→4+·14d ← 4+→4·17d</t>
+        </is>
+      </c>
       <c r="Z16" s="2" t="inlineStr"/>
       <c r="AA16" s="2" t="inlineStr"/>
-      <c r="AB16" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC16" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AD16" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="n">
-        <v>-51.69</v>
+        <v>-14.72</v>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>-7.28</v>
+        <v>-8.49</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>2.95</v>
+        <v>-1.14</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>6.07</v>
+        <v>-1.71</v>
       </c>
       <c r="AJ16" s="2" t="n">
-        <v>51.7</v>
+        <v>0.3</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="AL16" s="2" t="inlineStr"/>
-      <c r="AM16" s="2" t="inlineStr"/>
+      <c r="AM16" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="AN16" s="2" t="inlineStr"/>
       <c r="AO16" s="2" t="inlineStr"/>
       <c r="AP16" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>0.972</v>
+        <v>1.042</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>1.033</v>
+        <v>1.065</v>
       </c>
       <c r="AS16" s="2" t="n">
-        <v>1.067</v>
+        <v>1.095</v>
       </c>
       <c r="AT16" s="2" t="n">
-        <v>1.09</v>
+        <v>1.12</v>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>1.119</v>
+        <v>1.149</v>
       </c>
       <c r="AV16" s="2" t="n">
-        <v>1.119</v>
+        <v>1.187</v>
       </c>
       <c r="AW16" s="2" t="n">
-        <v>1.247</v>
+        <v>1.228</v>
       </c>
       <c r="AX16" s="2" t="n">
-        <v>-3.0683</v>
+        <v>-2.2184</v>
       </c>
       <c r="AY16" s="2" t="n">
-        <v>-2.0239</v>
+        <v>-1.3227</v>
       </c>
       <c r="AZ16" s="2" t="n">
-        <v>-0.7447</v>
+        <v>-0.6039</v>
       </c>
       <c r="BA16" s="2" t="n">
-        <v>-0.5687</v>
+        <v>-0.6807</v>
       </c>
       <c r="BB16" s="2" t="n">
-        <v>-0.5169</v>
+        <v>-0.1472</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.005</v>
+        <v>0.9</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-0.29</v>
+        <v>14.64</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -2956,41 +2958,45 @@
         <v>9</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="V17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W17" s="2" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y17" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>2A→1·20d</t>
+        </is>
+      </c>
       <c r="Z17" s="2" t="inlineStr"/>
       <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr"/>
@@ -2998,87 +3004,87 @@
       <c r="AD17" s="2" t="inlineStr"/>
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="n">
-        <v>-16.68</v>
+        <v>17.95</v>
       </c>
       <c r="AG17" s="2" t="n">
-        <v>-7.47</v>
+        <v>2.66</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>-1.18</v>
+        <v>-4.84</v>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>-1.72</v>
+        <v>-8.390000000000001</v>
       </c>
       <c r="AJ17" s="2" t="n">
-        <v>1.2</v>
+        <v>-6.8</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="AL17" s="2" t="inlineStr"/>
       <c r="AM17" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="AN17" s="2" t="inlineStr"/>
       <c r="AO17" s="2" t="inlineStr"/>
       <c r="AP17" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>1.126</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>1.161</v>
+        <v>0.982</v>
       </c>
       <c r="AS17" s="2" t="n">
-        <v>1.2</v>
+        <v>1.023</v>
       </c>
       <c r="AT17" s="2" t="n">
-        <v>1.229</v>
+        <v>1.041</v>
       </c>
       <c r="AU17" s="2" t="n">
-        <v>1.263</v>
+        <v>1.069</v>
       </c>
       <c r="AV17" s="2" t="n">
-        <v>1.305</v>
+        <v>1.17</v>
       </c>
       <c r="AW17" s="2" t="n">
-        <v>1.35</v>
+        <v>1.029</v>
       </c>
       <c r="AX17" s="2" t="n">
-        <v>-2.6518</v>
+        <v>-3.9433</v>
       </c>
       <c r="AY17" s="2" t="n">
-        <v>-1.5372</v>
+        <v>-1.4312</v>
       </c>
       <c r="AZ17" s="2" t="n">
-        <v>-0.6868</v>
+        <v>-1.1299</v>
       </c>
       <c r="BA17" s="2" t="n">
-        <v>-0.7208</v>
+        <v>-0.3963</v>
       </c>
       <c r="BB17" s="2" t="n">
-        <v>-0.1668</v>
+        <v>0.1795</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.887</v>
+        <v>0.863</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>14.64</v>
+        <v>85.37</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -3088,137 +3094,143 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>1111111111</t>
         </is>
       </c>
       <c r="V18" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W18" s="2" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="Y18" s="2" t="inlineStr">
         <is>
-          <t>1B→1A·1d ← 2A→1B·20d</t>
+          <t>2B→2A·6d</t>
         </is>
       </c>
       <c r="Z18" s="2" t="inlineStr"/>
       <c r="AA18" s="2" t="inlineStr"/>
-      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="n">
-        <v>0.5</v>
+        <v>7.01</v>
       </c>
       <c r="AG18" s="2" t="n">
-        <v>3.16</v>
+        <v>19.92</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>-7.75</v>
+        <v>4.19</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>-8.9</v>
+        <v>12.85</v>
       </c>
       <c r="AJ18" s="2" t="n">
-        <v>-6.4</v>
+        <v>99.3</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="AL18" s="2" t="inlineStr"/>
-      <c r="AM18" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="AN18" s="2" t="inlineStr"/>
+        <v>56</v>
+      </c>
+      <c r="AL18" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="AM18" s="2" t="inlineStr"/>
+      <c r="AN18" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AO18" s="2" t="inlineStr"/>
       <c r="AP18" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>3.342</v>
+        <v>0.862</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>3.826</v>
+        <v>0.854</v>
       </c>
       <c r="AS18" s="2" t="n">
-        <v>4.142</v>
+        <v>0.848</v>
       </c>
       <c r="AT18" s="2" t="n">
-        <v>4.264</v>
+        <v>0.844</v>
       </c>
       <c r="AU18" s="2" t="n">
-        <v>4.421</v>
+        <v>0.831</v>
       </c>
       <c r="AV18" s="2" t="n">
-        <v>4.876</v>
+        <v>0.805</v>
       </c>
       <c r="AW18" s="2" t="n">
-        <v>4.298</v>
+        <v>0.799</v>
       </c>
       <c r="AX18" s="2" t="n">
-        <v>-7.3119</v>
+        <v>0.7857</v>
       </c>
       <c r="AY18" s="2" t="n">
-        <v>-3.1327</v>
+        <v>0.3273</v>
       </c>
       <c r="AZ18" s="2" t="n">
-        <v>-1.7851</v>
+        <v>0.3288</v>
       </c>
       <c r="BA18" s="2" t="n">
-        <v>-0.6997</v>
+        <v>0.2736</v>
       </c>
       <c r="BB18" s="2" t="n">
-        <v>0.005</v>
+        <v>0.0701</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.853</v>
+        <v>1.001</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>85.37</v>
+        <v>-8.65</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -3227,83 +3239,83 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V19" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W19" s="2" t="n">
-        <v>6</v>
+        <v>151</v>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>4+(周J超卖·日线纠缠)</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
-          <t>3→2A·6d</t>
+          <t>4→4+·13d</t>
         </is>
       </c>
       <c r="Z19" s="2" t="inlineStr"/>
       <c r="AA19" s="2" t="inlineStr"/>
-      <c r="AB19" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC19" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AB19" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="n">
-        <v>-7.2</v>
+        <v>-54.96</v>
       </c>
       <c r="AG19" s="2" t="n">
-        <v>18.81</v>
+        <v>-13.34</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>5.08</v>
+        <v>5.36</v>
       </c>
       <c r="AI19" s="2" t="n">
-        <v>11.82</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AJ19" s="2" t="n">
-        <v>99.09999999999999</v>
+        <v>24.8</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>81</v>
+        <v>38</v>
       </c>
       <c r="AL19" s="2" t="inlineStr"/>
       <c r="AM19" s="2" t="inlineStr"/>
-      <c r="AN19" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AN19" s="2" t="inlineStr"/>
       <c r="AO19" s="2" t="inlineStr"/>
       <c r="AP19" s="2" t="inlineStr">
         <is>
@@ -3311,58 +3323,58 @@
         </is>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>1.549</v>
+        <v>1.008</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>1.619</v>
+        <v>1.008</v>
       </c>
       <c r="AS19" s="2" t="n">
-        <v>1.651</v>
+        <v>1.014</v>
       </c>
       <c r="AT19" s="2" t="n">
-        <v>1.658</v>
+        <v>1.028</v>
       </c>
       <c r="AU19" s="2" t="n">
-        <v>1.644</v>
+        <v>1.07</v>
       </c>
       <c r="AV19" s="2" t="n">
-        <v>1.6</v>
+        <v>1.076</v>
       </c>
       <c r="AW19" s="2" t="n">
-        <v>1.593</v>
+        <v>1.209</v>
       </c>
       <c r="AX19" s="2" t="n">
-        <v>-1.9117</v>
+        <v>-0.4502</v>
       </c>
       <c r="AY19" s="2" t="n">
-        <v>-1.0189</v>
+        <v>-0.4374</v>
       </c>
       <c r="AZ19" s="2" t="n">
-        <v>-0.2205</v>
+        <v>-0.4243</v>
       </c>
       <c r="BA19" s="2" t="n">
-        <v>-0.0097</v>
+        <v>-0.457</v>
       </c>
       <c r="BB19" s="2" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.5496</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.002</v>
+        <v>1.712</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-8.65</v>
+        <v>-5.36</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -3371,30 +3383,28 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
@@ -3403,43 +3413,43 @@
         </is>
       </c>
       <c r="W20" s="2" t="n">
-        <v>151</v>
+        <v>9</v>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y20" s="2" t="inlineStr"/>
+          <t>4+(周J超卖·日线纠缠)</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>4→4+·4d ← 4+→4·6d ← 1→4+·9d</t>
+        </is>
+      </c>
       <c r="Z20" s="2" t="inlineStr"/>
       <c r="AA20" s="2" t="inlineStr"/>
-      <c r="AB20" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="AB20" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="n">
-        <v>-54.94</v>
+        <v>-22.42</v>
       </c>
       <c r="AG20" s="2" t="n">
-        <v>-12.42</v>
+        <v>-1.16</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>5.28</v>
+        <v>3.21</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>8.119999999999999</v>
+        <v>3.63</v>
       </c>
       <c r="AJ20" s="2" t="n">
-        <v>25.8</v>
+        <v>12</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="AL20" s="2" t="inlineStr"/>
       <c r="AM20" s="2" t="inlineStr"/>
@@ -3447,62 +3457,62 @@
       <c r="AO20" s="2" t="inlineStr"/>
       <c r="AP20" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>1.008</v>
+        <v>1.729</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>1.008</v>
+        <v>1.741</v>
       </c>
       <c r="AS20" s="2" t="n">
-        <v>1.014</v>
+        <v>1.774</v>
       </c>
       <c r="AT20" s="2" t="n">
-        <v>1.028</v>
+        <v>1.81</v>
       </c>
       <c r="AU20" s="2" t="n">
-        <v>1.07</v>
+        <v>1.819</v>
       </c>
       <c r="AV20" s="2" t="n">
-        <v>1.076</v>
+        <v>1.812</v>
       </c>
       <c r="AW20" s="2" t="n">
-        <v>1.209</v>
+        <v>1.876</v>
       </c>
       <c r="AX20" s="2" t="n">
-        <v>-0.4451</v>
+        <v>-1.0503</v>
       </c>
       <c r="AY20" s="2" t="n">
-        <v>-0.4348</v>
+        <v>-1.0089</v>
       </c>
       <c r="AZ20" s="2" t="n">
-        <v>-0.4233</v>
+        <v>-0.364</v>
       </c>
       <c r="BA20" s="2" t="n">
-        <v>-0.4566</v>
+        <v>-0.1214</v>
       </c>
       <c r="BB20" s="2" t="n">
-        <v>-0.5494</v>
+        <v>-0.2242</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.709</v>
+        <v>2.321</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-5.36</v>
+        <v>110.91</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -3511,188 +3521,204 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N21" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0111111011</t>
         </is>
       </c>
       <c r="V21" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W21" s="2" t="n">
-        <v>9</v>
+        <v>99</v>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2B</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr">
         <is>
-          <t>1A→4·9d ← 1B→1A·19d</t>
+          <t>2C→2B·5d ← 2B→2C·18d</t>
         </is>
       </c>
       <c r="Z21" s="2" t="inlineStr"/>
       <c r="AA21" s="2" t="inlineStr"/>
-      <c r="AB21" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC21" s="2" t="inlineStr"/>
+      <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="inlineStr"/>
       <c r="AF21" s="2" t="n">
-        <v>-22.46</v>
+        <v>28.55</v>
       </c>
       <c r="AG21" s="2" t="n">
-        <v>-1.41</v>
+        <v>29.03</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>1.85</v>
+        <v>0.46</v>
       </c>
       <c r="AI21" s="2" t="n">
-        <v>3.21</v>
+        <v>12.87</v>
       </c>
       <c r="AJ21" s="2" t="n">
-        <v>15.1</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="AL21" s="2" t="inlineStr"/>
+        <v>23</v>
+      </c>
+      <c r="AL21" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
       <c r="AM21" s="2" t="inlineStr"/>
-      <c r="AN21" s="2" t="inlineStr"/>
+      <c r="AN21" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AO21" s="2" t="inlineStr"/>
       <c r="AP21" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>1.729</v>
+        <v>2.379</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>1.741</v>
+        <v>2.356</v>
       </c>
       <c r="AS21" s="2" t="n">
-        <v>1.774</v>
+        <v>2.3</v>
       </c>
       <c r="AT21" s="2" t="n">
-        <v>1.81</v>
+        <v>2.275</v>
       </c>
       <c r="AU21" s="2" t="n">
-        <v>1.819</v>
+        <v>2.247</v>
       </c>
       <c r="AV21" s="2" t="n">
-        <v>1.812</v>
+        <v>2.215</v>
       </c>
       <c r="AW21" s="2" t="n">
-        <v>1.876</v>
+        <v>2.042</v>
       </c>
       <c r="AX21" s="2" t="n">
-        <v>-1.0591</v>
+        <v>1.0622</v>
       </c>
       <c r="AY21" s="2" t="n">
-        <v>-1.0132</v>
+        <v>0.8881</v>
       </c>
       <c r="AZ21" s="2" t="n">
-        <v>-0.3657</v>
+        <v>0.6552</v>
       </c>
       <c r="BA21" s="2" t="n">
-        <v>-0.1223</v>
+        <v>0.3504</v>
       </c>
       <c r="BB21" s="2" t="n">
-        <v>-0.2246</v>
+        <v>0.2855</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2.334</v>
+        <v>1.348</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>110.91</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
+        <v>6.69</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="n">
-        <v>-9</v>
+        <v>13</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y22" s="2" t="inlineStr">
         <is>
-          <t>2B→2A·1d ← 2C→2B·5d ← 2B→2C·18d</t>
+          <t>4+→4·2d ← 4→4+·4d ← 4+→4·7d</t>
         </is>
       </c>
       <c r="Z22" s="2" t="inlineStr"/>
@@ -3701,107 +3727,101 @@
       <c r="AC22" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD22" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
       <c r="AF22" s="2" t="n">
-        <v>4.81</v>
+        <v>-27.96</v>
       </c>
       <c r="AG22" s="2" t="n">
-        <v>31.93</v>
+        <v>-16.28</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>5.74</v>
+        <v>-2.98</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>15.36</v>
+        <v>-3.07</v>
       </c>
       <c r="AJ22" s="2" t="n">
-        <v>85.40000000000001</v>
+        <v>-0.1</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>63</v>
+        <v>11</v>
       </c>
       <c r="AL22" s="2" t="inlineStr"/>
-      <c r="AM22" s="2" t="inlineStr"/>
+      <c r="AM22" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="AN22" s="2" t="inlineStr"/>
       <c r="AO22" s="2" t="inlineStr"/>
       <c r="AP22" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>10.043</v>
+        <v>1.408</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>10.857</v>
+        <v>1.429</v>
       </c>
       <c r="AS22" s="2" t="n">
-        <v>11.042</v>
+        <v>1.464</v>
       </c>
       <c r="AT22" s="2" t="n">
-        <v>11.069</v>
+        <v>1.503</v>
       </c>
       <c r="AU22" s="2" t="n">
-        <v>11.055</v>
+        <v>1.56</v>
       </c>
       <c r="AV22" s="2" t="n">
-        <v>10.984</v>
+        <v>1.687</v>
       </c>
       <c r="AW22" s="2" t="n">
-        <v>10.166</v>
+        <v>1.8</v>
       </c>
       <c r="AX22" s="2" t="n">
-        <v>-3.1142</v>
+        <v>-1.6486</v>
       </c>
       <c r="AY22" s="2" t="n">
-        <v>-1.2436</v>
+        <v>-1.2648</v>
       </c>
       <c r="AZ22" s="2" t="n">
-        <v>-0.2137</v>
+        <v>-0.6054</v>
       </c>
       <c r="BA22" s="2" t="n">
-        <v>-0.08799999999999999</v>
+        <v>-0.966</v>
       </c>
       <c r="BB22" s="2" t="n">
-        <v>0.0481</v>
+        <v>-0.2796</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.337</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>6.69</v>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>79.97</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>1</v>
@@ -3810,125 +3830,127 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
+          <t>0010000000</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
           <t>0000000000</t>
         </is>
       </c>
-      <c r="U23" s="2" t="inlineStr">
-        <is>
-          <t>0000000000</t>
-        </is>
-      </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W23" s="2" t="n">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y23" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>2A→1·6d</t>
+        </is>
+      </c>
       <c r="Z23" s="2" t="inlineStr"/>
       <c r="AA23" s="2" t="inlineStr"/>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="n">
-        <v>-28.12</v>
+        <v>16.33</v>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>-16.13</v>
+        <v>-0.62</v>
       </c>
       <c r="AH23" s="2" t="n">
-        <v>-2.33</v>
+        <v>-9.65</v>
       </c>
       <c r="AI23" s="2" t="n">
-        <v>-3.19</v>
+        <v>-21.88</v>
       </c>
       <c r="AJ23" s="2" t="n">
-        <v>0.2</v>
+        <v>5.2</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AL23" s="2" t="inlineStr"/>
       <c r="AM23" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="AN23" s="2" t="inlineStr"/>
       <c r="AO23" s="2" t="inlineStr"/>
       <c r="AP23" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>1.406</v>
+        <v>0.86</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>1.428</v>
+        <v>0.916</v>
       </c>
       <c r="AS23" s="2" t="n">
-        <v>1.464</v>
+        <v>0.984</v>
       </c>
       <c r="AT23" s="2" t="n">
-        <v>1.503</v>
+        <v>0.999</v>
       </c>
       <c r="AU23" s="2" t="n">
-        <v>1.56</v>
+        <v>1.005</v>
       </c>
       <c r="AV23" s="2" t="n">
-        <v>1.687</v>
+        <v>1.108</v>
       </c>
       <c r="AW23" s="2" t="n">
-        <v>1.8</v>
+        <v>0.975</v>
       </c>
       <c r="AX23" s="2" t="n">
-        <v>-1.6873</v>
+        <v>-5.309</v>
       </c>
       <c r="AY23" s="2" t="n">
-        <v>-1.2839</v>
+        <v>-2.1096</v>
       </c>
       <c r="AZ23" s="2" t="n">
-        <v>-0.6126</v>
+        <v>-0.7655999999999999</v>
       </c>
       <c r="BA23" s="2" t="n">
-        <v>-0.9693000000000001</v>
+        <v>-0.628</v>
       </c>
       <c r="BB23" s="2" t="n">
-        <v>-0.2812</v>
+        <v>0.1633</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>1.25</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>79.97</v>
+        <v>55.37</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -3938,149 +3960,161 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0100111100</t>
         </is>
       </c>
       <c r="U24" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0100111110</t>
         </is>
       </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W24" s="2" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>2C(减速)</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr">
         <is>
-          <t>1B→1A·1d ← 2A→1B·6d</t>
+          <t>2A→2C·2d ← 2B→2A·13d ← 3→2B·17d</t>
         </is>
       </c>
       <c r="Z24" s="2" t="inlineStr"/>
       <c r="AA24" s="2" t="inlineStr"/>
-      <c r="AB24" s="2" t="inlineStr"/>
-      <c r="AC24" s="2" t="inlineStr"/>
+      <c r="AB24" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC24" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="n">
-        <v>1.83</v>
+        <v>24.58</v>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>2.35</v>
+        <v>17.63</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>-11.41</v>
+        <v>0.7</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>-18.37</v>
+        <v>0.48</v>
       </c>
       <c r="AJ24" s="2" t="n">
-        <v>7.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AL24" s="2" t="inlineStr"/>
-      <c r="AM24" s="2" t="n">
-        <v>14</v>
-      </c>
+      <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr"/>
       <c r="AO24" s="2" t="inlineStr"/>
       <c r="AP24" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>2.256</v>
+        <v>1.283</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>2.587</v>
+        <v>1.273</v>
       </c>
       <c r="AS24" s="2" t="n">
-        <v>2.87</v>
+        <v>1.275</v>
       </c>
       <c r="AT24" s="2" t="n">
-        <v>2.944</v>
+        <v>1.29</v>
       </c>
       <c r="AU24" s="2" t="n">
-        <v>2.983</v>
+        <v>1.273</v>
       </c>
       <c r="AV24" s="2" t="n">
-        <v>3.307</v>
+        <v>1.241</v>
       </c>
       <c r="AW24" s="2" t="n">
-        <v>2.915</v>
+        <v>1.207</v>
       </c>
       <c r="AX24" s="2" t="n">
-        <v>-8.070499999999999</v>
+        <v>0.3059</v>
       </c>
       <c r="AY24" s="2" t="n">
-        <v>-3.4839</v>
+        <v>-0.1895</v>
       </c>
       <c r="AZ24" s="2" t="n">
-        <v>-1.3181</v>
+        <v>0.3571</v>
       </c>
       <c r="BA24" s="2" t="n">
-        <v>-0.8793</v>
+        <v>0.1031</v>
       </c>
       <c r="BB24" s="2" t="n">
-        <v>0.0183</v>
+        <v>0.2458</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.244</v>
+        <v>0.714</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>55.37</v>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
+        <v>7.96</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
@@ -4093,7 +4127,7 @@
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0000000100</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr">
@@ -4103,135 +4137,121 @@
       </c>
       <c r="V25" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W25" s="2" t="n">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>1B(纠缠)</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y25" s="2" t="inlineStr">
         <is>
-          <t>2C→1B·1d ← 2A→2C·2d ← 3→2A·13d</t>
+          <t>4+→4·6d ← 4→4+·9d</t>
         </is>
       </c>
       <c r="Z25" s="2" t="inlineStr"/>
       <c r="AA25" s="2" t="inlineStr"/>
-      <c r="AB25" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC25" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AD25" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AB25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="n">
-        <v>9.039999999999999</v>
+        <v>-28.32</v>
       </c>
       <c r="AG25" s="2" t="n">
-        <v>21.2</v>
+        <v>-18.4</v>
       </c>
       <c r="AH25" s="2" t="n">
-        <v>7.48</v>
+        <v>-2.5</v>
       </c>
       <c r="AI25" s="2" t="n">
-        <v>7.01</v>
+        <v>-2.93</v>
       </c>
       <c r="AJ25" s="2" t="n">
-        <v>69.59999999999999</v>
+        <v>2</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="AL25" s="2" t="inlineStr"/>
-      <c r="AM25" s="2" t="inlineStr"/>
+      <c r="AM25" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AN25" s="2" t="inlineStr"/>
       <c r="AO25" s="2" t="inlineStr"/>
       <c r="AP25" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>2.665</v>
+        <v>0.746</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>2.808</v>
+        <v>0.76</v>
       </c>
       <c r="AS25" s="2" t="n">
-        <v>2.897</v>
+        <v>0.782</v>
       </c>
       <c r="AT25" s="2" t="n">
-        <v>2.962</v>
+        <v>0.796</v>
       </c>
       <c r="AU25" s="2" t="n">
-        <v>2.943</v>
+        <v>0.819</v>
       </c>
       <c r="AV25" s="2" t="n">
-        <v>2.885</v>
+        <v>0.895</v>
       </c>
       <c r="AW25" s="2" t="n">
-        <v>2.815</v>
+        <v>0.983</v>
       </c>
       <c r="AX25" s="2" t="n">
-        <v>-2.6454</v>
+        <v>-2.1631</v>
       </c>
       <c r="AY25" s="2" t="n">
-        <v>-1.6488</v>
+        <v>-1.1063</v>
       </c>
       <c r="AZ25" s="2" t="n">
-        <v>-0.2336</v>
+        <v>-0.4784</v>
       </c>
       <c r="BA25" s="2" t="n">
-        <v>-0.1984</v>
+        <v>-1.0643</v>
       </c>
       <c r="BB25" s="2" t="n">
-        <v>0.09039999999999999</v>
+        <v>-0.2832</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.711</v>
+        <v>0.521</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>7.96</v>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>89.25</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>1</v>
@@ -4240,14 +4260,14 @@
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
@@ -4257,18 +4277,22 @@
       </c>
       <c r="V26" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W26" s="2" t="n">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y26" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>2A→1·8d ← 3→2A·12d</t>
+        </is>
+      </c>
       <c r="Z26" s="2" t="inlineStr"/>
       <c r="AA26" s="2" t="inlineStr"/>
       <c r="AB26" s="2" t="inlineStr"/>
@@ -4276,94 +4300,104 @@
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="n">
-        <v>-28.4</v>
+        <v>12.26</v>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>-16.73</v>
+        <v>-3.14</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>-1.3</v>
+        <v>-10.42</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>-1.71</v>
+        <v>-21.45</v>
       </c>
       <c r="AJ26" s="2" t="n">
-        <v>2.7</v>
+        <v>8.9</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="AL26" s="2" t="inlineStr"/>
       <c r="AM26" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="AN26" s="2" t="inlineStr"/>
       <c r="AO26" s="2" t="inlineStr"/>
       <c r="AP26" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>0.745</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>0.76</v>
+        <v>0.595</v>
       </c>
       <c r="AS26" s="2" t="n">
-        <v>0.782</v>
+        <v>0.64</v>
       </c>
       <c r="AT26" s="2" t="n">
-        <v>0.796</v>
+        <v>0.648</v>
       </c>
       <c r="AU26" s="2" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.649</v>
       </c>
       <c r="AV26" s="2" t="n">
-        <v>0.895</v>
+        <v>0.718</v>
       </c>
       <c r="AW26" s="2" t="n">
-        <v>0.983</v>
+        <v>0.644</v>
       </c>
       <c r="AX26" s="2" t="n">
-        <v>-2.1828</v>
+        <v>-5.5798</v>
       </c>
       <c r="AY26" s="2" t="n">
-        <v>-1.1161</v>
+        <v>-2.0116</v>
       </c>
       <c r="AZ26" s="2" t="n">
-        <v>-0.4822</v>
+        <v>-0.6197</v>
       </c>
       <c r="BA26" s="2" t="n">
-        <v>-1.066</v>
+        <v>-0.7297</v>
       </c>
       <c r="BB26" s="2" t="n">
-        <v>-0.284</v>
+        <v>0.1226</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.519</v>
+        <v>2.07</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>89.25</v>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
+        <v>3.12</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="n">
@@ -4393,20 +4427,20 @@
       </c>
       <c r="V27" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W27" s="2" t="n">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y27" s="2" t="inlineStr">
         <is>
-          <t>1B→1A·1d ← 2A→1B·8d ← 3→2A·12d</t>
+          <t>4+→4·2d ← 4→4+·4d ← 4+→4·6d</t>
         </is>
       </c>
       <c r="Z27" s="2" t="inlineStr"/>
@@ -4416,129 +4450,119 @@
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="n">
-        <v>-5.32</v>
+        <v>-29.84</v>
       </c>
       <c r="AG27" s="2" t="n">
-        <v>0.71</v>
+        <v>-18.28</v>
       </c>
       <c r="AH27" s="2" t="n">
-        <v>-11.27</v>
+        <v>-3.27</v>
       </c>
       <c r="AI27" s="2" t="n">
-        <v>-17.14</v>
+        <v>-2.81</v>
       </c>
       <c r="AJ27" s="2" t="n">
-        <v>11.6</v>
+        <v>-1.4</v>
       </c>
       <c r="AK27" s="2" t="n">
         <v>11</v>
       </c>
       <c r="AL27" s="2" t="inlineStr"/>
       <c r="AM27" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AN27" s="2" t="inlineStr"/>
       <c r="AO27" s="2" t="inlineStr"/>
       <c r="AP27" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>2.832</v>
+        <v>2.166</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>3.308</v>
+        <v>2.199</v>
       </c>
       <c r="AS27" s="2" t="n">
-        <v>3.709</v>
+        <v>2.258</v>
       </c>
       <c r="AT27" s="2" t="n">
-        <v>3.8</v>
+        <v>2.306</v>
       </c>
       <c r="AU27" s="2" t="n">
-        <v>3.838</v>
+        <v>2.394</v>
       </c>
       <c r="AV27" s="2" t="n">
-        <v>4.279</v>
+        <v>2.611</v>
       </c>
       <c r="AW27" s="2" t="n">
-        <v>3.85</v>
+        <v>2.838</v>
       </c>
       <c r="AX27" s="2" t="n">
-        <v>-8.9693</v>
+        <v>-1.7804</v>
       </c>
       <c r="AY27" s="2" t="n">
-        <v>-3.7081</v>
+        <v>-1.1079</v>
       </c>
       <c r="AZ27" s="2" t="n">
-        <v>-1.3081</v>
+        <v>-0.5972</v>
       </c>
       <c r="BA27" s="2" t="n">
-        <v>-1.0401</v>
+        <v>-1.0365</v>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>-0.0532</v>
+        <v>-0.2984</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2.053</v>
+        <v>0.787</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>7.5</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="n">
         <v>13</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
-          <t>1111110111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>1111110111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V28" s="2" t="inlineStr">
@@ -4547,50 +4571,42 @@
         </is>
       </c>
       <c r="W28" s="2" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="Y28" s="2" t="inlineStr"/>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>4+→4·6d ← 4→4+·14d ← 4+→4·16d</t>
+        </is>
+      </c>
       <c r="Z28" s="2" t="inlineStr"/>
       <c r="AA28" s="2" t="inlineStr"/>
-      <c r="AB28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AB28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="inlineStr"/>
+      <c r="AD28" s="2" t="inlineStr"/>
+      <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="n">
-        <v>11.78</v>
+        <v>-17.65</v>
       </c>
       <c r="AG28" s="2" t="n">
-        <v>-17.3</v>
+        <v>-13.43</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>-1.58</v>
+        <v>-4.7</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>-2.1</v>
+        <v>-6.85</v>
       </c>
       <c r="AJ28" s="2" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="AK28" s="2" t="n">
-        <v>14</v>
-      </c>
+        <v>-5.4</v>
+      </c>
+      <c r="AK28" s="2" t="inlineStr"/>
       <c r="AL28" s="2" t="inlineStr"/>
-      <c r="AM28" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr"/>
       <c r="AO28" s="2" t="inlineStr"/>
       <c r="AP28" s="2" t="inlineStr">
@@ -4599,58 +4615,58 @@
         </is>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>0.952</v>
+        <v>0.828</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>0.821</v>
+        <v>0.861</v>
       </c>
       <c r="AS28" s="2" t="n">
-        <v>0.769</v>
+        <v>0.892</v>
       </c>
       <c r="AT28" s="2" t="n">
-        <v>0.76</v>
+        <v>0.912</v>
       </c>
       <c r="AU28" s="2" t="n">
-        <v>0.768</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="AV28" s="2" t="n">
-        <v>0.821</v>
+        <v>1.02</v>
       </c>
       <c r="AW28" s="2" t="n">
-        <v>0.885</v>
+        <v>1.024</v>
       </c>
       <c r="AX28" s="2" t="n">
-        <v>8.657999999999999</v>
+        <v>-2.8959</v>
       </c>
       <c r="AY28" s="2" t="n">
-        <v>4.0415</v>
+        <v>-1.6928</v>
       </c>
       <c r="AZ28" s="2" t="n">
-        <v>1.3653</v>
+        <v>-0.5815</v>
       </c>
       <c r="BA28" s="2" t="n">
-        <v>-0.1446</v>
+        <v>-0.8463000000000001</v>
       </c>
       <c r="BB28" s="2" t="n">
-        <v>0.1178</v>
+        <v>-0.1765</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.787</v>
+        <v>1.438</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>7.5</v>
+        <v>12.87</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -4661,10 +4677,10 @@
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -4673,7 +4689,7 @@
         <v>0</v>
       </c>
       <c r="S29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
@@ -4682,111 +4698,115 @@
       </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W29" s="2" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y29" s="2" t="inlineStr">
-        <is>
-          <t>1A→4·20d</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr"/>
       <c r="Z29" s="2" t="inlineStr"/>
       <c r="AA29" s="2" t="inlineStr"/>
-      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AB29" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AC29" s="2" t="inlineStr"/>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="n">
-        <v>-17.65</v>
+        <v>6.07</v>
       </c>
       <c r="AG29" s="2" t="n">
-        <v>-11.74</v>
+        <v>-1.15</v>
       </c>
       <c r="AH29" s="2" t="n">
-        <v>-5.62</v>
+        <v>-3.43</v>
       </c>
       <c r="AI29" s="2" t="n">
-        <v>-6.3</v>
+        <v>-7.23</v>
       </c>
       <c r="AJ29" s="2" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="AK29" s="2" t="inlineStr"/>
+        <v>-6.5</v>
+      </c>
+      <c r="AK29" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="AL29" s="2" t="inlineStr"/>
-      <c r="AM29" s="2" t="inlineStr"/>
+      <c r="AM29" s="2" t="n">
+        <v>14</v>
+      </c>
       <c r="AN29" s="2" t="inlineStr"/>
       <c r="AO29" s="2" t="inlineStr"/>
       <c r="AP29" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>0.828</v>
+        <v>1.49</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>0.861</v>
+        <v>1.562</v>
       </c>
       <c r="AS29" s="2" t="n">
-        <v>0.892</v>
+        <v>1.629</v>
       </c>
       <c r="AT29" s="2" t="n">
-        <v>0.913</v>
+        <v>1.659</v>
       </c>
       <c r="AU29" s="2" t="n">
-        <v>0.9409999999999999</v>
+        <v>1.703</v>
       </c>
       <c r="AV29" s="2" t="n">
-        <v>1.02</v>
+        <v>1.834</v>
       </c>
       <c r="AW29" s="2" t="n">
-        <v>1.024</v>
+        <v>1.676</v>
       </c>
       <c r="AX29" s="2" t="n">
-        <v>-2.8959</v>
+        <v>-3.8596</v>
       </c>
       <c r="AY29" s="2" t="n">
-        <v>-1.6928</v>
+        <v>-1.5157</v>
       </c>
       <c r="AZ29" s="2" t="n">
-        <v>-0.5815</v>
+        <v>-1.0734</v>
       </c>
       <c r="BA29" s="2" t="n">
-        <v>-0.8463000000000001</v>
+        <v>-0.4752</v>
       </c>
       <c r="BB29" s="2" t="n">
-        <v>-0.1765</v>
+        <v>0.0607</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.418</v>
+        <v>0.329</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>12.87</v>
+        <v>52.3</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -4796,29 +4816,27 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0100111100</t>
         </is>
       </c>
       <c r="U30" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0010111000</t>
         </is>
       </c>
       <c r="V30" s="2" t="inlineStr">
@@ -4827,16 +4845,16 @@
         </is>
       </c>
       <c r="W30" s="2" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y30" s="2" t="inlineStr">
         <is>
-          <t>1B→1A·2d</t>
+          <t>1A→1·3d ← 1B→1A·6d ← 1A→1B·7d</t>
         </is>
       </c>
       <c r="Z30" s="2" t="inlineStr"/>
@@ -4846,87 +4864,85 @@
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="n">
-        <v>5.76</v>
+        <v>-2.78</v>
       </c>
       <c r="AG30" s="2" t="n">
-        <v>-0.99</v>
+        <v>7.74</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>-7.4</v>
+        <v>0.66</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>-8.1</v>
+        <v>8.27</v>
       </c>
       <c r="AJ30" s="2" t="n">
-        <v>-6.3</v>
+        <v>67.2</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="AL30" s="2" t="inlineStr"/>
-      <c r="AM30" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr"/>
       <c r="AO30" s="2" t="inlineStr"/>
       <c r="AP30" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>1.486</v>
+        <v>0.336</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>1.56</v>
+        <v>0.339</v>
       </c>
       <c r="AS30" s="2" t="n">
-        <v>1.628</v>
+        <v>0.339</v>
       </c>
       <c r="AT30" s="2" t="n">
-        <v>1.658</v>
+        <v>0.339</v>
       </c>
       <c r="AU30" s="2" t="n">
-        <v>1.703</v>
+        <v>0.341</v>
       </c>
       <c r="AV30" s="2" t="n">
-        <v>1.833</v>
+        <v>0.326</v>
       </c>
       <c r="AW30" s="2" t="n">
-        <v>1.676</v>
+        <v>0.336</v>
       </c>
       <c r="AX30" s="2" t="n">
-        <v>-3.9213</v>
+        <v>-0.6756</v>
       </c>
       <c r="AY30" s="2" t="n">
-        <v>-1.5467</v>
+        <v>-0.118</v>
       </c>
       <c r="AZ30" s="2" t="n">
-        <v>-1.0854</v>
+        <v>0.2082</v>
       </c>
       <c r="BA30" s="2" t="n">
-        <v>-0.4808</v>
+        <v>0.0615</v>
       </c>
       <c r="BB30" s="2" t="n">
-        <v>0.0576</v>
+        <v>-0.0278</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.328</v>
+        <v>0.417</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>52.3</v>
+        <v>-1.36</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -4940,41 +4956,43 @@
       <c r="N31" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S31" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0000000100</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010110</t>
         </is>
       </c>
       <c r="V31" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W31" s="2" t="n">
-        <v>33</v>
+        <v>192</v>
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>4+(周J超卖·日线纠缠)</t>
         </is>
       </c>
       <c r="Y31" s="2" t="inlineStr">
         <is>
-          <t>1B→1A·1d</t>
+          <t>4→4+·14d</t>
         </is>
       </c>
       <c r="Z31" s="2" t="inlineStr"/>
@@ -4984,22 +5002,22 @@
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="n">
-        <v>-20.1</v>
+        <v>-37.27</v>
       </c>
       <c r="AG31" s="2" t="n">
-        <v>7.43</v>
+        <v>-5.34</v>
       </c>
       <c r="AH31" s="2" t="n">
-        <v>-1.64</v>
+        <v>3.77</v>
       </c>
       <c r="AI31" s="2" t="n">
-        <v>6.5</v>
+        <v>9.33</v>
       </c>
       <c r="AJ31" s="2" t="n">
-        <v>69.7</v>
+        <v>52</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="AL31" s="2" t="inlineStr"/>
       <c r="AM31" s="2" t="inlineStr"/>
@@ -5011,40 +5029,40 @@
         </is>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>0.907</v>
+        <v>0.417</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>0.986</v>
+        <v>0.414</v>
       </c>
       <c r="AS31" s="2" t="n">
-        <v>1.021</v>
+        <v>0.413</v>
       </c>
       <c r="AT31" s="2" t="n">
-        <v>1.034</v>
+        <v>0.417</v>
       </c>
       <c r="AU31" s="2" t="n">
-        <v>1.05</v>
+        <v>0.425</v>
       </c>
       <c r="AV31" s="2" t="n">
-        <v>1.009</v>
+        <v>0.422</v>
       </c>
       <c r="AW31" s="2" t="n">
-        <v>1.044</v>
+        <v>0.469</v>
       </c>
       <c r="AX31" s="2" t="n">
-        <v>-4.068</v>
+        <v>0.2368</v>
       </c>
       <c r="AY31" s="2" t="n">
-        <v>-1.8332</v>
+        <v>-0.3888</v>
       </c>
       <c r="AZ31" s="2" t="n">
-        <v>-0.4772</v>
+        <v>-0.1053</v>
       </c>
       <c r="BA31" s="2" t="n">
-        <v>-0.2961</v>
+        <v>-0.2478</v>
       </c>
       <c r="BB31" s="2" t="n">
-        <v>-0.201</v>
+        <v>-0.3727</v>
       </c>
     </row>
   </sheetData>
@@ -5311,7 +5329,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stage (Weinstein 大阶段 v2引擎 2026-10-15: EMA30W(150日EMA)锚+双确认斜率): 锚斜率=EMA30W变化年化(4周×13 与 13周×3.88 双确认)。2=双确认均&gt;+8% 4=均&lt;-6%(不对称,跌快于涨); 放平带(-6%~+8%)按52周位置+价格确认分1/3: 3=pos52w&gt;0.55且价≥0.95×EMA30W 1=pos&lt;0.45且价≤1.05×EMA30W, 0.45~0.55滞回维持原状态。NA=历史&lt;300交易日</t>
+          <t xml:space="preserve">  Stage (Weinstein 大阶段 v2.1引擎: EMA30W(150日EMA)锚, 判定优先级从高到低): ①均线排列覆盖: MA20&gt;MA50&gt;MA100&gt;MA150(简单均线)多头排列→强制Stage2; MA20&lt;MA50&lt;MA100&lt;MA150空头排列→强制Stage4(忽略斜率, 解决慢磨盲区) ②斜率双确认: EMA30W变化年化(4周×13与13周×3.88)均&gt;+8%→2; 均&lt;-6%→4(不对称) ③放平带: 52周位置+价格确认分1/3(3:pos&gt;0.55且价≥0.95×EMA30W; 1:pos&lt;0.45且价≤1.05×; 0.45~0.55滞回)。NA=历史&lt;300交易日</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5350,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  子档(v2): 1A=价&lt;EMA10W且EMA10W≤EMA30W 1B=站上EMA10W或金叉 2A=修复态(2区回调未满配)或刚确立(进2区/金叉≤10日) 2B=满配多头排列(slope10&gt;0·EMA10W&gt;EMA30W·10日前也是) 2C=满配+延伸/减速/顶背离; 3/4不分档。括号内标记: 1B→纠缠(&lt;3%)·周线底背离; 2C→延伸(&gt;25%)·减速·顶背离</t>
+          <t xml:space="preserve">  子档(v2.1): 4+=止跌(日线MA5/10/20纠缠+快线&gt;慢线+周J超卖或底背离, 价&lt;EMA10W) | 1=过渡(价&lt;EMA10W) | 1A=早期修复(价≥EMA10W) | 1B=强筑底(站稳MA5/10/20全三条+全部斜率上行+周MACD DIF&gt;DEA; 标记:预金叉·纠缠·底背离) | 2A=修复态或刚确立(≤10日) | 2B=满配(slope10&gt;0·EMA10W&gt;EMA30W·10日前也是) | 2C=满配+延伸/减速/顶背离 | 3/4不分档。4+的标记: 周J超卖·底背离·日线纠缠; 2C的标记: 延伸(&gt;25%)·减速·顶背离</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-16
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$BB$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$BC$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB31"/>
+  <dimension ref="A1:BC31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -525,6 +525,7 @@
     <col width="11" customWidth="1" min="52" max="52"/>
     <col width="11" customWidth="1" min="53" max="53"/>
     <col width="11" customWidth="1" min="54" max="54"/>
+    <col width="11" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -650,150 +651,155 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>子档标记</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>子档变化</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>1→2</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>3→4</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>KDJ Cross</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>日MACD Cross</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>5_10 Cross</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>10_50 Cross</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>年线斜率</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300_1W</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300_4W</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>风险度</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>动量</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>DS信号</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>B距今</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>S距今</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>急杀</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>周线档</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>5D MV</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>10D MV</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>20D MV</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>30D MV</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>50D MV</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>100D MV</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>200D MV</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>10D斜率</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>20D斜率</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>50D斜率</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>100D斜率</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>200D斜率</t>
         </is>
@@ -862,80 +868,81 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>1→4·4d</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr"/>
       <c r="AA2" s="2" t="inlineStr"/>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr"/>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
-      <c r="AF2" s="2" t="n">
+      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="n">
         <v>-8.5</v>
       </c>
-      <c r="AG2" s="2" t="n">
+      <c r="AH2" s="2" t="n">
         <v>-8.359999999999999</v>
       </c>
-      <c r="AH2" s="2" t="n">
+      <c r="AI2" s="2" t="n">
         <v>-4.75</v>
       </c>
-      <c r="AI2" s="2" t="n">
+      <c r="AJ2" s="2" t="n">
         <v>-9.5</v>
       </c>
-      <c r="AJ2" s="2" t="n">
+      <c r="AK2" s="2" t="n">
         <v>-5.9</v>
       </c>
-      <c r="AK2" s="2" t="n">
+      <c r="AL2" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL2" s="2" t="inlineStr"/>
-      <c r="AM2" s="2" t="n">
+      <c r="AM2" s="2" t="inlineStr"/>
+      <c r="AN2" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AN2" s="2" t="inlineStr"/>
       <c r="AO2" s="2" t="inlineStr"/>
-      <c r="AP2" s="2" t="inlineStr">
+      <c r="AP2" s="2" t="inlineStr"/>
+      <c r="AQ2" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AQ2" s="2" t="n">
+      <c r="AR2" s="2" t="n">
         <v>2.944</v>
       </c>
-      <c r="AR2" s="2" t="n">
+      <c r="AS2" s="2" t="n">
         <v>3.056</v>
       </c>
-      <c r="AS2" s="2" t="n">
+      <c r="AT2" s="2" t="n">
         <v>3.205</v>
       </c>
-      <c r="AT2" s="2" t="n">
+      <c r="AU2" s="2" t="n">
         <v>3.268</v>
       </c>
-      <c r="AU2" s="2" t="n">
+      <c r="AV2" s="2" t="n">
         <v>3.371</v>
       </c>
-      <c r="AV2" s="2" t="n">
+      <c r="AW2" s="2" t="n">
         <v>3.658</v>
       </c>
-      <c r="AW2" s="2" t="n">
+      <c r="AX2" s="2" t="n">
         <v>3.521</v>
       </c>
-      <c r="AX2" s="2" t="n">
+      <c r="AY2" s="2" t="n">
         <v>-3.5352</v>
       </c>
-      <c r="AY2" s="2" t="n">
+      <c r="AZ2" s="2" t="n">
         <v>-1.6342</v>
       </c>
-      <c r="AZ2" s="2" t="n">
+      <c r="BA2" s="2" t="n">
         <v>-0.8365</v>
       </c>
-      <c r="BA2" s="2" t="n">
+      <c r="BB2" s="2" t="n">
         <v>-0.7159</v>
       </c>
-      <c r="BB2" s="2" t="n">
+      <c r="BC2" s="2" t="n">
         <v>-0.08500000000000001</v>
       </c>
     </row>
@@ -1002,80 +1009,81 @@
           <t>1</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr">
         <is>
           <t>4+→1·8d ← 1→4+·9d</t>
         </is>
       </c>
-      <c r="Z3" s="2" t="inlineStr"/>
       <c r="AA3" s="2" t="inlineStr"/>
-      <c r="AB3" s="2" t="n">
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AC3" s="2" t="inlineStr"/>
       <c r="AD3" s="2" t="inlineStr"/>
       <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="n">
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="n">
         <v>-12.91</v>
       </c>
-      <c r="AG3" s="2" t="n">
+      <c r="AH3" s="2" t="n">
         <v>3.05</v>
       </c>
-      <c r="AH3" s="2" t="n">
+      <c r="AI3" s="2" t="n">
         <v>4.14</v>
       </c>
-      <c r="AI3" s="2" t="n">
+      <c r="AJ3" s="2" t="n">
         <v>5.13</v>
       </c>
-      <c r="AJ3" s="2" t="n">
+      <c r="AK3" s="2" t="n">
         <v>48.5</v>
       </c>
-      <c r="AK3" s="2" t="n">
+      <c r="AL3" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="AL3" s="2" t="inlineStr"/>
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr"/>
       <c r="AO3" s="2" t="inlineStr"/>
-      <c r="AP3" s="2" t="inlineStr">
+      <c r="AP3" s="2" t="inlineStr"/>
+      <c r="AQ3" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ3" s="2" t="n">
+      <c r="AR3" s="2" t="n">
         <v>1.423</v>
       </c>
-      <c r="AR3" s="2" t="n">
+      <c r="AS3" s="2" t="n">
         <v>1.431</v>
       </c>
-      <c r="AS3" s="2" t="n">
+      <c r="AT3" s="2" t="n">
         <v>1.444</v>
       </c>
-      <c r="AT3" s="2" t="n">
+      <c r="AU3" s="2" t="n">
         <v>1.46</v>
       </c>
-      <c r="AU3" s="2" t="n">
+      <c r="AV3" s="2" t="n">
         <v>1.48</v>
       </c>
-      <c r="AV3" s="2" t="n">
+      <c r="AW3" s="2" t="n">
         <v>1.463</v>
       </c>
-      <c r="AW3" s="2" t="n">
+      <c r="AX3" s="2" t="n">
         <v>1.511</v>
       </c>
-      <c r="AX3" s="2" t="n">
+      <c r="AY3" s="2" t="n">
         <v>-0.6111</v>
       </c>
-      <c r="AY3" s="2" t="n">
+      <c r="AZ3" s="2" t="n">
         <v>-0.5956</v>
       </c>
-      <c r="AZ3" s="2" t="n">
+      <c r="BA3" s="2" t="n">
         <v>-0.252</v>
       </c>
-      <c r="BA3" s="2" t="n">
+      <c r="BB3" s="2" t="n">
         <v>-0.1896</v>
       </c>
-      <c r="BB3" s="2" t="n">
+      <c r="BC3" s="2" t="n">
         <v>-0.1291</v>
       </c>
     </row>
@@ -1137,85 +1145,90 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>4+(底背离·日线纠缠)</t>
+          <t>4+</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
+          <t>底背离·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
           <t>4→4+·3d ← 4+→4·4d ← 4→4+·20d</t>
         </is>
       </c>
-      <c r="Z4" s="2" t="inlineStr"/>
       <c r="AA4" s="2" t="inlineStr"/>
-      <c r="AB4" s="2" t="inlineStr">
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AC4" s="2" t="inlineStr"/>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
-      <c r="AF4" s="2" t="n">
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="n">
         <v>-24.3</v>
       </c>
-      <c r="AG4" s="2" t="n">
+      <c r="AH4" s="2" t="n">
         <v>0.03</v>
       </c>
-      <c r="AH4" s="2" t="n">
+      <c r="AI4" s="2" t="n">
         <v>4.78</v>
       </c>
-      <c r="AI4" s="2" t="n">
+      <c r="AJ4" s="2" t="n">
         <v>8.33</v>
       </c>
-      <c r="AJ4" s="2" t="n">
+      <c r="AK4" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="AK4" s="2" t="n">
+      <c r="AL4" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="AL4" s="2" t="inlineStr"/>
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr"/>
       <c r="AO4" s="2" t="inlineStr"/>
-      <c r="AP4" s="2" t="inlineStr">
+      <c r="AP4" s="2" t="inlineStr"/>
+      <c r="AQ4" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ4" s="2" t="n">
+      <c r="AR4" s="2" t="n">
         <v>0.661</v>
-      </c>
-      <c r="AR4" s="2" t="n">
-        <v>0.656</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>0.656</v>
       </c>
       <c r="AT4" s="2" t="n">
+        <v>0.656</v>
+      </c>
+      <c r="AU4" s="2" t="n">
         <v>0.662</v>
       </c>
-      <c r="AU4" s="2" t="n">
+      <c r="AV4" s="2" t="n">
         <v>0.667</v>
       </c>
-      <c r="AV4" s="2" t="n">
+      <c r="AW4" s="2" t="n">
         <v>0.659</v>
       </c>
-      <c r="AW4" s="2" t="n">
+      <c r="AX4" s="2" t="n">
         <v>0.714</v>
       </c>
-      <c r="AX4" s="2" t="n">
+      <c r="AY4" s="2" t="n">
         <v>0.2711</v>
       </c>
-      <c r="AY4" s="2" t="n">
+      <c r="AZ4" s="2" t="n">
         <v>-0.3545</v>
       </c>
-      <c r="AZ4" s="2" t="n">
+      <c r="BA4" s="2" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="BA4" s="2" t="n">
+      <c r="BB4" s="2" t="n">
         <v>-0.1886</v>
       </c>
-      <c r="BB4" s="2" t="n">
+      <c r="BC4" s="2" t="n">
         <v>-0.243</v>
       </c>
     </row>
@@ -1288,86 +1301,87 @@
           <t>2B</t>
         </is>
       </c>
-      <c r="Y5" s="2" t="inlineStr">
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>2A→2B·4d ← 3→2A·15d</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr"/>
       <c r="AA5" s="2" t="inlineStr"/>
-      <c r="AB5" s="2" t="n">
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AC5" s="2" t="inlineStr">
+      <c r="AD5" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr"/>
-      <c r="AF5" s="2" t="n">
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="n">
         <v>58.36</v>
       </c>
-      <c r="AG5" s="2" t="n">
+      <c r="AH5" s="2" t="n">
         <v>39.38</v>
       </c>
-      <c r="AH5" s="2" t="n">
+      <c r="AI5" s="2" t="n">
         <v>-4.54</v>
       </c>
-      <c r="AI5" s="2" t="n">
+      <c r="AJ5" s="2" t="n">
         <v>13.86</v>
       </c>
-      <c r="AJ5" s="2" t="n">
+      <c r="AK5" s="2" t="n">
         <v>98.59999999999999</v>
       </c>
-      <c r="AK5" s="2" t="n">
+      <c r="AL5" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="AL5" s="2" t="inlineStr"/>
       <c r="AM5" s="2" t="inlineStr"/>
-      <c r="AN5" s="2" t="n">
+      <c r="AN5" s="2" t="inlineStr"/>
+      <c r="AO5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="AO5" s="2" t="inlineStr"/>
-      <c r="AP5" s="2" t="inlineStr">
+      <c r="AP5" s="2" t="inlineStr"/>
+      <c r="AQ5" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ5" s="2" t="n">
+      <c r="AR5" s="2" t="n">
         <v>1.874</v>
       </c>
-      <c r="AR5" s="2" t="n">
+      <c r="AS5" s="2" t="n">
         <v>1.836</v>
       </c>
-      <c r="AS5" s="2" t="n">
+      <c r="AT5" s="2" t="n">
         <v>1.798</v>
       </c>
-      <c r="AT5" s="2" t="n">
+      <c r="AU5" s="2" t="n">
         <v>1.75</v>
       </c>
-      <c r="AU5" s="2" t="n">
+      <c r="AV5" s="2" t="n">
         <v>1.657</v>
       </c>
-      <c r="AV5" s="2" t="n">
+      <c r="AW5" s="2" t="n">
         <v>1.59</v>
       </c>
-      <c r="AW5" s="2" t="n">
+      <c r="AX5" s="2" t="n">
         <v>1.529</v>
       </c>
-      <c r="AX5" s="2" t="n">
+      <c r="AY5" s="2" t="n">
         <v>2.0247</v>
       </c>
-      <c r="AY5" s="2" t="n">
+      <c r="AZ5" s="2" t="n">
         <v>1.2621</v>
       </c>
-      <c r="AZ5" s="2" t="n">
+      <c r="BA5" s="2" t="n">
         <v>1.2166</v>
       </c>
-      <c r="BA5" s="2" t="n">
+      <c r="BB5" s="2" t="n">
         <v>0.361</v>
       </c>
-      <c r="BB5" s="2" t="n">
+      <c r="BC5" s="2" t="n">
         <v>0.5836</v>
       </c>
     </row>
@@ -1432,80 +1446,81 @@
           <t>1</t>
         </is>
       </c>
-      <c r="Y6" s="2" t="inlineStr">
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr">
         <is>
           <t>3→1·3d ← 1+→3·12d ← 1→1+·13d</t>
         </is>
       </c>
-      <c r="Z6" s="2" t="inlineStr"/>
       <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="inlineStr"/>
-      <c r="AC6" s="2" t="n">
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
-      <c r="AF6" s="2" t="n">
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="n">
         <v>-7.18</v>
       </c>
-      <c r="AG6" s="2" t="n">
+      <c r="AH6" s="2" t="n">
         <v>7.08</v>
       </c>
-      <c r="AH6" s="2" t="n">
+      <c r="AI6" s="2" t="n">
         <v>0.12</v>
       </c>
-      <c r="AI6" s="2" t="n">
+      <c r="AJ6" s="2" t="n">
         <v>7.47</v>
       </c>
-      <c r="AJ6" s="2" t="n">
+      <c r="AK6" s="2" t="n">
         <v>45.7</v>
       </c>
-      <c r="AK6" s="2" t="n">
+      <c r="AL6" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="AL6" s="2" t="inlineStr"/>
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr"/>
       <c r="AO6" s="2" t="inlineStr"/>
-      <c r="AP6" s="2" t="inlineStr">
+      <c r="AP6" s="2" t="inlineStr"/>
+      <c r="AQ6" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ6" s="2" t="n">
+      <c r="AR6" s="2" t="n">
         <v>0.823</v>
       </c>
-      <c r="AR6" s="2" t="n">
+      <c r="AS6" s="2" t="n">
         <v>0.835</v>
       </c>
-      <c r="AS6" s="2" t="n">
+      <c r="AT6" s="2" t="n">
         <v>0.836</v>
       </c>
-      <c r="AT6" s="2" t="n">
+      <c r="AU6" s="2" t="n">
         <v>0.841</v>
       </c>
-      <c r="AU6" s="2" t="n">
+      <c r="AV6" s="2" t="n">
         <v>0.86</v>
       </c>
-      <c r="AV6" s="2" t="n">
+      <c r="AW6" s="2" t="n">
         <v>0.828</v>
       </c>
-      <c r="AW6" s="2" t="n">
+      <c r="AX6" s="2" t="n">
         <v>0.832</v>
       </c>
-      <c r="AX6" s="2" t="n">
+      <c r="AY6" s="2" t="n">
         <v>-0.9651999999999999</v>
       </c>
-      <c r="AY6" s="2" t="n">
+      <c r="AZ6" s="2" t="n">
         <v>-0.3397</v>
       </c>
-      <c r="AZ6" s="2" t="n">
+      <c r="BA6" s="2" t="n">
         <v>-0.1821</v>
       </c>
-      <c r="BA6" s="2" t="n">
+      <c r="BB6" s="2" t="n">
         <v>0.0717</v>
       </c>
-      <c r="BB6" s="2" t="n">
+      <c r="BC6" s="2" t="n">
         <v>-0.0718</v>
       </c>
     </row>
@@ -1575,75 +1590,76 @@
       <c r="Y7" s="2" t="inlineStr"/>
       <c r="Z7" s="2" t="inlineStr"/>
       <c r="AA7" s="2" t="inlineStr"/>
-      <c r="AB7" s="2" t="inlineStr">
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
-      <c r="AF7" s="2" t="n">
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="n">
         <v>-6.44</v>
       </c>
-      <c r="AG7" s="2" t="n">
+      <c r="AH7" s="2" t="n">
         <v>5.72</v>
       </c>
-      <c r="AH7" s="2" t="n">
+      <c r="AI7" s="2" t="n">
         <v>1.91</v>
       </c>
-      <c r="AI7" s="2" t="n">
+      <c r="AJ7" s="2" t="n">
         <v>4.47</v>
       </c>
-      <c r="AJ7" s="2" t="n">
+      <c r="AK7" s="2" t="n">
         <v>10.5</v>
       </c>
-      <c r="AK7" s="2" t="n">
+      <c r="AL7" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="AL7" s="2" t="inlineStr"/>
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr"/>
       <c r="AO7" s="2" t="inlineStr"/>
-      <c r="AP7" s="2" t="inlineStr">
+      <c r="AP7" s="2" t="inlineStr"/>
+      <c r="AQ7" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ7" s="2" t="n">
+      <c r="AR7" s="2" t="n">
         <v>2.907</v>
       </c>
-      <c r="AR7" s="2" t="n">
+      <c r="AS7" s="2" t="n">
         <v>2.92</v>
       </c>
-      <c r="AS7" s="2" t="n">
+      <c r="AT7" s="2" t="n">
         <v>2.953</v>
       </c>
-      <c r="AT7" s="2" t="n">
+      <c r="AU7" s="2" t="n">
         <v>2.979</v>
       </c>
-      <c r="AU7" s="2" t="n">
+      <c r="AV7" s="2" t="n">
         <v>2.996</v>
       </c>
-      <c r="AV7" s="2" t="n">
+      <c r="AW7" s="2" t="n">
         <v>3.006</v>
       </c>
-      <c r="AW7" s="2" t="n">
+      <c r="AX7" s="2" t="n">
         <v>3.038</v>
       </c>
-      <c r="AX7" s="2" t="n">
+      <c r="AY7" s="2" t="n">
         <v>-0.7278</v>
       </c>
-      <c r="AY7" s="2" t="n">
+      <c r="AZ7" s="2" t="n">
         <v>-0.5137</v>
       </c>
-      <c r="AZ7" s="2" t="n">
+      <c r="BA7" s="2" t="n">
         <v>-0.2413</v>
       </c>
-      <c r="BA7" s="2" t="n">
+      <c r="BB7" s="2" t="n">
         <v>-0.1261</v>
       </c>
-      <c r="BB7" s="2" t="n">
+      <c r="BC7" s="2" t="n">
         <v>-0.0644</v>
       </c>
     </row>
@@ -1719,77 +1735,78 @@
       <c r="Y8" s="2" t="inlineStr"/>
       <c r="Z8" s="2" t="inlineStr"/>
       <c r="AA8" s="2" t="inlineStr"/>
-      <c r="AB8" s="2" t="inlineStr">
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="AC8" s="2" t="inlineStr"/>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="inlineStr"/>
-      <c r="AF8" s="2" t="n">
+      <c r="AF8" s="2" t="inlineStr"/>
+      <c r="AG8" s="2" t="n">
         <v>-7.07</v>
       </c>
-      <c r="AG8" s="2" t="n">
+      <c r="AH8" s="2" t="n">
         <v>1.36</v>
       </c>
-      <c r="AH8" s="2" t="n">
+      <c r="AI8" s="2" t="n">
         <v>-0.04</v>
       </c>
-      <c r="AI8" s="2" t="n">
+      <c r="AJ8" s="2" t="n">
         <v>0.24</v>
       </c>
-      <c r="AJ8" s="2" t="n">
+      <c r="AK8" s="2" t="n">
         <v>-4.2</v>
       </c>
-      <c r="AK8" s="2" t="n">
+      <c r="AL8" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL8" s="2" t="inlineStr"/>
-      <c r="AM8" s="2" t="n">
+      <c r="AM8" s="2" t="inlineStr"/>
+      <c r="AN8" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AN8" s="2" t="inlineStr"/>
       <c r="AO8" s="2" t="inlineStr"/>
-      <c r="AP8" s="2" t="inlineStr">
+      <c r="AP8" s="2" t="inlineStr"/>
+      <c r="AQ8" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AQ8" s="2" t="n">
+      <c r="AR8" s="2" t="n">
         <v>4.325</v>
       </c>
-      <c r="AR8" s="2" t="n">
+      <c r="AS8" s="2" t="n">
         <v>4.38</v>
       </c>
-      <c r="AS8" s="2" t="n">
+      <c r="AT8" s="2" t="n">
         <v>4.477</v>
       </c>
-      <c r="AT8" s="2" t="n">
+      <c r="AU8" s="2" t="n">
         <v>4.534</v>
       </c>
-      <c r="AU8" s="2" t="n">
+      <c r="AV8" s="2" t="n">
         <v>4.598</v>
       </c>
-      <c r="AV8" s="2" t="n">
+      <c r="AW8" s="2" t="n">
         <v>4.727</v>
       </c>
-      <c r="AW8" s="2" t="n">
+      <c r="AX8" s="2" t="n">
         <v>4.711</v>
       </c>
-      <c r="AX8" s="2" t="n">
+      <c r="AY8" s="2" t="n">
         <v>-1.4979</v>
       </c>
-      <c r="AY8" s="2" t="n">
+      <c r="AZ8" s="2" t="n">
         <v>-0.86</v>
       </c>
-      <c r="AZ8" s="2" t="n">
+      <c r="BA8" s="2" t="n">
         <v>-0.4262</v>
       </c>
-      <c r="BA8" s="2" t="n">
+      <c r="BB8" s="2" t="n">
         <v>-0.3204</v>
       </c>
-      <c r="BB8" s="2" t="n">
+      <c r="BC8" s="2" t="n">
         <v>-0.0707</v>
       </c>
     </row>
@@ -1856,81 +1873,82 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr">
         <is>
           <t>1→4·5d</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr"/>
       <c r="AA9" s="2" t="inlineStr"/>
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="inlineStr"/>
-      <c r="AF9" s="2" t="n">
-        <v>-0</v>
-      </c>
+      <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="2" t="n">
         <v>-2.67</v>
       </c>
-      <c r="AH9" s="2" t="n">
+      <c r="AI9" s="2" t="n">
         <v>-3.47</v>
       </c>
-      <c r="AI9" s="2" t="n">
+      <c r="AJ9" s="2" t="n">
         <v>-4.92</v>
       </c>
-      <c r="AJ9" s="2" t="n">
+      <c r="AK9" s="2" t="n">
         <v>3.5</v>
       </c>
-      <c r="AK9" s="2" t="n">
+      <c r="AL9" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL9" s="2" t="inlineStr"/>
-      <c r="AM9" s="2" t="n">
+      <c r="AM9" s="2" t="inlineStr"/>
+      <c r="AN9" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AN9" s="2" t="inlineStr"/>
       <c r="AO9" s="2" t="inlineStr"/>
-      <c r="AP9" s="2" t="inlineStr">
+      <c r="AP9" s="2" t="inlineStr"/>
+      <c r="AQ9" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AQ9" s="2" t="n">
+      <c r="AR9" s="2" t="n">
         <v>7.07</v>
       </c>
-      <c r="AR9" s="2" t="n">
+      <c r="AS9" s="2" t="n">
         <v>7.267</v>
       </c>
-      <c r="AS9" s="2" t="n">
+      <c r="AT9" s="2" t="n">
         <v>7.499</v>
       </c>
-      <c r="AT9" s="2" t="n">
+      <c r="AU9" s="2" t="n">
         <v>7.61</v>
       </c>
-      <c r="AU9" s="2" t="n">
+      <c r="AV9" s="2" t="n">
         <v>7.701</v>
       </c>
-      <c r="AV9" s="2" t="n">
+      <c r="AW9" s="2" t="n">
         <v>8.006</v>
       </c>
-      <c r="AW9" s="2" t="n">
+      <c r="AX9" s="2" t="n">
         <v>8.015000000000001</v>
       </c>
-      <c r="AX9" s="2" t="n">
+      <c r="AY9" s="2" t="n">
         <v>-2.5246</v>
       </c>
-      <c r="AY9" s="2" t="n">
+      <c r="AZ9" s="2" t="n">
         <v>-1.172</v>
       </c>
-      <c r="AZ9" s="2" t="n">
+      <c r="BA9" s="2" t="n">
         <v>-0.3577</v>
       </c>
-      <c r="BA9" s="2" t="n">
+      <c r="BB9" s="2" t="n">
         <v>-0.4898</v>
       </c>
-      <c r="BB9" s="2" t="n">
-        <v>-0</v>
+      <c r="BC9" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1996,88 +2014,89 @@
           <t>2A</t>
         </is>
       </c>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr">
         <is>
           <t>3→2A·11d ← 2B→3·13d</t>
         </is>
       </c>
-      <c r="Z10" s="2" t="inlineStr"/>
       <c r="AA10" s="2" t="inlineStr"/>
-      <c r="AB10" s="2" t="inlineStr">
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="inlineStr"/>
-      <c r="AF10" s="2" t="n">
+      <c r="AF10" s="2" t="inlineStr"/>
+      <c r="AG10" s="2" t="n">
         <v>16.97</v>
       </c>
-      <c r="AG10" s="2" t="n">
+      <c r="AH10" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="AH10" s="2" t="n">
+      <c r="AI10" s="2" t="n">
         <v>3.13</v>
       </c>
-      <c r="AI10" s="2" t="n">
+      <c r="AJ10" s="2" t="n">
         <v>6.36</v>
       </c>
-      <c r="AJ10" s="2" t="n">
+      <c r="AK10" s="2" t="n">
         <v>85.40000000000001</v>
       </c>
-      <c r="AK10" s="2" t="n">
+      <c r="AL10" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="AL10" s="2" t="inlineStr">
+      <c r="AM10" s="2" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="AM10" s="2" t="inlineStr"/>
-      <c r="AN10" s="2" t="n">
+      <c r="AN10" s="2" t="inlineStr"/>
+      <c r="AO10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AO10" s="2" t="inlineStr"/>
-      <c r="AP10" s="2" t="inlineStr">
+      <c r="AP10" s="2" t="inlineStr"/>
+      <c r="AQ10" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ10" s="2" t="n">
+      <c r="AR10" s="2" t="n">
         <v>3.451</v>
       </c>
-      <c r="AR10" s="2" t="n">
+      <c r="AS10" s="2" t="n">
         <v>3.406</v>
       </c>
-      <c r="AS10" s="2" t="n">
+      <c r="AT10" s="2" t="n">
         <v>3.396</v>
       </c>
-      <c r="AT10" s="2" t="n">
+      <c r="AU10" s="2" t="n">
         <v>3.415</v>
       </c>
-      <c r="AU10" s="2" t="n">
+      <c r="AV10" s="2" t="n">
         <v>3.379</v>
       </c>
-      <c r="AV10" s="2" t="n">
+      <c r="AW10" s="2" t="n">
         <v>3.271</v>
       </c>
-      <c r="AW10" s="2" t="n">
+      <c r="AX10" s="2" t="n">
         <v>3.228</v>
       </c>
-      <c r="AX10" s="2" t="n">
+      <c r="AY10" s="2" t="n">
         <v>0.7047</v>
       </c>
-      <c r="AY10" s="2" t="n">
+      <c r="AZ10" s="2" t="n">
         <v>0.0372</v>
       </c>
-      <c r="AZ10" s="2" t="n">
+      <c r="BA10" s="2" t="n">
         <v>0.3147</v>
       </c>
-      <c r="BA10" s="2" t="n">
+      <c r="BB10" s="2" t="n">
         <v>0.18</v>
       </c>
-      <c r="BB10" s="2" t="n">
+      <c r="BC10" s="2" t="n">
         <v>0.1697</v>
       </c>
     </row>
@@ -2141,91 +2160,96 @@
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>4+(周J超卖·日线纠缠)</t>
+          <t>4+</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
           <t>4→4+·4d ← 1→4·5d</t>
         </is>
       </c>
-      <c r="Z11" s="2" t="inlineStr"/>
       <c r="AA11" s="2" t="inlineStr"/>
       <c r="AB11" s="2" t="inlineStr"/>
-      <c r="AC11" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AC11" s="2" t="inlineStr"/>
       <c r="AD11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AE11" s="2" t="inlineStr"/>
-      <c r="AF11" s="2" t="n">
+      <c r="AE11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF11" s="2" t="inlineStr"/>
+      <c r="AG11" s="2" t="n">
         <v>-19.4</v>
       </c>
-      <c r="AG11" s="2" t="n">
+      <c r="AH11" s="2" t="n">
         <v>2.64</v>
       </c>
-      <c r="AH11" s="2" t="n">
+      <c r="AI11" s="2" t="n">
         <v>6.26</v>
       </c>
-      <c r="AI11" s="2" t="n">
+      <c r="AJ11" s="2" t="n">
         <v>6.57</v>
       </c>
-      <c r="AJ11" s="2" t="n">
+      <c r="AK11" s="2" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="AK11" s="2" t="n">
+      <c r="AL11" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="AL11" s="2" t="inlineStr">
+      <c r="AM11" s="2" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="AM11" s="2" t="n">
+      <c r="AN11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AN11" s="2" t="inlineStr"/>
       <c r="AO11" s="2" t="inlineStr"/>
-      <c r="AP11" s="2" t="inlineStr">
+      <c r="AP11" s="2" t="inlineStr"/>
+      <c r="AQ11" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ11" s="2" t="n">
+      <c r="AR11" s="2" t="n">
         <v>0.495</v>
       </c>
-      <c r="AR11" s="2" t="n">
+      <c r="AS11" s="2" t="n">
         <v>0.493</v>
       </c>
-      <c r="AS11" s="2" t="n">
+      <c r="AT11" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="AT11" s="2" t="n">
+      <c r="AU11" s="2" t="n">
         <v>0.509</v>
       </c>
-      <c r="AU11" s="2" t="n">
+      <c r="AV11" s="2" t="n">
         <v>0.513</v>
       </c>
-      <c r="AV11" s="2" t="n">
+      <c r="AW11" s="2" t="n">
         <v>0.516</v>
       </c>
-      <c r="AW11" s="2" t="n">
+      <c r="AX11" s="2" t="n">
         <v>0.53</v>
       </c>
-      <c r="AX11" s="2" t="n">
+      <c r="AY11" s="2" t="n">
         <v>-0.6145</v>
       </c>
-      <c r="AY11" s="2" t="n">
+      <c r="AZ11" s="2" t="n">
         <v>-0.7127</v>
       </c>
-      <c r="AZ11" s="2" t="n">
+      <c r="BA11" s="2" t="n">
         <v>-0.3321</v>
       </c>
-      <c r="BA11" s="2" t="n">
+      <c r="BB11" s="2" t="n">
         <v>-0.0654</v>
       </c>
-      <c r="BB11" s="2" t="n">
+      <c r="BC11" s="2" t="n">
         <v>-0.194</v>
       </c>
     </row>
@@ -2290,82 +2314,83 @@
           <t>1</t>
         </is>
       </c>
-      <c r="Y12" s="2" t="inlineStr">
+      <c r="Y12" s="2" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr">
         <is>
           <t>1+→1·6d ← 1→1+·7d ← 1+→1·11d</t>
         </is>
       </c>
-      <c r="Z12" s="2" t="inlineStr"/>
       <c r="AA12" s="2" t="inlineStr"/>
       <c r="AB12" s="2" t="inlineStr"/>
-      <c r="AC12" s="2" t="n">
+      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD12" s="2" t="n">
+      <c r="AE12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AE12" s="2" t="inlineStr"/>
-      <c r="AF12" s="2" t="n">
+      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AG12" s="2" t="n">
         <v>-4.86</v>
       </c>
-      <c r="AG12" s="2" t="n">
+      <c r="AH12" s="2" t="n">
         <v>11.28</v>
       </c>
-      <c r="AH12" s="2" t="n">
+      <c r="AI12" s="2" t="n">
         <v>2.49</v>
       </c>
-      <c r="AI12" s="2" t="n">
+      <c r="AJ12" s="2" t="n">
         <v>11.94</v>
       </c>
-      <c r="AJ12" s="2" t="n">
+      <c r="AK12" s="2" t="n">
         <v>61.1</v>
       </c>
-      <c r="AK12" s="2" t="n">
+      <c r="AL12" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="AL12" s="2" t="inlineStr"/>
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr"/>
       <c r="AO12" s="2" t="inlineStr"/>
-      <c r="AP12" s="2" t="inlineStr">
+      <c r="AP12" s="2" t="inlineStr"/>
+      <c r="AQ12" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ12" s="2" t="n">
+      <c r="AR12" s="2" t="n">
         <v>0.377</v>
       </c>
-      <c r="AR12" s="2" t="n">
+      <c r="AS12" s="2" t="n">
         <v>0.378</v>
       </c>
-      <c r="AS12" s="2" t="n">
+      <c r="AT12" s="2" t="n">
         <v>0.376</v>
       </c>
-      <c r="AT12" s="2" t="n">
+      <c r="AU12" s="2" t="n">
         <v>0.377</v>
       </c>
-      <c r="AU12" s="2" t="n">
+      <c r="AV12" s="2" t="n">
         <v>0.383</v>
       </c>
-      <c r="AV12" s="2" t="n">
+      <c r="AW12" s="2" t="n">
         <v>0.365</v>
       </c>
-      <c r="AW12" s="2" t="n">
+      <c r="AX12" s="2" t="n">
         <v>0.371</v>
       </c>
-      <c r="AX12" s="2" t="n">
+      <c r="AY12" s="2" t="n">
         <v>-0.1859</v>
       </c>
-      <c r="AY12" s="2" t="n">
+      <c r="AZ12" s="2" t="n">
         <v>-0.0283</v>
       </c>
-      <c r="AZ12" s="2" t="n">
+      <c r="BA12" s="2" t="n">
         <v>0.1005</v>
       </c>
-      <c r="BA12" s="2" t="n">
+      <c r="BB12" s="2" t="n">
         <v>0.1451</v>
       </c>
-      <c r="BB12" s="2" t="n">
+      <c r="BC12" s="2" t="n">
         <v>-0.0486</v>
       </c>
     </row>
@@ -2427,83 +2452,88 @@
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>4+(周J超卖·日线纠缠)</t>
+          <t>4+</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
           <t>4→4+·4d ← 4+→4·6d ← 1→4+·9d</t>
         </is>
       </c>
-      <c r="Z13" s="2" t="inlineStr"/>
       <c r="AA13" s="2" t="inlineStr"/>
-      <c r="AB13" s="2" t="n">
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
       <c r="AE13" s="2" t="inlineStr"/>
-      <c r="AF13" s="2" t="n">
+      <c r="AF13" s="2" t="inlineStr"/>
+      <c r="AG13" s="2" t="n">
         <v>-20.65</v>
       </c>
-      <c r="AG13" s="2" t="n">
+      <c r="AH13" s="2" t="n">
         <v>1.57</v>
       </c>
-      <c r="AH13" s="2" t="n">
+      <c r="AI13" s="2" t="n">
         <v>4.3</v>
       </c>
-      <c r="AI13" s="2" t="n">
+      <c r="AJ13" s="2" t="n">
         <v>4.63</v>
       </c>
-      <c r="AJ13" s="2" t="n">
+      <c r="AK13" s="2" t="n">
         <v>15.8</v>
       </c>
-      <c r="AK13" s="2" t="n">
+      <c r="AL13" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="AL13" s="2" t="inlineStr"/>
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr"/>
       <c r="AO13" s="2" t="inlineStr"/>
-      <c r="AP13" s="2" t="inlineStr">
+      <c r="AP13" s="2" t="inlineStr"/>
+      <c r="AQ13" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
-      </c>
-      <c r="AQ13" s="2" t="n">
-        <v>0.76</v>
       </c>
       <c r="AR13" s="2" t="n">
         <v>0.76</v>
       </c>
       <c r="AS13" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="AT13" s="2" t="n">
         <v>0.773</v>
       </c>
-      <c r="AT13" s="2" t="n">
+      <c r="AU13" s="2" t="n">
         <v>0.785</v>
       </c>
-      <c r="AU13" s="2" t="n">
+      <c r="AV13" s="2" t="n">
         <v>0.789</v>
       </c>
-      <c r="AV13" s="2" t="n">
+      <c r="AW13" s="2" t="n">
         <v>0.786</v>
       </c>
-      <c r="AW13" s="2" t="n">
+      <c r="AX13" s="2" t="n">
         <v>0.824</v>
       </c>
-      <c r="AX13" s="2" t="n">
+      <c r="AY13" s="2" t="n">
         <v>-0.8008999999999999</v>
       </c>
-      <c r="AY13" s="2" t="n">
+      <c r="AZ13" s="2" t="n">
         <v>-0.8296</v>
       </c>
-      <c r="AZ13" s="2" t="n">
+      <c r="BA13" s="2" t="n">
         <v>-0.3245</v>
       </c>
-      <c r="BA13" s="2" t="n">
+      <c r="BB13" s="2" t="n">
         <v>-0.0723</v>
       </c>
-      <c r="BB13" s="2" t="n">
+      <c r="BC13" s="2" t="n">
         <v>-0.2065</v>
       </c>
     </row>
@@ -2570,78 +2600,79 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y14" s="2" t="inlineStr">
+      <c r="Y14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr">
         <is>
           <t>1→4·15d</t>
         </is>
       </c>
-      <c r="Z14" s="2" t="inlineStr"/>
       <c r="AA14" s="2" t="inlineStr"/>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="inlineStr"/>
-      <c r="AF14" s="2" t="n">
+      <c r="AF14" s="2" t="inlineStr"/>
+      <c r="AG14" s="2" t="n">
         <v>-5.08</v>
       </c>
-      <c r="AG14" s="2" t="n">
+      <c r="AH14" s="2" t="n">
         <v>-4.11</v>
       </c>
-      <c r="AH14" s="2" t="n">
+      <c r="AI14" s="2" t="n">
         <v>-3.61</v>
       </c>
-      <c r="AI14" s="2" t="n">
+      <c r="AJ14" s="2" t="n">
         <v>-4.49</v>
       </c>
-      <c r="AJ14" s="2" t="n">
+      <c r="AK14" s="2" t="n">
         <v>17.8</v>
       </c>
-      <c r="AK14" s="2" t="n">
+      <c r="AL14" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL14" s="2" t="inlineStr"/>
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr"/>
       <c r="AO14" s="2" t="inlineStr"/>
-      <c r="AP14" s="2" t="inlineStr">
+      <c r="AP14" s="2" t="inlineStr"/>
+      <c r="AQ14" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ14" s="2" t="n">
+      <c r="AR14" s="2" t="n">
         <v>2.826</v>
       </c>
-      <c r="AR14" s="2" t="n">
+      <c r="AS14" s="2" t="n">
         <v>2.903</v>
       </c>
-      <c r="AS14" s="2" t="n">
+      <c r="AT14" s="2" t="n">
         <v>2.995</v>
       </c>
-      <c r="AT14" s="2" t="n">
+      <c r="AU14" s="2" t="n">
         <v>3.031</v>
       </c>
-      <c r="AU14" s="2" t="n">
+      <c r="AV14" s="2" t="n">
         <v>3.041</v>
       </c>
-      <c r="AV14" s="2" t="n">
+      <c r="AW14" s="2" t="n">
         <v>3.178</v>
       </c>
-      <c r="AW14" s="2" t="n">
+      <c r="AX14" s="2" t="n">
         <v>3.212</v>
       </c>
-      <c r="AX14" s="2" t="n">
+      <c r="AY14" s="2" t="n">
         <v>-2.5593</v>
       </c>
-      <c r="AY14" s="2" t="n">
+      <c r="AZ14" s="2" t="n">
         <v>-1.1037</v>
       </c>
-      <c r="AZ14" s="2" t="n">
+      <c r="BA14" s="2" t="n">
         <v>-0.0916</v>
       </c>
-      <c r="BA14" s="2" t="n">
+      <c r="BB14" s="2" t="n">
         <v>-0.5706</v>
       </c>
-      <c r="BB14" s="2" t="n">
+      <c r="BC14" s="2" t="n">
         <v>-0.0508</v>
       </c>
     </row>
@@ -2708,80 +2739,81 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y15" s="2" t="inlineStr">
+      <c r="Y15" s="2" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr">
         <is>
           <t>4+→4·6d ← 4→4+·11d ← 4+→4·14d</t>
         </is>
       </c>
-      <c r="Z15" s="2" t="inlineStr"/>
       <c r="AA15" s="2" t="inlineStr"/>
-      <c r="AB15" s="2" t="n">
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="inlineStr"/>
       <c r="AE15" s="2" t="inlineStr"/>
-      <c r="AF15" s="2" t="n">
+      <c r="AF15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="n">
         <v>-15.62</v>
       </c>
-      <c r="AG15" s="2" t="n">
+      <c r="AH15" s="2" t="n">
         <v>-9.56</v>
       </c>
-      <c r="AH15" s="2" t="n">
+      <c r="AI15" s="2" t="n">
         <v>-2.31</v>
       </c>
-      <c r="AI15" s="2" t="n">
+      <c r="AJ15" s="2" t="n">
         <v>-3.42</v>
       </c>
-      <c r="AJ15" s="2" t="n">
+      <c r="AK15" s="2" t="n">
         <v>23.4</v>
       </c>
-      <c r="AK15" s="2" t="n">
+      <c r="AL15" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="AL15" s="2" t="inlineStr"/>
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr"/>
       <c r="AO15" s="2" t="inlineStr"/>
-      <c r="AP15" s="2" t="inlineStr">
+      <c r="AP15" s="2" t="inlineStr"/>
+      <c r="AQ15" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ15" s="2" t="n">
+      <c r="AR15" s="2" t="n">
         <v>1.065</v>
       </c>
-      <c r="AR15" s="2" t="n">
+      <c r="AS15" s="2" t="n">
         <v>1.085</v>
       </c>
-      <c r="AS15" s="2" t="n">
+      <c r="AT15" s="2" t="n">
         <v>1.122</v>
       </c>
-      <c r="AT15" s="2" t="n">
+      <c r="AU15" s="2" t="n">
         <v>1.129</v>
       </c>
-      <c r="AU15" s="2" t="n">
+      <c r="AV15" s="2" t="n">
         <v>1.128</v>
       </c>
-      <c r="AV15" s="2" t="n">
+      <c r="AW15" s="2" t="n">
         <v>1.181</v>
       </c>
-      <c r="AW15" s="2" t="n">
+      <c r="AX15" s="2" t="n">
         <v>1.298</v>
       </c>
-      <c r="AX15" s="2" t="n">
+      <c r="AY15" s="2" t="n">
         <v>-2.1542</v>
       </c>
-      <c r="AY15" s="2" t="n">
+      <c r="AZ15" s="2" t="n">
         <v>-1.0315</v>
       </c>
-      <c r="AZ15" s="2" t="n">
+      <c r="BA15" s="2" t="n">
         <v>-0.1159</v>
       </c>
-      <c r="BA15" s="2" t="n">
+      <c r="BB15" s="2" t="n">
         <v>-0.7454</v>
       </c>
-      <c r="BB15" s="2" t="n">
+      <c r="BC15" s="2" t="n">
         <v>-0.1562</v>
       </c>
     </row>
@@ -2848,80 +2880,81 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y16" s="2" t="inlineStr">
+      <c r="Y16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr">
         <is>
           <t>4+→4·6d ← 4→4+·14d ← 4+→4·17d</t>
         </is>
       </c>
-      <c r="Z16" s="2" t="inlineStr"/>
       <c r="AA16" s="2" t="inlineStr"/>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
-      <c r="AF16" s="2" t="n">
+      <c r="AF16" s="2" t="inlineStr"/>
+      <c r="AG16" s="2" t="n">
         <v>-14.72</v>
       </c>
-      <c r="AG16" s="2" t="n">
+      <c r="AH16" s="2" t="n">
         <v>-8.49</v>
       </c>
-      <c r="AH16" s="2" t="n">
+      <c r="AI16" s="2" t="n">
         <v>-1.14</v>
       </c>
-      <c r="AI16" s="2" t="n">
+      <c r="AJ16" s="2" t="n">
         <v>-1.71</v>
       </c>
-      <c r="AJ16" s="2" t="n">
+      <c r="AK16" s="2" t="n">
         <v>0.3</v>
       </c>
-      <c r="AK16" s="2" t="n">
+      <c r="AL16" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AL16" s="2" t="inlineStr"/>
-      <c r="AM16" s="2" t="n">
+      <c r="AM16" s="2" t="inlineStr"/>
+      <c r="AN16" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="AN16" s="2" t="inlineStr"/>
       <c r="AO16" s="2" t="inlineStr"/>
-      <c r="AP16" s="2" t="inlineStr">
+      <c r="AP16" s="2" t="inlineStr"/>
+      <c r="AQ16" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AQ16" s="2" t="n">
+      <c r="AR16" s="2" t="n">
         <v>1.042</v>
       </c>
-      <c r="AR16" s="2" t="n">
+      <c r="AS16" s="2" t="n">
         <v>1.065</v>
       </c>
-      <c r="AS16" s="2" t="n">
+      <c r="AT16" s="2" t="n">
         <v>1.095</v>
       </c>
-      <c r="AT16" s="2" t="n">
+      <c r="AU16" s="2" t="n">
         <v>1.12</v>
       </c>
-      <c r="AU16" s="2" t="n">
+      <c r="AV16" s="2" t="n">
         <v>1.149</v>
       </c>
-      <c r="AV16" s="2" t="n">
+      <c r="AW16" s="2" t="n">
         <v>1.187</v>
       </c>
-      <c r="AW16" s="2" t="n">
+      <c r="AX16" s="2" t="n">
         <v>1.228</v>
       </c>
-      <c r="AX16" s="2" t="n">
+      <c r="AY16" s="2" t="n">
         <v>-2.2184</v>
       </c>
-      <c r="AY16" s="2" t="n">
+      <c r="AZ16" s="2" t="n">
         <v>-1.3227</v>
       </c>
-      <c r="AZ16" s="2" t="n">
+      <c r="BA16" s="2" t="n">
         <v>-0.6039</v>
       </c>
-      <c r="BA16" s="2" t="n">
+      <c r="BB16" s="2" t="n">
         <v>-0.6807</v>
       </c>
-      <c r="BB16" s="2" t="n">
+      <c r="BC16" s="2" t="n">
         <v>-0.1472</v>
       </c>
     </row>
@@ -2988,80 +3021,81 @@
           <t>1</t>
         </is>
       </c>
-      <c r="Y17" s="2" t="inlineStr">
+      <c r="Y17" s="2" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr">
         <is>
           <t>2A→1·20d</t>
         </is>
       </c>
-      <c r="Z17" s="2" t="inlineStr"/>
       <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
       <c r="AD17" s="2" t="inlineStr"/>
       <c r="AE17" s="2" t="inlineStr"/>
-      <c r="AF17" s="2" t="n">
+      <c r="AF17" s="2" t="inlineStr"/>
+      <c r="AG17" s="2" t="n">
         <v>17.95</v>
       </c>
-      <c r="AG17" s="2" t="n">
+      <c r="AH17" s="2" t="n">
         <v>2.66</v>
       </c>
-      <c r="AH17" s="2" t="n">
+      <c r="AI17" s="2" t="n">
         <v>-4.84</v>
       </c>
-      <c r="AI17" s="2" t="n">
+      <c r="AJ17" s="2" t="n">
         <v>-8.390000000000001</v>
       </c>
-      <c r="AJ17" s="2" t="n">
+      <c r="AK17" s="2" t="n">
         <v>-6.8</v>
       </c>
-      <c r="AK17" s="2" t="n">
+      <c r="AL17" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL17" s="2" t="inlineStr"/>
-      <c r="AM17" s="2" t="n">
+      <c r="AM17" s="2" t="inlineStr"/>
+      <c r="AN17" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="AN17" s="2" t="inlineStr"/>
       <c r="AO17" s="2" t="inlineStr"/>
-      <c r="AP17" s="2" t="inlineStr">
+      <c r="AP17" s="2" t="inlineStr"/>
+      <c r="AQ17" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ17" s="2" t="n">
+      <c r="AR17" s="2" t="n">
         <v>0.9350000000000001</v>
       </c>
-      <c r="AR17" s="2" t="n">
+      <c r="AS17" s="2" t="n">
         <v>0.982</v>
       </c>
-      <c r="AS17" s="2" t="n">
+      <c r="AT17" s="2" t="n">
         <v>1.023</v>
       </c>
-      <c r="AT17" s="2" t="n">
+      <c r="AU17" s="2" t="n">
         <v>1.041</v>
       </c>
-      <c r="AU17" s="2" t="n">
+      <c r="AV17" s="2" t="n">
         <v>1.069</v>
       </c>
-      <c r="AV17" s="2" t="n">
+      <c r="AW17" s="2" t="n">
         <v>1.17</v>
       </c>
-      <c r="AW17" s="2" t="n">
+      <c r="AX17" s="2" t="n">
         <v>1.029</v>
       </c>
-      <c r="AX17" s="2" t="n">
+      <c r="AY17" s="2" t="n">
         <v>-3.9433</v>
       </c>
-      <c r="AY17" s="2" t="n">
+      <c r="AZ17" s="2" t="n">
         <v>-1.4312</v>
       </c>
-      <c r="AZ17" s="2" t="n">
+      <c r="BA17" s="2" t="n">
         <v>-1.1299</v>
       </c>
-      <c r="BA17" s="2" t="n">
+      <c r="BB17" s="2" t="n">
         <v>-0.3963</v>
       </c>
-      <c r="BB17" s="2" t="n">
+      <c r="BC17" s="2" t="n">
         <v>0.1795</v>
       </c>
     </row>
@@ -3126,88 +3160,89 @@
           <t>2A</t>
         </is>
       </c>
-      <c r="Y18" s="2" t="inlineStr">
+      <c r="Y18" s="2" t="inlineStr"/>
+      <c r="Z18" s="2" t="inlineStr">
         <is>
           <t>2B→2A·6d</t>
         </is>
       </c>
-      <c r="Z18" s="2" t="inlineStr"/>
       <c r="AA18" s="2" t="inlineStr"/>
-      <c r="AB18" s="2" t="inlineStr">
+      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
-      <c r="AF18" s="2" t="n">
+      <c r="AF18" s="2" t="inlineStr"/>
+      <c r="AG18" s="2" t="n">
         <v>7.01</v>
       </c>
-      <c r="AG18" s="2" t="n">
+      <c r="AH18" s="2" t="n">
         <v>19.92</v>
       </c>
-      <c r="AH18" s="2" t="n">
+      <c r="AI18" s="2" t="n">
         <v>4.19</v>
       </c>
-      <c r="AI18" s="2" t="n">
+      <c r="AJ18" s="2" t="n">
         <v>12.85</v>
       </c>
-      <c r="AJ18" s="2" t="n">
+      <c r="AK18" s="2" t="n">
         <v>99.3</v>
       </c>
-      <c r="AK18" s="2" t="n">
+      <c r="AL18" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="AL18" s="2" t="inlineStr">
+      <c r="AM18" s="2" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="AM18" s="2" t="inlineStr"/>
-      <c r="AN18" s="2" t="n">
+      <c r="AN18" s="2" t="inlineStr"/>
+      <c r="AO18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AO18" s="2" t="inlineStr"/>
-      <c r="AP18" s="2" t="inlineStr">
+      <c r="AP18" s="2" t="inlineStr"/>
+      <c r="AQ18" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ18" s="2" t="n">
+      <c r="AR18" s="2" t="n">
         <v>0.862</v>
       </c>
-      <c r="AR18" s="2" t="n">
+      <c r="AS18" s="2" t="n">
         <v>0.854</v>
       </c>
-      <c r="AS18" s="2" t="n">
+      <c r="AT18" s="2" t="n">
         <v>0.848</v>
       </c>
-      <c r="AT18" s="2" t="n">
+      <c r="AU18" s="2" t="n">
         <v>0.844</v>
       </c>
-      <c r="AU18" s="2" t="n">
+      <c r="AV18" s="2" t="n">
         <v>0.831</v>
       </c>
-      <c r="AV18" s="2" t="n">
+      <c r="AW18" s="2" t="n">
         <v>0.805</v>
       </c>
-      <c r="AW18" s="2" t="n">
+      <c r="AX18" s="2" t="n">
         <v>0.799</v>
       </c>
-      <c r="AX18" s="2" t="n">
+      <c r="AY18" s="2" t="n">
         <v>0.7857</v>
       </c>
-      <c r="AY18" s="2" t="n">
+      <c r="AZ18" s="2" t="n">
         <v>0.3273</v>
       </c>
-      <c r="AZ18" s="2" t="n">
+      <c r="BA18" s="2" t="n">
         <v>0.3288</v>
       </c>
-      <c r="BA18" s="2" t="n">
+      <c r="BB18" s="2" t="n">
         <v>0.2736</v>
       </c>
-      <c r="BB18" s="2" t="n">
+      <c r="BC18" s="2" t="n">
         <v>0.0701</v>
       </c>
     </row>
@@ -3271,87 +3306,92 @@
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>4+(周J超卖·日线纠缠)</t>
+          <t>4+</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
           <t>4→4+·13d</t>
         </is>
       </c>
-      <c r="Z19" s="2" t="inlineStr"/>
       <c r="AA19" s="2" t="inlineStr"/>
-      <c r="AB19" s="2" t="inlineStr">
+      <c r="AB19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AC19" s="2" t="inlineStr"/>
-      <c r="AD19" s="2" t="n">
+      <c r="AD19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AE19" s="2" t="inlineStr"/>
-      <c r="AF19" s="2" t="n">
+      <c r="AF19" s="2" t="inlineStr"/>
+      <c r="AG19" s="2" t="n">
         <v>-54.96</v>
       </c>
-      <c r="AG19" s="2" t="n">
+      <c r="AH19" s="2" t="n">
         <v>-13.34</v>
       </c>
-      <c r="AH19" s="2" t="n">
+      <c r="AI19" s="2" t="n">
         <v>5.36</v>
       </c>
-      <c r="AI19" s="2" t="n">
+      <c r="AJ19" s="2" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="AJ19" s="2" t="n">
+      <c r="AK19" s="2" t="n">
         <v>24.8</v>
       </c>
-      <c r="AK19" s="2" t="n">
+      <c r="AL19" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="AL19" s="2" t="inlineStr"/>
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr"/>
       <c r="AO19" s="2" t="inlineStr"/>
-      <c r="AP19" s="2" t="inlineStr">
+      <c r="AP19" s="2" t="inlineStr"/>
+      <c r="AQ19" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
-      </c>
-      <c r="AQ19" s="2" t="n">
-        <v>1.008</v>
       </c>
       <c r="AR19" s="2" t="n">
         <v>1.008</v>
       </c>
       <c r="AS19" s="2" t="n">
+        <v>1.008</v>
+      </c>
+      <c r="AT19" s="2" t="n">
         <v>1.014</v>
       </c>
-      <c r="AT19" s="2" t="n">
+      <c r="AU19" s="2" t="n">
         <v>1.028</v>
       </c>
-      <c r="AU19" s="2" t="n">
+      <c r="AV19" s="2" t="n">
         <v>1.07</v>
       </c>
-      <c r="AV19" s="2" t="n">
+      <c r="AW19" s="2" t="n">
         <v>1.076</v>
       </c>
-      <c r="AW19" s="2" t="n">
+      <c r="AX19" s="2" t="n">
         <v>1.209</v>
       </c>
-      <c r="AX19" s="2" t="n">
+      <c r="AY19" s="2" t="n">
         <v>-0.4502</v>
       </c>
-      <c r="AY19" s="2" t="n">
+      <c r="AZ19" s="2" t="n">
         <v>-0.4374</v>
       </c>
-      <c r="AZ19" s="2" t="n">
+      <c r="BA19" s="2" t="n">
         <v>-0.4243</v>
       </c>
-      <c r="BA19" s="2" t="n">
+      <c r="BB19" s="2" t="n">
         <v>-0.457</v>
       </c>
-      <c r="BB19" s="2" t="n">
+      <c r="BC19" s="2" t="n">
         <v>-0.5496</v>
       </c>
     </row>
@@ -3413,83 +3453,88 @@
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>4+(周J超卖·日线纠缠)</t>
+          <t>4+</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
         <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
           <t>4→4+·4d ← 4+→4·6d ← 1→4+·9d</t>
         </is>
       </c>
-      <c r="Z20" s="2" t="inlineStr"/>
       <c r="AA20" s="2" t="inlineStr"/>
-      <c r="AB20" s="2" t="n">
+      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AC20" s="2" t="inlineStr"/>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
-      <c r="AF20" s="2" t="n">
+      <c r="AF20" s="2" t="inlineStr"/>
+      <c r="AG20" s="2" t="n">
         <v>-22.42</v>
       </c>
-      <c r="AG20" s="2" t="n">
+      <c r="AH20" s="2" t="n">
         <v>-1.16</v>
       </c>
-      <c r="AH20" s="2" t="n">
+      <c r="AI20" s="2" t="n">
         <v>3.21</v>
       </c>
-      <c r="AI20" s="2" t="n">
+      <c r="AJ20" s="2" t="n">
         <v>3.63</v>
       </c>
-      <c r="AJ20" s="2" t="n">
+      <c r="AK20" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AK20" s="2" t="n">
+      <c r="AL20" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="AL20" s="2" t="inlineStr"/>
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr"/>
       <c r="AO20" s="2" t="inlineStr"/>
-      <c r="AP20" s="2" t="inlineStr">
+      <c r="AP20" s="2" t="inlineStr"/>
+      <c r="AQ20" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ20" s="2" t="n">
+      <c r="AR20" s="2" t="n">
         <v>1.729</v>
       </c>
-      <c r="AR20" s="2" t="n">
+      <c r="AS20" s="2" t="n">
         <v>1.741</v>
       </c>
-      <c r="AS20" s="2" t="n">
+      <c r="AT20" s="2" t="n">
         <v>1.774</v>
       </c>
-      <c r="AT20" s="2" t="n">
+      <c r="AU20" s="2" t="n">
         <v>1.81</v>
       </c>
-      <c r="AU20" s="2" t="n">
+      <c r="AV20" s="2" t="n">
         <v>1.819</v>
       </c>
-      <c r="AV20" s="2" t="n">
+      <c r="AW20" s="2" t="n">
         <v>1.812</v>
       </c>
-      <c r="AW20" s="2" t="n">
+      <c r="AX20" s="2" t="n">
         <v>1.876</v>
       </c>
-      <c r="AX20" s="2" t="n">
+      <c r="AY20" s="2" t="n">
         <v>-1.0503</v>
       </c>
-      <c r="AY20" s="2" t="n">
+      <c r="AZ20" s="2" t="n">
         <v>-1.0089</v>
       </c>
-      <c r="AZ20" s="2" t="n">
+      <c r="BA20" s="2" t="n">
         <v>-0.364</v>
       </c>
-      <c r="BA20" s="2" t="n">
+      <c r="BB20" s="2" t="n">
         <v>-0.1214</v>
       </c>
-      <c r="BB20" s="2" t="n">
+      <c r="BC20" s="2" t="n">
         <v>-0.2242</v>
       </c>
     </row>
@@ -3558,88 +3603,89 @@
           <t>2B</t>
         </is>
       </c>
-      <c r="Y21" s="2" t="inlineStr">
+      <c r="Y21" s="2" t="inlineStr"/>
+      <c r="Z21" s="2" t="inlineStr">
         <is>
           <t>2C→2B·5d ← 2B→2C·18d</t>
         </is>
       </c>
-      <c r="Z21" s="2" t="inlineStr"/>
       <c r="AA21" s="2" t="inlineStr"/>
       <c r="AB21" s="2" t="inlineStr"/>
-      <c r="AC21" s="2" t="inlineStr">
+      <c r="AC21" s="2" t="inlineStr"/>
+      <c r="AD21" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="inlineStr"/>
-      <c r="AF21" s="2" t="n">
+      <c r="AF21" s="2" t="inlineStr"/>
+      <c r="AG21" s="2" t="n">
         <v>28.55</v>
       </c>
-      <c r="AG21" s="2" t="n">
+      <c r="AH21" s="2" t="n">
         <v>29.03</v>
       </c>
-      <c r="AH21" s="2" t="n">
+      <c r="AI21" s="2" t="n">
         <v>0.46</v>
       </c>
-      <c r="AI21" s="2" t="n">
+      <c r="AJ21" s="2" t="n">
         <v>12.87</v>
       </c>
-      <c r="AJ21" s="2" t="n">
+      <c r="AK21" s="2" t="n">
         <v>85.09999999999999</v>
       </c>
-      <c r="AK21" s="2" t="n">
+      <c r="AL21" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="AL21" s="2" t="inlineStr">
+      <c r="AM21" s="2" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="AM21" s="2" t="inlineStr"/>
-      <c r="AN21" s="2" t="n">
+      <c r="AN21" s="2" t="inlineStr"/>
+      <c r="AO21" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AO21" s="2" t="inlineStr"/>
-      <c r="AP21" s="2" t="inlineStr">
+      <c r="AP21" s="2" t="inlineStr"/>
+      <c r="AQ21" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ21" s="2" t="n">
+      <c r="AR21" s="2" t="n">
         <v>2.379</v>
       </c>
-      <c r="AR21" s="2" t="n">
+      <c r="AS21" s="2" t="n">
         <v>2.356</v>
       </c>
-      <c r="AS21" s="2" t="n">
+      <c r="AT21" s="2" t="n">
         <v>2.3</v>
       </c>
-      <c r="AT21" s="2" t="n">
+      <c r="AU21" s="2" t="n">
         <v>2.275</v>
       </c>
-      <c r="AU21" s="2" t="n">
+      <c r="AV21" s="2" t="n">
         <v>2.247</v>
       </c>
-      <c r="AV21" s="2" t="n">
+      <c r="AW21" s="2" t="n">
         <v>2.215</v>
       </c>
-      <c r="AW21" s="2" t="n">
+      <c r="AX21" s="2" t="n">
         <v>2.042</v>
       </c>
-      <c r="AX21" s="2" t="n">
+      <c r="AY21" s="2" t="n">
         <v>1.0622</v>
       </c>
-      <c r="AY21" s="2" t="n">
+      <c r="AZ21" s="2" t="n">
         <v>0.8881</v>
       </c>
-      <c r="AZ21" s="2" t="n">
+      <c r="BA21" s="2" t="n">
         <v>0.6552</v>
       </c>
-      <c r="BA21" s="2" t="n">
+      <c r="BB21" s="2" t="n">
         <v>0.3504</v>
       </c>
-      <c r="BB21" s="2" t="n">
+      <c r="BC21" s="2" t="n">
         <v>0.2855</v>
       </c>
     </row>
@@ -3712,82 +3758,83 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y22" s="2" t="inlineStr">
+      <c r="Y22" s="2" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr">
         <is>
           <t>4+→4·2d ← 4→4+·4d ← 4+→4·7d</t>
         </is>
       </c>
-      <c r="Z22" s="2" t="inlineStr"/>
       <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="n">
+      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AD22" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="inlineStr"/>
-      <c r="AF22" s="2" t="n">
+      <c r="AF22" s="2" t="inlineStr"/>
+      <c r="AG22" s="2" t="n">
         <v>-27.96</v>
       </c>
-      <c r="AG22" s="2" t="n">
+      <c r="AH22" s="2" t="n">
         <v>-16.28</v>
       </c>
-      <c r="AH22" s="2" t="n">
+      <c r="AI22" s="2" t="n">
         <v>-2.98</v>
       </c>
-      <c r="AI22" s="2" t="n">
+      <c r="AJ22" s="2" t="n">
         <v>-3.07</v>
       </c>
-      <c r="AJ22" s="2" t="n">
+      <c r="AK22" s="2" t="n">
         <v>-0.1</v>
       </c>
-      <c r="AK22" s="2" t="n">
+      <c r="AL22" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL22" s="2" t="inlineStr"/>
-      <c r="AM22" s="2" t="n">
+      <c r="AM22" s="2" t="inlineStr"/>
+      <c r="AN22" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AN22" s="2" t="inlineStr"/>
       <c r="AO22" s="2" t="inlineStr"/>
-      <c r="AP22" s="2" t="inlineStr">
+      <c r="AP22" s="2" t="inlineStr"/>
+      <c r="AQ22" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AQ22" s="2" t="n">
+      <c r="AR22" s="2" t="n">
         <v>1.408</v>
       </c>
-      <c r="AR22" s="2" t="n">
+      <c r="AS22" s="2" t="n">
         <v>1.429</v>
       </c>
-      <c r="AS22" s="2" t="n">
+      <c r="AT22" s="2" t="n">
         <v>1.464</v>
       </c>
-      <c r="AT22" s="2" t="n">
+      <c r="AU22" s="2" t="n">
         <v>1.503</v>
       </c>
-      <c r="AU22" s="2" t="n">
+      <c r="AV22" s="2" t="n">
         <v>1.56</v>
       </c>
-      <c r="AV22" s="2" t="n">
+      <c r="AW22" s="2" t="n">
         <v>1.687</v>
       </c>
-      <c r="AW22" s="2" t="n">
+      <c r="AX22" s="2" t="n">
         <v>1.8</v>
       </c>
-      <c r="AX22" s="2" t="n">
+      <c r="AY22" s="2" t="n">
         <v>-1.6486</v>
       </c>
-      <c r="AY22" s="2" t="n">
+      <c r="AZ22" s="2" t="n">
         <v>-1.2648</v>
       </c>
-      <c r="AZ22" s="2" t="n">
+      <c r="BA22" s="2" t="n">
         <v>-0.6054</v>
       </c>
-      <c r="BA22" s="2" t="n">
+      <c r="BB22" s="2" t="n">
         <v>-0.966</v>
       </c>
-      <c r="BB22" s="2" t="n">
+      <c r="BC22" s="2" t="n">
         <v>-0.2796</v>
       </c>
     </row>
@@ -3854,80 +3901,81 @@
           <t>1</t>
         </is>
       </c>
-      <c r="Y23" s="2" t="inlineStr">
+      <c r="Y23" s="2" t="inlineStr"/>
+      <c r="Z23" s="2" t="inlineStr">
         <is>
           <t>2A→1·6d</t>
         </is>
       </c>
-      <c r="Z23" s="2" t="inlineStr"/>
       <c r="AA23" s="2" t="inlineStr"/>
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
       <c r="AE23" s="2" t="inlineStr"/>
-      <c r="AF23" s="2" t="n">
+      <c r="AF23" s="2" t="inlineStr"/>
+      <c r="AG23" s="2" t="n">
         <v>16.33</v>
       </c>
-      <c r="AG23" s="2" t="n">
+      <c r="AH23" s="2" t="n">
         <v>-0.62</v>
       </c>
-      <c r="AH23" s="2" t="n">
+      <c r="AI23" s="2" t="n">
         <v>-9.65</v>
       </c>
-      <c r="AI23" s="2" t="n">
+      <c r="AJ23" s="2" t="n">
         <v>-21.88</v>
       </c>
-      <c r="AJ23" s="2" t="n">
+      <c r="AK23" s="2" t="n">
         <v>5.2</v>
       </c>
-      <c r="AK23" s="2" t="n">
+      <c r="AL23" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL23" s="2" t="inlineStr"/>
-      <c r="AM23" s="2" t="n">
+      <c r="AM23" s="2" t="inlineStr"/>
+      <c r="AN23" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="AN23" s="2" t="inlineStr"/>
       <c r="AO23" s="2" t="inlineStr"/>
-      <c r="AP23" s="2" t="inlineStr">
+      <c r="AP23" s="2" t="inlineStr"/>
+      <c r="AQ23" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ23" s="2" t="n">
+      <c r="AR23" s="2" t="n">
         <v>0.86</v>
       </c>
-      <c r="AR23" s="2" t="n">
+      <c r="AS23" s="2" t="n">
         <v>0.916</v>
       </c>
-      <c r="AS23" s="2" t="n">
+      <c r="AT23" s="2" t="n">
         <v>0.984</v>
       </c>
-      <c r="AT23" s="2" t="n">
+      <c r="AU23" s="2" t="n">
         <v>0.999</v>
       </c>
-      <c r="AU23" s="2" t="n">
+      <c r="AV23" s="2" t="n">
         <v>1.005</v>
       </c>
-      <c r="AV23" s="2" t="n">
+      <c r="AW23" s="2" t="n">
         <v>1.108</v>
       </c>
-      <c r="AW23" s="2" t="n">
+      <c r="AX23" s="2" t="n">
         <v>0.975</v>
       </c>
-      <c r="AX23" s="2" t="n">
+      <c r="AY23" s="2" t="n">
         <v>-5.309</v>
       </c>
-      <c r="AY23" s="2" t="n">
+      <c r="AZ23" s="2" t="n">
         <v>-2.1096</v>
       </c>
-      <c r="AZ23" s="2" t="n">
+      <c r="BA23" s="2" t="n">
         <v>-0.7655999999999999</v>
       </c>
-      <c r="BA23" s="2" t="n">
+      <c r="BB23" s="2" t="n">
         <v>-0.628</v>
       </c>
-      <c r="BB23" s="2" t="n">
+      <c r="BC23" s="2" t="n">
         <v>0.1633</v>
       </c>
     </row>
@@ -3989,85 +4037,90 @@
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>2C(减速)</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr">
         <is>
+          <t>减速</t>
+        </is>
+      </c>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
           <t>2A→2C·2d ← 2B→2A·13d ← 3→2B·17d</t>
         </is>
       </c>
-      <c r="Z24" s="2" t="inlineStr"/>
       <c r="AA24" s="2" t="inlineStr"/>
-      <c r="AB24" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD24" s="2" t="inlineStr"/>
+      <c r="AD24" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AE24" s="2" t="inlineStr"/>
-      <c r="AF24" s="2" t="n">
+      <c r="AF24" s="2" t="inlineStr"/>
+      <c r="AG24" s="2" t="n">
         <v>24.58</v>
       </c>
-      <c r="AG24" s="2" t="n">
+      <c r="AH24" s="2" t="n">
         <v>17.63</v>
       </c>
-      <c r="AH24" s="2" t="n">
+      <c r="AI24" s="2" t="n">
         <v>0.7</v>
       </c>
-      <c r="AI24" s="2" t="n">
+      <c r="AJ24" s="2" t="n">
         <v>0.48</v>
       </c>
-      <c r="AJ24" s="2" t="n">
+      <c r="AK24" s="2" t="n">
         <v>68.59999999999999</v>
       </c>
-      <c r="AK24" s="2" t="n">
+      <c r="AL24" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="AL24" s="2" t="inlineStr"/>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr"/>
       <c r="AO24" s="2" t="inlineStr"/>
-      <c r="AP24" s="2" t="inlineStr">
+      <c r="AP24" s="2" t="inlineStr"/>
+      <c r="AQ24" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ24" s="2" t="n">
+      <c r="AR24" s="2" t="n">
         <v>1.283</v>
       </c>
-      <c r="AR24" s="2" t="n">
+      <c r="AS24" s="2" t="n">
         <v>1.273</v>
       </c>
-      <c r="AS24" s="2" t="n">
+      <c r="AT24" s="2" t="n">
         <v>1.275</v>
       </c>
-      <c r="AT24" s="2" t="n">
+      <c r="AU24" s="2" t="n">
         <v>1.29</v>
       </c>
-      <c r="AU24" s="2" t="n">
+      <c r="AV24" s="2" t="n">
         <v>1.273</v>
       </c>
-      <c r="AV24" s="2" t="n">
+      <c r="AW24" s="2" t="n">
         <v>1.241</v>
       </c>
-      <c r="AW24" s="2" t="n">
+      <c r="AX24" s="2" t="n">
         <v>1.207</v>
       </c>
-      <c r="AX24" s="2" t="n">
+      <c r="AY24" s="2" t="n">
         <v>0.3059</v>
       </c>
-      <c r="AY24" s="2" t="n">
+      <c r="AZ24" s="2" t="n">
         <v>-0.1895</v>
       </c>
-      <c r="AZ24" s="2" t="n">
+      <c r="BA24" s="2" t="n">
         <v>0.3571</v>
       </c>
-      <c r="BA24" s="2" t="n">
+      <c r="BB24" s="2" t="n">
         <v>0.1031</v>
       </c>
-      <c r="BB24" s="2" t="n">
+      <c r="BC24" s="2" t="n">
         <v>0.2458</v>
       </c>
     </row>
@@ -4144,80 +4197,81 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y25" s="2" t="inlineStr">
+      <c r="Y25" s="2" t="inlineStr"/>
+      <c r="Z25" s="2" t="inlineStr">
         <is>
           <t>4+→4·6d ← 4→4+·9d</t>
         </is>
       </c>
-      <c r="Z25" s="2" t="inlineStr"/>
       <c r="AA25" s="2" t="inlineStr"/>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="inlineStr"/>
-      <c r="AF25" s="2" t="n">
+      <c r="AF25" s="2" t="inlineStr"/>
+      <c r="AG25" s="2" t="n">
         <v>-28.32</v>
       </c>
-      <c r="AG25" s="2" t="n">
+      <c r="AH25" s="2" t="n">
         <v>-18.4</v>
       </c>
-      <c r="AH25" s="2" t="n">
+      <c r="AI25" s="2" t="n">
         <v>-2.5</v>
       </c>
-      <c r="AI25" s="2" t="n">
+      <c r="AJ25" s="2" t="n">
         <v>-2.93</v>
       </c>
-      <c r="AJ25" s="2" t="n">
+      <c r="AK25" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="AK25" s="2" t="n">
+      <c r="AL25" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AL25" s="2" t="inlineStr"/>
-      <c r="AM25" s="2" t="n">
+      <c r="AM25" s="2" t="inlineStr"/>
+      <c r="AN25" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AN25" s="2" t="inlineStr"/>
       <c r="AO25" s="2" t="inlineStr"/>
-      <c r="AP25" s="2" t="inlineStr">
+      <c r="AP25" s="2" t="inlineStr"/>
+      <c r="AQ25" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AQ25" s="2" t="n">
+      <c r="AR25" s="2" t="n">
         <v>0.746</v>
       </c>
-      <c r="AR25" s="2" t="n">
+      <c r="AS25" s="2" t="n">
         <v>0.76</v>
       </c>
-      <c r="AS25" s="2" t="n">
+      <c r="AT25" s="2" t="n">
         <v>0.782</v>
       </c>
-      <c r="AT25" s="2" t="n">
+      <c r="AU25" s="2" t="n">
         <v>0.796</v>
       </c>
-      <c r="AU25" s="2" t="n">
+      <c r="AV25" s="2" t="n">
         <v>0.819</v>
       </c>
-      <c r="AV25" s="2" t="n">
+      <c r="AW25" s="2" t="n">
         <v>0.895</v>
       </c>
-      <c r="AW25" s="2" t="n">
+      <c r="AX25" s="2" t="n">
         <v>0.983</v>
       </c>
-      <c r="AX25" s="2" t="n">
+      <c r="AY25" s="2" t="n">
         <v>-2.1631</v>
       </c>
-      <c r="AY25" s="2" t="n">
+      <c r="AZ25" s="2" t="n">
         <v>-1.1063</v>
       </c>
-      <c r="AZ25" s="2" t="n">
+      <c r="BA25" s="2" t="n">
         <v>-0.4784</v>
       </c>
-      <c r="BA25" s="2" t="n">
+      <c r="BB25" s="2" t="n">
         <v>-1.0643</v>
       </c>
-      <c r="BB25" s="2" t="n">
+      <c r="BC25" s="2" t="n">
         <v>-0.2832</v>
       </c>
     </row>
@@ -4284,80 +4338,81 @@
           <t>1</t>
         </is>
       </c>
-      <c r="Y26" s="2" t="inlineStr">
+      <c r="Y26" s="2" t="inlineStr"/>
+      <c r="Z26" s="2" t="inlineStr">
         <is>
           <t>2A→1·8d ← 3→2A·12d</t>
         </is>
       </c>
-      <c r="Z26" s="2" t="inlineStr"/>
       <c r="AA26" s="2" t="inlineStr"/>
       <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr"/>
-      <c r="AF26" s="2" t="n">
+      <c r="AF26" s="2" t="inlineStr"/>
+      <c r="AG26" s="2" t="n">
         <v>12.26</v>
       </c>
-      <c r="AG26" s="2" t="n">
+      <c r="AH26" s="2" t="n">
         <v>-3.14</v>
       </c>
-      <c r="AH26" s="2" t="n">
+      <c r="AI26" s="2" t="n">
         <v>-10.42</v>
       </c>
-      <c r="AI26" s="2" t="n">
+      <c r="AJ26" s="2" t="n">
         <v>-21.45</v>
       </c>
-      <c r="AJ26" s="2" t="n">
+      <c r="AK26" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="AK26" s="2" t="n">
+      <c r="AL26" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL26" s="2" t="inlineStr"/>
-      <c r="AM26" s="2" t="n">
+      <c r="AM26" s="2" t="inlineStr"/>
+      <c r="AN26" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="AN26" s="2" t="inlineStr"/>
       <c r="AO26" s="2" t="inlineStr"/>
-      <c r="AP26" s="2" t="inlineStr">
+      <c r="AP26" s="2" t="inlineStr"/>
+      <c r="AQ26" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ26" s="2" t="n">
+      <c r="AR26" s="2" t="n">
         <v>0.5590000000000001</v>
       </c>
-      <c r="AR26" s="2" t="n">
+      <c r="AS26" s="2" t="n">
         <v>0.595</v>
       </c>
-      <c r="AS26" s="2" t="n">
+      <c r="AT26" s="2" t="n">
         <v>0.64</v>
       </c>
-      <c r="AT26" s="2" t="n">
+      <c r="AU26" s="2" t="n">
         <v>0.648</v>
       </c>
-      <c r="AU26" s="2" t="n">
+      <c r="AV26" s="2" t="n">
         <v>0.649</v>
       </c>
-      <c r="AV26" s="2" t="n">
+      <c r="AW26" s="2" t="n">
         <v>0.718</v>
       </c>
-      <c r="AW26" s="2" t="n">
+      <c r="AX26" s="2" t="n">
         <v>0.644</v>
       </c>
-      <c r="AX26" s="2" t="n">
+      <c r="AY26" s="2" t="n">
         <v>-5.5798</v>
       </c>
-      <c r="AY26" s="2" t="n">
+      <c r="AZ26" s="2" t="n">
         <v>-2.0116</v>
       </c>
-      <c r="AZ26" s="2" t="n">
+      <c r="BA26" s="2" t="n">
         <v>-0.6197</v>
       </c>
-      <c r="BA26" s="2" t="n">
+      <c r="BB26" s="2" t="n">
         <v>-0.7297</v>
       </c>
-      <c r="BB26" s="2" t="n">
+      <c r="BC26" s="2" t="n">
         <v>0.1226</v>
       </c>
     </row>
@@ -4434,80 +4489,81 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y27" s="2" t="inlineStr">
+      <c r="Y27" s="2" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr">
         <is>
           <t>4+→4·2d ← 4→4+·4d ← 4+→4·6d</t>
         </is>
       </c>
-      <c r="Z27" s="2" t="inlineStr"/>
       <c r="AA27" s="2" t="inlineStr"/>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="inlineStr"/>
       <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
-      <c r="AF27" s="2" t="n">
+      <c r="AF27" s="2" t="inlineStr"/>
+      <c r="AG27" s="2" t="n">
         <v>-29.84</v>
       </c>
-      <c r="AG27" s="2" t="n">
+      <c r="AH27" s="2" t="n">
         <v>-18.28</v>
       </c>
-      <c r="AH27" s="2" t="n">
+      <c r="AI27" s="2" t="n">
         <v>-3.27</v>
       </c>
-      <c r="AI27" s="2" t="n">
+      <c r="AJ27" s="2" t="n">
         <v>-2.81</v>
       </c>
-      <c r="AJ27" s="2" t="n">
+      <c r="AK27" s="2" t="n">
         <v>-1.4</v>
       </c>
-      <c r="AK27" s="2" t="n">
+      <c r="AL27" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL27" s="2" t="inlineStr"/>
-      <c r="AM27" s="2" t="n">
+      <c r="AM27" s="2" t="inlineStr"/>
+      <c r="AN27" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AN27" s="2" t="inlineStr"/>
       <c r="AO27" s="2" t="inlineStr"/>
-      <c r="AP27" s="2" t="inlineStr">
+      <c r="AP27" s="2" t="inlineStr"/>
+      <c r="AQ27" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AQ27" s="2" t="n">
+      <c r="AR27" s="2" t="n">
         <v>2.166</v>
       </c>
-      <c r="AR27" s="2" t="n">
+      <c r="AS27" s="2" t="n">
         <v>2.199</v>
       </c>
-      <c r="AS27" s="2" t="n">
+      <c r="AT27" s="2" t="n">
         <v>2.258</v>
       </c>
-      <c r="AT27" s="2" t="n">
+      <c r="AU27" s="2" t="n">
         <v>2.306</v>
       </c>
-      <c r="AU27" s="2" t="n">
+      <c r="AV27" s="2" t="n">
         <v>2.394</v>
       </c>
-      <c r="AV27" s="2" t="n">
+      <c r="AW27" s="2" t="n">
         <v>2.611</v>
       </c>
-      <c r="AW27" s="2" t="n">
+      <c r="AX27" s="2" t="n">
         <v>2.838</v>
       </c>
-      <c r="AX27" s="2" t="n">
+      <c r="AY27" s="2" t="n">
         <v>-1.7804</v>
       </c>
-      <c r="AY27" s="2" t="n">
+      <c r="AZ27" s="2" t="n">
         <v>-1.1079</v>
       </c>
-      <c r="AZ27" s="2" t="n">
+      <c r="BA27" s="2" t="n">
         <v>-0.5972</v>
       </c>
-      <c r="BA27" s="2" t="n">
+      <c r="BB27" s="2" t="n">
         <v>-1.0365</v>
       </c>
-      <c r="BB27" s="2" t="n">
+      <c r="BC27" s="2" t="n">
         <v>-0.2984</v>
       </c>
     </row>
@@ -4574,76 +4630,77 @@
           <t>4</t>
         </is>
       </c>
-      <c r="Y28" s="2" t="inlineStr">
+      <c r="Y28" s="2" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr">
         <is>
           <t>4+→4·6d ← 4→4+·14d ← 4+→4·16d</t>
         </is>
       </c>
-      <c r="Z28" s="2" t="inlineStr"/>
       <c r="AA28" s="2" t="inlineStr"/>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="inlineStr"/>
-      <c r="AF28" s="2" t="n">
+      <c r="AF28" s="2" t="inlineStr"/>
+      <c r="AG28" s="2" t="n">
         <v>-17.65</v>
       </c>
-      <c r="AG28" s="2" t="n">
+      <c r="AH28" s="2" t="n">
         <v>-13.43</v>
       </c>
-      <c r="AH28" s="2" t="n">
+      <c r="AI28" s="2" t="n">
         <v>-4.7</v>
       </c>
-      <c r="AI28" s="2" t="n">
+      <c r="AJ28" s="2" t="n">
         <v>-6.85</v>
       </c>
-      <c r="AJ28" s="2" t="n">
+      <c r="AK28" s="2" t="n">
         <v>-5.4</v>
       </c>
-      <c r="AK28" s="2" t="inlineStr"/>
       <c r="AL28" s="2" t="inlineStr"/>
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr"/>
       <c r="AO28" s="2" t="inlineStr"/>
-      <c r="AP28" s="2" t="inlineStr">
+      <c r="AP28" s="2" t="inlineStr"/>
+      <c r="AQ28" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AQ28" s="2" t="n">
+      <c r="AR28" s="2" t="n">
         <v>0.828</v>
       </c>
-      <c r="AR28" s="2" t="n">
+      <c r="AS28" s="2" t="n">
         <v>0.861</v>
       </c>
-      <c r="AS28" s="2" t="n">
+      <c r="AT28" s="2" t="n">
         <v>0.892</v>
       </c>
-      <c r="AT28" s="2" t="n">
+      <c r="AU28" s="2" t="n">
         <v>0.912</v>
       </c>
-      <c r="AU28" s="2" t="n">
+      <c r="AV28" s="2" t="n">
         <v>0.9409999999999999</v>
       </c>
-      <c r="AV28" s="2" t="n">
+      <c r="AW28" s="2" t="n">
         <v>1.02</v>
       </c>
-      <c r="AW28" s="2" t="n">
+      <c r="AX28" s="2" t="n">
         <v>1.024</v>
       </c>
-      <c r="AX28" s="2" t="n">
+      <c r="AY28" s="2" t="n">
         <v>-2.8959</v>
       </c>
-      <c r="AY28" s="2" t="n">
+      <c r="AZ28" s="2" t="n">
         <v>-1.6928</v>
       </c>
-      <c r="AZ28" s="2" t="n">
+      <c r="BA28" s="2" t="n">
         <v>-0.5815</v>
       </c>
-      <c r="BA28" s="2" t="n">
+      <c r="BB28" s="2" t="n">
         <v>-0.8463000000000001</v>
       </c>
-      <c r="BB28" s="2" t="n">
+      <c r="BC28" s="2" t="n">
         <v>-0.1765</v>
       </c>
     </row>
@@ -4713,77 +4770,78 @@
       <c r="Y29" s="2" t="inlineStr"/>
       <c r="Z29" s="2" t="inlineStr"/>
       <c r="AA29" s="2" t="inlineStr"/>
-      <c r="AB29" s="2" t="inlineStr">
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="AC29" s="2" t="inlineStr"/>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
-      <c r="AF29" s="2" t="n">
+      <c r="AF29" s="2" t="inlineStr"/>
+      <c r="AG29" s="2" t="n">
         <v>6.07</v>
       </c>
-      <c r="AG29" s="2" t="n">
+      <c r="AH29" s="2" t="n">
         <v>-1.15</v>
       </c>
-      <c r="AH29" s="2" t="n">
+      <c r="AI29" s="2" t="n">
         <v>-3.43</v>
       </c>
-      <c r="AI29" s="2" t="n">
+      <c r="AJ29" s="2" t="n">
         <v>-7.23</v>
       </c>
-      <c r="AJ29" s="2" t="n">
+      <c r="AK29" s="2" t="n">
         <v>-6.5</v>
       </c>
-      <c r="AK29" s="2" t="n">
+      <c r="AL29" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AL29" s="2" t="inlineStr"/>
-      <c r="AM29" s="2" t="n">
+      <c r="AM29" s="2" t="inlineStr"/>
+      <c r="AN29" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="AN29" s="2" t="inlineStr"/>
       <c r="AO29" s="2" t="inlineStr"/>
-      <c r="AP29" s="2" t="inlineStr">
+      <c r="AP29" s="2" t="inlineStr"/>
+      <c r="AQ29" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AQ29" s="2" t="n">
+      <c r="AR29" s="2" t="n">
         <v>1.49</v>
       </c>
-      <c r="AR29" s="2" t="n">
+      <c r="AS29" s="2" t="n">
         <v>1.562</v>
       </c>
-      <c r="AS29" s="2" t="n">
+      <c r="AT29" s="2" t="n">
         <v>1.629</v>
       </c>
-      <c r="AT29" s="2" t="n">
+      <c r="AU29" s="2" t="n">
         <v>1.659</v>
       </c>
-      <c r="AU29" s="2" t="n">
+      <c r="AV29" s="2" t="n">
         <v>1.703</v>
       </c>
-      <c r="AV29" s="2" t="n">
+      <c r="AW29" s="2" t="n">
         <v>1.834</v>
       </c>
-      <c r="AW29" s="2" t="n">
+      <c r="AX29" s="2" t="n">
         <v>1.676</v>
       </c>
-      <c r="AX29" s="2" t="n">
+      <c r="AY29" s="2" t="n">
         <v>-3.8596</v>
       </c>
-      <c r="AY29" s="2" t="n">
+      <c r="AZ29" s="2" t="n">
         <v>-1.5157</v>
       </c>
-      <c r="AZ29" s="2" t="n">
+      <c r="BA29" s="2" t="n">
         <v>-1.0734</v>
       </c>
-      <c r="BA29" s="2" t="n">
+      <c r="BB29" s="2" t="n">
         <v>-0.4752</v>
       </c>
-      <c r="BB29" s="2" t="n">
+      <c r="BC29" s="2" t="n">
         <v>0.0607</v>
       </c>
     </row>
@@ -4848,49 +4906,47 @@
           <t>1</t>
         </is>
       </c>
-      <c r="Y30" s="2" t="inlineStr">
+      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr">
         <is>
           <t>1+→1·6d ← 1→1+·7d ← 1+→1·10d</t>
         </is>
       </c>
-      <c r="Z30" s="2" t="inlineStr"/>
       <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
-      <c r="AF30" s="2" t="n">
+      <c r="AF30" s="2" t="inlineStr"/>
+      <c r="AG30" s="2" t="n">
         <v>-2.78</v>
       </c>
-      <c r="AG30" s="2" t="n">
+      <c r="AH30" s="2" t="n">
         <v>7.74</v>
       </c>
-      <c r="AH30" s="2" t="n">
+      <c r="AI30" s="2" t="n">
         <v>0.66</v>
       </c>
-      <c r="AI30" s="2" t="n">
+      <c r="AJ30" s="2" t="n">
         <v>8.27</v>
       </c>
-      <c r="AJ30" s="2" t="n">
+      <c r="AK30" s="2" t="n">
         <v>67.2</v>
       </c>
-      <c r="AK30" s="2" t="n">
+      <c r="AL30" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="AL30" s="2" t="inlineStr"/>
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr"/>
       <c r="AO30" s="2" t="inlineStr"/>
-      <c r="AP30" s="2" t="inlineStr">
+      <c r="AP30" s="2" t="inlineStr"/>
+      <c r="AQ30" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ30" s="2" t="n">
+      <c r="AR30" s="2" t="n">
         <v>0.336</v>
-      </c>
-      <c r="AR30" s="2" t="n">
-        <v>0.339</v>
       </c>
       <c r="AS30" s="2" t="n">
         <v>0.339</v>
@@ -4899,27 +4955,30 @@
         <v>0.339</v>
       </c>
       <c r="AU30" s="2" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="AV30" s="2" t="n">
         <v>0.341</v>
       </c>
-      <c r="AV30" s="2" t="n">
+      <c r="AW30" s="2" t="n">
         <v>0.326</v>
       </c>
-      <c r="AW30" s="2" t="n">
+      <c r="AX30" s="2" t="n">
         <v>0.336</v>
       </c>
-      <c r="AX30" s="2" t="n">
+      <c r="AY30" s="2" t="n">
         <v>-0.6756</v>
       </c>
-      <c r="AY30" s="2" t="n">
+      <c r="AZ30" s="2" t="n">
         <v>-0.118</v>
       </c>
-      <c r="AZ30" s="2" t="n">
+      <c r="BA30" s="2" t="n">
         <v>0.2082</v>
       </c>
-      <c r="BA30" s="2" t="n">
+      <c r="BB30" s="2" t="n">
         <v>0.0615</v>
       </c>
-      <c r="BB30" s="2" t="n">
+      <c r="BC30" s="2" t="n">
         <v>-0.0278</v>
       </c>
     </row>
@@ -4983,86 +5042,91 @@
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>4+(周J超卖·日线纠缠)</t>
+          <t>4+</t>
         </is>
       </c>
       <c r="Y31" s="2" t="inlineStr">
         <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
           <t>4→4+·14d</t>
         </is>
       </c>
-      <c r="Z31" s="2" t="inlineStr"/>
       <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
-      <c r="AF31" s="2" t="n">
+      <c r="AF31" s="2" t="inlineStr"/>
+      <c r="AG31" s="2" t="n">
         <v>-37.27</v>
       </c>
-      <c r="AG31" s="2" t="n">
+      <c r="AH31" s="2" t="n">
         <v>-5.34</v>
       </c>
-      <c r="AH31" s="2" t="n">
+      <c r="AI31" s="2" t="n">
         <v>3.77</v>
       </c>
-      <c r="AI31" s="2" t="n">
+      <c r="AJ31" s="2" t="n">
         <v>9.33</v>
       </c>
-      <c r="AJ31" s="2" t="n">
+      <c r="AK31" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="AK31" s="2" t="n">
+      <c r="AL31" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="AL31" s="2" t="inlineStr"/>
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr"/>
       <c r="AO31" s="2" t="inlineStr"/>
-      <c r="AP31" s="2" t="inlineStr">
+      <c r="AP31" s="2" t="inlineStr"/>
+      <c r="AQ31" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AQ31" s="2" t="n">
+      <c r="AR31" s="2" t="n">
         <v>0.417</v>
       </c>
-      <c r="AR31" s="2" t="n">
+      <c r="AS31" s="2" t="n">
         <v>0.414</v>
       </c>
-      <c r="AS31" s="2" t="n">
+      <c r="AT31" s="2" t="n">
         <v>0.413</v>
       </c>
-      <c r="AT31" s="2" t="n">
+      <c r="AU31" s="2" t="n">
         <v>0.417</v>
       </c>
-      <c r="AU31" s="2" t="n">
+      <c r="AV31" s="2" t="n">
         <v>0.425</v>
       </c>
-      <c r="AV31" s="2" t="n">
+      <c r="AW31" s="2" t="n">
         <v>0.422</v>
       </c>
-      <c r="AW31" s="2" t="n">
+      <c r="AX31" s="2" t="n">
         <v>0.469</v>
       </c>
-      <c r="AX31" s="2" t="n">
+      <c r="AY31" s="2" t="n">
         <v>0.2368</v>
       </c>
-      <c r="AY31" s="2" t="n">
+      <c r="AZ31" s="2" t="n">
         <v>-0.3888</v>
       </c>
-      <c r="AZ31" s="2" t="n">
+      <c r="BA31" s="2" t="n">
         <v>-0.1053</v>
       </c>
-      <c r="BA31" s="2" t="n">
+      <c r="BB31" s="2" t="n">
         <v>-0.2478</v>
       </c>
-      <c r="BB31" s="2" t="n">
+      <c r="BC31" s="2" t="n">
         <v>-0.3727</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB1"/>
+  <autoFilter ref="A1:BC1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5073,7 +5137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5325,7 +5389,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stage (Weinstein 大阶段 v2.1引擎: EMA30W(150日EMA)锚, 判定优先级从高到低): ①均线排列覆盖: MA20&gt;MA50&gt;MA100&gt;MA150(简单均线)多头排列→强制Stage2; MA20&lt;MA50&lt;MA100&lt;MA150空头排列→强制Stage4(忽略斜率, 解决慢磨盲区) ②斜率双确认: EMA30W变化年化(4周×13与13周×3.88)均&gt;+8%→2; 均&lt;-6%→4(不对称) ③放平带: 52周位置+价格确认分1/3(3:pos&gt;0.55且价≥0.95×EMA30W; 1:pos&lt;0.45且价≤1.05×; 0.45~0.55滞回)。NA=历史&lt;300交易日</t>
+          <t xml:space="preserve">  Stage (Weinstein 大阶段 v2.2引擎: EMA30W(150日EMA)锚, 判定优先级从高到低): ①均线排列覆盖: MA20&gt;MA50&gt;MA100&gt;MA150(简单均线)多头排列→强制Stage2; MA20&lt;MA50&lt;MA100&lt;MA150空头排列→强制Stage4(忽略斜率, 解决慢磨盲区) ②斜率双确认: EMA30W变化年化(4周×13与13周×3.88)均&gt;+8%→2; 均&lt;-6%→4(不对称) ③放平带: 52周位置+价格确认分1/3(3:pos&gt;0.55且价≥0.95×EMA30W; 1:pos&lt;0.45且价≤1.05×; 0.45~0.55滞回)。降级层(v2.2): 151-252根新股→①可用②仅≥215根③用上市以来位置, 标记列带'新'; ≤150根→NA</t>
         </is>
       </c>
     </row>
@@ -5346,133 +5410,140 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  子档(v2.1): 4+=止跌(日线MA5/10/20纠缠+快线&gt;慢线+周J超卖或底背离, 价&lt;EMA10W) | 1=筑底(不区分价格vs EMA10W) | 1+=强筑底(站稳MA5/10/20全三条+全上行+周MACD DIF&gt;DEA; 标记:预金叉·纠缠·底背离) | 2A=修复态或刚确立(≤10日) | 2B=满配(slope10&gt;0·EMA10W&gt;EMA30W·10日前也是) | 2C=满配+延伸/减速/顶背离 | 3/4不分档。4+的标记: 周J超卖·底背离·日线纠缠; 2C的标记: 延伸(&gt;25%)·减速·顶背离</t>
+          <t xml:space="preserve">  子档(v2.1): 4+=止跌(日线MA5/10/20纠缠+快线&gt;慢线+周J超卖或底背离, 价&lt;EMA10W) | 1=筑底(不区分价格vs EMA10W) | 1+=强筑底(站稳MA5/10/20全三条+全上行+周MACD DIF&gt;DEA) | 2A=修复态或刚确立(≤10日) | 2B=满配(slope10&gt;0·EMA10W&gt;EMA30W·10日前也是) | 2C=满配+延伸/减速/顶背离 | 3/4不分档</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  子档标记: 状态描述列(与子档列分开)。4+→周J超卖·底背离·日线纠缠(止跌命中条件); 1+→预金叉(EMA10W/30W将≤20日内纠缠或金叉)·纠缠·底背离; 2C→延伸(价超EMA30W达25%)·减速·顶背离; 新=降级层(上市151-252根弱规则档)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  子档变化: 近20日内最近3次子档转换, 新→旧 (如 '1A→1B·5d ← 2A→2B·12d')</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr"/>
-    </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>【④ 企稳上行 — Cross】</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
+          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
+          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
+          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
+          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">    有过零但不稳定(whipsaw/暴涨驱动等脏交叉) → 0; 无过零但两线持续重叠(近5日rel&lt;0.2%) → 0; 其余空</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr"/>
-    </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>【⑦ 均线 MV 与年化斜率】(最右 12 列)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ND MV: N日收盘均线(前复权)最新值, N=5/10/20/30/50/100/200。历史不足N个交易日留空</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ND斜率: (N日均线最新 ÷ 5个交易日前的N日均线 - 1) ×52, 年化小数(0.1=10%)。N=10/20/50/100/200, 正值=均线上行</t>
+          <t xml:space="preserve">  ND MV: N日收盘均线(前复权)最新值, N=5/10/20/30/50/100/200。历史不足N个交易日留空</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  ND斜率: (N日均线最新 ÷ 5个交易日前的N日均线 - 1) ×52, 年化小数(0.1=10%)。N=10/20/50/100/200, 正值=均线上行</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">           (与【⑤】年线斜率列的×100百分比口径不同, 本列为原始×52; 不足N+5个交易日留空)</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr"/>
-    </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>【⑤ ETF 专属 — 趋势/Mansfield RS】</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
+          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  MRS_沪深300_1W / MRS_沪深300_4W: MRS_沪深300 分数的 5日 / 20日 变化</t>
         </is>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-18
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$BD$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$BF$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD31"/>
+  <dimension ref="A1:BF31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -527,6 +527,8 @@
     <col width="11" customWidth="1" min="54" max="54"/>
     <col width="11" customWidth="1" min="55" max="55"/>
     <col width="11" customWidth="1" min="56" max="56"/>
+    <col width="11" customWidth="1" min="57" max="57"/>
+    <col width="11" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -672,140 +674,150 @@
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
+          <t>SOS晋升</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>SOW降级</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
           <t>KDJ Cross</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>日MACD Cross</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>周MACD Cross</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>5_10 Cross</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>10_50 Cross</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>年线斜率</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300_1W</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>MRS_沪深300_4W</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>风险度</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>动量</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>DS信号</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>B距今</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>S距今</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>急杀</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>周线档</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>5D MV</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>10D MV</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>20D MV</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>30D MV</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>50D MV</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>100D MV</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>200D MV</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>10D斜率</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>20D斜率</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>50D斜率</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>100D斜率</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>200D斜率</t>
         </is>
@@ -867,7 +879,7 @@
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
@@ -875,11 +887,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr"/>
-      <c r="Z2" s="2" t="inlineStr">
-        <is>
-          <t>1→4·5d</t>
-        </is>
-      </c>
+      <c r="Z2" s="2" t="inlineStr"/>
       <c r="AA2" s="2" t="inlineStr"/>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr"/>
@@ -887,69 +895,71 @@
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr"/>
-      <c r="AH2" s="2" t="n">
+      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AI2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="n">
         <v>-10.15</v>
       </c>
-      <c r="AI2" s="2" t="n">
+      <c r="AK2" s="2" t="n">
         <v>-9.01</v>
       </c>
-      <c r="AJ2" s="2" t="n">
+      <c r="AL2" s="2" t="n">
         <v>-5.58</v>
       </c>
-      <c r="AK2" s="2" t="n">
+      <c r="AM2" s="2" t="n">
         <v>-10.16</v>
       </c>
-      <c r="AL2" s="2" t="n">
+      <c r="AN2" s="2" t="n">
         <v>-6.5</v>
       </c>
-      <c r="AM2" s="2" t="n">
+      <c r="AO2" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AN2" s="2" t="inlineStr"/>
-      <c r="AO2" s="2" t="n">
+      <c r="AP2" s="2" t="inlineStr"/>
+      <c r="AQ2" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AP2" s="2" t="inlineStr"/>
-      <c r="AQ2" s="2" t="inlineStr"/>
-      <c r="AR2" s="2" t="inlineStr">
+      <c r="AR2" s="2" t="inlineStr"/>
+      <c r="AS2" s="2" t="inlineStr"/>
+      <c r="AT2" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AS2" s="2" t="n">
+      <c r="AU2" s="2" t="n">
         <v>2.889</v>
       </c>
-      <c r="AT2" s="2" t="n">
+      <c r="AV2" s="2" t="n">
         <v>3.003</v>
       </c>
-      <c r="AU2" s="2" t="n">
+      <c r="AW2" s="2" t="n">
         <v>3.177</v>
       </c>
-      <c r="AV2" s="2" t="n">
+      <c r="AX2" s="2" t="n">
         <v>3.245</v>
       </c>
-      <c r="AW2" s="2" t="n">
+      <c r="AY2" s="2" t="n">
         <v>3.362</v>
       </c>
-      <c r="AX2" s="2" t="n">
+      <c r="AZ2" s="2" t="n">
         <v>3.646</v>
       </c>
-      <c r="AY2" s="2" t="n">
+      <c r="BA2" s="2" t="n">
         <v>3.519</v>
       </c>
-      <c r="AZ2" s="2" t="n">
+      <c r="BB2" s="2" t="n">
         <v>-3.9913</v>
       </c>
-      <c r="BA2" s="2" t="n">
+      <c r="BC2" s="2" t="n">
         <v>-1.8798</v>
       </c>
-      <c r="BB2" s="2" t="n">
+      <c r="BD2" s="2" t="n">
         <v>-0.8233</v>
       </c>
-      <c r="BC2" s="2" t="n">
+      <c r="BE2" s="2" t="n">
         <v>-0.7401</v>
       </c>
-      <c r="BD2" s="2" t="n">
+      <c r="BF2" s="2" t="n">
         <v>-0.1015</v>
       </c>
     </row>
@@ -1003,97 +1013,99 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W3" s="2" t="n">
-        <v>42</v>
+        <v>103</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr"/>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>4+→1·9d ← 1→4+·10d</t>
+          <t>4+→4·6d ← 4→4+·15d</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr"/>
       <c r="AB3" s="2" t="inlineStr"/>
-      <c r="AC3" s="2" t="inlineStr">
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="n">
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF3" s="2" t="inlineStr"/>
-      <c r="AG3" s="2" t="inlineStr"/>
-      <c r="AH3" s="2" t="n">
+      <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="n">
         <v>-12.67</v>
       </c>
-      <c r="AI3" s="2" t="n">
+      <c r="AK3" s="2" t="n">
         <v>3.51</v>
       </c>
-      <c r="AJ3" s="2" t="n">
+      <c r="AL3" s="2" t="n">
         <v>3.46</v>
       </c>
-      <c r="AK3" s="2" t="n">
+      <c r="AM3" s="2" t="n">
         <v>5.98</v>
       </c>
-      <c r="AL3" s="2" t="n">
+      <c r="AN3" s="2" t="n">
         <v>46.7</v>
       </c>
-      <c r="AM3" s="2" t="n">
+      <c r="AO3" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="AN3" s="2" t="inlineStr"/>
-      <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr"/>
       <c r="AQ3" s="2" t="inlineStr"/>
-      <c r="AR3" s="2" t="inlineStr">
+      <c r="AR3" s="2" t="inlineStr"/>
+      <c r="AS3" s="2" t="inlineStr"/>
+      <c r="AT3" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS3" s="2" t="n">
+      <c r="AU3" s="2" t="n">
         <v>1.423</v>
       </c>
-      <c r="AT3" s="2" t="n">
+      <c r="AV3" s="2" t="n">
         <v>1.428</v>
       </c>
-      <c r="AU3" s="2" t="n">
+      <c r="AW3" s="2" t="n">
         <v>1.442</v>
       </c>
-      <c r="AV3" s="2" t="n">
+      <c r="AX3" s="2" t="n">
         <v>1.458</v>
       </c>
-      <c r="AW3" s="2" t="n">
+      <c r="AY3" s="2" t="n">
         <v>1.478</v>
       </c>
-      <c r="AX3" s="2" t="n">
+      <c r="AZ3" s="2" t="n">
         <v>1.463</v>
       </c>
-      <c r="AY3" s="2" t="n">
+      <c r="BA3" s="2" t="n">
         <v>1.51</v>
       </c>
-      <c r="AZ3" s="2" t="n">
+      <c r="BB3" s="2" t="n">
         <v>-0.6667</v>
       </c>
-      <c r="BA3" s="2" t="n">
+      <c r="BC3" s="2" t="n">
         <v>-0.5765</v>
       </c>
-      <c r="BB3" s="2" t="n">
+      <c r="BD3" s="2" t="n">
         <v>-0.2809</v>
       </c>
-      <c r="BC3" s="2" t="n">
+      <c r="BE3" s="2" t="n">
         <v>-0.1776</v>
       </c>
-      <c r="BD3" s="2" t="n">
+      <c r="BF3" s="2" t="n">
         <v>-0.1267</v>
       </c>
     </row>
@@ -1159,93 +1171,95 @@
         </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>16</v>
+        <v>152</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2A→2B·5d ← 3→2A·16d</t>
+          <t>2A→2C·7d</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr"/>
       <c r="AB4" s="2" t="inlineStr"/>
-      <c r="AC4" s="2" t="n">
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD4" s="2" t="n">
+      <c r="AF4" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AE4" s="2" t="inlineStr"/>
-      <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
-      <c r="AH4" s="2" t="n">
+      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="n">
         <v>57.14</v>
       </c>
-      <c r="AI4" s="2" t="n">
+      <c r="AK4" s="2" t="n">
         <v>39.33</v>
       </c>
-      <c r="AJ4" s="2" t="n">
+      <c r="AL4" s="2" t="n">
         <v>-3.4</v>
       </c>
-      <c r="AK4" s="2" t="n">
+      <c r="AM4" s="2" t="n">
         <v>12.35</v>
       </c>
-      <c r="AL4" s="2" t="n">
+      <c r="AN4" s="2" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="AM4" s="2" t="n">
+      <c r="AO4" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="AN4" s="2" t="inlineStr"/>
-      <c r="AO4" s="2" t="inlineStr"/>
-      <c r="AP4" s="2" t="n">
+      <c r="AP4" s="2" t="inlineStr"/>
+      <c r="AQ4" s="2" t="inlineStr"/>
+      <c r="AR4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AQ4" s="2" t="inlineStr"/>
-      <c r="AR4" s="2" t="inlineStr">
+      <c r="AS4" s="2" t="inlineStr"/>
+      <c r="AT4" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS4" s="2" t="n">
+      <c r="AU4" s="2" t="n">
         <v>1.856</v>
       </c>
-      <c r="AT4" s="2" t="n">
+      <c r="AV4" s="2" t="n">
         <v>1.845</v>
       </c>
-      <c r="AU4" s="2" t="n">
+      <c r="AW4" s="2" t="n">
         <v>1.801</v>
       </c>
-      <c r="AV4" s="2" t="n">
+      <c r="AX4" s="2" t="n">
         <v>1.761</v>
       </c>
-      <c r="AW4" s="2" t="n">
+      <c r="AY4" s="2" t="n">
         <v>1.664</v>
       </c>
-      <c r="AX4" s="2" t="n">
+      <c r="AZ4" s="2" t="n">
         <v>1.592</v>
       </c>
-      <c r="AY4" s="2" t="n">
+      <c r="BA4" s="2" t="n">
         <v>1.533</v>
       </c>
-      <c r="AZ4" s="2" t="n">
+      <c r="BB4" s="2" t="n">
         <v>1.8057</v>
       </c>
-      <c r="BA4" s="2" t="n">
+      <c r="BC4" s="2" t="n">
         <v>0.963</v>
       </c>
-      <c r="BB4" s="2" t="n">
+      <c r="BD4" s="2" t="n">
         <v>1.1789</v>
       </c>
-      <c r="BC4" s="2" t="n">
+      <c r="BE4" s="2" t="n">
         <v>0.3268</v>
       </c>
-      <c r="BD4" s="2" t="n">
+      <c r="BF4" s="2" t="n">
         <v>0.5714</v>
       </c>
     </row>
@@ -1299,7 +1313,7 @@
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W5" s="2" t="n">
@@ -1307,87 +1321,89 @@
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>3→1·4d ← 1+→3·13d ← 1→1+·14d</t>
+          <t>1→4·4d ← 1+→1·7d ← 1→1+·8d</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr"/>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="n">
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AE5" s="2" t="n">
+      <c r="AG5" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF5" s="2" t="inlineStr"/>
-      <c r="AG5" s="2" t="inlineStr"/>
-      <c r="AH5" s="2" t="n">
+      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="n">
         <v>-7.99</v>
       </c>
-      <c r="AI5" s="2" t="n">
+      <c r="AK5" s="2" t="n">
         <v>5.16</v>
       </c>
-      <c r="AJ5" s="2" t="n">
+      <c r="AL5" s="2" t="n">
         <v>-2.18</v>
       </c>
-      <c r="AK5" s="2" t="n">
+      <c r="AM5" s="2" t="n">
         <v>6.86</v>
       </c>
-      <c r="AL5" s="2" t="n">
+      <c r="AN5" s="2" t="n">
         <v>41.9</v>
       </c>
-      <c r="AM5" s="2" t="n">
+      <c r="AO5" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="AN5" s="2" t="inlineStr"/>
-      <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr"/>
       <c r="AQ5" s="2" t="inlineStr"/>
-      <c r="AR5" s="2" t="inlineStr">
+      <c r="AR5" s="2" t="inlineStr"/>
+      <c r="AS5" s="2" t="inlineStr"/>
+      <c r="AT5" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS5" s="2" t="n">
+      <c r="AU5" s="2" t="n">
         <v>0.8129999999999999</v>
       </c>
-      <c r="AT5" s="2" t="n">
+      <c r="AV5" s="2" t="n">
         <v>0.831</v>
       </c>
-      <c r="AU5" s="2" t="n">
+      <c r="AW5" s="2" t="n">
         <v>0.835</v>
       </c>
-      <c r="AV5" s="2" t="n">
+      <c r="AX5" s="2" t="n">
         <v>0.838</v>
       </c>
-      <c r="AW5" s="2" t="n">
+      <c r="AY5" s="2" t="n">
         <v>0.859</v>
       </c>
-      <c r="AX5" s="2" t="n">
+      <c r="AZ5" s="2" t="n">
         <v>0.828</v>
       </c>
-      <c r="AY5" s="2" t="n">
+      <c r="BA5" s="2" t="n">
         <v>0.831</v>
       </c>
-      <c r="AZ5" s="2" t="n">
+      <c r="BB5" s="2" t="n">
         <v>-1.3175</v>
       </c>
-      <c r="BA5" s="2" t="n">
+      <c r="BC5" s="2" t="n">
         <v>-0.3924</v>
       </c>
-      <c r="BB5" s="2" t="n">
+      <c r="BD5" s="2" t="n">
         <v>-0.1822</v>
       </c>
-      <c r="BC5" s="2" t="n">
+      <c r="BE5" s="2" t="n">
         <v>0.0692</v>
       </c>
-      <c r="BD5" s="2" t="n">
+      <c r="BF5" s="2" t="n">
         <v>-0.0799</v>
       </c>
     </row>
@@ -1443,11 +1459,11 @@
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W6" s="2" t="n">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
@@ -1457,79 +1473,81 @@
       <c r="Y6" s="2" t="inlineStr"/>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1→4·1d</t>
+          <t>4+→4·20d</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="inlineStr"/>
-      <c r="AC6" s="2" t="n">
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="inlineStr"/>
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
-      <c r="AH6" s="2" t="n">
+      <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="n">
         <v>-6.64</v>
       </c>
-      <c r="AI6" s="2" t="n">
+      <c r="AK6" s="2" t="n">
         <v>5.25</v>
       </c>
-      <c r="AJ6" s="2" t="n">
+      <c r="AL6" s="2" t="n">
         <v>1.6</v>
       </c>
-      <c r="AK6" s="2" t="n">
+      <c r="AM6" s="2" t="n">
         <v>3.64</v>
       </c>
-      <c r="AL6" s="2" t="n">
+      <c r="AN6" s="2" t="n">
         <v>8.5</v>
       </c>
-      <c r="AM6" s="2" t="n">
+      <c r="AO6" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="AN6" s="2" t="inlineStr"/>
-      <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr"/>
       <c r="AQ6" s="2" t="inlineStr"/>
-      <c r="AR6" s="2" t="inlineStr">
+      <c r="AR6" s="2" t="inlineStr"/>
+      <c r="AS6" s="2" t="inlineStr"/>
+      <c r="AT6" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS6" s="2" t="n">
+      <c r="AU6" s="2" t="n">
         <v>2.897</v>
       </c>
-      <c r="AT6" s="2" t="n">
+      <c r="AV6" s="2" t="n">
         <v>2.91</v>
       </c>
-      <c r="AU6" s="2" t="n">
+      <c r="AW6" s="2" t="n">
         <v>2.945</v>
       </c>
-      <c r="AV6" s="2" t="n">
+      <c r="AX6" s="2" t="n">
         <v>2.974</v>
       </c>
-      <c r="AW6" s="2" t="n">
+      <c r="AY6" s="2" t="n">
         <v>2.993</v>
       </c>
-      <c r="AX6" s="2" t="n">
+      <c r="AZ6" s="2" t="n">
         <v>3.005</v>
       </c>
-      <c r="AY6" s="2" t="n">
+      <c r="BA6" s="2" t="n">
         <v>3.037</v>
       </c>
-      <c r="AZ6" s="2" t="n">
+      <c r="BB6" s="2" t="n">
         <v>-0.8248</v>
       </c>
-      <c r="BA6" s="2" t="n">
+      <c r="BC6" s="2" t="n">
         <v>-0.5478</v>
       </c>
-      <c r="BB6" s="2" t="n">
+      <c r="BD6" s="2" t="n">
         <v>-0.2399</v>
       </c>
-      <c r="BC6" s="2" t="n">
+      <c r="BE6" s="2" t="n">
         <v>-0.1192</v>
       </c>
-      <c r="BD6" s="2" t="n">
+      <c r="BF6" s="2" t="n">
         <v>-0.0664</v>
       </c>
     </row>
@@ -1591,7 +1609,7 @@
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W7" s="2" t="n">
@@ -1603,85 +1621,83 @@
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr"/>
-      <c r="Z7" s="2" t="inlineStr">
-        <is>
-          <t>1→4·1d</t>
-        </is>
-      </c>
+      <c r="Z7" s="2" t="inlineStr"/>
       <c r="AA7" s="2" t="inlineStr"/>
       <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr">
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
-      <c r="AH7" s="2" t="n">
+      <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="n">
         <v>-7.54</v>
       </c>
-      <c r="AI7" s="2" t="n">
+      <c r="AK7" s="2" t="n">
         <v>1.09</v>
       </c>
-      <c r="AJ7" s="2" t="n">
+      <c r="AL7" s="2" t="n">
         <v>-0.05</v>
       </c>
-      <c r="AK7" s="2" t="n">
+      <c r="AM7" s="2" t="n">
         <v>-0.11</v>
       </c>
-      <c r="AL7" s="2" t="n">
+      <c r="AN7" s="2" t="n">
         <v>-4.4</v>
       </c>
-      <c r="AM7" s="2" t="n">
+      <c r="AO7" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AN7" s="2" t="inlineStr"/>
-      <c r="AO7" s="2" t="n">
+      <c r="AP7" s="2" t="inlineStr"/>
+      <c r="AQ7" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="AP7" s="2" t="inlineStr"/>
-      <c r="AQ7" s="2" t="inlineStr"/>
-      <c r="AR7" s="2" t="inlineStr">
+      <c r="AR7" s="2" t="inlineStr"/>
+      <c r="AS7" s="2" t="inlineStr"/>
+      <c r="AT7" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AS7" s="2" t="n">
+      <c r="AU7" s="2" t="n">
         <v>4.296</v>
       </c>
-      <c r="AT7" s="2" t="n">
+      <c r="AV7" s="2" t="n">
         <v>4.352</v>
       </c>
-      <c r="AU7" s="2" t="n">
+      <c r="AW7" s="2" t="n">
         <v>4.458</v>
       </c>
-      <c r="AV7" s="2" t="n">
+      <c r="AX7" s="2" t="n">
         <v>4.52</v>
       </c>
-      <c r="AW7" s="2" t="n">
+      <c r="AY7" s="2" t="n">
         <v>4.59</v>
       </c>
-      <c r="AX7" s="2" t="n">
+      <c r="AZ7" s="2" t="n">
         <v>4.721</v>
       </c>
-      <c r="AY7" s="2" t="n">
+      <c r="BA7" s="2" t="n">
         <v>4.71</v>
       </c>
-      <c r="AZ7" s="2" t="n">
+      <c r="BB7" s="2" t="n">
         <v>-1.6553</v>
       </c>
-      <c r="BA7" s="2" t="n">
+      <c r="BC7" s="2" t="n">
         <v>-0.9454</v>
       </c>
-      <c r="BB7" s="2" t="n">
+      <c r="BD7" s="2" t="n">
         <v>-0.4195</v>
       </c>
-      <c r="BC7" s="2" t="n">
+      <c r="BE7" s="2" t="n">
         <v>-0.3212</v>
       </c>
-      <c r="BD7" s="2" t="n">
+      <c r="BF7" s="2" t="n">
         <v>-0.07539999999999999</v>
       </c>
     </row>
@@ -1747,7 +1763,7 @@
         </is>
       </c>
       <c r="W8" s="2" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
@@ -1755,11 +1771,7 @@
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr"/>
-      <c r="Z8" s="2" t="inlineStr">
-        <is>
-          <t>1→4·6d</t>
-        </is>
-      </c>
+      <c r="Z8" s="2" t="inlineStr"/>
       <c r="AA8" s="2" t="inlineStr"/>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr"/>
@@ -1767,69 +1779,71 @@
       <c r="AE8" s="2" t="inlineStr"/>
       <c r="AF8" s="2" t="inlineStr"/>
       <c r="AG8" s="2" t="inlineStr"/>
-      <c r="AH8" s="2" t="n">
+      <c r="AH8" s="2" t="inlineStr"/>
+      <c r="AI8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="n">
         <v>-1.4</v>
       </c>
-      <c r="AI8" s="2" t="n">
+      <c r="AK8" s="2" t="n">
         <v>-2.66</v>
       </c>
-      <c r="AJ8" s="2" t="n">
+      <c r="AL8" s="2" t="n">
         <v>-3.32</v>
       </c>
-      <c r="AK8" s="2" t="n">
+      <c r="AM8" s="2" t="n">
         <v>-4.83</v>
       </c>
-      <c r="AL8" s="2" t="n">
+      <c r="AN8" s="2" t="n">
         <v>1.8</v>
       </c>
-      <c r="AM8" s="2" t="n">
+      <c r="AO8" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AN8" s="2" t="inlineStr"/>
-      <c r="AO8" s="2" t="n">
+      <c r="AP8" s="2" t="inlineStr"/>
+      <c r="AQ8" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="AP8" s="2" t="inlineStr"/>
-      <c r="AQ8" s="2" t="inlineStr"/>
-      <c r="AR8" s="2" t="inlineStr">
+      <c r="AR8" s="2" t="inlineStr"/>
+      <c r="AS8" s="2" t="inlineStr"/>
+      <c r="AT8" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AS8" s="2" t="n">
+      <c r="AU8" s="2" t="n">
         <v>6.973</v>
       </c>
-      <c r="AT8" s="2" t="n">
+      <c r="AV8" s="2" t="n">
         <v>7.181</v>
       </c>
-      <c r="AU8" s="2" t="n">
+      <c r="AW8" s="2" t="n">
         <v>7.451</v>
       </c>
-      <c r="AV8" s="2" t="n">
+      <c r="AX8" s="2" t="n">
         <v>7.569</v>
       </c>
-      <c r="AW8" s="2" t="n">
+      <c r="AY8" s="2" t="n">
         <v>7.688</v>
       </c>
-      <c r="AX8" s="2" t="n">
+      <c r="AZ8" s="2" t="n">
         <v>7.986</v>
       </c>
-      <c r="AY8" s="2" t="n">
+      <c r="BA8" s="2" t="n">
         <v>8.012</v>
       </c>
-      <c r="AZ8" s="2" t="n">
+      <c r="BB8" s="2" t="n">
         <v>-2.8417</v>
       </c>
-      <c r="BA8" s="2" t="n">
+      <c r="BC8" s="2" t="n">
         <v>-1.3238</v>
       </c>
-      <c r="BB8" s="2" t="n">
+      <c r="BD8" s="2" t="n">
         <v>-0.368</v>
       </c>
-      <c r="BC8" s="2" t="n">
+      <c r="BE8" s="2" t="n">
         <v>-0.5048</v>
       </c>
-      <c r="BD8" s="2" t="n">
+      <c r="BF8" s="2" t="n">
         <v>-0.014</v>
       </c>
     </row>
@@ -1887,7 +1901,7 @@
         </is>
       </c>
       <c r="W9" s="2" t="n">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
@@ -1901,81 +1915,83 @@
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·1d ← 3→2A·12d ← 2B→3·14d</t>
+          <t>2A→2C·17d</t>
         </is>
       </c>
       <c r="AA9" s="2" t="inlineStr"/>
       <c r="AB9" s="2" t="inlineStr"/>
-      <c r="AC9" s="2" t="n">
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AE9" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD9" s="2" t="inlineStr"/>
-      <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
-      <c r="AH9" s="2" t="n">
+      <c r="AH9" s="2" t="inlineStr"/>
+      <c r="AI9" s="2" t="inlineStr"/>
+      <c r="AJ9" s="2" t="n">
         <v>17.27</v>
       </c>
-      <c r="AI9" s="2" t="n">
+      <c r="AK9" s="2" t="n">
         <v>19.59</v>
       </c>
-      <c r="AJ9" s="2" t="n">
+      <c r="AL9" s="2" t="n">
         <v>3.48</v>
       </c>
-      <c r="AK9" s="2" t="n">
+      <c r="AM9" s="2" t="n">
         <v>7.2</v>
       </c>
-      <c r="AL9" s="2" t="n">
+      <c r="AN9" s="2" t="n">
         <v>85.59999999999999</v>
       </c>
-      <c r="AM9" s="2" t="n">
+      <c r="AO9" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="AN9" s="2" t="inlineStr"/>
-      <c r="AO9" s="2" t="inlineStr"/>
-      <c r="AP9" s="2" t="n">
+      <c r="AP9" s="2" t="inlineStr"/>
+      <c r="AQ9" s="2" t="inlineStr"/>
+      <c r="AR9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AQ9" s="2" t="inlineStr"/>
-      <c r="AR9" s="2" t="inlineStr">
+      <c r="AS9" s="2" t="inlineStr"/>
+      <c r="AT9" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS9" s="2" t="n">
+      <c r="AU9" s="2" t="n">
         <v>3.451</v>
       </c>
-      <c r="AT9" s="2" t="n">
+      <c r="AV9" s="2" t="n">
         <v>3.414</v>
       </c>
-      <c r="AU9" s="2" t="n">
+      <c r="AW9" s="2" t="n">
         <v>3.393</v>
       </c>
-      <c r="AV9" s="2" t="n">
+      <c r="AX9" s="2" t="n">
         <v>3.413</v>
       </c>
-      <c r="AW9" s="2" t="n">
+      <c r="AY9" s="2" t="n">
         <v>3.381</v>
       </c>
-      <c r="AX9" s="2" t="n">
+      <c r="AZ9" s="2" t="n">
         <v>3.273</v>
       </c>
-      <c r="AY9" s="2" t="n">
+      <c r="BA9" s="2" t="n">
         <v>3.23</v>
       </c>
-      <c r="AZ9" s="2" t="n">
+      <c r="BB9" s="2" t="n">
         <v>0.6859</v>
       </c>
-      <c r="BA9" s="2" t="n">
+      <c r="BC9" s="2" t="n">
         <v>0.008</v>
       </c>
-      <c r="BB9" s="2" t="n">
+      <c r="BD9" s="2" t="n">
         <v>0.3042</v>
       </c>
-      <c r="BC9" s="2" t="n">
+      <c r="BE9" s="2" t="n">
         <v>0.1843</v>
       </c>
-      <c r="BD9" s="2" t="n">
+      <c r="BF9" s="2" t="n">
         <v>0.1727</v>
       </c>
     </row>
@@ -2035,7 +2051,7 @@
         </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>6</v>
+        <v>69</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
@@ -2045,85 +2061,87 @@
       <c r="Y10" s="2" t="inlineStr"/>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>1→4·6d</t>
+          <t>4+→4·10d ← 4→4+·20d</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE10" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AG10" s="2" t="inlineStr"/>
+      <c r="AG10" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AH10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI10" s="2" t="inlineStr"/>
+      <c r="AJ10" s="2" t="n">
         <v>-19.08</v>
       </c>
-      <c r="AI10" s="2" t="n">
+      <c r="AK10" s="2" t="n">
         <v>1.73</v>
       </c>
-      <c r="AJ10" s="2" t="n">
+      <c r="AL10" s="2" t="n">
         <v>3.26</v>
       </c>
-      <c r="AK10" s="2" t="n">
+      <c r="AM10" s="2" t="n">
         <v>4.5</v>
       </c>
-      <c r="AL10" s="2" t="n">
+      <c r="AN10" s="2" t="n">
         <v>8.6</v>
       </c>
-      <c r="AM10" s="2" t="n">
+      <c r="AO10" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AN10" s="2" t="inlineStr"/>
-      <c r="AO10" s="2" t="n">
+      <c r="AP10" s="2" t="inlineStr"/>
+      <c r="AQ10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP10" s="2" t="inlineStr"/>
-      <c r="AQ10" s="2" t="inlineStr"/>
-      <c r="AR10" s="2" t="inlineStr">
+      <c r="AR10" s="2" t="inlineStr"/>
+      <c r="AS10" s="2" t="inlineStr"/>
+      <c r="AT10" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS10" s="2" t="n">
+      <c r="AU10" s="2" t="n">
         <v>0.495</v>
       </c>
-      <c r="AT10" s="2" t="n">
+      <c r="AV10" s="2" t="n">
         <v>0.493</v>
       </c>
-      <c r="AU10" s="2" t="n">
+      <c r="AW10" s="2" t="n">
         <v>0.499</v>
       </c>
-      <c r="AV10" s="2" t="n">
+      <c r="AX10" s="2" t="n">
         <v>0.507</v>
       </c>
-      <c r="AW10" s="2" t="n">
+      <c r="AY10" s="2" t="n">
         <v>0.513</v>
       </c>
-      <c r="AX10" s="2" t="n">
+      <c r="AZ10" s="2" t="n">
         <v>0.516</v>
       </c>
-      <c r="AY10" s="2" t="n">
+      <c r="BA10" s="2" t="n">
         <v>0.53</v>
       </c>
-      <c r="AZ10" s="2" t="n">
+      <c r="BB10" s="2" t="n">
         <v>-0.6566</v>
       </c>
-      <c r="BA10" s="2" t="n">
+      <c r="BC10" s="2" t="n">
         <v>-0.6994</v>
       </c>
-      <c r="BB10" s="2" t="n">
+      <c r="BD10" s="2" t="n">
         <v>-0.3166</v>
       </c>
-      <c r="BC10" s="2" t="n">
+      <c r="BE10" s="2" t="n">
         <v>-0.0453</v>
       </c>
-      <c r="BD10" s="2" t="n">
+      <c r="BF10" s="2" t="n">
         <v>-0.1908</v>
       </c>
     </row>
@@ -2177,97 +2195,103 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W11" s="2" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Y11" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>1+→1·7d ← 1→1+·8d ← 1+→1·11d</t>
+          <t>4→4+·1d ← 1→4·4d ← 1+→1·7d</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr"/>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
-      <c r="AD11" s="2" t="n">
+      <c r="AD11" s="2" t="inlineStr"/>
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AE11" s="2" t="inlineStr">
+      <c r="AG11" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AF11" s="2" t="inlineStr"/>
-      <c r="AG11" s="2" t="inlineStr"/>
-      <c r="AH11" s="2" t="n">
+      <c r="AH11" s="2" t="inlineStr"/>
+      <c r="AI11" s="2" t="inlineStr"/>
+      <c r="AJ11" s="2" t="n">
         <v>-5.29</v>
       </c>
-      <c r="AI11" s="2" t="n">
+      <c r="AK11" s="2" t="n">
         <v>8.25</v>
       </c>
-      <c r="AJ11" s="2" t="n">
+      <c r="AL11" s="2" t="n">
         <v>0.17</v>
       </c>
-      <c r="AK11" s="2" t="n">
+      <c r="AM11" s="2" t="n">
         <v>9.609999999999999</v>
       </c>
-      <c r="AL11" s="2" t="n">
+      <c r="AN11" s="2" t="n">
         <v>58.5</v>
       </c>
-      <c r="AM11" s="2" t="n">
+      <c r="AO11" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="AN11" s="2" t="inlineStr"/>
-      <c r="AO11" s="2" t="inlineStr"/>
       <c r="AP11" s="2" t="inlineStr"/>
       <c r="AQ11" s="2" t="inlineStr"/>
-      <c r="AR11" s="2" t="inlineStr">
+      <c r="AR11" s="2" t="inlineStr"/>
+      <c r="AS11" s="2" t="inlineStr"/>
+      <c r="AT11" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS11" s="2" t="n">
+      <c r="AU11" s="2" t="n">
         <v>0.375</v>
       </c>
-      <c r="AT11" s="2" t="n">
+      <c r="AV11" s="2" t="n">
         <v>0.378</v>
       </c>
-      <c r="AU11" s="2" t="n">
+      <c r="AW11" s="2" t="n">
         <v>0.376</v>
       </c>
-      <c r="AV11" s="2" t="n">
+      <c r="AX11" s="2" t="n">
         <v>0.377</v>
       </c>
-      <c r="AW11" s="2" t="n">
+      <c r="AY11" s="2" t="n">
         <v>0.382</v>
       </c>
-      <c r="AX11" s="2" t="n">
+      <c r="AZ11" s="2" t="n">
         <v>0.366</v>
       </c>
-      <c r="AY11" s="2" t="n">
+      <c r="BA11" s="2" t="n">
         <v>0.371</v>
       </c>
-      <c r="AZ11" s="2" t="n">
+      <c r="BB11" s="2" t="n">
         <v>-0.4024</v>
       </c>
-      <c r="BA11" s="2" t="n">
+      <c r="BC11" s="2" t="n">
         <v>-0.0495</v>
       </c>
-      <c r="BB11" s="2" t="n">
+      <c r="BD11" s="2" t="n">
         <v>0.0677</v>
       </c>
-      <c r="BC11" s="2" t="n">
+      <c r="BE11" s="2" t="n">
         <v>0.1593</v>
       </c>
-      <c r="BD11" s="2" t="n">
+      <c r="BF11" s="2" t="n">
         <v>-0.0529</v>
       </c>
     </row>
@@ -2327,7 +2351,7 @@
         </is>
       </c>
       <c r="W12" s="2" t="n">
-        <v>10</v>
+        <v>146</v>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
@@ -2337,81 +2361,83 @@
       <c r="Y12" s="2" t="inlineStr"/>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>4+→4·7d ← 1→4+·10d</t>
+          <t>4+→4·7d ← 4→4+·10d</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr"/>
       <c r="AB12" s="2" t="inlineStr"/>
-      <c r="AC12" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AG12" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF12" s="2" t="inlineStr"/>
-      <c r="AG12" s="2" t="inlineStr"/>
-      <c r="AH12" s="2" t="n">
+      <c r="AH12" s="2" t="inlineStr"/>
+      <c r="AI12" s="2" t="inlineStr"/>
+      <c r="AJ12" s="2" t="n">
         <v>-21.3</v>
       </c>
-      <c r="AI12" s="2" t="n">
+      <c r="AK12" s="2" t="n">
         <v>0.93</v>
       </c>
-      <c r="AJ12" s="2" t="n">
+      <c r="AL12" s="2" t="n">
         <v>2.22</v>
       </c>
-      <c r="AK12" s="2" t="n">
+      <c r="AM12" s="2" t="n">
         <v>2.79</v>
       </c>
-      <c r="AL12" s="2" t="n">
+      <c r="AN12" s="2" t="n">
         <v>13.1</v>
       </c>
-      <c r="AM12" s="2" t="n">
+      <c r="AO12" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="AN12" s="2" t="inlineStr"/>
-      <c r="AO12" s="2" t="inlineStr"/>
       <c r="AP12" s="2" t="inlineStr"/>
       <c r="AQ12" s="2" t="inlineStr"/>
-      <c r="AR12" s="2" t="inlineStr">
+      <c r="AR12" s="2" t="inlineStr"/>
+      <c r="AS12" s="2" t="inlineStr"/>
+      <c r="AT12" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS12" s="2" t="n">
+      <c r="AU12" s="2" t="n">
         <v>0.758</v>
       </c>
-      <c r="AT12" s="2" t="n">
+      <c r="AV12" s="2" t="n">
         <v>0.759</v>
       </c>
-      <c r="AU12" s="2" t="n">
+      <c r="AW12" s="2" t="n">
         <v>0.77</v>
       </c>
-      <c r="AV12" s="2" t="n">
+      <c r="AX12" s="2" t="n">
         <v>0.783</v>
       </c>
-      <c r="AW12" s="2" t="n">
+      <c r="AY12" s="2" t="n">
         <v>0.787</v>
       </c>
-      <c r="AX12" s="2" t="n">
+      <c r="AZ12" s="2" t="n">
         <v>0.786</v>
       </c>
-      <c r="AY12" s="2" t="n">
+      <c r="BA12" s="2" t="n">
         <v>0.823</v>
       </c>
-      <c r="AZ12" s="2" t="n">
+      <c r="BB12" s="2" t="n">
         <v>-0.8631</v>
       </c>
-      <c r="BA12" s="2" t="n">
+      <c r="BC12" s="2" t="n">
         <v>-0.8290999999999999</v>
       </c>
-      <c r="BB12" s="2" t="n">
+      <c r="BD12" s="2" t="n">
         <v>-0.3277</v>
       </c>
-      <c r="BC12" s="2" t="n">
+      <c r="BE12" s="2" t="n">
         <v>-0.0526</v>
       </c>
-      <c r="BD12" s="2" t="n">
+      <c r="BF12" s="2" t="n">
         <v>-0.213</v>
       </c>
     </row>
@@ -2477,7 +2503,7 @@
         </is>
       </c>
       <c r="W13" s="2" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
@@ -2485,11 +2511,7 @@
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr"/>
-      <c r="Z13" s="2" t="inlineStr">
-        <is>
-          <t>1→4·16d</t>
-        </is>
-      </c>
+      <c r="Z13" s="2" t="inlineStr"/>
       <c r="AA13" s="2" t="inlineStr"/>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
@@ -2497,67 +2519,69 @@
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="inlineStr"/>
-      <c r="AH13" s="2" t="n">
+      <c r="AH13" s="2" t="inlineStr"/>
+      <c r="AI13" s="2" t="inlineStr"/>
+      <c r="AJ13" s="2" t="n">
         <v>-6.34</v>
       </c>
-      <c r="AI13" s="2" t="n">
+      <c r="AK13" s="2" t="n">
         <v>-3.74</v>
       </c>
-      <c r="AJ13" s="2" t="n">
+      <c r="AL13" s="2" t="n">
         <v>-3.25</v>
       </c>
-      <c r="AK13" s="2" t="n">
+      <c r="AM13" s="2" t="n">
         <v>-4.04</v>
       </c>
-      <c r="AL13" s="2" t="n">
+      <c r="AN13" s="2" t="n">
         <v>14.4</v>
       </c>
-      <c r="AM13" s="2" t="n">
+      <c r="AO13" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AN13" s="2" t="inlineStr"/>
-      <c r="AO13" s="2" t="inlineStr"/>
       <c r="AP13" s="2" t="inlineStr"/>
       <c r="AQ13" s="2" t="inlineStr"/>
-      <c r="AR13" s="2" t="inlineStr">
+      <c r="AR13" s="2" t="inlineStr"/>
+      <c r="AS13" s="2" t="inlineStr"/>
+      <c r="AT13" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS13" s="2" t="n">
+      <c r="AU13" s="2" t="n">
         <v>2.789</v>
       </c>
-      <c r="AT13" s="2" t="n">
+      <c r="AV13" s="2" t="n">
         <v>2.868</v>
       </c>
-      <c r="AU13" s="2" t="n">
+      <c r="AW13" s="2" t="n">
         <v>2.977</v>
       </c>
-      <c r="AV13" s="2" t="n">
+      <c r="AX13" s="2" t="n">
         <v>3.018</v>
       </c>
-      <c r="AW13" s="2" t="n">
+      <c r="AY13" s="2" t="n">
         <v>3.04</v>
       </c>
-      <c r="AX13" s="2" t="n">
+      <c r="AZ13" s="2" t="n">
         <v>3.171</v>
       </c>
-      <c r="AY13" s="2" t="n">
+      <c r="BA13" s="2" t="n">
         <v>3.212</v>
       </c>
-      <c r="AZ13" s="2" t="n">
+      <c r="BB13" s="2" t="n">
         <v>-2.9216</v>
       </c>
-      <c r="BA13" s="2" t="n">
+      <c r="BC13" s="2" t="n">
         <v>-1.2647</v>
       </c>
-      <c r="BB13" s="2" t="n">
+      <c r="BD13" s="2" t="n">
         <v>-0.1163</v>
       </c>
-      <c r="BC13" s="2" t="n">
+      <c r="BE13" s="2" t="n">
         <v>-0.5944</v>
       </c>
-      <c r="BD13" s="2" t="n">
+      <c r="BF13" s="2" t="n">
         <v>-0.0634</v>
       </c>
     </row>
@@ -2611,97 +2635,103 @@
       </c>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W14" s="2" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Y14" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>1+→1·7d ← 1→1+·8d ← 1+→1·11d</t>
+          <t>4→4+·1d ← 4+→4·7d ← 4→4+·8d</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr"/>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
-      <c r="AD14" s="2" t="n">
+      <c r="AD14" s="2" t="inlineStr"/>
+      <c r="AE14" s="2" t="inlineStr"/>
+      <c r="AF14" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AE14" s="2" t="inlineStr">
+      <c r="AG14" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AF14" s="2" t="inlineStr"/>
-      <c r="AG14" s="2" t="inlineStr"/>
-      <c r="AH14" s="2" t="n">
+      <c r="AH14" s="2" t="inlineStr"/>
+      <c r="AI14" s="2" t="inlineStr"/>
+      <c r="AJ14" s="2" t="n">
         <v>-3.9</v>
       </c>
-      <c r="AI14" s="2" t="n">
+      <c r="AK14" s="2" t="n">
         <v>5.35</v>
       </c>
-      <c r="AJ14" s="2" t="n">
+      <c r="AL14" s="2" t="n">
         <v>-2.3</v>
       </c>
-      <c r="AK14" s="2" t="n">
+      <c r="AM14" s="2" t="n">
         <v>6.43</v>
       </c>
-      <c r="AL14" s="2" t="n">
+      <c r="AN14" s="2" t="n">
         <v>63.6</v>
       </c>
-      <c r="AM14" s="2" t="n">
+      <c r="AO14" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="AN14" s="2" t="inlineStr"/>
-      <c r="AO14" s="2" t="inlineStr"/>
       <c r="AP14" s="2" t="inlineStr"/>
       <c r="AQ14" s="2" t="inlineStr"/>
-      <c r="AR14" s="2" t="inlineStr">
+      <c r="AR14" s="2" t="inlineStr"/>
+      <c r="AS14" s="2" t="inlineStr"/>
+      <c r="AT14" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS14" s="2" t="n">
+      <c r="AU14" s="2" t="n">
         <v>0.332</v>
       </c>
-      <c r="AT14" s="2" t="n">
+      <c r="AV14" s="2" t="n">
         <v>0.337</v>
       </c>
-      <c r="AU14" s="2" t="n">
+      <c r="AW14" s="2" t="n">
         <v>0.338</v>
       </c>
-      <c r="AV14" s="2" t="n">
+      <c r="AX14" s="2" t="n">
         <v>0.338</v>
       </c>
-      <c r="AW14" s="2" t="n">
+      <c r="AY14" s="2" t="n">
         <v>0.341</v>
       </c>
-      <c r="AX14" s="2" t="n">
+      <c r="AZ14" s="2" t="n">
         <v>0.326</v>
       </c>
-      <c r="AY14" s="2" t="n">
+      <c r="BA14" s="2" t="n">
         <v>0.336</v>
       </c>
-      <c r="AZ14" s="2" t="n">
+      <c r="BB14" s="2" t="n">
         <v>-1.0291</v>
       </c>
-      <c r="BA14" s="2" t="n">
+      <c r="BC14" s="2" t="n">
         <v>-0.2211</v>
       </c>
-      <c r="BB14" s="2" t="n">
+      <c r="BD14" s="2" t="n">
         <v>0.1491</v>
       </c>
-      <c r="BC14" s="2" t="n">
+      <c r="BE14" s="2" t="n">
         <v>0.0548</v>
       </c>
-      <c r="BD14" s="2" t="n">
+      <c r="BF14" s="2" t="n">
         <v>-0.039</v>
       </c>
     </row>
@@ -2771,79 +2801,81 @@
       <c r="Y15" s="2" t="inlineStr"/>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>4+→4·10d ← 4→4+·15d</t>
+          <t>4+→4·12d ← 4→4+·15d</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="inlineStr"/>
-      <c r="AC15" s="2" t="n">
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr"/>
       <c r="AG15" s="2" t="inlineStr"/>
-      <c r="AH15" s="2" t="n">
+      <c r="AH15" s="2" t="inlineStr"/>
+      <c r="AI15" s="2" t="inlineStr"/>
+      <c r="AJ15" s="2" t="n">
         <v>-16.67</v>
       </c>
-      <c r="AI15" s="2" t="n">
+      <c r="AK15" s="2" t="n">
         <v>-7.19</v>
       </c>
-      <c r="AJ15" s="2" t="n">
+      <c r="AL15" s="2" t="n">
         <v>1.29</v>
       </c>
-      <c r="AK15" s="2" t="n">
+      <c r="AM15" s="2" t="n">
         <v>-1.6</v>
       </c>
-      <c r="AL15" s="2" t="n">
+      <c r="AN15" s="2" t="n">
         <v>21.6</v>
       </c>
-      <c r="AM15" s="2" t="n">
+      <c r="AO15" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="AN15" s="2" t="inlineStr"/>
-      <c r="AO15" s="2" t="inlineStr"/>
       <c r="AP15" s="2" t="inlineStr"/>
       <c r="AQ15" s="2" t="inlineStr"/>
-      <c r="AR15" s="2" t="inlineStr">
+      <c r="AR15" s="2" t="inlineStr"/>
+      <c r="AS15" s="2" t="inlineStr"/>
+      <c r="AT15" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS15" s="2" t="n">
+      <c r="AU15" s="2" t="n">
         <v>1.061</v>
       </c>
-      <c r="AT15" s="2" t="n">
+      <c r="AV15" s="2" t="n">
         <v>1.078</v>
       </c>
-      <c r="AU15" s="2" t="n">
+      <c r="AW15" s="2" t="n">
         <v>1.116</v>
       </c>
-      <c r="AV15" s="2" t="n">
+      <c r="AX15" s="2" t="n">
         <v>1.127</v>
       </c>
-      <c r="AW15" s="2" t="n">
+      <c r="AY15" s="2" t="n">
         <v>1.128</v>
       </c>
-      <c r="AX15" s="2" t="n">
+      <c r="AZ15" s="2" t="n">
         <v>1.178</v>
       </c>
-      <c r="AY15" s="2" t="n">
+      <c r="BA15" s="2" t="n">
         <v>1.297</v>
       </c>
-      <c r="AZ15" s="2" t="n">
+      <c r="BB15" s="2" t="n">
         <v>-2.2119</v>
       </c>
-      <c r="BA15" s="2" t="n">
+      <c r="BC15" s="2" t="n">
         <v>-1.1776</v>
       </c>
-      <c r="BB15" s="2" t="n">
+      <c r="BD15" s="2" t="n">
         <v>-0.1113</v>
       </c>
-      <c r="BC15" s="2" t="n">
+      <c r="BE15" s="2" t="n">
         <v>-0.707</v>
       </c>
-      <c r="BD15" s="2" t="n">
+      <c r="BF15" s="2" t="n">
         <v>-0.1667</v>
       </c>
     </row>
@@ -2905,7 +2937,7 @@
         </is>
       </c>
       <c r="W16" s="2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
@@ -2921,69 +2953,71 @@
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr"/>
       <c r="AG16" s="2" t="inlineStr"/>
-      <c r="AH16" s="2" t="n">
+      <c r="AH16" s="2" t="inlineStr"/>
+      <c r="AI16" s="2" t="inlineStr"/>
+      <c r="AJ16" s="2" t="n">
         <v>-15.15</v>
       </c>
-      <c r="AI16" s="2" t="n">
+      <c r="AK16" s="2" t="n">
         <v>-8.779999999999999</v>
       </c>
-      <c r="AJ16" s="2" t="n">
+      <c r="AL16" s="2" t="n">
         <v>-2.44</v>
       </c>
-      <c r="AK16" s="2" t="n">
+      <c r="AM16" s="2" t="n">
         <v>-1.95</v>
       </c>
-      <c r="AL16" s="2" t="n">
+      <c r="AN16" s="2" t="n">
         <v>-0.5</v>
       </c>
-      <c r="AM16" s="2" t="n">
+      <c r="AO16" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="AN16" s="2" t="inlineStr"/>
-      <c r="AO16" s="2" t="n">
+      <c r="AP16" s="2" t="inlineStr"/>
+      <c r="AQ16" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="AP16" s="2" t="inlineStr"/>
-      <c r="AQ16" s="2" t="inlineStr"/>
-      <c r="AR16" s="2" t="inlineStr">
+      <c r="AR16" s="2" t="inlineStr"/>
+      <c r="AS16" s="2" t="inlineStr"/>
+      <c r="AT16" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AS16" s="2" t="n">
+      <c r="AU16" s="2" t="n">
         <v>1.029</v>
       </c>
-      <c r="AT16" s="2" t="n">
+      <c r="AV16" s="2" t="n">
         <v>1.054</v>
       </c>
-      <c r="AU16" s="2" t="n">
+      <c r="AW16" s="2" t="n">
         <v>1.09</v>
       </c>
-      <c r="AV16" s="2" t="n">
+      <c r="AX16" s="2" t="n">
         <v>1.115</v>
       </c>
-      <c r="AW16" s="2" t="n">
+      <c r="AY16" s="2" t="n">
         <v>1.148</v>
       </c>
-      <c r="AX16" s="2" t="n">
+      <c r="AZ16" s="2" t="n">
         <v>1.184</v>
       </c>
-      <c r="AY16" s="2" t="n">
+      <c r="BA16" s="2" t="n">
         <v>1.228</v>
       </c>
-      <c r="AZ16" s="2" t="n">
+      <c r="BB16" s="2" t="n">
         <v>-2.5727</v>
       </c>
-      <c r="BA16" s="2" t="n">
+      <c r="BC16" s="2" t="n">
         <v>-1.3651</v>
       </c>
-      <c r="BB16" s="2" t="n">
+      <c r="BD16" s="2" t="n">
         <v>-0.5793</v>
       </c>
-      <c r="BC16" s="2" t="n">
+      <c r="BE16" s="2" t="n">
         <v>-0.6806</v>
       </c>
-      <c r="BD16" s="2" t="n">
+      <c r="BF16" s="2" t="n">
         <v>-0.1515</v>
       </c>
     </row>
@@ -3039,19 +3073,23 @@
       </c>
       <c r="V17" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W17" s="2" t="n">
-        <v>21</v>
+        <v>299</v>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr"/>
-      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2C→2A·4d</t>
+        </is>
+      </c>
       <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
@@ -3059,67 +3097,69 @@
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="inlineStr"/>
       <c r="AG17" s="2" t="inlineStr"/>
-      <c r="AH17" s="2" t="n">
+      <c r="AH17" s="2" t="inlineStr"/>
+      <c r="AI17" s="2" t="inlineStr"/>
+      <c r="AJ17" s="2" t="n">
         <v>16.51</v>
       </c>
-      <c r="AI17" s="2" t="n">
+      <c r="AK17" s="2" t="n">
         <v>1.71</v>
       </c>
-      <c r="AJ17" s="2" t="n">
+      <c r="AL17" s="2" t="n">
         <v>-5.38</v>
       </c>
-      <c r="AK17" s="2" t="n">
+      <c r="AM17" s="2" t="n">
         <v>-9.06</v>
       </c>
-      <c r="AL17" s="2" t="n">
+      <c r="AN17" s="2" t="n">
         <v>-7.2</v>
       </c>
-      <c r="AM17" s="2" t="n">
+      <c r="AO17" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AN17" s="2" t="inlineStr"/>
-      <c r="AO17" s="2" t="inlineStr"/>
       <c r="AP17" s="2" t="inlineStr"/>
       <c r="AQ17" s="2" t="inlineStr"/>
-      <c r="AR17" s="2" t="inlineStr">
+      <c r="AR17" s="2" t="inlineStr"/>
+      <c r="AS17" s="2" t="inlineStr"/>
+      <c r="AT17" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS17" s="2" t="n">
+      <c r="AU17" s="2" t="n">
         <v>0.92</v>
       </c>
-      <c r="AT17" s="2" t="n">
+      <c r="AV17" s="2" t="n">
         <v>0.963</v>
       </c>
-      <c r="AU17" s="2" t="n">
+      <c r="AW17" s="2" t="n">
         <v>1.016</v>
       </c>
-      <c r="AV17" s="2" t="n">
+      <c r="AX17" s="2" t="n">
         <v>1.033</v>
       </c>
-      <c r="AW17" s="2" t="n">
+      <c r="AY17" s="2" t="n">
         <v>1.066</v>
       </c>
-      <c r="AX17" s="2" t="n">
+      <c r="AZ17" s="2" t="n">
         <v>1.167</v>
       </c>
-      <c r="AY17" s="2" t="n">
+      <c r="BA17" s="2" t="n">
         <v>1.03</v>
       </c>
-      <c r="AZ17" s="2" t="n">
+      <c r="BB17" s="2" t="n">
         <v>-4.4706</v>
       </c>
-      <c r="BA17" s="2" t="n">
+      <c r="BC17" s="2" t="n">
         <v>-1.554</v>
       </c>
-      <c r="BB17" s="2" t="n">
+      <c r="BD17" s="2" t="n">
         <v>-1.0542</v>
       </c>
-      <c r="BC17" s="2" t="n">
+      <c r="BE17" s="2" t="n">
         <v>-0.4634</v>
       </c>
-      <c r="BD17" s="2" t="n">
+      <c r="BF17" s="2" t="n">
         <v>0.1651</v>
       </c>
     </row>
@@ -3177,93 +3217,99 @@
         </is>
       </c>
       <c r="W18" s="2" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>2A</t>
-        </is>
-      </c>
-      <c r="Y18" s="2" t="inlineStr"/>
+          <t>2C</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>减速</t>
+        </is>
+      </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>2B→2A·7d</t>
+          <t>2A→2C·13d</t>
         </is>
       </c>
       <c r="AA18" s="2" t="inlineStr"/>
       <c r="AB18" s="2" t="inlineStr"/>
-      <c r="AC18" s="2" t="inlineStr">
+      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AD18" s="2" t="inlineStr"/>
+      <c r="AE18" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr"/>
       <c r="AG18" s="2" t="inlineStr"/>
-      <c r="AH18" s="2" t="n">
+      <c r="AH18" s="2" t="inlineStr"/>
+      <c r="AI18" s="2" t="inlineStr"/>
+      <c r="AJ18" s="2" t="n">
         <v>7.85</v>
       </c>
-      <c r="AI18" s="2" t="n">
+      <c r="AK18" s="2" t="n">
         <v>19.84</v>
       </c>
-      <c r="AJ18" s="2" t="n">
+      <c r="AL18" s="2" t="n">
         <v>5.55</v>
       </c>
-      <c r="AK18" s="2" t="n">
+      <c r="AM18" s="2" t="n">
         <v>10.78</v>
       </c>
-      <c r="AL18" s="2" t="n">
+      <c r="AN18" s="2" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="AM18" s="2" t="n">
+      <c r="AO18" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="AN18" s="2" t="inlineStr"/>
-      <c r="AO18" s="2" t="inlineStr"/>
-      <c r="AP18" s="2" t="n">
+      <c r="AP18" s="2" t="inlineStr"/>
+      <c r="AQ18" s="2" t="inlineStr"/>
+      <c r="AR18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AQ18" s="2" t="inlineStr"/>
-      <c r="AR18" s="2" t="inlineStr">
+      <c r="AS18" s="2" t="inlineStr"/>
+      <c r="AT18" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS18" s="2" t="n">
+      <c r="AU18" s="2" t="n">
         <v>0.865</v>
       </c>
-      <c r="AT18" s="2" t="n">
+      <c r="AV18" s="2" t="n">
         <v>0.856</v>
       </c>
-      <c r="AU18" s="2" t="n">
+      <c r="AW18" s="2" t="n">
         <v>0.848</v>
       </c>
-      <c r="AV18" s="2" t="n">
+      <c r="AX18" s="2" t="n">
         <v>0.845</v>
       </c>
-      <c r="AW18" s="2" t="n">
+      <c r="AY18" s="2" t="n">
         <v>0.832</v>
       </c>
-      <c r="AX18" s="2" t="n">
+      <c r="AZ18" s="2" t="n">
         <v>0.806</v>
       </c>
-      <c r="AY18" s="2" t="n">
+      <c r="BA18" s="2" t="n">
         <v>0.8</v>
       </c>
-      <c r="AZ18" s="2" t="n">
+      <c r="BB18" s="2" t="n">
         <v>0.8586</v>
       </c>
-      <c r="BA18" s="2" t="n">
+      <c r="BC18" s="2" t="n">
         <v>0.3302</v>
       </c>
-      <c r="BB18" s="2" t="n">
+      <c r="BD18" s="2" t="n">
         <v>0.2995</v>
       </c>
-      <c r="BC18" s="2" t="n">
+      <c r="BE18" s="2" t="n">
         <v>0.2902</v>
       </c>
-      <c r="BD18" s="2" t="n">
+      <c r="BF18" s="2" t="n">
         <v>0.0785</v>
       </c>
     </row>
@@ -3323,7 +3369,7 @@
         </is>
       </c>
       <c r="W19" s="2" t="n">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
@@ -3345,71 +3391,73 @@
       <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr"/>
-      <c r="AF19" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AF19" s="2" t="inlineStr"/>
       <c r="AG19" s="2" t="inlineStr"/>
       <c r="AH19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="2" t="inlineStr"/>
+      <c r="AJ19" s="2" t="n">
         <v>-54.22</v>
       </c>
-      <c r="AI19" s="2" t="n">
+      <c r="AK19" s="2" t="n">
         <v>-12.4</v>
       </c>
-      <c r="AJ19" s="2" t="n">
+      <c r="AL19" s="2" t="n">
         <v>4.52</v>
       </c>
-      <c r="AK19" s="2" t="n">
+      <c r="AM19" s="2" t="n">
         <v>10.15</v>
       </c>
-      <c r="AL19" s="2" t="n">
+      <c r="AN19" s="2" t="n">
         <v>24.5</v>
       </c>
-      <c r="AM19" s="2" t="n">
+      <c r="AO19" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="AN19" s="2" t="inlineStr"/>
-      <c r="AO19" s="2" t="inlineStr"/>
       <c r="AP19" s="2" t="inlineStr"/>
       <c r="AQ19" s="2" t="inlineStr"/>
-      <c r="AR19" s="2" t="inlineStr">
+      <c r="AR19" s="2" t="inlineStr"/>
+      <c r="AS19" s="2" t="inlineStr"/>
+      <c r="AT19" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS19" s="2" t="n">
+      <c r="AU19" s="2" t="n">
         <v>1.01</v>
       </c>
-      <c r="AT19" s="2" t="n">
+      <c r="AV19" s="2" t="n">
         <v>1.006</v>
       </c>
-      <c r="AU19" s="2" t="n">
+      <c r="AW19" s="2" t="n">
         <v>1.014</v>
       </c>
-      <c r="AV19" s="2" t="n">
+      <c r="AX19" s="2" t="n">
         <v>1.026</v>
       </c>
-      <c r="AW19" s="2" t="n">
+      <c r="AY19" s="2" t="n">
         <v>1.067</v>
       </c>
-      <c r="AX19" s="2" t="n">
+      <c r="AZ19" s="2" t="n">
         <v>1.074</v>
       </c>
-      <c r="AY19" s="2" t="n">
+      <c r="BA19" s="2" t="n">
         <v>1.207</v>
       </c>
-      <c r="AZ19" s="2" t="n">
+      <c r="BB19" s="2" t="n">
         <v>-0.5168</v>
       </c>
-      <c r="BA19" s="2" t="n">
+      <c r="BC19" s="2" t="n">
         <v>-0.3515</v>
       </c>
-      <c r="BB19" s="2" t="n">
+      <c r="BD19" s="2" t="n">
         <v>-0.4588</v>
       </c>
-      <c r="BC19" s="2" t="n">
+      <c r="BE19" s="2" t="n">
         <v>-0.444</v>
       </c>
-      <c r="BD19" s="2" t="n">
+      <c r="BF19" s="2" t="n">
         <v>-0.5422</v>
       </c>
     </row>
@@ -3467,7 +3515,7 @@
         </is>
       </c>
       <c r="W20" s="2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
@@ -3477,81 +3525,83 @@
       <c r="Y20" s="2" t="inlineStr"/>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>4+→4·7d ← 1→4+·10d</t>
+          <t>4+→4·7d ← 4→4+·10d ← 2A→4·20d</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr"/>
       <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AC20" s="2" t="inlineStr"/>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF20" s="2" t="inlineStr"/>
+      <c r="AG20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF20" s="2" t="inlineStr"/>
-      <c r="AG20" s="2" t="inlineStr"/>
-      <c r="AH20" s="2" t="n">
+      <c r="AH20" s="2" t="inlineStr"/>
+      <c r="AI20" s="2" t="inlineStr"/>
+      <c r="AJ20" s="2" t="n">
         <v>-22.29</v>
       </c>
-      <c r="AI20" s="2" t="n">
+      <c r="AK20" s="2" t="n">
         <v>-1.15</v>
       </c>
-      <c r="AJ20" s="2" t="n">
+      <c r="AL20" s="2" t="n">
         <v>2.67</v>
       </c>
-      <c r="AK20" s="2" t="n">
+      <c r="AM20" s="2" t="n">
         <v>2.81</v>
       </c>
-      <c r="AL20" s="2" t="n">
+      <c r="AN20" s="2" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="AM20" s="2" t="n">
+      <c r="AO20" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="AN20" s="2" t="inlineStr"/>
-      <c r="AO20" s="2" t="inlineStr"/>
       <c r="AP20" s="2" t="inlineStr"/>
       <c r="AQ20" s="2" t="inlineStr"/>
-      <c r="AR20" s="2" t="inlineStr">
+      <c r="AR20" s="2" t="inlineStr"/>
+      <c r="AS20" s="2" t="inlineStr"/>
+      <c r="AT20" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS20" s="2" t="n">
+      <c r="AU20" s="2" t="n">
         <v>1.726</v>
       </c>
-      <c r="AT20" s="2" t="n">
+      <c r="AV20" s="2" t="n">
         <v>1.735</v>
       </c>
-      <c r="AU20" s="2" t="n">
+      <c r="AW20" s="2" t="n">
         <v>1.767</v>
       </c>
-      <c r="AV20" s="2" t="n">
+      <c r="AX20" s="2" t="n">
         <v>1.803</v>
       </c>
-      <c r="AW20" s="2" t="n">
+      <c r="AY20" s="2" t="n">
         <v>1.816</v>
       </c>
-      <c r="AX20" s="2" t="n">
+      <c r="AZ20" s="2" t="n">
         <v>1.811</v>
       </c>
-      <c r="AY20" s="2" t="n">
+      <c r="BA20" s="2" t="n">
         <v>1.875</v>
       </c>
-      <c r="AZ20" s="2" t="n">
+      <c r="BB20" s="2" t="n">
         <v>-1.1406</v>
       </c>
-      <c r="BA20" s="2" t="n">
+      <c r="BC20" s="2" t="n">
         <v>-1.0099</v>
       </c>
-      <c r="BB20" s="2" t="n">
+      <c r="BD20" s="2" t="n">
         <v>-0.3407</v>
       </c>
-      <c r="BC20" s="2" t="n">
+      <c r="BE20" s="2" t="n">
         <v>-0.1052</v>
       </c>
-      <c r="BD20" s="2" t="n">
+      <c r="BF20" s="2" t="n">
         <v>-0.2229</v>
       </c>
     </row>
@@ -3613,91 +3663,89 @@
         </is>
       </c>
       <c r="W21" s="2" t="n">
-        <v>100</v>
+        <v>128</v>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr"/>
-      <c r="Z21" s="2" t="inlineStr">
-        <is>
-          <t>2C→2B·6d ← 2B→2C·19d</t>
-        </is>
-      </c>
+      <c r="Z21" s="2" t="inlineStr"/>
       <c r="AA21" s="2" t="inlineStr"/>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
       <c r="AD21" s="2" t="inlineStr"/>
-      <c r="AE21" s="2" t="n">
+      <c r="AE21" s="2" t="inlineStr"/>
+      <c r="AF21" s="2" t="inlineStr"/>
+      <c r="AG21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AF21" s="2" t="inlineStr"/>
-      <c r="AG21" s="2" t="inlineStr"/>
-      <c r="AH21" s="2" t="n">
+      <c r="AH21" s="2" t="inlineStr"/>
+      <c r="AI21" s="2" t="inlineStr"/>
+      <c r="AJ21" s="2" t="n">
         <v>28.63</v>
       </c>
-      <c r="AI21" s="2" t="n">
+      <c r="AK21" s="2" t="n">
         <v>30.63</v>
       </c>
-      <c r="AJ21" s="2" t="n">
+      <c r="AL21" s="2" t="n">
         <v>1.18</v>
       </c>
-      <c r="AK21" s="2" t="n">
+      <c r="AM21" s="2" t="n">
         <v>14.75</v>
       </c>
-      <c r="AL21" s="2" t="n">
+      <c r="AN21" s="2" t="n">
         <v>86.09999999999999</v>
       </c>
-      <c r="AM21" s="2" t="n">
+      <c r="AO21" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="AN21" s="2" t="inlineStr"/>
-      <c r="AO21" s="2" t="inlineStr"/>
-      <c r="AP21" s="2" t="n">
+      <c r="AP21" s="2" t="inlineStr"/>
+      <c r="AQ21" s="2" t="inlineStr"/>
+      <c r="AR21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AQ21" s="2" t="inlineStr"/>
-      <c r="AR21" s="2" t="inlineStr">
+      <c r="AS21" s="2" t="inlineStr"/>
+      <c r="AT21" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS21" s="2" t="n">
+      <c r="AU21" s="2" t="n">
         <v>2.37</v>
       </c>
-      <c r="AT21" s="2" t="n">
+      <c r="AV21" s="2" t="n">
         <v>2.36</v>
       </c>
-      <c r="AU21" s="2" t="n">
+      <c r="AW21" s="2" t="n">
         <v>2.307</v>
       </c>
-      <c r="AV21" s="2" t="n">
+      <c r="AX21" s="2" t="n">
         <v>2.279</v>
       </c>
-      <c r="AW21" s="2" t="n">
+      <c r="AY21" s="2" t="n">
         <v>2.254</v>
       </c>
-      <c r="AX21" s="2" t="n">
+      <c r="AZ21" s="2" t="n">
         <v>2.217</v>
       </c>
-      <c r="AY21" s="2" t="n">
+      <c r="BA21" s="2" t="n">
         <v>2.044</v>
       </c>
-      <c r="AZ21" s="2" t="n">
+      <c r="BB21" s="2" t="n">
         <v>0.7547</v>
       </c>
-      <c r="BA21" s="2" t="n">
+      <c r="BC21" s="2" t="n">
         <v>0.8098</v>
       </c>
-      <c r="BB21" s="2" t="n">
+      <c r="BD21" s="2" t="n">
         <v>0.6761</v>
       </c>
-      <c r="BC21" s="2" t="n">
+      <c r="BE21" s="2" t="n">
         <v>0.3483</v>
       </c>
-      <c r="BD21" s="2" t="n">
+      <c r="BF21" s="2" t="n">
         <v>0.2863</v>
       </c>
     </row>
@@ -3761,7 +3809,7 @@
         </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
@@ -3773,75 +3821,77 @@
       <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
-      <c r="AD22" s="2" t="n">
+      <c r="AD22" s="2" t="inlineStr"/>
+      <c r="AE22" s="2" t="inlineStr"/>
+      <c r="AF22" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AE22" s="2" t="inlineStr"/>
-      <c r="AF22" s="2" t="inlineStr"/>
       <c r="AG22" s="2" t="inlineStr"/>
-      <c r="AH22" s="2" t="n">
+      <c r="AH22" s="2" t="inlineStr"/>
+      <c r="AI22" s="2" t="inlineStr"/>
+      <c r="AJ22" s="2" t="n">
         <v>-28.82</v>
       </c>
-      <c r="AI22" s="2" t="n">
+      <c r="AK22" s="2" t="n">
         <v>-16.69</v>
       </c>
-      <c r="AJ22" s="2" t="n">
+      <c r="AL22" s="2" t="n">
         <v>-4.9</v>
       </c>
-      <c r="AK22" s="2" t="n">
+      <c r="AM22" s="2" t="n">
         <v>-2.68</v>
       </c>
-      <c r="AL22" s="2" t="n">
+      <c r="AN22" s="2" t="n">
         <v>-0.6</v>
       </c>
-      <c r="AM22" s="2" t="n">
+      <c r="AO22" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="AN22" s="2" t="inlineStr"/>
-      <c r="AO22" s="2" t="n">
+      <c r="AP22" s="2" t="inlineStr"/>
+      <c r="AQ22" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AP22" s="2" t="inlineStr"/>
-      <c r="AQ22" s="2" t="inlineStr"/>
-      <c r="AR22" s="2" t="inlineStr">
+      <c r="AR22" s="2" t="inlineStr"/>
+      <c r="AS22" s="2" t="inlineStr"/>
+      <c r="AT22" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AS22" s="2" t="n">
+      <c r="AU22" s="2" t="n">
         <v>1.381</v>
       </c>
-      <c r="AT22" s="2" t="n">
+      <c r="AV22" s="2" t="n">
         <v>1.416</v>
       </c>
-      <c r="AU22" s="2" t="n">
+      <c r="AW22" s="2" t="n">
         <v>1.455</v>
       </c>
-      <c r="AV22" s="2" t="n">
+      <c r="AX22" s="2" t="n">
         <v>1.493</v>
       </c>
-      <c r="AW22" s="2" t="n">
+      <c r="AY22" s="2" t="n">
         <v>1.555</v>
       </c>
-      <c r="AX22" s="2" t="n">
+      <c r="AZ22" s="2" t="n">
         <v>1.68</v>
       </c>
-      <c r="AY22" s="2" t="n">
+      <c r="BA22" s="2" t="n">
         <v>1.798</v>
       </c>
-      <c r="AZ22" s="2" t="n">
+      <c r="BB22" s="2" t="n">
         <v>-2.0794</v>
       </c>
-      <c r="BA22" s="2" t="n">
+      <c r="BC22" s="2" t="n">
         <v>-1.4063</v>
       </c>
-      <c r="BB22" s="2" t="n">
+      <c r="BD22" s="2" t="n">
         <v>-0.6909</v>
       </c>
-      <c r="BC22" s="2" t="n">
+      <c r="BE22" s="2" t="n">
         <v>-0.9959</v>
       </c>
-      <c r="BD22" s="2" t="n">
+      <c r="BF22" s="2" t="n">
         <v>-0.2882</v>
       </c>
     </row>
@@ -3903,21 +3953,21 @@
       </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W23" s="2" t="n">
-        <v>7</v>
+        <v>299</v>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="Y23" s="2" t="inlineStr"/>
       <c r="Z23" s="2" t="inlineStr">
         <is>
-          <t>2A→1·7d</t>
+          <t>2C→2A·12d</t>
         </is>
       </c>
       <c r="AA23" s="2" t="inlineStr"/>
@@ -3927,67 +3977,69 @@
       <c r="AE23" s="2" t="inlineStr"/>
       <c r="AF23" s="2" t="inlineStr"/>
       <c r="AG23" s="2" t="inlineStr"/>
-      <c r="AH23" s="2" t="n">
+      <c r="AH23" s="2" t="inlineStr"/>
+      <c r="AI23" s="2" t="inlineStr"/>
+      <c r="AJ23" s="2" t="n">
         <v>14.05</v>
       </c>
-      <c r="AI23" s="2" t="n">
+      <c r="AK23" s="2" t="n">
         <v>-1.3</v>
       </c>
-      <c r="AJ23" s="2" t="n">
+      <c r="AL23" s="2" t="n">
         <v>-8.699999999999999</v>
       </c>
-      <c r="AK23" s="2" t="n">
+      <c r="AM23" s="2" t="n">
         <v>-22.04</v>
       </c>
-      <c r="AL23" s="2" t="n">
+      <c r="AN23" s="2" t="n">
         <v>3.2</v>
       </c>
-      <c r="AM23" s="2" t="n">
+      <c r="AO23" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="AN23" s="2" t="inlineStr"/>
-      <c r="AO23" s="2" t="inlineStr"/>
       <c r="AP23" s="2" t="inlineStr"/>
       <c r="AQ23" s="2" t="inlineStr"/>
-      <c r="AR23" s="2" t="inlineStr">
+      <c r="AR23" s="2" t="inlineStr"/>
+      <c r="AS23" s="2" t="inlineStr"/>
+      <c r="AT23" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS23" s="2" t="n">
+      <c r="AU23" s="2" t="n">
         <v>0.841</v>
       </c>
-      <c r="AT23" s="2" t="n">
+      <c r="AV23" s="2" t="n">
         <v>0.893</v>
       </c>
-      <c r="AU23" s="2" t="n">
+      <c r="AW23" s="2" t="n">
         <v>0.972</v>
       </c>
-      <c r="AV23" s="2" t="n">
+      <c r="AX23" s="2" t="n">
         <v>0.991</v>
       </c>
-      <c r="AW23" s="2" t="n">
+      <c r="AY23" s="2" t="n">
         <v>1.004</v>
       </c>
-      <c r="AX23" s="2" t="n">
+      <c r="AZ23" s="2" t="n">
         <v>1.104</v>
       </c>
-      <c r="AY23" s="2" t="n">
+      <c r="BA23" s="2" t="n">
         <v>0.975</v>
       </c>
-      <c r="AZ23" s="2" t="n">
+      <c r="BB23" s="2" t="n">
         <v>-5.8576</v>
       </c>
-      <c r="BA23" s="2" t="n">
+      <c r="BC23" s="2" t="n">
         <v>-2.4715</v>
       </c>
-      <c r="BB23" s="2" t="n">
+      <c r="BD23" s="2" t="n">
         <v>-0.6881</v>
       </c>
-      <c r="BC23" s="2" t="n">
+      <c r="BE23" s="2" t="n">
         <v>-0.667</v>
       </c>
-      <c r="BD23" s="2" t="n">
+      <c r="BF23" s="2" t="n">
         <v>0.1405</v>
       </c>
     </row>
@@ -4045,7 +4097,7 @@
         </is>
       </c>
       <c r="W24" s="2" t="n">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
@@ -4054,90 +4106,92 @@
       </c>
       <c r="Y24" s="2" t="inlineStr">
         <is>
-          <t>减速</t>
+          <t>减速·周MACD将死叉</t>
         </is>
       </c>
       <c r="Z24" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·3d ← 2B→2A·14d ← 3→2B·18d</t>
+          <t>2A→2C·12d</t>
         </is>
       </c>
       <c r="AA24" s="2" t="inlineStr"/>
       <c r="AB24" s="2" t="inlineStr"/>
-      <c r="AC24" s="2" t="n">
+      <c r="AC24" s="2" t="inlineStr"/>
+      <c r="AD24" s="2" t="inlineStr"/>
+      <c r="AE24" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AD24" s="2" t="n">
+      <c r="AF24" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AE24" s="2" t="inlineStr">
+      <c r="AG24" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
         </is>
       </c>
-      <c r="AF24" s="2" t="inlineStr"/>
-      <c r="AG24" s="2" t="inlineStr"/>
-      <c r="AH24" s="2" t="n">
+      <c r="AH24" s="2" t="inlineStr"/>
+      <c r="AI24" s="2" t="inlineStr"/>
+      <c r="AJ24" s="2" t="n">
         <v>24.26</v>
       </c>
-      <c r="AI24" s="2" t="n">
+      <c r="AK24" s="2" t="n">
         <v>18.77</v>
       </c>
-      <c r="AJ24" s="2" t="n">
+      <c r="AL24" s="2" t="n">
         <v>0.4</v>
       </c>
-      <c r="AK24" s="2" t="n">
+      <c r="AM24" s="2" t="n">
         <v>3.02</v>
       </c>
-      <c r="AL24" s="2" t="n">
+      <c r="AN24" s="2" t="n">
         <v>68.2</v>
       </c>
-      <c r="AM24" s="2" t="n">
+      <c r="AO24" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="AN24" s="2" t="inlineStr"/>
-      <c r="AO24" s="2" t="inlineStr"/>
       <c r="AP24" s="2" t="inlineStr"/>
       <c r="AQ24" s="2" t="inlineStr"/>
-      <c r="AR24" s="2" t="inlineStr">
+      <c r="AR24" s="2" t="inlineStr"/>
+      <c r="AS24" s="2" t="inlineStr"/>
+      <c r="AT24" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS24" s="2" t="n">
+      <c r="AU24" s="2" t="n">
         <v>1.277</v>
       </c>
-      <c r="AT24" s="2" t="n">
+      <c r="AV24" s="2" t="n">
         <v>1.272</v>
       </c>
-      <c r="AU24" s="2" t="n">
+      <c r="AW24" s="2" t="n">
         <v>1.272</v>
       </c>
-      <c r="AV24" s="2" t="n">
+      <c r="AX24" s="2" t="n">
         <v>1.288</v>
       </c>
-      <c r="AW24" s="2" t="n">
+      <c r="AY24" s="2" t="n">
         <v>1.274</v>
       </c>
-      <c r="AX24" s="2" t="n">
+      <c r="AZ24" s="2" t="n">
         <v>1.241</v>
       </c>
-      <c r="AY24" s="2" t="n">
+      <c r="BA24" s="2" t="n">
         <v>1.208</v>
       </c>
-      <c r="AZ24" s="2" t="n">
+      <c r="BB24" s="2" t="n">
         <v>0.1367</v>
       </c>
-      <c r="BA24" s="2" t="n">
+      <c r="BC24" s="2" t="n">
         <v>-0.2955</v>
       </c>
-      <c r="BB24" s="2" t="n">
+      <c r="BD24" s="2" t="n">
         <v>0.3603</v>
       </c>
-      <c r="BC24" s="2" t="n">
+      <c r="BE24" s="2" t="n">
         <v>0.0888</v>
       </c>
-      <c r="BD24" s="2" t="n">
+      <c r="BF24" s="2" t="n">
         <v>0.2426</v>
       </c>
     </row>
@@ -4203,7 +4257,7 @@
         </is>
       </c>
       <c r="W25" s="2" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
@@ -4214,78 +4268,80 @@
       <c r="Z25" s="2" t="inlineStr"/>
       <c r="AA25" s="2" t="inlineStr"/>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="inlineStr">
+      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AD25" s="2" t="inlineStr"/>
+      <c r="AE25" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="AD25" s="2" t="inlineStr"/>
-      <c r="AE25" s="2" t="inlineStr"/>
       <c r="AF25" s="2" t="inlineStr"/>
       <c r="AG25" s="2" t="inlineStr"/>
-      <c r="AH25" s="2" t="n">
+      <c r="AH25" s="2" t="inlineStr"/>
+      <c r="AI25" s="2" t="inlineStr"/>
+      <c r="AJ25" s="2" t="n">
         <v>-29.33</v>
       </c>
-      <c r="AI25" s="2" t="n">
+      <c r="AK25" s="2" t="n">
         <v>-18.1</v>
       </c>
-      <c r="AJ25" s="2" t="n">
+      <c r="AL25" s="2" t="n">
         <v>-2.33</v>
       </c>
-      <c r="AK25" s="2" t="n">
+      <c r="AM25" s="2" t="n">
         <v>-2.15</v>
       </c>
-      <c r="AL25" s="2" t="n">
+      <c r="AN25" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="AM25" s="2" t="n">
+      <c r="AO25" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="AN25" s="2" t="inlineStr"/>
-      <c r="AO25" s="2" t="n">
+      <c r="AP25" s="2" t="inlineStr"/>
+      <c r="AQ25" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AP25" s="2" t="inlineStr"/>
-      <c r="AQ25" s="2" t="inlineStr"/>
-      <c r="AR25" s="2" t="inlineStr">
+      <c r="AR25" s="2" t="inlineStr"/>
+      <c r="AS25" s="2" t="inlineStr"/>
+      <c r="AT25" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AS25" s="2" t="n">
+      <c r="AU25" s="2" t="n">
         <v>0.736</v>
       </c>
-      <c r="AT25" s="2" t="n">
+      <c r="AV25" s="2" t="n">
         <v>0.753</v>
       </c>
-      <c r="AU25" s="2" t="n">
+      <c r="AW25" s="2" t="n">
         <v>0.777</v>
       </c>
-      <c r="AV25" s="2" t="n">
+      <c r="AX25" s="2" t="n">
         <v>0.791</v>
       </c>
-      <c r="AW25" s="2" t="n">
+      <c r="AY25" s="2" t="n">
         <v>0.8169999999999999</v>
       </c>
-      <c r="AX25" s="2" t="n">
+      <c r="AZ25" s="2" t="n">
         <v>0.891</v>
       </c>
-      <c r="AY25" s="2" t="n">
+      <c r="BA25" s="2" t="n">
         <v>0.982</v>
       </c>
-      <c r="AZ25" s="2" t="n">
+      <c r="BB25" s="2" t="n">
         <v>-2.4799</v>
       </c>
-      <c r="BA25" s="2" t="n">
+      <c r="BC25" s="2" t="n">
         <v>-1.2595</v>
       </c>
-      <c r="BB25" s="2" t="n">
+      <c r="BD25" s="2" t="n">
         <v>-0.4956</v>
       </c>
-      <c r="BC25" s="2" t="n">
+      <c r="BE25" s="2" t="n">
         <v>-1.0848</v>
       </c>
-      <c r="BD25" s="2" t="n">
+      <c r="BF25" s="2" t="n">
         <v>-0.2933</v>
       </c>
     </row>
@@ -4347,21 +4403,21 @@
       </c>
       <c r="V26" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W26" s="2" t="n">
-        <v>9</v>
+        <v>299</v>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="Y26" s="2" t="inlineStr"/>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>2A→1·9d ← 3→2A·13d</t>
+          <t>2C→2A·19d</t>
         </is>
       </c>
       <c r="AA26" s="2" t="inlineStr"/>
@@ -4371,67 +4427,69 @@
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr"/>
       <c r="AG26" s="2" t="inlineStr"/>
-      <c r="AH26" s="2" t="n">
+      <c r="AH26" s="2" t="inlineStr"/>
+      <c r="AI26" s="2" t="inlineStr"/>
+      <c r="AJ26" s="2" t="n">
         <v>9.67</v>
       </c>
-      <c r="AI26" s="2" t="n">
+      <c r="AK26" s="2" t="n">
         <v>-3.14</v>
       </c>
-      <c r="AJ26" s="2" t="n">
+      <c r="AL26" s="2" t="n">
         <v>-9.74</v>
       </c>
-      <c r="AK26" s="2" t="n">
+      <c r="AM26" s="2" t="n">
         <v>-20.8</v>
       </c>
-      <c r="AL26" s="2" t="n">
+      <c r="AN26" s="2" t="n">
         <v>6.5</v>
       </c>
-      <c r="AM26" s="2" t="n">
+      <c r="AO26" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="AN26" s="2" t="inlineStr"/>
-      <c r="AO26" s="2" t="inlineStr"/>
       <c r="AP26" s="2" t="inlineStr"/>
       <c r="AQ26" s="2" t="inlineStr"/>
-      <c r="AR26" s="2" t="inlineStr">
+      <c r="AR26" s="2" t="inlineStr"/>
+      <c r="AS26" s="2" t="inlineStr"/>
+      <c r="AT26" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS26" s="2" t="n">
+      <c r="AU26" s="2" t="n">
         <v>0.545</v>
       </c>
-      <c r="AT26" s="2" t="n">
+      <c r="AV26" s="2" t="n">
         <v>0.579</v>
       </c>
-      <c r="AU26" s="2" t="n">
+      <c r="AW26" s="2" t="n">
         <v>0.633</v>
       </c>
-      <c r="AV26" s="2" t="n">
+      <c r="AX26" s="2" t="n">
         <v>0.643</v>
       </c>
-      <c r="AW26" s="2" t="n">
+      <c r="AY26" s="2" t="n">
         <v>0.648</v>
       </c>
-      <c r="AX26" s="2" t="n">
+      <c r="AZ26" s="2" t="n">
         <v>0.715</v>
       </c>
-      <c r="AY26" s="2" t="n">
+      <c r="BA26" s="2" t="n">
         <v>0.644</v>
       </c>
-      <c r="AZ26" s="2" t="n">
+      <c r="BB26" s="2" t="n">
         <v>-6.1583</v>
       </c>
-      <c r="BA26" s="2" t="n">
+      <c r="BC26" s="2" t="n">
         <v>-2.3924</v>
       </c>
-      <c r="BB26" s="2" t="n">
+      <c r="BD26" s="2" t="n">
         <v>-0.5481</v>
       </c>
-      <c r="BC26" s="2" t="n">
+      <c r="BE26" s="2" t="n">
         <v>-0.7674</v>
       </c>
-      <c r="BD26" s="2" t="n">
+      <c r="BF26" s="2" t="n">
         <v>0.09669999999999999</v>
       </c>
     </row>
@@ -4497,7 +4555,7 @@
         </is>
       </c>
       <c r="W27" s="2" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
@@ -4513,69 +4571,71 @@
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr"/>
       <c r="AG27" s="2" t="inlineStr"/>
-      <c r="AH27" s="2" t="n">
+      <c r="AH27" s="2" t="inlineStr"/>
+      <c r="AI27" s="2" t="inlineStr"/>
+      <c r="AJ27" s="2" t="n">
         <v>-30.85</v>
       </c>
-      <c r="AI27" s="2" t="n">
+      <c r="AK27" s="2" t="n">
         <v>-18.57</v>
       </c>
-      <c r="AJ27" s="2" t="n">
+      <c r="AL27" s="2" t="n">
         <v>-4.07</v>
       </c>
-      <c r="AK27" s="2" t="n">
+      <c r="AM27" s="2" t="n">
         <v>-2.97</v>
       </c>
-      <c r="AL27" s="2" t="n">
+      <c r="AN27" s="2" t="n">
         <v>-1.7</v>
       </c>
-      <c r="AM27" s="2" t="n">
+      <c r="AO27" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="AN27" s="2" t="inlineStr"/>
-      <c r="AO27" s="2" t="n">
+      <c r="AP27" s="2" t="inlineStr"/>
+      <c r="AQ27" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="AP27" s="2" t="inlineStr"/>
-      <c r="AQ27" s="2" t="inlineStr"/>
-      <c r="AR27" s="2" t="inlineStr">
+      <c r="AR27" s="2" t="inlineStr"/>
+      <c r="AS27" s="2" t="inlineStr"/>
+      <c r="AT27" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AS27" s="2" t="n">
+      <c r="AU27" s="2" t="n">
         <v>2.129</v>
       </c>
-      <c r="AT27" s="2" t="n">
+      <c r="AV27" s="2" t="n">
         <v>2.179</v>
       </c>
-      <c r="AU27" s="2" t="n">
+      <c r="AW27" s="2" t="n">
         <v>2.245</v>
       </c>
-      <c r="AV27" s="2" t="n">
+      <c r="AX27" s="2" t="n">
         <v>2.292</v>
       </c>
-      <c r="AW27" s="2" t="n">
+      <c r="AY27" s="2" t="n">
         <v>2.388</v>
       </c>
-      <c r="AX27" s="2" t="n">
+      <c r="AZ27" s="2" t="n">
         <v>2.6</v>
       </c>
-      <c r="AY27" s="2" t="n">
+      <c r="BA27" s="2" t="n">
         <v>2.835</v>
       </c>
-      <c r="AZ27" s="2" t="n">
+      <c r="BB27" s="2" t="n">
         <v>-2.1392</v>
       </c>
-      <c r="BA27" s="2" t="n">
+      <c r="BC27" s="2" t="n">
         <v>-1.2899</v>
       </c>
-      <c r="BB27" s="2" t="n">
+      <c r="BD27" s="2" t="n">
         <v>-0.6471</v>
       </c>
-      <c r="BC27" s="2" t="n">
+      <c r="BE27" s="2" t="n">
         <v>-1.0579</v>
       </c>
-      <c r="BD27" s="2" t="n">
+      <c r="BF27" s="2" t="n">
         <v>-0.3085</v>
       </c>
     </row>
@@ -4641,7 +4701,7 @@
         </is>
       </c>
       <c r="W28" s="2" t="n">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
@@ -4657,65 +4717,67 @@
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr"/>
       <c r="AG28" s="2" t="inlineStr"/>
-      <c r="AH28" s="2" t="n">
+      <c r="AH28" s="2" t="inlineStr"/>
+      <c r="AI28" s="2" t="inlineStr"/>
+      <c r="AJ28" s="2" t="n">
         <v>-18.47</v>
       </c>
-      <c r="AI28" s="2" t="n">
+      <c r="AK28" s="2" t="n">
         <v>-12.78</v>
       </c>
-      <c r="AJ28" s="2" t="n">
+      <c r="AL28" s="2" t="n">
         <v>-4.08</v>
       </c>
-      <c r="AK28" s="2" t="n">
+      <c r="AM28" s="2" t="n">
         <v>-5.15</v>
       </c>
-      <c r="AL28" s="2" t="n">
+      <c r="AN28" s="2" t="n">
         <v>-5.7</v>
       </c>
-      <c r="AM28" s="2" t="inlineStr"/>
-      <c r="AN28" s="2" t="inlineStr"/>
       <c r="AO28" s="2" t="inlineStr"/>
       <c r="AP28" s="2" t="inlineStr"/>
       <c r="AQ28" s="2" t="inlineStr"/>
-      <c r="AR28" s="2" t="inlineStr">
+      <c r="AR28" s="2" t="inlineStr"/>
+      <c r="AS28" s="2" t="inlineStr"/>
+      <c r="AT28" s="2" t="inlineStr">
         <is>
           <t>背离</t>
         </is>
       </c>
-      <c r="AS28" s="2" t="n">
+      <c r="AU28" s="2" t="n">
         <v>0.8139999999999999</v>
       </c>
-      <c r="AT28" s="2" t="n">
+      <c r="AV28" s="2" t="n">
         <v>0.849</v>
       </c>
-      <c r="AU28" s="2" t="n">
+      <c r="AW28" s="2" t="n">
         <v>0.885</v>
       </c>
-      <c r="AV28" s="2" t="n">
+      <c r="AX28" s="2" t="n">
         <v>0.907</v>
       </c>
-      <c r="AW28" s="2" t="n">
+      <c r="AY28" s="2" t="n">
         <v>0.9389999999999999</v>
       </c>
-      <c r="AX28" s="2" t="n">
+      <c r="AZ28" s="2" t="n">
         <v>1.016</v>
       </c>
-      <c r="AY28" s="2" t="n">
+      <c r="BA28" s="2" t="n">
         <v>1.024</v>
       </c>
-      <c r="AZ28" s="2" t="n">
+      <c r="BB28" s="2" t="n">
         <v>-3.3313</v>
       </c>
-      <c r="BA28" s="2" t="n">
+      <c r="BC28" s="2" t="n">
         <v>-1.8203</v>
       </c>
-      <c r="BB28" s="2" t="n">
+      <c r="BD28" s="2" t="n">
         <v>-0.6035</v>
       </c>
-      <c r="BC28" s="2" t="n">
+      <c r="BE28" s="2" t="n">
         <v>-0.9025</v>
       </c>
-      <c r="BD28" s="2" t="n">
+      <c r="BF28" s="2" t="n">
         <v>-0.1847</v>
       </c>
     </row>
@@ -4771,19 +4833,23 @@
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W29" s="2" t="n">
-        <v>24</v>
+        <v>299</v>
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="Y29" s="2" t="inlineStr"/>
-      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>2C→2A·5d</t>
+        </is>
+      </c>
       <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="inlineStr"/>
@@ -4791,69 +4857,71 @@
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr"/>
       <c r="AG29" s="2" t="inlineStr"/>
-      <c r="AH29" s="2" t="n">
+      <c r="AH29" s="2" t="inlineStr"/>
+      <c r="AI29" s="2" t="inlineStr"/>
+      <c r="AJ29" s="2" t="n">
         <v>4.83</v>
       </c>
-      <c r="AI29" s="2" t="n">
+      <c r="AK29" s="2" t="n">
         <v>-1.82</v>
       </c>
-      <c r="AJ29" s="2" t="n">
+      <c r="AL29" s="2" t="n">
         <v>-4.15</v>
       </c>
-      <c r="AK29" s="2" t="n">
+      <c r="AM29" s="2" t="n">
         <v>-7.62</v>
       </c>
-      <c r="AL29" s="2" t="n">
+      <c r="AN29" s="2" t="n">
         <v>-6.8</v>
       </c>
-      <c r="AM29" s="2" t="n">
+      <c r="AO29" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="AN29" s="2" t="inlineStr"/>
-      <c r="AO29" s="2" t="n">
+      <c r="AP29" s="2" t="inlineStr"/>
+      <c r="AQ29" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="AP29" s="2" t="inlineStr"/>
-      <c r="AQ29" s="2" t="inlineStr"/>
-      <c r="AR29" s="2" t="inlineStr">
+      <c r="AR29" s="2" t="inlineStr"/>
+      <c r="AS29" s="2" t="inlineStr"/>
+      <c r="AT29" s="2" t="inlineStr">
         <is>
           <t>无背离</t>
         </is>
       </c>
-      <c r="AS29" s="2" t="n">
+      <c r="AU29" s="2" t="n">
         <v>1.468</v>
       </c>
-      <c r="AT29" s="2" t="n">
+      <c r="AV29" s="2" t="n">
         <v>1.533</v>
       </c>
-      <c r="AU29" s="2" t="n">
+      <c r="AW29" s="2" t="n">
         <v>1.617</v>
       </c>
-      <c r="AV29" s="2" t="n">
+      <c r="AX29" s="2" t="n">
         <v>1.647</v>
       </c>
-      <c r="AW29" s="2" t="n">
+      <c r="AY29" s="2" t="n">
         <v>1.698</v>
       </c>
-      <c r="AX29" s="2" t="n">
+      <c r="AZ29" s="2" t="n">
         <v>1.829</v>
       </c>
-      <c r="AY29" s="2" t="n">
+      <c r="BA29" s="2" t="n">
         <v>1.676</v>
       </c>
-      <c r="AZ29" s="2" t="n">
+      <c r="BB29" s="2" t="n">
         <v>-4.2937</v>
       </c>
-      <c r="BA29" s="2" t="n">
+      <c r="BC29" s="2" t="n">
         <v>-1.6274</v>
       </c>
-      <c r="BB29" s="2" t="n">
+      <c r="BD29" s="2" t="n">
         <v>-1.0129</v>
       </c>
-      <c r="BC29" s="2" t="n">
+      <c r="BE29" s="2" t="n">
         <v>-0.5259</v>
       </c>
-      <c r="BD29" s="2" t="n">
+      <c r="BF29" s="2" t="n">
         <v>0.0483</v>
       </c>
     </row>
@@ -4911,7 +4979,7 @@
         </is>
       </c>
       <c r="W30" s="2" t="n">
-        <v>173</v>
+        <v>209</v>
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
@@ -4923,7 +4991,11 @@
           <t>站稳短均·底背离·日线纠缠</t>
         </is>
       </c>
-      <c r="Z30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>4→4+·20d</t>
+        </is>
+      </c>
       <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
@@ -4931,67 +5003,69 @@
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr"/>
       <c r="AG30" s="2" t="inlineStr"/>
-      <c r="AH30" s="2" t="n">
+      <c r="AH30" s="2" t="inlineStr"/>
+      <c r="AI30" s="2" t="inlineStr"/>
+      <c r="AJ30" s="2" t="n">
         <v>-24.07</v>
       </c>
-      <c r="AI30" s="2" t="n">
+      <c r="AK30" s="2" t="n">
         <v>1.05</v>
       </c>
-      <c r="AJ30" s="2" t="n">
+      <c r="AL30" s="2" t="n">
         <v>4.69</v>
       </c>
-      <c r="AK30" s="2" t="n">
+      <c r="AM30" s="2" t="n">
         <v>10.37</v>
       </c>
-      <c r="AL30" s="2" t="n">
+      <c r="AN30" s="2" t="n">
         <v>67.90000000000001</v>
       </c>
-      <c r="AM30" s="2" t="n">
+      <c r="AO30" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="AN30" s="2" t="inlineStr"/>
-      <c r="AO30" s="2" t="inlineStr"/>
       <c r="AP30" s="2" t="inlineStr"/>
       <c r="AQ30" s="2" t="inlineStr"/>
-      <c r="AR30" s="2" t="inlineStr">
+      <c r="AR30" s="2" t="inlineStr"/>
+      <c r="AS30" s="2" t="inlineStr"/>
+      <c r="AT30" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS30" s="2" t="n">
+      <c r="AU30" s="2" t="n">
         <v>0.663</v>
       </c>
-      <c r="AT30" s="2" t="n">
+      <c r="AV30" s="2" t="n">
         <v>0.658</v>
       </c>
-      <c r="AU30" s="2" t="n">
+      <c r="AW30" s="2" t="n">
         <v>0.656</v>
       </c>
-      <c r="AV30" s="2" t="n">
+      <c r="AX30" s="2" t="n">
         <v>0.662</v>
       </c>
-      <c r="AW30" s="2" t="n">
+      <c r="AY30" s="2" t="n">
         <v>0.667</v>
       </c>
-      <c r="AX30" s="2" t="n">
+      <c r="AZ30" s="2" t="n">
         <v>0.659</v>
       </c>
-      <c r="AY30" s="2" t="n">
+      <c r="BA30" s="2" t="n">
         <v>0.713</v>
       </c>
-      <c r="AZ30" s="2" t="n">
+      <c r="BB30" s="2" t="n">
         <v>0.3422</v>
       </c>
-      <c r="BA30" s="2" t="n">
+      <c r="BC30" s="2" t="n">
         <v>-0.3388</v>
       </c>
-      <c r="BB30" s="2" t="n">
+      <c r="BD30" s="2" t="n">
         <v>-0.0888</v>
       </c>
-      <c r="BC30" s="2" t="n">
+      <c r="BE30" s="2" t="n">
         <v>-0.1683</v>
       </c>
-      <c r="BD30" s="2" t="n">
+      <c r="BF30" s="2" t="n">
         <v>-0.2407</v>
       </c>
     </row>
@@ -5051,7 +5125,7 @@
         </is>
       </c>
       <c r="W31" s="2" t="n">
-        <v>193</v>
+        <v>217</v>
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
@@ -5075,72 +5149,74 @@
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr"/>
       <c r="AG31" s="2" t="inlineStr"/>
-      <c r="AH31" s="2" t="n">
+      <c r="AH31" s="2" t="inlineStr"/>
+      <c r="AI31" s="2" t="inlineStr"/>
+      <c r="AJ31" s="2" t="n">
         <v>-37.04</v>
       </c>
-      <c r="AI31" s="2" t="n">
+      <c r="AK31" s="2" t="n">
         <v>-4.41</v>
       </c>
-      <c r="AJ31" s="2" t="n">
+      <c r="AL31" s="2" t="n">
         <v>4.32</v>
       </c>
-      <c r="AK31" s="2" t="n">
+      <c r="AM31" s="2" t="n">
         <v>11.25</v>
       </c>
-      <c r="AL31" s="2" t="n">
+      <c r="AN31" s="2" t="n">
         <v>53.1</v>
       </c>
-      <c r="AM31" s="2" t="n">
+      <c r="AO31" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="AN31" s="2" t="inlineStr"/>
-      <c r="AO31" s="2" t="inlineStr"/>
       <c r="AP31" s="2" t="inlineStr"/>
       <c r="AQ31" s="2" t="inlineStr"/>
-      <c r="AR31" s="2" t="inlineStr">
+      <c r="AR31" s="2" t="inlineStr"/>
+      <c r="AS31" s="2" t="inlineStr"/>
+      <c r="AT31" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
         </is>
       </c>
-      <c r="AS31" s="2" t="n">
+      <c r="AU31" s="2" t="n">
         <v>0.417</v>
       </c>
-      <c r="AT31" s="2" t="n">
+      <c r="AV31" s="2" t="n">
         <v>0.415</v>
       </c>
-      <c r="AU31" s="2" t="n">
+      <c r="AW31" s="2" t="n">
         <v>0.413</v>
       </c>
-      <c r="AV31" s="2" t="n">
+      <c r="AX31" s="2" t="n">
         <v>0.417</v>
       </c>
-      <c r="AW31" s="2" t="n">
+      <c r="AY31" s="2" t="n">
         <v>0.424</v>
       </c>
-      <c r="AX31" s="2" t="n">
+      <c r="AZ31" s="2" t="n">
         <v>0.422</v>
       </c>
-      <c r="AY31" s="2" t="n">
+      <c r="BA31" s="2" t="n">
         <v>0.468</v>
       </c>
-      <c r="AZ31" s="2" t="n">
+      <c r="BB31" s="2" t="n">
         <v>0.2645</v>
       </c>
-      <c r="BA31" s="2" t="n">
+      <c r="BC31" s="2" t="n">
         <v>-0.3561</v>
       </c>
-      <c r="BB31" s="2" t="n">
+      <c r="BD31" s="2" t="n">
         <v>-0.1659</v>
       </c>
-      <c r="BC31" s="2" t="n">
+      <c r="BE31" s="2" t="n">
         <v>-0.2365</v>
       </c>
-      <c r="BD31" s="2" t="n">
+      <c r="BF31" s="2" t="n">
         <v>-0.3704</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BD1"/>
+  <autoFilter ref="A1:BF1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5151,7 +5227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A65"/>
+  <dimension ref="A1:A66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5403,182 +5479,189 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stage (Weinstein 大阶段 v2.4引擎: EMA30W(150日EMA)锚, 判定优先级从高到低): ①均线排列覆盖: MA20&gt;MA50&gt;MA100&gt;MA150(简单均线)多头排列→强制Stage2; MA20&lt;MA50&lt;MA100&lt;MA150空头排列→强制Stage4(忽略斜率, 解决慢磨盲区) ②斜率双确认: EMA30W变化年化(4周×13与13周×3.88)均&gt;+8%→2; 均&lt;-6%→4(不对称) ③放平带: 52周位置+价格确认分1/3(3:pos&gt;0.55且价≥0.95×EMA30W; 1:pos&lt;0.45且价≤1.05×; 0.45~0.55滞回)。降级层(v2.2): 151-252根新股→①可用②仅≥215根③用上市以来位置, 标记列带'新'; ≤150根→NA</t>
+          <t xml:space="preserve">  Stage (Weinstein 大阶段 3.0引擎: 10W/30W全线SMA(50/150日), 锚=SMA30W): 优先级: ②′交叉通道(2A条件:金叉状态+M1+M2)→2 | ①均线排列覆盖: 四线全多头→强制2, 全空头→强制4 | ②斜率双确认(SMA30W 4周×13与13周×3.88年化)均&gt;+8%→2, 均&lt;-6%→4 | ③放平带: 低位(pos&lt;0.45且价≤1.05×锚)须慢门+4-先行情境→1否则4; 高位(pos&gt;0.55且价≥0.95×锚)须慢门镜像+2-先行情境→3否则2; 0.45~0.55滞回。慢门(10日年化斜率, delta=斜率10日变化): S1 SMA30W delta&gt;0, S2 SMA10W delta&gt;0, S3 10W改善&gt;30W, S4 sl10&gt;-6%(&gt;+8%临毕业保留); 镜像S1′-S4′全部取反(S4′: sl10&lt;+8%)。情境: has4=自上次退出Stage2以来出现过Stage4(起点种子:回撤≥25%); has2=自上次退出Stage1以来出现过Stage2(种子:涨幅≥30%)。降级层(v2.2): 151-252根新股弱规则标'新'; ≤150根→NA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stage持续: 处于当前大阶段的天数 (3交易日防抖, 转换日期回填至真实穿越点)</t>
+          <t xml:space="preserve">  SOS晋升/SOW降级 (⓪车道, 每bar后处理, 豁免一切门): 近10日SOS(放量2×+RS超额BM≥2%+中大阳+收盘上1/3+P1多头≥2项)且价&gt;SMA30W → 4/4+→1/1+, 1→1+, 1+→2/2A; 近10日SOW(镜像: 放量+RS跑输+中大阴+收盘下1/3+P1空头)且价&lt;SMA30W → 2/2C→3/3-, 3→3-, 3-→4。SOS晋升/SOW降级列=1表示该窗口当前激活</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1→2 / 3→4: 大阶段转换信号, 'Nd'=N个交易日前触发。触发后≤10个交易日持续显示(追溯保留); 转换后又跌回/回升的信号自动作废</t>
+          <t xml:space="preserve">  Stage持续: 处于当前大阶段的天数 (3交易日防抖, 转换日期回填至真实穿越点)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  子档(v2.4): 4+=基础双路径+必要条件: A止跌(纠缠/快慢线+周J超卖或底背离, 价&lt;EMA10W) ∨ B短期修复(站稳MA5/10/20三条) ; 均须周MACD柱为正(DIF&gt;DEA)或预计≤1周金叉(v2.4收紧) | 1=筑底(不区分价格vs EMA10W) | 1+=强筑底(站稳MA5/10/20全三条+全上行+周MACD DIF&gt;DEA) | 2A=修复态或刚确立(≤10日) | 2B=满配(slope10&gt;0·EMA10W&gt;EMA30W·10日前也是) | 2C=满配+延伸/减速/顶背离 | 3/4不分档</t>
+          <t xml:space="preserve">  1→2 / 3→4: 大阶段转换信号, 'Nd'=N个交易日前触发。触发后≤10个交易日持续显示(追溯保留); 转换后又跌回/回升的信号自动作废</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  子档标记: 状态描述列(与子档列分开)。4+→站稳短均(路径B)·周J超卖·底背离·日线纠缠(路径A); 1+→预金叉(EMA10W/30W将≤20日内纠缠或金叉)·纠缠·底背离; 2C→延伸(价超EMA30W达25%)·减速·顶背离; 新=降级层(上市151-252根弱规则档)</t>
+          <t xml:space="preserve">  子档(3.0): 4+ = A止跌((纠缠∨MA5&gt;MA20)+(周J超卖∨底背离)+价&lt;SMA10W) ∨ B站稳短均(MA5/10/20三条) ; 均须周MACD柱为正或≤1周将金叉 | 1 = 筑底(过准入, 不满足1+) | 1+ = α(站稳三均线+全上行+周MACD金叉+RS&gt;0) ∨ β(SOS直通) | 2A = 金叉状态(已金叉≤20日∨纠缠&lt;3%∨外推≤20日金叉)+M1(sl10&gt;+8%且delta&gt;0)+M2(d30&gt;+5pp) | 2B = 大致多头(SMA10W&gt;SMA30W且10日前也是)+斜率好(30W双确认&gt;+8%∨完整四线多头) | 2C = 2B基础+衰竭信号(本轮闩锁): ATR延伸99%分位∨50D斜率delta首次转负∨周线顶背离∨周MACD死叉或将死叉 | 3 = 筑顶过渡 | 3- = 跌破三均线+全下行+周MACD死叉+RS&lt;0 | 4 = 默认。生命周期 4→4+→1→1+→2A→2B→2C→3→3-→4, SOS/SOW可跳级</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  子档标记: 4+→站稳短均·周J超卖·底背离·日线纠缠; 1+→SOS突破(β持有)·预金叉·纠缠·底背离; 2C→ATR延伸·减速·顶背离·周MACD(将)死叉; 3-→预死叉·纠缠·顶背离; 新=降级层新股</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  子档变化: 近20日内最近3次子档转换, 新→旧 (如 '1A→1B·5d ← 2A→2B·12d')</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>【④ 企稳上行 — Cross】</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
+          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
+          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
+          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  周MACD Cross (2026-10-16): 周线(W-FRI)MACD DIF/DEA交叉。过去4周内金叉=1/死叉=-1;</t>
+          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    按近两周gap变化率外推预计下周内交叉=预1/预-1; 否则空</t>
+          <t xml:space="preserve">  周MACD Cross (2026-10-16): 周线(W-FRI)MACD DIF/DEA交叉。过去4周内金叉=1/死叉=-1;</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  日MACD Cross 死叉窗口放宽: 死叉≤5日均标-1 (金叉仍≤2日; 与周线列回看风格一致, 2026-10-16)</t>
+          <t xml:space="preserve">    按近两周gap变化率外推预计下周内交叉=预1/预-1; 否则空</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
+          <t xml:space="preserve">  日MACD Cross 死叉窗口放宽: 死叉≤5日均标-1 (金叉仍≤2日; 与周线列回看风格一致, 2026-10-16)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">    有过零但不稳定(whipsaw/暴涨驱动等脏交叉) → 0; 无过零但两线持续重叠(近5日rel&lt;0.2%) → 0; 其余空</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr"/>
-    </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>【⑦ 均线 MV 与年化斜率】(最右 12 列)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ND MV: N日收盘均线(前复权)最新值, N=5/10/20/30/50/100/200。历史不足N个交易日留空</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ND斜率: (N日均线最新 ÷ 5个交易日前的N日均线 - 1) ×52, 年化小数(0.1=10%)。N=10/20/50/100/200, 正值=均线上行</t>
+          <t xml:space="preserve">  ND MV: N日收盘均线(前复权)最新值, N=5/10/20/30/50/100/200。历史不足N个交易日留空</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  ND斜率: (N日均线最新 ÷ 5个交易日前的N日均线 - 1) ×52, 年化小数(0.1=10%)。N=10/20/50/100/200, 正值=均线上行</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">           (与【⑤】年线斜率列的×100百分比口径不同, 本列为原始×52; 不足N+5个交易日留空)</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr"/>
-    </row>
     <row r="62">
-      <c r="A62" s="6" t="inlineStr">
+      <c r="A62" s="5" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>【⑤ ETF 专属 — 趋势/Mansfield RS】</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
+          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MRS_沪深300: Mansfield RS vs 沪深300指数(000300.SH, jianxin) = (个股/HS300)/(252日均线)-1 ×100。正=跑赢沪深300 (兜底: 510300.SH ETF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  MRS_沪深300_1W / MRS_沪深300_4W: MRS_沪深300 分数的 5日 / 20日 变化</t>
         </is>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-19
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.789</v>
+        <v>2.762</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-0.51</v>
@@ -852,7 +852,7 @@
         <v>9</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
@@ -898,26 +898,26 @@
       <c r="AH2" s="2" t="inlineStr"/>
       <c r="AI2" s="2" t="inlineStr"/>
       <c r="AJ2" s="2" t="n">
-        <v>-10.15</v>
+        <v>-10.84</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>-9.01</v>
+        <v>-9.949999999999999</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>-5.58</v>
+        <v>-4.61</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>-10.16</v>
+        <v>-11.39</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-6.5</v>
+        <v>-6.9</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="AP2" s="2" t="inlineStr"/>
       <c r="AQ2" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AR2" s="2" t="inlineStr"/>
       <c r="AS2" s="2" t="inlineStr"/>
@@ -927,40 +927,40 @@
         </is>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>2.889</v>
+        <v>2.844</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>3.003</v>
+        <v>2.964</v>
       </c>
       <c r="AW2" s="2" t="n">
-        <v>3.177</v>
+        <v>3.148</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>3.245</v>
+        <v>3.222</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>3.362</v>
+        <v>3.349</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>3.646</v>
+        <v>3.636</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>3.519</v>
+        <v>3.518</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>-3.9913</v>
+        <v>-4.0242</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>-1.8798</v>
+        <v>-2.0927</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>-0.8233</v>
+        <v>-0.8506</v>
       </c>
       <c r="BE2" s="2" t="n">
-        <v>-0.7401</v>
+        <v>-0.757</v>
       </c>
       <c r="BF2" s="2" t="n">
-        <v>-0.1015</v>
+        <v>-0.1084</v>
       </c>
     </row>
     <row r="3">
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="W3" s="2" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
@@ -1027,41 +1027,43 @@
       <c r="Y3" s="2" t="inlineStr"/>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>4+→4·6d ← 4→4+·15d</t>
+          <t>4+→4·7d ← 4→4+·16d</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr"/>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
       <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="inlineStr">
+      <c r="AE3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF3" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="n">
-        <v>-12.67</v>
+        <v>-12.47</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>3.51</v>
+        <v>3.43</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>3.46</v>
+        <v>2.25</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>5.98</v>
+        <v>5.69</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>46.7</v>
+        <v>44.8</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="AP3" s="2" t="inlineStr"/>
       <c r="AQ3" s="2" t="inlineStr"/>
@@ -1073,153 +1075,147 @@
         </is>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>1.423</v>
+        <v>1.421</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>1.428</v>
+        <v>1.425</v>
       </c>
       <c r="AW3" s="2" t="n">
-        <v>1.442</v>
+        <v>1.44</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>1.458</v>
+        <v>1.455</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>1.478</v>
+        <v>1.476</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>1.463</v>
+        <v>1.462</v>
       </c>
       <c r="BA3" s="2" t="n">
         <v>1.51</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>-0.6667</v>
+        <v>-0.6987</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>-0.5765</v>
+        <v>-0.4999</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>-0.2809</v>
+        <v>-0.3244</v>
       </c>
       <c r="BE3" s="2" t="n">
-        <v>-0.1776</v>
+        <v>-0.1622</v>
       </c>
       <c r="BF3" s="2" t="n">
-        <v>-0.1267</v>
+        <v>-0.1247</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.836</v>
+        <v>0.666</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>95.31</v>
+        <v>-2.04</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>0000010110</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>0111111111</t>
+          <t>0001010100</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>152</v>
+        <v>210</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>2C</t>
-        </is>
-      </c>
-      <c r="Y4" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·7d</t>
+          <t>4→4+·2d ← 4+→4·3d ← 4→4+·4d</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr"/>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
       <c r="AD4" s="2" t="inlineStr"/>
-      <c r="AE4" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AF4" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="n">
-        <v>57.14</v>
+        <v>-24.3</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>39.33</v>
+        <v>0.86</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>-3.4</v>
+        <v>3.02</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>12.35</v>
+        <v>10.55</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>97.40000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="AP4" s="2" t="inlineStr"/>
       <c r="AQ4" s="2" t="inlineStr"/>
-      <c r="AR4" s="2" t="n">
-        <v>3</v>
-      </c>
+      <c r="AR4" s="2" t="inlineStr"/>
       <c r="AS4" s="2" t="inlineStr"/>
       <c r="AT4" s="2" t="inlineStr">
         <is>
@@ -1227,143 +1223,159 @@
         </is>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>1.856</v>
+        <v>0.663</v>
       </c>
       <c r="AV4" s="2" t="n">
-        <v>1.845</v>
+        <v>0.66</v>
       </c>
       <c r="AW4" s="2" t="n">
-        <v>1.801</v>
+        <v>0.656</v>
       </c>
       <c r="AX4" s="2" t="n">
-        <v>1.761</v>
+        <v>0.662</v>
       </c>
       <c r="AY4" s="2" t="n">
-        <v>1.664</v>
+        <v>0.666</v>
       </c>
       <c r="AZ4" s="2" t="n">
-        <v>1.592</v>
+        <v>0.659</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>1.533</v>
+        <v>0.712</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>1.8057</v>
+        <v>0.3971</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>0.963</v>
+        <v>-0.2249</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>1.1789</v>
+        <v>-0.1526</v>
       </c>
       <c r="BE4" s="2" t="n">
-        <v>0.3268</v>
+        <v>-0.1449</v>
       </c>
       <c r="BF4" s="2" t="n">
-        <v>0.5714</v>
+        <v>-0.243</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.796</v>
+        <v>1.809</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>7.37</v>
+        <v>95.31</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>0010011000</t>
+          <t>0111111101</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>0010011000</t>
+          <t>0111111101</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W5" s="2" t="n">
-        <v>4</v>
+        <v>153</v>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>1→4·4d ← 1+→1·7d ← 1→1+·8d</t>
+          <t>2A→2C·8d</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr"/>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AF5" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AG5" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AI5" s="2" t="inlineStr"/>
       <c r="AJ5" s="2" t="n">
-        <v>-7.99</v>
+        <v>56.16</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>5.16</v>
+        <v>36.9</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>-2.18</v>
+        <v>-2.52</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>6.86</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>41.9</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="AP5" s="2" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="AP5" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AQ5" s="2" t="inlineStr"/>
-      <c r="AR5" s="2" t="inlineStr"/>
+      <c r="AR5" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AS5" s="2" t="inlineStr"/>
       <c r="AT5" s="2" t="inlineStr">
         <is>
@@ -1371,58 +1383,58 @@
         </is>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>0.8129999999999999</v>
+        <v>1.843</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>0.831</v>
+        <v>1.85</v>
       </c>
       <c r="AW5" s="2" t="n">
-        <v>0.835</v>
+        <v>1.804</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>0.838</v>
+        <v>1.77</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>0.859</v>
+        <v>1.67</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>0.828</v>
+        <v>1.593</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>0.831</v>
+        <v>1.536</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>-1.3175</v>
+        <v>1.5781</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>-0.3924</v>
+        <v>0.7354000000000001</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>-0.1822</v>
+        <v>1.1625</v>
       </c>
       <c r="BE5" s="2" t="n">
-        <v>0.0692</v>
+        <v>0.2944</v>
       </c>
       <c r="BF5" s="2" t="n">
-        <v>-0.0799</v>
+        <v>0.5616</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2.866</v>
+        <v>0.804</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2.9</v>
+        <v>7.37</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -1432,29 +1444,27 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0010011000</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
@@ -1463,7 +1473,7 @@
         </is>
       </c>
       <c r="W6" s="2" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
@@ -1473,37 +1483,43 @@
       <c r="Y6" s="2" t="inlineStr"/>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>4+→4·20d</t>
+          <t>1→4·5d ← 1+→1·8d ← 1→1+·9d</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
       <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF6" s="2" t="inlineStr"/>
-      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF6" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AG6" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AH6" s="2" t="inlineStr"/>
       <c r="AI6" s="2" t="inlineStr"/>
       <c r="AJ6" s="2" t="n">
-        <v>-6.64</v>
+        <v>-7.75</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>5.25</v>
+        <v>6.16</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>1.6</v>
+        <v>-0.31</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>3.64</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>8.5</v>
+        <v>38.9</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AP6" s="2" t="inlineStr"/>
       <c r="AQ6" s="2" t="inlineStr"/>
@@ -1515,78 +1531,72 @@
         </is>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>2.897</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>2.91</v>
+        <v>0.827</v>
       </c>
       <c r="AW6" s="2" t="n">
-        <v>2.945</v>
+        <v>0.835</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>2.974</v>
+        <v>0.836</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>2.993</v>
+        <v>0.858</v>
       </c>
       <c r="AZ6" s="2" t="n">
-        <v>3.005</v>
+        <v>0.828</v>
       </c>
       <c r="BA6" s="2" t="n">
-        <v>3.037</v>
+        <v>0.831</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>-0.8248</v>
+        <v>-1.538</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>-0.5478</v>
+        <v>-0.3433</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>-0.2399</v>
+        <v>-0.2184</v>
       </c>
       <c r="BE6" s="2" t="n">
-        <v>-0.1192</v>
+        <v>0.0591</v>
       </c>
       <c r="BF6" s="2" t="n">
-        <v>-0.0664</v>
+        <v>-0.0775</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4.236</v>
+        <v>2.886</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>2.9</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="n">
         <v>13</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -1613,7 +1623,7 @@
         </is>
       </c>
       <c r="W7" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
@@ -1626,37 +1636,33 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AE7" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
       <c r="AI7" s="2" t="inlineStr"/>
       <c r="AJ7" s="2" t="n">
-        <v>-7.54</v>
+        <v>-6.71</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>1.09</v>
+        <v>5.86</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>-0.05</v>
+        <v>1.05</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>-0.11</v>
+        <v>4.56</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>-4.4</v>
+        <v>7.7</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="AP7" s="2" t="inlineStr"/>
-      <c r="AQ7" s="2" t="n">
-        <v>14</v>
-      </c>
+      <c r="AQ7" s="2" t="inlineStr"/>
       <c r="AR7" s="2" t="inlineStr"/>
       <c r="AS7" s="2" t="inlineStr"/>
       <c r="AT7" s="2" t="inlineStr">
@@ -1665,58 +1671,58 @@
         </is>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>4.296</v>
+        <v>2.887</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>4.352</v>
+        <v>2.907</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>4.458</v>
+        <v>2.941</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>4.52</v>
+        <v>2.969</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>4.59</v>
+        <v>2.99</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>4.721</v>
+        <v>3.003</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>4.71</v>
+        <v>3.036</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>-1.6553</v>
+        <v>-0.8138</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>-0.9454</v>
+        <v>-0.5403</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>-0.4195</v>
+        <v>-0.2501</v>
       </c>
       <c r="BE7" s="2" t="n">
-        <v>-0.3212</v>
+        <v>-0.1135</v>
       </c>
       <c r="BF7" s="2" t="n">
-        <v>-0.07539999999999999</v>
+        <v>-0.06710000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>6.809</v>
+        <v>4.24</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.97</v>
+        <v>4.58</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -1733,28 +1739,28 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
@@ -1776,32 +1782,34 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr"/>
       <c r="AD8" s="2" t="inlineStr"/>
-      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AF8" s="2" t="inlineStr"/>
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr"/>
       <c r="AI8" s="2" t="inlineStr"/>
       <c r="AJ8" s="2" t="n">
-        <v>-1.4</v>
+        <v>-7.73</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>-2.66</v>
+        <v>1.1</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>-3.32</v>
+        <v>-0.15</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>-4.83</v>
+        <v>-0.11</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>1.8</v>
+        <v>-4.4</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="AP8" s="2" t="inlineStr"/>
       <c r="AQ8" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AR8" s="2" t="inlineStr"/>
       <c r="AS8" s="2" t="inlineStr"/>
@@ -1811,68 +1819,76 @@
         </is>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>6.973</v>
+        <v>4.271</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>7.181</v>
+        <v>4.334</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>7.451</v>
+        <v>4.441</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>7.569</v>
+        <v>4.504</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>7.688</v>
+        <v>4.581</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>7.986</v>
+        <v>4.715</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>8.012</v>
+        <v>4.707</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>-2.8417</v>
+        <v>-1.6112</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>-1.3238</v>
+        <v>-0.9956</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>-0.368</v>
+        <v>-0.4363</v>
       </c>
       <c r="BE8" s="2" t="n">
-        <v>-0.5048</v>
+        <v>-0.3201</v>
       </c>
       <c r="BF8" s="2" t="n">
-        <v>-0.014</v>
+        <v>-0.07729999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.43</v>
+        <v>6.83</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>41.01</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
+        <v>0.97</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
       </c>
@@ -1880,137 +1896,131 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>0111111111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W9" s="2" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>2C</t>
-        </is>
-      </c>
-      <c r="Y9" s="2" t="inlineStr">
-        <is>
-          <t>减速</t>
-        </is>
-      </c>
-      <c r="Z9" s="2" t="inlineStr">
-        <is>
-          <t>2A→2C·17d</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr"/>
       <c r="AA9" s="2" t="inlineStr"/>
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="inlineStr"/>
-      <c r="AE9" s="2" t="n">
-        <v>-1</v>
+      <c r="AE9" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr"/>
       <c r="AI9" s="2" t="inlineStr"/>
       <c r="AJ9" s="2" t="n">
-        <v>17.27</v>
+        <v>-2.05</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>19.59</v>
+        <v>-2.48</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>3.48</v>
+        <v>-1.59</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>7.2</v>
+        <v>-3.75</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>85.59999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="AP9" s="2" t="inlineStr"/>
-      <c r="AQ9" s="2" t="inlineStr"/>
-      <c r="AR9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AQ9" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="AR9" s="2" t="inlineStr"/>
       <c r="AS9" s="2" t="inlineStr"/>
       <c r="AT9" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>3.451</v>
+        <v>6.915</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>3.414</v>
+        <v>7.121</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>3.393</v>
+        <v>7.412</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>3.413</v>
+        <v>7.533</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>3.381</v>
+        <v>7.675</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>3.273</v>
+        <v>7.972</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>3.23</v>
+        <v>8.010999999999999</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>0.6859</v>
+        <v>-2.8013</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>0.008</v>
+        <v>-1.4078</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>0.3042</v>
+        <v>-0.402</v>
       </c>
       <c r="BE9" s="2" t="n">
-        <v>0.1843</v>
+        <v>-0.5077</v>
       </c>
       <c r="BF9" s="2" t="n">
-        <v>0.1727</v>
+        <v>-0.0205</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.493</v>
+        <v>3.463</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>-0.8100000000000001</v>
+        <v>41.01</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -2019,148 +2029,152 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>1111111101</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y10" s="2" t="inlineStr"/>
+          <t>2C</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>减速</t>
+        </is>
+      </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>4+→4·10d ← 4→4+·20d</t>
+          <t>2A→2C·18d</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="inlineStr"/>
-      <c r="AE10" s="2" t="inlineStr"/>
-      <c r="AF10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG10" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AH10" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE10" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF10" s="2" t="inlineStr"/>
+      <c r="AG10" s="2" t="inlineStr"/>
+      <c r="AH10" s="2" t="inlineStr"/>
       <c r="AI10" s="2" t="inlineStr"/>
       <c r="AJ10" s="2" t="n">
-        <v>-19.08</v>
+        <v>17.73</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>1.73</v>
+        <v>20.5</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>3.26</v>
+        <v>3.16</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>4.5</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>8.6</v>
+        <v>86.5</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="AP10" s="2" t="inlineStr"/>
-      <c r="AQ10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR10" s="2" t="inlineStr"/>
+        <v>59</v>
+      </c>
+      <c r="AP10" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="AQ10" s="2" t="inlineStr"/>
+      <c r="AR10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AS10" s="2" t="inlineStr"/>
       <c r="AT10" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>0.495</v>
+        <v>3.454</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>0.493</v>
+        <v>3.426</v>
       </c>
       <c r="AW10" s="2" t="n">
-        <v>0.499</v>
+        <v>3.395</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>0.507</v>
+        <v>3.413</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>0.513</v>
+        <v>3.384</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>0.516</v>
+        <v>3.276</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>0.53</v>
+        <v>3.232</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>-0.6566</v>
+        <v>0.7040999999999999</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>-0.6994</v>
+        <v>0.0346</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>-0.3166</v>
+        <v>0.2837</v>
       </c>
       <c r="BE10" s="2" t="n">
-        <v>-0.0453</v>
+        <v>0.1948</v>
       </c>
       <c r="BF10" s="2" t="n">
-        <v>-0.1908</v>
+        <v>0.1773</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.367</v>
+        <v>0.493</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>9.880000000000001</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -2169,28 +2183,30 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>0010111000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>0010111000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V11" s="2" t="inlineStr">
@@ -2199,21 +2215,17 @@
         </is>
       </c>
       <c r="W11" s="2" t="n">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
-        </is>
-      </c>
-      <c r="Y11" s="2" t="inlineStr">
-        <is>
-          <t>周J超卖·日线纠缠</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr"/>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>4→4+·1d ← 1→4·4d ← 1+→1·7d</t>
+          <t>4+→4·11d</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr"/>
@@ -2222,95 +2234,95 @@
       <c r="AD11" s="2" t="inlineStr"/>
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG11" s="2" t="n">
         <v>-1</v>
-      </c>
-      <c r="AG11" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
       </c>
       <c r="AH11" s="2" t="inlineStr"/>
       <c r="AI11" s="2" t="inlineStr"/>
       <c r="AJ11" s="2" t="n">
-        <v>-5.29</v>
+        <v>-19.04</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>8.25</v>
+        <v>1.67</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>0.17</v>
+        <v>2.48</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>9.609999999999999</v>
+        <v>6.34</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>58.5</v>
+        <v>7.5</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="AP11" s="2" t="inlineStr"/>
-      <c r="AQ11" s="2" t="inlineStr"/>
+      <c r="AQ11" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AR11" s="2" t="inlineStr"/>
       <c r="AS11" s="2" t="inlineStr"/>
       <c r="AT11" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>0.375</v>
+        <v>0.494</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>0.378</v>
+        <v>0.493</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>0.376</v>
+        <v>0.498</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>0.377</v>
+        <v>0.506</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>0.382</v>
+        <v>0.512</v>
       </c>
       <c r="AZ11" s="2" t="n">
-        <v>0.366</v>
+        <v>0.516</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>0.371</v>
+        <v>0.529</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>-0.4024</v>
+        <v>-0.5222</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>-0.0495</v>
+        <v>-0.5985</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>0.0677</v>
+        <v>-0.3271</v>
       </c>
       <c r="BE11" s="2" t="n">
-        <v>0.1593</v>
+        <v>-0.0383</v>
       </c>
       <c r="BF11" s="2" t="n">
-        <v>-0.0529</v>
+        <v>-0.1904</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.754</v>
+        <v>0.373</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-4.85</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -2319,9 +2331,7 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
         <v>2</v>
@@ -2330,19 +2340,19 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0010111010</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0010111000</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
@@ -2351,49 +2361,59 @@
         </is>
       </c>
       <c r="W12" s="2" t="n">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y12" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>4+→4·7d ← 4→4+·10d</t>
+          <t>4→4+·2d ← 1→4·5d ← 1+→1·8d</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr"/>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="inlineStr"/>
-      <c r="AE12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF12" s="2" t="inlineStr"/>
-      <c r="AG12" s="2" t="n">
+      <c r="AE12" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF12" s="2" t="n">
         <v>-1</v>
+      </c>
+      <c r="AG12" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="AH12" s="2" t="inlineStr"/>
       <c r="AI12" s="2" t="inlineStr"/>
       <c r="AJ12" s="2" t="n">
-        <v>-21.3</v>
+        <v>-4.79</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>0.93</v>
+        <v>10</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>2.22</v>
+        <v>1.42</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>2.79</v>
+        <v>11.56</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>13.1</v>
+        <v>57.2</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="AP12" s="2" t="inlineStr"/>
       <c r="AQ12" s="2" t="inlineStr"/>
@@ -2401,82 +2421,76 @@
       <c r="AS12" s="2" t="inlineStr"/>
       <c r="AT12" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU12" s="2" t="n">
-        <v>0.758</v>
+        <v>0.373</v>
       </c>
       <c r="AV12" s="2" t="n">
-        <v>0.759</v>
+        <v>0.377</v>
       </c>
       <c r="AW12" s="2" t="n">
-        <v>0.77</v>
+        <v>0.377</v>
       </c>
       <c r="AX12" s="2" t="n">
-        <v>0.783</v>
+        <v>0.376</v>
       </c>
       <c r="AY12" s="2" t="n">
-        <v>0.787</v>
+        <v>0.382</v>
       </c>
       <c r="AZ12" s="2" t="n">
-        <v>0.786</v>
+        <v>0.366</v>
       </c>
       <c r="BA12" s="2" t="n">
-        <v>0.823</v>
+        <v>0.371</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>-0.8631</v>
+        <v>-0.5206</v>
       </c>
       <c r="BC12" s="2" t="n">
-        <v>-0.8290999999999999</v>
+        <v>0.0141</v>
       </c>
       <c r="BD12" s="2" t="n">
-        <v>-0.3277</v>
+        <v>0.0188</v>
       </c>
       <c r="BE12" s="2" t="n">
-        <v>-0.0526</v>
+        <v>0.1666</v>
       </c>
       <c r="BF12" s="2" t="n">
-        <v>-0.213</v>
+        <v>-0.0479</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>2.719</v>
+        <v>0.756</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4.11</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>-4.85</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="n">
+      <c r="L13" s="2" t="n">
         <v>13</v>
       </c>
+      <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
@@ -2485,16 +2499,16 @@
         <v>1</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V13" s="2" t="inlineStr">
@@ -2503,7 +2517,7 @@
         </is>
       </c>
       <c r="W13" s="2" t="n">
-        <v>50</v>
+        <v>147</v>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
@@ -2511,33 +2525,45 @@
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr"/>
-      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>4+→4·8d ← 4→4+·11d</t>
+        </is>
+      </c>
       <c r="AA13" s="2" t="inlineStr"/>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
-      <c r="AE13" s="2" t="inlineStr"/>
-      <c r="AF13" s="2" t="inlineStr"/>
-      <c r="AG13" s="2" t="inlineStr"/>
+      <c r="AE13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF13" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AG13" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AH13" s="2" t="inlineStr"/>
       <c r="AI13" s="2" t="inlineStr"/>
       <c r="AJ13" s="2" t="n">
-        <v>-6.34</v>
+        <v>-22.19</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>-3.74</v>
+        <v>1.12</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>-3.25</v>
+        <v>1.35</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>-4.04</v>
+        <v>4.39</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>14.4</v>
+        <v>11</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="AP13" s="2" t="inlineStr"/>
       <c r="AQ13" s="2" t="inlineStr"/>
@@ -2549,88 +2575,96 @@
         </is>
       </c>
       <c r="AU13" s="2" t="n">
-        <v>2.789</v>
+        <v>0.756</v>
       </c>
       <c r="AV13" s="2" t="n">
-        <v>2.868</v>
+        <v>0.758</v>
       </c>
       <c r="AW13" s="2" t="n">
-        <v>2.977</v>
+        <v>0.769</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>3.018</v>
+        <v>0.782</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>3.04</v>
+        <v>0.786</v>
       </c>
       <c r="AZ13" s="2" t="n">
-        <v>3.171</v>
+        <v>0.786</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>3.212</v>
+        <v>0.822</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>-2.9216</v>
+        <v>-0.7759</v>
       </c>
       <c r="BC13" s="2" t="n">
-        <v>-1.2647</v>
+        <v>-0.7512</v>
       </c>
       <c r="BD13" s="2" t="n">
-        <v>-0.1163</v>
+        <v>-0.3528</v>
       </c>
       <c r="BE13" s="2" t="n">
-        <v>-0.5944</v>
+        <v>-0.0437</v>
       </c>
       <c r="BF13" s="2" t="n">
-        <v>-0.0634</v>
+        <v>-0.2219</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.322</v>
+        <v>2.722</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>12.17</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+        <v>4.11</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N14" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>0000011100</t>
+          <t>0000000100</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V14" s="2" t="inlineStr">
@@ -2639,52 +2673,42 @@
         </is>
       </c>
       <c r="W14" s="2" t="n">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
-        </is>
-      </c>
-      <c r="Y14" s="2" t="inlineStr">
-        <is>
-          <t>周J超卖·日线纠缠</t>
-        </is>
-      </c>
-      <c r="Z14" s="2" t="inlineStr">
-        <is>
-          <t>4→4+·1d ← 4+→4·7d ← 4→4+·8d</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr"/>
       <c r="AA14" s="2" t="inlineStr"/>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="inlineStr"/>
-      <c r="AE14" s="2" t="inlineStr"/>
-      <c r="AF14" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AG14" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="AE14" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF14" s="2" t="inlineStr"/>
+      <c r="AG14" s="2" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr"/>
       <c r="AI14" s="2" t="inlineStr"/>
       <c r="AJ14" s="2" t="n">
-        <v>-3.9</v>
+        <v>-6.86</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>5.35</v>
+        <v>-3.73</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>-2.3</v>
+        <v>-2.07</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>6.43</v>
+        <v>-2.68</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>63.6</v>
+        <v>11.7</v>
       </c>
       <c r="AO14" s="2" t="n">
         <v>21</v>
@@ -2695,62 +2719,62 @@
       <c r="AS14" s="2" t="inlineStr"/>
       <c r="AT14" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>0.332</v>
+        <v>2.762</v>
       </c>
       <c r="AV14" s="2" t="n">
-        <v>0.337</v>
+        <v>2.843</v>
       </c>
       <c r="AW14" s="2" t="n">
-        <v>0.338</v>
+        <v>2.963</v>
       </c>
       <c r="AX14" s="2" t="n">
-        <v>0.338</v>
+        <v>3.005</v>
       </c>
       <c r="AY14" s="2" t="n">
-        <v>0.341</v>
+        <v>3.038</v>
       </c>
       <c r="AZ14" s="2" t="n">
-        <v>0.326</v>
+        <v>3.164</v>
       </c>
       <c r="BA14" s="2" t="n">
-        <v>0.336</v>
+        <v>3.212</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>-1.0291</v>
+        <v>-2.9018</v>
       </c>
       <c r="BC14" s="2" t="n">
-        <v>-0.2211</v>
+        <v>-1.358</v>
       </c>
       <c r="BD14" s="2" t="n">
-        <v>0.1491</v>
+        <v>-0.1731</v>
       </c>
       <c r="BE14" s="2" t="n">
-        <v>0.0548</v>
+        <v>-0.6018</v>
       </c>
       <c r="BF14" s="2" t="n">
-        <v>-0.039</v>
+        <v>-0.06859999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.059</v>
+        <v>0.326</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>71.16</v>
+        <v>12.17</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -2760,29 +2784,27 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0000011100</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
@@ -2791,47 +2813,59 @@
         </is>
       </c>
       <c r="W15" s="2" t="n">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y15" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>4+→4·12d ← 4→4+·15d</t>
+          <t>4→4+·2d ← 4+→4·8d ← 4→4+·9d</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF15" s="2" t="inlineStr"/>
-      <c r="AG15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF15" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AG15" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AH15" s="2" t="inlineStr"/>
       <c r="AI15" s="2" t="inlineStr"/>
       <c r="AJ15" s="2" t="n">
-        <v>-16.67</v>
+        <v>-4.59</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>-7.19</v>
+        <v>6.65</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>1.29</v>
+        <v>-1.48</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>-1.6</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>21.6</v>
+        <v>61.1</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="AP15" s="2" t="inlineStr"/>
       <c r="AQ15" s="2" t="inlineStr"/>
@@ -2839,62 +2873,62 @@
       <c r="AS15" s="2" t="inlineStr"/>
       <c r="AT15" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU15" s="2" t="n">
-        <v>1.061</v>
+        <v>0.329</v>
       </c>
       <c r="AV15" s="2" t="n">
-        <v>1.078</v>
+        <v>0.335</v>
       </c>
       <c r="AW15" s="2" t="n">
-        <v>1.116</v>
+        <v>0.338</v>
       </c>
       <c r="AX15" s="2" t="n">
-        <v>1.127</v>
+        <v>0.338</v>
       </c>
       <c r="AY15" s="2" t="n">
-        <v>1.128</v>
+        <v>0.341</v>
       </c>
       <c r="AZ15" s="2" t="n">
-        <v>1.178</v>
+        <v>0.326</v>
       </c>
       <c r="BA15" s="2" t="n">
-        <v>1.297</v>
+        <v>0.336</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>-2.2119</v>
+        <v>-1.2427</v>
       </c>
       <c r="BC15" s="2" t="n">
-        <v>-1.1776</v>
+        <v>-0.2382</v>
       </c>
       <c r="BD15" s="2" t="n">
-        <v>-0.1113</v>
+        <v>0.0607</v>
       </c>
       <c r="BE15" s="2" t="n">
-        <v>-0.707</v>
+        <v>0.0399</v>
       </c>
       <c r="BF15" s="2" t="n">
-        <v>-0.1667</v>
+        <v>-0.0459</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.004</v>
+        <v>1.073</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>-0.29</v>
+        <v>71.16</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -2903,41 +2937,39 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="n">
         <v>9</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
+          <t>0000000100</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
           <t>0000000000</t>
         </is>
       </c>
-      <c r="U16" s="2" t="inlineStr">
-        <is>
-          <t>0000000000</t>
-        </is>
-      </c>
       <c r="V16" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
       <c r="W16" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
@@ -2945,38 +2977,46 @@
         </is>
       </c>
       <c r="Y16" s="2" t="inlineStr"/>
-      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>4+→4·13d ← 4→4+·16d</t>
+        </is>
+      </c>
       <c r="AA16" s="2" t="inlineStr"/>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
       <c r="AD16" s="2" t="inlineStr"/>
-      <c r="AE16" s="2" t="inlineStr"/>
-      <c r="AF16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF16" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AG16" s="2" t="inlineStr"/>
       <c r="AH16" s="2" t="inlineStr"/>
       <c r="AI16" s="2" t="inlineStr"/>
       <c r="AJ16" s="2" t="n">
-        <v>-15.15</v>
+        <v>-16.6</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>-8.779999999999999</v>
+        <v>-6.05</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>-2.44</v>
+        <v>3.83</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>-1.95</v>
+        <v>-0.25</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>-0.5</v>
+        <v>20.6</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="AP16" s="2" t="inlineStr"/>
-      <c r="AQ16" s="2" t="n">
-        <v>11</v>
-      </c>
+      <c r="AQ16" s="2" t="inlineStr"/>
       <c r="AR16" s="2" t="inlineStr"/>
       <c r="AS16" s="2" t="inlineStr"/>
       <c r="AT16" s="2" t="inlineStr">
@@ -2985,58 +3025,58 @@
         </is>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>1.029</v>
+        <v>1.064</v>
       </c>
       <c r="AV16" s="2" t="n">
-        <v>1.054</v>
+        <v>1.076</v>
       </c>
       <c r="AW16" s="2" t="n">
-        <v>1.09</v>
+        <v>1.111</v>
       </c>
       <c r="AX16" s="2" t="n">
-        <v>1.115</v>
+        <v>1.126</v>
       </c>
       <c r="AY16" s="2" t="n">
-        <v>1.148</v>
+        <v>1.127</v>
       </c>
       <c r="AZ16" s="2" t="n">
-        <v>1.184</v>
+        <v>1.175</v>
       </c>
       <c r="BA16" s="2" t="n">
-        <v>1.228</v>
+        <v>1.296</v>
       </c>
       <c r="BB16" s="2" t="n">
-        <v>-2.5727</v>
+        <v>-1.8733</v>
       </c>
       <c r="BC16" s="2" t="n">
-        <v>-1.3651</v>
+        <v>-1.1914</v>
       </c>
       <c r="BD16" s="2" t="n">
-        <v>-0.5793</v>
+        <v>-0.1123</v>
       </c>
       <c r="BE16" s="2" t="n">
-        <v>-0.6806</v>
+        <v>-0.6667999999999999</v>
       </c>
       <c r="BF16" s="2" t="n">
-        <v>-0.1515</v>
+        <v>-0.166</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.893</v>
+        <v>1.017</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>4.85</v>
+        <v>-0.29</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -3045,140 +3085,144 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M17" s="2" t="n">
         <v>9</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V17" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W17" s="2" t="n">
-        <v>299</v>
+        <v>61</v>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr"/>
-      <c r="Z17" s="2" t="inlineStr">
-        <is>
-          <t>2C→2A·4d</t>
-        </is>
-      </c>
+      <c r="Z17" s="2" t="inlineStr"/>
       <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
       <c r="AD17" s="2" t="inlineStr"/>
-      <c r="AE17" s="2" t="inlineStr"/>
+      <c r="AE17" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AF17" s="2" t="inlineStr"/>
       <c r="AG17" s="2" t="inlineStr"/>
       <c r="AH17" s="2" t="inlineStr"/>
       <c r="AI17" s="2" t="inlineStr"/>
       <c r="AJ17" s="2" t="n">
-        <v>16.51</v>
+        <v>-14.74</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>1.71</v>
+        <v>-7.56</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>-5.38</v>
+        <v>-0.39</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>-9.06</v>
+        <v>-0.15</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>-7.2</v>
+        <v>-0.7</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="AP17" s="2" t="inlineStr"/>
-      <c r="AQ17" s="2" t="inlineStr"/>
+      <c r="AQ17" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="AR17" s="2" t="inlineStr"/>
       <c r="AS17" s="2" t="inlineStr"/>
       <c r="AT17" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU17" s="2" t="n">
-        <v>0.92</v>
+        <v>1.022</v>
       </c>
       <c r="AV17" s="2" t="n">
-        <v>0.963</v>
+        <v>1.046</v>
       </c>
       <c r="AW17" s="2" t="n">
-        <v>1.016</v>
+        <v>1.084</v>
       </c>
       <c r="AX17" s="2" t="n">
-        <v>1.033</v>
+        <v>1.109</v>
       </c>
       <c r="AY17" s="2" t="n">
-        <v>1.066</v>
+        <v>1.144</v>
       </c>
       <c r="AZ17" s="2" t="n">
-        <v>1.167</v>
+        <v>1.181</v>
       </c>
       <c r="BA17" s="2" t="n">
-        <v>1.03</v>
+        <v>1.226</v>
       </c>
       <c r="BB17" s="2" t="n">
-        <v>-4.4706</v>
+        <v>-2.5357</v>
       </c>
       <c r="BC17" s="2" t="n">
-        <v>-1.554</v>
+        <v>-1.3398</v>
       </c>
       <c r="BD17" s="2" t="n">
-        <v>-1.0542</v>
+        <v>-0.6205000000000001</v>
       </c>
       <c r="BE17" s="2" t="n">
-        <v>-0.4634</v>
+        <v>-0.6693</v>
       </c>
       <c r="BF17" s="2" t="n">
-        <v>0.1651</v>
+        <v>-0.1474</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.864</v>
+        <v>0.875</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>73.68000000000001</v>
+        <v>4.85</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -3188,27 +3232,29 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N18" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>0111111001</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>1111111111</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="V18" s="2" t="inlineStr">
@@ -3217,100 +3263,90 @@
         </is>
       </c>
       <c r="W18" s="2" t="n">
-        <v>53</v>
+        <v>299</v>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>2C</t>
-        </is>
-      </c>
-      <c r="Y18" s="2" t="inlineStr">
-        <is>
-          <t>减速</t>
-        </is>
-      </c>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr"/>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·13d</t>
+          <t>2C→2A·5d</t>
         </is>
       </c>
       <c r="AA18" s="2" t="inlineStr"/>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="AE18" s="2" t="inlineStr"/>
       <c r="AF18" s="2" t="inlineStr"/>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="inlineStr"/>
       <c r="AI18" s="2" t="inlineStr"/>
       <c r="AJ18" s="2" t="n">
-        <v>7.85</v>
+        <v>15.53</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>19.84</v>
+        <v>-0.49</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>5.55</v>
+        <v>-5.57</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>10.78</v>
+        <v>-10.58</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>-7.7</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="AP18" s="2" t="inlineStr"/>
       <c r="AQ18" s="2" t="inlineStr"/>
-      <c r="AR18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AR18" s="2" t="inlineStr"/>
       <c r="AS18" s="2" t="inlineStr"/>
       <c r="AT18" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AU18" s="2" t="n">
-        <v>0.865</v>
+        <v>0.906</v>
       </c>
       <c r="AV18" s="2" t="n">
-        <v>0.856</v>
+        <v>0.947</v>
       </c>
       <c r="AW18" s="2" t="n">
-        <v>0.848</v>
+        <v>1.008</v>
       </c>
       <c r="AX18" s="2" t="n">
-        <v>0.845</v>
+        <v>1.026</v>
       </c>
       <c r="AY18" s="2" t="n">
-        <v>0.832</v>
+        <v>1.062</v>
       </c>
       <c r="AZ18" s="2" t="n">
-        <v>0.806</v>
+        <v>1.165</v>
       </c>
       <c r="BA18" s="2" t="n">
-        <v>0.8</v>
+        <v>1.031</v>
       </c>
       <c r="BB18" s="2" t="n">
-        <v>0.8586</v>
+        <v>-4.5679</v>
       </c>
       <c r="BC18" s="2" t="n">
-        <v>0.3302</v>
+        <v>-1.7029</v>
       </c>
       <c r="BD18" s="2" t="n">
-        <v>0.2995</v>
+        <v>-0.9969</v>
       </c>
       <c r="BE18" s="2" t="n">
-        <v>0.2902</v>
+        <v>-0.5215</v>
       </c>
       <c r="BF18" s="2" t="n">
-        <v>0.0785</v>
+        <v>0.1553</v>
       </c>
     </row>
     <row r="19">
@@ -3325,7 +3361,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.011</v>
+        <v>1.006</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>-8.65</v>
@@ -3342,20 +3378,20 @@
       </c>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>0000000010</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
@@ -3369,7 +3405,7 @@
         </is>
       </c>
       <c r="W19" s="2" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
@@ -3383,37 +3419,39 @@
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>4→4+·14d</t>
+          <t>4→4+·15d</t>
         </is>
       </c>
       <c r="AA19" s="2" t="inlineStr"/>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="inlineStr"/>
-      <c r="AE19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AF19" s="2" t="inlineStr"/>
       <c r="AG19" s="2" t="inlineStr"/>
-      <c r="AH19" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AH19" s="2" t="inlineStr"/>
       <c r="AI19" s="2" t="inlineStr"/>
       <c r="AJ19" s="2" t="n">
-        <v>-54.22</v>
+        <v>-53.4</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>-12.4</v>
+        <v>-12.75</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>4.52</v>
+        <v>2.94</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>10.15</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>24.5</v>
+        <v>23.1</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="AP19" s="2" t="inlineStr"/>
       <c r="AQ19" s="2" t="inlineStr"/>
@@ -3425,40 +3463,40 @@
         </is>
       </c>
       <c r="AU19" s="2" t="n">
-        <v>1.01</v>
+        <v>1.009</v>
       </c>
       <c r="AV19" s="2" t="n">
-        <v>1.006</v>
+        <v>1.005</v>
       </c>
       <c r="AW19" s="2" t="n">
         <v>1.014</v>
       </c>
       <c r="AX19" s="2" t="n">
-        <v>1.026</v>
+        <v>1.023</v>
       </c>
       <c r="AY19" s="2" t="n">
-        <v>1.067</v>
+        <v>1.064</v>
       </c>
       <c r="AZ19" s="2" t="n">
-        <v>1.074</v>
+        <v>1.073</v>
       </c>
       <c r="BA19" s="2" t="n">
-        <v>1.207</v>
+        <v>1.204</v>
       </c>
       <c r="BB19" s="2" t="n">
-        <v>-0.5168</v>
+        <v>-0.5478</v>
       </c>
       <c r="BC19" s="2" t="n">
-        <v>-0.3515</v>
+        <v>-0.2527</v>
       </c>
       <c r="BD19" s="2" t="n">
-        <v>-0.4588</v>
+        <v>-0.5405</v>
       </c>
       <c r="BE19" s="2" t="n">
-        <v>-0.444</v>
+        <v>-0.4131</v>
       </c>
       <c r="BF19" s="2" t="n">
-        <v>-0.5422</v>
+        <v>-0.534</v>
       </c>
     </row>
     <row r="20">
@@ -3473,7 +3511,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.713</v>
+        <v>1.717</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>-7.05</v>
@@ -3488,7 +3526,7 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
@@ -3497,7 +3535,7 @@
         <v>2</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3544,7 @@
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
@@ -3515,7 +3553,7 @@
         </is>
       </c>
       <c r="W20" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
@@ -3525,7 +3563,7 @@
       <c r="Y20" s="2" t="inlineStr"/>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>4+→4·7d ← 4→4+·10d ← 2A→4·20d</t>
+          <t>4+→4·8d ← 4→4+·11d</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr"/>
@@ -3542,22 +3580,22 @@
       <c r="AH20" s="2" t="inlineStr"/>
       <c r="AI20" s="2" t="inlineStr"/>
       <c r="AJ20" s="2" t="n">
-        <v>-22.29</v>
+        <v>-22.41</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>-1.15</v>
+        <v>-0.96</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>2.67</v>
+        <v>1.72</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>2.81</v>
+        <v>3.97</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>9.300000000000001</v>
+        <v>7.1</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AP20" s="2" t="inlineStr"/>
       <c r="AQ20" s="2" t="inlineStr"/>
@@ -3565,44 +3603,44 @@
       <c r="AS20" s="2" t="inlineStr"/>
       <c r="AT20" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU20" s="2" t="n">
-        <v>1.726</v>
+        <v>1.721</v>
       </c>
       <c r="AV20" s="2" t="n">
-        <v>1.735</v>
+        <v>1.731</v>
       </c>
       <c r="AW20" s="2" t="n">
-        <v>1.767</v>
+        <v>1.762</v>
       </c>
       <c r="AX20" s="2" t="n">
-        <v>1.803</v>
+        <v>1.797</v>
       </c>
       <c r="AY20" s="2" t="n">
-        <v>1.816</v>
+        <v>1.814</v>
       </c>
       <c r="AZ20" s="2" t="n">
-        <v>1.811</v>
+        <v>1.81</v>
       </c>
       <c r="BA20" s="2" t="n">
-        <v>1.875</v>
+        <v>1.873</v>
       </c>
       <c r="BB20" s="2" t="n">
-        <v>-1.1406</v>
+        <v>-1.0621</v>
       </c>
       <c r="BC20" s="2" t="n">
-        <v>-1.0099</v>
+        <v>-0.9117</v>
       </c>
       <c r="BD20" s="2" t="n">
-        <v>-0.3407</v>
+        <v>-0.3463</v>
       </c>
       <c r="BE20" s="2" t="n">
-        <v>-0.1052</v>
+        <v>-0.1003</v>
       </c>
       <c r="BF20" s="2" t="n">
-        <v>-0.2229</v>
+        <v>-0.2241</v>
       </c>
     </row>
     <row r="21">
@@ -3617,7 +3655,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.356</v>
+        <v>2.345</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>110.91</v>
@@ -3645,7 +3683,7 @@
         <v>8</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
@@ -3654,7 +3692,7 @@
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>0111111011</t>
+          <t>0111111001</t>
         </is>
       </c>
       <c r="V21" s="2" t="inlineStr">
@@ -3663,7 +3701,7 @@
         </is>
       </c>
       <c r="W21" s="2" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
@@ -3677,34 +3715,38 @@
       <c r="AC21" s="2" t="inlineStr"/>
       <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="inlineStr"/>
-      <c r="AF21" s="2" t="inlineStr"/>
+      <c r="AF21" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AG21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AH21" s="2" t="inlineStr"/>
+      <c r="AH21" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AI21" s="2" t="inlineStr"/>
       <c r="AJ21" s="2" t="n">
-        <v>28.63</v>
+        <v>28.59</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>30.63</v>
+        <v>29.69</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>1.18</v>
+        <v>-0.54</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>14.75</v>
+        <v>13.9</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>86.09999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="AP21" s="2" t="inlineStr"/>
       <c r="AQ21" s="2" t="inlineStr"/>
       <c r="AR21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS21" s="2" t="inlineStr"/>
       <c r="AT21" s="2" t="inlineStr">
@@ -3713,40 +3755,40 @@
         </is>
       </c>
       <c r="AU21" s="2" t="n">
-        <v>2.37</v>
+        <v>2.359</v>
       </c>
       <c r="AV21" s="2" t="n">
-        <v>2.36</v>
+        <v>2.364</v>
       </c>
       <c r="AW21" s="2" t="n">
-        <v>2.307</v>
+        <v>2.314</v>
       </c>
       <c r="AX21" s="2" t="n">
-        <v>2.279</v>
+        <v>2.283</v>
       </c>
       <c r="AY21" s="2" t="n">
-        <v>2.254</v>
+        <v>2.258</v>
       </c>
       <c r="AZ21" s="2" t="n">
-        <v>2.217</v>
+        <v>2.22</v>
       </c>
       <c r="BA21" s="2" t="n">
-        <v>2.044</v>
+        <v>2.046</v>
       </c>
       <c r="BB21" s="2" t="n">
-        <v>0.7547</v>
+        <v>0.5505</v>
       </c>
       <c r="BC21" s="2" t="n">
-        <v>0.8098</v>
+        <v>0.7678</v>
       </c>
       <c r="BD21" s="2" t="n">
-        <v>0.6761</v>
+        <v>0.6449</v>
       </c>
       <c r="BE21" s="2" t="n">
-        <v>0.3483</v>
+        <v>0.3353</v>
       </c>
       <c r="BF21" s="2" t="n">
-        <v>0.2863</v>
+        <v>0.2859</v>
       </c>
     </row>
     <row r="22">
@@ -3761,7 +3803,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.342</v>
+        <v>1.338</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>3.97</v>
@@ -3809,7 +3851,7 @@
         </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
@@ -3830,26 +3872,26 @@
       <c r="AH22" s="2" t="inlineStr"/>
       <c r="AI22" s="2" t="inlineStr"/>
       <c r="AJ22" s="2" t="n">
-        <v>-28.82</v>
+        <v>-29.25</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>-16.69</v>
+        <v>-16.96</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>-4.9</v>
+        <v>-3.94</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>-2.68</v>
+        <v>-1.79</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>-0.6</v>
+        <v>-1</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="AP22" s="2" t="inlineStr"/>
       <c r="AQ22" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AR22" s="2" t="inlineStr"/>
       <c r="AS22" s="2" t="inlineStr"/>
@@ -3859,40 +3901,40 @@
         </is>
       </c>
       <c r="AU22" s="2" t="n">
-        <v>1.381</v>
+        <v>1.36</v>
       </c>
       <c r="AV22" s="2" t="n">
-        <v>1.416</v>
+        <v>1.407</v>
       </c>
       <c r="AW22" s="2" t="n">
-        <v>1.455</v>
+        <v>1.448</v>
       </c>
       <c r="AX22" s="2" t="n">
-        <v>1.493</v>
+        <v>1.483</v>
       </c>
       <c r="AY22" s="2" t="n">
-        <v>1.555</v>
+        <v>1.55</v>
       </c>
       <c r="AZ22" s="2" t="n">
-        <v>1.68</v>
+        <v>1.673</v>
       </c>
       <c r="BA22" s="2" t="n">
-        <v>1.798</v>
+        <v>1.796</v>
       </c>
       <c r="BB22" s="2" t="n">
-        <v>-2.0794</v>
+        <v>-2.2152</v>
       </c>
       <c r="BC22" s="2" t="n">
-        <v>-1.4063</v>
+        <v>-1.4796</v>
       </c>
       <c r="BD22" s="2" t="n">
-        <v>-0.6909</v>
+        <v>-0.7996</v>
       </c>
       <c r="BE22" s="2" t="n">
-        <v>-0.9959</v>
+        <v>-1.0283</v>
       </c>
       <c r="BF22" s="2" t="n">
-        <v>-0.2882</v>
+        <v>-0.2925</v>
       </c>
     </row>
     <row r="23">
@@ -3930,7 +3972,7 @@
         <v>9</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -3939,7 +3981,7 @@
         <v>1</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
@@ -3948,7 +3990,7 @@
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="V23" s="2" t="inlineStr">
@@ -3967,35 +4009,39 @@
       <c r="Y23" s="2" t="inlineStr"/>
       <c r="Z23" s="2" t="inlineStr">
         <is>
-          <t>2C→2A·12d</t>
+          <t>2C→2A·13d</t>
         </is>
       </c>
       <c r="AA23" s="2" t="inlineStr"/>
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
-      <c r="AE23" s="2" t="inlineStr"/>
+      <c r="AE23" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AF23" s="2" t="inlineStr"/>
       <c r="AG23" s="2" t="inlineStr"/>
       <c r="AH23" s="2" t="inlineStr"/>
       <c r="AI23" s="2" t="inlineStr"/>
       <c r="AJ23" s="2" t="n">
-        <v>14.05</v>
+        <v>13.77</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>-1.3</v>
+        <v>-1.46</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>-8.699999999999999</v>
+        <v>-4.48</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>-22.04</v>
+        <v>-23.34</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>3.2</v>
+        <v>1.7</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AP23" s="2" t="inlineStr"/>
       <c r="AQ23" s="2" t="inlineStr"/>
@@ -4007,40 +4053,40 @@
         </is>
       </c>
       <c r="AU23" s="2" t="n">
-        <v>0.841</v>
+        <v>0.83</v>
       </c>
       <c r="AV23" s="2" t="n">
-        <v>0.893</v>
+        <v>0.877</v>
       </c>
       <c r="AW23" s="2" t="n">
-        <v>0.972</v>
+        <v>0.96</v>
       </c>
       <c r="AX23" s="2" t="n">
-        <v>0.991</v>
+        <v>0.984</v>
       </c>
       <c r="AY23" s="2" t="n">
-        <v>1.004</v>
+        <v>1.001</v>
       </c>
       <c r="AZ23" s="2" t="n">
-        <v>1.104</v>
+        <v>1.101</v>
       </c>
       <c r="BA23" s="2" t="n">
-        <v>0.975</v>
+        <v>0.976</v>
       </c>
       <c r="BB23" s="2" t="n">
-        <v>-5.8576</v>
+        <v>-5.7327</v>
       </c>
       <c r="BC23" s="2" t="n">
-        <v>-2.4715</v>
+        <v>-2.7839</v>
       </c>
       <c r="BD23" s="2" t="n">
-        <v>-0.6881</v>
+        <v>-0.638</v>
       </c>
       <c r="BE23" s="2" t="n">
-        <v>-0.667</v>
+        <v>-0.6761</v>
       </c>
       <c r="BF23" s="2" t="n">
-        <v>0.1405</v>
+        <v>0.1377</v>
       </c>
     </row>
     <row r="24">
@@ -4055,7 +4101,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.265</v>
+        <v>1.279</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>46.54</v>
@@ -4076,28 +4122,28 @@
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>6</v>
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
+          <t>0111111100</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
           <t>0110111100</t>
         </is>
       </c>
-      <c r="U24" s="2" t="inlineStr">
-        <is>
-          <t>0100111110</t>
-        </is>
-      </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="W24" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
@@ -4111,15 +4157,17 @@
       </c>
       <c r="Z24" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·12d</t>
+          <t>2A→2C·13d</t>
         </is>
       </c>
       <c r="AA24" s="2" t="inlineStr"/>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="inlineStr"/>
       <c r="AD24" s="2" t="inlineStr"/>
-      <c r="AE24" s="2" t="n">
-        <v>-1</v>
+      <c r="AE24" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="AF24" s="2" t="n">
         <v>-1</v>
@@ -4130,24 +4178,26 @@
         </is>
       </c>
       <c r="AH24" s="2" t="inlineStr"/>
-      <c r="AI24" s="2" t="inlineStr"/>
+      <c r="AI24" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AJ24" s="2" t="n">
-        <v>24.26</v>
+        <v>24.79</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>18.77</v>
+        <v>19.8</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>0.4</v>
+        <v>2.94</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>3.02</v>
+        <v>5.56</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>68.2</v>
+        <v>68.5</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="AP24" s="2" t="inlineStr"/>
       <c r="AQ24" s="2" t="inlineStr"/>
@@ -4159,40 +4209,40 @@
         </is>
       </c>
       <c r="AU24" s="2" t="n">
-        <v>1.277</v>
+        <v>1.278</v>
       </c>
       <c r="AV24" s="2" t="n">
-        <v>1.272</v>
+        <v>1.274</v>
       </c>
       <c r="AW24" s="2" t="n">
         <v>1.272</v>
       </c>
       <c r="AX24" s="2" t="n">
-        <v>1.288</v>
+        <v>1.286</v>
       </c>
       <c r="AY24" s="2" t="n">
-        <v>1.274</v>
+        <v>1.276</v>
       </c>
       <c r="AZ24" s="2" t="n">
-        <v>1.241</v>
+        <v>1.242</v>
       </c>
       <c r="BA24" s="2" t="n">
-        <v>1.208</v>
+        <v>1.21</v>
       </c>
       <c r="BB24" s="2" t="n">
-        <v>0.1367</v>
+        <v>0.0944</v>
       </c>
       <c r="BC24" s="2" t="n">
-        <v>-0.2955</v>
+        <v>-0.2741</v>
       </c>
       <c r="BD24" s="2" t="n">
-        <v>0.3603</v>
+        <v>0.3513</v>
       </c>
       <c r="BE24" s="2" t="n">
-        <v>0.0888</v>
+        <v>0.1001</v>
       </c>
       <c r="BF24" s="2" t="n">
-        <v>0.2426</v>
+        <v>0.2479</v>
       </c>
     </row>
     <row r="25">
@@ -4207,7 +4257,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.717</v>
+        <v>0.723</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>3.22</v>
@@ -4257,7 +4307,7 @@
         </is>
       </c>
       <c r="W25" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
@@ -4280,26 +4330,26 @@
       <c r="AH25" s="2" t="inlineStr"/>
       <c r="AI25" s="2" t="inlineStr"/>
       <c r="AJ25" s="2" t="n">
-        <v>-29.33</v>
+        <v>-29.2</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>-18.1</v>
+        <v>-17.44</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>-2.33</v>
+        <v>-1.73</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>-2.15</v>
+        <v>-0.65</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="AP25" s="2" t="inlineStr"/>
       <c r="AQ25" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AR25" s="2" t="inlineStr"/>
       <c r="AS25" s="2" t="inlineStr"/>
@@ -4309,40 +4359,40 @@
         </is>
       </c>
       <c r="AU25" s="2" t="n">
-        <v>0.736</v>
+        <v>0.729</v>
       </c>
       <c r="AV25" s="2" t="n">
-        <v>0.753</v>
+        <v>0.748</v>
       </c>
       <c r="AW25" s="2" t="n">
-        <v>0.777</v>
+        <v>0.774</v>
       </c>
       <c r="AX25" s="2" t="n">
-        <v>0.791</v>
+        <v>0.787</v>
       </c>
       <c r="AY25" s="2" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="AZ25" s="2" t="n">
-        <v>0.891</v>
+        <v>0.888</v>
       </c>
       <c r="BA25" s="2" t="n">
-        <v>0.982</v>
+        <v>0.981</v>
       </c>
       <c r="BB25" s="2" t="n">
-        <v>-2.4799</v>
+        <v>-2.451</v>
       </c>
       <c r="BC25" s="2" t="n">
-        <v>-1.2595</v>
+        <v>-1.3449</v>
       </c>
       <c r="BD25" s="2" t="n">
-        <v>-0.4956</v>
+        <v>-0.5493</v>
       </c>
       <c r="BE25" s="2" t="n">
-        <v>-1.0848</v>
+        <v>-1.0903</v>
       </c>
       <c r="BF25" s="2" t="n">
-        <v>-0.2933</v>
+        <v>-0.292</v>
       </c>
     </row>
     <row r="26">
@@ -4357,7 +4407,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.522</v>
+        <v>0.523</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>3.91</v>
@@ -4380,7 +4430,7 @@
         <v>13</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
@@ -4417,35 +4467,39 @@
       <c r="Y26" s="2" t="inlineStr"/>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>2C→2A·19d</t>
+          <t>2C→2A·20d</t>
         </is>
       </c>
       <c r="AA26" s="2" t="inlineStr"/>
       <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
-      <c r="AE26" s="2" t="inlineStr"/>
+      <c r="AE26" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AF26" s="2" t="inlineStr"/>
       <c r="AG26" s="2" t="inlineStr"/>
       <c r="AH26" s="2" t="inlineStr"/>
       <c r="AI26" s="2" t="inlineStr"/>
       <c r="AJ26" s="2" t="n">
-        <v>9.67</v>
+        <v>9.48</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>-3.14</v>
+        <v>-3.12</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>-9.74</v>
+        <v>-4.91</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>-20.8</v>
+        <v>-22.28</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>6.5</v>
+        <v>4.8</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AP26" s="2" t="inlineStr"/>
       <c r="AQ26" s="2" t="inlineStr"/>
@@ -4453,44 +4507,44 @@
       <c r="AS26" s="2" t="inlineStr"/>
       <c r="AT26" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU26" s="2" t="n">
-        <v>0.545</v>
+        <v>0.537</v>
       </c>
       <c r="AV26" s="2" t="n">
-        <v>0.579</v>
+        <v>0.569</v>
       </c>
       <c r="AW26" s="2" t="n">
-        <v>0.633</v>
+        <v>0.625</v>
       </c>
       <c r="AX26" s="2" t="n">
-        <v>0.643</v>
+        <v>0.638</v>
       </c>
       <c r="AY26" s="2" t="n">
-        <v>0.648</v>
+        <v>0.647</v>
       </c>
       <c r="AZ26" s="2" t="n">
-        <v>0.715</v>
+        <v>0.713</v>
       </c>
       <c r="BA26" s="2" t="n">
-        <v>0.644</v>
+        <v>0.645</v>
       </c>
       <c r="BB26" s="2" t="n">
-        <v>-6.1583</v>
+        <v>-5.9869</v>
       </c>
       <c r="BC26" s="2" t="n">
-        <v>-2.3924</v>
+        <v>-2.7022</v>
       </c>
       <c r="BD26" s="2" t="n">
-        <v>-0.5481</v>
+        <v>-0.5097</v>
       </c>
       <c r="BE26" s="2" t="n">
-        <v>-0.7674</v>
+        <v>-0.7603</v>
       </c>
       <c r="BF26" s="2" t="n">
-        <v>0.09669999999999999</v>
+        <v>0.0948</v>
       </c>
     </row>
     <row r="27">
@@ -4505,7 +4559,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2.064</v>
+        <v>2.058</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>2.27</v>
@@ -4524,9 +4578,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
         <v>1</v>
       </c>
@@ -4555,7 +4607,7 @@
         </is>
       </c>
       <c r="W27" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
@@ -4574,26 +4626,26 @@
       <c r="AH27" s="2" t="inlineStr"/>
       <c r="AI27" s="2" t="inlineStr"/>
       <c r="AJ27" s="2" t="n">
-        <v>-30.85</v>
+        <v>-31.18</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>-18.57</v>
+        <v>-18.85</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>-4.07</v>
+        <v>-3.85</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>-2.97</v>
+        <v>-2.43</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>-1.7</v>
+        <v>-2</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AP27" s="2" t="inlineStr"/>
       <c r="AQ27" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AR27" s="2" t="inlineStr"/>
       <c r="AS27" s="2" t="inlineStr"/>
@@ -4603,40 +4655,40 @@
         </is>
       </c>
       <c r="AU27" s="2" t="n">
-        <v>2.129</v>
+        <v>2.097</v>
       </c>
       <c r="AV27" s="2" t="n">
-        <v>2.179</v>
+        <v>2.165</v>
       </c>
       <c r="AW27" s="2" t="n">
-        <v>2.245</v>
+        <v>2.233</v>
       </c>
       <c r="AX27" s="2" t="n">
-        <v>2.292</v>
+        <v>2.279</v>
       </c>
       <c r="AY27" s="2" t="n">
-        <v>2.388</v>
+        <v>2.381</v>
       </c>
       <c r="AZ27" s="2" t="n">
-        <v>2.6</v>
+        <v>2.59</v>
       </c>
       <c r="BA27" s="2" t="n">
-        <v>2.835</v>
+        <v>2.833</v>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>-2.1392</v>
+        <v>-2.2243</v>
       </c>
       <c r="BC27" s="2" t="n">
-        <v>-1.2899</v>
+        <v>-1.4254</v>
       </c>
       <c r="BD27" s="2" t="n">
-        <v>-0.6471</v>
+        <v>-0.729</v>
       </c>
       <c r="BE27" s="2" t="n">
-        <v>-1.0579</v>
+        <v>-1.0784</v>
       </c>
       <c r="BF27" s="2" t="n">
-        <v>-0.3085</v>
+        <v>-0.3118</v>
       </c>
     </row>
     <row r="28">
@@ -4651,7 +4703,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.793</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>3.87</v>
@@ -4671,7 +4723,7 @@
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>2</v>
@@ -4701,7 +4753,7 @@
         </is>
       </c>
       <c r="W28" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
@@ -4714,25 +4766,27 @@
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
-      <c r="AE28" s="2" t="inlineStr"/>
+      <c r="AE28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AF28" s="2" t="inlineStr"/>
       <c r="AG28" s="2" t="inlineStr"/>
       <c r="AH28" s="2" t="inlineStr"/>
       <c r="AI28" s="2" t="inlineStr"/>
       <c r="AJ28" s="2" t="n">
-        <v>-18.47</v>
+        <v>-18.03</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>-12.78</v>
+        <v>-10.26</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>-4.08</v>
+        <v>0.08</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>-5.15</v>
+        <v>-1.85</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>-5.7</v>
+        <v>-5.1</v>
       </c>
       <c r="AO28" s="2" t="inlineStr"/>
       <c r="AP28" s="2" t="inlineStr"/>
@@ -4745,40 +4799,40 @@
         </is>
       </c>
       <c r="AU28" s="2" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="AV28" s="2" t="n">
-        <v>0.849</v>
+        <v>0.841</v>
       </c>
       <c r="AW28" s="2" t="n">
-        <v>0.885</v>
+        <v>0.88</v>
       </c>
       <c r="AX28" s="2" t="n">
-        <v>0.907</v>
+        <v>0.902</v>
       </c>
       <c r="AY28" s="2" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="AZ28" s="2" t="n">
-        <v>1.016</v>
+        <v>1.013</v>
       </c>
       <c r="BA28" s="2" t="n">
-        <v>1.024</v>
+        <v>1.023</v>
       </c>
       <c r="BB28" s="2" t="n">
-        <v>-3.3313</v>
+        <v>-3.2848</v>
       </c>
       <c r="BC28" s="2" t="n">
-        <v>-1.8203</v>
+        <v>-1.8214</v>
       </c>
       <c r="BD28" s="2" t="n">
-        <v>-0.6035</v>
+        <v>-0.6671</v>
       </c>
       <c r="BE28" s="2" t="n">
-        <v>-0.9025</v>
+        <v>-0.9473</v>
       </c>
       <c r="BF28" s="2" t="n">
-        <v>-0.1847</v>
+        <v>-0.1803</v>
       </c>
     </row>
     <row r="29">
@@ -4793,7 +4847,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.43</v>
+        <v>1.405</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>5.56</v>
@@ -4847,7 +4901,7 @@
       <c r="Y29" s="2" t="inlineStr"/>
       <c r="Z29" s="2" t="inlineStr">
         <is>
-          <t>2C→2A·5d</t>
+          <t>2C→2A·6d</t>
         </is>
       </c>
       <c r="AA29" s="2" t="inlineStr"/>
@@ -4860,27 +4914,25 @@
       <c r="AH29" s="2" t="inlineStr"/>
       <c r="AI29" s="2" t="inlineStr"/>
       <c r="AJ29" s="2" t="n">
-        <v>4.83</v>
+        <v>4.08</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>-1.82</v>
+        <v>-3.63</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>-4.15</v>
+        <v>-4.29</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>-7.62</v>
+        <v>-8.99</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-6.8</v>
+        <v>-7.4</v>
       </c>
       <c r="AO29" s="2" t="n">
         <v>21</v>
       </c>
       <c r="AP29" s="2" t="inlineStr"/>
-      <c r="AQ29" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AQ29" s="2" t="inlineStr"/>
       <c r="AR29" s="2" t="inlineStr"/>
       <c r="AS29" s="2" t="inlineStr"/>
       <c r="AT29" s="2" t="inlineStr">
@@ -4889,58 +4941,58 @@
         </is>
       </c>
       <c r="AU29" s="2" t="n">
-        <v>1.468</v>
+        <v>1.448</v>
       </c>
       <c r="AV29" s="2" t="n">
-        <v>1.533</v>
+        <v>1.509</v>
       </c>
       <c r="AW29" s="2" t="n">
-        <v>1.617</v>
+        <v>1.606</v>
       </c>
       <c r="AX29" s="2" t="n">
-        <v>1.647</v>
+        <v>1.635</v>
       </c>
       <c r="AY29" s="2" t="n">
-        <v>1.698</v>
+        <v>1.692</v>
       </c>
       <c r="AZ29" s="2" t="n">
-        <v>1.829</v>
+        <v>1.824</v>
       </c>
       <c r="BA29" s="2" t="n">
         <v>1.676</v>
       </c>
       <c r="BB29" s="2" t="n">
-        <v>-4.2937</v>
+        <v>-4.3557</v>
       </c>
       <c r="BC29" s="2" t="n">
-        <v>-1.6274</v>
+        <v>-1.748</v>
       </c>
       <c r="BD29" s="2" t="n">
-        <v>-1.0129</v>
+        <v>-0.9835</v>
       </c>
       <c r="BE29" s="2" t="n">
-        <v>-0.5259</v>
+        <v>-0.5679</v>
       </c>
       <c r="BF29" s="2" t="n">
-        <v>0.0483</v>
+        <v>0.0408</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.667</v>
+        <v>0.423</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-2.04</v>
+        <v>-1.36</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -4952,25 +5004,27 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O30" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="n">
         <v>2</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>0001010000</t>
+          <t>0000010010</t>
         </is>
       </c>
       <c r="U30" s="2" t="inlineStr">
         <is>
-          <t>0001010110</t>
+          <t>0001010100</t>
         </is>
       </c>
       <c r="V30" s="2" t="inlineStr">
@@ -4979,7 +5033,7 @@
         </is>
       </c>
       <c r="W30" s="2" t="n">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
@@ -4988,12 +5042,12 @@
       </c>
       <c r="Y30" s="2" t="inlineStr">
         <is>
-          <t>站稳短均·底背离·日线纠缠</t>
+          <t>站稳短均·日线纠缠</t>
         </is>
       </c>
       <c r="Z30" s="2" t="inlineStr">
         <is>
-          <t>4→4+·20d</t>
+          <t>4→4+·16d</t>
         </is>
       </c>
       <c r="AA30" s="2" t="inlineStr"/>
@@ -5006,22 +5060,22 @@
       <c r="AH30" s="2" t="inlineStr"/>
       <c r="AI30" s="2" t="inlineStr"/>
       <c r="AJ30" s="2" t="n">
-        <v>-24.07</v>
+        <v>-37.19</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>1.05</v>
+        <v>-3.98</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>4.69</v>
+        <v>4</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>10.37</v>
+        <v>12.05</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>67.90000000000001</v>
+        <v>54.3</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="AP30" s="2" t="inlineStr"/>
       <c r="AQ30" s="2" t="inlineStr"/>
@@ -5033,58 +5087,58 @@
         </is>
       </c>
       <c r="AU30" s="2" t="n">
-        <v>0.663</v>
+        <v>0.418</v>
       </c>
       <c r="AV30" s="2" t="n">
-        <v>0.658</v>
+        <v>0.417</v>
       </c>
       <c r="AW30" s="2" t="n">
-        <v>0.656</v>
+        <v>0.414</v>
       </c>
       <c r="AX30" s="2" t="n">
-        <v>0.662</v>
+        <v>0.417</v>
       </c>
       <c r="AY30" s="2" t="n">
-        <v>0.667</v>
+        <v>0.424</v>
       </c>
       <c r="AZ30" s="2" t="n">
-        <v>0.659</v>
+        <v>0.421</v>
       </c>
       <c r="BA30" s="2" t="n">
-        <v>0.713</v>
+        <v>0.467</v>
       </c>
       <c r="BB30" s="2" t="n">
-        <v>0.3422</v>
+        <v>0.3771</v>
       </c>
       <c r="BC30" s="2" t="n">
-        <v>-0.3388</v>
+        <v>-0.1948</v>
       </c>
       <c r="BD30" s="2" t="n">
-        <v>-0.0888</v>
+        <v>-0.2464</v>
       </c>
       <c r="BE30" s="2" t="n">
-        <v>-0.1683</v>
+        <v>-0.217</v>
       </c>
       <c r="BF30" s="2" t="n">
-        <v>-0.2407</v>
+        <v>-0.3719</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.421</v>
+        <v>0.877</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>-1.36</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -5096,50 +5150,48 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O31" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="S31" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>0000010010</t>
+          <t>1111111101</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr">
         <is>
-          <t>0001010110</t>
+          <t>1111111101</t>
         </is>
       </c>
       <c r="V31" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W31" s="2" t="n">
-        <v>217</v>
+        <v>54</v>
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="Y31" s="2" t="inlineStr">
         <is>
-          <t>站稳短均·日线纠缠</t>
+          <t>减速</t>
         </is>
       </c>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>4→4+·15d</t>
+          <t>2A→2C·14d</t>
         </is>
       </c>
       <c r="AA31" s="2" t="inlineStr"/>
@@ -5152,26 +5204,28 @@
       <c r="AH31" s="2" t="inlineStr"/>
       <c r="AI31" s="2" t="inlineStr"/>
       <c r="AJ31" s="2" t="n">
-        <v>-37.04</v>
+        <v>8.66</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>-4.41</v>
+        <v>21.42</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>4.32</v>
+        <v>3.99</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>11.25</v>
+        <v>12.21</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>53.1</v>
+        <v>100.7</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="AP31" s="2" t="inlineStr"/>
       <c r="AQ31" s="2" t="inlineStr"/>
-      <c r="AR31" s="2" t="inlineStr"/>
+      <c r="AR31" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AS31" s="2" t="inlineStr"/>
       <c r="AT31" s="2" t="inlineStr">
         <is>
@@ -5179,40 +5233,40 @@
         </is>
       </c>
       <c r="AU31" s="2" t="n">
-        <v>0.417</v>
+        <v>0.867</v>
       </c>
       <c r="AV31" s="2" t="n">
-        <v>0.415</v>
+        <v>0.86</v>
       </c>
       <c r="AW31" s="2" t="n">
-        <v>0.413</v>
+        <v>0.85</v>
       </c>
       <c r="AX31" s="2" t="n">
-        <v>0.417</v>
+        <v>0.847</v>
       </c>
       <c r="AY31" s="2" t="n">
-        <v>0.424</v>
+        <v>0.833</v>
       </c>
       <c r="AZ31" s="2" t="n">
-        <v>0.422</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="BA31" s="2" t="n">
-        <v>0.468</v>
+        <v>0.8</v>
       </c>
       <c r="BB31" s="2" t="n">
-        <v>0.2645</v>
+        <v>0.9107</v>
       </c>
       <c r="BC31" s="2" t="n">
-        <v>-0.3561</v>
+        <v>0.3606</v>
       </c>
       <c r="BD31" s="2" t="n">
-        <v>-0.1659</v>
+        <v>0.2701</v>
       </c>
       <c r="BE31" s="2" t="n">
-        <v>-0.2365</v>
+        <v>0.3042</v>
       </c>
       <c r="BF31" s="2" t="n">
-        <v>-0.3704</v>
+        <v>0.0866</v>
       </c>
     </row>
   </sheetData>
@@ -5243,7 +5297,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-16 | 30 只</t>
+          <t>截至: 2026-10-19 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-20
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.762</v>
+        <v>2.756</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-0.51</v>
@@ -852,7 +852,7 @@
         <v>9</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
@@ -898,26 +898,26 @@
       <c r="AH2" s="2" t="inlineStr"/>
       <c r="AI2" s="2" t="inlineStr"/>
       <c r="AJ2" s="2" t="n">
-        <v>-10.84</v>
+        <v>-12.25</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>-9.949999999999999</v>
+        <v>-9.65</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>-4.61</v>
+        <v>-4.28</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>-11.39</v>
+        <v>-10.58</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-6.9</v>
+        <v>-7.3</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="AP2" s="2" t="inlineStr"/>
       <c r="AQ2" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AR2" s="2" t="inlineStr"/>
       <c r="AS2" s="2" t="inlineStr"/>
@@ -927,40 +927,40 @@
         </is>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>2.844</v>
+        <v>2.801</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>2.964</v>
+        <v>2.923</v>
       </c>
       <c r="AW2" s="2" t="n">
-        <v>3.148</v>
+        <v>3.12</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>3.222</v>
+        <v>3.199</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>3.349</v>
+        <v>3.338</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>3.636</v>
+        <v>3.624</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>3.518</v>
+        <v>3.516</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>-4.0242</v>
+        <v>-4.0182</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>-2.0927</v>
+        <v>-2.1931</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>-0.8506</v>
+        <v>-0.8326</v>
       </c>
       <c r="BE2" s="2" t="n">
-        <v>-0.757</v>
+        <v>-0.7865</v>
       </c>
       <c r="BF2" s="2" t="n">
-        <v>-0.1084</v>
+        <v>-0.1225</v>
       </c>
     </row>
     <row r="3">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.418</v>
+        <v>1.402</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>-2.87</v>
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="W3" s="2" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
       <c r="Y3" s="2" t="inlineStr"/>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>4+→4·7d ← 4→4+·16d</t>
+          <t>4+→4·8d ← 4→4+·17d</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr"/>
@@ -1035,35 +1035,31 @@
       <c r="AC3" s="2" t="inlineStr"/>
       <c r="AD3" s="2" t="inlineStr"/>
       <c r="AE3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF3" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="n">
-        <v>-12.47</v>
+        <v>-12.77</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>3.43</v>
+        <v>2.83</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>2.25</v>
+        <v>1.32</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>5.69</v>
+        <v>4.09</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>44.8</v>
+        <v>42</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="AP3" s="2" t="inlineStr"/>
       <c r="AQ3" s="2" t="inlineStr"/>
@@ -1075,40 +1071,40 @@
         </is>
       </c>
       <c r="AU3" s="2" t="n">
+        <v>1.416</v>
+      </c>
+      <c r="AV3" s="2" t="n">
         <v>1.421</v>
       </c>
-      <c r="AV3" s="2" t="n">
-        <v>1.425</v>
-      </c>
       <c r="AW3" s="2" t="n">
-        <v>1.44</v>
+        <v>1.437</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>1.455</v>
+        <v>1.452</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>1.476</v>
+        <v>1.473</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>1.462</v>
+        <v>1.461</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>1.51</v>
+        <v>1.509</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>-0.6987</v>
+        <v>-0.7244</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>-0.4999</v>
+        <v>-0.4858</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>-0.3244</v>
+        <v>-0.372</v>
       </c>
       <c r="BE3" s="2" t="n">
-        <v>-0.1622</v>
+        <v>-0.1644</v>
       </c>
       <c r="BF3" s="2" t="n">
-        <v>-0.1247</v>
+        <v>-0.1277</v>
       </c>
     </row>
     <row r="4">
@@ -1123,7 +1119,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.666</v>
+        <v>0.664</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>-2.04</v>
@@ -1144,19 +1140,19 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>0000010110</t>
+          <t>0000010100</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>0001010100</t>
+          <t>0001010110</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
@@ -1165,7 +1161,7 @@
         </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
@@ -1179,39 +1175,37 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>4→4+·2d ← 4+→4·3d ← 4→4+·4d</t>
+          <t>4→4+·3d ← 4+→4·4d ← 4→4+·5d</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr"/>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
       <c r="AD4" s="2" t="inlineStr"/>
-      <c r="AE4" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="AE4" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="n">
-        <v>-24.3</v>
+        <v>-24.47</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>0.86</v>
+        <v>1.16</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>3.02</v>
+        <v>4.13</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>10.55</v>
+        <v>10.27</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>68.7</v>
+        <v>68.3</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="AP4" s="2" t="inlineStr"/>
       <c r="AQ4" s="2" t="inlineStr"/>
@@ -1223,10 +1217,10 @@
         </is>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>0.663</v>
+        <v>0.664</v>
       </c>
       <c r="AV4" s="2" t="n">
-        <v>0.66</v>
+        <v>0.661</v>
       </c>
       <c r="AW4" s="2" t="n">
         <v>0.656</v>
@@ -1244,19 +1238,19 @@
         <v>0.712</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>0.3971</v>
+        <v>0.5321</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>-0.2249</v>
+        <v>-0.0988</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>-0.1526</v>
+        <v>-0.1853</v>
       </c>
       <c r="BE4" s="2" t="n">
-        <v>-0.1449</v>
+        <v>-0.1198</v>
       </c>
       <c r="BF4" s="2" t="n">
-        <v>-0.243</v>
+        <v>-0.2447</v>
       </c>
     </row>
     <row r="5">
@@ -1271,7 +1265,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.809</v>
+        <v>1.827</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>95.31</v>
@@ -1294,7 +1288,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -1321,7 +1315,7 @@
         </is>
       </c>
       <c r="W5" s="2" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
@@ -1331,16 +1325,14 @@
       <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·10d</t>
+          <t>2A→2C·11d</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr"/>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AE5" s="2" t="inlineStr"/>
       <c r="AF5" s="2" t="n">
         <v>-1</v>
       </c>
@@ -1350,31 +1342,27 @@
       </c>
       <c r="AI5" s="2" t="inlineStr"/>
       <c r="AJ5" s="2" t="n">
-        <v>56.16</v>
+        <v>55.35</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>36.9</v>
+        <v>38.74</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>-2.52</v>
+        <v>-0.44</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>9.720000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="AP5" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="AP5" s="2" t="inlineStr"/>
       <c r="AQ5" s="2" t="inlineStr"/>
       <c r="AR5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="inlineStr"/>
       <c r="AT5" s="2" t="inlineStr">
@@ -1383,40 +1371,40 @@
         </is>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>1.843</v>
+        <v>1.834</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>1.85</v>
+        <v>1.855</v>
       </c>
       <c r="AW5" s="2" t="n">
-        <v>1.804</v>
+        <v>1.806</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>1.77</v>
+        <v>1.776</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>1.67</v>
+        <v>1.677</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>1.593</v>
+        <v>1.595</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>1.536</v>
+        <v>1.539</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>1.5781</v>
+        <v>1.3605</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>0.7354000000000001</v>
+        <v>0.5264</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>1.1625</v>
+        <v>1.113</v>
       </c>
       <c r="BE5" s="2" t="n">
-        <v>0.2944</v>
+        <v>0.2894</v>
       </c>
       <c r="BF5" s="2" t="n">
-        <v>0.5616</v>
+        <v>0.5535</v>
       </c>
     </row>
     <row r="6">
@@ -1431,7 +1419,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.804</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>7.37</v>
@@ -1446,7 +1434,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
@@ -1455,7 +1443,7 @@
         <v>3</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
@@ -1464,7 +1452,7 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0010011000</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
@@ -1473,7 +1461,7 @@
         </is>
       </c>
       <c r="W6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
@@ -1483,7 +1471,7 @@
       <c r="Y6" s="2" t="inlineStr"/>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1→4·5d ← 1+→1·8d ← 1→1+·9d</t>
+          <t>1→4·6d ← 1+→1·9d ← 1→1+·10d</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr"/>
@@ -1504,22 +1492,22 @@
       <c r="AH6" s="2" t="inlineStr"/>
       <c r="AI6" s="2" t="inlineStr"/>
       <c r="AJ6" s="2" t="n">
-        <v>-7.75</v>
+        <v>-7.19</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>6.16</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>-0.31</v>
+        <v>2.68</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>9.140000000000001</v>
+        <v>7.21</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>38.9</v>
+        <v>35.5</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="AP6" s="2" t="inlineStr"/>
       <c r="AQ6" s="2" t="inlineStr"/>
@@ -1531,16 +1519,16 @@
         </is>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>0.827</v>
+        <v>0.824</v>
       </c>
       <c r="AW6" s="2" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="AX6" s="2" t="n">
         <v>0.835</v>
-      </c>
-      <c r="AX6" s="2" t="n">
-        <v>0.836</v>
       </c>
       <c r="AY6" s="2" t="n">
         <v>0.858</v>
@@ -1552,19 +1540,19 @@
         <v>0.831</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>-1.538</v>
+        <v>-1.4242</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>-0.3433</v>
+        <v>-0.3251</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>-0.2184</v>
+        <v>-0.1884</v>
       </c>
       <c r="BE6" s="2" t="n">
-        <v>0.0591</v>
+        <v>0.06660000000000001</v>
       </c>
       <c r="BF6" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-0.07190000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -1579,7 +1567,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.886</v>
+        <v>2.877</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>2.9</v>
@@ -1596,7 +1584,7 @@
         <v>13</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -1623,7 +1611,7 @@
         </is>
       </c>
       <c r="W7" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
@@ -1644,22 +1632,22 @@
       <c r="AH7" s="2" t="inlineStr"/>
       <c r="AI7" s="2" t="inlineStr"/>
       <c r="AJ7" s="2" t="n">
-        <v>-6.71</v>
+        <v>-7.11</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>5.86</v>
+        <v>6.08</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>1.05</v>
+        <v>1.53</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>4.56</v>
+        <v>4.26</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>7.7</v>
+        <v>6.6</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="AP7" s="2" t="inlineStr"/>
       <c r="AQ7" s="2" t="inlineStr"/>
@@ -1671,40 +1659,40 @@
         </is>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>2.887</v>
+        <v>2.879</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>2.907</v>
+        <v>2.902</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>2.941</v>
+        <v>2.936</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>2.969</v>
+        <v>2.963</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>2.99</v>
+        <v>2.988</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>3.003</v>
+        <v>3.002</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>3.036</v>
+        <v>3.035</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>-0.8138</v>
+        <v>-0.7454</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>-0.5403</v>
+        <v>-0.54</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>-0.2501</v>
+        <v>-0.2422</v>
       </c>
       <c r="BE7" s="2" t="n">
         <v>-0.1135</v>
       </c>
       <c r="BF7" s="2" t="n">
-        <v>-0.06710000000000001</v>
+        <v>-0.0711</v>
       </c>
     </row>
     <row r="8">
@@ -1719,7 +1707,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.24</v>
+        <v>4.22</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>4.58</v>
@@ -1769,7 +1757,7 @@
         </is>
       </c>
       <c r="W8" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
@@ -1783,34 +1771,32 @@
       <c r="AC8" s="2" t="inlineStr"/>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF8" s="2" t="inlineStr"/>
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr"/>
       <c r="AI8" s="2" t="inlineStr"/>
       <c r="AJ8" s="2" t="n">
-        <v>-7.73</v>
+        <v>-8.41</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>1.1</v>
+        <v>1.15</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.04</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>-0.11</v>
+        <v>-0.14</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-4.4</v>
+        <v>-4.7</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="AP8" s="2" t="inlineStr"/>
-      <c r="AQ8" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AQ8" s="2" t="inlineStr"/>
       <c r="AR8" s="2" t="inlineStr"/>
       <c r="AS8" s="2" t="inlineStr"/>
       <c r="AT8" s="2" t="inlineStr">
@@ -1819,40 +1805,40 @@
         </is>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>4.271</v>
+        <v>4.247</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>4.334</v>
+        <v>4.314</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>4.441</v>
+        <v>4.425</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>4.504</v>
+        <v>4.489</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>4.581</v>
+        <v>4.574</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>4.715</v>
+        <v>4.709</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>4.707</v>
+        <v>4.706</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>-1.6112</v>
+        <v>-1.5432</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>-0.9956</v>
+        <v>-1.0238</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>-0.4363</v>
+        <v>-0.4305</v>
       </c>
       <c r="BE8" s="2" t="n">
-        <v>-0.3201</v>
+        <v>-0.3325</v>
       </c>
       <c r="BF8" s="2" t="n">
-        <v>-0.07729999999999999</v>
+        <v>-0.08409999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1867,7 +1853,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6.83</v>
+        <v>6.871</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0.97</v>
@@ -1917,7 +1903,7 @@
         </is>
       </c>
       <c r="W9" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
@@ -1940,27 +1926,25 @@
       <c r="AH9" s="2" t="inlineStr"/>
       <c r="AI9" s="2" t="inlineStr"/>
       <c r="AJ9" s="2" t="n">
-        <v>-2.05</v>
+        <v>-2.81</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>-2.48</v>
+        <v>-1.38</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>-1.59</v>
+        <v>-0.55</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>-3.75</v>
+        <v>-3.1</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>0.7</v>
+        <v>-0.1</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="AP9" s="2" t="inlineStr"/>
-      <c r="AQ9" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AQ9" s="2" t="inlineStr"/>
       <c r="AR9" s="2" t="inlineStr"/>
       <c r="AS9" s="2" t="inlineStr"/>
       <c r="AT9" s="2" t="inlineStr">
@@ -1969,40 +1953,40 @@
         </is>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>6.915</v>
+        <v>6.867</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>7.121</v>
+        <v>7.06</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>7.412</v>
+        <v>7.376</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>7.533</v>
+        <v>7.496</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>7.675</v>
+        <v>7.664</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>7.972</v>
+        <v>7.955</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>8.010999999999999</v>
+        <v>8.01</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>-2.8013</v>
+        <v>-2.7212</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>-1.4078</v>
+        <v>-1.4361</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>-0.402</v>
+        <v>-0.3936</v>
       </c>
       <c r="BE9" s="2" t="n">
-        <v>-0.5077</v>
+        <v>-0.527</v>
       </c>
       <c r="BF9" s="2" t="n">
-        <v>-0.0205</v>
+        <v>-0.0281</v>
       </c>
     </row>
     <row r="10">
@@ -2017,7 +2001,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.463</v>
+        <v>3.416</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>41.01</v>
@@ -2041,7 +2025,7 @@
         <v>9</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
@@ -2050,7 +2034,7 @@
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>1111111101</t>
+          <t>0111111101</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -2059,7 +2043,7 @@
         </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
@@ -2076,41 +2060,35 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="inlineStr"/>
-      <c r="AE10" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AE10" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="AF10" s="2" t="inlineStr"/>
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="inlineStr"/>
       <c r="AI10" s="2" t="inlineStr"/>
       <c r="AJ10" s="2" t="n">
-        <v>17.73</v>
+        <v>17.47</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>20.5</v>
+        <v>19.38</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>3.16</v>
+        <v>0.91</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>8.970000000000001</v>
+        <v>7.64</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>86.5</v>
+        <v>86.2</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="AP10" s="2" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="AP10" s="2" t="inlineStr"/>
       <c r="AQ10" s="2" t="inlineStr"/>
       <c r="AR10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS10" s="2" t="inlineStr"/>
       <c r="AT10" s="2" t="inlineStr">
@@ -2119,40 +2097,40 @@
         </is>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>3.454</v>
+        <v>3.443</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>3.426</v>
+        <v>3.435</v>
       </c>
       <c r="AW10" s="2" t="n">
-        <v>3.395</v>
+        <v>3.396</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>3.413</v>
+        <v>3.411</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>3.384</v>
+        <v>3.387</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>3.276</v>
+        <v>3.279</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>3.232</v>
+        <v>3.235</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.7040999999999999</v>
+        <v>0.7065</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>0.0346</v>
+        <v>-0.0203</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>0.2837</v>
+        <v>0.2492</v>
       </c>
       <c r="BE10" s="2" t="n">
-        <v>0.1948</v>
+        <v>0.1962</v>
       </c>
       <c r="BF10" s="2" t="n">
-        <v>0.1773</v>
+        <v>0.1747</v>
       </c>
     </row>
     <row r="11">
@@ -2167,7 +2145,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.493</v>
+        <v>0.486</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>-0.8100000000000001</v>
@@ -2211,7 +2189,7 @@
         </is>
       </c>
       <c r="W11" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
@@ -2221,43 +2199,43 @@
       <c r="Y11" s="2" t="inlineStr"/>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>4+→4·11d</t>
+          <t>4+→4·12d</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr"/>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
       <c r="AD11" s="2" t="inlineStr"/>
-      <c r="AE11" s="2" t="inlineStr"/>
-      <c r="AF11" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE11" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AF11" s="2" t="inlineStr"/>
       <c r="AG11" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="AH11" s="2" t="inlineStr"/>
       <c r="AI11" s="2" t="inlineStr"/>
       <c r="AJ11" s="2" t="n">
-        <v>-19.04</v>
+        <v>-19.79</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>1.67</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>2.48</v>
+        <v>1.28</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>6.34</v>
+        <v>5.32</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>7.5</v>
+        <v>5.3</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="AP11" s="2" t="inlineStr"/>
       <c r="AQ11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR11" s="2" t="inlineStr"/>
       <c r="AS11" s="2" t="inlineStr"/>
@@ -2267,19 +2245,19 @@
         </is>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>0.494</v>
+        <v>0.493</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>0.493</v>
+        <v>0.492</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>0.498</v>
+        <v>0.497</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>0.506</v>
+        <v>0.505</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>0.512</v>
+        <v>0.511</v>
       </c>
       <c r="AZ11" s="2" t="n">
         <v>0.516</v>
@@ -2288,19 +2266,19 @@
         <v>0.529</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>-0.5222</v>
+        <v>-0.419</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>-0.5985</v>
+        <v>-0.5433</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>-0.3271</v>
+        <v>-0.3436</v>
       </c>
       <c r="BE11" s="2" t="n">
-        <v>-0.0383</v>
+        <v>-0.0423</v>
       </c>
       <c r="BF11" s="2" t="n">
-        <v>-0.1904</v>
+        <v>-0.1979</v>
       </c>
     </row>
     <row r="12">
@@ -2315,7 +2293,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.373</v>
+        <v>0.377</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>9.880000000000001</v>
@@ -2343,7 +2321,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>0010111010</t>
+          <t>0110111000</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -2357,7 +2335,7 @@
         </is>
       </c>
       <c r="W12" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
@@ -2371,45 +2349,41 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>4→4+·2d ← 1→4·5d ← 1+→1·8d</t>
+          <t>4→4+·3d ← 1→4·6d ← 1+→1·9d</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr"/>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="inlineStr"/>
-      <c r="AE12" s="2" t="inlineStr">
+      <c r="AE12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF12" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="AF12" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AG12" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="AG12" s="2" t="inlineStr"/>
       <c r="AH12" s="2" t="inlineStr"/>
       <c r="AI12" s="2" t="inlineStr"/>
       <c r="AJ12" s="2" t="n">
-        <v>-4.79</v>
+        <v>-4.09</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>10</v>
+        <v>11.75</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>1.42</v>
+        <v>3.7</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>11.56</v>
+        <v>10.65</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>57.2</v>
+        <v>56.1</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="AP12" s="2" t="inlineStr"/>
       <c r="AQ12" s="2" t="inlineStr"/>
@@ -2421,7 +2395,7 @@
         </is>
       </c>
       <c r="AU12" s="2" t="n">
-        <v>0.373</v>
+        <v>0.374</v>
       </c>
       <c r="AV12" s="2" t="n">
         <v>0.377</v>
@@ -2442,19 +2416,19 @@
         <v>0.371</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>-0.5206</v>
+        <v>-0.3854</v>
       </c>
       <c r="BC12" s="2" t="n">
-        <v>0.0141</v>
+        <v>0.0619</v>
       </c>
       <c r="BD12" s="2" t="n">
-        <v>0.0188</v>
+        <v>0.0056</v>
       </c>
       <c r="BE12" s="2" t="n">
-        <v>0.1666</v>
+        <v>0.1836</v>
       </c>
       <c r="BF12" s="2" t="n">
-        <v>-0.0479</v>
+        <v>-0.0409</v>
       </c>
     </row>
     <row r="13">
@@ -2469,7 +2443,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.756</v>
+        <v>0.744</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>-4.85</v>
@@ -2513,7 +2487,7 @@
         </is>
       </c>
       <c r="W13" s="2" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
@@ -2523,43 +2497,41 @@
       <c r="Y13" s="2" t="inlineStr"/>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>4+→4·8d ← 4→4+·11d</t>
+          <t>4+→4·9d ← 4→4+·12d</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr"/>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
-      <c r="AE13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF13" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="AE13" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="AH13" s="2" t="inlineStr"/>
       <c r="AI13" s="2" t="inlineStr"/>
       <c r="AJ13" s="2" t="n">
-        <v>-22.19</v>
+        <v>-23.75</v>
       </c>
       <c r="AK13" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AL13" s="2" t="n">
         <v>1.12</v>
       </c>
-      <c r="AL13" s="2" t="n">
-        <v>1.35</v>
-      </c>
       <c r="AM13" s="2" t="n">
-        <v>4.39</v>
+        <v>2.98</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>11</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="AP13" s="2" t="inlineStr"/>
       <c r="AQ13" s="2" t="inlineStr"/>
@@ -2571,40 +2543,40 @@
         </is>
       </c>
       <c r="AU13" s="2" t="n">
-        <v>0.756</v>
+        <v>0.753</v>
       </c>
       <c r="AV13" s="2" t="n">
-        <v>0.758</v>
+        <v>0.757</v>
       </c>
       <c r="AW13" s="2" t="n">
-        <v>0.769</v>
+        <v>0.767</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>0.782</v>
+        <v>0.78</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>0.786</v>
+        <v>0.785</v>
       </c>
       <c r="AZ13" s="2" t="n">
         <v>0.786</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>0.822</v>
+        <v>0.821</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>-0.7759</v>
+        <v>-0.6716</v>
       </c>
       <c r="BC13" s="2" t="n">
-        <v>-0.7512</v>
+        <v>-0.7277</v>
       </c>
       <c r="BD13" s="2" t="n">
-        <v>-0.3528</v>
+        <v>-0.3798</v>
       </c>
       <c r="BE13" s="2" t="n">
-        <v>-0.0437</v>
+        <v>-0.0419</v>
       </c>
       <c r="BF13" s="2" t="n">
-        <v>-0.2219</v>
+        <v>-0.2375</v>
       </c>
     </row>
     <row r="14">
@@ -2619,7 +2591,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.722</v>
+        <v>2.752</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>4.11</v>
@@ -2669,7 +2641,7 @@
         </is>
       </c>
       <c r="W14" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
@@ -2682,32 +2654,30 @@
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="inlineStr"/>
-      <c r="AE14" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AE14" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AF14" s="2" t="inlineStr"/>
       <c r="AG14" s="2" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr"/>
       <c r="AI14" s="2" t="inlineStr"/>
       <c r="AJ14" s="2" t="n">
-        <v>-6.86</v>
+        <v>-7.32</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>-3.73</v>
+        <v>-2.17</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>-2.07</v>
+        <v>-0.7</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>-2.68</v>
+        <v>-2.39</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>11.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="AP14" s="2" t="inlineStr"/>
       <c r="AQ14" s="2" t="inlineStr"/>
@@ -2719,40 +2689,40 @@
         </is>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>2.762</v>
+        <v>2.742</v>
       </c>
       <c r="AV14" s="2" t="n">
-        <v>2.843</v>
+        <v>2.821</v>
       </c>
       <c r="AW14" s="2" t="n">
-        <v>2.963</v>
+        <v>2.949</v>
       </c>
       <c r="AX14" s="2" t="n">
-        <v>3.005</v>
+        <v>2.992</v>
       </c>
       <c r="AY14" s="2" t="n">
-        <v>3.038</v>
+        <v>3.036</v>
       </c>
       <c r="AZ14" s="2" t="n">
-        <v>3.164</v>
+        <v>3.157</v>
       </c>
       <c r="BA14" s="2" t="n">
-        <v>3.212</v>
+        <v>3.211</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>-2.9018</v>
+        <v>-2.8135</v>
       </c>
       <c r="BC14" s="2" t="n">
-        <v>-1.358</v>
+        <v>-1.3958</v>
       </c>
       <c r="BD14" s="2" t="n">
-        <v>-0.1731</v>
+        <v>-0.186</v>
       </c>
       <c r="BE14" s="2" t="n">
-        <v>-0.6018</v>
+        <v>-0.6204</v>
       </c>
       <c r="BF14" s="2" t="n">
-        <v>-0.06859999999999999</v>
+        <v>-0.0732</v>
       </c>
     </row>
     <row r="15">
@@ -2767,7 +2737,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.326</v>
+        <v>0.333</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>12.17</v>
@@ -2788,19 +2758,19 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>0000011100</t>
+          <t>0100111100</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0010111000</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
@@ -2809,7 +2779,7 @@
         </is>
       </c>
       <c r="W15" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
@@ -2823,45 +2793,37 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>4→4+·2d ← 4+→4·8d ← 4→4+·9d</t>
+          <t>4→4+·3d ← 4+→4·9d ← 4→4+·10d</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="AF15" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AG15" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="AE15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="inlineStr"/>
       <c r="AH15" s="2" t="inlineStr"/>
       <c r="AI15" s="2" t="inlineStr"/>
       <c r="AJ15" s="2" t="n">
-        <v>-4.59</v>
+        <v>-4.74</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>6.65</v>
+        <v>9.57</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>-1.48</v>
+        <v>2.72</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>8.640000000000001</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>61.1</v>
+        <v>59.5</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="AP15" s="2" t="inlineStr"/>
       <c r="AQ15" s="2" t="inlineStr"/>
@@ -2873,7 +2835,7 @@
         </is>
       </c>
       <c r="AU15" s="2" t="n">
-        <v>0.329</v>
+        <v>0.328</v>
       </c>
       <c r="AV15" s="2" t="n">
         <v>0.335</v>
@@ -2882,7 +2844,7 @@
         <v>0.338</v>
       </c>
       <c r="AX15" s="2" t="n">
-        <v>0.338</v>
+        <v>0.337</v>
       </c>
       <c r="AY15" s="2" t="n">
         <v>0.341</v>
@@ -2891,22 +2853,22 @@
         <v>0.326</v>
       </c>
       <c r="BA15" s="2" t="n">
-        <v>0.336</v>
+        <v>0.335</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>-1.2427</v>
+        <v>-1.1402</v>
       </c>
       <c r="BC15" s="2" t="n">
-        <v>-0.2382</v>
+        <v>-0.2309</v>
       </c>
       <c r="BD15" s="2" t="n">
-        <v>0.0607</v>
+        <v>0.0401</v>
       </c>
       <c r="BE15" s="2" t="n">
-        <v>0.0399</v>
+        <v>0.0466</v>
       </c>
       <c r="BF15" s="2" t="n">
-        <v>-0.0459</v>
+        <v>-0.0474</v>
       </c>
     </row>
     <row r="16">
@@ -2921,7 +2883,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.073</v>
+        <v>1.07</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>71.16</v>
@@ -2938,7 +2900,7 @@
         <v>9</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -2965,7 +2927,7 @@
         </is>
       </c>
       <c r="W16" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
@@ -2975,7 +2937,7 @@
       <c r="Y16" s="2" t="inlineStr"/>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>4+→4·13d ← 4→4+·16d</t>
+          <t>4+→4·14d ← 4→4+·17d</t>
         </is>
       </c>
       <c r="AA16" s="2" t="inlineStr"/>
@@ -2985,34 +2947,36 @@
       <c r="AE16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AF16" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="AF16" s="2" t="inlineStr"/>
       <c r="AG16" s="2" t="inlineStr"/>
       <c r="AH16" s="2" t="inlineStr"/>
       <c r="AI16" s="2" t="inlineStr"/>
       <c r="AJ16" s="2" t="n">
-        <v>-16.6</v>
+        <v>-16.87</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>-6.05</v>
+        <v>-5.8</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>3.83</v>
+        <v>1.76</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>-0.25</v>
+        <v>0.78</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>20.6</v>
+        <v>19.6</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="AP16" s="2" t="inlineStr"/>
-      <c r="AQ16" s="2" t="inlineStr"/>
+        <v>54</v>
+      </c>
+      <c r="AP16" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="AQ16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AR16" s="2" t="inlineStr"/>
       <c r="AS16" s="2" t="inlineStr"/>
       <c r="AT16" s="2" t="inlineStr">
@@ -3021,58 +2985,58 @@
         </is>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>1.064</v>
+        <v>1.061</v>
       </c>
       <c r="AV16" s="2" t="n">
-        <v>1.076</v>
+        <v>1.073</v>
       </c>
       <c r="AW16" s="2" t="n">
-        <v>1.111</v>
+        <v>1.107</v>
       </c>
       <c r="AX16" s="2" t="n">
-        <v>1.126</v>
+        <v>1.123</v>
       </c>
       <c r="AY16" s="2" t="n">
         <v>1.127</v>
       </c>
       <c r="AZ16" s="2" t="n">
-        <v>1.175</v>
+        <v>1.172</v>
       </c>
       <c r="BA16" s="2" t="n">
-        <v>1.296</v>
+        <v>1.295</v>
       </c>
       <c r="BB16" s="2" t="n">
-        <v>-1.8733</v>
+        <v>-1.5978</v>
       </c>
       <c r="BC16" s="2" t="n">
-        <v>-1.1914</v>
+        <v>-1.218</v>
       </c>
       <c r="BD16" s="2" t="n">
-        <v>-0.1123</v>
+        <v>-0.1206</v>
       </c>
       <c r="BE16" s="2" t="n">
-        <v>-0.6667999999999999</v>
+        <v>-0.6614</v>
       </c>
       <c r="BF16" s="2" t="n">
-        <v>-0.166</v>
+        <v>-0.1687</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.017</v>
+        <v>0.419</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-0.29</v>
+        <v>-1.36</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -3081,32 +3045,28 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010010</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0001010100</t>
         </is>
       </c>
       <c r="V17" s="2" t="inlineStr">
@@ -3115,110 +3075,114 @@
         </is>
       </c>
       <c r="W17" s="2" t="n">
-        <v>61</v>
+        <v>219</v>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y17" s="2" t="inlineStr"/>
-      <c r="Z17" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>4→4+·17d</t>
+        </is>
+      </c>
       <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
       <c r="AD17" s="2" t="inlineStr"/>
-      <c r="AE17" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AE17" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="AF17" s="2" t="inlineStr"/>
       <c r="AG17" s="2" t="inlineStr"/>
       <c r="AH17" s="2" t="inlineStr"/>
       <c r="AI17" s="2" t="inlineStr"/>
       <c r="AJ17" s="2" t="n">
-        <v>-14.74</v>
+        <v>-37.04</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>-7.56</v>
+        <v>-4.3</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>-0.39</v>
+        <v>4.11</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>-0.15</v>
+        <v>11.01</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>-0.7</v>
+        <v>54.6</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="AP17" s="2" t="inlineStr"/>
-      <c r="AQ17" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="AQ17" s="2" t="inlineStr"/>
       <c r="AR17" s="2" t="inlineStr"/>
       <c r="AS17" s="2" t="inlineStr"/>
       <c r="AT17" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU17" s="2" t="n">
-        <v>1.022</v>
+        <v>0.419</v>
       </c>
       <c r="AV17" s="2" t="n">
-        <v>1.046</v>
+        <v>0.418</v>
       </c>
       <c r="AW17" s="2" t="n">
-        <v>1.084</v>
+        <v>0.414</v>
       </c>
       <c r="AX17" s="2" t="n">
-        <v>1.109</v>
+        <v>0.418</v>
       </c>
       <c r="AY17" s="2" t="n">
-        <v>1.144</v>
+        <v>0.423</v>
       </c>
       <c r="AZ17" s="2" t="n">
-        <v>1.181</v>
+        <v>0.421</v>
       </c>
       <c r="BA17" s="2" t="n">
-        <v>1.226</v>
+        <v>0.467</v>
       </c>
       <c r="BB17" s="2" t="n">
-        <v>-2.5357</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="BC17" s="2" t="n">
-        <v>-1.3398</v>
+        <v>-0.04</v>
       </c>
       <c r="BD17" s="2" t="n">
-        <v>-0.6205000000000001</v>
+        <v>-0.3061</v>
       </c>
       <c r="BE17" s="2" t="n">
-        <v>-0.6693</v>
+        <v>-0.1992</v>
       </c>
       <c r="BF17" s="2" t="n">
-        <v>-0.1474</v>
+        <v>-0.3704</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.875</v>
+        <v>1.027</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>4.85</v>
+        <v>-0.29</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -3227,140 +3191,146 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M18" s="2" t="n">
         <v>9</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W18" s="2" t="n">
-        <v>299</v>
+        <v>62</v>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>2C</t>
-        </is>
-      </c>
-      <c r="Y18" s="2" t="inlineStr">
-        <is>
-          <t>顶背离·周MACD死叉</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr"/>
       <c r="Z18" s="2" t="inlineStr"/>
       <c r="AA18" s="2" t="inlineStr"/>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="inlineStr"/>
-      <c r="AF18" s="2" t="inlineStr"/>
+      <c r="AE18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF18" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="inlineStr"/>
       <c r="AI18" s="2" t="inlineStr"/>
       <c r="AJ18" s="2" t="n">
-        <v>15.53</v>
+        <v>-14.86</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>-0.49</v>
+        <v>-6.09</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>-5.57</v>
+        <v>0.84</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>-10.58</v>
+        <v>0.72</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-7.7</v>
+        <v>-0.4</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="AP18" s="2" t="inlineStr"/>
-      <c r="AQ18" s="2" t="inlineStr"/>
+      <c r="AQ18" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="AR18" s="2" t="inlineStr"/>
       <c r="AS18" s="2" t="inlineStr"/>
       <c r="AT18" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU18" s="2" t="n">
-        <v>0.906</v>
+        <v>1.017</v>
       </c>
       <c r="AV18" s="2" t="n">
-        <v>0.947</v>
+        <v>1.04</v>
       </c>
       <c r="AW18" s="2" t="n">
-        <v>1.008</v>
+        <v>1.08</v>
       </c>
       <c r="AX18" s="2" t="n">
-        <v>1.026</v>
+        <v>1.104</v>
       </c>
       <c r="AY18" s="2" t="n">
-        <v>1.062</v>
+        <v>1.141</v>
       </c>
       <c r="AZ18" s="2" t="n">
-        <v>1.165</v>
+        <v>1.178</v>
       </c>
       <c r="BA18" s="2" t="n">
-        <v>1.031</v>
+        <v>1.226</v>
       </c>
       <c r="BB18" s="2" t="n">
-        <v>-4.5679</v>
+        <v>-2.431</v>
       </c>
       <c r="BC18" s="2" t="n">
-        <v>-1.7029</v>
+        <v>-1.2783</v>
       </c>
       <c r="BD18" s="2" t="n">
-        <v>-0.9969</v>
+        <v>-0.6187</v>
       </c>
       <c r="BE18" s="2" t="n">
-        <v>-0.5215</v>
+        <v>-0.6704</v>
       </c>
       <c r="BF18" s="2" t="n">
-        <v>0.1553</v>
+        <v>-0.1486</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.006</v>
+        <v>0.882</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>-8.65</v>
+        <v>4.85</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -3369,62 +3339,58 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="M19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N19" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="V19" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W19" s="2" t="n">
-        <v>156</v>
+        <v>299</v>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
-          <t>周J超卖·日线纠缠</t>
-        </is>
-      </c>
-      <c r="Z19" s="2" t="inlineStr">
-        <is>
-          <t>4→4+·15d</t>
-        </is>
-      </c>
+          <t>顶背离·周MACD死叉</t>
+        </is>
+      </c>
+      <c r="Z19" s="2" t="inlineStr"/>
       <c r="AA19" s="2" t="inlineStr"/>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
+          <t>预1</t>
         </is>
       </c>
       <c r="AF19" s="2" t="inlineStr"/>
@@ -3432,22 +3398,22 @@
       <c r="AH19" s="2" t="inlineStr"/>
       <c r="AI19" s="2" t="inlineStr"/>
       <c r="AJ19" s="2" t="n">
-        <v>-53.4</v>
+        <v>14.32</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>-12.75</v>
+        <v>0.82</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>2.94</v>
+        <v>-4.36</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>8.640000000000001</v>
+        <v>-8.06</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>23.1</v>
+        <v>-7.8</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="AP19" s="2" t="inlineStr"/>
       <c r="AQ19" s="2" t="inlineStr"/>
@@ -3455,62 +3421,62 @@
       <c r="AS19" s="2" t="inlineStr"/>
       <c r="AT19" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AU19" s="2" t="n">
-        <v>1.009</v>
+        <v>0.893</v>
       </c>
       <c r="AV19" s="2" t="n">
-        <v>1.005</v>
+        <v>0.931</v>
       </c>
       <c r="AW19" s="2" t="n">
-        <v>1.014</v>
+        <v>1.002</v>
       </c>
       <c r="AX19" s="2" t="n">
-        <v>1.023</v>
+        <v>1.017</v>
       </c>
       <c r="AY19" s="2" t="n">
-        <v>1.064</v>
+        <v>1.06</v>
       </c>
       <c r="AZ19" s="2" t="n">
-        <v>1.073</v>
+        <v>1.161</v>
       </c>
       <c r="BA19" s="2" t="n">
-        <v>1.204</v>
+        <v>1.031</v>
       </c>
       <c r="BB19" s="2" t="n">
-        <v>-0.5478</v>
+        <v>-4.6538</v>
       </c>
       <c r="BC19" s="2" t="n">
-        <v>-0.2527</v>
+        <v>-1.7275</v>
       </c>
       <c r="BD19" s="2" t="n">
-        <v>-0.5405</v>
+        <v>-0.8512999999999999</v>
       </c>
       <c r="BE19" s="2" t="n">
-        <v>-0.4131</v>
+        <v>-0.5915</v>
       </c>
       <c r="BF19" s="2" t="n">
-        <v>-0.534</v>
+        <v>0.1432</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.717</v>
+        <v>0.866</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-7.05</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -3522,44 +3488,48 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>1111111101</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W20" s="2" t="n">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y20" s="2" t="inlineStr"/>
+          <t>2C</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>减速</t>
+        </is>
+      </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>4+→4·8d ← 4→4+·11d</t>
+          <t>2A→2C·15d</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr"/>
@@ -3567,94 +3537,94 @@
       <c r="AC20" s="2" t="inlineStr"/>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF20" s="2" t="inlineStr"/>
-      <c r="AG20" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AG20" s="2" t="inlineStr"/>
       <c r="AH20" s="2" t="inlineStr"/>
       <c r="AI20" s="2" t="inlineStr"/>
       <c r="AJ20" s="2" t="n">
-        <v>-22.41</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>-0.96</v>
+        <v>20.44</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>1.72</v>
+        <v>3.29</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>3.97</v>
+        <v>9.35</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>7.1</v>
+        <v>100.6</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="AP20" s="2" t="inlineStr"/>
       <c r="AQ20" s="2" t="inlineStr"/>
-      <c r="AR20" s="2" t="inlineStr"/>
+      <c r="AR20" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="AS20" s="2" t="inlineStr"/>
       <c r="AT20" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU20" s="2" t="n">
-        <v>1.721</v>
+        <v>0.867</v>
       </c>
       <c r="AV20" s="2" t="n">
-        <v>1.731</v>
+        <v>0.863</v>
       </c>
       <c r="AW20" s="2" t="n">
-        <v>1.762</v>
+        <v>0.85</v>
       </c>
       <c r="AX20" s="2" t="n">
-        <v>1.797</v>
+        <v>0.849</v>
       </c>
       <c r="AY20" s="2" t="n">
-        <v>1.814</v>
+        <v>0.833</v>
       </c>
       <c r="AZ20" s="2" t="n">
-        <v>1.81</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="BA20" s="2" t="n">
-        <v>1.873</v>
+        <v>0.8</v>
       </c>
       <c r="BB20" s="2" t="n">
-        <v>-1.0621</v>
+        <v>0.908</v>
       </c>
       <c r="BC20" s="2" t="n">
-        <v>-0.9117</v>
+        <v>0.3015</v>
       </c>
       <c r="BD20" s="2" t="n">
-        <v>-0.3463</v>
+        <v>0.2396</v>
       </c>
       <c r="BE20" s="2" t="n">
-        <v>-0.1003</v>
+        <v>0.3117</v>
       </c>
       <c r="BF20" s="2" t="n">
-        <v>-0.2241</v>
+        <v>0.08790000000000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.345</v>
+        <v>0.996</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>110.91</v>
+        <v>-8.65</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -3664,86 +3634,90 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="n">
-        <v>-13</v>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>-9</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>0111111001</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V21" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W21" s="2" t="n">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>2C</t>
-        </is>
-      </c>
-      <c r="Y21" s="2" t="inlineStr"/>
-      <c r="Z21" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr">
+        <is>
+          <t>周J超卖·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>4→4+·16d</t>
+        </is>
+      </c>
       <c r="AA21" s="2" t="inlineStr"/>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
       <c r="AD21" s="2" t="inlineStr"/>
-      <c r="AE21" s="2" t="inlineStr"/>
-      <c r="AF21" s="2" t="n">
+      <c r="AE21" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AG21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH21" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AF21" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="AG21" s="2" t="inlineStr"/>
+      <c r="AH21" s="2" t="inlineStr"/>
       <c r="AI21" s="2" t="inlineStr"/>
       <c r="AJ21" s="2" t="n">
-        <v>28.59</v>
+        <v>-52.85</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>29.69</v>
+        <v>-12.98</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>-0.54</v>
+        <v>2.8</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>13.9</v>
+        <v>8</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>86.5</v>
+        <v>20.9</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AP21" s="2" t="inlineStr"/>
       <c r="AQ21" s="2" t="inlineStr"/>
-      <c r="AR21" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AR21" s="2" t="inlineStr"/>
       <c r="AS21" s="2" t="inlineStr"/>
       <c r="AT21" s="2" t="inlineStr">
         <is>
@@ -3751,94 +3725,88 @@
         </is>
       </c>
       <c r="AU21" s="2" t="n">
-        <v>2.359</v>
+        <v>1.008</v>
       </c>
       <c r="AV21" s="2" t="n">
-        <v>2.364</v>
+        <v>1.004</v>
       </c>
       <c r="AW21" s="2" t="n">
-        <v>2.314</v>
+        <v>1.013</v>
       </c>
       <c r="AX21" s="2" t="n">
-        <v>2.283</v>
+        <v>1.02</v>
       </c>
       <c r="AY21" s="2" t="n">
-        <v>2.258</v>
+        <v>1.061</v>
       </c>
       <c r="AZ21" s="2" t="n">
-        <v>2.22</v>
+        <v>1.071</v>
       </c>
       <c r="BA21" s="2" t="n">
-        <v>2.046</v>
+        <v>1.202</v>
       </c>
       <c r="BB21" s="2" t="n">
-        <v>0.5505</v>
+        <v>-0.462</v>
       </c>
       <c r="BC21" s="2" t="n">
-        <v>0.7678</v>
+        <v>-0.174</v>
       </c>
       <c r="BD21" s="2" t="n">
-        <v>0.6449</v>
+        <v>-0.6343</v>
       </c>
       <c r="BE21" s="2" t="n">
-        <v>0.3353</v>
+        <v>-0.3994</v>
       </c>
       <c r="BF21" s="2" t="n">
-        <v>0.2859</v>
+        <v>-0.5285</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.338</v>
+        <v>1.659</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>3.97</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>-7.05</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000001000</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V22" s="2" t="inlineStr">
@@ -3847,7 +3815,7 @@
         </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
@@ -3855,40 +3823,44 @@
         </is>
       </c>
       <c r="Y22" s="2" t="inlineStr"/>
-      <c r="Z22" s="2" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>4+→4·9d ← 4→4+·12d</t>
+        </is>
+      </c>
       <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
       <c r="AD22" s="2" t="inlineStr"/>
-      <c r="AE22" s="2" t="inlineStr"/>
-      <c r="AF22" s="2" t="n">
+      <c r="AE22" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AG22" s="2" t="inlineStr"/>
+      <c r="AF22" s="2" t="inlineStr"/>
+      <c r="AG22" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AH22" s="2" t="inlineStr"/>
       <c r="AI22" s="2" t="inlineStr"/>
       <c r="AJ22" s="2" t="n">
-        <v>-29.25</v>
+        <v>-23.96</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>-16.96</v>
+        <v>-3.72</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>-3.94</v>
+        <v>-1.12</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>-1.79</v>
+        <v>0.84</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>-1</v>
+        <v>4.3</v>
       </c>
       <c r="AO22" s="2" t="n">
         <v>17</v>
       </c>
       <c r="AP22" s="2" t="inlineStr"/>
-      <c r="AQ22" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="AQ22" s="2" t="inlineStr"/>
       <c r="AR22" s="2" t="inlineStr"/>
       <c r="AS22" s="2" t="inlineStr"/>
       <c r="AT22" s="2" t="inlineStr">
@@ -3897,96 +3869,90 @@
         </is>
       </c>
       <c r="AU22" s="2" t="n">
-        <v>1.36</v>
+        <v>1.706</v>
       </c>
       <c r="AV22" s="2" t="n">
-        <v>1.407</v>
+        <v>1.722</v>
       </c>
       <c r="AW22" s="2" t="n">
-        <v>1.448</v>
+        <v>1.755</v>
       </c>
       <c r="AX22" s="2" t="n">
-        <v>1.483</v>
+        <v>1.789</v>
       </c>
       <c r="AY22" s="2" t="n">
-        <v>1.55</v>
+        <v>1.81</v>
       </c>
       <c r="AZ22" s="2" t="n">
-        <v>1.673</v>
+        <v>1.809</v>
       </c>
       <c r="BA22" s="2" t="n">
-        <v>1.796</v>
+        <v>1.871</v>
       </c>
       <c r="BB22" s="2" t="n">
-        <v>-2.2152</v>
+        <v>-1.1257</v>
       </c>
       <c r="BC22" s="2" t="n">
-        <v>-1.4796</v>
+        <v>-0.9198</v>
       </c>
       <c r="BD22" s="2" t="n">
-        <v>-0.7996</v>
+        <v>-0.3707</v>
       </c>
       <c r="BE22" s="2" t="n">
-        <v>-1.0283</v>
+        <v>-0.1167</v>
       </c>
       <c r="BF22" s="2" t="n">
-        <v>-0.2925</v>
+        <v>-0.2396</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>2.334</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>3.37</v>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>110.91</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="N23" s="2" t="n">
-        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0111111101</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0111111001</t>
         </is>
       </c>
       <c r="V23" s="2" t="inlineStr">
@@ -3995,264 +3961,258 @@
         </is>
       </c>
       <c r="W23" s="2" t="n">
-        <v>299</v>
+        <v>130</v>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
           <t>2C</t>
         </is>
       </c>
-      <c r="Y23" s="2" t="inlineStr">
-        <is>
-          <t>周MACD死叉</t>
-        </is>
-      </c>
+      <c r="Y23" s="2" t="inlineStr"/>
       <c r="Z23" s="2" t="inlineStr"/>
       <c r="AA23" s="2" t="inlineStr"/>
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
-      <c r="AE23" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="AF23" s="2" t="inlineStr"/>
-      <c r="AG23" s="2" t="inlineStr"/>
-      <c r="AH23" s="2" t="inlineStr"/>
+      <c r="AE23" s="2" t="inlineStr"/>
+      <c r="AF23" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AG23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH23" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AI23" s="2" t="inlineStr"/>
       <c r="AJ23" s="2" t="n">
-        <v>13.77</v>
+        <v>28.61</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>-1.46</v>
+        <v>29.57</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>-4.48</v>
+        <v>0.51</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>-23.34</v>
+        <v>13.65</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>1.7</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="AP23" s="2" t="inlineStr"/>
       <c r="AQ23" s="2" t="inlineStr"/>
-      <c r="AR23" s="2" t="inlineStr"/>
+      <c r="AR23" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="AS23" s="2" t="inlineStr"/>
       <c r="AT23" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU23" s="2" t="n">
-        <v>0.83</v>
+        <v>2.351</v>
       </c>
       <c r="AV23" s="2" t="n">
-        <v>0.877</v>
+        <v>2.366</v>
       </c>
       <c r="AW23" s="2" t="n">
-        <v>0.96</v>
+        <v>2.322</v>
       </c>
       <c r="AX23" s="2" t="n">
-        <v>0.984</v>
+        <v>2.286</v>
       </c>
       <c r="AY23" s="2" t="n">
-        <v>1.001</v>
+        <v>2.262</v>
       </c>
       <c r="AZ23" s="2" t="n">
-        <v>1.101</v>
+        <v>2.222</v>
       </c>
       <c r="BA23" s="2" t="n">
-        <v>0.976</v>
+        <v>2.048</v>
       </c>
       <c r="BB23" s="2" t="n">
-        <v>-5.7327</v>
+        <v>0.3665</v>
       </c>
       <c r="BC23" s="2" t="n">
-        <v>-2.7839</v>
+        <v>0.7698</v>
       </c>
       <c r="BD23" s="2" t="n">
-        <v>-0.638</v>
+        <v>0.6201</v>
       </c>
       <c r="BE23" s="2" t="n">
-        <v>-0.6761</v>
+        <v>0.3144</v>
       </c>
       <c r="BF23" s="2" t="n">
-        <v>0.1377</v>
+        <v>0.2861</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.279</v>
+        <v>1.34</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>46.54</v>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+        <v>3.97</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
-          <t>0111111100</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U24" s="2" t="inlineStr">
         <is>
-          <t>0110111100</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W24" s="2" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>2C</t>
-        </is>
-      </c>
-      <c r="Y24" s="2" t="inlineStr">
-        <is>
-          <t>减速·周MACD将死叉</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr"/>
       <c r="Z24" s="2" t="inlineStr"/>
       <c r="AA24" s="2" t="inlineStr"/>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="inlineStr"/>
       <c r="AD24" s="2" t="inlineStr"/>
-      <c r="AE24" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="AE24" s="2" t="inlineStr"/>
       <c r="AF24" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AG24" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="AG24" s="2" t="inlineStr"/>
       <c r="AH24" s="2" t="inlineStr"/>
-      <c r="AI24" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AI24" s="2" t="inlineStr"/>
       <c r="AJ24" s="2" t="n">
-        <v>24.79</v>
+        <v>-29.75</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>19.8</v>
+        <v>-16.33</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>2.94</v>
+        <v>-1.25</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>5.56</v>
+        <v>-2.81</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>68.5</v>
+        <v>-1.3</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="AP24" s="2" t="inlineStr"/>
-      <c r="AQ24" s="2" t="inlineStr"/>
+      <c r="AQ24" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="AR24" s="2" t="inlineStr"/>
       <c r="AS24" s="2" t="inlineStr"/>
       <c r="AT24" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU24" s="2" t="n">
-        <v>1.278</v>
+        <v>1.347</v>
       </c>
       <c r="AV24" s="2" t="n">
-        <v>1.274</v>
+        <v>1.396</v>
       </c>
       <c r="AW24" s="2" t="n">
-        <v>1.272</v>
+        <v>1.439</v>
       </c>
       <c r="AX24" s="2" t="n">
-        <v>1.286</v>
+        <v>1.474</v>
       </c>
       <c r="AY24" s="2" t="n">
-        <v>1.276</v>
+        <v>1.544</v>
       </c>
       <c r="AZ24" s="2" t="n">
-        <v>1.242</v>
+        <v>1.666</v>
       </c>
       <c r="BA24" s="2" t="n">
-        <v>1.21</v>
+        <v>1.794</v>
       </c>
       <c r="BB24" s="2" t="n">
-        <v>0.0944</v>
+        <v>-2.2516</v>
       </c>
       <c r="BC24" s="2" t="n">
-        <v>-0.2741</v>
+        <v>-1.51</v>
       </c>
       <c r="BD24" s="2" t="n">
-        <v>0.3513</v>
+        <v>-0.85</v>
       </c>
       <c r="BE24" s="2" t="n">
-        <v>0.1001</v>
+        <v>-1.0584</v>
       </c>
       <c r="BF24" s="2" t="n">
-        <v>0.2479</v>
+        <v>-0.2975</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.723</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -4281,166 +4241,158 @@
         <v>1</v>
       </c>
       <c r="S25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="V25" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W25" s="2" t="n">
-        <v>72</v>
+        <v>299</v>
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y25" s="2" t="inlineStr"/>
+          <t>2C</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>减速·周MACD死叉</t>
+        </is>
+      </c>
       <c r="Z25" s="2" t="inlineStr"/>
       <c r="AA25" s="2" t="inlineStr"/>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
-      <c r="AE25" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AE25" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AF25" s="2" t="inlineStr"/>
       <c r="AG25" s="2" t="inlineStr"/>
       <c r="AH25" s="2" t="inlineStr"/>
       <c r="AI25" s="2" t="inlineStr"/>
       <c r="AJ25" s="2" t="n">
-        <v>-29.2</v>
+        <v>12.43</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>-17.44</v>
+        <v>-0.15</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>-1.73</v>
+        <v>-5.15</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>-0.65</v>
+        <v>-19.02</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="AP25" s="2" t="inlineStr"/>
-      <c r="AQ25" s="2" t="n">
-        <v>14</v>
-      </c>
+      <c r="AQ25" s="2" t="inlineStr"/>
       <c r="AR25" s="2" t="inlineStr"/>
       <c r="AS25" s="2" t="inlineStr"/>
       <c r="AT25" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AU25" s="2" t="n">
-        <v>0.729</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="AV25" s="2" t="n">
-        <v>0.748</v>
+        <v>0.861</v>
       </c>
       <c r="AW25" s="2" t="n">
-        <v>0.774</v>
+        <v>0.95</v>
       </c>
       <c r="AX25" s="2" t="n">
-        <v>0.787</v>
+        <v>0.976</v>
       </c>
       <c r="AY25" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>1</v>
       </c>
       <c r="AZ25" s="2" t="n">
-        <v>0.888</v>
+        <v>1.098</v>
       </c>
       <c r="BA25" s="2" t="n">
-        <v>0.981</v>
+        <v>0.976</v>
       </c>
       <c r="BB25" s="2" t="n">
-        <v>-2.451</v>
+        <v>-5.6324</v>
       </c>
       <c r="BC25" s="2" t="n">
-        <v>-1.3449</v>
+        <v>-2.8877</v>
       </c>
       <c r="BD25" s="2" t="n">
-        <v>-0.5493</v>
+        <v>-0.5487</v>
       </c>
       <c r="BE25" s="2" t="n">
-        <v>-1.0903</v>
+        <v>-0.7284</v>
       </c>
       <c r="BF25" s="2" t="n">
-        <v>-0.292</v>
+        <v>0.1243</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.523</v>
+        <v>1.254</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>46.54</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0100111100</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000111100</t>
         </is>
       </c>
       <c r="V26" s="2" t="inlineStr">
@@ -4449,7 +4401,7 @@
         </is>
       </c>
       <c r="W26" s="2" t="n">
-        <v>299</v>
+        <v>55</v>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
@@ -4458,7 +4410,7 @@
       </c>
       <c r="Y26" s="2" t="inlineStr">
         <is>
-          <t>周MACD死叉</t>
+          <t>减速·周MACD将死叉</t>
         </is>
       </c>
       <c r="Z26" s="2" t="inlineStr"/>
@@ -4466,32 +4418,34 @@
       <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
-      <c r="AE26" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="AF26" s="2" t="inlineStr"/>
-      <c r="AG26" s="2" t="inlineStr"/>
-      <c r="AH26" s="2" t="inlineStr"/>
+      <c r="AE26" s="2" t="inlineStr"/>
+      <c r="AF26" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AG26" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH26" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AI26" s="2" t="inlineStr"/>
       <c r="AJ26" s="2" t="n">
-        <v>9.48</v>
+        <v>24.46</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>-3.12</v>
+        <v>17.97</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>-4.91</v>
+        <v>-0.74</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>-22.28</v>
+        <v>4.78</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>4.8</v>
+        <v>67.7</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="AP26" s="2" t="inlineStr"/>
       <c r="AQ26" s="2" t="inlineStr"/>
@@ -4499,62 +4453,62 @@
       <c r="AS26" s="2" t="inlineStr"/>
       <c r="AT26" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU26" s="2" t="n">
-        <v>0.537</v>
+        <v>1.27</v>
       </c>
       <c r="AV26" s="2" t="n">
-        <v>0.569</v>
+        <v>1.275</v>
       </c>
       <c r="AW26" s="2" t="n">
-        <v>0.625</v>
+        <v>1.27</v>
       </c>
       <c r="AX26" s="2" t="n">
-        <v>0.638</v>
+        <v>1.282</v>
       </c>
       <c r="AY26" s="2" t="n">
-        <v>0.647</v>
+        <v>1.277</v>
       </c>
       <c r="AZ26" s="2" t="n">
-        <v>0.713</v>
+        <v>1.243</v>
       </c>
       <c r="BA26" s="2" t="n">
-        <v>0.645</v>
+        <v>1.211</v>
       </c>
       <c r="BB26" s="2" t="n">
-        <v>-5.9869</v>
+        <v>0.0891</v>
       </c>
       <c r="BC26" s="2" t="n">
-        <v>-2.7022</v>
+        <v>-0.3573</v>
       </c>
       <c r="BD26" s="2" t="n">
-        <v>-0.5097</v>
+        <v>0.3283</v>
       </c>
       <c r="BE26" s="2" t="n">
-        <v>-0.7603</v>
+        <v>0.1054</v>
       </c>
       <c r="BF26" s="2" t="n">
-        <v>0.0948</v>
+        <v>0.2446</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2.058</v>
+        <v>0.718</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>2.27</v>
+        <v>3.22</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -4570,36 +4524,38 @@
       </c>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
+          <t>0000000100</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
           <t>0000000000</t>
         </is>
       </c>
-      <c r="U27" s="2" t="inlineStr">
-        <is>
-          <t>0000000000</t>
-        </is>
-      </c>
       <c r="V27" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
       <c r="W27" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
@@ -4618,22 +4574,22 @@
       <c r="AH27" s="2" t="inlineStr"/>
       <c r="AI27" s="2" t="inlineStr"/>
       <c r="AJ27" s="2" t="n">
-        <v>-31.18</v>
+        <v>-29.81</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>-18.85</v>
+        <v>-17.53</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>-3.85</v>
+        <v>-1.2</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>-2.43</v>
+        <v>-1.3</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>-2</v>
+        <v>0.9</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="AP27" s="2" t="inlineStr"/>
       <c r="AQ27" s="2" t="n">
@@ -4647,58 +4603,58 @@
         </is>
       </c>
       <c r="AU27" s="2" t="n">
-        <v>2.097</v>
+        <v>0.722</v>
       </c>
       <c r="AV27" s="2" t="n">
-        <v>2.165</v>
+        <v>0.743</v>
       </c>
       <c r="AW27" s="2" t="n">
-        <v>2.233</v>
+        <v>0.77</v>
       </c>
       <c r="AX27" s="2" t="n">
-        <v>2.279</v>
+        <v>0.783</v>
       </c>
       <c r="AY27" s="2" t="n">
-        <v>2.381</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="AZ27" s="2" t="n">
-        <v>2.59</v>
+        <v>0.884</v>
       </c>
       <c r="BA27" s="2" t="n">
-        <v>2.833</v>
+        <v>0.98</v>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>-2.2243</v>
+        <v>-2.3788</v>
       </c>
       <c r="BC27" s="2" t="n">
-        <v>-1.4254</v>
+        <v>-1.3801</v>
       </c>
       <c r="BD27" s="2" t="n">
-        <v>-0.729</v>
+        <v>-0.5959</v>
       </c>
       <c r="BE27" s="2" t="n">
-        <v>-1.0784</v>
+        <v>-1.1159</v>
       </c>
       <c r="BF27" s="2" t="n">
-        <v>-0.3118</v>
+        <v>-0.2981</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.529</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>3.87</v>
+        <v>3.91</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -4715,44 +4671,48 @@
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
+          <t>0010000000</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
           <t>0000000000</t>
         </is>
       </c>
-      <c r="U28" s="2" t="inlineStr">
-        <is>
-          <t>0000000000</t>
-        </is>
-      </c>
       <c r="V28" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W28" s="2" t="n">
-        <v>50</v>
+        <v>299</v>
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y28" s="2" t="inlineStr"/>
+          <t>2C</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>减速·周MACD死叉</t>
+        </is>
+      </c>
       <c r="Z28" s="2" t="inlineStr"/>
       <c r="AA28" s="2" t="inlineStr"/>
       <c r="AB28" s="2" t="inlineStr"/>
@@ -4766,21 +4726,23 @@
       <c r="AH28" s="2" t="inlineStr"/>
       <c r="AI28" s="2" t="inlineStr"/>
       <c r="AJ28" s="2" t="n">
-        <v>-18.03</v>
+        <v>8.25</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>-10.26</v>
+        <v>-1.56</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>0.08</v>
+        <v>-5.35</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>-1.85</v>
+        <v>-18.13</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>-5.1</v>
-      </c>
-      <c r="AO28" s="2" t="inlineStr"/>
+        <v>3.4</v>
+      </c>
+      <c r="AO28" s="2" t="n">
+        <v>39</v>
+      </c>
       <c r="AP28" s="2" t="inlineStr"/>
       <c r="AQ28" s="2" t="inlineStr"/>
       <c r="AR28" s="2" t="inlineStr"/>
@@ -4791,72 +4753,76 @@
         </is>
       </c>
       <c r="AU28" s="2" t="n">
-        <v>0.8090000000000001</v>
+        <v>0.529</v>
       </c>
       <c r="AV28" s="2" t="n">
-        <v>0.841</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="AW28" s="2" t="n">
-        <v>0.88</v>
+        <v>0.619</v>
       </c>
       <c r="AX28" s="2" t="n">
-        <v>0.902</v>
+        <v>0.633</v>
       </c>
       <c r="AY28" s="2" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.646</v>
       </c>
       <c r="AZ28" s="2" t="n">
-        <v>1.013</v>
+        <v>0.711</v>
       </c>
       <c r="BA28" s="2" t="n">
-        <v>1.023</v>
+        <v>0.645</v>
       </c>
       <c r="BB28" s="2" t="n">
-        <v>-3.2848</v>
+        <v>-5.7894</v>
       </c>
       <c r="BC28" s="2" t="n">
-        <v>-1.8214</v>
+        <v>-2.8154</v>
       </c>
       <c r="BD28" s="2" t="n">
-        <v>-0.6671</v>
+        <v>-0.4441</v>
       </c>
       <c r="BE28" s="2" t="n">
-        <v>-0.9473</v>
+        <v>-0.7949000000000001</v>
       </c>
       <c r="BF28" s="2" t="n">
-        <v>-0.1803</v>
+        <v>0.0825</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.405</v>
+        <v>2.041</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>5.56</v>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
+        <v>2.27</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -4865,7 +4831,7 @@
         <v>0</v>
       </c>
       <c r="S29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
@@ -4874,28 +4840,24 @@
       </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W29" s="2" t="n">
-        <v>299</v>
+        <v>73</v>
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y29" s="2" t="inlineStr"/>
-      <c r="Z29" s="2" t="inlineStr">
-        <is>
-          <t>2C→2A·1d</t>
-        </is>
-      </c>
+      <c r="Z29" s="2" t="inlineStr"/>
       <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="inlineStr"/>
@@ -4906,22 +4868,22 @@
       <c r="AH29" s="2" t="inlineStr"/>
       <c r="AI29" s="2" t="inlineStr"/>
       <c r="AJ29" s="2" t="n">
-        <v>4.08</v>
+        <v>-32.07</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>-3.63</v>
+        <v>-19</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>-4.29</v>
+        <v>-2.42</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>-8.99</v>
+        <v>-3.85</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-7.4</v>
+        <v>-2.2</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="AP29" s="2" t="inlineStr"/>
       <c r="AQ29" s="2" t="inlineStr"/>
@@ -4929,94 +4891,100 @@
       <c r="AS29" s="2" t="inlineStr"/>
       <c r="AT29" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU29" s="2" t="n">
-        <v>1.448</v>
+        <v>2.071</v>
       </c>
       <c r="AV29" s="2" t="n">
-        <v>1.509</v>
+        <v>2.146</v>
       </c>
       <c r="AW29" s="2" t="n">
-        <v>1.606</v>
+        <v>2.218</v>
       </c>
       <c r="AX29" s="2" t="n">
-        <v>1.635</v>
+        <v>2.264</v>
       </c>
       <c r="AY29" s="2" t="n">
-        <v>1.692</v>
+        <v>2.371</v>
       </c>
       <c r="AZ29" s="2" t="n">
-        <v>1.824</v>
+        <v>2.577</v>
       </c>
       <c r="BA29" s="2" t="n">
-        <v>1.676</v>
+        <v>2.828</v>
       </c>
       <c r="BB29" s="2" t="n">
-        <v>-4.3557</v>
+        <v>-2.2781</v>
       </c>
       <c r="BC29" s="2" t="n">
-        <v>-1.748</v>
+        <v>-1.5237</v>
       </c>
       <c r="BD29" s="2" t="n">
-        <v>-0.9835</v>
+        <v>-0.7755</v>
       </c>
       <c r="BE29" s="2" t="n">
-        <v>-0.5679</v>
+        <v>-1.1075</v>
       </c>
       <c r="BF29" s="2" t="n">
-        <v>0.0408</v>
+        <v>-0.3207</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.423</v>
+        <v>0.842</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-1.36</v>
-      </c>
-      <c r="E30" s="2" t="inlineStr"/>
+        <v>3.87</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N30" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O30" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>0000010010</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U30" s="2" t="inlineStr">
         <is>
-          <t>0001010100</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V30" s="2" t="inlineStr">
@@ -5025,112 +4993,108 @@
         </is>
       </c>
       <c r="W30" s="2" t="n">
-        <v>218</v>
+        <v>51</v>
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
-        </is>
-      </c>
-      <c r="Y30" s="2" t="inlineStr">
-        <is>
-          <t>站稳短均·日线纠缠</t>
-        </is>
-      </c>
-      <c r="Z30" s="2" t="inlineStr">
-        <is>
-          <t>4→4+·16d</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr"/>
       <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
-      <c r="AE30" s="2" t="inlineStr"/>
-      <c r="AF30" s="2" t="inlineStr"/>
+      <c r="AE30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF30" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AG30" s="2" t="inlineStr"/>
       <c r="AH30" s="2" t="inlineStr"/>
       <c r="AI30" s="2" t="inlineStr"/>
       <c r="AJ30" s="2" t="n">
-        <v>-37.19</v>
+        <v>-17.03</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>-3.98</v>
+        <v>-6.85</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>12.05</v>
+        <v>0.5</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>54.3</v>
-      </c>
-      <c r="AO30" s="2" t="n">
-        <v>76</v>
-      </c>
+        <v>-3.8</v>
+      </c>
+      <c r="AO30" s="2" t="inlineStr"/>
       <c r="AP30" s="2" t="inlineStr"/>
       <c r="AQ30" s="2" t="inlineStr"/>
       <c r="AR30" s="2" t="inlineStr"/>
       <c r="AS30" s="2" t="inlineStr"/>
       <c r="AT30" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU30" s="2" t="n">
-        <v>0.418</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AV30" s="2" t="n">
-        <v>0.417</v>
+        <v>0.835</v>
       </c>
       <c r="AW30" s="2" t="n">
-        <v>0.414</v>
+        <v>0.877</v>
       </c>
       <c r="AX30" s="2" t="n">
-        <v>0.417</v>
+        <v>0.898</v>
       </c>
       <c r="AY30" s="2" t="n">
-        <v>0.424</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="AZ30" s="2" t="n">
-        <v>0.421</v>
+        <v>1.009</v>
       </c>
       <c r="BA30" s="2" t="n">
-        <v>0.467</v>
+        <v>1.023</v>
       </c>
       <c r="BB30" s="2" t="n">
-        <v>0.3771</v>
+        <v>-3.0812</v>
       </c>
       <c r="BC30" s="2" t="n">
-        <v>-0.1948</v>
+        <v>-1.6985</v>
       </c>
       <c r="BD30" s="2" t="n">
-        <v>-0.2464</v>
+        <v>-0.6840000000000001</v>
       </c>
       <c r="BE30" s="2" t="n">
-        <v>-0.217</v>
+        <v>-0.9701</v>
       </c>
       <c r="BF30" s="2" t="n">
-        <v>-0.3719</v>
+        <v>-0.1703</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.877</v>
+        <v>1.417</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>73.68000000000001</v>
+        <v>5.56</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -5140,27 +5104,29 @@
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N31" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S31" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>1111111101</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr">
         <is>
-          <t>1111111101</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="V31" s="2" t="inlineStr">
@@ -5169,96 +5135,94 @@
         </is>
       </c>
       <c r="W31" s="2" t="n">
-        <v>54</v>
+        <v>299</v>
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>2C</t>
-        </is>
-      </c>
-      <c r="Y31" s="2" t="inlineStr">
-        <is>
-          <t>减速</t>
-        </is>
-      </c>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·14d</t>
+          <t>2C→2A·2d</t>
         </is>
       </c>
       <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
-      <c r="AE31" s="2" t="inlineStr"/>
+      <c r="AE31" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AF31" s="2" t="inlineStr"/>
       <c r="AG31" s="2" t="inlineStr"/>
       <c r="AH31" s="2" t="inlineStr"/>
       <c r="AI31" s="2" t="inlineStr"/>
       <c r="AJ31" s="2" t="n">
-        <v>8.66</v>
+        <v>2.98</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>21.42</v>
+        <v>-2.29</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>3.99</v>
+        <v>-3.26</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>12.21</v>
+        <v>-6.62</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>100.7</v>
+        <v>-7.5</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="AP31" s="2" t="inlineStr"/>
       <c r="AQ31" s="2" t="inlineStr"/>
-      <c r="AR31" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AR31" s="2" t="inlineStr"/>
       <c r="AS31" s="2" t="inlineStr"/>
       <c r="AT31" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AU31" s="2" t="n">
-        <v>0.867</v>
+        <v>1.43</v>
       </c>
       <c r="AV31" s="2" t="n">
-        <v>0.86</v>
+        <v>1.486</v>
       </c>
       <c r="AW31" s="2" t="n">
-        <v>0.85</v>
+        <v>1.596</v>
       </c>
       <c r="AX31" s="2" t="n">
-        <v>0.847</v>
+        <v>1.623</v>
       </c>
       <c r="AY31" s="2" t="n">
-        <v>0.833</v>
+        <v>1.688</v>
       </c>
       <c r="AZ31" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>1.819</v>
       </c>
       <c r="BA31" s="2" t="n">
-        <v>0.8</v>
+        <v>1.676</v>
       </c>
       <c r="BB31" s="2" t="n">
-        <v>0.9107</v>
+        <v>-4.4142</v>
       </c>
       <c r="BC31" s="2" t="n">
-        <v>0.3606</v>
+        <v>-1.7553</v>
       </c>
       <c r="BD31" s="2" t="n">
-        <v>0.2701</v>
+        <v>-0.8761</v>
       </c>
       <c r="BE31" s="2" t="n">
-        <v>0.3042</v>
+        <v>-0.6224</v>
       </c>
       <c r="BF31" s="2" t="n">
-        <v>0.0866</v>
+        <v>0.0298</v>
       </c>
     </row>
   </sheetData>
@@ -5289,7 +5253,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-19 | 30 只</t>
+          <t>截至: 2026-10-20 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-21
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.756</v>
+        <v>2.713</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-0.51</v>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
@@ -898,27 +898,25 @@
       <c r="AH2" s="2" t="inlineStr"/>
       <c r="AI2" s="2" t="inlineStr"/>
       <c r="AJ2" s="2" t="n">
-        <v>-12.25</v>
+        <v>-13.17</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>-9.65</v>
+        <v>-10.18</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>-4.28</v>
+        <v>-3.43</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>-10.58</v>
+        <v>-10.63</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-7.3</v>
+        <v>-7.7</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="AP2" s="2" t="inlineStr"/>
-      <c r="AQ2" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AQ2" s="2" t="inlineStr"/>
       <c r="AR2" s="2" t="inlineStr"/>
       <c r="AS2" s="2" t="inlineStr"/>
       <c r="AT2" s="2" t="inlineStr">
@@ -927,40 +925,40 @@
         </is>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>2.801</v>
+        <v>2.765</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>2.923</v>
+        <v>2.879</v>
       </c>
       <c r="AW2" s="2" t="n">
-        <v>3.12</v>
+        <v>3.093</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>3.199</v>
+        <v>3.175</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>3.338</v>
+        <v>3.322</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>3.624</v>
+        <v>3.61</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>3.516</v>
+        <v>3.514</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>-4.0182</v>
+        <v>-3.9395</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>-2.1931</v>
+        <v>-2.2658</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>-0.8326</v>
+        <v>-0.9385</v>
       </c>
       <c r="BE2" s="2" t="n">
-        <v>-0.7865</v>
+        <v>-0.8297</v>
       </c>
       <c r="BF2" s="2" t="n">
-        <v>-0.1225</v>
+        <v>-0.1317</v>
       </c>
     </row>
     <row r="3">
@@ -975,7 +973,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.402</v>
+        <v>1.389</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>-2.87</v>
@@ -990,7 +988,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -1017,7 +1015,7 @@
         </is>
       </c>
       <c r="W3" s="2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
@@ -1027,7 +1025,7 @@
       <c r="Y3" s="2" t="inlineStr"/>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>4+→4·8d ← 4→4+·17d</t>
+          <t>4+→4·9d ← 4→4+·18d</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr"/>
@@ -1044,22 +1042,22 @@
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="n">
-        <v>-12.77</v>
+        <v>-13.3</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>2.83</v>
+        <v>2.94</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>1.32</v>
+        <v>-0.46</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>4.09</v>
+        <v>4.16</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>42</v>
+        <v>38.2</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="AP3" s="2" t="inlineStr"/>
       <c r="AQ3" s="2" t="inlineStr"/>
@@ -1071,40 +1069,40 @@
         </is>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>1.416</v>
+        <v>1.407</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>1.421</v>
+        <v>1.414</v>
       </c>
       <c r="AW3" s="2" t="n">
-        <v>1.437</v>
+        <v>1.434</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>1.452</v>
+        <v>1.448</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>1.473</v>
+        <v>1.47</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>1.461</v>
+        <v>1.459</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>1.509</v>
+        <v>1.508</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>-0.7244</v>
+        <v>-0.785</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>-0.4858</v>
+        <v>-0.5037</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>-0.372</v>
+        <v>-0.4243</v>
       </c>
       <c r="BE3" s="2" t="n">
-        <v>-0.1644</v>
+        <v>-0.1783</v>
       </c>
       <c r="BF3" s="2" t="n">
-        <v>-0.1277</v>
+        <v>-0.133</v>
       </c>
     </row>
     <row r="4">
@@ -1119,7 +1117,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.664</v>
+        <v>0.657</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>-2.04</v>
@@ -1134,7 +1132,7 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
@@ -1143,7 +1141,7 @@
         <v>2</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
@@ -1152,7 +1150,7 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>0001010110</t>
+          <t>0000010110</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
@@ -1161,21 +1159,17 @@
         </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
-        </is>
-      </c>
-      <c r="Y4" s="2" t="inlineStr">
-        <is>
-          <t>站稳短均·日线纠缠</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>4→4+·3d ← 4+→4·4d ← 4→4+·5d</t>
+          <t>4+→4·1d ← 4→4+·4d ← 4+→4·5d</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr"/>
@@ -1185,27 +1179,31 @@
       <c r="AE4" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="n">
-        <v>-24.47</v>
+        <v>-25.04</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>4.13</v>
+        <v>2.1</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>10.27</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>68.3</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="AP4" s="2" t="inlineStr"/>
       <c r="AQ4" s="2" t="inlineStr"/>
@@ -1217,40 +1215,40 @@
         </is>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>0.664</v>
+        <v>0.663</v>
       </c>
       <c r="AV4" s="2" t="n">
         <v>0.661</v>
       </c>
       <c r="AW4" s="2" t="n">
-        <v>0.656</v>
+        <v>0.657</v>
       </c>
       <c r="AX4" s="2" t="n">
-        <v>0.662</v>
+        <v>0.661</v>
       </c>
       <c r="AY4" s="2" t="n">
-        <v>0.666</v>
+        <v>0.665</v>
       </c>
       <c r="AZ4" s="2" t="n">
-        <v>0.659</v>
+        <v>0.658</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>0.712</v>
+        <v>0.711</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>0.5321</v>
+        <v>0.4921</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>-0.0988</v>
+        <v>-0.004</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>-0.1853</v>
+        <v>-0.2025</v>
       </c>
       <c r="BE4" s="2" t="n">
-        <v>-0.1198</v>
+        <v>-0.1088</v>
       </c>
       <c r="BF4" s="2" t="n">
-        <v>-0.2447</v>
+        <v>-0.2504</v>
       </c>
     </row>
     <row r="5">
@@ -1265,7 +1263,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.827</v>
+        <v>1.81</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>95.31</v>
@@ -1315,7 +1313,7 @@
         </is>
       </c>
       <c r="W5" s="2" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
@@ -1325,7 +1323,7 @@
       <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·11d</t>
+          <t>2A→2C·12d</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr"/>
@@ -1337,32 +1335,30 @@
         <v>-1</v>
       </c>
       <c r="AG5" s="2" t="inlineStr"/>
-      <c r="AH5" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AH5" s="2" t="inlineStr"/>
       <c r="AI5" s="2" t="inlineStr"/>
       <c r="AJ5" s="2" t="n">
-        <v>55.35</v>
+        <v>53.99</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>38.74</v>
+        <v>38.51</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>-0.44</v>
+        <v>-2.3</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>9.5</v>
+        <v>7.94</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>94.40000000000001</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="AP5" s="2" t="inlineStr"/>
       <c r="AQ5" s="2" t="inlineStr"/>
       <c r="AR5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS5" s="2" t="inlineStr"/>
       <c r="AT5" s="2" t="inlineStr">
@@ -1371,40 +1367,40 @@
         </is>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>1.834</v>
+        <v>1.823</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>1.855</v>
+        <v>1.859</v>
       </c>
       <c r="AW5" s="2" t="n">
-        <v>1.806</v>
+        <v>1.807</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>1.776</v>
+        <v>1.781</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>1.677</v>
+        <v>1.683</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>1.595</v>
+        <v>1.597</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>1.539</v>
+        <v>1.542</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>1.3605</v>
+        <v>1.0997</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>0.5264</v>
+        <v>0.3826</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>1.113</v>
+        <v>1.0469</v>
       </c>
       <c r="BE5" s="2" t="n">
-        <v>0.2894</v>
+        <v>0.3042</v>
       </c>
       <c r="BF5" s="2" t="n">
-        <v>0.5535</v>
+        <v>0.5399</v>
       </c>
     </row>
     <row r="6">
@@ -1434,7 +1430,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
@@ -1461,7 +1457,7 @@
         </is>
       </c>
       <c r="W6" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
@@ -1471,43 +1467,39 @@
       <c r="Y6" s="2" t="inlineStr"/>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1→4·6d ← 1+→1·9d ← 1→1+·10d</t>
+          <t>1→4·7d ← 1+→1·10d ← 1→1+·11d</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
       <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="AF6" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AE6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="AH6" s="2" t="inlineStr"/>
       <c r="AI6" s="2" t="inlineStr"/>
       <c r="AJ6" s="2" t="n">
-        <v>-7.19</v>
+        <v>-6.28</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>8.220000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>2.68</v>
+        <v>3.56</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>7.21</v>
+        <v>8.5</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>35.5</v>
+        <v>32.5</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="AP6" s="2" t="inlineStr"/>
       <c r="AQ6" s="2" t="inlineStr"/>
@@ -1519,40 +1511,40 @@
         </is>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>0.824</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="AW6" s="2" t="n">
         <v>0.834</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>0.835</v>
+        <v>0.834</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>0.858</v>
+        <v>0.857</v>
       </c>
       <c r="AZ6" s="2" t="n">
-        <v>0.828</v>
+        <v>0.829</v>
       </c>
       <c r="BA6" s="2" t="n">
         <v>0.831</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>-1.4242</v>
+        <v>-1.4338</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>-0.3251</v>
+        <v>-0.2266</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>-0.1884</v>
+        <v>-0.2043</v>
       </c>
       <c r="BE6" s="2" t="n">
-        <v>0.06660000000000001</v>
+        <v>0.0779</v>
       </c>
       <c r="BF6" s="2" t="n">
-        <v>-0.07190000000000001</v>
+        <v>-0.06279999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -1567,7 +1559,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.877</v>
+        <v>2.856</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>2.9</v>
@@ -1611,7 +1603,7 @@
         </is>
       </c>
       <c r="W7" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
@@ -1625,29 +1617,29 @@
       <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
       <c r="AI7" s="2" t="inlineStr"/>
       <c r="AJ7" s="2" t="n">
-        <v>-7.11</v>
+        <v>-7.62</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>6.08</v>
+        <v>6.32</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>1.53</v>
+        <v>1.25</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>4.26</v>
+        <v>4.45</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>6.6</v>
+        <v>4.6</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="AP7" s="2" t="inlineStr"/>
       <c r="AQ7" s="2" t="inlineStr"/>
@@ -1659,40 +1651,40 @@
         </is>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>2.879</v>
+        <v>2.872</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>2.902</v>
+        <v>2.894</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>2.936</v>
+        <v>2.93</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>2.963</v>
+        <v>2.956</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>2.988</v>
+        <v>2.985</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>3.002</v>
+        <v>3</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>3.035</v>
+        <v>3.034</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>-0.7454</v>
+        <v>-0.6762</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>-0.54</v>
+        <v>-0.5206</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>-0.2422</v>
+        <v>-0.2414</v>
       </c>
       <c r="BE7" s="2" t="n">
-        <v>-0.1135</v>
+        <v>-0.1252</v>
       </c>
       <c r="BF7" s="2" t="n">
-        <v>-0.0711</v>
+        <v>-0.0762</v>
       </c>
     </row>
     <row r="8">
@@ -1707,7 +1699,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.22</v>
+        <v>4.185</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>4.58</v>
@@ -1757,7 +1749,7 @@
         </is>
       </c>
       <c r="W8" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
@@ -1778,22 +1770,22 @@
       <c r="AH8" s="2" t="inlineStr"/>
       <c r="AI8" s="2" t="inlineStr"/>
       <c r="AJ8" s="2" t="n">
-        <v>-8.41</v>
+        <v>-9.01</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>1.15</v>
+        <v>1.29</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>-0.04</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.02</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-4.7</v>
+        <v>-5.3</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="AP8" s="2" t="inlineStr"/>
       <c r="AQ8" s="2" t="inlineStr"/>
@@ -1805,40 +1797,40 @@
         </is>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>4.247</v>
+        <v>4.224</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>4.314</v>
+        <v>4.289</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>4.425</v>
+        <v>4.407</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>4.489</v>
+        <v>4.472</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>4.574</v>
+        <v>4.565</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>4.709</v>
+        <v>4.701</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>4.706</v>
+        <v>4.704</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>-1.5432</v>
+        <v>-1.4698</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>-1.0238</v>
+        <v>-1.0322</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>-0.4305</v>
+        <v>-0.461</v>
       </c>
       <c r="BE8" s="2" t="n">
-        <v>-0.3325</v>
+        <v>-0.3542</v>
       </c>
       <c r="BF8" s="2" t="n">
-        <v>-0.08409999999999999</v>
+        <v>-0.0901</v>
       </c>
     </row>
     <row r="9">
@@ -1853,7 +1845,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6.871</v>
+        <v>6.864</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0.97</v>
@@ -1903,7 +1895,7 @@
         </is>
       </c>
       <c r="W9" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
@@ -1916,32 +1908,30 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="inlineStr"/>
-      <c r="AE9" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AE9" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr"/>
       <c r="AI9" s="2" t="inlineStr"/>
       <c r="AJ9" s="2" t="n">
-        <v>-2.81</v>
+        <v>-3.39</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>-1.38</v>
+        <v>-0.52</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>-0.55</v>
+        <v>0.17</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>-3.1</v>
+        <v>-2.78</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.9</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="AP9" s="2" t="inlineStr"/>
       <c r="AQ9" s="2" t="inlineStr"/>
@@ -1953,40 +1943,40 @@
         </is>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>6.867</v>
+        <v>6.834</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>7.06</v>
+        <v>6.998</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>7.376</v>
+        <v>7.338</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>7.496</v>
+        <v>7.461</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>7.664</v>
+        <v>7.648</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>7.955</v>
+        <v>7.936</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>8.01</v>
+        <v>8.007999999999999</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>-2.7212</v>
+        <v>-2.5961</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>-1.4361</v>
+        <v>-1.4292</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>-0.3936</v>
+        <v>-0.4341</v>
       </c>
       <c r="BE9" s="2" t="n">
-        <v>-0.527</v>
+        <v>-0.5481</v>
       </c>
       <c r="BF9" s="2" t="n">
-        <v>-0.0281</v>
+        <v>-0.0339</v>
       </c>
     </row>
     <row r="10">
@@ -2001,7 +1991,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.416</v>
+        <v>3.385</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>41.01</v>
@@ -2022,19 +2012,19 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>8</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>0111111111</t>
+          <t>0110111101</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>0110111111</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -2043,7 +2033,7 @@
         </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
@@ -2060,35 +2050,37 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="inlineStr"/>
-      <c r="AE10" s="2" t="n">
+      <c r="AE10" s="2" t="inlineStr"/>
+      <c r="AF10" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF10" s="2" t="inlineStr"/>
       <c r="AG10" s="2" t="inlineStr"/>
-      <c r="AH10" s="2" t="inlineStr"/>
+      <c r="AH10" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AI10" s="2" t="inlineStr"/>
       <c r="AJ10" s="2" t="n">
-        <v>17.47</v>
+        <v>16.38</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>19.38</v>
+        <v>19.33</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>0.91</v>
+        <v>-1.54</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>7.64</v>
+        <v>7.62</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>86.2</v>
+        <v>85.2</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="AP10" s="2" t="inlineStr"/>
       <c r="AQ10" s="2" t="inlineStr"/>
       <c r="AR10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS10" s="2" t="inlineStr"/>
       <c r="AT10" s="2" t="inlineStr">
@@ -2097,40 +2089,40 @@
         </is>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>3.443</v>
+        <v>3.42</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>3.435</v>
+        <v>3.437</v>
       </c>
       <c r="AW10" s="2" t="n">
         <v>3.396</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>3.411</v>
+        <v>3.408</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>3.387</v>
+        <v>3.39</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>3.279</v>
+        <v>3.281</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>3.235</v>
+        <v>3.237</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.7065</v>
+        <v>0.548</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>-0.0203</v>
+        <v>-0.0586</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>0.2492</v>
+        <v>0.2122</v>
       </c>
       <c r="BE10" s="2" t="n">
-        <v>0.1962</v>
+        <v>0.1829</v>
       </c>
       <c r="BF10" s="2" t="n">
-        <v>0.1747</v>
+        <v>0.1638</v>
       </c>
     </row>
     <row r="11">
@@ -2145,7 +2137,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.486</v>
+        <v>0.482</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>-0.8100000000000001</v>
@@ -2189,7 +2181,7 @@
         </is>
       </c>
       <c r="W11" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
@@ -2199,7 +2191,7 @@
       <c r="Y11" s="2" t="inlineStr"/>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>4+→4·12d</t>
+          <t>4+→4·13d</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr"/>
@@ -2209,33 +2201,37 @@
       <c r="AE11" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AG11" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AH11" s="2" t="inlineStr"/>
+      <c r="AH11" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AI11" s="2" t="inlineStr"/>
       <c r="AJ11" s="2" t="n">
-        <v>-19.79</v>
+        <v>-20.74</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>1</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>1.28</v>
+        <v>0.27</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>5.32</v>
+        <v>5.17</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>5.3</v>
+        <v>3.3</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="AP11" s="2" t="inlineStr"/>
       <c r="AQ11" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR11" s="2" t="inlineStr"/>
       <c r="AS11" s="2" t="inlineStr"/>
@@ -2245,40 +2241,40 @@
         </is>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>0.493</v>
+        <v>0.49</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>0.492</v>
+        <v>0.491</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>0.497</v>
+        <v>0.496</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>0.505</v>
+        <v>0.503</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>0.511</v>
+        <v>0.51</v>
       </c>
       <c r="AZ11" s="2" t="n">
-        <v>0.516</v>
+        <v>0.515</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>0.529</v>
+        <v>0.528</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>-0.419</v>
+        <v>-0.3469</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>-0.5433</v>
+        <v>-0.5084</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>-0.3436</v>
+        <v>-0.3845</v>
       </c>
       <c r="BE11" s="2" t="n">
-        <v>-0.0423</v>
+        <v>-0.0534</v>
       </c>
       <c r="BF11" s="2" t="n">
-        <v>-0.1979</v>
+        <v>-0.2074</v>
       </c>
     </row>
     <row r="12">
@@ -2293,7 +2289,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.377</v>
+        <v>0.376</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>9.880000000000001</v>
@@ -2308,20 +2304,20 @@
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>4</v>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>0110111000</t>
+          <t>0010111000</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -2335,7 +2331,7 @@
         </is>
       </c>
       <c r="W12" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
@@ -2349,7 +2345,7 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>4→4+·3d ← 1→4·6d ← 1+→1·9d</t>
+          <t>4→4+·4d ← 1→4·7d ← 1+→1·10d</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr"/>
@@ -2359,28 +2355,26 @@
       <c r="AE12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AF12" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AF12" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="AG12" s="2" t="inlineStr"/>
       <c r="AH12" s="2" t="inlineStr"/>
       <c r="AI12" s="2" t="inlineStr"/>
       <c r="AJ12" s="2" t="n">
-        <v>-4.09</v>
+        <v>-3.46</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>11.75</v>
+        <v>12.55</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>3.7</v>
+        <v>3.56</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>10.65</v>
+        <v>11.53</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>56.1</v>
+        <v>55</v>
       </c>
       <c r="AO12" s="2" t="n">
         <v>62</v>
@@ -2398,7 +2392,7 @@
         <v>0.374</v>
       </c>
       <c r="AV12" s="2" t="n">
-        <v>0.377</v>
+        <v>0.376</v>
       </c>
       <c r="AW12" s="2" t="n">
         <v>0.377</v>
@@ -2410,25 +2404,25 @@
         <v>0.382</v>
       </c>
       <c r="AZ12" s="2" t="n">
-        <v>0.366</v>
+        <v>0.367</v>
       </c>
       <c r="BA12" s="2" t="n">
         <v>0.371</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>-0.3854</v>
+        <v>-0.411</v>
       </c>
       <c r="BC12" s="2" t="n">
-        <v>0.0619</v>
+        <v>0.1451</v>
       </c>
       <c r="BD12" s="2" t="n">
-        <v>0.0056</v>
+        <v>-0.0355</v>
       </c>
       <c r="BE12" s="2" t="n">
-        <v>0.1836</v>
+        <v>0.1992</v>
       </c>
       <c r="BF12" s="2" t="n">
-        <v>-0.0409</v>
+        <v>-0.0346</v>
       </c>
     </row>
     <row r="13">
@@ -2443,7 +2437,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.744</v>
+        <v>0.739</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>-4.85</v>
@@ -2458,7 +2452,9 @@
       <c r="L13" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="M13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N13" s="2" t="n">
         <v>2</v>
       </c>
@@ -2487,7 +2483,7 @@
         </is>
       </c>
       <c r="W13" s="2" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
@@ -2497,17 +2493,15 @@
       <c r="Y13" s="2" t="inlineStr"/>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>4+→4·9d ← 4→4+·12d</t>
+          <t>4+→4·10d ← 4→4+·13d</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr"/>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
-      <c r="AE13" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="AE13" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="n">
@@ -2516,22 +2510,22 @@
       <c r="AH13" s="2" t="inlineStr"/>
       <c r="AI13" s="2" t="inlineStr"/>
       <c r="AJ13" s="2" t="n">
-        <v>-23.75</v>
+        <v>-25.36</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>0.05</v>
+        <v>0.37</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>1.12</v>
+        <v>0.72</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>2.98</v>
+        <v>3.33</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>8.300000000000001</v>
+        <v>5.4</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AP13" s="2" t="inlineStr"/>
       <c r="AQ13" s="2" t="inlineStr"/>
@@ -2543,40 +2537,40 @@
         </is>
       </c>
       <c r="AU13" s="2" t="n">
-        <v>0.753</v>
+        <v>0.75</v>
       </c>
       <c r="AV13" s="2" t="n">
-        <v>0.757</v>
+        <v>0.755</v>
       </c>
       <c r="AW13" s="2" t="n">
-        <v>0.767</v>
+        <v>0.765</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>0.78</v>
+        <v>0.777</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>0.785</v>
+        <v>0.784</v>
       </c>
       <c r="AZ13" s="2" t="n">
         <v>0.786</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>0.821</v>
+        <v>0.82</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>-0.6716</v>
+        <v>-0.5877</v>
       </c>
       <c r="BC13" s="2" t="n">
-        <v>-0.7277</v>
+        <v>-0.704</v>
       </c>
       <c r="BD13" s="2" t="n">
-        <v>-0.3798</v>
+        <v>-0.4029</v>
       </c>
       <c r="BE13" s="2" t="n">
-        <v>-0.0419</v>
+        <v>-0.0481</v>
       </c>
       <c r="BF13" s="2" t="n">
-        <v>-0.2375</v>
+        <v>-0.2536</v>
       </c>
     </row>
     <row r="14">
@@ -2591,7 +2585,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.752</v>
+        <v>2.749</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>4.11</v>
@@ -2620,14 +2614,14 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
@@ -2641,7 +2635,7 @@
         </is>
       </c>
       <c r="W14" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
@@ -2662,22 +2656,22 @@
       <c r="AH14" s="2" t="inlineStr"/>
       <c r="AI14" s="2" t="inlineStr"/>
       <c r="AJ14" s="2" t="n">
-        <v>-7.32</v>
+        <v>-7.66</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>-2.17</v>
+        <v>-1.32</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>-0.7</v>
+        <v>0.3</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>-2.39</v>
+        <v>-1.94</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>9.800000000000001</v>
+        <v>8</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="AP14" s="2" t="inlineStr"/>
       <c r="AQ14" s="2" t="inlineStr"/>
@@ -2689,40 +2683,40 @@
         </is>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>2.742</v>
+        <v>2.73</v>
       </c>
       <c r="AV14" s="2" t="n">
-        <v>2.821</v>
+        <v>2.798</v>
       </c>
       <c r="AW14" s="2" t="n">
-        <v>2.949</v>
+        <v>2.935</v>
       </c>
       <c r="AX14" s="2" t="n">
-        <v>2.992</v>
+        <v>2.979</v>
       </c>
       <c r="AY14" s="2" t="n">
-        <v>3.036</v>
+        <v>3.032</v>
       </c>
       <c r="AZ14" s="2" t="n">
-        <v>3.157</v>
+        <v>3.149</v>
       </c>
       <c r="BA14" s="2" t="n">
-        <v>3.211</v>
+        <v>3.21</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>-2.8135</v>
+        <v>-2.6421</v>
       </c>
       <c r="BC14" s="2" t="n">
-        <v>-1.3958</v>
+        <v>-1.3864</v>
       </c>
       <c r="BD14" s="2" t="n">
-        <v>-0.186</v>
+        <v>-0.2392</v>
       </c>
       <c r="BE14" s="2" t="n">
-        <v>-0.6204</v>
+        <v>-0.638</v>
       </c>
       <c r="BF14" s="2" t="n">
-        <v>-0.0732</v>
+        <v>-0.0766</v>
       </c>
     </row>
     <row r="15">
@@ -2737,7 +2731,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.333</v>
+        <v>0.332</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>12.17</v>
@@ -2752,20 +2746,20 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S15" s="2" t="n">
         <v>4</v>
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>0100111100</t>
+          <t>0000111100</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
@@ -2779,7 +2773,7 @@
         </is>
       </c>
       <c r="W15" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
@@ -2793,7 +2787,7 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>4→4+·3d ← 4+→4·9d ← 4→4+·10d</t>
+          <t>4→4+·4d ← 4+→4·10d ← 4→4+·11d</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr"/>
@@ -2808,22 +2802,22 @@
       <c r="AH15" s="2" t="inlineStr"/>
       <c r="AI15" s="2" t="inlineStr"/>
       <c r="AJ15" s="2" t="n">
-        <v>-4.74</v>
+        <v>-5.19</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>9.57</v>
+        <v>10.34</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>2.72</v>
+        <v>2.91</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>8.710000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>59.5</v>
+        <v>57.8</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="AP15" s="2" t="inlineStr"/>
       <c r="AQ15" s="2" t="inlineStr"/>
@@ -2838,7 +2832,7 @@
         <v>0.328</v>
       </c>
       <c r="AV15" s="2" t="n">
-        <v>0.335</v>
+        <v>0.333</v>
       </c>
       <c r="AW15" s="2" t="n">
         <v>0.338</v>
@@ -2856,19 +2850,19 @@
         <v>0.335</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>-1.1402</v>
+        <v>-1.165</v>
       </c>
       <c r="BC15" s="2" t="n">
-        <v>-0.2309</v>
+        <v>-0.1624</v>
       </c>
       <c r="BD15" s="2" t="n">
-        <v>0.0401</v>
+        <v>-0.0029</v>
       </c>
       <c r="BE15" s="2" t="n">
         <v>0.0466</v>
       </c>
       <c r="BF15" s="2" t="n">
-        <v>-0.0474</v>
+        <v>-0.0519</v>
       </c>
     </row>
     <row r="16">
@@ -2883,7 +2877,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.07</v>
+        <v>1.063</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>71.16</v>
@@ -2900,7 +2894,7 @@
         <v>9</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -2927,7 +2921,7 @@
         </is>
       </c>
       <c r="W16" s="2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
@@ -2937,45 +2931,39 @@
       <c r="Y16" s="2" t="inlineStr"/>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>4+→4·14d ← 4→4+·17d</t>
+          <t>4+→4·15d ← 4→4+·18d</t>
         </is>
       </c>
       <c r="AA16" s="2" t="inlineStr"/>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
       <c r="AD16" s="2" t="inlineStr"/>
-      <c r="AE16" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr"/>
       <c r="AG16" s="2" t="inlineStr"/>
       <c r="AH16" s="2" t="inlineStr"/>
       <c r="AI16" s="2" t="inlineStr"/>
       <c r="AJ16" s="2" t="n">
-        <v>-16.87</v>
+        <v>-17.48</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>-5.8</v>
+        <v>-5.5</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>1.76</v>
+        <v>1.47</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>0.78</v>
+        <v>1.23</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>19.6</v>
+        <v>18.3</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="AP16" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="AP16" s="2" t="inlineStr"/>
       <c r="AQ16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR16" s="2" t="inlineStr"/>
       <c r="AS16" s="2" t="inlineStr"/>
@@ -2985,40 +2973,40 @@
         </is>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>1.061</v>
+        <v>1.059</v>
       </c>
       <c r="AV16" s="2" t="n">
-        <v>1.073</v>
+        <v>1.069</v>
       </c>
       <c r="AW16" s="2" t="n">
-        <v>1.107</v>
+        <v>1.103</v>
       </c>
       <c r="AX16" s="2" t="n">
-        <v>1.123</v>
+        <v>1.121</v>
       </c>
       <c r="AY16" s="2" t="n">
-        <v>1.127</v>
+        <v>1.126</v>
       </c>
       <c r="AZ16" s="2" t="n">
-        <v>1.172</v>
+        <v>1.169</v>
       </c>
       <c r="BA16" s="2" t="n">
         <v>1.295</v>
       </c>
       <c r="BB16" s="2" t="n">
-        <v>-1.5978</v>
+        <v>-1.3461</v>
       </c>
       <c r="BC16" s="2" t="n">
-        <v>-1.218</v>
+        <v>-1.1951</v>
       </c>
       <c r="BD16" s="2" t="n">
-        <v>-0.1206</v>
+        <v>-0.1667</v>
       </c>
       <c r="BE16" s="2" t="n">
-        <v>-0.6614</v>
+        <v>-0.6684</v>
       </c>
       <c r="BF16" s="2" t="n">
-        <v>-0.1687</v>
+        <v>-0.1748</v>
       </c>
     </row>
     <row r="17">
@@ -3033,7 +3021,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.419</v>
+        <v>0.409</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>-1.36</v>
@@ -3046,7 +3034,9 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N17" s="2" t="n">
         <v>3</v>
       </c>
@@ -3054,42 +3044,38 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="S17" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
+          <t>0000000000</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
           <t>0000010010</t>
         </is>
       </c>
-      <c r="U17" s="2" t="inlineStr">
-        <is>
-          <t>0001010100</t>
-        </is>
-      </c>
       <c r="V17" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
       <c r="W17" s="2" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
-        </is>
-      </c>
-      <c r="Y17" s="2" t="inlineStr">
-        <is>
-          <t>站稳短均·日线纠缠</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr"/>
       <c r="Z17" s="2" t="inlineStr">
         <is>
-          <t>4→4+·17d</t>
+          <t>4+→4·1d ← 4→4+·18d</t>
         </is>
       </c>
       <c r="AA17" s="2" t="inlineStr"/>
@@ -3099,27 +3085,31 @@
       <c r="AE17" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF17" s="2" t="inlineStr"/>
+      <c r="AF17" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AG17" s="2" t="inlineStr"/>
       <c r="AH17" s="2" t="inlineStr"/>
       <c r="AI17" s="2" t="inlineStr"/>
       <c r="AJ17" s="2" t="n">
-        <v>-37.04</v>
+        <v>-37.47</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>-4.3</v>
+        <v>-5.51</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>4.11</v>
+        <v>1.77</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>11.01</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>54.6</v>
+        <v>52.9</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="AP17" s="2" t="inlineStr"/>
       <c r="AQ17" s="2" t="inlineStr"/>
@@ -3131,40 +3121,40 @@
         </is>
       </c>
       <c r="AU17" s="2" t="n">
-        <v>0.419</v>
+        <v>0.418</v>
       </c>
       <c r="AV17" s="2" t="n">
-        <v>0.418</v>
+        <v>0.417</v>
       </c>
       <c r="AW17" s="2" t="n">
         <v>0.414</v>
       </c>
       <c r="AX17" s="2" t="n">
-        <v>0.418</v>
+        <v>0.417</v>
       </c>
       <c r="AY17" s="2" t="n">
-        <v>0.423</v>
+        <v>0.422</v>
       </c>
       <c r="AZ17" s="2" t="n">
         <v>0.421</v>
       </c>
       <c r="BA17" s="2" t="n">
-        <v>0.467</v>
+        <v>0.466</v>
       </c>
       <c r="BB17" s="2" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.4763</v>
       </c>
       <c r="BC17" s="2" t="n">
-        <v>-0.04</v>
+        <v>0.0684</v>
       </c>
       <c r="BD17" s="2" t="n">
-        <v>-0.3061</v>
+        <v>-0.3448</v>
       </c>
       <c r="BE17" s="2" t="n">
-        <v>-0.1992</v>
+        <v>-0.2017</v>
       </c>
       <c r="BF17" s="2" t="n">
-        <v>-0.3704</v>
+        <v>-0.3747</v>
       </c>
     </row>
     <row r="18">
@@ -3179,7 +3169,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.027</v>
+        <v>1.034</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>-0.29</v>
@@ -3198,7 +3188,7 @@
         <v>9</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -3225,7 +3215,7 @@
         </is>
       </c>
       <c r="W18" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
@@ -3250,26 +3240,30 @@
       <c r="AH18" s="2" t="inlineStr"/>
       <c r="AI18" s="2" t="inlineStr"/>
       <c r="AJ18" s="2" t="n">
-        <v>-14.86</v>
+        <v>-14.6</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>-6.09</v>
+        <v>-4.54</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>0.84</v>
+        <v>2.92</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>0.72</v>
+        <v>1.97</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-0.4</v>
+        <v>0.1</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="AP18" s="2" t="inlineStr"/>
+        <v>57</v>
+      </c>
+      <c r="AP18" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="AQ18" s="2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AR18" s="2" t="inlineStr"/>
       <c r="AS18" s="2" t="inlineStr"/>
@@ -3279,40 +3273,40 @@
         </is>
       </c>
       <c r="AU18" s="2" t="n">
-        <v>1.017</v>
+        <v>1.018</v>
       </c>
       <c r="AV18" s="2" t="n">
-        <v>1.04</v>
+        <v>1.035</v>
       </c>
       <c r="AW18" s="2" t="n">
-        <v>1.08</v>
+        <v>1.077</v>
       </c>
       <c r="AX18" s="2" t="n">
-        <v>1.104</v>
+        <v>1.099</v>
       </c>
       <c r="AY18" s="2" t="n">
-        <v>1.141</v>
+        <v>1.138</v>
       </c>
       <c r="AZ18" s="2" t="n">
-        <v>1.178</v>
+        <v>1.176</v>
       </c>
       <c r="BA18" s="2" t="n">
         <v>1.226</v>
       </c>
       <c r="BB18" s="2" t="n">
-        <v>-2.431</v>
+        <v>-2.0909</v>
       </c>
       <c r="BC18" s="2" t="n">
-        <v>-1.2783</v>
+        <v>-1.1841</v>
       </c>
       <c r="BD18" s="2" t="n">
-        <v>-0.6187</v>
+        <v>-0.6611</v>
       </c>
       <c r="BE18" s="2" t="n">
-        <v>-0.6704</v>
+        <v>-0.6623</v>
       </c>
       <c r="BF18" s="2" t="n">
-        <v>-0.1486</v>
+        <v>-0.146</v>
       </c>
     </row>
     <row r="19">
@@ -3327,7 +3321,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.882</v>
+        <v>0.887</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>4.85</v>
@@ -3344,7 +3338,7 @@
         <v>9</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
@@ -3388,32 +3382,30 @@
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="inlineStr"/>
-      <c r="AE19" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AE19" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AF19" s="2" t="inlineStr"/>
       <c r="AG19" s="2" t="inlineStr"/>
       <c r="AH19" s="2" t="inlineStr"/>
       <c r="AI19" s="2" t="inlineStr"/>
       <c r="AJ19" s="2" t="n">
-        <v>14.32</v>
+        <v>13.87</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>0.82</v>
+        <v>2.32</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>-4.36</v>
+        <v>-0.84</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>-8.06</v>
+        <v>-9.24</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>-7.8</v>
+        <v>-7.9</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="AP19" s="2" t="inlineStr"/>
       <c r="AQ19" s="2" t="inlineStr"/>
@@ -3425,40 +3417,40 @@
         </is>
       </c>
       <c r="AU19" s="2" t="n">
-        <v>0.893</v>
+        <v>0.887</v>
       </c>
       <c r="AV19" s="2" t="n">
-        <v>0.931</v>
+        <v>0.918</v>
       </c>
       <c r="AW19" s="2" t="n">
-        <v>1.002</v>
+        <v>0.995</v>
       </c>
       <c r="AX19" s="2" t="n">
-        <v>1.017</v>
+        <v>1.011</v>
       </c>
       <c r="AY19" s="2" t="n">
-        <v>1.06</v>
+        <v>1.056</v>
       </c>
       <c r="AZ19" s="2" t="n">
-        <v>1.161</v>
+        <v>1.158</v>
       </c>
       <c r="BA19" s="2" t="n">
         <v>1.031</v>
       </c>
       <c r="BB19" s="2" t="n">
-        <v>-4.6538</v>
+        <v>-4.3714</v>
       </c>
       <c r="BC19" s="2" t="n">
-        <v>-1.7275</v>
+        <v>-1.7489</v>
       </c>
       <c r="BD19" s="2" t="n">
-        <v>-0.8512999999999999</v>
+        <v>-0.8003</v>
       </c>
       <c r="BE19" s="2" t="n">
-        <v>-0.5915</v>
+        <v>-0.6767</v>
       </c>
       <c r="BF19" s="2" t="n">
-        <v>0.1432</v>
+        <v>0.1387</v>
       </c>
     </row>
     <row r="20">
@@ -3473,7 +3465,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.866</v>
+        <v>0.862</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>73.68000000000001</v>
@@ -3494,19 +3486,19 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>0111111111</t>
+          <t>0111111101</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>1111111101</t>
+          <t>0111111101</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
@@ -3515,7 +3507,7 @@
         </is>
       </c>
       <c r="W20" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
@@ -3529,7 +3521,7 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·15d</t>
+          <t>2A→2C·16d</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr"/>
@@ -3539,32 +3531,40 @@
       <c r="AE20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF20" s="2" t="inlineStr"/>
+      <c r="AF20" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AG20" s="2" t="inlineStr"/>
       <c r="AH20" s="2" t="inlineStr"/>
       <c r="AI20" s="2" t="inlineStr"/>
       <c r="AJ20" s="2" t="n">
-        <v>8.789999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>20.44</v>
+        <v>20.95</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>3.29</v>
+        <v>2.14</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>9.35</v>
+        <v>10.82</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>100.6</v>
+        <v>100</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="AP20" s="2" t="inlineStr"/>
+        <v>45</v>
+      </c>
+      <c r="AP20" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
       <c r="AQ20" s="2" t="inlineStr"/>
       <c r="AR20" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS20" s="2" t="inlineStr"/>
       <c r="AT20" s="2" t="inlineStr">
@@ -3573,40 +3573,40 @@
         </is>
       </c>
       <c r="AU20" s="2" t="n">
-        <v>0.867</v>
+        <v>0.866</v>
       </c>
       <c r="AV20" s="2" t="n">
-        <v>0.863</v>
+        <v>0.864</v>
       </c>
       <c r="AW20" s="2" t="n">
-        <v>0.85</v>
+        <v>0.851</v>
       </c>
       <c r="AX20" s="2" t="n">
         <v>0.849</v>
       </c>
       <c r="AY20" s="2" t="n">
-        <v>0.833</v>
+        <v>0.834</v>
       </c>
       <c r="AZ20" s="2" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="BA20" s="2" t="n">
         <v>0.8</v>
       </c>
       <c r="BB20" s="2" t="n">
-        <v>0.908</v>
+        <v>0.8012</v>
       </c>
       <c r="BC20" s="2" t="n">
-        <v>0.3015</v>
+        <v>0.2796</v>
       </c>
       <c r="BD20" s="2" t="n">
-        <v>0.2396</v>
+        <v>0.2444</v>
       </c>
       <c r="BE20" s="2" t="n">
-        <v>0.3117</v>
+        <v>0.3119</v>
       </c>
       <c r="BF20" s="2" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.083</v>
       </c>
     </row>
     <row r="21">
@@ -3621,7 +3621,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.996</v>
+        <v>0.98</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>-8.65</v>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="W21" s="2" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>4→4+·16d</t>
+          <t>4→4+·17d</t>
         </is>
       </c>
       <c r="AA21" s="2" t="inlineStr"/>
@@ -3695,25 +3695,27 @@
         </is>
       </c>
       <c r="AG21" s="2" t="inlineStr"/>
-      <c r="AH21" s="2" t="inlineStr"/>
+      <c r="AH21" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AI21" s="2" t="inlineStr"/>
       <c r="AJ21" s="2" t="n">
-        <v>-52.85</v>
+        <v>-53.06</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>-12.98</v>
+        <v>-13.37</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>2.8</v>
+        <v>-0.95</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>8</v>
+        <v>6.09</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>20.9</v>
+        <v>17.2</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="AP21" s="2" t="inlineStr"/>
       <c r="AQ21" s="2" t="inlineStr"/>
@@ -3725,40 +3727,40 @@
         </is>
       </c>
       <c r="AU21" s="2" t="n">
-        <v>1.008</v>
+        <v>0.999</v>
       </c>
       <c r="AV21" s="2" t="n">
-        <v>1.004</v>
+        <v>1.001</v>
       </c>
       <c r="AW21" s="2" t="n">
-        <v>1.013</v>
+        <v>1.011</v>
       </c>
       <c r="AX21" s="2" t="n">
-        <v>1.02</v>
+        <v>1.018</v>
       </c>
       <c r="AY21" s="2" t="n">
-        <v>1.061</v>
+        <v>1.057</v>
       </c>
       <c r="AZ21" s="2" t="n">
-        <v>1.071</v>
+        <v>1.069</v>
       </c>
       <c r="BA21" s="2" t="n">
-        <v>1.202</v>
+        <v>1.199</v>
       </c>
       <c r="BB21" s="2" t="n">
-        <v>-0.462</v>
+        <v>-0.4734</v>
       </c>
       <c r="BC21" s="2" t="n">
-        <v>-0.174</v>
+        <v>-0.2433</v>
       </c>
       <c r="BD21" s="2" t="n">
-        <v>-0.6343</v>
+        <v>-0.7574</v>
       </c>
       <c r="BE21" s="2" t="n">
-        <v>-0.3994</v>
+        <v>-0.4038</v>
       </c>
       <c r="BF21" s="2" t="n">
-        <v>-0.5285</v>
+        <v>-0.5306</v>
       </c>
     </row>
     <row r="22">
@@ -3773,7 +3775,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.659</v>
+        <v>1.646</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>-7.05</v>
@@ -3801,7 +3803,7 @@
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>0000001000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
@@ -3815,7 +3817,7 @@
         </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
@@ -3825,7 +3827,7 @@
       <c r="Y22" s="2" t="inlineStr"/>
       <c r="Z22" s="2" t="inlineStr">
         <is>
-          <t>4+→4·9d ← 4→4+·12d</t>
+          <t>4+→4·10d ← 4→4+·13d</t>
         </is>
       </c>
       <c r="AA22" s="2" t="inlineStr"/>
@@ -3842,22 +3844,22 @@
       <c r="AH22" s="2" t="inlineStr"/>
       <c r="AI22" s="2" t="inlineStr"/>
       <c r="AJ22" s="2" t="n">
-        <v>-23.96</v>
+        <v>-25.65</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>-3.72</v>
+        <v>-3.45</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>-1.12</v>
+        <v>-2.04</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>0.84</v>
+        <v>1.11</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>4.3</v>
+        <v>1.5</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="AP22" s="2" t="inlineStr"/>
       <c r="AQ22" s="2" t="inlineStr"/>
@@ -3869,40 +3871,40 @@
         </is>
       </c>
       <c r="AU22" s="2" t="n">
-        <v>1.706</v>
+        <v>1.689</v>
       </c>
       <c r="AV22" s="2" t="n">
-        <v>1.722</v>
+        <v>1.71</v>
       </c>
       <c r="AW22" s="2" t="n">
-        <v>1.755</v>
+        <v>1.748</v>
       </c>
       <c r="AX22" s="2" t="n">
-        <v>1.789</v>
+        <v>1.781</v>
       </c>
       <c r="AY22" s="2" t="n">
-        <v>1.81</v>
+        <v>1.807</v>
       </c>
       <c r="AZ22" s="2" t="n">
-        <v>1.809</v>
+        <v>1.808</v>
       </c>
       <c r="BA22" s="2" t="n">
-        <v>1.871</v>
+        <v>1.869</v>
       </c>
       <c r="BB22" s="2" t="n">
-        <v>-1.1257</v>
+        <v>-1.2261</v>
       </c>
       <c r="BC22" s="2" t="n">
-        <v>-0.9198</v>
+        <v>-0.968</v>
       </c>
       <c r="BD22" s="2" t="n">
-        <v>-0.3707</v>
+        <v>-0.4202</v>
       </c>
       <c r="BE22" s="2" t="n">
-        <v>-0.1167</v>
+        <v>-0.1414</v>
       </c>
       <c r="BF22" s="2" t="n">
-        <v>-0.2396</v>
+        <v>-0.2565</v>
       </c>
     </row>
     <row r="23">
@@ -3917,7 +3919,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.334</v>
+        <v>2.311</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>110.91</v>
@@ -3934,7 +3936,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -3947,7 +3949,7 @@
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>0111111011</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
@@ -3961,7 +3963,7 @@
         </is>
       </c>
       <c r="W23" s="2" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
@@ -3981,32 +3983,30 @@
       <c r="AG23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AH23" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AH23" s="2" t="inlineStr"/>
       <c r="AI23" s="2" t="inlineStr"/>
       <c r="AJ23" s="2" t="n">
-        <v>28.61</v>
+        <v>27.96</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>29.57</v>
+        <v>29.34</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>0.51</v>
+        <v>-2.59</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>13.65</v>
+        <v>12.51</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>86.40000000000001</v>
+        <v>85.5</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="AP23" s="2" t="inlineStr"/>
       <c r="AQ23" s="2" t="inlineStr"/>
       <c r="AR23" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AS23" s="2" t="inlineStr"/>
       <c r="AT23" s="2" t="inlineStr">
@@ -4015,40 +4015,40 @@
         </is>
       </c>
       <c r="AU23" s="2" t="n">
-        <v>2.351</v>
+        <v>2.333</v>
       </c>
       <c r="AV23" s="2" t="n">
-        <v>2.366</v>
+        <v>2.361</v>
       </c>
       <c r="AW23" s="2" t="n">
-        <v>2.322</v>
+        <v>2.327</v>
       </c>
       <c r="AX23" s="2" t="n">
-        <v>2.286</v>
+        <v>2.289</v>
       </c>
       <c r="AY23" s="2" t="n">
-        <v>2.262</v>
+        <v>2.265</v>
       </c>
       <c r="AZ23" s="2" t="n">
-        <v>2.222</v>
+        <v>2.223</v>
       </c>
       <c r="BA23" s="2" t="n">
-        <v>2.048</v>
+        <v>2.051</v>
       </c>
       <c r="BB23" s="2" t="n">
-        <v>0.3665</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="BC23" s="2" t="n">
-        <v>0.7698</v>
+        <v>0.7091</v>
       </c>
       <c r="BD23" s="2" t="n">
-        <v>0.6201</v>
+        <v>0.5199</v>
       </c>
       <c r="BE23" s="2" t="n">
-        <v>0.3144</v>
+        <v>0.2544</v>
       </c>
       <c r="BF23" s="2" t="n">
-        <v>0.2861</v>
+        <v>0.2796</v>
       </c>
     </row>
     <row r="24">
@@ -4063,7 +4063,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.34</v>
+        <v>1.293</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>3.97</v>
@@ -4111,7 +4111,7 @@
         </is>
       </c>
       <c r="W24" s="2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
@@ -4125,33 +4125,31 @@
       <c r="AC24" s="2" t="inlineStr"/>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="inlineStr"/>
-      <c r="AF24" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AF24" s="2" t="inlineStr"/>
       <c r="AG24" s="2" t="inlineStr"/>
       <c r="AH24" s="2" t="inlineStr"/>
       <c r="AI24" s="2" t="inlineStr"/>
       <c r="AJ24" s="2" t="n">
-        <v>-29.75</v>
+        <v>-30.1</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>-16.33</v>
+        <v>-18.4</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>-1.25</v>
+        <v>-2.27</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>-2.81</v>
+        <v>-4.14</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>-1.3</v>
+        <v>-1.8</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="AP24" s="2" t="inlineStr"/>
       <c r="AQ24" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AR24" s="2" t="inlineStr"/>
       <c r="AS24" s="2" t="inlineStr"/>
@@ -4161,40 +4159,40 @@
         </is>
       </c>
       <c r="AU24" s="2" t="n">
-        <v>1.347</v>
+        <v>1.332</v>
       </c>
       <c r="AV24" s="2" t="n">
-        <v>1.396</v>
+        <v>1.38</v>
       </c>
       <c r="AW24" s="2" t="n">
-        <v>1.439</v>
+        <v>1.43</v>
       </c>
       <c r="AX24" s="2" t="n">
-        <v>1.474</v>
+        <v>1.464</v>
       </c>
       <c r="AY24" s="2" t="n">
-        <v>1.544</v>
+        <v>1.537</v>
       </c>
       <c r="AZ24" s="2" t="n">
-        <v>1.666</v>
+        <v>1.659</v>
       </c>
       <c r="BA24" s="2" t="n">
-        <v>1.794</v>
+        <v>1.791</v>
       </c>
       <c r="BB24" s="2" t="n">
-        <v>-2.2516</v>
+        <v>-2.3355</v>
       </c>
       <c r="BC24" s="2" t="n">
-        <v>-1.51</v>
+        <v>-1.5472</v>
       </c>
       <c r="BD24" s="2" t="n">
-        <v>-0.85</v>
+        <v>-0.9353</v>
       </c>
       <c r="BE24" s="2" t="n">
-        <v>-1.0584</v>
+        <v>-1.081</v>
       </c>
       <c r="BF24" s="2" t="n">
-        <v>-0.2975</v>
+        <v>-0.301</v>
       </c>
     </row>
     <row r="25">
@@ -4209,7 +4207,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.823</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>3.37</v>
@@ -4232,7 +4230,7 @@
         <v>9</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
@@ -4284,22 +4282,22 @@
       <c r="AH25" s="2" t="inlineStr"/>
       <c r="AI25" s="2" t="inlineStr"/>
       <c r="AJ25" s="2" t="n">
-        <v>12.43</v>
+        <v>12.01</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>-0.15</v>
+        <v>1.84</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>-5.15</v>
+        <v>-0.51</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>-19.02</v>
+        <v>-17.04</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>0.5</v>
+        <v>-0.4</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="AP25" s="2" t="inlineStr"/>
       <c r="AQ25" s="2" t="inlineStr"/>
@@ -4311,40 +4309,40 @@
         </is>
       </c>
       <c r="AU25" s="2" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="AV25" s="2" t="n">
-        <v>0.861</v>
+        <v>0.847</v>
       </c>
       <c r="AW25" s="2" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AX25" s="2" t="n">
-        <v>0.976</v>
+        <v>0.969</v>
       </c>
       <c r="AY25" s="2" t="n">
-        <v>1</v>
+        <v>0.996</v>
       </c>
       <c r="AZ25" s="2" t="n">
-        <v>1.098</v>
+        <v>1.094</v>
       </c>
       <c r="BA25" s="2" t="n">
         <v>0.976</v>
       </c>
       <c r="BB25" s="2" t="n">
-        <v>-5.6324</v>
+        <v>-5.2646</v>
       </c>
       <c r="BC25" s="2" t="n">
-        <v>-2.8877</v>
+        <v>-2.8928</v>
       </c>
       <c r="BD25" s="2" t="n">
-        <v>-0.5487</v>
+        <v>-0.6046</v>
       </c>
       <c r="BE25" s="2" t="n">
-        <v>-0.7284</v>
+        <v>-0.7766</v>
       </c>
       <c r="BF25" s="2" t="n">
-        <v>0.1243</v>
+        <v>0.1201</v>
       </c>
     </row>
     <row r="26">
@@ -4359,7 +4357,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.254</v>
+        <v>1.237</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>46.54</v>
@@ -4383,16 +4381,16 @@
         <v>5</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>0100111100</t>
+          <t>0110011100</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
         <is>
-          <t>0000111100</t>
+          <t>0000111000</t>
         </is>
       </c>
       <c r="V26" s="2" t="inlineStr">
@@ -4401,7 +4399,7 @@
         </is>
       </c>
       <c r="W26" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
@@ -4430,22 +4428,22 @@
       </c>
       <c r="AI26" s="2" t="inlineStr"/>
       <c r="AJ26" s="2" t="n">
-        <v>24.46</v>
+        <v>22.89</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>17.97</v>
+        <v>17.36</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>-0.74</v>
+        <v>-3.84</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>4.78</v>
+        <v>3.78</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>67.7</v>
+        <v>66.2</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="AP26" s="2" t="inlineStr"/>
       <c r="AQ26" s="2" t="inlineStr"/>
@@ -4457,40 +4455,40 @@
         </is>
       </c>
       <c r="AU26" s="2" t="n">
-        <v>1.27</v>
+        <v>1.257</v>
       </c>
       <c r="AV26" s="2" t="n">
-        <v>1.275</v>
+        <v>1.273</v>
       </c>
       <c r="AW26" s="2" t="n">
-        <v>1.27</v>
+        <v>1.269</v>
       </c>
       <c r="AX26" s="2" t="n">
-        <v>1.282</v>
+        <v>1.278</v>
       </c>
       <c r="AY26" s="2" t="n">
-        <v>1.277</v>
+        <v>1.279</v>
       </c>
       <c r="AZ26" s="2" t="n">
         <v>1.243</v>
       </c>
       <c r="BA26" s="2" t="n">
-        <v>1.211</v>
+        <v>1.212</v>
       </c>
       <c r="BB26" s="2" t="n">
-        <v>0.0891</v>
+        <v>-0.0332</v>
       </c>
       <c r="BC26" s="2" t="n">
-        <v>-0.3573</v>
+        <v>-0.4259</v>
       </c>
       <c r="BD26" s="2" t="n">
-        <v>0.3283</v>
+        <v>0.2756</v>
       </c>
       <c r="BE26" s="2" t="n">
-        <v>0.1054</v>
+        <v>0.0919</v>
       </c>
       <c r="BF26" s="2" t="n">
-        <v>0.2446</v>
+        <v>0.2289</v>
       </c>
     </row>
     <row r="27">
@@ -4505,7 +4503,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.718</v>
+        <v>0.717</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>3.22</v>
@@ -4555,7 +4553,7 @@
         </is>
       </c>
       <c r="W27" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
@@ -4568,33 +4566,35 @@
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="inlineStr"/>
       <c r="AD27" s="2" t="inlineStr"/>
-      <c r="AE27" s="2" t="inlineStr"/>
+      <c r="AE27" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AF27" s="2" t="inlineStr"/>
       <c r="AG27" s="2" t="inlineStr"/>
       <c r="AH27" s="2" t="inlineStr"/>
       <c r="AI27" s="2" t="inlineStr"/>
       <c r="AJ27" s="2" t="n">
-        <v>-29.81</v>
+        <v>-29.92</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>-17.53</v>
+        <v>-16.79</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>-1.2</v>
+        <v>-0.06</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>-1.3</v>
+        <v>-0.51</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="AP27" s="2" t="inlineStr"/>
-      <c r="AQ27" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="AQ27" s="2" t="inlineStr"/>
       <c r="AR27" s="2" t="inlineStr"/>
       <c r="AS27" s="2" t="inlineStr"/>
       <c r="AT27" s="2" t="inlineStr">
@@ -4603,40 +4603,40 @@
         </is>
       </c>
       <c r="AU27" s="2" t="n">
-        <v>0.722</v>
+        <v>0.718</v>
       </c>
       <c r="AV27" s="2" t="n">
-        <v>0.743</v>
+        <v>0.737</v>
       </c>
       <c r="AW27" s="2" t="n">
-        <v>0.77</v>
+        <v>0.767</v>
       </c>
       <c r="AX27" s="2" t="n">
-        <v>0.783</v>
+        <v>0.78</v>
       </c>
       <c r="AY27" s="2" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AZ27" s="2" t="n">
-        <v>0.884</v>
+        <v>0.88</v>
       </c>
       <c r="BA27" s="2" t="n">
-        <v>0.98</v>
+        <v>0.979</v>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>-2.3788</v>
+        <v>-2.2682</v>
       </c>
       <c r="BC27" s="2" t="n">
-        <v>-1.3801</v>
+        <v>-1.3509</v>
       </c>
       <c r="BD27" s="2" t="n">
-        <v>-0.5959</v>
+        <v>-0.6603</v>
       </c>
       <c r="BE27" s="2" t="n">
-        <v>-1.1159</v>
+        <v>-1.1453</v>
       </c>
       <c r="BF27" s="2" t="n">
-        <v>-0.2981</v>
+        <v>-0.2992</v>
       </c>
     </row>
     <row r="28">
@@ -4651,7 +4651,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.529</v>
+        <v>0.535</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>3.91</v>
@@ -4674,25 +4674,25 @@
         <v>13</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S28" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
+          <t>0000000000</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
           <t>0010000000</t>
-        </is>
-      </c>
-      <c r="U28" s="2" t="inlineStr">
-        <is>
-          <t>0000000000</t>
         </is>
       </c>
       <c r="V28" s="2" t="inlineStr">
@@ -4726,22 +4726,22 @@
       <c r="AH28" s="2" t="inlineStr"/>
       <c r="AI28" s="2" t="inlineStr"/>
       <c r="AJ28" s="2" t="n">
-        <v>8.25</v>
+        <v>7.82</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>-1.56</v>
+        <v>0.43</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>-5.35</v>
+        <v>-0.28</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>-18.13</v>
+        <v>-16.04</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>3.4</v>
+        <v>2.4</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="AP28" s="2" t="inlineStr"/>
       <c r="AQ28" s="2" t="inlineStr"/>
@@ -4753,40 +4753,40 @@
         </is>
       </c>
       <c r="AU28" s="2" t="n">
-        <v>0.529</v>
+        <v>0.526</v>
       </c>
       <c r="AV28" s="2" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="AW28" s="2" t="n">
-        <v>0.619</v>
+        <v>0.613</v>
       </c>
       <c r="AX28" s="2" t="n">
-        <v>0.633</v>
+        <v>0.629</v>
       </c>
       <c r="AY28" s="2" t="n">
-        <v>0.646</v>
+        <v>0.644</v>
       </c>
       <c r="AZ28" s="2" t="n">
-        <v>0.711</v>
+        <v>0.709</v>
       </c>
       <c r="BA28" s="2" t="n">
         <v>0.645</v>
       </c>
       <c r="BB28" s="2" t="n">
-        <v>-5.7894</v>
+        <v>-5.3626</v>
       </c>
       <c r="BC28" s="2" t="n">
-        <v>-2.8154</v>
+        <v>-2.8221</v>
       </c>
       <c r="BD28" s="2" t="n">
-        <v>-0.4441</v>
+        <v>-0.5248</v>
       </c>
       <c r="BE28" s="2" t="n">
-        <v>-0.7949000000000001</v>
+        <v>-0.8229</v>
       </c>
       <c r="BF28" s="2" t="n">
-        <v>0.0825</v>
+        <v>0.07820000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -4801,7 +4801,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2.041</v>
+        <v>1.984</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>2.27</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="W29" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
@@ -4868,22 +4868,22 @@
       <c r="AH29" s="2" t="inlineStr"/>
       <c r="AI29" s="2" t="inlineStr"/>
       <c r="AJ29" s="2" t="n">
-        <v>-32.07</v>
+        <v>-32.58</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>-19</v>
+        <v>-20.48</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>-2.42</v>
+        <v>-3.19</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>-3.85</v>
+        <v>-5.07</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-2.2</v>
+        <v>-2.6</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="AP29" s="2" t="inlineStr"/>
       <c r="AQ29" s="2" t="inlineStr"/>
@@ -4895,40 +4895,40 @@
         </is>
       </c>
       <c r="AU29" s="2" t="n">
-        <v>2.071</v>
+        <v>2.044</v>
       </c>
       <c r="AV29" s="2" t="n">
-        <v>2.146</v>
+        <v>2.122</v>
       </c>
       <c r="AW29" s="2" t="n">
-        <v>2.218</v>
+        <v>2.204</v>
       </c>
       <c r="AX29" s="2" t="n">
-        <v>2.264</v>
+        <v>2.251</v>
       </c>
       <c r="AY29" s="2" t="n">
-        <v>2.371</v>
+        <v>2.363</v>
       </c>
       <c r="AZ29" s="2" t="n">
-        <v>2.577</v>
+        <v>2.567</v>
       </c>
       <c r="BA29" s="2" t="n">
-        <v>2.828</v>
+        <v>2.826</v>
       </c>
       <c r="BB29" s="2" t="n">
-        <v>-2.2781</v>
+        <v>-2.4056</v>
       </c>
       <c r="BC29" s="2" t="n">
-        <v>-1.5237</v>
+        <v>-1.6205</v>
       </c>
       <c r="BD29" s="2" t="n">
-        <v>-0.7755</v>
+        <v>-0.8685</v>
       </c>
       <c r="BE29" s="2" t="n">
-        <v>-1.1075</v>
+        <v>-1.1352</v>
       </c>
       <c r="BF29" s="2" t="n">
-        <v>-0.3207</v>
+        <v>-0.3258</v>
       </c>
     </row>
     <row r="30">
@@ -4943,7 +4943,7 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.842</v>
+        <v>0.837</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>3.87</v>
@@ -4993,7 +4993,7 @@
         </is>
       </c>
       <c r="W30" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
@@ -5009,28 +5009,24 @@
       <c r="AE30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AF30" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="AF30" s="2" t="inlineStr"/>
       <c r="AG30" s="2" t="inlineStr"/>
       <c r="AH30" s="2" t="inlineStr"/>
       <c r="AI30" s="2" t="inlineStr"/>
       <c r="AJ30" s="2" t="n">
-        <v>-17.03</v>
+        <v>-15.82</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>-6.85</v>
+        <v>-6.45</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>3.6</v>
+        <v>5.3</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>0.5</v>
+        <v>1.06</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>-3.8</v>
+        <v>-2.6</v>
       </c>
       <c r="AO30" s="2" t="inlineStr"/>
       <c r="AP30" s="2" t="inlineStr"/>
@@ -5043,40 +5039,40 @@
         </is>
       </c>
       <c r="AU30" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="AV30" s="2" t="n">
-        <v>0.835</v>
+        <v>0.829</v>
       </c>
       <c r="AW30" s="2" t="n">
-        <v>0.877</v>
+        <v>0.873</v>
       </c>
       <c r="AX30" s="2" t="n">
-        <v>0.898</v>
+        <v>0.894</v>
       </c>
       <c r="AY30" s="2" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.93</v>
       </c>
       <c r="AZ30" s="2" t="n">
-        <v>1.009</v>
+        <v>1.005</v>
       </c>
       <c r="BA30" s="2" t="n">
-        <v>1.023</v>
+        <v>1.022</v>
       </c>
       <c r="BB30" s="2" t="n">
-        <v>-3.0812</v>
+        <v>-2.7615</v>
       </c>
       <c r="BC30" s="2" t="n">
-        <v>-1.6985</v>
+        <v>-1.5121</v>
       </c>
       <c r="BD30" s="2" t="n">
-        <v>-0.6840000000000001</v>
+        <v>-0.733</v>
       </c>
       <c r="BE30" s="2" t="n">
-        <v>-0.9701</v>
+        <v>-0.9781</v>
       </c>
       <c r="BF30" s="2" t="n">
-        <v>-0.1703</v>
+        <v>-0.1582</v>
       </c>
     </row>
     <row r="31">
@@ -5091,7 +5087,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.417</v>
+        <v>1.418</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>5.56</v>
@@ -5131,53 +5127,51 @@
       </c>
       <c r="V31" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W31" s="2" t="n">
-        <v>299</v>
+        <v>3</v>
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>2C→2A·2d</t>
+          <t>2C→4·3d</t>
         </is>
       </c>
       <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
-      <c r="AE31" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AE31" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AF31" s="2" t="inlineStr"/>
       <c r="AG31" s="2" t="inlineStr"/>
       <c r="AH31" s="2" t="inlineStr"/>
       <c r="AI31" s="2" t="inlineStr"/>
       <c r="AJ31" s="2" t="n">
-        <v>2.98</v>
+        <v>2.61</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>-2.29</v>
+        <v>-1.27</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>-3.26</v>
+        <v>-0.29</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>-6.62</v>
+        <v>-7.87</v>
       </c>
       <c r="AN31" s="2" t="n">
         <v>-7.5</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="AP31" s="2" t="inlineStr"/>
       <c r="AQ31" s="2" t="inlineStr"/>
@@ -5189,40 +5183,40 @@
         </is>
       </c>
       <c r="AU31" s="2" t="n">
-        <v>1.43</v>
+        <v>1.422</v>
       </c>
       <c r="AV31" s="2" t="n">
-        <v>1.486</v>
+        <v>1.466</v>
       </c>
       <c r="AW31" s="2" t="n">
-        <v>1.596</v>
+        <v>1.585</v>
       </c>
       <c r="AX31" s="2" t="n">
-        <v>1.623</v>
+        <v>1.613</v>
       </c>
       <c r="AY31" s="2" t="n">
-        <v>1.688</v>
+        <v>1.682</v>
       </c>
       <c r="AZ31" s="2" t="n">
-        <v>1.819</v>
+        <v>1.813</v>
       </c>
       <c r="BA31" s="2" t="n">
-        <v>1.676</v>
+        <v>1.677</v>
       </c>
       <c r="BB31" s="2" t="n">
-        <v>-4.4142</v>
+        <v>-4.1644</v>
       </c>
       <c r="BC31" s="2" t="n">
-        <v>-1.7553</v>
+        <v>-1.7625</v>
       </c>
       <c r="BD31" s="2" t="n">
-        <v>-0.8761</v>
+        <v>-0.8557</v>
       </c>
       <c r="BE31" s="2" t="n">
-        <v>-0.6224</v>
+        <v>-0.6901</v>
       </c>
       <c r="BF31" s="2" t="n">
-        <v>0.0298</v>
+        <v>0.0261</v>
       </c>
     </row>
   </sheetData>
@@ -5253,7 +5247,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-20 | 30 只</t>
+          <t>截至: 2026-10-21 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-22
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.713</v>
+        <v>2.592</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-0.51</v>
@@ -852,7 +852,7 @@
         <v>9</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
@@ -891,29 +891,31 @@
       <c r="AA2" s="2" t="inlineStr"/>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr"/>
-      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr"/>
       <c r="AH2" s="2" t="inlineStr"/>
       <c r="AI2" s="2" t="inlineStr"/>
       <c r="AJ2" s="2" t="n">
-        <v>-13.17</v>
+        <v>-14.26</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>-10.18</v>
+        <v>-12.55</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>-3.43</v>
+        <v>-4.19</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>-10.63</v>
+        <v>-14.16</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-7.7</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="AP2" s="2" t="inlineStr"/>
       <c r="AQ2" s="2" t="inlineStr"/>
@@ -925,40 +927,40 @@
         </is>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>2.765</v>
+        <v>2.722</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>2.879</v>
+        <v>2.833</v>
       </c>
       <c r="AW2" s="2" t="n">
-        <v>3.093</v>
+        <v>3.056</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>3.175</v>
+        <v>3.151</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>3.322</v>
+        <v>3.303</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>3.61</v>
+        <v>3.596</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>3.514</v>
+        <v>3.511</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>-3.9395</v>
+        <v>-3.7913</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>-2.2658</v>
+        <v>-2.4245</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>-0.9385</v>
+        <v>-1.0566</v>
       </c>
       <c r="BE2" s="2" t="n">
-        <v>-0.8297</v>
+        <v>-0.8815</v>
       </c>
       <c r="BF2" s="2" t="n">
-        <v>-0.1317</v>
+        <v>-0.1426</v>
       </c>
     </row>
     <row r="3">
@@ -973,7 +975,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.389</v>
+        <v>1.345</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>-2.87</v>
@@ -988,7 +990,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -1015,7 +1017,7 @@
         </is>
       </c>
       <c r="W3" s="2" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
@@ -1025,7 +1027,7 @@
       <c r="Y3" s="2" t="inlineStr"/>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>4+→4·9d ← 4→4+·18d</t>
+          <t>4+→4·10d ← 4→4+·19d</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr"/>
@@ -1042,22 +1044,22 @@
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="n">
-        <v>-13.3</v>
+        <v>-14.11</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>2.94</v>
+        <v>1.53</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>-0.46</v>
+        <v>-1.52</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>4.16</v>
+        <v>3.44</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>38.2</v>
+        <v>31.9</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="AP3" s="2" t="inlineStr"/>
       <c r="AQ3" s="2" t="inlineStr"/>
@@ -1069,40 +1071,40 @@
         </is>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>1.407</v>
+        <v>1.395</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>1.414</v>
+        <v>1.409</v>
       </c>
       <c r="AW3" s="2" t="n">
-        <v>1.434</v>
+        <v>1.429</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>1.448</v>
+        <v>1.444</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>1.47</v>
+        <v>1.467</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>1.459</v>
+        <v>1.458</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>1.508</v>
+        <v>1.507</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>-0.785</v>
+        <v>-0.8188</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>-0.5037</v>
+        <v>-0.57</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>-0.4243</v>
+        <v>-0.4718</v>
       </c>
       <c r="BE3" s="2" t="n">
-        <v>-0.1783</v>
+        <v>-0.1973</v>
       </c>
       <c r="BF3" s="2" t="n">
-        <v>-0.133</v>
+        <v>-0.1411</v>
       </c>
     </row>
     <row r="4">
@@ -1117,7 +1119,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.657</v>
+        <v>0.654</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>-2.04</v>
@@ -1138,14 +1140,14 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>0000010100</t>
+          <t>0000010110</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -1159,7 +1161,7 @@
         </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
@@ -1169,7 +1171,7 @@
       <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>4+→4·1d ← 4→4+·4d ← 4+→4·5d</t>
+          <t>4+→4·2d ← 4→4+·5d ← 4+→4·6d</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr"/>
@@ -1188,22 +1190,22 @@
       <c r="AH4" s="2" t="inlineStr"/>
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="n">
-        <v>-25.04</v>
+        <v>-25.83</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>1.13</v>
+        <v>2.61</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>2.1</v>
+        <v>2.58</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>9.949999999999999</v>
+        <v>12.76</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>66.59999999999999</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="AP4" s="2" t="inlineStr"/>
       <c r="AQ4" s="2" t="inlineStr"/>
@@ -1215,7 +1217,7 @@
         </is>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>0.663</v>
+        <v>0.662</v>
       </c>
       <c r="AV4" s="2" t="n">
         <v>0.661</v>
@@ -1233,22 +1235,22 @@
         <v>0.658</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>0.711</v>
+        <v>0.71</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>0.4921</v>
+        <v>0.468</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>-0.004</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>-0.2025</v>
+        <v>-0.2042</v>
       </c>
       <c r="BE4" s="2" t="n">
-        <v>-0.1088</v>
+        <v>-0.0978</v>
       </c>
       <c r="BF4" s="2" t="n">
-        <v>-0.2504</v>
+        <v>-0.2583</v>
       </c>
     </row>
     <row r="5">
@@ -1263,7 +1265,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.81</v>
+        <v>1.829</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>95.31</v>
@@ -1292,28 +1294,28 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S5" s="2" t="n">
         <v>8</v>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
+          <t>0111111111</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
           <t>0111111101</t>
         </is>
       </c>
-      <c r="U5" s="2" t="inlineStr">
-        <is>
-          <t>0111111101</t>
-        </is>
-      </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="W5" s="2" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
@@ -1323,14 +1325,18 @@
       <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·12d</t>
+          <t>2A→2C·13d</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr"/>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="n">
         <v>-1</v>
       </c>
@@ -1338,27 +1344,27 @@
       <c r="AH5" s="2" t="inlineStr"/>
       <c r="AI5" s="2" t="inlineStr"/>
       <c r="AJ5" s="2" t="n">
-        <v>53.99</v>
+        <v>53.21</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>38.51</v>
+        <v>42.28</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>-2.3</v>
+        <v>2.9</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>7.94</v>
+        <v>10.31</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>92.90000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="AP5" s="2" t="inlineStr"/>
       <c r="AQ5" s="2" t="inlineStr"/>
       <c r="AR5" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS5" s="2" t="inlineStr"/>
       <c r="AT5" s="2" t="inlineStr">
@@ -1367,40 +1373,40 @@
         </is>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>1.823</v>
+        <v>1.822</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>1.859</v>
+        <v>1.848</v>
       </c>
       <c r="AW5" s="2" t="n">
-        <v>1.807</v>
+        <v>1.808</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>1.781</v>
+        <v>1.786</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>1.683</v>
+        <v>1.691</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>1.597</v>
+        <v>1.6</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>1.542</v>
+        <v>1.545</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>1.0997</v>
+        <v>0.3512</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>0.3826</v>
+        <v>0.2849</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>1.0469</v>
+        <v>1.0544</v>
       </c>
       <c r="BE5" s="2" t="n">
-        <v>0.3042</v>
+        <v>0.332</v>
       </c>
       <c r="BF5" s="2" t="n">
-        <v>0.5399</v>
+        <v>0.5321</v>
       </c>
     </row>
     <row r="6">
@@ -1415,7 +1421,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.791</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>7.37</v>
@@ -1436,19 +1442,19 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>0010011000</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>0010011000</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
@@ -1457,7 +1463,7 @@
         </is>
       </c>
       <c r="W6" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
@@ -1467,7 +1473,7 @@
       <c r="Y6" s="2" t="inlineStr"/>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1→4·7d ← 1+→1·10d ← 1→1+·11d</t>
+          <t>1→4·8d ← 1+→1·11d ← 1→1+·12d</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr"/>
@@ -1475,7 +1481,7 @@
       <c r="AC6" s="2" t="inlineStr"/>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="n">
@@ -1484,22 +1490,22 @@
       <c r="AH6" s="2" t="inlineStr"/>
       <c r="AI6" s="2" t="inlineStr"/>
       <c r="AJ6" s="2" t="n">
-        <v>-6.28</v>
+        <v>-6.5</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>9.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>3.56</v>
+        <v>1.01</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>8.5</v>
+        <v>7.41</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>32.5</v>
+        <v>27</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="AP6" s="2" t="inlineStr"/>
       <c r="AQ6" s="2" t="inlineStr"/>
@@ -1511,19 +1517,19 @@
         </is>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.804</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="AW6" s="2" t="n">
-        <v>0.834</v>
+        <v>0.832</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>0.834</v>
+        <v>0.832</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>0.857</v>
+        <v>0.856</v>
       </c>
       <c r="AZ6" s="2" t="n">
         <v>0.829</v>
@@ -1532,19 +1538,19 @@
         <v>0.831</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>-1.4338</v>
+        <v>-1.3694</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>-0.2266</v>
+        <v>-0.2518</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>-0.2043</v>
+        <v>-0.2468</v>
       </c>
       <c r="BE6" s="2" t="n">
-        <v>0.0779</v>
+        <v>0.076</v>
       </c>
       <c r="BF6" s="2" t="n">
-        <v>-0.06279999999999999</v>
+        <v>-0.065</v>
       </c>
     </row>
     <row r="7">
@@ -1559,7 +1565,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.856</v>
+        <v>2.836</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>2.9</v>
@@ -1603,7 +1609,7 @@
         </is>
       </c>
       <c r="W7" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
@@ -1624,22 +1630,22 @@
       <c r="AH7" s="2" t="inlineStr"/>
       <c r="AI7" s="2" t="inlineStr"/>
       <c r="AJ7" s="2" t="n">
-        <v>-7.62</v>
+        <v>-8.17</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>6.32</v>
+        <v>7.52</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>1.25</v>
+        <v>1.81</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>4.45</v>
+        <v>5.57</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>4.6</v>
+        <v>2.5</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="AP7" s="2" t="inlineStr"/>
       <c r="AQ7" s="2" t="inlineStr"/>
@@ -1651,40 +1657,40 @@
         </is>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>2.872</v>
+        <v>2.864</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>2.894</v>
+        <v>2.885</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>2.93</v>
+        <v>2.923</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>2.956</v>
+        <v>2.95</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>2.985</v>
+        <v>2.981</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>3</v>
+        <v>2.998</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>3.034</v>
+        <v>3.033</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>-0.6762</v>
+        <v>-0.6028</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>-0.5206</v>
+        <v>-0.5194</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>-0.2414</v>
+        <v>-0.257</v>
       </c>
       <c r="BE7" s="2" t="n">
-        <v>-0.1252</v>
+        <v>-0.1354</v>
       </c>
       <c r="BF7" s="2" t="n">
-        <v>-0.0762</v>
+        <v>-0.08169999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1699,7 +1705,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.185</v>
+        <v>4.107</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>4.58</v>
@@ -1719,7 +1725,7 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>1</v>
@@ -1749,7 +1755,7 @@
         </is>
       </c>
       <c r="W8" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
@@ -1770,22 +1776,22 @@
       <c r="AH8" s="2" t="inlineStr"/>
       <c r="AI8" s="2" t="inlineStr"/>
       <c r="AJ8" s="2" t="n">
-        <v>-9.01</v>
+        <v>-9.73</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>1.29</v>
+        <v>1.25</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.11</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>-0.02</v>
+        <v>0.03</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-5.3</v>
+        <v>-5.8</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="AP8" s="2" t="inlineStr"/>
       <c r="AQ8" s="2" t="inlineStr"/>
@@ -1797,40 +1803,40 @@
         </is>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>4.224</v>
+        <v>4.198</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>4.289</v>
+        <v>4.261</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>4.407</v>
+        <v>4.385</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>4.472</v>
+        <v>4.455</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>4.565</v>
+        <v>4.553</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>4.701</v>
+        <v>4.693</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>4.704</v>
+        <v>4.702</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>-1.4698</v>
+        <v>-1.4027</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>-1.0322</v>
+        <v>-1.0642</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>-0.461</v>
+        <v>-0.5052</v>
       </c>
       <c r="BE8" s="2" t="n">
-        <v>-0.3542</v>
+        <v>-0.3808</v>
       </c>
       <c r="BF8" s="2" t="n">
-        <v>-0.0901</v>
+        <v>-0.0973</v>
       </c>
     </row>
     <row r="9">
@@ -1845,7 +1851,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6.864</v>
+        <v>6.684</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0.97</v>
@@ -1895,7 +1901,7 @@
         </is>
       </c>
       <c r="W9" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
@@ -1909,29 +1915,29 @@
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr"/>
       <c r="AI9" s="2" t="inlineStr"/>
       <c r="AJ9" s="2" t="n">
-        <v>-3.39</v>
+        <v>-3.77</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>-0.52</v>
+        <v>-1.37</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>0.17</v>
+        <v>1.31</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>-2.78</v>
+        <v>-4.5</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>-0.9</v>
+        <v>-2.3</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="AP9" s="2" t="inlineStr"/>
       <c r="AQ9" s="2" t="inlineStr"/>
@@ -1943,40 +1949,40 @@
         </is>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>6.834</v>
+        <v>6.813</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>6.998</v>
+        <v>6.941</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>7.338</v>
+        <v>7.289</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>7.461</v>
+        <v>7.428</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>7.648</v>
+        <v>7.628</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>7.936</v>
+        <v>7.92</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>8.007999999999999</v>
+        <v>8.009</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>-2.5961</v>
+        <v>-2.3315</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>-1.4292</v>
+        <v>-1.4529</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>-0.4341</v>
+        <v>-0.4881</v>
       </c>
       <c r="BE9" s="2" t="n">
-        <v>-0.5481</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="BF9" s="2" t="n">
-        <v>-0.0339</v>
+        <v>-0.0377</v>
       </c>
     </row>
     <row r="10">
@@ -1991,7 +1997,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.385</v>
+        <v>3.327</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>41.01</v>
@@ -2012,19 +2018,19 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>0110111101</t>
+          <t>0110111100</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>0110111111</t>
+          <t>0110111100</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -2033,7 +2039,7 @@
         </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
@@ -2054,33 +2060,41 @@
       <c r="AF10" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AG10" s="2" t="inlineStr"/>
+      <c r="AG10" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AH10" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="AI10" s="2" t="inlineStr"/>
       <c r="AJ10" s="2" t="n">
-        <v>16.38</v>
+        <v>15.49</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>19.33</v>
+        <v>19.35</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>-1.54</v>
+        <v>0.36</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>7.62</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>85.2</v>
+        <v>82.5</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="AP10" s="2" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="AP10" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AQ10" s="2" t="inlineStr"/>
       <c r="AR10" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS10" s="2" t="inlineStr"/>
       <c r="AT10" s="2" t="inlineStr">
@@ -2089,40 +2103,40 @@
         </is>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>3.42</v>
+        <v>3.404</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>3.437</v>
+        <v>3.428</v>
       </c>
       <c r="AW10" s="2" t="n">
-        <v>3.396</v>
+        <v>3.394</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>3.408</v>
+        <v>3.405</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>3.39</v>
+        <v>3.392</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>3.281</v>
+        <v>3.282</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>3.237</v>
+        <v>3.238</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.548</v>
+        <v>0.3266</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>-0.0586</v>
+        <v>-0.0186</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>0.2122</v>
+        <v>0.2016</v>
       </c>
       <c r="BE10" s="2" t="n">
-        <v>0.1829</v>
+        <v>0.176</v>
       </c>
       <c r="BF10" s="2" t="n">
-        <v>0.1638</v>
+        <v>0.1549</v>
       </c>
     </row>
     <row r="11">
@@ -2137,7 +2151,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.482</v>
+        <v>0.477</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>-0.8100000000000001</v>
@@ -2181,7 +2195,7 @@
         </is>
       </c>
       <c r="W11" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
@@ -2191,7 +2205,7 @@
       <c r="Y11" s="2" t="inlineStr"/>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>4+→4·13d</t>
+          <t>4+→4·14d</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr"/>
@@ -2212,26 +2226,26 @@
       </c>
       <c r="AI11" s="2" t="inlineStr"/>
       <c r="AJ11" s="2" t="n">
-        <v>-20.74</v>
+        <v>-22.07</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>1</v>
+        <v>1.87</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>0.27</v>
+        <v>-0.77</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>5.17</v>
+        <v>6.22</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>3.3</v>
+        <v>1.1</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="AP11" s="2" t="inlineStr"/>
       <c r="AQ11" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR11" s="2" t="inlineStr"/>
       <c r="AS11" s="2" t="inlineStr"/>
@@ -2241,19 +2255,19 @@
         </is>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>0.49</v>
+        <v>0.486</v>
       </c>
       <c r="AV11" s="2" t="n">
         <v>0.491</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>0.496</v>
+        <v>0.495</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>0.503</v>
+        <v>0.502</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>0.51</v>
+        <v>0.509</v>
       </c>
       <c r="AZ11" s="2" t="n">
         <v>0.515</v>
@@ -2262,19 +2276,19 @@
         <v>0.528</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>-0.3469</v>
+        <v>-0.2846</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>-0.5084</v>
+        <v>-0.5354</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>-0.3845</v>
+        <v>-0.4275</v>
       </c>
       <c r="BE11" s="2" t="n">
-        <v>-0.0534</v>
+        <v>-0.0726</v>
       </c>
       <c r="BF11" s="2" t="n">
-        <v>-0.2074</v>
+        <v>-0.2207</v>
       </c>
     </row>
     <row r="12">
@@ -2289,7 +2303,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.376</v>
+        <v>0.368</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>9.880000000000001</v>
@@ -2310,28 +2324,28 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>4</v>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
+          <t>0000111000</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
           <t>0010111000</t>
         </is>
       </c>
-      <c r="U12" s="2" t="inlineStr">
-        <is>
-          <t>0010111000</t>
-        </is>
-      </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
       <c r="W12" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
@@ -2345,7 +2359,7 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>4→4+·4d ← 1→4·7d ← 1+→1·10d</t>
+          <t>4→4+·5d ← 1→4·8d ← 1+→1·11d</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr"/>
@@ -2353,31 +2367,33 @@
       <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF12" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AG12" s="2" t="inlineStr"/>
+      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AG12" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AH12" s="2" t="inlineStr"/>
       <c r="AI12" s="2" t="inlineStr"/>
       <c r="AJ12" s="2" t="n">
-        <v>-3.46</v>
+        <v>-3.88</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>12.55</v>
+        <v>12.27</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>3.56</v>
+        <v>0.99</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>11.53</v>
+        <v>11.84</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>55</v>
+        <v>51.5</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="AP12" s="2" t="inlineStr"/>
       <c r="AQ12" s="2" t="inlineStr"/>
@@ -2389,10 +2405,10 @@
         </is>
       </c>
       <c r="AU12" s="2" t="n">
-        <v>0.374</v>
+        <v>0.372</v>
       </c>
       <c r="AV12" s="2" t="n">
-        <v>0.376</v>
+        <v>0.375</v>
       </c>
       <c r="AW12" s="2" t="n">
         <v>0.377</v>
@@ -2410,19 +2426,19 @@
         <v>0.371</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>-0.411</v>
+        <v>-0.5068</v>
       </c>
       <c r="BC12" s="2" t="n">
-        <v>0.1451</v>
+        <v>0.1168</v>
       </c>
       <c r="BD12" s="2" t="n">
-        <v>-0.0355</v>
+        <v>-0.0975</v>
       </c>
       <c r="BE12" s="2" t="n">
-        <v>0.1992</v>
+        <v>0.199</v>
       </c>
       <c r="BF12" s="2" t="n">
-        <v>-0.0346</v>
+        <v>-0.0388</v>
       </c>
     </row>
     <row r="13">
@@ -2437,7 +2453,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.739</v>
+        <v>0.733</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>-4.85</v>
@@ -2483,7 +2499,7 @@
         </is>
       </c>
       <c r="W13" s="2" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
@@ -2493,7 +2509,7 @@
       <c r="Y13" s="2" t="inlineStr"/>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>4+→4·10d ← 4→4+·13d</t>
+          <t>4+→4·11d ← 4→4+·14d</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr"/>
@@ -2510,22 +2526,22 @@
       <c r="AH13" s="2" t="inlineStr"/>
       <c r="AI13" s="2" t="inlineStr"/>
       <c r="AJ13" s="2" t="n">
-        <v>-25.36</v>
+        <v>-27.14</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>0.37</v>
+        <v>1.47</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>0.72</v>
+        <v>-0.1</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>3.33</v>
+        <v>4.9</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>5.4</v>
+        <v>2.6</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="AP13" s="2" t="inlineStr"/>
       <c r="AQ13" s="2" t="inlineStr"/>
@@ -2537,40 +2553,40 @@
         </is>
       </c>
       <c r="AU13" s="2" t="n">
-        <v>0.75</v>
+        <v>0.745</v>
       </c>
       <c r="AV13" s="2" t="n">
-        <v>0.755</v>
+        <v>0.752</v>
       </c>
       <c r="AW13" s="2" t="n">
-        <v>0.765</v>
+        <v>0.762</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>0.777</v>
+        <v>0.774</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>0.784</v>
+        <v>0.782</v>
       </c>
       <c r="AZ13" s="2" t="n">
-        <v>0.786</v>
+        <v>0.785</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>0.82</v>
+        <v>0.819</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>-0.5877</v>
+        <v>-0.5276999999999999</v>
       </c>
       <c r="BC13" s="2" t="n">
-        <v>-0.704</v>
+        <v>-0.7161</v>
       </c>
       <c r="BD13" s="2" t="n">
-        <v>-0.4029</v>
+        <v>-0.431</v>
       </c>
       <c r="BE13" s="2" t="n">
-        <v>-0.0481</v>
+        <v>-0.064</v>
       </c>
       <c r="BF13" s="2" t="n">
-        <v>-0.2536</v>
+        <v>-0.2714</v>
       </c>
     </row>
     <row r="14">
@@ -2585,7 +2601,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.749</v>
+        <v>2.672</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>4.11</v>
@@ -2635,7 +2651,7 @@
         </is>
       </c>
       <c r="W14" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
@@ -2649,29 +2665,29 @@
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF14" s="2" t="inlineStr"/>
       <c r="AG14" s="2" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr"/>
       <c r="AI14" s="2" t="inlineStr"/>
       <c r="AJ14" s="2" t="n">
-        <v>-7.66</v>
+        <v>-7.82</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>-1.32</v>
+        <v>-2.33</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>0.3</v>
+        <v>1.79</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>-1.94</v>
+        <v>-4.11</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>8</v>
+        <v>5.3</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="AP14" s="2" t="inlineStr"/>
       <c r="AQ14" s="2" t="inlineStr"/>
@@ -2683,40 +2699,40 @@
         </is>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>2.73</v>
+        <v>2.724</v>
       </c>
       <c r="AV14" s="2" t="n">
-        <v>2.798</v>
+        <v>2.776</v>
       </c>
       <c r="AW14" s="2" t="n">
-        <v>2.935</v>
+        <v>2.916</v>
       </c>
       <c r="AX14" s="2" t="n">
-        <v>2.979</v>
+        <v>2.967</v>
       </c>
       <c r="AY14" s="2" t="n">
-        <v>3.032</v>
+        <v>3.025</v>
       </c>
       <c r="AZ14" s="2" t="n">
-        <v>3.149</v>
+        <v>3.142</v>
       </c>
       <c r="BA14" s="2" t="n">
         <v>3.21</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>-2.6421</v>
+        <v>-2.3121</v>
       </c>
       <c r="BC14" s="2" t="n">
-        <v>-1.3864</v>
+        <v>-1.4095</v>
       </c>
       <c r="BD14" s="2" t="n">
-        <v>-0.2392</v>
+        <v>-0.3056</v>
       </c>
       <c r="BE14" s="2" t="n">
-        <v>-0.638</v>
+        <v>-0.6384</v>
       </c>
       <c r="BF14" s="2" t="n">
-        <v>-0.0766</v>
+        <v>-0.07820000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -2731,7 +2747,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.332</v>
+        <v>0.326</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>12.17</v>
@@ -2752,19 +2768,19 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>0000111100</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>0010111000</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
@@ -2773,7 +2789,7 @@
         </is>
       </c>
       <c r="W15" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
@@ -2787,37 +2803,43 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>4→4+·4d ← 4+→4·10d ← 4→4+·11d</t>
+          <t>4→4+·5d ← 4+→4·11d ← 4→4+·12d</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="n">
-        <v>1</v>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="AF15" s="2" t="inlineStr"/>
-      <c r="AG15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AH15" s="2" t="inlineStr"/>
       <c r="AI15" s="2" t="inlineStr"/>
       <c r="AJ15" s="2" t="n">
-        <v>-5.19</v>
+        <v>-5.96</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>10.34</v>
+        <v>10.37</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>2.91</v>
+        <v>2.63</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>9.31</v>
+        <v>9.08</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>57.8</v>
+        <v>54.9</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="AP15" s="2" t="inlineStr"/>
       <c r="AQ15" s="2" t="inlineStr"/>
@@ -2832,10 +2854,10 @@
         <v>0.328</v>
       </c>
       <c r="AV15" s="2" t="n">
-        <v>0.333</v>
+        <v>0.332</v>
       </c>
       <c r="AW15" s="2" t="n">
-        <v>0.338</v>
+        <v>0.337</v>
       </c>
       <c r="AX15" s="2" t="n">
         <v>0.337</v>
@@ -2850,19 +2872,19 @@
         <v>0.335</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>-1.165</v>
+        <v>-1.0587</v>
       </c>
       <c r="BC15" s="2" t="n">
-        <v>-0.1624</v>
+        <v>-0.1699</v>
       </c>
       <c r="BD15" s="2" t="n">
-        <v>-0.0029</v>
+        <v>-0.045</v>
       </c>
       <c r="BE15" s="2" t="n">
-        <v>0.0466</v>
+        <v>0.0501</v>
       </c>
       <c r="BF15" s="2" t="n">
-        <v>-0.0519</v>
+        <v>-0.0596</v>
       </c>
     </row>
     <row r="16">
@@ -2877,7 +2899,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.063</v>
+        <v>1.038</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>71.16</v>
@@ -2921,7 +2943,7 @@
         </is>
       </c>
       <c r="W16" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
@@ -2931,39 +2953,43 @@
       <c r="Y16" s="2" t="inlineStr"/>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>4+→4·15d ← 4→4+·18d</t>
+          <t>4+→4·16d ← 4→4+·19d</t>
         </is>
       </c>
       <c r="AA16" s="2" t="inlineStr"/>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
       <c r="AD16" s="2" t="inlineStr"/>
-      <c r="AE16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AF16" s="2" t="inlineStr"/>
       <c r="AG16" s="2" t="inlineStr"/>
       <c r="AH16" s="2" t="inlineStr"/>
       <c r="AI16" s="2" t="inlineStr"/>
       <c r="AJ16" s="2" t="n">
-        <v>-17.48</v>
+        <v>-17.79</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>-5.5</v>
+        <v>-5.98</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>1.47</v>
+        <v>3.58</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>1.23</v>
+        <v>0.44</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>18.3</v>
+        <v>16</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="AP16" s="2" t="inlineStr"/>
       <c r="AQ16" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR16" s="2" t="inlineStr"/>
       <c r="AS16" s="2" t="inlineStr"/>
@@ -2973,40 +2999,40 @@
         </is>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>1.059</v>
+        <v>1.061</v>
       </c>
       <c r="AV16" s="2" t="n">
-        <v>1.069</v>
+        <v>1.063</v>
       </c>
       <c r="AW16" s="2" t="n">
-        <v>1.103</v>
+        <v>1.098</v>
       </c>
       <c r="AX16" s="2" t="n">
-        <v>1.121</v>
+        <v>1.117</v>
       </c>
       <c r="AY16" s="2" t="n">
-        <v>1.126</v>
+        <v>1.124</v>
       </c>
       <c r="AZ16" s="2" t="n">
-        <v>1.169</v>
+        <v>1.166</v>
       </c>
       <c r="BA16" s="2" t="n">
-        <v>1.295</v>
+        <v>1.293</v>
       </c>
       <c r="BB16" s="2" t="n">
-        <v>-1.3461</v>
+        <v>-1.0638</v>
       </c>
       <c r="BC16" s="2" t="n">
-        <v>-1.1951</v>
+        <v>-1.1173</v>
       </c>
       <c r="BD16" s="2" t="n">
-        <v>-0.1667</v>
+        <v>-0.1991</v>
       </c>
       <c r="BE16" s="2" t="n">
-        <v>-0.6684</v>
+        <v>-0.6545</v>
       </c>
       <c r="BF16" s="2" t="n">
-        <v>-0.1748</v>
+        <v>-0.1779</v>
       </c>
     </row>
     <row r="17">
@@ -3021,7 +3047,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.409</v>
+        <v>0.404</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>-1.36</v>
@@ -3044,19 +3070,19 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>0000010010</t>
+          <t>0000010000</t>
         </is>
       </c>
       <c r="V17" s="2" t="inlineStr">
@@ -3065,7 +3091,7 @@
         </is>
       </c>
       <c r="W17" s="2" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
@@ -3075,7 +3101,7 @@
       <c r="Y17" s="2" t="inlineStr"/>
       <c r="Z17" s="2" t="inlineStr">
         <is>
-          <t>4+→4·1d ← 4→4+·18d</t>
+          <t>4+→4·2d ← 4→4+·19d</t>
         </is>
       </c>
       <c r="AA17" s="2" t="inlineStr"/>
@@ -3085,31 +3111,31 @@
       <c r="AE17" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF17" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="AF17" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="AG17" s="2" t="inlineStr"/>
-      <c r="AH17" s="2" t="inlineStr"/>
+      <c r="AH17" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AI17" s="2" t="inlineStr"/>
       <c r="AJ17" s="2" t="n">
-        <v>-37.47</v>
+        <v>-38.41</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>-5.51</v>
+        <v>-4.88</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>1.77</v>
+        <v>0.46</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>9.550000000000001</v>
+        <v>11</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>52.9</v>
+        <v>50.3</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="AP17" s="2" t="inlineStr"/>
       <c r="AQ17" s="2" t="inlineStr"/>
@@ -3121,16 +3147,16 @@
         </is>
       </c>
       <c r="AU17" s="2" t="n">
-        <v>0.418</v>
+        <v>0.415</v>
       </c>
       <c r="AV17" s="2" t="n">
-        <v>0.417</v>
+        <v>0.416</v>
       </c>
       <c r="AW17" s="2" t="n">
         <v>0.414</v>
       </c>
       <c r="AX17" s="2" t="n">
-        <v>0.417</v>
+        <v>0.416</v>
       </c>
       <c r="AY17" s="2" t="n">
         <v>0.422</v>
@@ -3139,22 +3165,22 @@
         <v>0.421</v>
       </c>
       <c r="BA17" s="2" t="n">
-        <v>0.466</v>
+        <v>0.465</v>
       </c>
       <c r="BB17" s="2" t="n">
-        <v>0.4763</v>
+        <v>0.2875</v>
       </c>
       <c r="BC17" s="2" t="n">
-        <v>0.0684</v>
+        <v>0.09909999999999999</v>
       </c>
       <c r="BD17" s="2" t="n">
-        <v>-0.3448</v>
+        <v>-0.3791</v>
       </c>
       <c r="BE17" s="2" t="n">
-        <v>-0.2017</v>
+        <v>-0.2083</v>
       </c>
       <c r="BF17" s="2" t="n">
-        <v>-0.3747</v>
+        <v>-0.3841</v>
       </c>
     </row>
     <row r="18">
@@ -3169,7 +3195,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.034</v>
+        <v>1.015</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>-0.29</v>
@@ -3215,7 +3241,7 @@
         </is>
       </c>
       <c r="W18" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
@@ -3228,42 +3254,36 @@
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF18" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="AE18" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="AF18" s="2" t="inlineStr"/>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="inlineStr"/>
       <c r="AI18" s="2" t="inlineStr"/>
       <c r="AJ18" s="2" t="n">
-        <v>-14.6</v>
+        <v>-14.03</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>-4.54</v>
+        <v>-4.41</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>2.92</v>
+        <v>4.08</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>1.97</v>
+        <v>1.62</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="AP18" s="2" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="AP18" s="2" t="inlineStr"/>
       <c r="AQ18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR18" s="2" t="inlineStr"/>
       <c r="AS18" s="2" t="inlineStr"/>
@@ -3273,40 +3293,40 @@
         </is>
       </c>
       <c r="AU18" s="2" t="n">
-        <v>1.018</v>
+        <v>1.019</v>
       </c>
       <c r="AV18" s="2" t="n">
-        <v>1.035</v>
+        <v>1.03</v>
       </c>
       <c r="AW18" s="2" t="n">
-        <v>1.077</v>
+        <v>1.071</v>
       </c>
       <c r="AX18" s="2" t="n">
-        <v>1.099</v>
+        <v>1.092</v>
       </c>
       <c r="AY18" s="2" t="n">
-        <v>1.138</v>
+        <v>1.133</v>
       </c>
       <c r="AZ18" s="2" t="n">
-        <v>1.176</v>
+        <v>1.172</v>
       </c>
       <c r="BA18" s="2" t="n">
-        <v>1.226</v>
+        <v>1.224</v>
       </c>
       <c r="BB18" s="2" t="n">
-        <v>-2.0909</v>
+        <v>-1.6602</v>
       </c>
       <c r="BC18" s="2" t="n">
-        <v>-1.1841</v>
+        <v>-1.1285</v>
       </c>
       <c r="BD18" s="2" t="n">
-        <v>-0.6611</v>
+        <v>-0.7368</v>
       </c>
       <c r="BE18" s="2" t="n">
-        <v>-0.6623</v>
+        <v>-0.6352</v>
       </c>
       <c r="BF18" s="2" t="n">
-        <v>-0.146</v>
+        <v>-0.1403</v>
       </c>
     </row>
     <row r="19">
@@ -3321,7 +3341,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.887</v>
+        <v>0.865</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>4.85</v>
@@ -3383,29 +3403,29 @@
       <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="inlineStr"/>
       <c r="AE19" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF19" s="2" t="inlineStr"/>
       <c r="AG19" s="2" t="inlineStr"/>
       <c r="AH19" s="2" t="inlineStr"/>
       <c r="AI19" s="2" t="inlineStr"/>
       <c r="AJ19" s="2" t="n">
-        <v>13.87</v>
+        <v>13.54</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>2.32</v>
+        <v>1.59</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>-0.84</v>
+        <v>-1.07</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>-9.24</v>
+        <v>-13.92</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>-7.9</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="AP19" s="2" t="inlineStr"/>
       <c r="AQ19" s="2" t="inlineStr"/>
@@ -3417,40 +3437,40 @@
         </is>
       </c>
       <c r="AU19" s="2" t="n">
-        <v>0.887</v>
+        <v>0.881</v>
       </c>
       <c r="AV19" s="2" t="n">
-        <v>0.918</v>
+        <v>0.908</v>
       </c>
       <c r="AW19" s="2" t="n">
-        <v>0.995</v>
+        <v>0.985</v>
       </c>
       <c r="AX19" s="2" t="n">
-        <v>1.011</v>
+        <v>1.004</v>
       </c>
       <c r="AY19" s="2" t="n">
-        <v>1.056</v>
+        <v>1.052</v>
       </c>
       <c r="AZ19" s="2" t="n">
-        <v>1.158</v>
+        <v>1.154</v>
       </c>
       <c r="BA19" s="2" t="n">
-        <v>1.031</v>
+        <v>1.032</v>
       </c>
       <c r="BB19" s="2" t="n">
-        <v>-4.3714</v>
+        <v>-3.9244</v>
       </c>
       <c r="BC19" s="2" t="n">
-        <v>-1.7489</v>
+        <v>-1.9164</v>
       </c>
       <c r="BD19" s="2" t="n">
-        <v>-0.8003</v>
+        <v>-0.8404</v>
       </c>
       <c r="BE19" s="2" t="n">
-        <v>-0.6767</v>
+        <v>-0.7413</v>
       </c>
       <c r="BF19" s="2" t="n">
-        <v>0.1387</v>
+        <v>0.1354</v>
       </c>
     </row>
     <row r="20">
@@ -3465,7 +3485,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.862</v>
+        <v>0.863</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>73.68000000000001</v>
@@ -3480,25 +3500,25 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
@@ -3507,7 +3527,7 @@
         </is>
       </c>
       <c r="W20" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
@@ -3521,7 +3541,7 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·16d</t>
+          <t>2A→2C·17d</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr"/>
@@ -3531,40 +3551,32 @@
       <c r="AE20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF20" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="AF20" s="2" t="inlineStr"/>
       <c r="AG20" s="2" t="inlineStr"/>
       <c r="AH20" s="2" t="inlineStr"/>
       <c r="AI20" s="2" t="inlineStr"/>
       <c r="AJ20" s="2" t="n">
-        <v>8.300000000000001</v>
+        <v>7.94</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>20.95</v>
+        <v>23.23</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>2.14</v>
+        <v>3.31</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>10.82</v>
+        <v>14.36</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>100</v>
+        <v>99.5</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="AP20" s="2" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="AP20" s="2" t="inlineStr"/>
       <c r="AQ20" s="2" t="inlineStr"/>
       <c r="AR20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS20" s="2" t="inlineStr"/>
       <c r="AT20" s="2" t="inlineStr">
@@ -3579,34 +3591,34 @@
         <v>0.864</v>
       </c>
       <c r="AW20" s="2" t="n">
-        <v>0.851</v>
+        <v>0.853</v>
       </c>
       <c r="AX20" s="2" t="n">
-        <v>0.849</v>
+        <v>0.85</v>
       </c>
       <c r="AY20" s="2" t="n">
-        <v>0.834</v>
+        <v>0.836</v>
       </c>
       <c r="AZ20" s="2" t="n">
-        <v>0.8090000000000001</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="BA20" s="2" t="n">
-        <v>0.8</v>
+        <v>0.801</v>
       </c>
       <c r="BB20" s="2" t="n">
-        <v>0.8012</v>
+        <v>0.6399</v>
       </c>
       <c r="BC20" s="2" t="n">
-        <v>0.2796</v>
+        <v>0.2884</v>
       </c>
       <c r="BD20" s="2" t="n">
-        <v>0.2444</v>
+        <v>0.2666</v>
       </c>
       <c r="BE20" s="2" t="n">
-        <v>0.3119</v>
+        <v>0.3142</v>
       </c>
       <c r="BF20" s="2" t="n">
-        <v>0.083</v>
+        <v>0.0794</v>
       </c>
     </row>
     <row r="21">
@@ -3621,7 +3633,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>-8.65</v>
@@ -3638,7 +3650,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -3665,7 +3677,7 @@
         </is>
       </c>
       <c r="W21" s="2" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
@@ -3679,7 +3691,7 @@
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>4→4+·17d</t>
+          <t>4→4+·18d</t>
         </is>
       </c>
       <c r="AA21" s="2" t="inlineStr"/>
@@ -3689,33 +3701,33 @@
       <c r="AE21" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF21" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="AG21" s="2" t="inlineStr"/>
+      <c r="AF21" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AG21" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AH21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AI21" s="2" t="inlineStr"/>
       <c r="AJ21" s="2" t="n">
-        <v>-53.06</v>
+        <v>-53.84</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>-13.37</v>
+        <v>-16.07</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>-0.95</v>
+        <v>-2.73</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>6.09</v>
+        <v>4.43</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>17.2</v>
+        <v>13.8</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="AP21" s="2" t="inlineStr"/>
       <c r="AQ21" s="2" t="inlineStr"/>
@@ -3727,40 +3739,40 @@
         </is>
       </c>
       <c r="AU21" s="2" t="n">
-        <v>0.999</v>
+        <v>0.985</v>
       </c>
       <c r="AV21" s="2" t="n">
-        <v>1.001</v>
+        <v>0.996</v>
       </c>
       <c r="AW21" s="2" t="n">
-        <v>1.011</v>
+        <v>1.006</v>
       </c>
       <c r="AX21" s="2" t="n">
-        <v>1.018</v>
+        <v>1.014</v>
       </c>
       <c r="AY21" s="2" t="n">
-        <v>1.057</v>
+        <v>1.052</v>
       </c>
       <c r="AZ21" s="2" t="n">
-        <v>1.069</v>
+        <v>1.067</v>
       </c>
       <c r="BA21" s="2" t="n">
-        <v>1.199</v>
+        <v>1.197</v>
       </c>
       <c r="BB21" s="2" t="n">
-        <v>-0.4734</v>
+        <v>-0.5883</v>
       </c>
       <c r="BC21" s="2" t="n">
-        <v>-0.2433</v>
+        <v>-0.3898</v>
       </c>
       <c r="BD21" s="2" t="n">
-        <v>-0.7574</v>
+        <v>-0.8827</v>
       </c>
       <c r="BE21" s="2" t="n">
-        <v>-0.4038</v>
+        <v>-0.4137</v>
       </c>
       <c r="BF21" s="2" t="n">
-        <v>-0.5306</v>
+        <v>-0.5384</v>
       </c>
     </row>
     <row r="22">
@@ -3775,7 +3787,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.646</v>
+        <v>1.59</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>-7.05</v>
@@ -3796,19 +3808,19 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V22" s="2" t="inlineStr">
@@ -3817,7 +3829,7 @@
         </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
@@ -3827,7 +3839,7 @@
       <c r="Y22" s="2" t="inlineStr"/>
       <c r="Z22" s="2" t="inlineStr">
         <is>
-          <t>4+→4·10d ← 4→4+·13d</t>
+          <t>4+→4·11d ← 4→4+·14d</t>
         </is>
       </c>
       <c r="AA22" s="2" t="inlineStr"/>
@@ -3844,22 +3856,22 @@
       <c r="AH22" s="2" t="inlineStr"/>
       <c r="AI22" s="2" t="inlineStr"/>
       <c r="AJ22" s="2" t="n">
-        <v>-25.65</v>
+        <v>-27.69</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>-3.45</v>
+        <v>-4.89</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>-2.04</v>
+        <v>-3.73</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>1.11</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>1.5</v>
+        <v>-1</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AP22" s="2" t="inlineStr"/>
       <c r="AQ22" s="2" t="inlineStr"/>
@@ -3871,40 +3883,40 @@
         </is>
       </c>
       <c r="AU22" s="2" t="n">
-        <v>1.689</v>
+        <v>1.665</v>
       </c>
       <c r="AV22" s="2" t="n">
-        <v>1.71</v>
+        <v>1.697</v>
       </c>
       <c r="AW22" s="2" t="n">
-        <v>1.748</v>
+        <v>1.737</v>
       </c>
       <c r="AX22" s="2" t="n">
-        <v>1.781</v>
+        <v>1.772</v>
       </c>
       <c r="AY22" s="2" t="n">
-        <v>1.807</v>
+        <v>1.802</v>
       </c>
       <c r="AZ22" s="2" t="n">
-        <v>1.808</v>
+        <v>1.806</v>
       </c>
       <c r="BA22" s="2" t="n">
-        <v>1.869</v>
+        <v>1.866</v>
       </c>
       <c r="BB22" s="2" t="n">
-        <v>-1.2261</v>
+        <v>-1.3228</v>
       </c>
       <c r="BC22" s="2" t="n">
-        <v>-0.968</v>
+        <v>-1.0772</v>
       </c>
       <c r="BD22" s="2" t="n">
-        <v>-0.4202</v>
+        <v>-0.4917</v>
       </c>
       <c r="BE22" s="2" t="n">
-        <v>-0.1414</v>
+        <v>-0.1745</v>
       </c>
       <c r="BF22" s="2" t="n">
-        <v>-0.2565</v>
+        <v>-0.2769</v>
       </c>
     </row>
     <row r="23">
@@ -3919,7 +3931,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.311</v>
+        <v>2.262</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>110.91</v>
@@ -3942,19 +3954,19 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>0111111011</t>
+          <t>0010111011</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>0111111001</t>
+          <t>0010111000</t>
         </is>
       </c>
       <c r="V23" s="2" t="inlineStr">
@@ -3963,7 +3975,7 @@
         </is>
       </c>
       <c r="W23" s="2" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
@@ -3981,32 +3993,36 @@
         <v>-1</v>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AH23" s="2" t="inlineStr"/>
       <c r="AI23" s="2" t="inlineStr"/>
       <c r="AJ23" s="2" t="n">
-        <v>27.96</v>
+        <v>27.25</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>29.34</v>
+        <v>28.77</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>-2.59</v>
+        <v>-0.26</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>12.51</v>
+        <v>11.7</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>85.5</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="AP23" s="2" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="AP23" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AQ23" s="2" t="inlineStr"/>
       <c r="AR23" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AS23" s="2" t="inlineStr"/>
       <c r="AT23" s="2" t="inlineStr">
@@ -4015,16 +4031,16 @@
         </is>
       </c>
       <c r="AU23" s="2" t="n">
-        <v>2.333</v>
+        <v>2.322</v>
       </c>
       <c r="AV23" s="2" t="n">
-        <v>2.361</v>
+        <v>2.35</v>
       </c>
       <c r="AW23" s="2" t="n">
-        <v>2.327</v>
+        <v>2.33</v>
       </c>
       <c r="AX23" s="2" t="n">
-        <v>2.289</v>
+        <v>2.291</v>
       </c>
       <c r="AY23" s="2" t="n">
         <v>2.265</v>
@@ -4033,22 +4049,22 @@
         <v>2.223</v>
       </c>
       <c r="BA23" s="2" t="n">
-        <v>2.051</v>
+        <v>2.052</v>
       </c>
       <c r="BB23" s="2" t="n">
-        <v>0.09089999999999999</v>
+        <v>-0.128</v>
       </c>
       <c r="BC23" s="2" t="n">
-        <v>0.7091</v>
+        <v>0.6592</v>
       </c>
       <c r="BD23" s="2" t="n">
-        <v>0.5199</v>
+        <v>0.4022</v>
       </c>
       <c r="BE23" s="2" t="n">
-        <v>0.2544</v>
+        <v>0.2078</v>
       </c>
       <c r="BF23" s="2" t="n">
-        <v>0.2796</v>
+        <v>0.2725</v>
       </c>
     </row>
     <row r="24">
@@ -4063,7 +4079,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.293</v>
+        <v>1.268</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>3.97</v>
@@ -4082,7 +4098,9 @@
       </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N24" s="2" t="n">
         <v>1</v>
       </c>
@@ -4111,7 +4129,7 @@
         </is>
       </c>
       <c r="W24" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
@@ -4130,26 +4148,26 @@
       <c r="AH24" s="2" t="inlineStr"/>
       <c r="AI24" s="2" t="inlineStr"/>
       <c r="AJ24" s="2" t="n">
-        <v>-30.1</v>
+        <v>-30.93</v>
       </c>
       <c r="AK24" s="2" t="n">
         <v>-18.4</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>-2.27</v>
+        <v>-2.11</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>-4.14</v>
+        <v>-3.62</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>-1.8</v>
+        <v>-2.3</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AP24" s="2" t="inlineStr"/>
       <c r="AQ24" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AR24" s="2" t="inlineStr"/>
       <c r="AS24" s="2" t="inlineStr"/>
@@ -4159,40 +4177,40 @@
         </is>
       </c>
       <c r="AU24" s="2" t="n">
-        <v>1.332</v>
+        <v>1.316</v>
       </c>
       <c r="AV24" s="2" t="n">
-        <v>1.38</v>
+        <v>1.362</v>
       </c>
       <c r="AW24" s="2" t="n">
-        <v>1.43</v>
+        <v>1.419</v>
       </c>
       <c r="AX24" s="2" t="n">
-        <v>1.464</v>
+        <v>1.454</v>
       </c>
       <c r="AY24" s="2" t="n">
-        <v>1.537</v>
+        <v>1.529</v>
       </c>
       <c r="AZ24" s="2" t="n">
-        <v>1.659</v>
+        <v>1.651</v>
       </c>
       <c r="BA24" s="2" t="n">
-        <v>1.791</v>
+        <v>1.789</v>
       </c>
       <c r="BB24" s="2" t="n">
-        <v>-2.3355</v>
+        <v>-2.4483</v>
       </c>
       <c r="BC24" s="2" t="n">
-        <v>-1.5472</v>
+        <v>-1.5965</v>
       </c>
       <c r="BD24" s="2" t="n">
-        <v>-0.9353</v>
+        <v>-1.0304</v>
       </c>
       <c r="BE24" s="2" t="n">
-        <v>-1.081</v>
+        <v>-1.1085</v>
       </c>
       <c r="BF24" s="2" t="n">
-        <v>-0.301</v>
+        <v>-0.3093</v>
       </c>
     </row>
     <row r="25">
@@ -4207,7 +4225,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.823</v>
+        <v>0.776</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>3.37</v>
@@ -4230,25 +4248,25 @@
         <v>9</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S25" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V25" s="2" t="inlineStr">
@@ -4275,29 +4293,29 @@
       <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
       <c r="AE25" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF25" s="2" t="inlineStr"/>
       <c r="AG25" s="2" t="inlineStr"/>
       <c r="AH25" s="2" t="inlineStr"/>
       <c r="AI25" s="2" t="inlineStr"/>
       <c r="AJ25" s="2" t="n">
-        <v>12.01</v>
+        <v>11.37</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>1.84</v>
+        <v>-2.25</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>-0.51</v>
+        <v>-1.63</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>-17.04</v>
+        <v>-24.65</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>-0.4</v>
+        <v>-2</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="AP25" s="2" t="inlineStr"/>
       <c r="AQ25" s="2" t="inlineStr"/>
@@ -4309,40 +4327,40 @@
         </is>
       </c>
       <c r="AU25" s="2" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.805</v>
       </c>
       <c r="AV25" s="2" t="n">
-        <v>0.847</v>
+        <v>0.833</v>
       </c>
       <c r="AW25" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.927</v>
       </c>
       <c r="AX25" s="2" t="n">
-        <v>0.969</v>
+        <v>0.961</v>
       </c>
       <c r="AY25" s="2" t="n">
-        <v>0.996</v>
+        <v>0.992</v>
       </c>
       <c r="AZ25" s="2" t="n">
-        <v>1.094</v>
+        <v>1.09</v>
       </c>
       <c r="BA25" s="2" t="n">
-        <v>0.976</v>
+        <v>0.977</v>
       </c>
       <c r="BB25" s="2" t="n">
-        <v>-5.2646</v>
+        <v>-4.7381</v>
       </c>
       <c r="BC25" s="2" t="n">
-        <v>-2.8928</v>
+        <v>-3.0155</v>
       </c>
       <c r="BD25" s="2" t="n">
-        <v>-0.6046</v>
+        <v>-0.6901</v>
       </c>
       <c r="BE25" s="2" t="n">
-        <v>-0.7766</v>
+        <v>-0.8309</v>
       </c>
       <c r="BF25" s="2" t="n">
-        <v>0.1201</v>
+        <v>0.1137</v>
       </c>
     </row>
     <row r="26">
@@ -4357,7 +4375,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.237</v>
+        <v>1.202</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>46.54</v>
@@ -4378,19 +4396,19 @@
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>0110011100</t>
+          <t>0100011100</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
         <is>
-          <t>0000111000</t>
+          <t>0000011000</t>
         </is>
       </c>
       <c r="V26" s="2" t="inlineStr">
@@ -4399,7 +4417,7 @@
         </is>
       </c>
       <c r="W26" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
@@ -4423,27 +4441,25 @@
       <c r="AG26" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AH26" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AH26" s="2" t="inlineStr"/>
       <c r="AI26" s="2" t="inlineStr"/>
       <c r="AJ26" s="2" t="n">
-        <v>22.89</v>
+        <v>21.7</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>17.36</v>
+        <v>16.03</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>-3.84</v>
+        <v>-1.59</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>3.78</v>
+        <v>3.13</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>66.2</v>
+        <v>62.5</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="AP26" s="2" t="inlineStr"/>
       <c r="AQ26" s="2" t="inlineStr"/>
@@ -4455,16 +4471,16 @@
         </is>
       </c>
       <c r="AU26" s="2" t="n">
-        <v>1.257</v>
+        <v>1.248</v>
       </c>
       <c r="AV26" s="2" t="n">
-        <v>1.273</v>
+        <v>1.266</v>
       </c>
       <c r="AW26" s="2" t="n">
-        <v>1.269</v>
+        <v>1.266</v>
       </c>
       <c r="AX26" s="2" t="n">
-        <v>1.278</v>
+        <v>1.275</v>
       </c>
       <c r="AY26" s="2" t="n">
         <v>1.279</v>
@@ -4473,22 +4489,22 @@
         <v>1.243</v>
       </c>
       <c r="BA26" s="2" t="n">
-        <v>1.212</v>
+        <v>1.213</v>
       </c>
       <c r="BB26" s="2" t="n">
-        <v>-0.0332</v>
+        <v>-0.2988</v>
       </c>
       <c r="BC26" s="2" t="n">
-        <v>-0.4259</v>
+        <v>-0.3856</v>
       </c>
       <c r="BD26" s="2" t="n">
-        <v>0.2756</v>
+        <v>0.2572</v>
       </c>
       <c r="BE26" s="2" t="n">
-        <v>0.0919</v>
+        <v>0.0896</v>
       </c>
       <c r="BF26" s="2" t="n">
-        <v>0.2289</v>
+        <v>0.217</v>
       </c>
     </row>
     <row r="27">
@@ -4503,7 +4519,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.717</v>
+        <v>0.706</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>3.22</v>
@@ -4532,14 +4548,14 @@
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
@@ -4553,7 +4569,7 @@
         </is>
       </c>
       <c r="W27" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
@@ -4566,32 +4582,28 @@
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="inlineStr"/>
       <c r="AD27" s="2" t="inlineStr"/>
-      <c r="AE27" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr"/>
       <c r="AG27" s="2" t="inlineStr"/>
       <c r="AH27" s="2" t="inlineStr"/>
       <c r="AI27" s="2" t="inlineStr"/>
       <c r="AJ27" s="2" t="n">
-        <v>-29.92</v>
+        <v>-29.46</v>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>-16.79</v>
+        <v>-16.48</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>-0.06</v>
+        <v>1.91</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>-0.51</v>
+        <v>-0.8</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>0.5</v>
+        <v>-0.2</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="AP27" s="2" t="inlineStr"/>
       <c r="AQ27" s="2" t="inlineStr"/>
@@ -4603,40 +4615,40 @@
         </is>
       </c>
       <c r="AU27" s="2" t="n">
-        <v>0.718</v>
+        <v>0.716</v>
       </c>
       <c r="AV27" s="2" t="n">
-        <v>0.737</v>
+        <v>0.731</v>
       </c>
       <c r="AW27" s="2" t="n">
-        <v>0.767</v>
+        <v>0.762</v>
       </c>
       <c r="AX27" s="2" t="n">
-        <v>0.78</v>
+        <v>0.776</v>
       </c>
       <c r="AY27" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="AZ27" s="2" t="n">
-        <v>0.88</v>
+        <v>0.876</v>
       </c>
       <c r="BA27" s="2" t="n">
-        <v>0.979</v>
+        <v>0.978</v>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>-2.2682</v>
+        <v>-2.0039</v>
       </c>
       <c r="BC27" s="2" t="n">
-        <v>-1.3509</v>
+        <v>-1.3232</v>
       </c>
       <c r="BD27" s="2" t="n">
-        <v>-0.6603</v>
+        <v>-0.7217</v>
       </c>
       <c r="BE27" s="2" t="n">
-        <v>-1.1453</v>
+        <v>-1.1534</v>
       </c>
       <c r="BF27" s="2" t="n">
-        <v>-0.2992</v>
+        <v>-0.2946</v>
       </c>
     </row>
     <row r="28">
@@ -4651,7 +4663,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.535</v>
+        <v>0.503</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>3.91</v>
@@ -4671,10 +4683,10 @@
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
@@ -4683,7 +4695,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
@@ -4692,7 +4704,7 @@
       </c>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V28" s="2" t="inlineStr">
@@ -4719,29 +4731,29 @@
       <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF28" s="2" t="inlineStr"/>
       <c r="AG28" s="2" t="inlineStr"/>
       <c r="AH28" s="2" t="inlineStr"/>
       <c r="AI28" s="2" t="inlineStr"/>
       <c r="AJ28" s="2" t="n">
-        <v>7.82</v>
+        <v>7.32</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>0.43</v>
+        <v>-3.89</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.75</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>-16.04</v>
+        <v>-25.03</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="AP28" s="2" t="inlineStr"/>
       <c r="AQ28" s="2" t="inlineStr"/>
@@ -4753,40 +4765,40 @@
         </is>
       </c>
       <c r="AU28" s="2" t="n">
-        <v>0.526</v>
+        <v>0.522</v>
       </c>
       <c r="AV28" s="2" t="n">
-        <v>0.55</v>
+        <v>0.541</v>
       </c>
       <c r="AW28" s="2" t="n">
-        <v>0.613</v>
+        <v>0.604</v>
       </c>
       <c r="AX28" s="2" t="n">
-        <v>0.629</v>
+        <v>0.624</v>
       </c>
       <c r="AY28" s="2" t="n">
-        <v>0.644</v>
+        <v>0.641</v>
       </c>
       <c r="AZ28" s="2" t="n">
-        <v>0.709</v>
+        <v>0.706</v>
       </c>
       <c r="BA28" s="2" t="n">
         <v>0.645</v>
       </c>
       <c r="BB28" s="2" t="n">
-        <v>-5.3626</v>
+        <v>-4.7469</v>
       </c>
       <c r="BC28" s="2" t="n">
-        <v>-2.8221</v>
+        <v>-2.9621</v>
       </c>
       <c r="BD28" s="2" t="n">
-        <v>-0.5248</v>
+        <v>-0.6192</v>
       </c>
       <c r="BE28" s="2" t="n">
-        <v>-0.8229</v>
+        <v>-0.8521</v>
       </c>
       <c r="BF28" s="2" t="n">
-        <v>0.07820000000000001</v>
+        <v>0.0732</v>
       </c>
     </row>
     <row r="29">
@@ -4801,7 +4813,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.984</v>
+        <v>1.945</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>2.27</v>
@@ -4820,7 +4832,9 @@
       </c>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N29" s="2" t="n">
         <v>1</v>
       </c>
@@ -4849,7 +4863,7 @@
         </is>
       </c>
       <c r="W29" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
@@ -4868,22 +4882,22 @@
       <c r="AH29" s="2" t="inlineStr"/>
       <c r="AI29" s="2" t="inlineStr"/>
       <c r="AJ29" s="2" t="n">
-        <v>-32.58</v>
+        <v>-33.13</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>-20.48</v>
+        <v>-20.51</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>-3.19</v>
+        <v>-2.24</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>-5.07</v>
+        <v>-4.64</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>-2.6</v>
+        <v>-3</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AP29" s="2" t="inlineStr"/>
       <c r="AQ29" s="2" t="inlineStr"/>
@@ -4895,40 +4909,40 @@
         </is>
       </c>
       <c r="AU29" s="2" t="n">
-        <v>2.044</v>
+        <v>2.019</v>
       </c>
       <c r="AV29" s="2" t="n">
-        <v>2.122</v>
+        <v>2.093</v>
       </c>
       <c r="AW29" s="2" t="n">
-        <v>2.204</v>
+        <v>2.185</v>
       </c>
       <c r="AX29" s="2" t="n">
-        <v>2.251</v>
+        <v>2.237</v>
       </c>
       <c r="AY29" s="2" t="n">
-        <v>2.363</v>
+        <v>2.351</v>
       </c>
       <c r="AZ29" s="2" t="n">
-        <v>2.567</v>
+        <v>2.554</v>
       </c>
       <c r="BA29" s="2" t="n">
-        <v>2.826</v>
+        <v>2.822</v>
       </c>
       <c r="BB29" s="2" t="n">
-        <v>-2.4056</v>
+        <v>-2.5319</v>
       </c>
       <c r="BC29" s="2" t="n">
-        <v>-1.6205</v>
+        <v>-1.7091</v>
       </c>
       <c r="BD29" s="2" t="n">
-        <v>-0.8685</v>
+        <v>-0.9695</v>
       </c>
       <c r="BE29" s="2" t="n">
-        <v>-1.1352</v>
+        <v>-1.162</v>
       </c>
       <c r="BF29" s="2" t="n">
-        <v>-0.3258</v>
+        <v>-0.3313</v>
       </c>
     </row>
     <row r="30">
@@ -4943,7 +4957,7 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.837</v>
+        <v>0.829</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>3.87</v>
@@ -4966,7 +4980,7 @@
         <v>9</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -4993,7 +5007,7 @@
         </is>
       </c>
       <c r="W30" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
@@ -5006,27 +5020,25 @@
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
-      <c r="AE30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr"/>
       <c r="AG30" s="2" t="inlineStr"/>
       <c r="AH30" s="2" t="inlineStr"/>
       <c r="AI30" s="2" t="inlineStr"/>
       <c r="AJ30" s="2" t="n">
-        <v>-15.82</v>
+        <v>-14.26</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>-6.45</v>
+        <v>-5.55</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>5.3</v>
+        <v>7.88</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>1.06</v>
+        <v>1.93</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>-2.6</v>
+        <v>-1.9</v>
       </c>
       <c r="AO30" s="2" t="inlineStr"/>
       <c r="AP30" s="2" t="inlineStr"/>
@@ -5039,40 +5051,40 @@
         </is>
       </c>
       <c r="AU30" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.823</v>
       </c>
       <c r="AV30" s="2" t="n">
-        <v>0.829</v>
+        <v>0.826</v>
       </c>
       <c r="AW30" s="2" t="n">
-        <v>0.873</v>
+        <v>0.869</v>
       </c>
       <c r="AX30" s="2" t="n">
-        <v>0.894</v>
+        <v>0.89</v>
       </c>
       <c r="AY30" s="2" t="n">
-        <v>0.93</v>
+        <v>0.926</v>
       </c>
       <c r="AZ30" s="2" t="n">
-        <v>1.005</v>
+        <v>1.001</v>
       </c>
       <c r="BA30" s="2" t="n">
         <v>1.022</v>
       </c>
       <c r="BB30" s="2" t="n">
-        <v>-2.7615</v>
+        <v>-2.1491</v>
       </c>
       <c r="BC30" s="2" t="n">
-        <v>-1.5121</v>
+        <v>-1.3152</v>
       </c>
       <c r="BD30" s="2" t="n">
-        <v>-0.733</v>
+        <v>-0.7893</v>
       </c>
       <c r="BE30" s="2" t="n">
-        <v>-0.9781</v>
+        <v>-0.9641999999999999</v>
       </c>
       <c r="BF30" s="2" t="n">
-        <v>-0.1582</v>
+        <v>-0.1426</v>
       </c>
     </row>
     <row r="31">
@@ -5087,7 +5099,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.418</v>
+        <v>1.377</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>5.56</v>
@@ -5131,7 +5143,7 @@
         </is>
       </c>
       <c r="W31" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
@@ -5141,7 +5153,7 @@
       <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>2C→4·3d</t>
+          <t>2C→4·4d</t>
         </is>
       </c>
       <c r="AA31" s="2" t="inlineStr"/>
@@ -5149,29 +5161,29 @@
       <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF31" s="2" t="inlineStr"/>
       <c r="AG31" s="2" t="inlineStr"/>
       <c r="AH31" s="2" t="inlineStr"/>
       <c r="AI31" s="2" t="inlineStr"/>
       <c r="AJ31" s="2" t="n">
-        <v>2.61</v>
+        <v>2.25</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>-1.27</v>
+        <v>-2.34</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>-0.29</v>
+        <v>-1.18</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>-7.87</v>
+        <v>-12.65</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>-7.5</v>
+        <v>-7.9</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="AP31" s="2" t="inlineStr"/>
       <c r="AQ31" s="2" t="inlineStr"/>
@@ -5183,40 +5195,40 @@
         </is>
       </c>
       <c r="AU31" s="2" t="n">
-        <v>1.422</v>
+        <v>1.409</v>
       </c>
       <c r="AV31" s="2" t="n">
-        <v>1.466</v>
+        <v>1.45</v>
       </c>
       <c r="AW31" s="2" t="n">
-        <v>1.585</v>
+        <v>1.568</v>
       </c>
       <c r="AX31" s="2" t="n">
-        <v>1.613</v>
+        <v>1.602</v>
       </c>
       <c r="AY31" s="2" t="n">
-        <v>1.682</v>
+        <v>1.674</v>
       </c>
       <c r="AZ31" s="2" t="n">
-        <v>1.813</v>
+        <v>1.808</v>
       </c>
       <c r="BA31" s="2" t="n">
         <v>1.677</v>
       </c>
       <c r="BB31" s="2" t="n">
-        <v>-4.1644</v>
+        <v>-3.7262</v>
       </c>
       <c r="BC31" s="2" t="n">
-        <v>-1.7625</v>
+        <v>-1.9315</v>
       </c>
       <c r="BD31" s="2" t="n">
-        <v>-0.8557</v>
+        <v>-0.9025</v>
       </c>
       <c r="BE31" s="2" t="n">
-        <v>-0.6901</v>
+        <v>-0.7365</v>
       </c>
       <c r="BF31" s="2" t="n">
-        <v>0.0261</v>
+        <v>0.0225</v>
       </c>
     </row>
   </sheetData>
@@ -5247,7 +5259,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-21 | 30 只</t>
+          <t>截至: 2026-10-22 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-23
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.592</v>
+        <v>2.702</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-0.51</v>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
@@ -894,28 +894,30 @@
       <c r="AD2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr"/>
       <c r="AH2" s="2" t="inlineStr"/>
       <c r="AI2" s="2" t="inlineStr"/>
       <c r="AJ2" s="2" t="n">
-        <v>-14.26</v>
+        <v>-15.32</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>-12.55</v>
+        <v>-10.36</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>-4.19</v>
+        <v>-1.35</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>-14.16</v>
+        <v>-12.03</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>-8.199999999999999</v>
+        <v>-6.9</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="AP2" s="2" t="inlineStr"/>
       <c r="AQ2" s="2" t="inlineStr"/>
@@ -927,40 +929,40 @@
         </is>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>2.722</v>
+        <v>2.705</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>2.833</v>
+        <v>2.797</v>
       </c>
       <c r="AW2" s="2" t="n">
-        <v>3.056</v>
+        <v>3.025</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>3.151</v>
+        <v>3.13</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>3.303</v>
+        <v>3.286</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>3.596</v>
+        <v>3.582</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>3.511</v>
+        <v>3.509</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>-3.7913</v>
+        <v>-3.5786</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>-2.4245</v>
+        <v>-2.4855</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>-1.0566</v>
+        <v>-1.1701</v>
       </c>
       <c r="BE2" s="2" t="n">
-        <v>-0.8815</v>
+        <v>-0.9144</v>
       </c>
       <c r="BF2" s="2" t="n">
-        <v>-0.1426</v>
+        <v>-0.1532</v>
       </c>
     </row>
     <row r="3">
@@ -975,7 +977,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.345</v>
+        <v>1.36</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>-2.87</v>
@@ -990,7 +992,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -1017,7 +1019,7 @@
         </is>
       </c>
       <c r="W3" s="2" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
@@ -1027,15 +1029,17 @@
       <c r="Y3" s="2" t="inlineStr"/>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>4+→4·10d ← 4→4+·19d</t>
+          <t>4+→4·11d ← 4→4+·20d</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr"/>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
       <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="n">
-        <v>-1</v>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="n">
@@ -1044,22 +1048,22 @@
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="n">
-        <v>-14.11</v>
+        <v>-15.16</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>1.53</v>
+        <v>0.97</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>-1.52</v>
+        <v>-2.54</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>3.44</v>
+        <v>3.12</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>31.9</v>
+        <v>27.5</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AP3" s="2" t="inlineStr"/>
       <c r="AQ3" s="2" t="inlineStr"/>
@@ -1071,40 +1075,40 @@
         </is>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>1.395</v>
+        <v>1.383</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>1.409</v>
+        <v>1.403</v>
       </c>
       <c r="AW3" s="2" t="n">
-        <v>1.429</v>
+        <v>1.425</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>1.444</v>
+        <v>1.44</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>1.467</v>
+        <v>1.464</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>1.458</v>
+        <v>1.457</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>1.507</v>
+        <v>1.506</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>-0.8188</v>
+        <v>-0.9143</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.6293</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>-0.4718</v>
+        <v>-0.4893</v>
       </c>
       <c r="BE3" s="2" t="n">
-        <v>-0.1973</v>
+        <v>-0.209</v>
       </c>
       <c r="BF3" s="2" t="n">
-        <v>-0.1411</v>
+        <v>-0.1516</v>
       </c>
     </row>
     <row r="4">
@@ -1119,10 +1123,10 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.654</v>
+        <v>0.663</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-2.04</v>
+        <v>5.6</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -1134,7 +1138,7 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
@@ -1143,7 +1147,7 @@
         <v>3</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
@@ -1152,7 +1156,7 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>0000010110</t>
+          <t>0001010110</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
@@ -1161,51 +1165,55 @@
         </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y4" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>4+→4·2d ← 4→4+·5d ← 4+→4·6d</t>
+          <t>4→4+·1d ← 4+→4·3d ← 4→4+·6d</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr"/>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
       <c r="AD4" s="2" t="inlineStr"/>
-      <c r="AE4" s="2" t="n">
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF4" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="AG4" s="2" t="inlineStr"/>
-      <c r="AH4" s="2" t="inlineStr"/>
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="n">
-        <v>-25.83</v>
+        <v>-26.29</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>2.61</v>
+        <v>2.32</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>2.58</v>
+        <v>1.27</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>12.76</v>
+        <v>11.82</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>64.59999999999999</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="AP4" s="2" t="inlineStr"/>
       <c r="AQ4" s="2" t="inlineStr"/>
@@ -1217,13 +1225,13 @@
         </is>
       </c>
       <c r="AU4" s="2" t="n">
+        <v>0.661</v>
+      </c>
+      <c r="AV4" s="2" t="n">
         <v>0.662</v>
       </c>
-      <c r="AV4" s="2" t="n">
-        <v>0.661</v>
-      </c>
       <c r="AW4" s="2" t="n">
-        <v>0.657</v>
+        <v>0.658</v>
       </c>
       <c r="AX4" s="2" t="n">
         <v>0.661</v>
@@ -1235,22 +1243,22 @@
         <v>0.658</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>0.71</v>
+        <v>0.709</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>0.468</v>
+        <v>0.3163</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.1507</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>-0.2042</v>
+        <v>-0.1638</v>
       </c>
       <c r="BE4" s="2" t="n">
-        <v>-0.0978</v>
+        <v>-0.0876</v>
       </c>
       <c r="BF4" s="2" t="n">
-        <v>-0.2583</v>
+        <v>-0.2629</v>
       </c>
     </row>
     <row r="5">
@@ -1265,7 +1273,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.829</v>
+        <v>1.848</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>95.31</v>
@@ -1290,14 +1298,16 @@
       <c r="N5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="n">
         <v>9</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
@@ -1306,7 +1316,7 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
@@ -1315,7 +1325,7 @@
         </is>
       </c>
       <c r="W5" s="2" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
@@ -1325,7 +1335,7 @@
       <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·13d</t>
+          <t>2A→2C·14d</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr"/>
@@ -1344,27 +1354,27 @@
       <c r="AH5" s="2" t="inlineStr"/>
       <c r="AI5" s="2" t="inlineStr"/>
       <c r="AJ5" s="2" t="n">
-        <v>53.21</v>
+        <v>52.47</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>42.28</v>
+        <v>41.02</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>2.9</v>
+        <v>1.69</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>10.31</v>
+        <v>12.2</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="AP5" s="2" t="inlineStr"/>
       <c r="AQ5" s="2" t="inlineStr"/>
       <c r="AR5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AS5" s="2" t="inlineStr"/>
       <c r="AT5" s="2" t="inlineStr">
@@ -1373,40 +1383,40 @@
         </is>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>1.822</v>
+        <v>1.825</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>1.848</v>
+        <v>1.84</v>
       </c>
       <c r="AW5" s="2" t="n">
-        <v>1.808</v>
+        <v>1.811</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>1.786</v>
+        <v>1.792</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>1.691</v>
+        <v>1.699</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>1.6</v>
+        <v>1.603</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>1.545</v>
+        <v>1.548</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>0.3512</v>
+        <v>-0.1212</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>0.2849</v>
+        <v>0.2974</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>1.0544</v>
+        <v>1.0896</v>
       </c>
       <c r="BE5" s="2" t="n">
-        <v>0.332</v>
+        <v>0.3623</v>
       </c>
       <c r="BF5" s="2" t="n">
-        <v>0.5321</v>
+        <v>0.5247000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -1421,7 +1431,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.791</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>7.37</v>
@@ -1442,28 +1452,28 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
+          <t>0010011000</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
           <t>0000011000</t>
         </is>
       </c>
-      <c r="U6" s="2" t="inlineStr">
-        <is>
-          <t>0000011000</t>
-        </is>
-      </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
       <c r="W6" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
@@ -1473,7 +1483,7 @@
       <c r="Y6" s="2" t="inlineStr"/>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1→4·8d ← 1+→1·11d ← 1→1+·12d</t>
+          <t>1→4·9d ← 1+→1·12d ← 1→1+·13d</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr"/>
@@ -1481,7 +1491,7 @@
       <c r="AC6" s="2" t="inlineStr"/>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="n">
@@ -1490,22 +1500,22 @@
       <c r="AH6" s="2" t="inlineStr"/>
       <c r="AI6" s="2" t="inlineStr"/>
       <c r="AJ6" s="2" t="n">
-        <v>-6.5</v>
+        <v>-6.19</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>8.1</v>
+        <v>8.85</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>1.01</v>
+        <v>3.69</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>7.41</v>
+        <v>7.14</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>27</v>
+        <v>24.2</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="AP6" s="2" t="inlineStr"/>
       <c r="AQ6" s="2" t="inlineStr"/>
@@ -1517,40 +1527,40 @@
         </is>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>0.804</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AW6" s="2" t="n">
-        <v>0.832</v>
+        <v>0.831</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>0.832</v>
+        <v>0.831</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>0.856</v>
+        <v>0.855</v>
       </c>
       <c r="AZ6" s="2" t="n">
         <v>0.829</v>
       </c>
       <c r="BA6" s="2" t="n">
-        <v>0.831</v>
+        <v>0.83</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>-1.3694</v>
+        <v>-1.3017</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>-0.2518</v>
+        <v>-0.2366</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>-0.2468</v>
+        <v>-0.2591</v>
       </c>
       <c r="BE6" s="2" t="n">
-        <v>0.076</v>
+        <v>0.0974</v>
       </c>
       <c r="BF6" s="2" t="n">
-        <v>-0.065</v>
+        <v>-0.0619</v>
       </c>
     </row>
     <row r="7">
@@ -1565,7 +1575,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.836</v>
+        <v>2.869</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>2.9</v>
@@ -1582,7 +1592,7 @@
         <v>13</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -1609,7 +1619,7 @@
         </is>
       </c>
       <c r="W7" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
@@ -1623,29 +1633,29 @@
       <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
       <c r="AI7" s="2" t="inlineStr"/>
       <c r="AJ7" s="2" t="n">
-        <v>-8.17</v>
+        <v>-8.48</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>7.52</v>
+        <v>6.92</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>1.81</v>
+        <v>1.67</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>5.57</v>
+        <v>5.27</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>2.5</v>
+        <v>3.4</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="AP7" s="2" t="inlineStr"/>
       <c r="AQ7" s="2" t="inlineStr"/>
@@ -1657,40 +1667,40 @@
         </is>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>2.864</v>
+        <v>2.865</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>2.885</v>
+        <v>2.88</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>2.923</v>
+        <v>2.919</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>2.95</v>
+        <v>2.944</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>2.981</v>
+        <v>2.978</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>2.998</v>
+        <v>2.997</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>3.033</v>
+        <v>3.031</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>-0.6028</v>
+        <v>-0.527</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>-0.5194</v>
+        <v>-0.4665</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>-0.257</v>
+        <v>-0.2571</v>
       </c>
       <c r="BE7" s="2" t="n">
-        <v>-0.1354</v>
+        <v>-0.1313</v>
       </c>
       <c r="BF7" s="2" t="n">
-        <v>-0.08169999999999999</v>
+        <v>-0.0848</v>
       </c>
     </row>
     <row r="8">
@@ -1705,30 +1715,24 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.107</v>
+        <v>4.178</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>4.58</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="n">
         <v>9</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
@@ -1755,7 +1759,7 @@
         </is>
       </c>
       <c r="W8" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
@@ -1769,29 +1773,29 @@
       <c r="AC8" s="2" t="inlineStr"/>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AF8" s="2" t="inlineStr"/>
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr"/>
       <c r="AI8" s="2" t="inlineStr"/>
       <c r="AJ8" s="2" t="n">
-        <v>-9.73</v>
+        <v>-10.39</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>-0.11</v>
+        <v>0.17</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>-5.8</v>
+        <v>-4.2</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="AP8" s="2" t="inlineStr"/>
       <c r="AQ8" s="2" t="inlineStr"/>
@@ -1803,40 +1807,40 @@
         </is>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>4.198</v>
+        <v>4.186</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>4.261</v>
+        <v>4.241</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>4.385</v>
+        <v>4.368</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>4.455</v>
+        <v>4.441</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>4.553</v>
+        <v>4.542</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>4.693</v>
+        <v>4.685</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>4.702</v>
+        <v>4.7</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>-1.4027</v>
+        <v>-1.325</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>-1.0642</v>
+        <v>-1.0531</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>-0.5052</v>
+        <v>-0.5427</v>
       </c>
       <c r="BE8" s="2" t="n">
-        <v>-0.3808</v>
+        <v>-0.3944</v>
       </c>
       <c r="BF8" s="2" t="n">
-        <v>-0.0973</v>
+        <v>-0.1039</v>
       </c>
     </row>
     <row r="9">
@@ -1851,7 +1855,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6.684</v>
+        <v>6.857</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0.97</v>
@@ -1901,7 +1905,7 @@
         </is>
       </c>
       <c r="W9" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
@@ -1915,29 +1919,33 @@
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="inlineStr"/>
       <c r="AE9" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AF9" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AF9" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AG9" s="2" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr"/>
       <c r="AI9" s="2" t="inlineStr"/>
       <c r="AJ9" s="2" t="n">
-        <v>-3.77</v>
+        <v>-4.04</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>-1.37</v>
+        <v>-0.53</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>1.31</v>
+        <v>2.14</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>-4.5</v>
+        <v>-3.68</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>-2.3</v>
+        <v>-1.3</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="AP9" s="2" t="inlineStr"/>
       <c r="AQ9" s="2" t="inlineStr"/>
@@ -1949,40 +1957,40 @@
         </is>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>6.813</v>
+        <v>6.822</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>6.941</v>
+        <v>6.898</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>7.289</v>
+        <v>7.248</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>7.428</v>
+        <v>7.397</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>7.628</v>
+        <v>7.608</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>7.92</v>
+        <v>7.903</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>8.009</v>
+        <v>8.006</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>-2.3315</v>
+        <v>-2.0586</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>-1.4529</v>
+        <v>-1.424</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>-0.4881</v>
+        <v>-0.5496</v>
       </c>
       <c r="BE9" s="2" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.5496</v>
       </c>
       <c r="BF9" s="2" t="n">
-        <v>-0.0377</v>
+        <v>-0.0404</v>
       </c>
     </row>
     <row r="10">
@@ -1997,10 +2005,10 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.327</v>
+        <v>3.31</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>41.01</v>
+        <v>52.49</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -2018,19 +2026,19 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>0110111100</t>
+          <t>0100111100</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>0110111100</t>
+          <t>0110111000</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -2039,7 +2047,7 @@
         </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
@@ -2048,7 +2056,7 @@
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>减速</t>
+          <t>减速·周MACD将死叉</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr"/>
@@ -2065,36 +2073,30 @@
           <t>预-1</t>
         </is>
       </c>
-      <c r="AH10" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AH10" s="2" t="inlineStr"/>
       <c r="AI10" s="2" t="inlineStr"/>
       <c r="AJ10" s="2" t="n">
-        <v>15.49</v>
+        <v>14.58</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>19.35</v>
+        <v>16.63</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>0.36</v>
+        <v>-2.97</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>8.960000000000001</v>
+        <v>6.43</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>82.5</v>
+        <v>79.2</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="AP10" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="AP10" s="2" t="inlineStr"/>
       <c r="AQ10" s="2" t="inlineStr"/>
       <c r="AR10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS10" s="2" t="inlineStr"/>
       <c r="AT10" s="2" t="inlineStr">
@@ -2103,40 +2105,40 @@
         </is>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>3.404</v>
+        <v>3.38</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>3.428</v>
+        <v>3.416</v>
       </c>
       <c r="AW10" s="2" t="n">
-        <v>3.394</v>
+        <v>3.393</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>3.405</v>
+        <v>3.401</v>
       </c>
       <c r="AY10" s="2" t="n">
         <v>3.392</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>3.282</v>
+        <v>3.284</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>3.238</v>
+        <v>3.239</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.3266</v>
+        <v>0.0294</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>-0.0186</v>
+        <v>-0.0139</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>0.2016</v>
+        <v>0.172</v>
       </c>
       <c r="BE10" s="2" t="n">
-        <v>0.176</v>
+        <v>0.164</v>
       </c>
       <c r="BF10" s="2" t="n">
-        <v>0.1549</v>
+        <v>0.1458</v>
       </c>
     </row>
     <row r="11">
@@ -2151,7 +2153,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.477</v>
+        <v>0.484</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>-0.8100000000000001</v>
@@ -2195,7 +2197,7 @@
         </is>
       </c>
       <c r="W11" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
@@ -2205,15 +2207,17 @@
       <c r="Y11" s="2" t="inlineStr"/>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>4+→4·14d</t>
+          <t>4+→4·15d</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr"/>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
       <c r="AD11" s="2" t="inlineStr"/>
-      <c r="AE11" s="2" t="n">
-        <v>-1</v>
+      <c r="AE11" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="AF11" s="2" t="n">
         <v>-1</v>
@@ -2221,31 +2225,29 @@
       <c r="AG11" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AH11" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AH11" s="2" t="inlineStr"/>
       <c r="AI11" s="2" t="inlineStr"/>
       <c r="AJ11" s="2" t="n">
-        <v>-22.07</v>
+        <v>-22.73</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>1.87</v>
+        <v>1.67</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>-0.77</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>6.22</v>
+        <v>6.27</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="AP11" s="2" t="inlineStr"/>
       <c r="AQ11" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AR11" s="2" t="inlineStr"/>
       <c r="AS11" s="2" t="inlineStr"/>
@@ -2255,40 +2257,40 @@
         </is>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>0.486</v>
+        <v>0.484</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>0.491</v>
+        <v>0.49</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>0.495</v>
+        <v>0.494</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>0.502</v>
+        <v>0.5</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>0.509</v>
+        <v>0.508</v>
       </c>
       <c r="AZ11" s="2" t="n">
         <v>0.515</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>0.528</v>
+        <v>0.527</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>-0.2846</v>
+        <v>-0.3167</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>-0.5354</v>
+        <v>-0.4692</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>-0.4275</v>
+        <v>-0.4362</v>
       </c>
       <c r="BE11" s="2" t="n">
-        <v>-0.0726</v>
+        <v>-0.0796</v>
       </c>
       <c r="BF11" s="2" t="n">
-        <v>-0.2207</v>
+        <v>-0.2273</v>
       </c>
     </row>
     <row r="12">
@@ -2303,10 +2305,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.368</v>
+        <v>0.376</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>9.880000000000001</v>
+        <v>12.01</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -2324,19 +2326,19 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>0000111000</t>
+          <t>0010111010</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>0010111000</t>
+          <t>0010111010</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
@@ -2345,21 +2347,17 @@
         </is>
       </c>
       <c r="W12" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
-        </is>
-      </c>
-      <c r="Y12" s="2" t="inlineStr">
-        <is>
-          <t>周J超卖·日线纠缠</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr"/>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>4→4+·5d ← 1→4·8d ← 1+→1·11d</t>
+          <t>4+→4·1d ← 4→4+·6d ← 1→4·9d</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr"/>
@@ -2367,33 +2365,29 @@
       <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AF12" s="2" t="inlineStr"/>
-      <c r="AG12" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="AG12" s="2" t="inlineStr"/>
       <c r="AH12" s="2" t="inlineStr"/>
       <c r="AI12" s="2" t="inlineStr"/>
       <c r="AJ12" s="2" t="n">
-        <v>-3.88</v>
+        <v>-3.45</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>12.27</v>
+        <v>12.78</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>0.99</v>
+        <v>4.53</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>11.84</v>
+        <v>10.98</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>51.5</v>
+        <v>50</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="AP12" s="2" t="inlineStr"/>
       <c r="AQ12" s="2" t="inlineStr"/>
@@ -2405,10 +2399,10 @@
         </is>
       </c>
       <c r="AU12" s="2" t="n">
-        <v>0.372</v>
+        <v>0.374</v>
       </c>
       <c r="AV12" s="2" t="n">
-        <v>0.375</v>
+        <v>0.374</v>
       </c>
       <c r="AW12" s="2" t="n">
         <v>0.377</v>
@@ -2426,19 +2420,19 @@
         <v>0.371</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>-0.5068</v>
+        <v>-0.455</v>
       </c>
       <c r="BC12" s="2" t="n">
-        <v>0.1168</v>
+        <v>0.1575</v>
       </c>
       <c r="BD12" s="2" t="n">
-        <v>-0.0975</v>
+        <v>-0.0815</v>
       </c>
       <c r="BE12" s="2" t="n">
-        <v>0.199</v>
+        <v>0.2186</v>
       </c>
       <c r="BF12" s="2" t="n">
-        <v>-0.0388</v>
+        <v>-0.0345</v>
       </c>
     </row>
     <row r="13">
@@ -2453,7 +2447,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.733</v>
+        <v>0.747</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>-4.85</v>
@@ -2499,7 +2493,7 @@
         </is>
       </c>
       <c r="W13" s="2" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
@@ -2509,7 +2503,7 @@
       <c r="Y13" s="2" t="inlineStr"/>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>4+→4·11d ← 4→4+·14d</t>
+          <t>4+→4·12d ← 4→4+·15d</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr"/>
@@ -2517,7 +2511,7 @@
       <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
       <c r="AE13" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="n">
@@ -2526,22 +2520,22 @@
       <c r="AH13" s="2" t="inlineStr"/>
       <c r="AI13" s="2" t="inlineStr"/>
       <c r="AJ13" s="2" t="n">
-        <v>-27.14</v>
+        <v>-27.8</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>1.47</v>
+        <v>1.65</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>-0.1</v>
+        <v>0.72</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>4.9</v>
+        <v>5.47</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="AP13" s="2" t="inlineStr"/>
       <c r="AQ13" s="2" t="inlineStr"/>
@@ -2553,40 +2547,40 @@
         </is>
       </c>
       <c r="AU13" s="2" t="n">
-        <v>0.745</v>
+        <v>0.744</v>
       </c>
       <c r="AV13" s="2" t="n">
-        <v>0.752</v>
+        <v>0.751</v>
       </c>
       <c r="AW13" s="2" t="n">
-        <v>0.762</v>
+        <v>0.761</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>0.774</v>
+        <v>0.772</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>0.782</v>
+        <v>0.781</v>
       </c>
       <c r="AZ13" s="2" t="n">
         <v>0.785</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>0.819</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>-0.5276999999999999</v>
+        <v>-0.5243</v>
       </c>
       <c r="BC13" s="2" t="n">
-        <v>-0.7161</v>
+        <v>-0.6276</v>
       </c>
       <c r="BD13" s="2" t="n">
-        <v>-0.431</v>
+        <v>-0.4169</v>
       </c>
       <c r="BE13" s="2" t="n">
-        <v>-0.064</v>
+        <v>-0.0635</v>
       </c>
       <c r="BF13" s="2" t="n">
-        <v>-0.2714</v>
+        <v>-0.278</v>
       </c>
     </row>
     <row r="14">
@@ -2601,7 +2595,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2.672</v>
+        <v>2.742</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>4.11</v>
@@ -2651,7 +2645,7 @@
         </is>
       </c>
       <c r="W14" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
@@ -2665,29 +2659,33 @@
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AF14" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AF14" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AG14" s="2" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr"/>
       <c r="AI14" s="2" t="inlineStr"/>
       <c r="AJ14" s="2" t="n">
-        <v>-7.82</v>
+        <v>-7.89</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>-2.33</v>
+        <v>-1.37</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>1.79</v>
+        <v>2.36</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>-4.11</v>
+        <v>-3.05</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="AP14" s="2" t="inlineStr"/>
       <c r="AQ14" s="2" t="inlineStr"/>
@@ -2699,58 +2697,58 @@
         </is>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>2.724</v>
+        <v>2.726</v>
       </c>
       <c r="AV14" s="2" t="n">
-        <v>2.776</v>
+        <v>2.757</v>
       </c>
       <c r="AW14" s="2" t="n">
-        <v>2.916</v>
+        <v>2.897</v>
       </c>
       <c r="AX14" s="2" t="n">
-        <v>2.967</v>
+        <v>2.952</v>
       </c>
       <c r="AY14" s="2" t="n">
-        <v>3.025</v>
+        <v>3.017</v>
       </c>
       <c r="AZ14" s="2" t="n">
-        <v>3.142</v>
+        <v>3.132</v>
       </c>
       <c r="BA14" s="2" t="n">
-        <v>3.21</v>
+        <v>3.206</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>-2.3121</v>
+        <v>-1.9906</v>
       </c>
       <c r="BC14" s="2" t="n">
-        <v>-1.4095</v>
+        <v>-1.3829</v>
       </c>
       <c r="BD14" s="2" t="n">
-        <v>-0.3056</v>
+        <v>-0.3838</v>
       </c>
       <c r="BE14" s="2" t="n">
-        <v>-0.6384</v>
+        <v>-0.6185</v>
       </c>
       <c r="BF14" s="2" t="n">
-        <v>-0.07820000000000001</v>
+        <v>-0.0789</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.326</v>
+        <v>1.061</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>12.17</v>
+        <v>17.41</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -2760,27 +2758,29 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0000000100</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>0000011000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
@@ -2789,120 +2789,112 @@
         </is>
       </c>
       <c r="W15" s="2" t="n">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
-        </is>
-      </c>
-      <c r="Y15" s="2" t="inlineStr">
-        <is>
-          <t>周J超卖·日线纠缠</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr"/>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>4→4+·5d ← 4+→4·11d ← 4→4+·12d</t>
+          <t>4+→4·17d ← 4→4+·20d</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr"/>
-      <c r="AG15" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="AH15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="inlineStr"/>
+      <c r="AH15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AI15" s="2" t="inlineStr"/>
       <c r="AJ15" s="2" t="n">
-        <v>-5.96</v>
+        <v>-18.1</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>10.37</v>
+        <v>-5.5</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>2.63</v>
+        <v>1.69</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>9.08</v>
+        <v>1.13</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>54.9</v>
+        <v>15.7</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="AP15" s="2" t="inlineStr"/>
-      <c r="AQ15" s="2" t="inlineStr"/>
+      <c r="AQ15" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="AR15" s="2" t="inlineStr"/>
       <c r="AS15" s="2" t="inlineStr"/>
       <c r="AT15" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU15" s="2" t="n">
-        <v>0.328</v>
+        <v>1.061</v>
       </c>
       <c r="AV15" s="2" t="n">
-        <v>0.332</v>
+        <v>1.061</v>
       </c>
       <c r="AW15" s="2" t="n">
-        <v>0.337</v>
+        <v>1.093</v>
       </c>
       <c r="AX15" s="2" t="n">
-        <v>0.337</v>
+        <v>1.115</v>
       </c>
       <c r="AY15" s="2" t="n">
-        <v>0.341</v>
+        <v>1.122</v>
       </c>
       <c r="AZ15" s="2" t="n">
-        <v>0.326</v>
+        <v>1.163</v>
       </c>
       <c r="BA15" s="2" t="n">
-        <v>0.335</v>
+        <v>1.292</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>-1.0587</v>
+        <v>-0.8344</v>
       </c>
       <c r="BC15" s="2" t="n">
-        <v>-0.1699</v>
+        <v>-1.0301</v>
       </c>
       <c r="BD15" s="2" t="n">
-        <v>-0.045</v>
+        <v>-0.2545</v>
       </c>
       <c r="BE15" s="2" t="n">
-        <v>0.0501</v>
+        <v>-0.6342</v>
       </c>
       <c r="BF15" s="2" t="n">
-        <v>-0.0596</v>
+        <v>-0.181</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.038</v>
+        <v>0.415</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>71.16</v>
+        <v>6.28</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -2913,7 +2905,7 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>2</v>
@@ -2922,19 +2914,19 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0000010110</t>
         </is>
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0000010010</t>
         </is>
       </c>
       <c r="V16" s="2" t="inlineStr">
@@ -2943,7 +2935,7 @@
         </is>
       </c>
       <c r="W16" s="2" t="n">
-        <v>69</v>
+        <v>222</v>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
@@ -2953,7 +2945,7 @@
       <c r="Y16" s="2" t="inlineStr"/>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>4+→4·16d ← 4→4+·19d</t>
+          <t>4+→4·3d ← 4→4+·20d</t>
         </is>
       </c>
       <c r="AA16" s="2" t="inlineStr"/>
@@ -2962,95 +2954,97 @@
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="AF16" s="2" t="inlineStr"/>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF16" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AG16" s="2" t="inlineStr"/>
-      <c r="AH16" s="2" t="inlineStr"/>
+      <c r="AH16" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AI16" s="2" t="inlineStr"/>
       <c r="AJ16" s="2" t="n">
-        <v>-17.79</v>
+        <v>-38.74</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>-5.98</v>
+        <v>-3.79</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>3.58</v>
+        <v>0.62</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>0.44</v>
+        <v>11.57</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>16</v>
+        <v>50.2</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="AP16" s="2" t="inlineStr"/>
-      <c r="AQ16" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AQ16" s="2" t="inlineStr"/>
       <c r="AR16" s="2" t="inlineStr"/>
       <c r="AS16" s="2" t="inlineStr"/>
       <c r="AT16" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>1.061</v>
+        <v>0.414</v>
       </c>
       <c r="AV16" s="2" t="n">
-        <v>1.063</v>
+        <v>0.415</v>
       </c>
       <c r="AW16" s="2" t="n">
-        <v>1.098</v>
+        <v>0.414</v>
       </c>
       <c r="AX16" s="2" t="n">
-        <v>1.117</v>
+        <v>0.416</v>
       </c>
       <c r="AY16" s="2" t="n">
-        <v>1.124</v>
+        <v>0.421</v>
       </c>
       <c r="AZ16" s="2" t="n">
-        <v>1.166</v>
+        <v>0.42</v>
       </c>
       <c r="BA16" s="2" t="n">
-        <v>1.293</v>
+        <v>0.464</v>
       </c>
       <c r="BB16" s="2" t="n">
-        <v>-1.0638</v>
+        <v>0.0752</v>
       </c>
       <c r="BC16" s="2" t="n">
-        <v>-1.1173</v>
+        <v>0.125</v>
       </c>
       <c r="BD16" s="2" t="n">
-        <v>-0.1991</v>
+        <v>-0.3502</v>
       </c>
       <c r="BE16" s="2" t="n">
-        <v>-0.6545</v>
+        <v>-0.2136</v>
       </c>
       <c r="BF16" s="2" t="n">
-        <v>-0.1779</v>
+        <v>-0.3874</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.404</v>
+        <v>1.057</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-1.36</v>
+        <v>-0.29</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -3059,30 +3053,32 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M17" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>0000010000</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V17" s="2" t="inlineStr">
@@ -3091,7 +3087,7 @@
         </is>
       </c>
       <c r="W17" s="2" t="n">
-        <v>221</v>
+        <v>65</v>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
@@ -3099,106 +3095,106 @@
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr"/>
-      <c r="Z17" s="2" t="inlineStr">
-        <is>
-          <t>4+→4·2d ← 4→4+·19d</t>
-        </is>
-      </c>
+      <c r="Z17" s="2" t="inlineStr"/>
       <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
       <c r="AD17" s="2" t="inlineStr"/>
-      <c r="AE17" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AG17" s="2" t="inlineStr"/>
       <c r="AH17" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AI17" s="2" t="inlineStr"/>
       <c r="AJ17" s="2" t="n">
-        <v>-38.41</v>
+        <v>-13.02</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>-4.88</v>
+        <v>-2.1</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>0.46</v>
+        <v>6.68</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>11</v>
+        <v>3.87</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>50.3</v>
+        <v>1.9</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="AP17" s="2" t="inlineStr"/>
-      <c r="AQ17" s="2" t="inlineStr"/>
+        <v>65</v>
+      </c>
+      <c r="AP17" s="2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="AQ17" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AR17" s="2" t="inlineStr"/>
       <c r="AS17" s="2" t="inlineStr"/>
       <c r="AT17" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU17" s="2" t="n">
-        <v>0.415</v>
+        <v>1.03</v>
       </c>
       <c r="AV17" s="2" t="n">
-        <v>0.416</v>
+        <v>1.029</v>
       </c>
       <c r="AW17" s="2" t="n">
-        <v>0.414</v>
+        <v>1.069</v>
       </c>
       <c r="AX17" s="2" t="n">
-        <v>0.416</v>
+        <v>1.089</v>
       </c>
       <c r="AY17" s="2" t="n">
-        <v>0.422</v>
+        <v>1.13</v>
       </c>
       <c r="AZ17" s="2" t="n">
-        <v>0.421</v>
+        <v>1.17</v>
       </c>
       <c r="BA17" s="2" t="n">
-        <v>0.465</v>
+        <v>1.224</v>
       </c>
       <c r="BB17" s="2" t="n">
-        <v>0.2875</v>
+        <v>-1.1625</v>
       </c>
       <c r="BC17" s="2" t="n">
-        <v>0.09909999999999999</v>
+        <v>-0.9722</v>
       </c>
       <c r="BD17" s="2" t="n">
-        <v>-0.3791</v>
+        <v>-0.7951</v>
       </c>
       <c r="BE17" s="2" t="n">
-        <v>-0.2083</v>
+        <v>-0.5818</v>
       </c>
       <c r="BF17" s="2" t="n">
-        <v>-0.3841</v>
+        <v>-0.1302</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.015</v>
+        <v>0.891</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>-0.29</v>
+        <v>4.85</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -3207,144 +3203,146 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="n">
         <v>9</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010000000</t>
         </is>
       </c>
       <c r="V18" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W18" s="2" t="n">
-        <v>64</v>
+        <v>299</v>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y18" s="2" t="inlineStr"/>
+          <t>2C</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>顶背离·周MACD死叉</t>
+        </is>
+      </c>
       <c r="Z18" s="2" t="inlineStr"/>
       <c r="AA18" s="2" t="inlineStr"/>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="AF18" s="2" t="inlineStr"/>
+      <c r="AE18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF18" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="inlineStr"/>
       <c r="AI18" s="2" t="inlineStr"/>
       <c r="AJ18" s="2" t="n">
-        <v>-14.03</v>
+        <v>13.07</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>-4.41</v>
+        <v>2.83</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>4.08</v>
+        <v>1.13</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>1.62</v>
+        <v>-12.05</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>-0</v>
+        <v>-7.4</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="AP18" s="2" t="inlineStr"/>
-      <c r="AQ18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AQ18" s="2" t="inlineStr"/>
       <c r="AR18" s="2" t="inlineStr"/>
       <c r="AS18" s="2" t="inlineStr"/>
       <c r="AT18" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>无背离</t>
         </is>
       </c>
       <c r="AU18" s="2" t="n">
-        <v>1.019</v>
+        <v>0.88</v>
       </c>
       <c r="AV18" s="2" t="n">
-        <v>1.03</v>
+        <v>0.9</v>
       </c>
       <c r="AW18" s="2" t="n">
-        <v>1.071</v>
+        <v>0.977</v>
       </c>
       <c r="AX18" s="2" t="n">
-        <v>1.092</v>
+        <v>0.998</v>
       </c>
       <c r="AY18" s="2" t="n">
-        <v>1.133</v>
+        <v>1.047</v>
       </c>
       <c r="AZ18" s="2" t="n">
-        <v>1.172</v>
+        <v>1.151</v>
       </c>
       <c r="BA18" s="2" t="n">
-        <v>1.224</v>
+        <v>1.033</v>
       </c>
       <c r="BB18" s="2" t="n">
-        <v>-1.6602</v>
+        <v>-3.4025</v>
       </c>
       <c r="BC18" s="2" t="n">
-        <v>-1.1285</v>
+        <v>-1.9965</v>
       </c>
       <c r="BD18" s="2" t="n">
-        <v>-0.7368</v>
+        <v>-0.9307</v>
       </c>
       <c r="BE18" s="2" t="n">
-        <v>-0.6352</v>
+        <v>-0.7558</v>
       </c>
       <c r="BF18" s="2" t="n">
-        <v>-0.1403</v>
+        <v>0.1307</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.865</v>
+        <v>0.849</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>4.85</v>
+        <v>89.31999999999999</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -3354,29 +3352,27 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0111111111</t>
         </is>
       </c>
       <c r="V19" s="2" t="inlineStr">
@@ -3385,7 +3381,7 @@
         </is>
       </c>
       <c r="W19" s="2" t="n">
-        <v>299</v>
+        <v>58</v>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
@@ -3394,101 +3390,109 @@
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
-          <t>顶背离·周MACD死叉</t>
-        </is>
-      </c>
-      <c r="Z19" s="2" t="inlineStr"/>
+          <t>减速</t>
+        </is>
+      </c>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
+          <t>2A→2C·18d</t>
+        </is>
+      </c>
       <c r="AA19" s="2" t="inlineStr"/>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="inlineStr"/>
-      <c r="AE19" s="2" t="n">
+      <c r="AE19" s="2" t="inlineStr"/>
+      <c r="AF19" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF19" s="2" t="inlineStr"/>
       <c r="AG19" s="2" t="inlineStr"/>
-      <c r="AH19" s="2" t="inlineStr"/>
+      <c r="AH19" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="AI19" s="2" t="inlineStr"/>
       <c r="AJ19" s="2" t="n">
-        <v>13.54</v>
+        <v>7.32</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>1.59</v>
+        <v>19.08</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>-1.07</v>
+        <v>-0.76</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>-13.92</v>
+        <v>9.98</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>-8.199999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="AP19" s="2" t="inlineStr"/>
       <c r="AQ19" s="2" t="inlineStr"/>
-      <c r="AR19" s="2" t="inlineStr"/>
+      <c r="AR19" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="AS19" s="2" t="inlineStr"/>
       <c r="AT19" s="2" t="inlineStr">
         <is>
-          <t>无背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU19" s="2" t="n">
-        <v>0.881</v>
+        <v>0.863</v>
       </c>
       <c r="AV19" s="2" t="n">
-        <v>0.908</v>
+        <v>0.864</v>
       </c>
       <c r="AW19" s="2" t="n">
-        <v>0.985</v>
+        <v>0.853</v>
       </c>
       <c r="AX19" s="2" t="n">
-        <v>1.004</v>
+        <v>0.85</v>
       </c>
       <c r="AY19" s="2" t="n">
-        <v>1.052</v>
+        <v>0.836</v>
       </c>
       <c r="AZ19" s="2" t="n">
-        <v>1.154</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="BA19" s="2" t="n">
-        <v>1.032</v>
+        <v>0.801</v>
       </c>
       <c r="BB19" s="2" t="n">
-        <v>-3.9244</v>
+        <v>0.4801</v>
       </c>
       <c r="BC19" s="2" t="n">
-        <v>-1.9164</v>
+        <v>0.2913</v>
       </c>
       <c r="BD19" s="2" t="n">
-        <v>-0.8404</v>
+        <v>0.2915</v>
       </c>
       <c r="BE19" s="2" t="n">
-        <v>-0.7413</v>
+        <v>0.3048</v>
       </c>
       <c r="BF19" s="2" t="n">
-        <v>0.1354</v>
+        <v>0.0732</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.863</v>
+        <v>0.949</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>73.68000000000001</v>
+        <v>-8.65</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -3497,87 +3501,91 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>0111111111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>0111111111</t>
+          <t>0000000000</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W20" s="2" t="n">
-        <v>57</v>
+        <v>160</v>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>2C</t>
-        </is>
-      </c>
-      <c r="Y20" s="2" t="inlineStr">
-        <is>
-          <t>减速</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr"/>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>2A→2C·17d</t>
+          <t>4+→4·1d ← 4→4+·19d</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr"/>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
       <c r="AD20" s="2" t="inlineStr"/>
-      <c r="AE20" s="2" t="n">
+      <c r="AE20" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF20" s="2" t="inlineStr"/>
-      <c r="AG20" s="2" t="inlineStr"/>
+      <c r="AG20" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="AH20" s="2" t="inlineStr"/>
       <c r="AI20" s="2" t="inlineStr"/>
       <c r="AJ20" s="2" t="n">
-        <v>7.94</v>
+        <v>-54.97</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>23.23</v>
+        <v>-15.63</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>3.31</v>
+        <v>-3.23</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>14.36</v>
+        <v>5.33</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>99.5</v>
+        <v>11.8</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="AP20" s="2" t="inlineStr"/>
       <c r="AQ20" s="2" t="inlineStr"/>
-      <c r="AR20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AR20" s="2" t="inlineStr"/>
       <c r="AS20" s="2" t="inlineStr"/>
       <c r="AT20" s="2" t="inlineStr">
         <is>
@@ -3585,72 +3593,76 @@
         </is>
       </c>
       <c r="AU20" s="2" t="n">
-        <v>0.866</v>
+        <v>0.972</v>
       </c>
       <c r="AV20" s="2" t="n">
-        <v>0.864</v>
+        <v>0.991</v>
       </c>
       <c r="AW20" s="2" t="n">
-        <v>0.853</v>
+        <v>1.004</v>
       </c>
       <c r="AX20" s="2" t="n">
-        <v>0.85</v>
+        <v>1.011</v>
       </c>
       <c r="AY20" s="2" t="n">
-        <v>0.836</v>
+        <v>1.047</v>
       </c>
       <c r="AZ20" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.066</v>
       </c>
       <c r="BA20" s="2" t="n">
-        <v>0.801</v>
+        <v>1.194</v>
       </c>
       <c r="BB20" s="2" t="n">
-        <v>0.6399</v>
+        <v>-0.7907</v>
       </c>
       <c r="BC20" s="2" t="n">
-        <v>0.2884</v>
+        <v>-0.5308</v>
       </c>
       <c r="BD20" s="2" t="n">
-        <v>0.2666</v>
+        <v>-0.9667</v>
       </c>
       <c r="BE20" s="2" t="n">
-        <v>0.3142</v>
+        <v>-0.4149</v>
       </c>
       <c r="BF20" s="2" t="n">
-        <v>0.0794</v>
+        <v>-0.5497</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.93</v>
+        <v>1.624</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-8.65</v>
+        <v>-7.05</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>底背离</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -3677,21 +3689,17 @@
         </is>
       </c>
       <c r="W21" s="2" t="n">
-        <v>159</v>
+        <v>25</v>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>4+</t>
-        </is>
-      </c>
-      <c r="Y21" s="2" t="inlineStr">
-        <is>
-          <t>周J超卖·日线纠缠</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr"/>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>4→4+·18d</t>
+          <t>4+→4·12d ← 4→4+·15d</t>
         </is>
       </c>
       <c r="AA21" s="2" t="inlineStr"/>
@@ -3699,35 +3707,31 @@
       <c r="AC21" s="2" t="inlineStr"/>
       <c r="AD21" s="2" t="inlineStr"/>
       <c r="AE21" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AF21" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="AF21" s="2" t="inlineStr"/>
       <c r="AG21" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AH21" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AH21" s="2" t="inlineStr"/>
       <c r="AI21" s="2" t="inlineStr"/>
       <c r="AJ21" s="2" t="n">
-        <v>-53.84</v>
+        <v>-29.17</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>-16.07</v>
+        <v>-4.4</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>-2.73</v>
+        <v>-3.25</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>4.43</v>
+        <v>1.37</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>13.8</v>
+        <v>-1</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="AP21" s="2" t="inlineStr"/>
       <c r="AQ21" s="2" t="inlineStr"/>
@@ -3735,62 +3739,62 @@
       <c r="AS21" s="2" t="inlineStr"/>
       <c r="AT21" s="2" t="inlineStr">
         <is>
-          <t>柱≥0</t>
+          <t>背离</t>
         </is>
       </c>
       <c r="AU21" s="2" t="n">
-        <v>0.985</v>
+        <v>1.647</v>
       </c>
       <c r="AV21" s="2" t="n">
-        <v>0.996</v>
+        <v>1.686</v>
       </c>
       <c r="AW21" s="2" t="n">
-        <v>1.006</v>
+        <v>1.73</v>
       </c>
       <c r="AX21" s="2" t="n">
-        <v>1.014</v>
+        <v>1.764</v>
       </c>
       <c r="AY21" s="2" t="n">
-        <v>1.052</v>
+        <v>1.798</v>
       </c>
       <c r="AZ21" s="2" t="n">
-        <v>1.067</v>
+        <v>1.804</v>
       </c>
       <c r="BA21" s="2" t="n">
-        <v>1.197</v>
+        <v>1.864</v>
       </c>
       <c r="BB21" s="2" t="n">
-        <v>-0.5883</v>
+        <v>-1.4449</v>
       </c>
       <c r="BC21" s="2" t="n">
-        <v>-0.3898</v>
+        <v>-1.0961</v>
       </c>
       <c r="BD21" s="2" t="n">
-        <v>-0.8827</v>
+        <v>-0.5371</v>
       </c>
       <c r="BE21" s="2" t="n">
-        <v>-0.4137</v>
+        <v>-0.1961</v>
       </c>
       <c r="BF21" s="2" t="n">
-        <v>-0.5384</v>
+        <v>-0.2917</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.59</v>
+        <v>2.243</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>-7.05</v>
+        <v>110.91</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -3799,7 +3803,9 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -3808,133 +3814,139 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010111010</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0010111000</t>
         </is>
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>24</v>
+        <v>133</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y22" s="2" t="inlineStr"/>
-      <c r="Z22" s="2" t="inlineStr">
-        <is>
-          <t>4+→4·11d ← 4→4+·14d</t>
-        </is>
-      </c>
+          <t>2C</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>周MACD死叉</t>
+        </is>
+      </c>
+      <c r="Z22" s="2" t="inlineStr"/>
       <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
       <c r="AD22" s="2" t="inlineStr"/>
-      <c r="AE22" s="2" t="n">
+      <c r="AE22" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="AF22" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="AF22" s="2" t="inlineStr"/>
       <c r="AG22" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="AH22" s="2" t="inlineStr"/>
       <c r="AI22" s="2" t="inlineStr"/>
       <c r="AJ22" s="2" t="n">
-        <v>-27.69</v>
+        <v>25.23</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>-4.89</v>
+        <v>25.37</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>-3.73</v>
+        <v>-5.26</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>7.79</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>-1</v>
+        <v>79.8</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="AP22" s="2" t="inlineStr"/>
       <c r="AQ22" s="2" t="inlineStr"/>
-      <c r="AR22" s="2" t="inlineStr"/>
+      <c r="AR22" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="AS22" s="2" t="inlineStr"/>
       <c r="AT22" s="2" t="inlineStr">
         <is>
-          <t>背离</t>
+          <t>柱≥0</t>
         </is>
       </c>
       <c r="AU22" s="2" t="n">
-        <v>1.665</v>
+        <v>2.299</v>
       </c>
       <c r="AV22" s="2" t="n">
-        <v>1.697</v>
+        <v>2.335</v>
       </c>
       <c r="AW22" s="2" t="n">
-        <v>1.737</v>
+        <v>2.331</v>
       </c>
       <c r="AX22" s="2" t="n">
-        <v>1.772</v>
+        <v>2.293</v>
       </c>
       <c r="AY22" s="2" t="n">
-        <v>1.802</v>
+        <v>2.265</v>
       </c>
       <c r="AZ22" s="2" t="n">
-        <v>1.806</v>
+        <v>2.224</v>
       </c>
       <c r="BA22" s="2" t="n">
-        <v>1.866</v>
+        <v>2.054</v>
       </c>
       <c r="BB22" s="2" t="n">
-        <v>-1.3228</v>
+        <v>-0.5669</v>
       </c>
       <c r="BC22" s="2" t="n">
-        <v>-1.0772</v>
+        <v>0.5286</v>
       </c>
       <c r="BD22" s="2" t="n">
-        <v>-0.4917</v>
+        <v>0.2552</v>
       </c>
       <c r="BE22" s="2" t="n">
-        <v>-0.1745</v>
+        <v>0.1423</v>
       </c>
       <c r="BF22" s="2" t="n">
-        <v>-0.2769</v>
+        <v>0.2523</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B23" s="2" 